<commit_message>
Faltantes: nota en gestion + confirmacion jefe deposito; sync_stock via reporte directo
- Faltantes: nota de contexto al pasar a en_gestion (textarea inline)
- Faltantes: boton Confirmar recepcion para jefe_deposito en tickets resueltos
- Faltantes: tickets confirmados desaparecen de vista activa (filtro confirmado_en IS NULL)
- Faltantes: nuevo endpoint PATCH /api/faltantes/<id>/confirmar
- Header app: safe-area-inset-top para iPhone con Dynamic Island/notch
- sync_stock.py: reescrito usando alm_articulospordeposito.aspx en vez de scraping HTML
- stock_data.json: actualizado con 694 articulos con stock

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1018" uniqueCount="1018">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1022" uniqueCount="1022">
   <si>
     <t>Código</t>
   </si>
@@ -1917,6 +1917,18 @@
   </si>
   <si>
     <t>LEVOFLOXACINA 500 MG RICHET FA - 990100234</t>
+  </si>
+  <si>
+    <t>000024674</t>
+  </si>
+  <si>
+    <t>LEVOFLOXACINA 500MG X 7 COMPR - DUNCAN - 000024674</t>
+  </si>
+  <si>
+    <t>000024675</t>
+  </si>
+  <si>
+    <t>LEVOFLOXACINA 750 MG X 5 COMPR - BIOTENK - 000024675</t>
   </si>
   <si>
     <t>000015662</t>
@@ -3124,7 +3136,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A3:D477"/>
+  <dimension ref="A3:D479"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="3">
@@ -4776,7 +4788,7 @@
         <v>273</v>
       </c>
       <c r="D120" s="0">
-        <v>415</v>
+        <v>520</v>
       </c>
     </row>
     <row r="121">
@@ -4790,7 +4802,7 @@
         <v>35</v>
       </c>
       <c r="D121" s="0">
-        <v>415</v>
+        <v>520</v>
       </c>
     </row>
     <row r="122">
@@ -5042,7 +5054,7 @@
         <v>69</v>
       </c>
       <c r="D139" s="0">
-        <v>660</v>
+        <v>700</v>
       </c>
     </row>
     <row r="140">
@@ -5056,7 +5068,7 @@
         <v>35</v>
       </c>
       <c r="D140" s="0">
-        <v>651</v>
+        <v>700</v>
       </c>
     </row>
     <row r="141">
@@ -5196,7 +5208,7 @@
         <v>29</v>
       </c>
       <c r="D150" s="0">
-        <v>86457</v>
+        <v>86457.1</v>
       </c>
     </row>
     <row r="151">
@@ -5210,7 +5222,7 @@
         <v>29</v>
       </c>
       <c r="D151" s="0">
-        <v>108071</v>
+        <v>108071.4</v>
       </c>
     </row>
     <row r="152">
@@ -5224,7 +5236,7 @@
         <v>343</v>
       </c>
       <c r="D152" s="0">
-        <v>500</v>
+        <v>570</v>
       </c>
     </row>
     <row r="153">
@@ -5252,7 +5264,7 @@
         <v>140</v>
       </c>
       <c r="D154" s="0">
-        <v>500</v>
+        <v>570</v>
       </c>
     </row>
     <row r="155">
@@ -5266,7 +5278,7 @@
         <v>16</v>
       </c>
       <c r="D155" s="0">
-        <v>550</v>
+        <v>570</v>
       </c>
     </row>
     <row r="156">
@@ -6372,7 +6384,7 @@
         <v>29</v>
       </c>
       <c r="D234" s="0">
-        <v>12090.4</v>
+        <v>12682.6</v>
       </c>
     </row>
     <row r="235">
@@ -7058,7 +7070,7 @@
         <v>29</v>
       </c>
       <c r="D283" s="0">
-        <v>5238.8</v>
+        <v>7086.15</v>
       </c>
     </row>
     <row r="284">
@@ -7181,10 +7193,10 @@
         <v>636</v>
       </c>
       <c r="C292" s="0" t="s">
-        <v>89</v>
+        <v>140</v>
       </c>
       <c r="D292" s="0">
-        <v>299475</v>
+        <v>896</v>
       </c>
     </row>
     <row r="293">
@@ -7195,10 +7207,10 @@
         <v>638</v>
       </c>
       <c r="C293" s="0" t="s">
-        <v>194</v>
+        <v>129</v>
       </c>
       <c r="D293" s="0">
-        <v>17440</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="294">
@@ -7209,10 +7221,10 @@
         <v>640</v>
       </c>
       <c r="C294" s="0" t="s">
-        <v>194</v>
+        <v>89</v>
       </c>
       <c r="D294" s="0">
-        <v>6000</v>
+        <v>299475</v>
       </c>
     </row>
     <row r="295">
@@ -7226,7 +7238,7 @@
         <v>194</v>
       </c>
       <c r="D295" s="0">
-        <v>4390</v>
+        <v>17440</v>
       </c>
     </row>
     <row r="296">
@@ -7237,10 +7249,10 @@
         <v>644</v>
       </c>
       <c r="C296" s="0" t="s">
-        <v>273</v>
+        <v>194</v>
       </c>
       <c r="D296" s="0">
-        <v>2250</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="297">
@@ -7254,7 +7266,7 @@
         <v>194</v>
       </c>
       <c r="D297" s="0">
-        <v>3355</v>
+        <v>4390</v>
       </c>
     </row>
     <row r="298">
@@ -7265,10 +7277,10 @@
         <v>648</v>
       </c>
       <c r="C298" s="0" t="s">
-        <v>199</v>
+        <v>273</v>
       </c>
       <c r="D298" s="0">
-        <v>7500</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="299">
@@ -7279,10 +7291,10 @@
         <v>650</v>
       </c>
       <c r="C299" s="0" t="s">
-        <v>89</v>
+        <v>194</v>
       </c>
       <c r="D299" s="0">
-        <v>23958</v>
+        <v>3355</v>
       </c>
     </row>
     <row r="300">
@@ -7293,10 +7305,10 @@
         <v>652</v>
       </c>
       <c r="C300" s="0" t="s">
-        <v>89</v>
+        <v>199</v>
       </c>
       <c r="D300" s="0">
-        <v>239580</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="301">
@@ -7307,10 +7319,10 @@
         <v>654</v>
       </c>
       <c r="C301" s="0" t="s">
-        <v>51</v>
+        <v>89</v>
       </c>
       <c r="D301" s="0">
-        <v>130</v>
+        <v>23958</v>
       </c>
     </row>
     <row r="302">
@@ -7321,10 +7333,10 @@
         <v>656</v>
       </c>
       <c r="C302" s="0" t="s">
-        <v>22</v>
+        <v>89</v>
       </c>
       <c r="D302" s="0">
-        <v>285.6</v>
+        <v>239580</v>
       </c>
     </row>
     <row r="303">
@@ -7335,10 +7347,10 @@
         <v>658</v>
       </c>
       <c r="C303" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="D303" s="0">
-        <v>338</v>
+        <v>130</v>
       </c>
     </row>
     <row r="304">
@@ -7349,52 +7361,52 @@
         <v>660</v>
       </c>
       <c r="C304" s="0" t="s">
-        <v>661</v>
+        <v>22</v>
       </c>
       <c r="D304" s="0">
-        <v>770</v>
+        <v>285.6</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="0" t="s">
+        <v>661</v>
+      </c>
+      <c r="B305" s="0" t="s">
         <v>662</v>
       </c>
-      <c r="B305" s="0" t="s">
-        <v>663</v>
-      </c>
       <c r="C305" s="0" t="s">
-        <v>664</v>
+        <v>22</v>
       </c>
       <c r="D305" s="0">
-        <v>770</v>
+        <v>338</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="0" t="s">
+        <v>663</v>
+      </c>
+      <c r="B306" s="0" t="s">
+        <v>664</v>
+      </c>
+      <c r="C306" s="0" t="s">
         <v>665</v>
       </c>
-      <c r="B306" s="0" t="s">
-        <v>666</v>
-      </c>
-      <c r="C306" s="0" t="s">
-        <v>16</v>
-      </c>
       <c r="D306" s="0">
-        <v>780</v>
+        <v>770</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="0" t="s">
+        <v>666</v>
+      </c>
+      <c r="B307" s="0" t="s">
         <v>667</v>
       </c>
-      <c r="B307" s="0" t="s">
+      <c r="C307" s="0" t="s">
         <v>668</v>
       </c>
-      <c r="C307" s="0" t="s">
-        <v>22</v>
-      </c>
       <c r="D307" s="0">
-        <v>507.08</v>
+        <v>770</v>
       </c>
     </row>
     <row r="308">
@@ -7408,7 +7420,7 @@
         <v>16</v>
       </c>
       <c r="D308" s="0">
-        <v>450</v>
+        <v>780</v>
       </c>
     </row>
     <row r="309">
@@ -7419,10 +7431,10 @@
         <v>672</v>
       </c>
       <c r="C309" s="0" t="s">
-        <v>140</v>
+        <v>22</v>
       </c>
       <c r="D309" s="0">
-        <v>760</v>
+        <v>507.08</v>
       </c>
     </row>
     <row r="310">
@@ -7433,10 +7445,10 @@
         <v>674</v>
       </c>
       <c r="C310" s="0" t="s">
-        <v>273</v>
+        <v>16</v>
       </c>
       <c r="D310" s="0">
-        <v>5900</v>
+        <v>450</v>
       </c>
     </row>
     <row r="311">
@@ -7447,10 +7459,10 @@
         <v>676</v>
       </c>
       <c r="C311" s="0" t="s">
-        <v>273</v>
+        <v>140</v>
       </c>
       <c r="D311" s="0">
-        <v>2900</v>
+        <v>760</v>
       </c>
     </row>
     <row r="312">
@@ -7461,10 +7473,10 @@
         <v>678</v>
       </c>
       <c r="C312" s="0" t="s">
-        <v>129</v>
+        <v>273</v>
       </c>
       <c r="D312" s="0">
-        <v>797.4</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="313">
@@ -7475,10 +7487,10 @@
         <v>680</v>
       </c>
       <c r="C313" s="0" t="s">
-        <v>129</v>
+        <v>273</v>
       </c>
       <c r="D313" s="0">
-        <v>519</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="314">
@@ -7492,7 +7504,7 @@
         <v>129</v>
       </c>
       <c r="D314" s="0">
-        <v>62</v>
+        <v>797.4</v>
       </c>
     </row>
     <row r="315">
@@ -7503,10 +7515,10 @@
         <v>684</v>
       </c>
       <c r="C315" s="0" t="s">
-        <v>89</v>
+        <v>129</v>
       </c>
       <c r="D315" s="0">
-        <v>11313.5</v>
+        <v>519</v>
       </c>
     </row>
     <row r="316">
@@ -7517,10 +7529,10 @@
         <v>686</v>
       </c>
       <c r="C316" s="0" t="s">
-        <v>35</v>
+        <v>129</v>
       </c>
       <c r="D316" s="0">
-        <v>418</v>
+        <v>62</v>
       </c>
     </row>
     <row r="317">
@@ -7531,10 +7543,10 @@
         <v>688</v>
       </c>
       <c r="C317" s="0" t="s">
-        <v>343</v>
+        <v>89</v>
       </c>
       <c r="D317" s="0">
-        <v>418</v>
+        <v>11313.5</v>
       </c>
     </row>
     <row r="318">
@@ -7545,10 +7557,10 @@
         <v>690</v>
       </c>
       <c r="C318" s="0" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="D318" s="0">
-        <v>377</v>
+        <v>418</v>
       </c>
     </row>
     <row r="319">
@@ -7559,10 +7571,10 @@
         <v>692</v>
       </c>
       <c r="C319" s="0" t="s">
-        <v>44</v>
+        <v>343</v>
       </c>
       <c r="D319" s="0">
-        <v>3860.67</v>
+        <v>418</v>
       </c>
     </row>
     <row r="320">
@@ -7573,10 +7585,10 @@
         <v>694</v>
       </c>
       <c r="C320" s="0" t="s">
-        <v>69</v>
+        <v>22</v>
       </c>
       <c r="D320" s="0">
-        <v>898</v>
+        <v>377</v>
       </c>
     </row>
     <row r="321">
@@ -7587,10 +7599,10 @@
         <v>696</v>
       </c>
       <c r="C321" s="0" t="s">
-        <v>115</v>
+        <v>44</v>
       </c>
       <c r="D321" s="0">
-        <v>4767</v>
+        <v>3860.67</v>
       </c>
     </row>
     <row r="322">
@@ -7601,10 +7613,10 @@
         <v>698</v>
       </c>
       <c r="C322" s="0" t="s">
-        <v>35</v>
+        <v>69</v>
       </c>
       <c r="D322" s="0">
-        <v>650</v>
+        <v>898</v>
       </c>
     </row>
     <row r="323">
@@ -7615,10 +7627,10 @@
         <v>700</v>
       </c>
       <c r="C323" s="0" t="s">
-        <v>69</v>
+        <v>115</v>
       </c>
       <c r="D323" s="0">
-        <v>650</v>
+        <v>4767</v>
       </c>
     </row>
     <row r="324">
@@ -7629,10 +7641,10 @@
         <v>702</v>
       </c>
       <c r="C324" s="0" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D324" s="0">
-        <v>1900</v>
+        <v>650</v>
       </c>
     </row>
     <row r="325">
@@ -7643,10 +7655,10 @@
         <v>704</v>
       </c>
       <c r="C325" s="0" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="D325" s="0">
-        <v>8318.75</v>
+        <v>650</v>
       </c>
     </row>
     <row r="326">
@@ -7657,38 +7669,38 @@
         <v>706</v>
       </c>
       <c r="C326" s="0" t="s">
-        <v>707</v>
+        <v>16</v>
       </c>
       <c r="D326" s="0">
-        <v>1800</v>
+        <v>1900</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="0" t="s">
+        <v>707</v>
+      </c>
+      <c r="B327" s="0" t="s">
         <v>708</v>
       </c>
-      <c r="B327" s="0" t="s">
-        <v>709</v>
-      </c>
       <c r="C327" s="0" t="s">
-        <v>140</v>
+        <v>89</v>
       </c>
       <c r="D327" s="0">
-        <v>900</v>
+        <v>8318.75</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="0" t="s">
+        <v>709</v>
+      </c>
+      <c r="B328" s="0" t="s">
         <v>710</v>
       </c>
-      <c r="B328" s="0" t="s">
+      <c r="C328" s="0" t="s">
         <v>711</v>
       </c>
-      <c r="C328" s="0" t="s">
-        <v>22</v>
-      </c>
       <c r="D328" s="0">
-        <v>1722</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="329">
@@ -7699,10 +7711,10 @@
         <v>713</v>
       </c>
       <c r="C329" s="0" t="s">
-        <v>35</v>
+        <v>140</v>
       </c>
       <c r="D329" s="0">
-        <v>456</v>
+        <v>900</v>
       </c>
     </row>
     <row r="330">
@@ -7713,10 +7725,10 @@
         <v>715</v>
       </c>
       <c r="C330" s="0" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="D330" s="0">
-        <v>45600</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="331">
@@ -7727,10 +7739,10 @@
         <v>717</v>
       </c>
       <c r="C331" s="0" t="s">
-        <v>140</v>
+        <v>35</v>
       </c>
       <c r="D331" s="0">
-        <v>1212</v>
+        <v>456</v>
       </c>
     </row>
     <row r="332">
@@ -7741,10 +7753,10 @@
         <v>719</v>
       </c>
       <c r="C332" s="0" t="s">
-        <v>140</v>
+        <v>35</v>
       </c>
       <c r="D332" s="0">
-        <v>1300</v>
+        <v>45600</v>
       </c>
     </row>
     <row r="333">
@@ -7758,7 +7770,7 @@
         <v>140</v>
       </c>
       <c r="D333" s="0">
-        <v>1500</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="334">
@@ -7772,7 +7784,7 @@
         <v>140</v>
       </c>
       <c r="D334" s="0">
-        <v>1400</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="335">
@@ -7783,10 +7795,10 @@
         <v>725</v>
       </c>
       <c r="C335" s="0" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="D335" s="0">
-        <v>300</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="336">
@@ -7797,10 +7809,10 @@
         <v>727</v>
       </c>
       <c r="C336" s="0" t="s">
-        <v>273</v>
+        <v>140</v>
       </c>
       <c r="D336" s="0">
-        <v>1450</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="337">
@@ -7811,10 +7823,10 @@
         <v>729</v>
       </c>
       <c r="C337" s="0" t="s">
-        <v>89</v>
+        <v>129</v>
       </c>
       <c r="D337" s="0">
-        <v>7986</v>
+        <v>300</v>
       </c>
     </row>
     <row r="338">
@@ -7825,10 +7837,10 @@
         <v>731</v>
       </c>
       <c r="C338" s="0" t="s">
-        <v>16</v>
+        <v>273</v>
       </c>
       <c r="D338" s="0">
-        <v>900</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="339">
@@ -7839,10 +7851,10 @@
         <v>733</v>
       </c>
       <c r="C339" s="0" t="s">
-        <v>273</v>
+        <v>89</v>
       </c>
       <c r="D339" s="0">
-        <v>520</v>
+        <v>7986</v>
       </c>
     </row>
     <row r="340">
@@ -7853,10 +7865,10 @@
         <v>735</v>
       </c>
       <c r="C340" s="0" t="s">
-        <v>458</v>
+        <v>16</v>
       </c>
       <c r="D340" s="0">
-        <v>64925</v>
+        <v>900</v>
       </c>
     </row>
     <row r="341">
@@ -7867,10 +7879,10 @@
         <v>737</v>
       </c>
       <c r="C341" s="0" t="s">
-        <v>16</v>
+        <v>273</v>
       </c>
       <c r="D341" s="0">
-        <v>1000</v>
+        <v>520</v>
       </c>
     </row>
     <row r="342">
@@ -7881,10 +7893,10 @@
         <v>739</v>
       </c>
       <c r="C342" s="0" t="s">
-        <v>22</v>
+        <v>458</v>
       </c>
       <c r="D342" s="0">
-        <v>1623</v>
+        <v>64925</v>
       </c>
     </row>
     <row r="343">
@@ -7895,10 +7907,10 @@
         <v>741</v>
       </c>
       <c r="C343" s="0" t="s">
-        <v>129</v>
+        <v>16</v>
       </c>
       <c r="D343" s="0">
-        <v>1116.03</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="344">
@@ -7909,10 +7921,10 @@
         <v>743</v>
       </c>
       <c r="C344" s="0" t="s">
-        <v>129</v>
+        <v>22</v>
       </c>
       <c r="D344" s="0">
-        <v>4028.88</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="345">
@@ -7923,10 +7935,10 @@
         <v>745</v>
       </c>
       <c r="C345" s="0" t="s">
-        <v>29</v>
+        <v>129</v>
       </c>
       <c r="D345" s="0">
-        <v>1869</v>
+        <v>1116.03</v>
       </c>
     </row>
     <row r="346">
@@ -7937,10 +7949,10 @@
         <v>747</v>
       </c>
       <c r="C346" s="0" t="s">
-        <v>16</v>
+        <v>129</v>
       </c>
       <c r="D346" s="0">
-        <v>420</v>
+        <v>4028.88</v>
       </c>
     </row>
     <row r="347">
@@ -7951,10 +7963,10 @@
         <v>749</v>
       </c>
       <c r="C347" s="0" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="D347" s="0">
-        <v>750</v>
+        <v>1869.6</v>
       </c>
     </row>
     <row r="348">
@@ -7968,7 +7980,7 @@
         <v>16</v>
       </c>
       <c r="D348" s="0">
-        <v>750</v>
+        <v>420</v>
       </c>
     </row>
     <row r="349">
@@ -7979,10 +7991,10 @@
         <v>753</v>
       </c>
       <c r="C349" s="0" t="s">
-        <v>362</v>
+        <v>16</v>
       </c>
       <c r="D349" s="0">
-        <v>134775.6</v>
+        <v>750</v>
       </c>
     </row>
     <row r="350">
@@ -7993,10 +8005,10 @@
         <v>755</v>
       </c>
       <c r="C350" s="0" t="s">
-        <v>362</v>
+        <v>16</v>
       </c>
       <c r="D350" s="0">
-        <v>175991.55</v>
+        <v>750</v>
       </c>
     </row>
     <row r="351">
@@ -8007,10 +8019,10 @@
         <v>757</v>
       </c>
       <c r="C351" s="0" t="s">
-        <v>69</v>
+        <v>362</v>
       </c>
       <c r="D351" s="0">
-        <v>3263</v>
+        <v>134775.6</v>
       </c>
     </row>
     <row r="352">
@@ -8021,10 +8033,10 @@
         <v>759</v>
       </c>
       <c r="C352" s="0" t="s">
-        <v>69</v>
+        <v>362</v>
       </c>
       <c r="D352" s="0">
-        <v>18027</v>
+        <v>175991.55</v>
       </c>
     </row>
     <row r="353">
@@ -8035,10 +8047,10 @@
         <v>761</v>
       </c>
       <c r="C353" s="0" t="s">
-        <v>273</v>
+        <v>69</v>
       </c>
       <c r="D353" s="0">
-        <v>515</v>
+        <v>3263</v>
       </c>
     </row>
     <row r="354">
@@ -8049,10 +8061,10 @@
         <v>763</v>
       </c>
       <c r="C354" s="0" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="D354" s="0">
-        <v>515</v>
+        <v>18027</v>
       </c>
     </row>
     <row r="355">
@@ -8063,10 +8075,10 @@
         <v>765</v>
       </c>
       <c r="C355" s="0" t="s">
-        <v>41</v>
+        <v>273</v>
       </c>
       <c r="D355" s="0">
-        <v>10154</v>
+        <v>515</v>
       </c>
     </row>
     <row r="356">
@@ -8077,10 +8089,10 @@
         <v>767</v>
       </c>
       <c r="C356" s="0" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="D356" s="0">
-        <v>9500</v>
+        <v>515</v>
       </c>
     </row>
     <row r="357">
@@ -8091,10 +8103,10 @@
         <v>769</v>
       </c>
       <c r="C357" s="0" t="s">
-        <v>458</v>
+        <v>41</v>
       </c>
       <c r="D357" s="0">
-        <v>207600</v>
+        <v>10154</v>
       </c>
     </row>
     <row r="358">
@@ -8105,10 +8117,10 @@
         <v>771</v>
       </c>
       <c r="C358" s="0" t="s">
-        <v>458</v>
+        <v>51</v>
       </c>
       <c r="D358" s="0">
-        <v>249000</v>
+        <v>9500</v>
       </c>
     </row>
     <row r="359">
@@ -8119,10 +8131,10 @@
         <v>773</v>
       </c>
       <c r="C359" s="0" t="s">
-        <v>69</v>
+        <v>458</v>
       </c>
       <c r="D359" s="0">
-        <v>10021.22</v>
+        <v>207600</v>
       </c>
     </row>
     <row r="360">
@@ -8133,10 +8145,10 @@
         <v>775</v>
       </c>
       <c r="C360" s="0" t="s">
-        <v>69</v>
+        <v>458</v>
       </c>
       <c r="D360" s="0">
-        <v>17710</v>
+        <v>249000</v>
       </c>
     </row>
     <row r="361">
@@ -8147,66 +8159,66 @@
         <v>777</v>
       </c>
       <c r="C361" s="0" t="s">
-        <v>778</v>
+        <v>69</v>
       </c>
       <c r="D361" s="0">
-        <v>1080</v>
+        <v>10021.22</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="0" t="s">
+        <v>778</v>
+      </c>
+      <c r="B362" s="0" t="s">
         <v>779</v>
       </c>
-      <c r="B362" s="0" t="s">
-        <v>780</v>
-      </c>
       <c r="C362" s="0" t="s">
-        <v>19</v>
+        <v>69</v>
       </c>
       <c r="D362" s="0">
-        <v>691</v>
+        <v>17710</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="0" t="s">
+        <v>780</v>
+      </c>
+      <c r="B363" s="0" t="s">
         <v>781</v>
       </c>
-      <c r="B363" s="0" t="s">
+      <c r="C363" s="0" t="s">
         <v>782</v>
       </c>
-      <c r="C363" s="0" t="s">
-        <v>783</v>
-      </c>
       <c r="D363" s="0">
-        <v>520</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="0" t="s">
+        <v>783</v>
+      </c>
+      <c r="B364" s="0" t="s">
         <v>784</v>
       </c>
-      <c r="B364" s="0" t="s">
-        <v>785</v>
-      </c>
       <c r="C364" s="0" t="s">
-        <v>783</v>
+        <v>19</v>
       </c>
       <c r="D364" s="0">
-        <v>300</v>
+        <v>691</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="0" t="s">
+        <v>785</v>
+      </c>
+      <c r="B365" s="0" t="s">
         <v>786</v>
       </c>
-      <c r="B365" s="0" t="s">
+      <c r="C365" s="0" t="s">
         <v>787</v>
       </c>
-      <c r="C365" s="0" t="s">
-        <v>16</v>
-      </c>
       <c r="D365" s="0">
-        <v>2200</v>
+        <v>520</v>
       </c>
     </row>
     <row r="366">
@@ -8217,10 +8229,10 @@
         <v>789</v>
       </c>
       <c r="C366" s="0" t="s">
-        <v>16</v>
+        <v>787</v>
       </c>
       <c r="D366" s="0">
-        <v>2500</v>
+        <v>300</v>
       </c>
     </row>
     <row r="367">
@@ -8231,10 +8243,10 @@
         <v>791</v>
       </c>
       <c r="C367" s="0" t="s">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="D367" s="0">
-        <v>4791.6</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="368">
@@ -8245,10 +8257,10 @@
         <v>793</v>
       </c>
       <c r="C368" s="0" t="s">
-        <v>69</v>
+        <v>16</v>
       </c>
       <c r="D368" s="0">
-        <v>2699.64</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="369">
@@ -8259,10 +8271,10 @@
         <v>795</v>
       </c>
       <c r="C369" s="0" t="s">
-        <v>35</v>
+        <v>89</v>
       </c>
       <c r="D369" s="0">
-        <v>3800</v>
+        <v>4791.6</v>
       </c>
     </row>
     <row r="370">
@@ -8273,10 +8285,10 @@
         <v>797</v>
       </c>
       <c r="C370" s="0" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="D370" s="0">
-        <v>4000</v>
+        <v>2699.64</v>
       </c>
     </row>
     <row r="371">
@@ -8287,7 +8299,7 @@
         <v>799</v>
       </c>
       <c r="C371" s="0" t="s">
-        <v>800</v>
+        <v>35</v>
       </c>
       <c r="D371" s="0">
         <v>3800</v>
@@ -8295,30 +8307,30 @@
     </row>
     <row r="372">
       <c r="A372" s="0" t="s">
+        <v>800</v>
+      </c>
+      <c r="B372" s="0" t="s">
         <v>801</v>
       </c>
-      <c r="B372" s="0" t="s">
-        <v>802</v>
-      </c>
       <c r="C372" s="0" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D372" s="0">
-        <v>353</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="0" t="s">
+        <v>802</v>
+      </c>
+      <c r="B373" s="0" t="s">
         <v>803</v>
       </c>
-      <c r="B373" s="0" t="s">
+      <c r="C373" s="0" t="s">
         <v>804</v>
       </c>
-      <c r="C373" s="0" t="s">
-        <v>346</v>
-      </c>
       <c r="D373" s="0">
-        <v>1800</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="374">
@@ -8329,10 +8341,10 @@
         <v>806</v>
       </c>
       <c r="C374" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D374" s="0">
-        <v>2100</v>
+        <v>353</v>
       </c>
     </row>
     <row r="375">
@@ -8343,10 +8355,10 @@
         <v>808</v>
       </c>
       <c r="C375" s="0" t="s">
-        <v>199</v>
+        <v>346</v>
       </c>
       <c r="D375" s="0">
-        <v>65537</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="376">
@@ -8357,10 +8369,10 @@
         <v>810</v>
       </c>
       <c r="C376" s="0" t="s">
-        <v>129</v>
+        <v>16</v>
       </c>
       <c r="D376" s="0">
-        <v>3820.86</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="377">
@@ -8371,10 +8383,10 @@
         <v>812</v>
       </c>
       <c r="C377" s="0" t="s">
-        <v>129</v>
+        <v>199</v>
       </c>
       <c r="D377" s="0">
-        <v>3962</v>
+        <v>65537</v>
       </c>
     </row>
     <row r="378">
@@ -8388,7 +8400,7 @@
         <v>129</v>
       </c>
       <c r="D378" s="0">
-        <v>5802.4</v>
+        <v>3820.86</v>
       </c>
     </row>
     <row r="379">
@@ -8399,10 +8411,10 @@
         <v>816</v>
       </c>
       <c r="C379" s="0" t="s">
-        <v>300</v>
+        <v>129</v>
       </c>
       <c r="D379" s="0">
-        <v>570</v>
+        <v>3962</v>
       </c>
     </row>
     <row r="380">
@@ -8413,10 +8425,10 @@
         <v>818</v>
       </c>
       <c r="C380" s="0" t="s">
-        <v>69</v>
+        <v>129</v>
       </c>
       <c r="D380" s="0">
-        <v>550</v>
+        <v>5802.4</v>
       </c>
     </row>
     <row r="381">
@@ -8427,10 +8439,10 @@
         <v>820</v>
       </c>
       <c r="C381" s="0" t="s">
-        <v>51</v>
+        <v>300</v>
       </c>
       <c r="D381" s="0">
-        <v>167</v>
+        <v>570</v>
       </c>
     </row>
     <row r="382">
@@ -8441,10 +8453,10 @@
         <v>822</v>
       </c>
       <c r="C382" s="0" t="s">
-        <v>29</v>
+        <v>69</v>
       </c>
       <c r="D382" s="0">
-        <v>586.2</v>
+        <v>550</v>
       </c>
     </row>
     <row r="383">
@@ -8455,10 +8467,10 @@
         <v>824</v>
       </c>
       <c r="C383" s="0" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="D383" s="0">
-        <v>101000</v>
+        <v>167</v>
       </c>
     </row>
     <row r="384">
@@ -8469,10 +8481,10 @@
         <v>826</v>
       </c>
       <c r="C384" s="0" t="s">
-        <v>115</v>
+        <v>29</v>
       </c>
       <c r="D384" s="0">
-        <v>6251</v>
+        <v>686.98</v>
       </c>
     </row>
     <row r="385">
@@ -8483,10 +8495,10 @@
         <v>828</v>
       </c>
       <c r="C385" s="0" t="s">
-        <v>89</v>
+        <v>58</v>
       </c>
       <c r="D385" s="0">
-        <v>1166</v>
+        <v>101000</v>
       </c>
     </row>
     <row r="386">
@@ -8497,10 +8509,10 @@
         <v>830</v>
       </c>
       <c r="C386" s="0" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="D386" s="0">
-        <v>360</v>
+        <v>6251</v>
       </c>
     </row>
     <row r="387">
@@ -8511,10 +8523,10 @@
         <v>832</v>
       </c>
       <c r="C387" s="0" t="s">
-        <v>140</v>
+        <v>89</v>
       </c>
       <c r="D387" s="0">
-        <v>450</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="388">
@@ -8528,7 +8540,7 @@
         <v>140</v>
       </c>
       <c r="D388" s="0">
-        <v>2050</v>
+        <v>360</v>
       </c>
     </row>
     <row r="389">
@@ -8539,10 +8551,10 @@
         <v>836</v>
       </c>
       <c r="C389" s="0" t="s">
-        <v>559</v>
+        <v>140</v>
       </c>
       <c r="D389" s="0">
-        <v>25192.82</v>
+        <v>450</v>
       </c>
     </row>
     <row r="390">
@@ -8553,10 +8565,10 @@
         <v>838</v>
       </c>
       <c r="C390" s="0" t="s">
-        <v>69</v>
+        <v>140</v>
       </c>
       <c r="D390" s="0">
-        <v>3500</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="391">
@@ -8567,10 +8579,10 @@
         <v>840</v>
       </c>
       <c r="C391" s="0" t="s">
-        <v>167</v>
+        <v>559</v>
       </c>
       <c r="D391" s="0">
-        <v>600</v>
+        <v>25192.82</v>
       </c>
     </row>
     <row r="392">
@@ -8581,38 +8593,38 @@
         <v>842</v>
       </c>
       <c r="C392" s="0" t="s">
-        <v>843</v>
+        <v>69</v>
       </c>
       <c r="D392" s="0">
-        <v>1080</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="0" t="s">
+        <v>843</v>
+      </c>
+      <c r="B393" s="0" t="s">
         <v>844</v>
       </c>
-      <c r="B393" s="0" t="s">
-        <v>845</v>
-      </c>
       <c r="C393" s="0" t="s">
-        <v>322</v>
+        <v>167</v>
       </c>
       <c r="D393" s="0">
-        <v>8628</v>
+        <v>600</v>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="0" t="s">
+        <v>845</v>
+      </c>
+      <c r="B394" s="0" t="s">
         <v>846</v>
       </c>
-      <c r="B394" s="0" t="s">
+      <c r="C394" s="0" t="s">
         <v>847</v>
       </c>
-      <c r="C394" s="0" t="s">
-        <v>322</v>
-      </c>
       <c r="D394" s="0">
-        <v>9125</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="395">
@@ -8623,10 +8635,10 @@
         <v>849</v>
       </c>
       <c r="C395" s="0" t="s">
-        <v>129</v>
+        <v>322</v>
       </c>
       <c r="D395" s="0">
-        <v>1080</v>
+        <v>8628</v>
       </c>
     </row>
     <row r="396">
@@ -8637,10 +8649,10 @@
         <v>851</v>
       </c>
       <c r="C396" s="0" t="s">
-        <v>129</v>
+        <v>322</v>
       </c>
       <c r="D396" s="0">
-        <v>4500</v>
+        <v>9125</v>
       </c>
     </row>
     <row r="397">
@@ -8651,10 +8663,10 @@
         <v>853</v>
       </c>
       <c r="C397" s="0" t="s">
-        <v>44</v>
+        <v>129</v>
       </c>
       <c r="D397" s="0">
-        <v>4194.88</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="398">
@@ -8665,10 +8677,10 @@
         <v>855</v>
       </c>
       <c r="C398" s="0" t="s">
-        <v>44</v>
+        <v>129</v>
       </c>
       <c r="D398" s="0">
-        <v>2139.28</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="399">
@@ -8682,7 +8694,7 @@
         <v>44</v>
       </c>
       <c r="D399" s="0">
-        <v>1699.1</v>
+        <v>4194.88</v>
       </c>
     </row>
     <row r="400">
@@ -8696,7 +8708,7 @@
         <v>44</v>
       </c>
       <c r="D400" s="0">
-        <v>3427.58</v>
+        <v>2139.28</v>
       </c>
     </row>
     <row r="401">
@@ -8710,7 +8722,7 @@
         <v>44</v>
       </c>
       <c r="D401" s="0">
-        <v>19700</v>
+        <v>1699.1</v>
       </c>
     </row>
     <row r="402">
@@ -8724,7 +8736,7 @@
         <v>44</v>
       </c>
       <c r="D402" s="0">
-        <v>1839.2</v>
+        <v>3427.58</v>
       </c>
     </row>
     <row r="403">
@@ -8738,7 +8750,7 @@
         <v>44</v>
       </c>
       <c r="D403" s="0">
-        <v>4215.45</v>
+        <v>19700</v>
       </c>
     </row>
     <row r="404">
@@ -8752,7 +8764,7 @@
         <v>44</v>
       </c>
       <c r="D404" s="0">
-        <v>3395.26</v>
+        <v>1839.2</v>
       </c>
     </row>
     <row r="405">
@@ -8763,10 +8775,10 @@
         <v>869</v>
       </c>
       <c r="C405" s="0" t="s">
-        <v>467</v>
+        <v>44</v>
       </c>
       <c r="D405" s="0">
-        <v>510</v>
+        <v>4215.45</v>
       </c>
     </row>
     <row r="406">
@@ -8777,10 +8789,10 @@
         <v>871</v>
       </c>
       <c r="C406" s="0" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D406" s="0">
-        <v>510</v>
+        <v>3395.26</v>
       </c>
     </row>
     <row r="407">
@@ -8791,35 +8803,35 @@
         <v>873</v>
       </c>
       <c r="C407" s="0" t="s">
-        <v>874</v>
+        <v>467</v>
       </c>
       <c r="D407" s="0">
-        <v>559</v>
+        <v>510</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="0" t="s">
+        <v>874</v>
+      </c>
+      <c r="B408" s="0" t="s">
         <v>875</v>
       </c>
-      <c r="B408" s="0" t="s">
-        <v>876</v>
-      </c>
       <c r="C408" s="0" t="s">
-        <v>874</v>
+        <v>38</v>
       </c>
       <c r="D408" s="0">
-        <v>559</v>
+        <v>510</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="0" t="s">
+        <v>876</v>
+      </c>
+      <c r="B409" s="0" t="s">
         <v>877</v>
       </c>
-      <c r="B409" s="0" t="s">
+      <c r="C409" s="0" t="s">
         <v>878</v>
-      </c>
-      <c r="C409" s="0" t="s">
-        <v>874</v>
       </c>
       <c r="D409" s="0">
         <v>559</v>
@@ -8833,10 +8845,10 @@
         <v>880</v>
       </c>
       <c r="C410" s="0" t="s">
-        <v>874</v>
+        <v>878</v>
       </c>
       <c r="D410" s="0">
-        <v>342</v>
+        <v>559</v>
       </c>
     </row>
     <row r="411">
@@ -8847,10 +8859,10 @@
         <v>882</v>
       </c>
       <c r="C411" s="0" t="s">
-        <v>874</v>
+        <v>878</v>
       </c>
       <c r="D411" s="0">
-        <v>342</v>
+        <v>559</v>
       </c>
     </row>
     <row r="412">
@@ -8861,7 +8873,7 @@
         <v>884</v>
       </c>
       <c r="C412" s="0" t="s">
-        <v>874</v>
+        <v>878</v>
       </c>
       <c r="D412" s="0">
         <v>342</v>
@@ -8875,10 +8887,10 @@
         <v>886</v>
       </c>
       <c r="C413" s="0" t="s">
-        <v>874</v>
+        <v>878</v>
       </c>
       <c r="D413" s="0">
-        <v>0</v>
+        <v>342</v>
       </c>
     </row>
     <row r="414">
@@ -8889,10 +8901,10 @@
         <v>888</v>
       </c>
       <c r="C414" s="0" t="s">
-        <v>874</v>
+        <v>878</v>
       </c>
       <c r="D414" s="0">
-        <v>0</v>
+        <v>342</v>
       </c>
     </row>
     <row r="415">
@@ -8903,10 +8915,10 @@
         <v>890</v>
       </c>
       <c r="C415" s="0" t="s">
-        <v>874</v>
+        <v>878</v>
       </c>
       <c r="D415" s="0">
-        <v>423</v>
+        <v>0</v>
       </c>
     </row>
     <row r="416">
@@ -8917,10 +8929,10 @@
         <v>892</v>
       </c>
       <c r="C416" s="0" t="s">
-        <v>69</v>
+        <v>878</v>
       </c>
       <c r="D416" s="0">
-        <v>15968</v>
+        <v>0</v>
       </c>
     </row>
     <row r="417">
@@ -8931,10 +8943,10 @@
         <v>894</v>
       </c>
       <c r="C417" s="0" t="s">
-        <v>109</v>
+        <v>878</v>
       </c>
       <c r="D417" s="0">
-        <v>14000</v>
+        <v>423</v>
       </c>
     </row>
     <row r="418">
@@ -8945,10 +8957,10 @@
         <v>896</v>
       </c>
       <c r="C418" s="0" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="D418" s="0">
-        <v>266200</v>
+        <v>15968</v>
       </c>
     </row>
     <row r="419">
@@ -8959,10 +8971,10 @@
         <v>898</v>
       </c>
       <c r="C419" s="0" t="s">
-        <v>89</v>
+        <v>109</v>
       </c>
       <c r="D419" s="0">
-        <v>194991.5</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="420">
@@ -8976,7 +8988,7 @@
         <v>89</v>
       </c>
       <c r="D420" s="0">
-        <v>289492.5</v>
+        <v>266200</v>
       </c>
     </row>
     <row r="421">
@@ -8987,38 +8999,38 @@
         <v>902</v>
       </c>
       <c r="C421" s="0" t="s">
-        <v>903</v>
+        <v>89</v>
       </c>
       <c r="D421" s="0">
-        <v>13722</v>
+        <v>194991.5</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="0" t="s">
+        <v>903</v>
+      </c>
+      <c r="B422" s="0" t="s">
         <v>904</v>
       </c>
-      <c r="B422" s="0" t="s">
-        <v>905</v>
-      </c>
       <c r="C422" s="0" t="s">
-        <v>903</v>
+        <v>89</v>
       </c>
       <c r="D422" s="0">
-        <v>15072</v>
+        <v>289492.5</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="0" t="s">
+        <v>905</v>
+      </c>
+      <c r="B423" s="0" t="s">
         <v>906</v>
       </c>
-      <c r="B423" s="0" t="s">
+      <c r="C423" s="0" t="s">
         <v>907</v>
       </c>
-      <c r="C423" s="0" t="s">
-        <v>903</v>
-      </c>
       <c r="D423" s="0">
-        <v>6555</v>
+        <v>13722</v>
       </c>
     </row>
     <row r="424">
@@ -9029,10 +9041,10 @@
         <v>909</v>
       </c>
       <c r="C424" s="0" t="s">
-        <v>903</v>
+        <v>907</v>
       </c>
       <c r="D424" s="0">
-        <v>8964.61</v>
+        <v>15072</v>
       </c>
     </row>
     <row r="425">
@@ -9043,10 +9055,10 @@
         <v>911</v>
       </c>
       <c r="C425" s="0" t="s">
-        <v>903</v>
+        <v>907</v>
       </c>
       <c r="D425" s="0">
-        <v>11735</v>
+        <v>6555</v>
       </c>
     </row>
     <row r="426">
@@ -9057,10 +9069,10 @@
         <v>913</v>
       </c>
       <c r="C426" s="0" t="s">
-        <v>69</v>
+        <v>907</v>
       </c>
       <c r="D426" s="0">
-        <v>3380</v>
+        <v>8964.61</v>
       </c>
     </row>
     <row r="427">
@@ -9071,10 +9083,10 @@
         <v>915</v>
       </c>
       <c r="C427" s="0" t="s">
-        <v>129</v>
+        <v>907</v>
       </c>
       <c r="D427" s="0">
-        <v>3822.39</v>
+        <v>11735</v>
       </c>
     </row>
     <row r="428">
@@ -9085,10 +9097,10 @@
         <v>917</v>
       </c>
       <c r="C428" s="0" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="D428" s="0">
-        <v>4393</v>
+        <v>3380</v>
       </c>
     </row>
     <row r="429">
@@ -9099,10 +9111,10 @@
         <v>919</v>
       </c>
       <c r="C429" s="0" t="s">
-        <v>51</v>
+        <v>129</v>
       </c>
       <c r="D429" s="0">
-        <v>1200</v>
+        <v>3822.39</v>
       </c>
     </row>
     <row r="430">
@@ -9113,10 +9125,10 @@
         <v>921</v>
       </c>
       <c r="C430" s="0" t="s">
-        <v>51</v>
+        <v>89</v>
       </c>
       <c r="D430" s="0">
-        <v>278</v>
+        <v>4393</v>
       </c>
     </row>
     <row r="431">
@@ -9130,7 +9142,7 @@
         <v>51</v>
       </c>
       <c r="D431" s="0">
-        <v>562</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="432">
@@ -9141,10 +9153,10 @@
         <v>925</v>
       </c>
       <c r="C432" s="0" t="s">
-        <v>359</v>
+        <v>51</v>
       </c>
       <c r="D432" s="0">
-        <v>65142</v>
+        <v>278</v>
       </c>
     </row>
     <row r="433">
@@ -9155,10 +9167,10 @@
         <v>927</v>
       </c>
       <c r="C433" s="0" t="s">
-        <v>359</v>
+        <v>51</v>
       </c>
       <c r="D433" s="0">
-        <v>23483</v>
+        <v>562</v>
       </c>
     </row>
     <row r="434">
@@ -9169,10 +9181,10 @@
         <v>929</v>
       </c>
       <c r="C434" s="0" t="s">
-        <v>29</v>
+        <v>359</v>
       </c>
       <c r="D434" s="0">
-        <v>5795.46</v>
+        <v>65142</v>
       </c>
     </row>
     <row r="435">
@@ -9183,10 +9195,10 @@
         <v>931</v>
       </c>
       <c r="C435" s="0" t="s">
-        <v>51</v>
+        <v>359</v>
       </c>
       <c r="D435" s="0">
-        <v>10985</v>
+        <v>23483</v>
       </c>
     </row>
     <row r="436">
@@ -9197,10 +9209,10 @@
         <v>933</v>
       </c>
       <c r="C436" s="0" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="D436" s="0">
-        <v>17425</v>
+        <v>5795.46</v>
       </c>
     </row>
     <row r="437">
@@ -9211,38 +9223,38 @@
         <v>935</v>
       </c>
       <c r="C437" s="0" t="s">
-        <v>936</v>
+        <v>51</v>
       </c>
       <c r="D437" s="0">
-        <v>1958</v>
+        <v>10985</v>
       </c>
     </row>
     <row r="438">
       <c r="A438" s="0" t="s">
+        <v>936</v>
+      </c>
+      <c r="B438" s="0" t="s">
         <v>937</v>
       </c>
-      <c r="B438" s="0" t="s">
-        <v>938</v>
-      </c>
       <c r="C438" s="0" t="s">
-        <v>89</v>
+        <v>51</v>
       </c>
       <c r="D438" s="0">
-        <v>209632.5</v>
+        <v>17425</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="0" t="s">
+        <v>938</v>
+      </c>
+      <c r="B439" s="0" t="s">
         <v>939</v>
       </c>
-      <c r="B439" s="0" t="s">
+      <c r="C439" s="0" t="s">
         <v>940</v>
       </c>
-      <c r="C439" s="0" t="s">
-        <v>559</v>
-      </c>
       <c r="D439" s="0">
-        <v>71176</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="440">
@@ -9253,10 +9265,10 @@
         <v>942</v>
       </c>
       <c r="C440" s="0" t="s">
-        <v>129</v>
+        <v>89</v>
       </c>
       <c r="D440" s="0">
-        <v>82</v>
+        <v>209632.5</v>
       </c>
     </row>
     <row r="441">
@@ -9267,10 +9279,10 @@
         <v>944</v>
       </c>
       <c r="C441" s="0" t="s">
-        <v>69</v>
+        <v>559</v>
       </c>
       <c r="D441" s="0">
-        <v>950</v>
+        <v>71176</v>
       </c>
     </row>
     <row r="442">
@@ -9281,10 +9293,10 @@
         <v>946</v>
       </c>
       <c r="C442" s="0" t="s">
-        <v>458</v>
+        <v>129</v>
       </c>
       <c r="D442" s="0">
-        <v>342641</v>
+        <v>82</v>
       </c>
     </row>
     <row r="443">
@@ -9295,10 +9307,10 @@
         <v>948</v>
       </c>
       <c r="C443" s="0" t="s">
-        <v>147</v>
+        <v>69</v>
       </c>
       <c r="D443" s="0">
-        <v>2200</v>
+        <v>950</v>
       </c>
     </row>
     <row r="444">
@@ -9309,10 +9321,10 @@
         <v>950</v>
       </c>
       <c r="C444" s="0" t="s">
-        <v>467</v>
+        <v>458</v>
       </c>
       <c r="D444" s="0">
-        <v>41000</v>
+        <v>342641</v>
       </c>
     </row>
     <row r="445">
@@ -9323,10 +9335,10 @@
         <v>952</v>
       </c>
       <c r="C445" s="0" t="s">
-        <v>69</v>
+        <v>147</v>
       </c>
       <c r="D445" s="0">
-        <v>9299</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="446">
@@ -9337,10 +9349,10 @@
         <v>954</v>
       </c>
       <c r="C446" s="0" t="s">
-        <v>874</v>
+        <v>467</v>
       </c>
       <c r="D446" s="0">
-        <v>595</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="447">
@@ -9351,10 +9363,10 @@
         <v>956</v>
       </c>
       <c r="C447" s="0" t="s">
-        <v>874</v>
+        <v>69</v>
       </c>
       <c r="D447" s="0">
-        <v>595</v>
+        <v>9299</v>
       </c>
     </row>
     <row r="448">
@@ -9365,7 +9377,7 @@
         <v>958</v>
       </c>
       <c r="C448" s="0" t="s">
-        <v>874</v>
+        <v>878</v>
       </c>
       <c r="D448" s="0">
         <v>595</v>
@@ -9379,10 +9391,10 @@
         <v>960</v>
       </c>
       <c r="C449" s="0" t="s">
-        <v>22</v>
+        <v>878</v>
       </c>
       <c r="D449" s="0">
-        <v>563.36</v>
+        <v>595</v>
       </c>
     </row>
     <row r="450">
@@ -9393,10 +9405,10 @@
         <v>962</v>
       </c>
       <c r="C450" s="0" t="s">
-        <v>16</v>
+        <v>878</v>
       </c>
       <c r="D450" s="0">
-        <v>3200</v>
+        <v>595</v>
       </c>
     </row>
     <row r="451">
@@ -9407,10 +9419,10 @@
         <v>964</v>
       </c>
       <c r="C451" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D451" s="0">
-        <v>2600</v>
+        <v>563.36</v>
       </c>
     </row>
     <row r="452">
@@ -9421,10 +9433,10 @@
         <v>966</v>
       </c>
       <c r="C452" s="0" t="s">
-        <v>273</v>
+        <v>16</v>
       </c>
       <c r="D452" s="0">
-        <v>3700</v>
+        <v>3200</v>
       </c>
     </row>
     <row r="453">
@@ -9435,7 +9447,7 @@
         <v>968</v>
       </c>
       <c r="C453" s="0" t="s">
-        <v>273</v>
+        <v>16</v>
       </c>
       <c r="D453" s="0">
         <v>2600</v>
@@ -9449,10 +9461,10 @@
         <v>970</v>
       </c>
       <c r="C454" s="0" t="s">
-        <v>16</v>
+        <v>273</v>
       </c>
       <c r="D454" s="0">
-        <v>2235</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="455">
@@ -9463,24 +9475,24 @@
         <v>972</v>
       </c>
       <c r="C455" s="0" t="s">
-        <v>16</v>
+        <v>273</v>
       </c>
       <c r="D455" s="0">
-        <v>3500</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="456">
       <c r="A456" s="0" t="s">
-        <v>380</v>
+        <v>973</v>
       </c>
       <c r="B456" s="0" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="C456" s="0" t="s">
-        <v>974</v>
+        <v>16</v>
       </c>
       <c r="D456" s="0">
-        <v>1</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="457">
@@ -9491,24 +9503,24 @@
         <v>976</v>
       </c>
       <c r="C457" s="0" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="D457" s="0">
-        <v>11886</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="0" t="s">
+        <v>380</v>
+      </c>
+      <c r="B458" s="0" t="s">
         <v>977</v>
       </c>
-      <c r="B458" s="0" t="s">
+      <c r="C458" s="0" t="s">
         <v>978</v>
       </c>
-      <c r="C458" s="0" t="s">
-        <v>359</v>
-      </c>
       <c r="D458" s="0">
-        <v>4000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="459">
@@ -9519,10 +9531,10 @@
         <v>980</v>
       </c>
       <c r="C459" s="0" t="s">
-        <v>359</v>
+        <v>29</v>
       </c>
       <c r="D459" s="0">
-        <v>11751</v>
+        <v>13075</v>
       </c>
     </row>
     <row r="460">
@@ -9533,10 +9545,10 @@
         <v>982</v>
       </c>
       <c r="C460" s="0" t="s">
-        <v>322</v>
+        <v>359</v>
       </c>
       <c r="D460" s="0">
-        <v>6000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="461">
@@ -9547,10 +9559,10 @@
         <v>984</v>
       </c>
       <c r="C461" s="0" t="s">
-        <v>322</v>
+        <v>359</v>
       </c>
       <c r="D461" s="0">
-        <v>3000</v>
+        <v>11751</v>
       </c>
     </row>
     <row r="462">
@@ -9561,10 +9573,10 @@
         <v>986</v>
       </c>
       <c r="C462" s="0" t="s">
-        <v>38</v>
+        <v>322</v>
       </c>
       <c r="D462" s="0">
-        <v>618</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="463">
@@ -9575,38 +9587,38 @@
         <v>988</v>
       </c>
       <c r="C463" s="0" t="s">
-        <v>989</v>
+        <v>322</v>
       </c>
       <c r="D463" s="0">
-        <v>24600</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="0" t="s">
+        <v>989</v>
+      </c>
+      <c r="B464" s="0" t="s">
         <v>990</v>
       </c>
-      <c r="B464" s="0" t="s">
-        <v>991</v>
-      </c>
       <c r="C464" s="0" t="s">
-        <v>102</v>
+        <v>38</v>
       </c>
       <c r="D464" s="0">
-        <v>0</v>
+        <v>618</v>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="0" t="s">
+        <v>991</v>
+      </c>
+      <c r="B465" s="0" t="s">
         <v>992</v>
       </c>
-      <c r="B465" s="0" t="s">
+      <c r="C465" s="0" t="s">
         <v>993</v>
       </c>
-      <c r="C465" s="0" t="s">
-        <v>89</v>
-      </c>
       <c r="D465" s="0">
-        <v>28283.75</v>
+        <v>24600</v>
       </c>
     </row>
     <row r="466">
@@ -9617,10 +9629,10 @@
         <v>995</v>
       </c>
       <c r="C466" s="0" t="s">
-        <v>359</v>
+        <v>102</v>
       </c>
       <c r="D466" s="0">
-        <v>75529.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="467">
@@ -9631,10 +9643,10 @@
         <v>997</v>
       </c>
       <c r="C467" s="0" t="s">
-        <v>359</v>
+        <v>89</v>
       </c>
       <c r="D467" s="0">
-        <v>41613</v>
+        <v>28283.75</v>
       </c>
     </row>
     <row r="468">
@@ -9648,7 +9660,7 @@
         <v>359</v>
       </c>
       <c r="D468" s="0">
-        <v>87056</v>
+        <v>75529.41</v>
       </c>
     </row>
     <row r="469">
@@ -9662,7 +9674,7 @@
         <v>359</v>
       </c>
       <c r="D469" s="0">
-        <v>49243.16</v>
+        <v>41613</v>
       </c>
     </row>
     <row r="470">
@@ -9673,10 +9685,10 @@
         <v>1003</v>
       </c>
       <c r="C470" s="0" t="s">
-        <v>22</v>
+        <v>359</v>
       </c>
       <c r="D470" s="0">
-        <v>1600</v>
+        <v>87056</v>
       </c>
     </row>
     <row r="471">
@@ -9687,10 +9699,10 @@
         <v>1005</v>
       </c>
       <c r="C471" s="0" t="s">
-        <v>29</v>
+        <v>359</v>
       </c>
       <c r="D471" s="0">
-        <v>3270.2</v>
+        <v>49243.16</v>
       </c>
     </row>
     <row r="472">
@@ -9701,10 +9713,10 @@
         <v>1007</v>
       </c>
       <c r="C472" s="0" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D472" s="0">
-        <v>3905</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="473">
@@ -9718,7 +9730,7 @@
         <v>29</v>
       </c>
       <c r="D473" s="0">
-        <v>3950</v>
+        <v>3270.2</v>
       </c>
     </row>
     <row r="474">
@@ -9732,21 +9744,21 @@
         <v>29</v>
       </c>
       <c r="D474" s="0">
-        <v>3313.05</v>
+        <v>3905</v>
       </c>
     </row>
     <row r="475">
-      <c r="A475" s="2" t="s">
+      <c r="A475" s="0" t="s">
         <v>1012</v>
       </c>
-      <c r="B475" s="2" t="s">
+      <c r="B475" s="0" t="s">
         <v>1013</v>
       </c>
-      <c r="C475" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D475" s="2">
-        <v>0</v>
+      <c r="C475" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D475" s="0">
+        <v>3950.91</v>
       </c>
     </row>
     <row r="476">
@@ -9757,23 +9769,51 @@
         <v>1015</v>
       </c>
       <c r="C476" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D476" s="0">
+        <v>3313.05</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="2" t="s">
+        <v>1016</v>
+      </c>
+      <c r="B477" s="2" t="s">
+        <v>1017</v>
+      </c>
+      <c r="C477" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D477" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="0" t="s">
+        <v>1018</v>
+      </c>
+      <c r="B478" s="0" t="s">
+        <v>1019</v>
+      </c>
+      <c r="C478" s="0" t="s">
         <v>147</v>
       </c>
-      <c r="D476" s="0">
+      <c r="D478" s="0">
         <v>430</v>
       </c>
     </row>
-    <row r="477">
-      <c r="A477" s="0" t="s">
-        <v>1016</v>
-      </c>
-      <c r="B477" s="0" t="s">
-        <v>1017</v>
-      </c>
-      <c r="C477" s="0" t="s">
+    <row r="479">
+      <c r="A479" s="0" t="s">
+        <v>1020</v>
+      </c>
+      <c r="B479" s="0" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C479" s="0" t="s">
         <v>129</v>
       </c>
-      <c r="D477" s="0">
+      <c r="D479" s="0">
         <v>435</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: stock y precios actualizados 2026-06-16
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1022" uniqueCount="1022">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="1024">
   <si>
     <t>Código</t>
   </si>
@@ -2196,6 +2196,12 @@
   </si>
   <si>
     <t>NETOCUR BALSAMICO JBE. X 100ML - 000002445</t>
+  </si>
+  <si>
+    <t>000010797</t>
+  </si>
+  <si>
+    <t>NEUMOCORT 200mcg Aer. x 200 Dosis - 000010797</t>
   </si>
   <si>
     <t>000023836</t>
@@ -3136,7 +3142,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A3:D479"/>
+  <dimension ref="A3:D480"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="3">
@@ -3626,7 +3632,7 @@
         <v>89</v>
       </c>
       <c r="D37" s="0">
-        <v>21296</v>
+        <v>21961.5</v>
       </c>
     </row>
     <row r="38">
@@ -4480,7 +4486,7 @@
         <v>89</v>
       </c>
       <c r="D98" s="0">
-        <v>3327.5</v>
+        <v>2355.84</v>
       </c>
     </row>
     <row r="99">
@@ -4494,7 +4500,7 @@
         <v>89</v>
       </c>
       <c r="D99" s="0">
-        <v>3660.25</v>
+        <v>3533.76</v>
       </c>
     </row>
     <row r="100">
@@ -4676,7 +4682,7 @@
         <v>89</v>
       </c>
       <c r="D112" s="0">
-        <v>9317</v>
+        <v>9649.75</v>
       </c>
     </row>
     <row r="113">
@@ -7168,7 +7174,7 @@
         <v>89</v>
       </c>
       <c r="D290" s="0">
-        <v>32609</v>
+        <v>32609.5</v>
       </c>
     </row>
     <row r="291">
@@ -7224,7 +7230,7 @@
         <v>89</v>
       </c>
       <c r="D294" s="0">
-        <v>299475</v>
+        <v>306130</v>
       </c>
     </row>
     <row r="295">
@@ -7252,7 +7258,7 @@
         <v>194</v>
       </c>
       <c r="D296" s="0">
-        <v>6000</v>
+        <v>4390</v>
       </c>
     </row>
     <row r="297">
@@ -7686,7 +7692,7 @@
         <v>89</v>
       </c>
       <c r="D327" s="0">
-        <v>8318.75</v>
+        <v>7986</v>
       </c>
     </row>
     <row r="328">
@@ -7823,10 +7829,10 @@
         <v>729</v>
       </c>
       <c r="C337" s="0" t="s">
-        <v>129</v>
+        <v>249</v>
       </c>
       <c r="D337" s="0">
-        <v>300</v>
+        <v>11959</v>
       </c>
     </row>
     <row r="338">
@@ -7837,10 +7843,10 @@
         <v>731</v>
       </c>
       <c r="C338" s="0" t="s">
-        <v>273</v>
+        <v>129</v>
       </c>
       <c r="D338" s="0">
-        <v>1450</v>
+        <v>300</v>
       </c>
     </row>
     <row r="339">
@@ -7851,10 +7857,10 @@
         <v>733</v>
       </c>
       <c r="C339" s="0" t="s">
-        <v>89</v>
+        <v>273</v>
       </c>
       <c r="D339" s="0">
-        <v>7986</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="340">
@@ -7865,10 +7871,10 @@
         <v>735</v>
       </c>
       <c r="C340" s="0" t="s">
-        <v>16</v>
+        <v>89</v>
       </c>
       <c r="D340" s="0">
-        <v>900</v>
+        <v>7320.5</v>
       </c>
     </row>
     <row r="341">
@@ -7879,10 +7885,10 @@
         <v>737</v>
       </c>
       <c r="C341" s="0" t="s">
-        <v>273</v>
+        <v>16</v>
       </c>
       <c r="D341" s="0">
-        <v>520</v>
+        <v>900</v>
       </c>
     </row>
     <row r="342">
@@ -7893,10 +7899,10 @@
         <v>739</v>
       </c>
       <c r="C342" s="0" t="s">
-        <v>458</v>
+        <v>273</v>
       </c>
       <c r="D342" s="0">
-        <v>64925</v>
+        <v>520</v>
       </c>
     </row>
     <row r="343">
@@ -7907,10 +7913,10 @@
         <v>741</v>
       </c>
       <c r="C343" s="0" t="s">
-        <v>16</v>
+        <v>458</v>
       </c>
       <c r="D343" s="0">
-        <v>1000</v>
+        <v>64925</v>
       </c>
     </row>
     <row r="344">
@@ -7921,10 +7927,10 @@
         <v>743</v>
       </c>
       <c r="C344" s="0" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D344" s="0">
-        <v>1623</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="345">
@@ -7935,10 +7941,10 @@
         <v>745</v>
       </c>
       <c r="C345" s="0" t="s">
-        <v>129</v>
+        <v>22</v>
       </c>
       <c r="D345" s="0">
-        <v>1116.03</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="346">
@@ -7952,7 +7958,7 @@
         <v>129</v>
       </c>
       <c r="D346" s="0">
-        <v>4028.88</v>
+        <v>1116.03</v>
       </c>
     </row>
     <row r="347">
@@ -7963,10 +7969,10 @@
         <v>749</v>
       </c>
       <c r="C347" s="0" t="s">
-        <v>29</v>
+        <v>129</v>
       </c>
       <c r="D347" s="0">
-        <v>1869.6</v>
+        <v>4028.88</v>
       </c>
     </row>
     <row r="348">
@@ -7977,10 +7983,10 @@
         <v>751</v>
       </c>
       <c r="C348" s="0" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="D348" s="0">
-        <v>420</v>
+        <v>1869.6</v>
       </c>
     </row>
     <row r="349">
@@ -7994,7 +8000,7 @@
         <v>16</v>
       </c>
       <c r="D349" s="0">
-        <v>750</v>
+        <v>420</v>
       </c>
     </row>
     <row r="350">
@@ -8019,10 +8025,10 @@
         <v>757</v>
       </c>
       <c r="C351" s="0" t="s">
-        <v>362</v>
+        <v>16</v>
       </c>
       <c r="D351" s="0">
-        <v>134775.6</v>
+        <v>750</v>
       </c>
     </row>
     <row r="352">
@@ -8036,7 +8042,7 @@
         <v>362</v>
       </c>
       <c r="D352" s="0">
-        <v>175991.55</v>
+        <v>134775.6</v>
       </c>
     </row>
     <row r="353">
@@ -8047,10 +8053,10 @@
         <v>761</v>
       </c>
       <c r="C353" s="0" t="s">
-        <v>69</v>
+        <v>362</v>
       </c>
       <c r="D353" s="0">
-        <v>3263</v>
+        <v>175991.55</v>
       </c>
     </row>
     <row r="354">
@@ -8064,7 +8070,7 @@
         <v>69</v>
       </c>
       <c r="D354" s="0">
-        <v>18027</v>
+        <v>3263</v>
       </c>
     </row>
     <row r="355">
@@ -8075,10 +8081,10 @@
         <v>765</v>
       </c>
       <c r="C355" s="0" t="s">
-        <v>273</v>
+        <v>69</v>
       </c>
       <c r="D355" s="0">
-        <v>515</v>
+        <v>18027</v>
       </c>
     </row>
     <row r="356">
@@ -8089,7 +8095,7 @@
         <v>767</v>
       </c>
       <c r="C356" s="0" t="s">
-        <v>38</v>
+        <v>273</v>
       </c>
       <c r="D356" s="0">
         <v>515</v>
@@ -8103,10 +8109,10 @@
         <v>769</v>
       </c>
       <c r="C357" s="0" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D357" s="0">
-        <v>10154</v>
+        <v>515</v>
       </c>
     </row>
     <row r="358">
@@ -8117,10 +8123,10 @@
         <v>771</v>
       </c>
       <c r="C358" s="0" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="D358" s="0">
-        <v>9500</v>
+        <v>10154</v>
       </c>
     </row>
     <row r="359">
@@ -8131,10 +8137,10 @@
         <v>773</v>
       </c>
       <c r="C359" s="0" t="s">
-        <v>458</v>
+        <v>51</v>
       </c>
       <c r="D359" s="0">
-        <v>207600</v>
+        <v>9500</v>
       </c>
     </row>
     <row r="360">
@@ -8148,7 +8154,7 @@
         <v>458</v>
       </c>
       <c r="D360" s="0">
-        <v>249000</v>
+        <v>207600</v>
       </c>
     </row>
     <row r="361">
@@ -8159,10 +8165,10 @@
         <v>777</v>
       </c>
       <c r="C361" s="0" t="s">
-        <v>69</v>
+        <v>458</v>
       </c>
       <c r="D361" s="0">
-        <v>10021.22</v>
+        <v>249000</v>
       </c>
     </row>
     <row r="362">
@@ -8176,7 +8182,7 @@
         <v>69</v>
       </c>
       <c r="D362" s="0">
-        <v>17710</v>
+        <v>10021.22</v>
       </c>
     </row>
     <row r="363">
@@ -8187,24 +8193,24 @@
         <v>781</v>
       </c>
       <c r="C363" s="0" t="s">
-        <v>782</v>
+        <v>69</v>
       </c>
       <c r="D363" s="0">
-        <v>1080</v>
+        <v>17710</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="0" t="s">
+        <v>782</v>
+      </c>
+      <c r="B364" s="0" t="s">
         <v>783</v>
       </c>
-      <c r="B364" s="0" t="s">
+      <c r="C364" s="0" t="s">
         <v>784</v>
       </c>
-      <c r="C364" s="0" t="s">
-        <v>19</v>
-      </c>
       <c r="D364" s="0">
-        <v>691</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="365">
@@ -8215,24 +8221,24 @@
         <v>786</v>
       </c>
       <c r="C365" s="0" t="s">
-        <v>787</v>
+        <v>19</v>
       </c>
       <c r="D365" s="0">
-        <v>520</v>
+        <v>691</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="0" t="s">
+        <v>787</v>
+      </c>
+      <c r="B366" s="0" t="s">
         <v>788</v>
       </c>
-      <c r="B366" s="0" t="s">
+      <c r="C366" s="0" t="s">
         <v>789</v>
       </c>
-      <c r="C366" s="0" t="s">
-        <v>787</v>
-      </c>
       <c r="D366" s="0">
-        <v>300</v>
+        <v>520</v>
       </c>
     </row>
     <row r="367">
@@ -8243,10 +8249,10 @@
         <v>791</v>
       </c>
       <c r="C367" s="0" t="s">
-        <v>16</v>
+        <v>789</v>
       </c>
       <c r="D367" s="0">
-        <v>2200</v>
+        <v>300</v>
       </c>
     </row>
     <row r="368">
@@ -8260,7 +8266,7 @@
         <v>16</v>
       </c>
       <c r="D368" s="0">
-        <v>2500</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="369">
@@ -8271,10 +8277,10 @@
         <v>795</v>
       </c>
       <c r="C369" s="0" t="s">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="D369" s="0">
-        <v>4791.6</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="370">
@@ -8285,10 +8291,10 @@
         <v>797</v>
       </c>
       <c r="C370" s="0" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="D370" s="0">
-        <v>2699.64</v>
+        <v>4791.6</v>
       </c>
     </row>
     <row r="371">
@@ -8299,10 +8305,10 @@
         <v>799</v>
       </c>
       <c r="C371" s="0" t="s">
-        <v>35</v>
+        <v>69</v>
       </c>
       <c r="D371" s="0">
-        <v>3800</v>
+        <v>2699.64</v>
       </c>
     </row>
     <row r="372">
@@ -8313,10 +8319,10 @@
         <v>801</v>
       </c>
       <c r="C372" s="0" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D372" s="0">
-        <v>4000</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="373">
@@ -8327,24 +8333,24 @@
         <v>803</v>
       </c>
       <c r="C373" s="0" t="s">
-        <v>804</v>
+        <v>16</v>
       </c>
       <c r="D373" s="0">
-        <v>3800</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="0" t="s">
+        <v>804</v>
+      </c>
+      <c r="B374" s="0" t="s">
         <v>805</v>
       </c>
-      <c r="B374" s="0" t="s">
+      <c r="C374" s="0" t="s">
         <v>806</v>
       </c>
-      <c r="C374" s="0" t="s">
-        <v>22</v>
-      </c>
       <c r="D374" s="0">
-        <v>353</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="375">
@@ -8355,10 +8361,10 @@
         <v>808</v>
       </c>
       <c r="C375" s="0" t="s">
-        <v>346</v>
+        <v>22</v>
       </c>
       <c r="D375" s="0">
-        <v>1800</v>
+        <v>353</v>
       </c>
     </row>
     <row r="376">
@@ -8369,10 +8375,10 @@
         <v>810</v>
       </c>
       <c r="C376" s="0" t="s">
-        <v>16</v>
+        <v>346</v>
       </c>
       <c r="D376" s="0">
-        <v>2100</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="377">
@@ -8383,10 +8389,10 @@
         <v>812</v>
       </c>
       <c r="C377" s="0" t="s">
-        <v>199</v>
+        <v>16</v>
       </c>
       <c r="D377" s="0">
-        <v>65537</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="378">
@@ -8397,10 +8403,10 @@
         <v>814</v>
       </c>
       <c r="C378" s="0" t="s">
-        <v>129</v>
+        <v>199</v>
       </c>
       <c r="D378" s="0">
-        <v>3820.86</v>
+        <v>65537</v>
       </c>
     </row>
     <row r="379">
@@ -8414,7 +8420,7 @@
         <v>129</v>
       </c>
       <c r="D379" s="0">
-        <v>3962</v>
+        <v>3820.86</v>
       </c>
     </row>
     <row r="380">
@@ -8428,7 +8434,7 @@
         <v>129</v>
       </c>
       <c r="D380" s="0">
-        <v>5802.4</v>
+        <v>3962</v>
       </c>
     </row>
     <row r="381">
@@ -8439,10 +8445,10 @@
         <v>820</v>
       </c>
       <c r="C381" s="0" t="s">
-        <v>300</v>
+        <v>129</v>
       </c>
       <c r="D381" s="0">
-        <v>570</v>
+        <v>5802.4</v>
       </c>
     </row>
     <row r="382">
@@ -8453,10 +8459,10 @@
         <v>822</v>
       </c>
       <c r="C382" s="0" t="s">
-        <v>69</v>
+        <v>300</v>
       </c>
       <c r="D382" s="0">
-        <v>550</v>
+        <v>570</v>
       </c>
     </row>
     <row r="383">
@@ -8467,10 +8473,10 @@
         <v>824</v>
       </c>
       <c r="C383" s="0" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="D383" s="0">
-        <v>167</v>
+        <v>550</v>
       </c>
     </row>
     <row r="384">
@@ -8481,10 +8487,10 @@
         <v>826</v>
       </c>
       <c r="C384" s="0" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="D384" s="0">
-        <v>686.98</v>
+        <v>167</v>
       </c>
     </row>
     <row r="385">
@@ -8495,10 +8501,10 @@
         <v>828</v>
       </c>
       <c r="C385" s="0" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="D385" s="0">
-        <v>101000</v>
+        <v>686.98</v>
       </c>
     </row>
     <row r="386">
@@ -8509,10 +8515,10 @@
         <v>830</v>
       </c>
       <c r="C386" s="0" t="s">
-        <v>115</v>
+        <v>58</v>
       </c>
       <c r="D386" s="0">
-        <v>6251</v>
+        <v>101000</v>
       </c>
     </row>
     <row r="387">
@@ -8523,10 +8529,10 @@
         <v>832</v>
       </c>
       <c r="C387" s="0" t="s">
-        <v>89</v>
+        <v>115</v>
       </c>
       <c r="D387" s="0">
-        <v>1166</v>
+        <v>6251</v>
       </c>
     </row>
     <row r="388">
@@ -8537,10 +8543,10 @@
         <v>834</v>
       </c>
       <c r="C388" s="0" t="s">
-        <v>140</v>
+        <v>89</v>
       </c>
       <c r="D388" s="0">
-        <v>360</v>
+        <v>1164.66</v>
       </c>
     </row>
     <row r="389">
@@ -8554,7 +8560,7 @@
         <v>140</v>
       </c>
       <c r="D389" s="0">
-        <v>450</v>
+        <v>360</v>
       </c>
     </row>
     <row r="390">
@@ -8568,7 +8574,7 @@
         <v>140</v>
       </c>
       <c r="D390" s="0">
-        <v>2050</v>
+        <v>450</v>
       </c>
     </row>
     <row r="391">
@@ -8579,10 +8585,10 @@
         <v>840</v>
       </c>
       <c r="C391" s="0" t="s">
-        <v>559</v>
+        <v>140</v>
       </c>
       <c r="D391" s="0">
-        <v>25192.82</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="392">
@@ -8593,10 +8599,10 @@
         <v>842</v>
       </c>
       <c r="C392" s="0" t="s">
-        <v>69</v>
+        <v>559</v>
       </c>
       <c r="D392" s="0">
-        <v>3500</v>
+        <v>25192.82</v>
       </c>
     </row>
     <row r="393">
@@ -8607,10 +8613,10 @@
         <v>844</v>
       </c>
       <c r="C393" s="0" t="s">
-        <v>167</v>
+        <v>69</v>
       </c>
       <c r="D393" s="0">
-        <v>600</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="394">
@@ -8621,24 +8627,24 @@
         <v>846</v>
       </c>
       <c r="C394" s="0" t="s">
-        <v>847</v>
+        <v>167</v>
       </c>
       <c r="D394" s="0">
-        <v>1080</v>
+        <v>600</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="0" t="s">
+        <v>847</v>
+      </c>
+      <c r="B395" s="0" t="s">
         <v>848</v>
       </c>
-      <c r="B395" s="0" t="s">
+      <c r="C395" s="0" t="s">
         <v>849</v>
       </c>
-      <c r="C395" s="0" t="s">
-        <v>322</v>
-      </c>
       <c r="D395" s="0">
-        <v>8628</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="396">
@@ -8652,7 +8658,7 @@
         <v>322</v>
       </c>
       <c r="D396" s="0">
-        <v>9125</v>
+        <v>8628</v>
       </c>
     </row>
     <row r="397">
@@ -8663,10 +8669,10 @@
         <v>853</v>
       </c>
       <c r="C397" s="0" t="s">
-        <v>129</v>
+        <v>322</v>
       </c>
       <c r="D397" s="0">
-        <v>1080</v>
+        <v>9125</v>
       </c>
     </row>
     <row r="398">
@@ -8680,7 +8686,7 @@
         <v>129</v>
       </c>
       <c r="D398" s="0">
-        <v>4500</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="399">
@@ -8691,10 +8697,10 @@
         <v>857</v>
       </c>
       <c r="C399" s="0" t="s">
-        <v>44</v>
+        <v>129</v>
       </c>
       <c r="D399" s="0">
-        <v>4194.88</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="400">
@@ -8708,7 +8714,7 @@
         <v>44</v>
       </c>
       <c r="D400" s="0">
-        <v>2139.28</v>
+        <v>4194.88</v>
       </c>
     </row>
     <row r="401">
@@ -8722,7 +8728,7 @@
         <v>44</v>
       </c>
       <c r="D401" s="0">
-        <v>1699.1</v>
+        <v>2139.28</v>
       </c>
     </row>
     <row r="402">
@@ -8736,7 +8742,7 @@
         <v>44</v>
       </c>
       <c r="D402" s="0">
-        <v>3427.58</v>
+        <v>1699.1</v>
       </c>
     </row>
     <row r="403">
@@ -8750,7 +8756,7 @@
         <v>44</v>
       </c>
       <c r="D403" s="0">
-        <v>19700</v>
+        <v>3427.58</v>
       </c>
     </row>
     <row r="404">
@@ -8764,7 +8770,7 @@
         <v>44</v>
       </c>
       <c r="D404" s="0">
-        <v>1839.2</v>
+        <v>19700</v>
       </c>
     </row>
     <row r="405">
@@ -8778,7 +8784,7 @@
         <v>44</v>
       </c>
       <c r="D405" s="0">
-        <v>4215.45</v>
+        <v>1839.2</v>
       </c>
     </row>
     <row r="406">
@@ -8792,7 +8798,7 @@
         <v>44</v>
       </c>
       <c r="D406" s="0">
-        <v>3395.26</v>
+        <v>4215.45</v>
       </c>
     </row>
     <row r="407">
@@ -8803,10 +8809,10 @@
         <v>873</v>
       </c>
       <c r="C407" s="0" t="s">
-        <v>467</v>
+        <v>44</v>
       </c>
       <c r="D407" s="0">
-        <v>510</v>
+        <v>3395.26</v>
       </c>
     </row>
     <row r="408">
@@ -8817,7 +8823,7 @@
         <v>875</v>
       </c>
       <c r="C408" s="0" t="s">
-        <v>38</v>
+        <v>467</v>
       </c>
       <c r="D408" s="0">
         <v>510</v>
@@ -8831,21 +8837,21 @@
         <v>877</v>
       </c>
       <c r="C409" s="0" t="s">
-        <v>878</v>
+        <v>38</v>
       </c>
       <c r="D409" s="0">
-        <v>559</v>
+        <v>510</v>
       </c>
     </row>
     <row r="410">
       <c r="A410" s="0" t="s">
+        <v>878</v>
+      </c>
+      <c r="B410" s="0" t="s">
         <v>879</v>
       </c>
-      <c r="B410" s="0" t="s">
+      <c r="C410" s="0" t="s">
         <v>880</v>
-      </c>
-      <c r="C410" s="0" t="s">
-        <v>878</v>
       </c>
       <c r="D410" s="0">
         <v>559</v>
@@ -8859,7 +8865,7 @@
         <v>882</v>
       </c>
       <c r="C411" s="0" t="s">
-        <v>878</v>
+        <v>880</v>
       </c>
       <c r="D411" s="0">
         <v>559</v>
@@ -8873,10 +8879,10 @@
         <v>884</v>
       </c>
       <c r="C412" s="0" t="s">
-        <v>878</v>
+        <v>880</v>
       </c>
       <c r="D412" s="0">
-        <v>342</v>
+        <v>559</v>
       </c>
     </row>
     <row r="413">
@@ -8887,7 +8893,7 @@
         <v>886</v>
       </c>
       <c r="C413" s="0" t="s">
-        <v>878</v>
+        <v>880</v>
       </c>
       <c r="D413" s="0">
         <v>342</v>
@@ -8901,7 +8907,7 @@
         <v>888</v>
       </c>
       <c r="C414" s="0" t="s">
-        <v>878</v>
+        <v>880</v>
       </c>
       <c r="D414" s="0">
         <v>342</v>
@@ -8915,10 +8921,10 @@
         <v>890</v>
       </c>
       <c r="C415" s="0" t="s">
-        <v>878</v>
+        <v>880</v>
       </c>
       <c r="D415" s="0">
-        <v>0</v>
+        <v>342</v>
       </c>
     </row>
     <row r="416">
@@ -8929,7 +8935,7 @@
         <v>892</v>
       </c>
       <c r="C416" s="0" t="s">
-        <v>878</v>
+        <v>880</v>
       </c>
       <c r="D416" s="0">
         <v>0</v>
@@ -8943,10 +8949,10 @@
         <v>894</v>
       </c>
       <c r="C417" s="0" t="s">
-        <v>878</v>
+        <v>880</v>
       </c>
       <c r="D417" s="0">
-        <v>423</v>
+        <v>0</v>
       </c>
     </row>
     <row r="418">
@@ -8957,10 +8963,10 @@
         <v>896</v>
       </c>
       <c r="C418" s="0" t="s">
-        <v>69</v>
+        <v>880</v>
       </c>
       <c r="D418" s="0">
-        <v>15968</v>
+        <v>423</v>
       </c>
     </row>
     <row r="419">
@@ -8971,10 +8977,10 @@
         <v>898</v>
       </c>
       <c r="C419" s="0" t="s">
-        <v>109</v>
+        <v>69</v>
       </c>
       <c r="D419" s="0">
-        <v>14000</v>
+        <v>15968</v>
       </c>
     </row>
     <row r="420">
@@ -8985,10 +8991,10 @@
         <v>900</v>
       </c>
       <c r="C420" s="0" t="s">
-        <v>89</v>
+        <v>109</v>
       </c>
       <c r="D420" s="0">
-        <v>266200</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="421">
@@ -9002,7 +9008,7 @@
         <v>89</v>
       </c>
       <c r="D421" s="0">
-        <v>194991.5</v>
+        <v>266200</v>
       </c>
     </row>
     <row r="422">
@@ -9016,7 +9022,7 @@
         <v>89</v>
       </c>
       <c r="D422" s="0">
-        <v>289492.5</v>
+        <v>194991.5</v>
       </c>
     </row>
     <row r="423">
@@ -9027,24 +9033,24 @@
         <v>906</v>
       </c>
       <c r="C423" s="0" t="s">
-        <v>907</v>
+        <v>89</v>
       </c>
       <c r="D423" s="0">
-        <v>13722</v>
+        <v>289492.5</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="0" t="s">
+        <v>907</v>
+      </c>
+      <c r="B424" s="0" t="s">
         <v>908</v>
       </c>
-      <c r="B424" s="0" t="s">
+      <c r="C424" s="0" t="s">
         <v>909</v>
       </c>
-      <c r="C424" s="0" t="s">
-        <v>907</v>
-      </c>
       <c r="D424" s="0">
-        <v>15072</v>
+        <v>13722</v>
       </c>
     </row>
     <row r="425">
@@ -9055,10 +9061,10 @@
         <v>911</v>
       </c>
       <c r="C425" s="0" t="s">
-        <v>907</v>
+        <v>909</v>
       </c>
       <c r="D425" s="0">
-        <v>6555</v>
+        <v>15072</v>
       </c>
     </row>
     <row r="426">
@@ -9069,10 +9075,10 @@
         <v>913</v>
       </c>
       <c r="C426" s="0" t="s">
-        <v>907</v>
+        <v>909</v>
       </c>
       <c r="D426" s="0">
-        <v>8964.61</v>
+        <v>6555</v>
       </c>
     </row>
     <row r="427">
@@ -9083,10 +9089,10 @@
         <v>915</v>
       </c>
       <c r="C427" s="0" t="s">
-        <v>907</v>
+        <v>909</v>
       </c>
       <c r="D427" s="0">
-        <v>11735</v>
+        <v>8964.61</v>
       </c>
     </row>
     <row r="428">
@@ -9097,10 +9103,10 @@
         <v>917</v>
       </c>
       <c r="C428" s="0" t="s">
-        <v>69</v>
+        <v>909</v>
       </c>
       <c r="D428" s="0">
-        <v>3380</v>
+        <v>11735</v>
       </c>
     </row>
     <row r="429">
@@ -9111,10 +9117,10 @@
         <v>919</v>
       </c>
       <c r="C429" s="0" t="s">
-        <v>129</v>
+        <v>69</v>
       </c>
       <c r="D429" s="0">
-        <v>3822.39</v>
+        <v>3380</v>
       </c>
     </row>
     <row r="430">
@@ -9125,10 +9131,10 @@
         <v>921</v>
       </c>
       <c r="C430" s="0" t="s">
-        <v>89</v>
+        <v>129</v>
       </c>
       <c r="D430" s="0">
-        <v>4393</v>
+        <v>3822.39</v>
       </c>
     </row>
     <row r="431">
@@ -9139,10 +9145,10 @@
         <v>923</v>
       </c>
       <c r="C431" s="0" t="s">
-        <v>51</v>
+        <v>89</v>
       </c>
       <c r="D431" s="0">
-        <v>1200</v>
+        <v>4392.3</v>
       </c>
     </row>
     <row r="432">
@@ -9156,7 +9162,7 @@
         <v>51</v>
       </c>
       <c r="D432" s="0">
-        <v>278</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="433">
@@ -9170,7 +9176,7 @@
         <v>51</v>
       </c>
       <c r="D433" s="0">
-        <v>562</v>
+        <v>278</v>
       </c>
     </row>
     <row r="434">
@@ -9181,10 +9187,10 @@
         <v>929</v>
       </c>
       <c r="C434" s="0" t="s">
-        <v>359</v>
+        <v>51</v>
       </c>
       <c r="D434" s="0">
-        <v>65142</v>
+        <v>562</v>
       </c>
     </row>
     <row r="435">
@@ -9198,7 +9204,7 @@
         <v>359</v>
       </c>
       <c r="D435" s="0">
-        <v>23483</v>
+        <v>65142</v>
       </c>
     </row>
     <row r="436">
@@ -9209,10 +9215,10 @@
         <v>933</v>
       </c>
       <c r="C436" s="0" t="s">
-        <v>29</v>
+        <v>359</v>
       </c>
       <c r="D436" s="0">
-        <v>5795.46</v>
+        <v>23483</v>
       </c>
     </row>
     <row r="437">
@@ -9223,10 +9229,10 @@
         <v>935</v>
       </c>
       <c r="C437" s="0" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="D437" s="0">
-        <v>10985</v>
+        <v>5795.46</v>
       </c>
     </row>
     <row r="438">
@@ -9240,7 +9246,7 @@
         <v>51</v>
       </c>
       <c r="D438" s="0">
-        <v>17425</v>
+        <v>10985</v>
       </c>
     </row>
     <row r="439">
@@ -9251,24 +9257,24 @@
         <v>939</v>
       </c>
       <c r="C439" s="0" t="s">
-        <v>940</v>
+        <v>51</v>
       </c>
       <c r="D439" s="0">
-        <v>1958</v>
+        <v>17425</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="0" t="s">
+        <v>940</v>
+      </c>
+      <c r="B440" s="0" t="s">
         <v>941</v>
       </c>
-      <c r="B440" s="0" t="s">
+      <c r="C440" s="0" t="s">
         <v>942</v>
       </c>
-      <c r="C440" s="0" t="s">
-        <v>89</v>
-      </c>
       <c r="D440" s="0">
-        <v>209632.5</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="441">
@@ -9279,10 +9285,10 @@
         <v>944</v>
       </c>
       <c r="C441" s="0" t="s">
-        <v>559</v>
+        <v>89</v>
       </c>
       <c r="D441" s="0">
-        <v>71176</v>
+        <v>249562.5</v>
       </c>
     </row>
     <row r="442">
@@ -9293,10 +9299,10 @@
         <v>946</v>
       </c>
       <c r="C442" s="0" t="s">
-        <v>129</v>
+        <v>559</v>
       </c>
       <c r="D442" s="0">
-        <v>82</v>
+        <v>71176</v>
       </c>
     </row>
     <row r="443">
@@ -9307,10 +9313,10 @@
         <v>948</v>
       </c>
       <c r="C443" s="0" t="s">
-        <v>69</v>
+        <v>129</v>
       </c>
       <c r="D443" s="0">
-        <v>950</v>
+        <v>82</v>
       </c>
     </row>
     <row r="444">
@@ -9321,10 +9327,10 @@
         <v>950</v>
       </c>
       <c r="C444" s="0" t="s">
-        <v>458</v>
+        <v>69</v>
       </c>
       <c r="D444" s="0">
-        <v>342641</v>
+        <v>950</v>
       </c>
     </row>
     <row r="445">
@@ -9335,10 +9341,10 @@
         <v>952</v>
       </c>
       <c r="C445" s="0" t="s">
-        <v>147</v>
+        <v>458</v>
       </c>
       <c r="D445" s="0">
-        <v>2200</v>
+        <v>342641</v>
       </c>
     </row>
     <row r="446">
@@ -9349,10 +9355,10 @@
         <v>954</v>
       </c>
       <c r="C446" s="0" t="s">
-        <v>467</v>
+        <v>147</v>
       </c>
       <c r="D446" s="0">
-        <v>41000</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="447">
@@ -9363,10 +9369,10 @@
         <v>956</v>
       </c>
       <c r="C447" s="0" t="s">
-        <v>69</v>
+        <v>467</v>
       </c>
       <c r="D447" s="0">
-        <v>9299</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="448">
@@ -9377,10 +9383,10 @@
         <v>958</v>
       </c>
       <c r="C448" s="0" t="s">
-        <v>878</v>
+        <v>69</v>
       </c>
       <c r="D448" s="0">
-        <v>595</v>
+        <v>9299</v>
       </c>
     </row>
     <row r="449">
@@ -9391,7 +9397,7 @@
         <v>960</v>
       </c>
       <c r="C449" s="0" t="s">
-        <v>878</v>
+        <v>880</v>
       </c>
       <c r="D449" s="0">
         <v>595</v>
@@ -9405,7 +9411,7 @@
         <v>962</v>
       </c>
       <c r="C450" s="0" t="s">
-        <v>878</v>
+        <v>880</v>
       </c>
       <c r="D450" s="0">
         <v>595</v>
@@ -9419,10 +9425,10 @@
         <v>964</v>
       </c>
       <c r="C451" s="0" t="s">
-        <v>22</v>
+        <v>880</v>
       </c>
       <c r="D451" s="0">
-        <v>563.36</v>
+        <v>595</v>
       </c>
     </row>
     <row r="452">
@@ -9433,10 +9439,10 @@
         <v>966</v>
       </c>
       <c r="C452" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D452" s="0">
-        <v>3200</v>
+        <v>563.36</v>
       </c>
     </row>
     <row r="453">
@@ -9450,7 +9456,7 @@
         <v>16</v>
       </c>
       <c r="D453" s="0">
-        <v>2600</v>
+        <v>3200</v>
       </c>
     </row>
     <row r="454">
@@ -9461,10 +9467,10 @@
         <v>970</v>
       </c>
       <c r="C454" s="0" t="s">
-        <v>273</v>
+        <v>16</v>
       </c>
       <c r="D454" s="0">
-        <v>3700</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="455">
@@ -9478,7 +9484,7 @@
         <v>273</v>
       </c>
       <c r="D455" s="0">
-        <v>2600</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="456">
@@ -9489,10 +9495,10 @@
         <v>974</v>
       </c>
       <c r="C456" s="0" t="s">
-        <v>16</v>
+        <v>273</v>
       </c>
       <c r="D456" s="0">
-        <v>2235</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="457">
@@ -9506,35 +9512,35 @@
         <v>16</v>
       </c>
       <c r="D457" s="0">
-        <v>3500</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="0" t="s">
-        <v>380</v>
+        <v>977</v>
       </c>
       <c r="B458" s="0" t="s">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="C458" s="0" t="s">
-        <v>978</v>
+        <v>16</v>
       </c>
       <c r="D458" s="0">
-        <v>1</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="459">
       <c r="A459" s="0" t="s">
+        <v>380</v>
+      </c>
+      <c r="B459" s="0" t="s">
         <v>979</v>
       </c>
-      <c r="B459" s="0" t="s">
+      <c r="C459" s="0" t="s">
         <v>980</v>
       </c>
-      <c r="C459" s="0" t="s">
-        <v>29</v>
-      </c>
       <c r="D459" s="0">
-        <v>13075</v>
+        <v>1</v>
       </c>
     </row>
     <row r="460">
@@ -9545,10 +9551,10 @@
         <v>982</v>
       </c>
       <c r="C460" s="0" t="s">
-        <v>359</v>
+        <v>29</v>
       </c>
       <c r="D460" s="0">
-        <v>4000</v>
+        <v>13075</v>
       </c>
     </row>
     <row r="461">
@@ -9562,7 +9568,7 @@
         <v>359</v>
       </c>
       <c r="D461" s="0">
-        <v>11751</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="462">
@@ -9573,10 +9579,10 @@
         <v>986</v>
       </c>
       <c r="C462" s="0" t="s">
-        <v>322</v>
+        <v>359</v>
       </c>
       <c r="D462" s="0">
-        <v>6000</v>
+        <v>11751</v>
       </c>
     </row>
     <row r="463">
@@ -9590,7 +9596,7 @@
         <v>322</v>
       </c>
       <c r="D463" s="0">
-        <v>3000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="464">
@@ -9601,10 +9607,10 @@
         <v>990</v>
       </c>
       <c r="C464" s="0" t="s">
-        <v>38</v>
+        <v>322</v>
       </c>
       <c r="D464" s="0">
-        <v>618</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="465">
@@ -9615,24 +9621,24 @@
         <v>992</v>
       </c>
       <c r="C465" s="0" t="s">
-        <v>993</v>
+        <v>38</v>
       </c>
       <c r="D465" s="0">
-        <v>24600</v>
+        <v>618</v>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="0" t="s">
+        <v>993</v>
+      </c>
+      <c r="B466" s="0" t="s">
         <v>994</v>
       </c>
-      <c r="B466" s="0" t="s">
+      <c r="C466" s="0" t="s">
         <v>995</v>
       </c>
-      <c r="C466" s="0" t="s">
-        <v>102</v>
-      </c>
       <c r="D466" s="0">
-        <v>0</v>
+        <v>24600</v>
       </c>
     </row>
     <row r="467">
@@ -9643,10 +9649,10 @@
         <v>997</v>
       </c>
       <c r="C467" s="0" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="D467" s="0">
-        <v>28283.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="468">
@@ -9657,10 +9663,10 @@
         <v>999</v>
       </c>
       <c r="C468" s="0" t="s">
-        <v>359</v>
+        <v>89</v>
       </c>
       <c r="D468" s="0">
-        <v>75529.41</v>
+        <v>32942.25</v>
       </c>
     </row>
     <row r="469">
@@ -9674,7 +9680,7 @@
         <v>359</v>
       </c>
       <c r="D469" s="0">
-        <v>41613</v>
+        <v>75529.41</v>
       </c>
     </row>
     <row r="470">
@@ -9688,7 +9694,7 @@
         <v>359</v>
       </c>
       <c r="D470" s="0">
-        <v>87056</v>
+        <v>41613</v>
       </c>
     </row>
     <row r="471">
@@ -9702,7 +9708,7 @@
         <v>359</v>
       </c>
       <c r="D471" s="0">
-        <v>49243.16</v>
+        <v>87056</v>
       </c>
     </row>
     <row r="472">
@@ -9713,10 +9719,10 @@
         <v>1007</v>
       </c>
       <c r="C472" s="0" t="s">
-        <v>22</v>
+        <v>359</v>
       </c>
       <c r="D472" s="0">
-        <v>1600</v>
+        <v>49243.16</v>
       </c>
     </row>
     <row r="473">
@@ -9727,10 +9733,10 @@
         <v>1009</v>
       </c>
       <c r="C473" s="0" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D473" s="0">
-        <v>3270.2</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="474">
@@ -9744,7 +9750,7 @@
         <v>29</v>
       </c>
       <c r="D474" s="0">
-        <v>3905</v>
+        <v>3270.2</v>
       </c>
     </row>
     <row r="475">
@@ -9758,7 +9764,7 @@
         <v>29</v>
       </c>
       <c r="D475" s="0">
-        <v>3950.91</v>
+        <v>3905</v>
       </c>
     </row>
     <row r="476">
@@ -9772,35 +9778,35 @@
         <v>29</v>
       </c>
       <c r="D476" s="0">
+        <v>3950.91</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="0" t="s">
+        <v>1016</v>
+      </c>
+      <c r="B477" s="0" t="s">
+        <v>1017</v>
+      </c>
+      <c r="C477" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D477" s="0">
         <v>3313.05</v>
       </c>
     </row>
-    <row r="477">
-      <c r="A477" s="2" t="s">
-        <v>1016</v>
-      </c>
-      <c r="B477" s="2" t="s">
-        <v>1017</v>
-      </c>
-      <c r="C477" s="2" t="s">
+    <row r="478">
+      <c r="A478" s="2" t="s">
+        <v>1018</v>
+      </c>
+      <c r="B478" s="2" t="s">
+        <v>1019</v>
+      </c>
+      <c r="C478" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D477" s="2">
+      <c r="D478" s="2">
         <v>0</v>
-      </c>
-    </row>
-    <row r="478">
-      <c r="A478" s="0" t="s">
-        <v>1018</v>
-      </c>
-      <c r="B478" s="0" t="s">
-        <v>1019</v>
-      </c>
-      <c r="C478" s="0" t="s">
-        <v>147</v>
-      </c>
-      <c r="D478" s="0">
-        <v>430</v>
       </c>
     </row>
     <row r="479">
@@ -9811,9 +9817,23 @@
         <v>1021</v>
       </c>
       <c r="C479" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="D479" s="0">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="0" t="s">
+        <v>1022</v>
+      </c>
+      <c r="B480" s="0" t="s">
+        <v>1023</v>
+      </c>
+      <c r="C480" s="0" t="s">
         <v>129</v>
       </c>
-      <c r="D479" s="0">
+      <c r="D480" s="0">
         <v>435</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: stock y precios actualizados vie. 19/06/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -3226,7 +3226,7 @@
         <v>16</v>
       </c>
       <c r="D8" s="0">
-        <v>18500</v>
+        <v>19800</v>
       </c>
     </row>
     <row r="9">
@@ -3730,7 +3730,7 @@
         <v>16</v>
       </c>
       <c r="D44" s="0">
-        <v>2800</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="45">
@@ -3926,7 +3926,7 @@
         <v>16</v>
       </c>
       <c r="D58" s="0">
-        <v>440</v>
+        <v>484</v>
       </c>
     </row>
     <row r="59">
@@ -4122,7 +4122,7 @@
         <v>16</v>
       </c>
       <c r="D72" s="0">
-        <v>1770</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="73">
@@ -4444,7 +4444,7 @@
         <v>16</v>
       </c>
       <c r="D95" s="0">
-        <v>1600</v>
+        <v>1760</v>
       </c>
     </row>
     <row r="96">
@@ -4584,7 +4584,7 @@
         <v>16</v>
       </c>
       <c r="D105" s="0">
-        <v>1650</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="106">
@@ -4640,7 +4640,7 @@
         <v>249</v>
       </c>
       <c r="D109" s="0">
-        <v>2660</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="110">
@@ -5130,7 +5130,7 @@
         <v>16</v>
       </c>
       <c r="D144" s="0">
-        <v>400</v>
+        <v>500</v>
       </c>
     </row>
     <row r="145">
@@ -5186,7 +5186,7 @@
         <v>16</v>
       </c>
       <c r="D148" s="0">
-        <v>520</v>
+        <v>572</v>
       </c>
     </row>
     <row r="149">
@@ -6362,7 +6362,7 @@
         <v>16</v>
       </c>
       <c r="D232" s="0">
-        <v>1000</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="233">
@@ -6432,7 +6432,7 @@
         <v>16</v>
       </c>
       <c r="D237" s="0">
-        <v>750</v>
+        <v>825</v>
       </c>
     </row>
     <row r="238">
@@ -6446,7 +6446,7 @@
         <v>16</v>
       </c>
       <c r="D238" s="0">
-        <v>33</v>
+        <v>36.3</v>
       </c>
     </row>
     <row r="239">
@@ -6460,7 +6460,7 @@
         <v>16</v>
       </c>
       <c r="D239" s="0">
-        <v>495</v>
+        <v>544.5</v>
       </c>
     </row>
     <row r="240">
@@ -6558,7 +6558,7 @@
         <v>16</v>
       </c>
       <c r="D246" s="0">
-        <v>820</v>
+        <v>902</v>
       </c>
     </row>
     <row r="247">
@@ -6866,7 +6866,7 @@
         <v>16</v>
       </c>
       <c r="D268" s="0">
-        <v>1500</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="269">
@@ -6894,7 +6894,7 @@
         <v>16</v>
       </c>
       <c r="D270" s="0">
-        <v>1800</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="271">
@@ -6964,7 +6964,7 @@
         <v>16</v>
       </c>
       <c r="D275" s="0">
-        <v>6500</v>
+        <v>6700</v>
       </c>
     </row>
     <row r="276">
@@ -7426,7 +7426,7 @@
         <v>16</v>
       </c>
       <c r="D308" s="0">
-        <v>780</v>
+        <v>973.5</v>
       </c>
     </row>
     <row r="309">
@@ -7678,7 +7678,7 @@
         <v>16</v>
       </c>
       <c r="D326" s="0">
-        <v>1900</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="327">
@@ -7930,7 +7930,7 @@
         <v>16</v>
       </c>
       <c r="D344" s="0">
-        <v>1000</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="345">
@@ -8000,7 +8000,7 @@
         <v>16</v>
       </c>
       <c r="D349" s="0">
-        <v>420</v>
+        <v>450</v>
       </c>
     </row>
     <row r="350">
@@ -8014,7 +8014,7 @@
         <v>16</v>
       </c>
       <c r="D350" s="0">
-        <v>750</v>
+        <v>825</v>
       </c>
     </row>
     <row r="351">
@@ -8028,7 +8028,7 @@
         <v>16</v>
       </c>
       <c r="D351" s="0">
-        <v>750</v>
+        <v>825</v>
       </c>
     </row>
     <row r="352">
@@ -8280,7 +8280,7 @@
         <v>16</v>
       </c>
       <c r="D369" s="0">
-        <v>2500</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="370">
@@ -8392,7 +8392,7 @@
         <v>16</v>
       </c>
       <c r="D377" s="0">
-        <v>2100</v>
+        <v>2948</v>
       </c>
     </row>
     <row r="378">
@@ -9456,7 +9456,7 @@
         <v>16</v>
       </c>
       <c r="D453" s="0">
-        <v>3200</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="454">
@@ -9526,7 +9526,7 @@
         <v>16</v>
       </c>
       <c r="D458" s="0">
-        <v>3500</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="459">

</xml_diff>

<commit_message>
sync: stock y precios actualizados sáb. 20/06/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -3296,7 +3296,7 @@
         <v>29</v>
       </c>
       <c r="D13" s="0">
-        <v>129.36</v>
+        <v>132.08</v>
       </c>
     </row>
     <row r="14">
@@ -3464,7 +3464,7 @@
         <v>29</v>
       </c>
       <c r="D25" s="0">
-        <v>153.92</v>
+        <v>157.16</v>
       </c>
     </row>
     <row r="26">
@@ -4850,7 +4850,7 @@
         <v>29</v>
       </c>
       <c r="D124" s="0">
-        <v>6842.5</v>
+        <v>6986.2</v>
       </c>
     </row>
     <row r="125">
@@ -5200,7 +5200,7 @@
         <v>29</v>
       </c>
       <c r="D149" s="0">
-        <v>80100</v>
+        <v>97734</v>
       </c>
     </row>
     <row r="150">
@@ -5214,7 +5214,7 @@
         <v>29</v>
       </c>
       <c r="D150" s="0">
-        <v>86457.1</v>
+        <v>105490.7</v>
       </c>
     </row>
     <row r="151">
@@ -5228,7 +5228,7 @@
         <v>29</v>
       </c>
       <c r="D151" s="0">
-        <v>108071.4</v>
+        <v>131863.3</v>
       </c>
     </row>
     <row r="152">
@@ -5396,7 +5396,7 @@
         <v>29</v>
       </c>
       <c r="D163" s="0">
-        <v>930.5</v>
+        <v>950</v>
       </c>
     </row>
     <row r="164">
@@ -5788,7 +5788,7 @@
         <v>29</v>
       </c>
       <c r="D191" s="0">
-        <v>310.7</v>
+        <v>317.2</v>
       </c>
     </row>
     <row r="192">
@@ -6390,7 +6390,7 @@
         <v>29</v>
       </c>
       <c r="D234" s="0">
-        <v>12682.6</v>
+        <v>13304.2</v>
       </c>
     </row>
     <row r="235">
@@ -7076,7 +7076,7 @@
         <v>29</v>
       </c>
       <c r="D283" s="0">
-        <v>7086.15</v>
+        <v>7234.96</v>
       </c>
     </row>
     <row r="284">
@@ -7986,7 +7986,7 @@
         <v>29</v>
       </c>
       <c r="D348" s="0">
-        <v>1869.6</v>
+        <v>1908.8</v>
       </c>
     </row>
     <row r="349">
@@ -8504,7 +8504,7 @@
         <v>29</v>
       </c>
       <c r="D385" s="0">
-        <v>686.98</v>
+        <v>701.42</v>
       </c>
     </row>
     <row r="386">
@@ -9232,7 +9232,7 @@
         <v>29</v>
       </c>
       <c r="D437" s="0">
-        <v>5795.46</v>
+        <v>5917.17</v>
       </c>
     </row>
     <row r="438">
@@ -9554,7 +9554,7 @@
         <v>29</v>
       </c>
       <c r="D460" s="0">
-        <v>13075</v>
+        <v>13715</v>
       </c>
     </row>
     <row r="461">
@@ -9750,7 +9750,7 @@
         <v>29</v>
       </c>
       <c r="D474" s="0">
-        <v>3270.2</v>
+        <v>3338.9</v>
       </c>
     </row>
     <row r="475">
@@ -9764,7 +9764,7 @@
         <v>29</v>
       </c>
       <c r="D475" s="0">
-        <v>3905</v>
+        <v>3987</v>
       </c>
     </row>
     <row r="476">
@@ -9778,7 +9778,7 @@
         <v>29</v>
       </c>
       <c r="D476" s="0">
-        <v>3950.91</v>
+        <v>4010.17</v>
       </c>
     </row>
     <row r="477">
@@ -9792,7 +9792,7 @@
         <v>29</v>
       </c>
       <c r="D477" s="0">
-        <v>3313.05</v>
+        <v>3382.65</v>
       </c>
     </row>
     <row r="478">

</xml_diff>

<commit_message>
sync: stock y precios actualizados vie. 26/06/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1053" uniqueCount="1053">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="1055">
   <si>
     <t>Código</t>
   </si>
@@ -1749,6 +1749,12 @@
   </si>
   <si>
     <t>INSULINA NOVORAPID PENFILL 100UI CART. X 5 X 3ML - 000010280</t>
+  </si>
+  <si>
+    <t>000024454</t>
+  </si>
+  <si>
+    <t>IODOPOVIDONA SOL TOP 10% X 30ML - KLOPOXONA - 000024454</t>
   </si>
   <si>
     <t>000001887</t>
@@ -3229,7 +3235,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A3:D493"/>
+  <dimension ref="A3:D494"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="3">
@@ -5007,7 +5013,7 @@
         <v>16</v>
       </c>
       <c r="D129" s="0">
-        <v>4000</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="130">
@@ -5483,7 +5489,7 @@
         <v>368</v>
       </c>
       <c r="D163" s="0">
-        <v>44902.12</v>
+        <v>52972.83</v>
       </c>
     </row>
     <row r="164">
@@ -5679,7 +5685,7 @@
         <v>368</v>
       </c>
       <c r="D177" s="0">
-        <v>36105</v>
+        <v>36105.51</v>
       </c>
     </row>
     <row r="178">
@@ -6894,24 +6900,24 @@
         <v>580</v>
       </c>
       <c r="C264" s="0" t="s">
-        <v>581</v>
+        <v>16</v>
       </c>
       <c r="D264" s="0">
-        <v>26350</v>
+        <v>1760</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="0" t="s">
+        <v>581</v>
+      </c>
+      <c r="B265" s="0" t="s">
         <v>582</v>
       </c>
-      <c r="B265" s="0" t="s">
+      <c r="C265" s="0" t="s">
         <v>583</v>
       </c>
-      <c r="C265" s="0" t="s">
-        <v>478</v>
-      </c>
       <c r="D265" s="0">
-        <v>31250</v>
+        <v>26350</v>
       </c>
     </row>
     <row r="266">
@@ -6922,10 +6928,10 @@
         <v>585</v>
       </c>
       <c r="C266" s="0" t="s">
-        <v>51</v>
+        <v>478</v>
       </c>
       <c r="D266" s="0">
-        <v>34.98</v>
+        <v>31250</v>
       </c>
     </row>
     <row r="267">
@@ -6939,7 +6945,7 @@
         <v>51</v>
       </c>
       <c r="D267" s="0">
-        <v>65</v>
+        <v>34.98</v>
       </c>
     </row>
     <row r="268">
@@ -6953,7 +6959,7 @@
         <v>51</v>
       </c>
       <c r="D268" s="0">
-        <v>92</v>
+        <v>65</v>
       </c>
     </row>
     <row r="269">
@@ -6967,7 +6973,7 @@
         <v>51</v>
       </c>
       <c r="D269" s="0">
-        <v>33</v>
+        <v>92</v>
       </c>
     </row>
     <row r="270">
@@ -6981,7 +6987,7 @@
         <v>51</v>
       </c>
       <c r="D270" s="0">
-        <v>38.22</v>
+        <v>33</v>
       </c>
     </row>
     <row r="271">
@@ -6992,10 +6998,10 @@
         <v>595</v>
       </c>
       <c r="C271" s="0" t="s">
-        <v>331</v>
+        <v>51</v>
       </c>
       <c r="D271" s="0">
-        <v>300</v>
+        <v>38.22</v>
       </c>
     </row>
     <row r="272">
@@ -7009,7 +7015,7 @@
         <v>331</v>
       </c>
       <c r="D272" s="0">
-        <v>370</v>
+        <v>300</v>
       </c>
     </row>
     <row r="273">
@@ -7020,10 +7026,10 @@
         <v>599</v>
       </c>
       <c r="C273" s="0" t="s">
-        <v>352</v>
+        <v>331</v>
       </c>
       <c r="D273" s="0">
-        <v>400</v>
+        <v>370</v>
       </c>
     </row>
     <row r="274">
@@ -7034,10 +7040,10 @@
         <v>601</v>
       </c>
       <c r="C274" s="0" t="s">
-        <v>16</v>
+        <v>352</v>
       </c>
       <c r="D274" s="0">
-        <v>510</v>
+        <v>400</v>
       </c>
     </row>
     <row r="275">
@@ -7051,7 +7057,7 @@
         <v>16</v>
       </c>
       <c r="D275" s="0">
-        <v>1650</v>
+        <v>510</v>
       </c>
     </row>
     <row r="276">
@@ -7065,7 +7071,7 @@
         <v>16</v>
       </c>
       <c r="D276" s="0">
-        <v>2100</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="277">
@@ -7079,7 +7085,7 @@
         <v>16</v>
       </c>
       <c r="D277" s="0">
-        <v>1980</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="278">
@@ -7093,7 +7099,7 @@
         <v>16</v>
       </c>
       <c r="D278" s="0">
-        <v>2160</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="279">
@@ -7107,7 +7113,7 @@
         <v>16</v>
       </c>
       <c r="D279" s="0">
-        <v>1100</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="280">
@@ -7121,7 +7127,7 @@
         <v>16</v>
       </c>
       <c r="D280" s="0">
-        <v>2600</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="281">
@@ -7135,7 +7141,7 @@
         <v>16</v>
       </c>
       <c r="D281" s="0">
-        <v>2000</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="282">
@@ -7149,7 +7155,7 @@
         <v>16</v>
       </c>
       <c r="D282" s="0">
-        <v>6700</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="283">
@@ -7163,7 +7169,7 @@
         <v>16</v>
       </c>
       <c r="D283" s="0">
-        <v>1650</v>
+        <v>6700</v>
       </c>
     </row>
     <row r="284">
@@ -7177,7 +7183,7 @@
         <v>16</v>
       </c>
       <c r="D284" s="0">
-        <v>1035</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="285">
@@ -7191,7 +7197,7 @@
         <v>16</v>
       </c>
       <c r="D285" s="0">
-        <v>2600</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="286">
@@ -7205,7 +7211,7 @@
         <v>16</v>
       </c>
       <c r="D286" s="0">
-        <v>2200</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="287">
@@ -7216,10 +7222,10 @@
         <v>627</v>
       </c>
       <c r="C287" s="0" t="s">
-        <v>132</v>
+        <v>16</v>
       </c>
       <c r="D287" s="0">
-        <v>4045</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="288">
@@ -7233,7 +7239,7 @@
         <v>132</v>
       </c>
       <c r="D288" s="0">
-        <v>2081</v>
+        <v>4045</v>
       </c>
     </row>
     <row r="289">
@@ -7247,7 +7253,7 @@
         <v>132</v>
       </c>
       <c r="D289" s="0">
-        <v>998</v>
+        <v>2081</v>
       </c>
     </row>
     <row r="290">
@@ -7258,10 +7264,10 @@
         <v>633</v>
       </c>
       <c r="C290" s="0" t="s">
-        <v>29</v>
+        <v>132</v>
       </c>
       <c r="D290" s="0">
-        <v>7234.96</v>
+        <v>998</v>
       </c>
     </row>
     <row r="291">
@@ -7272,10 +7278,10 @@
         <v>635</v>
       </c>
       <c r="C291" s="0" t="s">
-        <v>115</v>
+        <v>29</v>
       </c>
       <c r="D291" s="0">
-        <v>1790</v>
+        <v>7234.96</v>
       </c>
     </row>
     <row r="292">
@@ -7289,7 +7295,7 @@
         <v>115</v>
       </c>
       <c r="D292" s="0">
-        <v>2859.96</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="293">
@@ -7303,7 +7309,7 @@
         <v>115</v>
       </c>
       <c r="D293" s="0">
-        <v>4800</v>
+        <v>2859.96</v>
       </c>
     </row>
     <row r="294">
@@ -7314,24 +7320,24 @@
         <v>641</v>
       </c>
       <c r="C294" s="0" t="s">
-        <v>642</v>
+        <v>115</v>
       </c>
       <c r="D294" s="0">
-        <v>0</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="0" t="s">
+        <v>642</v>
+      </c>
+      <c r="B295" s="0" t="s">
         <v>643</v>
       </c>
-      <c r="B295" s="0" t="s">
+      <c r="C295" s="0" t="s">
         <v>644</v>
       </c>
-      <c r="C295" s="0" t="s">
-        <v>29</v>
-      </c>
       <c r="D295" s="0">
-        <v>494</v>
+        <v>0</v>
       </c>
     </row>
     <row r="296">
@@ -7345,7 +7351,7 @@
         <v>29</v>
       </c>
       <c r="D296" s="0">
-        <v>665.3</v>
+        <v>494</v>
       </c>
     </row>
     <row r="297">
@@ -7356,10 +7362,10 @@
         <v>648</v>
       </c>
       <c r="C297" s="0" t="s">
-        <v>89</v>
+        <v>29</v>
       </c>
       <c r="D297" s="0">
-        <v>32609.5</v>
+        <v>665.3</v>
       </c>
     </row>
     <row r="298">
@@ -7373,7 +7379,7 @@
         <v>89</v>
       </c>
       <c r="D298" s="0">
-        <v>4525.4</v>
+        <v>32609.5</v>
       </c>
     </row>
     <row r="299">
@@ -7384,10 +7390,10 @@
         <v>652</v>
       </c>
       <c r="C299" s="0" t="s">
-        <v>143</v>
+        <v>89</v>
       </c>
       <c r="D299" s="0">
-        <v>896</v>
+        <v>4525.4</v>
       </c>
     </row>
     <row r="300">
@@ -7398,10 +7404,10 @@
         <v>654</v>
       </c>
       <c r="C300" s="0" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="D300" s="0">
-        <v>1280</v>
+        <v>896</v>
       </c>
     </row>
     <row r="301">
@@ -7412,10 +7418,10 @@
         <v>656</v>
       </c>
       <c r="C301" s="0" t="s">
-        <v>89</v>
+        <v>132</v>
       </c>
       <c r="D301" s="0">
-        <v>306130</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="302">
@@ -7426,10 +7432,10 @@
         <v>658</v>
       </c>
       <c r="C302" s="0" t="s">
-        <v>197</v>
+        <v>89</v>
       </c>
       <c r="D302" s="0">
-        <v>17440</v>
+        <v>306130</v>
       </c>
     </row>
     <row r="303">
@@ -7443,7 +7449,7 @@
         <v>197</v>
       </c>
       <c r="D303" s="0">
-        <v>4390</v>
+        <v>17440</v>
       </c>
     </row>
     <row r="304">
@@ -7468,10 +7474,10 @@
         <v>664</v>
       </c>
       <c r="C305" s="0" t="s">
-        <v>276</v>
+        <v>197</v>
       </c>
       <c r="D305" s="0">
-        <v>2250</v>
+        <v>4390</v>
       </c>
     </row>
     <row r="306">
@@ -7482,10 +7488,10 @@
         <v>666</v>
       </c>
       <c r="C306" s="0" t="s">
-        <v>197</v>
+        <v>276</v>
       </c>
       <c r="D306" s="0">
-        <v>3355</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="307">
@@ -7496,10 +7502,10 @@
         <v>668</v>
       </c>
       <c r="C307" s="0" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="D307" s="0">
-        <v>7500</v>
+        <v>3355</v>
       </c>
     </row>
     <row r="308">
@@ -7510,10 +7516,10 @@
         <v>670</v>
       </c>
       <c r="C308" s="0" t="s">
-        <v>89</v>
+        <v>202</v>
       </c>
       <c r="D308" s="0">
-        <v>23958</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="309">
@@ -7527,7 +7533,7 @@
         <v>89</v>
       </c>
       <c r="D309" s="0">
-        <v>239580</v>
+        <v>23958</v>
       </c>
     </row>
     <row r="310">
@@ -7538,10 +7544,10 @@
         <v>674</v>
       </c>
       <c r="C310" s="0" t="s">
-        <v>51</v>
+        <v>89</v>
       </c>
       <c r="D310" s="0">
-        <v>130</v>
+        <v>239580</v>
       </c>
     </row>
     <row r="311">
@@ -7552,10 +7558,10 @@
         <v>676</v>
       </c>
       <c r="C311" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="D311" s="0">
-        <v>285.6</v>
+        <v>130</v>
       </c>
     </row>
     <row r="312">
@@ -7569,7 +7575,7 @@
         <v>22</v>
       </c>
       <c r="D312" s="0">
-        <v>338</v>
+        <v>285.6</v>
       </c>
     </row>
     <row r="313">
@@ -7580,21 +7586,21 @@
         <v>680</v>
       </c>
       <c r="C313" s="0" t="s">
-        <v>681</v>
+        <v>22</v>
       </c>
       <c r="D313" s="0">
-        <v>770</v>
+        <v>338</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="0" t="s">
+        <v>681</v>
+      </c>
+      <c r="B314" s="0" t="s">
         <v>682</v>
       </c>
-      <c r="B314" s="0" t="s">
+      <c r="C314" s="0" t="s">
         <v>683</v>
-      </c>
-      <c r="C314" s="0" t="s">
-        <v>684</v>
       </c>
       <c r="D314" s="0">
         <v>770</v>
@@ -7602,16 +7608,16 @@
     </row>
     <row r="315">
       <c r="A315" s="0" t="s">
+        <v>684</v>
+      </c>
+      <c r="B315" s="0" t="s">
         <v>685</v>
       </c>
-      <c r="B315" s="0" t="s">
+      <c r="C315" s="0" t="s">
         <v>686</v>
       </c>
-      <c r="C315" s="0" t="s">
-        <v>16</v>
-      </c>
       <c r="D315" s="0">
-        <v>973.5</v>
+        <v>770</v>
       </c>
     </row>
     <row r="316">
@@ -7622,10 +7628,10 @@
         <v>688</v>
       </c>
       <c r="C316" s="0" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D316" s="0">
-        <v>507.08</v>
+        <v>973.5</v>
       </c>
     </row>
     <row r="317">
@@ -7636,10 +7642,10 @@
         <v>690</v>
       </c>
       <c r="C317" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D317" s="0">
-        <v>450</v>
+        <v>507.08</v>
       </c>
     </row>
     <row r="318">
@@ -7650,10 +7656,10 @@
         <v>692</v>
       </c>
       <c r="C318" s="0" t="s">
-        <v>143</v>
+        <v>16</v>
       </c>
       <c r="D318" s="0">
-        <v>760</v>
+        <v>450</v>
       </c>
     </row>
     <row r="319">
@@ -7664,10 +7670,10 @@
         <v>694</v>
       </c>
       <c r="C319" s="0" t="s">
-        <v>276</v>
+        <v>143</v>
       </c>
       <c r="D319" s="0">
-        <v>5900</v>
+        <v>760</v>
       </c>
     </row>
     <row r="320">
@@ -7681,7 +7687,7 @@
         <v>276</v>
       </c>
       <c r="D320" s="0">
-        <v>2900</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="321">
@@ -7692,10 +7698,10 @@
         <v>698</v>
       </c>
       <c r="C321" s="0" t="s">
-        <v>132</v>
+        <v>276</v>
       </c>
       <c r="D321" s="0">
-        <v>797.4</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="322">
@@ -7709,7 +7715,7 @@
         <v>132</v>
       </c>
       <c r="D322" s="0">
-        <v>519</v>
+        <v>797.4</v>
       </c>
     </row>
     <row r="323">
@@ -7723,7 +7729,7 @@
         <v>132</v>
       </c>
       <c r="D323" s="0">
-        <v>62</v>
+        <v>519</v>
       </c>
     </row>
     <row r="324">
@@ -7734,10 +7740,10 @@
         <v>704</v>
       </c>
       <c r="C324" s="0" t="s">
-        <v>89</v>
+        <v>132</v>
       </c>
       <c r="D324" s="0">
-        <v>11313.5</v>
+        <v>62</v>
       </c>
     </row>
     <row r="325">
@@ -7748,10 +7754,10 @@
         <v>706</v>
       </c>
       <c r="C325" s="0" t="s">
-        <v>35</v>
+        <v>89</v>
       </c>
       <c r="D325" s="0">
-        <v>418</v>
+        <v>11313.5</v>
       </c>
     </row>
     <row r="326">
@@ -7762,7 +7768,7 @@
         <v>708</v>
       </c>
       <c r="C326" s="0" t="s">
-        <v>352</v>
+        <v>35</v>
       </c>
       <c r="D326" s="0">
         <v>418</v>
@@ -7776,10 +7782,10 @@
         <v>710</v>
       </c>
       <c r="C327" s="0" t="s">
-        <v>22</v>
+        <v>352</v>
       </c>
       <c r="D327" s="0">
-        <v>377</v>
+        <v>418</v>
       </c>
     </row>
     <row r="328">
@@ -7790,10 +7796,10 @@
         <v>712</v>
       </c>
       <c r="C328" s="0" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="D328" s="0">
-        <v>3860.67</v>
+        <v>377</v>
       </c>
     </row>
     <row r="329">
@@ -7804,10 +7810,10 @@
         <v>714</v>
       </c>
       <c r="C329" s="0" t="s">
-        <v>69</v>
+        <v>44</v>
       </c>
       <c r="D329" s="0">
-        <v>898</v>
+        <v>3860.67</v>
       </c>
     </row>
     <row r="330">
@@ -7818,10 +7824,10 @@
         <v>716</v>
       </c>
       <c r="C330" s="0" t="s">
-        <v>115</v>
+        <v>69</v>
       </c>
       <c r="D330" s="0">
-        <v>4767</v>
+        <v>898</v>
       </c>
     </row>
     <row r="331">
@@ -7832,10 +7838,10 @@
         <v>718</v>
       </c>
       <c r="C331" s="0" t="s">
-        <v>35</v>
+        <v>115</v>
       </c>
       <c r="D331" s="0">
-        <v>650</v>
+        <v>4767</v>
       </c>
     </row>
     <row r="332">
@@ -7846,7 +7852,7 @@
         <v>720</v>
       </c>
       <c r="C332" s="0" t="s">
-        <v>69</v>
+        <v>35</v>
       </c>
       <c r="D332" s="0">
         <v>650</v>
@@ -7860,10 +7866,10 @@
         <v>722</v>
       </c>
       <c r="C333" s="0" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="D333" s="0">
-        <v>2178</v>
+        <v>650</v>
       </c>
     </row>
     <row r="334">
@@ -7874,10 +7880,10 @@
         <v>724</v>
       </c>
       <c r="C334" s="0" t="s">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="D334" s="0">
-        <v>7986</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="335">
@@ -7888,24 +7894,24 @@
         <v>726</v>
       </c>
       <c r="C335" s="0" t="s">
-        <v>727</v>
+        <v>89</v>
       </c>
       <c r="D335" s="0">
-        <v>1800</v>
+        <v>7986</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="0" t="s">
+        <v>727</v>
+      </c>
+      <c r="B336" s="0" t="s">
         <v>728</v>
       </c>
-      <c r="B336" s="0" t="s">
+      <c r="C336" s="0" t="s">
         <v>729</v>
       </c>
-      <c r="C336" s="0" t="s">
-        <v>143</v>
-      </c>
       <c r="D336" s="0">
-        <v>900</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="337">
@@ -7916,10 +7922,10 @@
         <v>731</v>
       </c>
       <c r="C337" s="0" t="s">
-        <v>22</v>
+        <v>143</v>
       </c>
       <c r="D337" s="0">
-        <v>1722</v>
+        <v>900</v>
       </c>
     </row>
     <row r="338">
@@ -7930,10 +7936,10 @@
         <v>733</v>
       </c>
       <c r="C338" s="0" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="D338" s="0">
-        <v>456</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="339">
@@ -7947,7 +7953,7 @@
         <v>35</v>
       </c>
       <c r="D339" s="0">
-        <v>45600</v>
+        <v>456</v>
       </c>
     </row>
     <row r="340">
@@ -7958,10 +7964,10 @@
         <v>737</v>
       </c>
       <c r="C340" s="0" t="s">
-        <v>143</v>
+        <v>35</v>
       </c>
       <c r="D340" s="0">
-        <v>750</v>
+        <v>45600</v>
       </c>
     </row>
     <row r="341">
@@ -7975,7 +7981,7 @@
         <v>143</v>
       </c>
       <c r="D341" s="0">
-        <v>1212</v>
+        <v>750</v>
       </c>
     </row>
     <row r="342">
@@ -7989,7 +7995,7 @@
         <v>143</v>
       </c>
       <c r="D342" s="0">
-        <v>1300</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="343">
@@ -8003,7 +8009,7 @@
         <v>143</v>
       </c>
       <c r="D343" s="0">
-        <v>1500</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="344">
@@ -8017,7 +8023,7 @@
         <v>143</v>
       </c>
       <c r="D344" s="0">
-        <v>1400</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="345">
@@ -8028,10 +8034,10 @@
         <v>747</v>
       </c>
       <c r="C345" s="0" t="s">
-        <v>252</v>
+        <v>143</v>
       </c>
       <c r="D345" s="0">
-        <v>11959</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="346">
@@ -8042,10 +8048,10 @@
         <v>749</v>
       </c>
       <c r="C346" s="0" t="s">
-        <v>132</v>
+        <v>252</v>
       </c>
       <c r="D346" s="0">
-        <v>300</v>
+        <v>11959</v>
       </c>
     </row>
     <row r="347">
@@ -8056,10 +8062,10 @@
         <v>751</v>
       </c>
       <c r="C347" s="0" t="s">
-        <v>276</v>
+        <v>132</v>
       </c>
       <c r="D347" s="0">
-        <v>1450</v>
+        <v>300</v>
       </c>
     </row>
     <row r="348">
@@ -8070,10 +8076,10 @@
         <v>753</v>
       </c>
       <c r="C348" s="0" t="s">
-        <v>89</v>
+        <v>276</v>
       </c>
       <c r="D348" s="0">
-        <v>7320.5</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="349">
@@ -8084,10 +8090,10 @@
         <v>755</v>
       </c>
       <c r="C349" s="0" t="s">
-        <v>16</v>
+        <v>89</v>
       </c>
       <c r="D349" s="0">
-        <v>900</v>
+        <v>7320.5</v>
       </c>
     </row>
     <row r="350">
@@ -8098,10 +8104,10 @@
         <v>757</v>
       </c>
       <c r="C350" s="0" t="s">
-        <v>276</v>
+        <v>16</v>
       </c>
       <c r="D350" s="0">
-        <v>520</v>
+        <v>900</v>
       </c>
     </row>
     <row r="351">
@@ -8112,10 +8118,10 @@
         <v>759</v>
       </c>
       <c r="C351" s="0" t="s">
-        <v>469</v>
+        <v>276</v>
       </c>
       <c r="D351" s="0">
-        <v>64925</v>
+        <v>520</v>
       </c>
     </row>
     <row r="352">
@@ -8126,10 +8132,10 @@
         <v>761</v>
       </c>
       <c r="C352" s="0" t="s">
-        <v>16</v>
+        <v>469</v>
       </c>
       <c r="D352" s="0">
-        <v>1100</v>
+        <v>64925</v>
       </c>
     </row>
     <row r="353">
@@ -8140,10 +8146,10 @@
         <v>763</v>
       </c>
       <c r="C353" s="0" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D353" s="0">
-        <v>1623</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="354">
@@ -8154,10 +8160,10 @@
         <v>765</v>
       </c>
       <c r="C354" s="0" t="s">
-        <v>132</v>
+        <v>22</v>
       </c>
       <c r="D354" s="0">
-        <v>1116.03</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="355">
@@ -8171,7 +8177,7 @@
         <v>132</v>
       </c>
       <c r="D355" s="0">
-        <v>4028.88</v>
+        <v>1116.03</v>
       </c>
     </row>
     <row r="356">
@@ -8182,10 +8188,10 @@
         <v>769</v>
       </c>
       <c r="C356" s="0" t="s">
-        <v>29</v>
+        <v>132</v>
       </c>
       <c r="D356" s="0">
-        <v>1650</v>
+        <v>4028.88</v>
       </c>
     </row>
     <row r="357">
@@ -8199,7 +8205,7 @@
         <v>29</v>
       </c>
       <c r="D357" s="0">
-        <v>1908.8</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="358">
@@ -8210,10 +8216,10 @@
         <v>773</v>
       </c>
       <c r="C358" s="0" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="D358" s="0">
-        <v>450</v>
+        <v>1908.8</v>
       </c>
     </row>
     <row r="359">
@@ -8227,7 +8233,7 @@
         <v>16</v>
       </c>
       <c r="D359" s="0">
-        <v>825</v>
+        <v>450</v>
       </c>
     </row>
     <row r="360">
@@ -8252,10 +8258,10 @@
         <v>779</v>
       </c>
       <c r="C361" s="0" t="s">
-        <v>371</v>
+        <v>16</v>
       </c>
       <c r="D361" s="0">
-        <v>134775.6</v>
+        <v>825</v>
       </c>
     </row>
     <row r="362">
@@ -8269,7 +8275,7 @@
         <v>371</v>
       </c>
       <c r="D362" s="0">
-        <v>175991.55</v>
+        <v>134775.6</v>
       </c>
     </row>
     <row r="363">
@@ -8280,10 +8286,10 @@
         <v>783</v>
       </c>
       <c r="C363" s="0" t="s">
-        <v>69</v>
+        <v>371</v>
       </c>
       <c r="D363" s="0">
-        <v>3263</v>
+        <v>175991.55</v>
       </c>
     </row>
     <row r="364">
@@ -8297,7 +8303,7 @@
         <v>69</v>
       </c>
       <c r="D364" s="0">
-        <v>18027</v>
+        <v>3263</v>
       </c>
     </row>
     <row r="365">
@@ -8308,10 +8314,10 @@
         <v>787</v>
       </c>
       <c r="C365" s="0" t="s">
-        <v>276</v>
+        <v>69</v>
       </c>
       <c r="D365" s="0">
-        <v>515</v>
+        <v>18027</v>
       </c>
     </row>
     <row r="366">
@@ -8322,38 +8328,38 @@
         <v>789</v>
       </c>
       <c r="C366" s="0" t="s">
-        <v>38</v>
+        <v>276</v>
       </c>
       <c r="D366" s="0">
         <v>515</v>
       </c>
     </row>
     <row r="367">
-      <c r="A367" s="2" t="s">
+      <c r="A367" s="0" t="s">
         <v>790</v>
       </c>
-      <c r="B367" s="2" t="s">
+      <c r="B367" s="0" t="s">
         <v>791</v>
       </c>
-      <c r="C367" s="2" t="s">
+      <c r="C367" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="D367" s="0">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="2" t="s">
+        <v>792</v>
+      </c>
+      <c r="B368" s="2" t="s">
+        <v>793</v>
+      </c>
+      <c r="C368" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D367" s="2">
+      <c r="D368" s="2">
         <v>10154</v>
-      </c>
-    </row>
-    <row r="368">
-      <c r="A368" s="0" t="s">
-        <v>792</v>
-      </c>
-      <c r="B368" s="0" t="s">
-        <v>793</v>
-      </c>
-      <c r="C368" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="D368" s="0">
-        <v>9500</v>
       </c>
     </row>
     <row r="369">
@@ -8364,10 +8370,10 @@
         <v>795</v>
       </c>
       <c r="C369" s="0" t="s">
-        <v>469</v>
+        <v>51</v>
       </c>
       <c r="D369" s="0">
-        <v>207558.08</v>
+        <v>9500</v>
       </c>
     </row>
     <row r="370">
@@ -8381,7 +8387,7 @@
         <v>469</v>
       </c>
       <c r="D370" s="0">
-        <v>249069.69</v>
+        <v>207558.08</v>
       </c>
     </row>
     <row r="371">
@@ -8392,10 +8398,10 @@
         <v>799</v>
       </c>
       <c r="C371" s="0" t="s">
-        <v>69</v>
+        <v>469</v>
       </c>
       <c r="D371" s="0">
-        <v>10021.22</v>
+        <v>249069.69</v>
       </c>
     </row>
     <row r="372">
@@ -8409,7 +8415,7 @@
         <v>69</v>
       </c>
       <c r="D372" s="0">
-        <v>17710</v>
+        <v>10021.22</v>
       </c>
     </row>
     <row r="373">
@@ -8420,24 +8426,24 @@
         <v>803</v>
       </c>
       <c r="C373" s="0" t="s">
-        <v>804</v>
+        <v>69</v>
       </c>
       <c r="D373" s="0">
-        <v>1080</v>
+        <v>17710</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="0" t="s">
+        <v>804</v>
+      </c>
+      <c r="B374" s="0" t="s">
         <v>805</v>
       </c>
-      <c r="B374" s="0" t="s">
+      <c r="C374" s="0" t="s">
         <v>806</v>
       </c>
-      <c r="C374" s="0" t="s">
-        <v>19</v>
-      </c>
       <c r="D374" s="0">
-        <v>691.03</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="375">
@@ -8448,24 +8454,24 @@
         <v>808</v>
       </c>
       <c r="C375" s="0" t="s">
-        <v>809</v>
+        <v>19</v>
       </c>
       <c r="D375" s="0">
-        <v>520</v>
+        <v>691.03</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="0" t="s">
+        <v>809</v>
+      </c>
+      <c r="B376" s="0" t="s">
         <v>810</v>
       </c>
-      <c r="B376" s="0" t="s">
+      <c r="C376" s="0" t="s">
         <v>811</v>
       </c>
-      <c r="C376" s="0" t="s">
-        <v>809</v>
-      </c>
       <c r="D376" s="0">
-        <v>300</v>
+        <v>520</v>
       </c>
     </row>
     <row r="377">
@@ -8476,10 +8482,10 @@
         <v>813</v>
       </c>
       <c r="C377" s="0" t="s">
-        <v>16</v>
+        <v>811</v>
       </c>
       <c r="D377" s="0">
-        <v>2200</v>
+        <v>300</v>
       </c>
     </row>
     <row r="378">
@@ -8493,7 +8499,7 @@
         <v>16</v>
       </c>
       <c r="D378" s="0">
-        <v>2800</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="379">
@@ -8504,10 +8510,10 @@
         <v>817</v>
       </c>
       <c r="C379" s="0" t="s">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="D379" s="0">
-        <v>4791.6</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="380">
@@ -8518,10 +8524,10 @@
         <v>819</v>
       </c>
       <c r="C380" s="0" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="D380" s="0">
-        <v>2699.64</v>
+        <v>4791.6</v>
       </c>
     </row>
     <row r="381">
@@ -8532,10 +8538,10 @@
         <v>821</v>
       </c>
       <c r="C381" s="0" t="s">
-        <v>35</v>
+        <v>69</v>
       </c>
       <c r="D381" s="0">
-        <v>3800</v>
+        <v>2699.64</v>
       </c>
     </row>
     <row r="382">
@@ -8546,10 +8552,10 @@
         <v>823</v>
       </c>
       <c r="C382" s="0" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D382" s="0">
-        <v>4000</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="383">
@@ -8560,24 +8566,24 @@
         <v>825</v>
       </c>
       <c r="C383" s="0" t="s">
-        <v>826</v>
+        <v>16</v>
       </c>
       <c r="D383" s="0">
-        <v>3800</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="384">
       <c r="A384" s="0" t="s">
+        <v>826</v>
+      </c>
+      <c r="B384" s="0" t="s">
         <v>827</v>
       </c>
-      <c r="B384" s="0" t="s">
+      <c r="C384" s="0" t="s">
         <v>828</v>
       </c>
-      <c r="C384" s="0" t="s">
-        <v>22</v>
-      </c>
       <c r="D384" s="0">
-        <v>353</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="385">
@@ -8588,10 +8594,10 @@
         <v>830</v>
       </c>
       <c r="C385" s="0" t="s">
-        <v>355</v>
+        <v>22</v>
       </c>
       <c r="D385" s="0">
-        <v>1800</v>
+        <v>353</v>
       </c>
     </row>
     <row r="386">
@@ -8602,10 +8608,10 @@
         <v>832</v>
       </c>
       <c r="C386" s="0" t="s">
-        <v>16</v>
+        <v>355</v>
       </c>
       <c r="D386" s="0">
-        <v>2948</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="387">
@@ -8616,10 +8622,10 @@
         <v>834</v>
       </c>
       <c r="C387" s="0" t="s">
-        <v>202</v>
+        <v>16</v>
       </c>
       <c r="D387" s="0">
-        <v>65537</v>
+        <v>2948</v>
       </c>
     </row>
     <row r="388">
@@ -8630,10 +8636,10 @@
         <v>836</v>
       </c>
       <c r="C388" s="0" t="s">
-        <v>132</v>
+        <v>202</v>
       </c>
       <c r="D388" s="0">
-        <v>3820.86</v>
+        <v>65537</v>
       </c>
     </row>
     <row r="389">
@@ -8647,7 +8653,7 @@
         <v>132</v>
       </c>
       <c r="D389" s="0">
-        <v>3962</v>
+        <v>3820.86</v>
       </c>
     </row>
     <row r="390">
@@ -8661,7 +8667,7 @@
         <v>132</v>
       </c>
       <c r="D390" s="0">
-        <v>5802.4</v>
+        <v>3962</v>
       </c>
     </row>
     <row r="391">
@@ -8672,10 +8678,10 @@
         <v>842</v>
       </c>
       <c r="C391" s="0" t="s">
-        <v>303</v>
+        <v>132</v>
       </c>
       <c r="D391" s="0">
-        <v>570</v>
+        <v>5802.4</v>
       </c>
     </row>
     <row r="392">
@@ -8686,10 +8692,10 @@
         <v>844</v>
       </c>
       <c r="C392" s="0" t="s">
-        <v>69</v>
+        <v>303</v>
       </c>
       <c r="D392" s="0">
-        <v>550</v>
+        <v>570</v>
       </c>
     </row>
     <row r="393">
@@ -8700,10 +8706,10 @@
         <v>846</v>
       </c>
       <c r="C393" s="0" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="D393" s="0">
-        <v>167</v>
+        <v>550</v>
       </c>
     </row>
     <row r="394">
@@ -8714,10 +8720,10 @@
         <v>848</v>
       </c>
       <c r="C394" s="0" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="D394" s="0">
-        <v>701.42</v>
+        <v>167</v>
       </c>
     </row>
     <row r="395">
@@ -8728,10 +8734,10 @@
         <v>850</v>
       </c>
       <c r="C395" s="0" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="D395" s="0">
-        <v>101000</v>
+        <v>701.42</v>
       </c>
     </row>
     <row r="396">
@@ -8742,10 +8748,10 @@
         <v>852</v>
       </c>
       <c r="C396" s="0" t="s">
-        <v>115</v>
+        <v>58</v>
       </c>
       <c r="D396" s="0">
-        <v>6251</v>
+        <v>101000</v>
       </c>
     </row>
     <row r="397">
@@ -8756,10 +8762,10 @@
         <v>854</v>
       </c>
       <c r="C397" s="0" t="s">
-        <v>368</v>
+        <v>115</v>
       </c>
       <c r="D397" s="0">
-        <v>857.67</v>
+        <v>6251</v>
       </c>
     </row>
     <row r="398">
@@ -8770,10 +8776,10 @@
         <v>856</v>
       </c>
       <c r="C398" s="0" t="s">
-        <v>89</v>
+        <v>368</v>
       </c>
       <c r="D398" s="0">
-        <v>1164.66</v>
+        <v>857.67</v>
       </c>
     </row>
     <row r="399">
@@ -8784,10 +8790,10 @@
         <v>858</v>
       </c>
       <c r="C399" s="0" t="s">
-        <v>143</v>
+        <v>89</v>
       </c>
       <c r="D399" s="0">
-        <v>360</v>
+        <v>1164.66</v>
       </c>
     </row>
     <row r="400">
@@ -8801,7 +8807,7 @@
         <v>143</v>
       </c>
       <c r="D400" s="0">
-        <v>450</v>
+        <v>360</v>
       </c>
     </row>
     <row r="401">
@@ -8815,7 +8821,7 @@
         <v>143</v>
       </c>
       <c r="D401" s="0">
-        <v>2050</v>
+        <v>450</v>
       </c>
     </row>
     <row r="402">
@@ -8826,10 +8832,10 @@
         <v>864</v>
       </c>
       <c r="C402" s="0" t="s">
-        <v>570</v>
+        <v>143</v>
       </c>
       <c r="D402" s="0">
-        <v>25192.82</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="403">
@@ -8840,10 +8846,10 @@
         <v>866</v>
       </c>
       <c r="C403" s="0" t="s">
-        <v>69</v>
+        <v>570</v>
       </c>
       <c r="D403" s="0">
-        <v>3500</v>
+        <v>25192.82</v>
       </c>
     </row>
     <row r="404">
@@ -8854,10 +8860,10 @@
         <v>868</v>
       </c>
       <c r="C404" s="0" t="s">
-        <v>170</v>
+        <v>69</v>
       </c>
       <c r="D404" s="0">
-        <v>600</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="405">
@@ -8868,24 +8874,24 @@
         <v>870</v>
       </c>
       <c r="C405" s="0" t="s">
-        <v>871</v>
+        <v>170</v>
       </c>
       <c r="D405" s="0">
-        <v>1080</v>
+        <v>600</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="0" t="s">
+        <v>871</v>
+      </c>
+      <c r="B406" s="0" t="s">
         <v>872</v>
       </c>
-      <c r="B406" s="0" t="s">
+      <c r="C406" s="0" t="s">
         <v>873</v>
       </c>
-      <c r="C406" s="0" t="s">
-        <v>331</v>
-      </c>
       <c r="D406" s="0">
-        <v>8628</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="407">
@@ -8899,7 +8905,7 @@
         <v>331</v>
       </c>
       <c r="D407" s="0">
-        <v>9125.1</v>
+        <v>8628</v>
       </c>
     </row>
     <row r="408">
@@ -8910,10 +8916,10 @@
         <v>877</v>
       </c>
       <c r="C408" s="0" t="s">
-        <v>41</v>
+        <v>331</v>
       </c>
       <c r="D408" s="0">
-        <v>27991.54</v>
+        <v>9125.1</v>
       </c>
     </row>
     <row r="409">
@@ -8924,10 +8930,10 @@
         <v>879</v>
       </c>
       <c r="C409" s="0" t="s">
-        <v>132</v>
+        <v>41</v>
       </c>
       <c r="D409" s="0">
-        <v>1080</v>
+        <v>27991.54</v>
       </c>
     </row>
     <row r="410">
@@ -8941,7 +8947,7 @@
         <v>132</v>
       </c>
       <c r="D410" s="0">
-        <v>4500</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="411">
@@ -8952,10 +8958,10 @@
         <v>883</v>
       </c>
       <c r="C411" s="0" t="s">
-        <v>44</v>
+        <v>132</v>
       </c>
       <c r="D411" s="0">
-        <v>4194.88</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="412">
@@ -8969,7 +8975,7 @@
         <v>44</v>
       </c>
       <c r="D412" s="0">
-        <v>2139.28</v>
+        <v>4194.88</v>
       </c>
     </row>
     <row r="413">
@@ -8983,7 +8989,7 @@
         <v>44</v>
       </c>
       <c r="D413" s="0">
-        <v>1699.1</v>
+        <v>2139.28</v>
       </c>
     </row>
     <row r="414">
@@ -8997,7 +9003,7 @@
         <v>44</v>
       </c>
       <c r="D414" s="0">
-        <v>3427.58</v>
+        <v>1699.1</v>
       </c>
     </row>
     <row r="415">
@@ -9011,7 +9017,7 @@
         <v>44</v>
       </c>
       <c r="D415" s="0">
-        <v>19700</v>
+        <v>3427.58</v>
       </c>
     </row>
     <row r="416">
@@ -9025,7 +9031,7 @@
         <v>44</v>
       </c>
       <c r="D416" s="0">
-        <v>1839.2</v>
+        <v>19700</v>
       </c>
     </row>
     <row r="417">
@@ -9039,7 +9045,7 @@
         <v>44</v>
       </c>
       <c r="D417" s="0">
-        <v>4215.45</v>
+        <v>1839.2</v>
       </c>
     </row>
     <row r="418">
@@ -9053,7 +9059,7 @@
         <v>44</v>
       </c>
       <c r="D418" s="0">
-        <v>3395.26</v>
+        <v>4215.45</v>
       </c>
     </row>
     <row r="419">
@@ -9064,10 +9070,10 @@
         <v>899</v>
       </c>
       <c r="C419" s="0" t="s">
-        <v>478</v>
+        <v>44</v>
       </c>
       <c r="D419" s="0">
-        <v>510</v>
+        <v>3395.26</v>
       </c>
     </row>
     <row r="420">
@@ -9078,7 +9084,7 @@
         <v>901</v>
       </c>
       <c r="C420" s="0" t="s">
-        <v>38</v>
+        <v>478</v>
       </c>
       <c r="D420" s="0">
         <v>510</v>
@@ -9092,21 +9098,21 @@
         <v>903</v>
       </c>
       <c r="C421" s="0" t="s">
-        <v>904</v>
+        <v>38</v>
       </c>
       <c r="D421" s="0">
-        <v>559</v>
+        <v>510</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="0" t="s">
+        <v>904</v>
+      </c>
+      <c r="B422" s="0" t="s">
         <v>905</v>
       </c>
-      <c r="B422" s="0" t="s">
+      <c r="C422" s="0" t="s">
         <v>906</v>
-      </c>
-      <c r="C422" s="0" t="s">
-        <v>904</v>
       </c>
       <c r="D422" s="0">
         <v>559</v>
@@ -9120,7 +9126,7 @@
         <v>908</v>
       </c>
       <c r="C423" s="0" t="s">
-        <v>904</v>
+        <v>906</v>
       </c>
       <c r="D423" s="0">
         <v>559</v>
@@ -9134,10 +9140,10 @@
         <v>910</v>
       </c>
       <c r="C424" s="0" t="s">
-        <v>904</v>
+        <v>906</v>
       </c>
       <c r="D424" s="0">
-        <v>342</v>
+        <v>559</v>
       </c>
     </row>
     <row r="425">
@@ -9148,7 +9154,7 @@
         <v>912</v>
       </c>
       <c r="C425" s="0" t="s">
-        <v>904</v>
+        <v>906</v>
       </c>
       <c r="D425" s="0">
         <v>342</v>
@@ -9162,7 +9168,7 @@
         <v>914</v>
       </c>
       <c r="C426" s="0" t="s">
-        <v>904</v>
+        <v>906</v>
       </c>
       <c r="D426" s="0">
         <v>342</v>
@@ -9176,10 +9182,10 @@
         <v>916</v>
       </c>
       <c r="C427" s="0" t="s">
-        <v>904</v>
+        <v>906</v>
       </c>
       <c r="D427" s="0">
-        <v>0</v>
+        <v>342</v>
       </c>
     </row>
     <row r="428">
@@ -9190,7 +9196,7 @@
         <v>918</v>
       </c>
       <c r="C428" s="0" t="s">
-        <v>904</v>
+        <v>906</v>
       </c>
       <c r="D428" s="0">
         <v>0</v>
@@ -9204,10 +9210,10 @@
         <v>920</v>
       </c>
       <c r="C429" s="0" t="s">
-        <v>904</v>
+        <v>906</v>
       </c>
       <c r="D429" s="0">
-        <v>423</v>
+        <v>0</v>
       </c>
     </row>
     <row r="430">
@@ -9218,10 +9224,10 @@
         <v>922</v>
       </c>
       <c r="C430" s="0" t="s">
-        <v>69</v>
+        <v>906</v>
       </c>
       <c r="D430" s="0">
-        <v>15968</v>
+        <v>423</v>
       </c>
     </row>
     <row r="431">
@@ -9232,10 +9238,10 @@
         <v>924</v>
       </c>
       <c r="C431" s="0" t="s">
-        <v>109</v>
+        <v>69</v>
       </c>
       <c r="D431" s="0">
-        <v>14000</v>
+        <v>15968</v>
       </c>
     </row>
     <row r="432">
@@ -9246,10 +9252,10 @@
         <v>926</v>
       </c>
       <c r="C432" s="0" t="s">
-        <v>132</v>
+        <v>109</v>
       </c>
       <c r="D432" s="0">
-        <v>14001</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="433">
@@ -9260,10 +9266,10 @@
         <v>928</v>
       </c>
       <c r="C433" s="0" t="s">
-        <v>89</v>
+        <v>132</v>
       </c>
       <c r="D433" s="0">
-        <v>266200</v>
+        <v>14001</v>
       </c>
     </row>
     <row r="434">
@@ -9277,7 +9283,7 @@
         <v>89</v>
       </c>
       <c r="D434" s="0">
-        <v>194991.5</v>
+        <v>266200</v>
       </c>
     </row>
     <row r="435">
@@ -9291,7 +9297,7 @@
         <v>89</v>
       </c>
       <c r="D435" s="0">
-        <v>289492.5</v>
+        <v>194991.5</v>
       </c>
     </row>
     <row r="436">
@@ -9302,24 +9308,24 @@
         <v>934</v>
       </c>
       <c r="C436" s="0" t="s">
-        <v>935</v>
+        <v>89</v>
       </c>
       <c r="D436" s="0">
-        <v>13722.52</v>
+        <v>289492.5</v>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="0" t="s">
+        <v>935</v>
+      </c>
+      <c r="B437" s="0" t="s">
         <v>936</v>
       </c>
-      <c r="B437" s="0" t="s">
+      <c r="C437" s="0" t="s">
         <v>937</v>
       </c>
-      <c r="C437" s="0" t="s">
-        <v>935</v>
-      </c>
       <c r="D437" s="0">
-        <v>15072</v>
+        <v>13722.52</v>
       </c>
     </row>
     <row r="438">
@@ -9330,10 +9336,10 @@
         <v>939</v>
       </c>
       <c r="C438" s="0" t="s">
-        <v>935</v>
+        <v>937</v>
       </c>
       <c r="D438" s="0">
-        <v>6555.64</v>
+        <v>15072</v>
       </c>
     </row>
     <row r="439">
@@ -9344,10 +9350,10 @@
         <v>941</v>
       </c>
       <c r="C439" s="0" t="s">
-        <v>935</v>
+        <v>937</v>
       </c>
       <c r="D439" s="0">
-        <v>8964.61</v>
+        <v>6555.64</v>
       </c>
     </row>
     <row r="440">
@@ -9358,10 +9364,10 @@
         <v>943</v>
       </c>
       <c r="C440" s="0" t="s">
-        <v>935</v>
+        <v>937</v>
       </c>
       <c r="D440" s="0">
-        <v>11735</v>
+        <v>8964.61</v>
       </c>
     </row>
     <row r="441">
@@ -9372,10 +9378,10 @@
         <v>945</v>
       </c>
       <c r="C441" s="0" t="s">
-        <v>69</v>
+        <v>937</v>
       </c>
       <c r="D441" s="0">
-        <v>3380</v>
+        <v>11735</v>
       </c>
     </row>
     <row r="442">
@@ -9386,10 +9392,10 @@
         <v>947</v>
       </c>
       <c r="C442" s="0" t="s">
-        <v>132</v>
+        <v>69</v>
       </c>
       <c r="D442" s="0">
-        <v>3822.39</v>
+        <v>3380</v>
       </c>
     </row>
     <row r="443">
@@ -9400,10 +9406,10 @@
         <v>949</v>
       </c>
       <c r="C443" s="0" t="s">
-        <v>89</v>
+        <v>132</v>
       </c>
       <c r="D443" s="0">
-        <v>4392.3</v>
+        <v>3822.39</v>
       </c>
     </row>
     <row r="444">
@@ -9414,24 +9420,24 @@
         <v>951</v>
       </c>
       <c r="C444" s="0" t="s">
-        <v>952</v>
+        <v>89</v>
       </c>
       <c r="D444" s="0">
-        <v>5254.41</v>
+        <v>4392.3</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="0" t="s">
+        <v>952</v>
+      </c>
+      <c r="B445" s="0" t="s">
         <v>953</v>
       </c>
-      <c r="B445" s="0" t="s">
+      <c r="C445" s="0" t="s">
         <v>954</v>
       </c>
-      <c r="C445" s="0" t="s">
-        <v>51</v>
-      </c>
       <c r="D445" s="0">
-        <v>1200</v>
+        <v>5254.41</v>
       </c>
     </row>
     <row r="446">
@@ -9445,7 +9451,7 @@
         <v>51</v>
       </c>
       <c r="D446" s="0">
-        <v>278</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="447">
@@ -9459,7 +9465,7 @@
         <v>51</v>
       </c>
       <c r="D447" s="0">
-        <v>562</v>
+        <v>278</v>
       </c>
     </row>
     <row r="448">
@@ -9470,10 +9476,10 @@
         <v>960</v>
       </c>
       <c r="C448" s="0" t="s">
-        <v>368</v>
+        <v>51</v>
       </c>
       <c r="D448" s="0">
-        <v>65142</v>
+        <v>562</v>
       </c>
     </row>
     <row r="449">
@@ -9487,7 +9493,7 @@
         <v>368</v>
       </c>
       <c r="D449" s="0">
-        <v>23483</v>
+        <v>65142.6</v>
       </c>
     </row>
     <row r="450">
@@ -9498,10 +9504,10 @@
         <v>964</v>
       </c>
       <c r="C450" s="0" t="s">
-        <v>29</v>
+        <v>368</v>
       </c>
       <c r="D450" s="0">
-        <v>5917.17</v>
+        <v>23482.7</v>
       </c>
     </row>
     <row r="451">
@@ -9512,10 +9518,10 @@
         <v>966</v>
       </c>
       <c r="C451" s="0" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="D451" s="0">
-        <v>10985</v>
+        <v>5917.17</v>
       </c>
     </row>
     <row r="452">
@@ -9529,7 +9535,7 @@
         <v>51</v>
       </c>
       <c r="D452" s="0">
-        <v>17425</v>
+        <v>10985</v>
       </c>
     </row>
     <row r="453">
@@ -9540,24 +9546,24 @@
         <v>970</v>
       </c>
       <c r="C453" s="0" t="s">
-        <v>971</v>
+        <v>51</v>
       </c>
       <c r="D453" s="0">
-        <v>1958</v>
+        <v>17425</v>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="0" t="s">
+        <v>971</v>
+      </c>
+      <c r="B454" s="0" t="s">
         <v>972</v>
       </c>
-      <c r="B454" s="0" t="s">
+      <c r="C454" s="0" t="s">
         <v>973</v>
       </c>
-      <c r="C454" s="0" t="s">
-        <v>89</v>
-      </c>
       <c r="D454" s="0">
-        <v>249562.5</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="455">
@@ -9568,10 +9574,10 @@
         <v>975</v>
       </c>
       <c r="C455" s="0" t="s">
-        <v>570</v>
+        <v>89</v>
       </c>
       <c r="D455" s="0">
-        <v>71176.4</v>
+        <v>249562.5</v>
       </c>
     </row>
     <row r="456">
@@ -9582,10 +9588,10 @@
         <v>977</v>
       </c>
       <c r="C456" s="0" t="s">
-        <v>132</v>
+        <v>570</v>
       </c>
       <c r="D456" s="0">
-        <v>82</v>
+        <v>71176.4</v>
       </c>
     </row>
     <row r="457">
@@ -9596,10 +9602,10 @@
         <v>979</v>
       </c>
       <c r="C457" s="0" t="s">
-        <v>69</v>
+        <v>132</v>
       </c>
       <c r="D457" s="0">
-        <v>950</v>
+        <v>82</v>
       </c>
     </row>
     <row r="458">
@@ -9610,10 +9616,10 @@
         <v>981</v>
       </c>
       <c r="C458" s="0" t="s">
-        <v>469</v>
+        <v>69</v>
       </c>
       <c r="D458" s="0">
-        <v>342641</v>
+        <v>950</v>
       </c>
     </row>
     <row r="459">
@@ -9624,10 +9630,10 @@
         <v>983</v>
       </c>
       <c r="C459" s="0" t="s">
-        <v>150</v>
+        <v>469</v>
       </c>
       <c r="D459" s="0">
-        <v>2200</v>
+        <v>342641</v>
       </c>
     </row>
     <row r="460">
@@ -9638,10 +9644,10 @@
         <v>985</v>
       </c>
       <c r="C460" s="0" t="s">
-        <v>478</v>
+        <v>150</v>
       </c>
       <c r="D460" s="0">
-        <v>41000</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="461">
@@ -9652,10 +9658,10 @@
         <v>987</v>
       </c>
       <c r="C461" s="0" t="s">
-        <v>69</v>
+        <v>478</v>
       </c>
       <c r="D461" s="0">
-        <v>9299</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="462">
@@ -9666,10 +9672,10 @@
         <v>989</v>
       </c>
       <c r="C462" s="0" t="s">
-        <v>904</v>
+        <v>69</v>
       </c>
       <c r="D462" s="0">
-        <v>595</v>
+        <v>9299</v>
       </c>
     </row>
     <row r="463">
@@ -9680,7 +9686,7 @@
         <v>991</v>
       </c>
       <c r="C463" s="0" t="s">
-        <v>904</v>
+        <v>906</v>
       </c>
       <c r="D463" s="0">
         <v>595</v>
@@ -9694,7 +9700,7 @@
         <v>993</v>
       </c>
       <c r="C464" s="0" t="s">
-        <v>904</v>
+        <v>906</v>
       </c>
       <c r="D464" s="0">
         <v>595</v>
@@ -9708,10 +9714,10 @@
         <v>995</v>
       </c>
       <c r="C465" s="0" t="s">
-        <v>22</v>
+        <v>906</v>
       </c>
       <c r="D465" s="0">
-        <v>563.36</v>
+        <v>595</v>
       </c>
     </row>
     <row r="466">
@@ -9722,10 +9728,10 @@
         <v>997</v>
       </c>
       <c r="C466" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D466" s="0">
-        <v>3520</v>
+        <v>563.36</v>
       </c>
     </row>
     <row r="467">
@@ -9739,7 +9745,7 @@
         <v>16</v>
       </c>
       <c r="D467" s="0">
-        <v>2600</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="468">
@@ -9750,10 +9756,10 @@
         <v>1001</v>
       </c>
       <c r="C468" s="0" t="s">
-        <v>276</v>
+        <v>16</v>
       </c>
       <c r="D468" s="0">
-        <v>3700</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="469">
@@ -9767,7 +9773,7 @@
         <v>276</v>
       </c>
       <c r="D469" s="0">
-        <v>2600</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="470">
@@ -9778,10 +9784,10 @@
         <v>1005</v>
       </c>
       <c r="C470" s="0" t="s">
-        <v>16</v>
+        <v>276</v>
       </c>
       <c r="D470" s="0">
-        <v>2235</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="471">
@@ -9795,35 +9801,35 @@
         <v>16</v>
       </c>
       <c r="D471" s="0">
-        <v>3850</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="0" t="s">
-        <v>389</v>
+        <v>1008</v>
       </c>
       <c r="B472" s="0" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="C472" s="0" t="s">
-        <v>1009</v>
+        <v>16</v>
       </c>
       <c r="D472" s="0">
-        <v>1</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="0" t="s">
+        <v>389</v>
+      </c>
+      <c r="B473" s="0" t="s">
         <v>1010</v>
       </c>
-      <c r="B473" s="0" t="s">
+      <c r="C473" s="0" t="s">
         <v>1011</v>
       </c>
-      <c r="C473" s="0" t="s">
-        <v>29</v>
-      </c>
       <c r="D473" s="0">
-        <v>13715</v>
+        <v>1</v>
       </c>
     </row>
     <row r="474">
@@ -9834,10 +9840,10 @@
         <v>1013</v>
       </c>
       <c r="C474" s="0" t="s">
-        <v>368</v>
+        <v>29</v>
       </c>
       <c r="D474" s="0">
-        <v>3859.93</v>
+        <v>13715</v>
       </c>
     </row>
     <row r="475">
@@ -9851,7 +9857,7 @@
         <v>368</v>
       </c>
       <c r="D475" s="0">
-        <v>11751.49</v>
+        <v>3859.93</v>
       </c>
     </row>
     <row r="476">
@@ -9862,10 +9868,10 @@
         <v>1017</v>
       </c>
       <c r="C476" s="0" t="s">
-        <v>331</v>
+        <v>368</v>
       </c>
       <c r="D476" s="0">
-        <v>6000</v>
+        <v>11751.49</v>
       </c>
     </row>
     <row r="477">
@@ -9879,7 +9885,7 @@
         <v>331</v>
       </c>
       <c r="D477" s="0">
-        <v>3000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="478">
@@ -9890,10 +9896,10 @@
         <v>1021</v>
       </c>
       <c r="C478" s="0" t="s">
-        <v>38</v>
+        <v>331</v>
       </c>
       <c r="D478" s="0">
-        <v>618</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="479">
@@ -9904,24 +9910,24 @@
         <v>1023</v>
       </c>
       <c r="C479" s="0" t="s">
-        <v>1024</v>
+        <v>38</v>
       </c>
       <c r="D479" s="0">
-        <v>24600</v>
+        <v>618</v>
       </c>
     </row>
     <row r="480">
       <c r="A480" s="0" t="s">
+        <v>1024</v>
+      </c>
+      <c r="B480" s="0" t="s">
         <v>1025</v>
       </c>
-      <c r="B480" s="0" t="s">
+      <c r="C480" s="0" t="s">
         <v>1026</v>
       </c>
-      <c r="C480" s="0" t="s">
-        <v>102</v>
-      </c>
       <c r="D480" s="0">
-        <v>0</v>
+        <v>24600</v>
       </c>
     </row>
     <row r="481">
@@ -9932,10 +9938,10 @@
         <v>1028</v>
       </c>
       <c r="C481" s="0" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="D481" s="0">
-        <v>32942.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="482">
@@ -9946,10 +9952,10 @@
         <v>1030</v>
       </c>
       <c r="C482" s="0" t="s">
-        <v>368</v>
+        <v>89</v>
       </c>
       <c r="D482" s="0">
-        <v>75529.41</v>
+        <v>32942.25</v>
       </c>
     </row>
     <row r="483">
@@ -9963,7 +9969,7 @@
         <v>368</v>
       </c>
       <c r="D483" s="0">
-        <v>41613</v>
+        <v>75529.71</v>
       </c>
     </row>
     <row r="484">
@@ -9977,7 +9983,7 @@
         <v>368</v>
       </c>
       <c r="D484" s="0">
-        <v>87056</v>
+        <v>41613.42</v>
       </c>
     </row>
     <row r="485">
@@ -9991,7 +9997,7 @@
         <v>368</v>
       </c>
       <c r="D485" s="0">
-        <v>49243.16</v>
+        <v>87056.42</v>
       </c>
     </row>
     <row r="486">
@@ -10002,10 +10008,10 @@
         <v>1038</v>
       </c>
       <c r="C486" s="0" t="s">
-        <v>22</v>
+        <v>368</v>
       </c>
       <c r="D486" s="0">
-        <v>1600</v>
+        <v>49243.16</v>
       </c>
     </row>
     <row r="487">
@@ -10016,10 +10022,10 @@
         <v>1040</v>
       </c>
       <c r="C487" s="0" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D487" s="0">
-        <v>3338.9</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="488">
@@ -10033,7 +10039,7 @@
         <v>29</v>
       </c>
       <c r="D488" s="0">
-        <v>3987</v>
+        <v>3338.9</v>
       </c>
     </row>
     <row r="489">
@@ -10047,7 +10053,7 @@
         <v>29</v>
       </c>
       <c r="D489" s="0">
-        <v>4010.17</v>
+        <v>3987</v>
       </c>
     </row>
     <row r="490">
@@ -10061,35 +10067,35 @@
         <v>29</v>
       </c>
       <c r="D490" s="0">
+        <v>4010.17</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="0" t="s">
+        <v>1047</v>
+      </c>
+      <c r="B491" s="0" t="s">
+        <v>1048</v>
+      </c>
+      <c r="C491" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D491" s="0">
         <v>3382.65</v>
       </c>
     </row>
-    <row r="491">
-      <c r="A491" s="2" t="s">
-        <v>1047</v>
-      </c>
-      <c r="B491" s="2" t="s">
-        <v>1048</v>
-      </c>
-      <c r="C491" s="2" t="s">
+    <row r="492">
+      <c r="A492" s="2" t="s">
+        <v>1049</v>
+      </c>
+      <c r="B492" s="2" t="s">
+        <v>1050</v>
+      </c>
+      <c r="C492" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D491" s="2">
+      <c r="D492" s="2">
         <v>0</v>
-      </c>
-    </row>
-    <row r="492">
-      <c r="A492" s="0" t="s">
-        <v>1049</v>
-      </c>
-      <c r="B492" s="0" t="s">
-        <v>1050</v>
-      </c>
-      <c r="C492" s="0" t="s">
-        <v>150</v>
-      </c>
-      <c r="D492" s="0">
-        <v>430</v>
       </c>
     </row>
     <row r="493">
@@ -10100,9 +10106,23 @@
         <v>1052</v>
       </c>
       <c r="C493" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="D493" s="0">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="0" t="s">
+        <v>1053</v>
+      </c>
+      <c r="B494" s="0" t="s">
+        <v>1054</v>
+      </c>
+      <c r="C494" s="0" t="s">
         <v>132</v>
       </c>
-      <c r="D493" s="0">
+      <c r="D494" s="0">
         <v>435</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: stock y precios actualizados sáb. 27/06/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="1055">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1057" uniqueCount="1057">
   <si>
     <t>Código</t>
   </si>
@@ -1818,6 +1818,12 @@
   </si>
   <si>
     <t>KETOROLAC AMP 30 MG X 2 ML / LAVIMAR - 000024327</t>
+  </si>
+  <si>
+    <t>000022228</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KETOROLAC LARJAN 30MG INY. AMP.  X 2 ML  X 1  - 000022228</t>
   </si>
   <si>
     <t>000023684</t>
@@ -3235,7 +3241,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A3:D494"/>
+  <dimension ref="A3:D495"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="3">
@@ -3459,7 +3465,7 @@
         <v>44</v>
       </c>
       <c r="D18" s="0">
-        <v>2547.8</v>
+        <v>2675.19</v>
       </c>
     </row>
     <row r="19">
@@ -3487,7 +3493,7 @@
         <v>44</v>
       </c>
       <c r="D20" s="0">
-        <v>21079.41</v>
+        <v>22133.38</v>
       </c>
     </row>
     <row r="21">
@@ -3977,7 +3983,7 @@
         <v>132</v>
       </c>
       <c r="D55" s="0">
-        <v>393</v>
+        <v>473.6</v>
       </c>
     </row>
     <row r="56">
@@ -3991,7 +3997,7 @@
         <v>132</v>
       </c>
       <c r="D56" s="0">
-        <v>482</v>
+        <v>584.3</v>
       </c>
     </row>
     <row r="57">
@@ -4173,7 +4179,7 @@
         <v>132</v>
       </c>
       <c r="D69" s="0">
-        <v>533</v>
+        <v>537</v>
       </c>
     </row>
     <row r="70">
@@ -4187,7 +4193,7 @@
         <v>132</v>
       </c>
       <c r="D70" s="0">
-        <v>620</v>
+        <v>705</v>
       </c>
     </row>
     <row r="71">
@@ -4453,7 +4459,7 @@
         <v>132</v>
       </c>
       <c r="D89" s="0">
-        <v>527.38</v>
+        <v>636.16</v>
       </c>
     </row>
     <row r="90">
@@ -4467,7 +4473,7 @@
         <v>132</v>
       </c>
       <c r="D90" s="0">
-        <v>451.64</v>
+        <v>543.06</v>
       </c>
     </row>
     <row r="91">
@@ -4705,7 +4711,7 @@
         <v>44</v>
       </c>
       <c r="D107" s="0">
-        <v>3816.26</v>
+        <v>4007.07</v>
       </c>
     </row>
     <row r="108">
@@ -4733,7 +4739,7 @@
         <v>132</v>
       </c>
       <c r="D109" s="0">
-        <v>975</v>
+        <v>980</v>
       </c>
     </row>
     <row r="110">
@@ -4985,7 +4991,7 @@
         <v>132</v>
       </c>
       <c r="D127" s="0">
-        <v>2713</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="128">
@@ -4999,7 +5005,7 @@
         <v>132</v>
       </c>
       <c r="D128" s="0">
-        <v>3200</v>
+        <v>6375</v>
       </c>
     </row>
     <row r="129">
@@ -5643,7 +5649,7 @@
         <v>132</v>
       </c>
       <c r="D174" s="0">
-        <v>2141.42</v>
+        <v>2762.43</v>
       </c>
     </row>
     <row r="175">
@@ -5657,7 +5663,7 @@
         <v>132</v>
       </c>
       <c r="D175" s="0">
-        <v>3371.4</v>
+        <v>3573.45</v>
       </c>
     </row>
     <row r="176">
@@ -5979,7 +5985,7 @@
         <v>44</v>
       </c>
       <c r="D198" s="0">
-        <v>4129.73</v>
+        <v>4336.22</v>
       </c>
     </row>
     <row r="199">
@@ -6203,7 +6209,7 @@
         <v>132</v>
       </c>
       <c r="D214" s="0">
-        <v>340</v>
+        <v>492.2</v>
       </c>
     </row>
     <row r="215">
@@ -6245,7 +6251,7 @@
         <v>51</v>
       </c>
       <c r="D217" s="0">
-        <v>4150</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="218">
@@ -6259,7 +6265,7 @@
         <v>51</v>
       </c>
       <c r="D218" s="0">
-        <v>4150</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="219">
@@ -6273,7 +6279,7 @@
         <v>51</v>
       </c>
       <c r="D219" s="0">
-        <v>4150</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="220">
@@ -6287,7 +6293,7 @@
         <v>489</v>
       </c>
       <c r="D220" s="0">
-        <v>250</v>
+        <v>265</v>
       </c>
     </row>
     <row r="221">
@@ -6301,7 +6307,7 @@
         <v>489</v>
       </c>
       <c r="D221" s="0">
-        <v>250</v>
+        <v>265</v>
       </c>
     </row>
     <row r="222">
@@ -6315,7 +6321,7 @@
         <v>489</v>
       </c>
       <c r="D222" s="0">
-        <v>250</v>
+        <v>265</v>
       </c>
     </row>
     <row r="223">
@@ -6329,7 +6335,7 @@
         <v>489</v>
       </c>
       <c r="D223" s="0">
-        <v>250</v>
+        <v>265</v>
       </c>
     </row>
     <row r="224">
@@ -6343,7 +6349,7 @@
         <v>489</v>
       </c>
       <c r="D224" s="0">
-        <v>250</v>
+        <v>265</v>
       </c>
     </row>
     <row r="225">
@@ -6357,7 +6363,7 @@
         <v>489</v>
       </c>
       <c r="D225" s="0">
-        <v>250</v>
+        <v>265</v>
       </c>
     </row>
     <row r="226">
@@ -6371,7 +6377,7 @@
         <v>502</v>
       </c>
       <c r="D226" s="0">
-        <v>5550</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="227">
@@ -6385,7 +6391,7 @@
         <v>505</v>
       </c>
       <c r="D227" s="0">
-        <v>5550</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="228">
@@ -6399,7 +6405,7 @@
         <v>502</v>
       </c>
       <c r="D228" s="0">
-        <v>5550</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="229">
@@ -6749,7 +6755,7 @@
         <v>132</v>
       </c>
       <c r="D253" s="0">
-        <v>415.15</v>
+        <v>430</v>
       </c>
     </row>
     <row r="254">
@@ -6763,7 +6769,7 @@
         <v>132</v>
       </c>
       <c r="D254" s="0">
-        <v>318.63</v>
+        <v>354.54</v>
       </c>
     </row>
     <row r="255">
@@ -7043,7 +7049,7 @@
         <v>352</v>
       </c>
       <c r="D274" s="0">
-        <v>400</v>
+        <v>450</v>
       </c>
     </row>
     <row r="275">
@@ -7054,10 +7060,10 @@
         <v>603</v>
       </c>
       <c r="C275" s="0" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="D275" s="0">
-        <v>510</v>
+        <v>450</v>
       </c>
     </row>
     <row r="276">
@@ -7071,7 +7077,7 @@
         <v>16</v>
       </c>
       <c r="D276" s="0">
-        <v>1650</v>
+        <v>450</v>
       </c>
     </row>
     <row r="277">
@@ -7085,7 +7091,7 @@
         <v>16</v>
       </c>
       <c r="D277" s="0">
-        <v>2100</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="278">
@@ -7099,7 +7105,7 @@
         <v>16</v>
       </c>
       <c r="D278" s="0">
-        <v>1980</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="279">
@@ -7113,7 +7119,7 @@
         <v>16</v>
       </c>
       <c r="D279" s="0">
-        <v>2160</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="280">
@@ -7127,7 +7133,7 @@
         <v>16</v>
       </c>
       <c r="D280" s="0">
-        <v>1100</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="281">
@@ -7141,7 +7147,7 @@
         <v>16</v>
       </c>
       <c r="D281" s="0">
-        <v>2600</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="282">
@@ -7155,7 +7161,7 @@
         <v>16</v>
       </c>
       <c r="D282" s="0">
-        <v>2000</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="283">
@@ -7169,7 +7175,7 @@
         <v>16</v>
       </c>
       <c r="D283" s="0">
-        <v>6700</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="284">
@@ -7183,7 +7189,7 @@
         <v>16</v>
       </c>
       <c r="D284" s="0">
-        <v>1650</v>
+        <v>6700</v>
       </c>
     </row>
     <row r="285">
@@ -7197,7 +7203,7 @@
         <v>16</v>
       </c>
       <c r="D285" s="0">
-        <v>1035</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="286">
@@ -7211,7 +7217,7 @@
         <v>16</v>
       </c>
       <c r="D286" s="0">
-        <v>2600</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="287">
@@ -7225,7 +7231,7 @@
         <v>16</v>
       </c>
       <c r="D287" s="0">
-        <v>2400</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="288">
@@ -7236,10 +7242,10 @@
         <v>629</v>
       </c>
       <c r="C288" s="0" t="s">
-        <v>132</v>
+        <v>16</v>
       </c>
       <c r="D288" s="0">
-        <v>4045</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="289">
@@ -7253,7 +7259,7 @@
         <v>132</v>
       </c>
       <c r="D289" s="0">
-        <v>2081</v>
+        <v>4497.2</v>
       </c>
     </row>
     <row r="290">
@@ -7267,7 +7273,7 @@
         <v>132</v>
       </c>
       <c r="D290" s="0">
-        <v>998</v>
+        <v>2328</v>
       </c>
     </row>
     <row r="291">
@@ -7278,10 +7284,10 @@
         <v>635</v>
       </c>
       <c r="C291" s="0" t="s">
-        <v>29</v>
+        <v>132</v>
       </c>
       <c r="D291" s="0">
-        <v>7234.96</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="292">
@@ -7292,10 +7298,10 @@
         <v>637</v>
       </c>
       <c r="C292" s="0" t="s">
-        <v>115</v>
+        <v>29</v>
       </c>
       <c r="D292" s="0">
-        <v>1790</v>
+        <v>7234.96</v>
       </c>
     </row>
     <row r="293">
@@ -7309,7 +7315,7 @@
         <v>115</v>
       </c>
       <c r="D293" s="0">
-        <v>2859.96</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="294">
@@ -7323,7 +7329,7 @@
         <v>115</v>
       </c>
       <c r="D294" s="0">
-        <v>4800</v>
+        <v>2859.96</v>
       </c>
     </row>
     <row r="295">
@@ -7334,24 +7340,24 @@
         <v>643</v>
       </c>
       <c r="C295" s="0" t="s">
-        <v>644</v>
+        <v>115</v>
       </c>
       <c r="D295" s="0">
-        <v>0</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="0" t="s">
+        <v>644</v>
+      </c>
+      <c r="B296" s="0" t="s">
         <v>645</v>
       </c>
-      <c r="B296" s="0" t="s">
+      <c r="C296" s="0" t="s">
         <v>646</v>
       </c>
-      <c r="C296" s="0" t="s">
-        <v>29</v>
-      </c>
       <c r="D296" s="0">
-        <v>494</v>
+        <v>0</v>
       </c>
     </row>
     <row r="297">
@@ -7365,7 +7371,7 @@
         <v>29</v>
       </c>
       <c r="D297" s="0">
-        <v>665.3</v>
+        <v>494</v>
       </c>
     </row>
     <row r="298">
@@ -7376,10 +7382,10 @@
         <v>650</v>
       </c>
       <c r="C298" s="0" t="s">
-        <v>89</v>
+        <v>29</v>
       </c>
       <c r="D298" s="0">
-        <v>32609.5</v>
+        <v>665.3</v>
       </c>
     </row>
     <row r="299">
@@ -7393,7 +7399,7 @@
         <v>89</v>
       </c>
       <c r="D299" s="0">
-        <v>4525.4</v>
+        <v>32609.5</v>
       </c>
     </row>
     <row r="300">
@@ -7404,10 +7410,10 @@
         <v>654</v>
       </c>
       <c r="C300" s="0" t="s">
-        <v>143</v>
+        <v>89</v>
       </c>
       <c r="D300" s="0">
-        <v>896</v>
+        <v>4525.4</v>
       </c>
     </row>
     <row r="301">
@@ -7418,10 +7424,10 @@
         <v>656</v>
       </c>
       <c r="C301" s="0" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="D301" s="0">
-        <v>1280</v>
+        <v>896</v>
       </c>
     </row>
     <row r="302">
@@ -7432,10 +7438,10 @@
         <v>658</v>
       </c>
       <c r="C302" s="0" t="s">
-        <v>89</v>
+        <v>132</v>
       </c>
       <c r="D302" s="0">
-        <v>306130</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="303">
@@ -7446,10 +7452,10 @@
         <v>660</v>
       </c>
       <c r="C303" s="0" t="s">
-        <v>197</v>
+        <v>89</v>
       </c>
       <c r="D303" s="0">
-        <v>17440</v>
+        <v>306130</v>
       </c>
     </row>
     <row r="304">
@@ -7463,7 +7469,7 @@
         <v>197</v>
       </c>
       <c r="D304" s="0">
-        <v>4390</v>
+        <v>17440</v>
       </c>
     </row>
     <row r="305">
@@ -7488,10 +7494,10 @@
         <v>666</v>
       </c>
       <c r="C306" s="0" t="s">
-        <v>276</v>
+        <v>197</v>
       </c>
       <c r="D306" s="0">
-        <v>2250</v>
+        <v>4390</v>
       </c>
     </row>
     <row r="307">
@@ -7502,10 +7508,10 @@
         <v>668</v>
       </c>
       <c r="C307" s="0" t="s">
-        <v>197</v>
+        <v>276</v>
       </c>
       <c r="D307" s="0">
-        <v>3355</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="308">
@@ -7516,10 +7522,10 @@
         <v>670</v>
       </c>
       <c r="C308" s="0" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="D308" s="0">
-        <v>7500</v>
+        <v>3355</v>
       </c>
     </row>
     <row r="309">
@@ -7530,10 +7536,10 @@
         <v>672</v>
       </c>
       <c r="C309" s="0" t="s">
-        <v>89</v>
+        <v>202</v>
       </c>
       <c r="D309" s="0">
-        <v>23958</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="310">
@@ -7547,7 +7553,7 @@
         <v>89</v>
       </c>
       <c r="D310" s="0">
-        <v>239580</v>
+        <v>23958</v>
       </c>
     </row>
     <row r="311">
@@ -7558,10 +7564,10 @@
         <v>676</v>
       </c>
       <c r="C311" s="0" t="s">
-        <v>51</v>
+        <v>89</v>
       </c>
       <c r="D311" s="0">
-        <v>130</v>
+        <v>239580</v>
       </c>
     </row>
     <row r="312">
@@ -7572,10 +7578,10 @@
         <v>678</v>
       </c>
       <c r="C312" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="D312" s="0">
-        <v>285.6</v>
+        <v>130</v>
       </c>
     </row>
     <row r="313">
@@ -7589,7 +7595,7 @@
         <v>22</v>
       </c>
       <c r="D313" s="0">
-        <v>338</v>
+        <v>285.6</v>
       </c>
     </row>
     <row r="314">
@@ -7600,21 +7606,21 @@
         <v>682</v>
       </c>
       <c r="C314" s="0" t="s">
-        <v>683</v>
+        <v>22</v>
       </c>
       <c r="D314" s="0">
-        <v>770</v>
+        <v>338</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="0" t="s">
+        <v>683</v>
+      </c>
+      <c r="B315" s="0" t="s">
         <v>684</v>
       </c>
-      <c r="B315" s="0" t="s">
+      <c r="C315" s="0" t="s">
         <v>685</v>
-      </c>
-      <c r="C315" s="0" t="s">
-        <v>686</v>
       </c>
       <c r="D315" s="0">
         <v>770</v>
@@ -7622,16 +7628,16 @@
     </row>
     <row r="316">
       <c r="A316" s="0" t="s">
+        <v>686</v>
+      </c>
+      <c r="B316" s="0" t="s">
         <v>687</v>
       </c>
-      <c r="B316" s="0" t="s">
+      <c r="C316" s="0" t="s">
         <v>688</v>
       </c>
-      <c r="C316" s="0" t="s">
-        <v>16</v>
-      </c>
       <c r="D316" s="0">
-        <v>973.5</v>
+        <v>770</v>
       </c>
     </row>
     <row r="317">
@@ -7642,10 +7648,10 @@
         <v>690</v>
       </c>
       <c r="C317" s="0" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D317" s="0">
-        <v>507.08</v>
+        <v>973.5</v>
       </c>
     </row>
     <row r="318">
@@ -7656,10 +7662,10 @@
         <v>692</v>
       </c>
       <c r="C318" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D318" s="0">
-        <v>450</v>
+        <v>507.08</v>
       </c>
     </row>
     <row r="319">
@@ -7670,10 +7676,10 @@
         <v>694</v>
       </c>
       <c r="C319" s="0" t="s">
-        <v>143</v>
+        <v>16</v>
       </c>
       <c r="D319" s="0">
-        <v>760</v>
+        <v>450</v>
       </c>
     </row>
     <row r="320">
@@ -7684,10 +7690,10 @@
         <v>696</v>
       </c>
       <c r="C320" s="0" t="s">
-        <v>276</v>
+        <v>143</v>
       </c>
       <c r="D320" s="0">
-        <v>5900</v>
+        <v>760</v>
       </c>
     </row>
     <row r="321">
@@ -7701,7 +7707,7 @@
         <v>276</v>
       </c>
       <c r="D321" s="0">
-        <v>2900</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="322">
@@ -7712,10 +7718,10 @@
         <v>700</v>
       </c>
       <c r="C322" s="0" t="s">
-        <v>132</v>
+        <v>276</v>
       </c>
       <c r="D322" s="0">
-        <v>797.4</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="323">
@@ -7729,7 +7735,7 @@
         <v>132</v>
       </c>
       <c r="D323" s="0">
-        <v>519</v>
+        <v>886.2</v>
       </c>
     </row>
     <row r="324">
@@ -7743,7 +7749,7 @@
         <v>132</v>
       </c>
       <c r="D324" s="0">
-        <v>62</v>
+        <v>589.9</v>
       </c>
     </row>
     <row r="325">
@@ -7754,10 +7760,10 @@
         <v>706</v>
       </c>
       <c r="C325" s="0" t="s">
-        <v>89</v>
+        <v>132</v>
       </c>
       <c r="D325" s="0">
-        <v>11313.5</v>
+        <v>65</v>
       </c>
     </row>
     <row r="326">
@@ -7768,10 +7774,10 @@
         <v>708</v>
       </c>
       <c r="C326" s="0" t="s">
-        <v>35</v>
+        <v>89</v>
       </c>
       <c r="D326" s="0">
-        <v>418</v>
+        <v>11313.5</v>
       </c>
     </row>
     <row r="327">
@@ -7782,7 +7788,7 @@
         <v>710</v>
       </c>
       <c r="C327" s="0" t="s">
-        <v>352</v>
+        <v>35</v>
       </c>
       <c r="D327" s="0">
         <v>418</v>
@@ -7796,10 +7802,10 @@
         <v>712</v>
       </c>
       <c r="C328" s="0" t="s">
-        <v>22</v>
+        <v>352</v>
       </c>
       <c r="D328" s="0">
-        <v>377</v>
+        <v>418</v>
       </c>
     </row>
     <row r="329">
@@ -7810,10 +7816,10 @@
         <v>714</v>
       </c>
       <c r="C329" s="0" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="D329" s="0">
-        <v>3860.67</v>
+        <v>377</v>
       </c>
     </row>
     <row r="330">
@@ -7824,10 +7830,10 @@
         <v>716</v>
       </c>
       <c r="C330" s="0" t="s">
-        <v>69</v>
+        <v>44</v>
       </c>
       <c r="D330" s="0">
-        <v>898</v>
+        <v>4053.7</v>
       </c>
     </row>
     <row r="331">
@@ -7838,10 +7844,10 @@
         <v>718</v>
       </c>
       <c r="C331" s="0" t="s">
-        <v>115</v>
+        <v>69</v>
       </c>
       <c r="D331" s="0">
-        <v>4767</v>
+        <v>898</v>
       </c>
     </row>
     <row r="332">
@@ -7852,10 +7858,10 @@
         <v>720</v>
       </c>
       <c r="C332" s="0" t="s">
-        <v>35</v>
+        <v>115</v>
       </c>
       <c r="D332" s="0">
-        <v>650</v>
+        <v>4767</v>
       </c>
     </row>
     <row r="333">
@@ -7866,7 +7872,7 @@
         <v>722</v>
       </c>
       <c r="C333" s="0" t="s">
-        <v>69</v>
+        <v>35</v>
       </c>
       <c r="D333" s="0">
         <v>650</v>
@@ -7880,10 +7886,10 @@
         <v>724</v>
       </c>
       <c r="C334" s="0" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="D334" s="0">
-        <v>2178</v>
+        <v>650</v>
       </c>
     </row>
     <row r="335">
@@ -7894,10 +7900,10 @@
         <v>726</v>
       </c>
       <c r="C335" s="0" t="s">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="D335" s="0">
-        <v>7986</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="336">
@@ -7908,24 +7914,24 @@
         <v>728</v>
       </c>
       <c r="C336" s="0" t="s">
-        <v>729</v>
+        <v>89</v>
       </c>
       <c r="D336" s="0">
-        <v>1800</v>
+        <v>7986</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="0" t="s">
+        <v>729</v>
+      </c>
+      <c r="B337" s="0" t="s">
         <v>730</v>
       </c>
-      <c r="B337" s="0" t="s">
+      <c r="C337" s="0" t="s">
         <v>731</v>
       </c>
-      <c r="C337" s="0" t="s">
-        <v>143</v>
-      </c>
       <c r="D337" s="0">
-        <v>900</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="338">
@@ -7936,10 +7942,10 @@
         <v>733</v>
       </c>
       <c r="C338" s="0" t="s">
-        <v>22</v>
+        <v>143</v>
       </c>
       <c r="D338" s="0">
-        <v>1722</v>
+        <v>900</v>
       </c>
     </row>
     <row r="339">
@@ -7950,10 +7956,10 @@
         <v>735</v>
       </c>
       <c r="C339" s="0" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="D339" s="0">
-        <v>456</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="340">
@@ -7967,7 +7973,7 @@
         <v>35</v>
       </c>
       <c r="D340" s="0">
-        <v>45600</v>
+        <v>456</v>
       </c>
     </row>
     <row r="341">
@@ -7978,10 +7984,10 @@
         <v>739</v>
       </c>
       <c r="C341" s="0" t="s">
-        <v>143</v>
+        <v>35</v>
       </c>
       <c r="D341" s="0">
-        <v>750</v>
+        <v>45600</v>
       </c>
     </row>
     <row r="342">
@@ -7995,7 +8001,7 @@
         <v>143</v>
       </c>
       <c r="D342" s="0">
-        <v>1212</v>
+        <v>750</v>
       </c>
     </row>
     <row r="343">
@@ -8009,7 +8015,7 @@
         <v>143</v>
       </c>
       <c r="D343" s="0">
-        <v>1300</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="344">
@@ -8023,7 +8029,7 @@
         <v>143</v>
       </c>
       <c r="D344" s="0">
-        <v>1500</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="345">
@@ -8037,7 +8043,7 @@
         <v>143</v>
       </c>
       <c r="D345" s="0">
-        <v>1400</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="346">
@@ -8048,10 +8054,10 @@
         <v>749</v>
       </c>
       <c r="C346" s="0" t="s">
-        <v>252</v>
+        <v>143</v>
       </c>
       <c r="D346" s="0">
-        <v>11959</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="347">
@@ -8062,10 +8068,10 @@
         <v>751</v>
       </c>
       <c r="C347" s="0" t="s">
-        <v>132</v>
+        <v>252</v>
       </c>
       <c r="D347" s="0">
-        <v>300</v>
+        <v>11959</v>
       </c>
     </row>
     <row r="348">
@@ -8076,10 +8082,10 @@
         <v>753</v>
       </c>
       <c r="C348" s="0" t="s">
-        <v>276</v>
+        <v>132</v>
       </c>
       <c r="D348" s="0">
-        <v>1450</v>
+        <v>345</v>
       </c>
     </row>
     <row r="349">
@@ -8090,10 +8096,10 @@
         <v>755</v>
       </c>
       <c r="C349" s="0" t="s">
-        <v>89</v>
+        <v>276</v>
       </c>
       <c r="D349" s="0">
-        <v>7320.5</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="350">
@@ -8104,10 +8110,10 @@
         <v>757</v>
       </c>
       <c r="C350" s="0" t="s">
-        <v>16</v>
+        <v>89</v>
       </c>
       <c r="D350" s="0">
-        <v>900</v>
+        <v>7320.5</v>
       </c>
     </row>
     <row r="351">
@@ -8118,10 +8124,10 @@
         <v>759</v>
       </c>
       <c r="C351" s="0" t="s">
-        <v>276</v>
+        <v>16</v>
       </c>
       <c r="D351" s="0">
-        <v>520</v>
+        <v>900</v>
       </c>
     </row>
     <row r="352">
@@ -8132,10 +8138,10 @@
         <v>761</v>
       </c>
       <c r="C352" s="0" t="s">
-        <v>469</v>
+        <v>276</v>
       </c>
       <c r="D352" s="0">
-        <v>64925</v>
+        <v>520</v>
       </c>
     </row>
     <row r="353">
@@ -8146,10 +8152,10 @@
         <v>763</v>
       </c>
       <c r="C353" s="0" t="s">
-        <v>16</v>
+        <v>469</v>
       </c>
       <c r="D353" s="0">
-        <v>1100</v>
+        <v>64925</v>
       </c>
     </row>
     <row r="354">
@@ -8160,10 +8166,10 @@
         <v>765</v>
       </c>
       <c r="C354" s="0" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D354" s="0">
-        <v>1623</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="355">
@@ -8174,10 +8180,10 @@
         <v>767</v>
       </c>
       <c r="C355" s="0" t="s">
-        <v>132</v>
+        <v>22</v>
       </c>
       <c r="D355" s="0">
-        <v>1116.03</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="356">
@@ -8191,7 +8197,7 @@
         <v>132</v>
       </c>
       <c r="D356" s="0">
-        <v>4028.88</v>
+        <v>1182.75</v>
       </c>
     </row>
     <row r="357">
@@ -8202,10 +8208,10 @@
         <v>771</v>
       </c>
       <c r="C357" s="0" t="s">
-        <v>29</v>
+        <v>132</v>
       </c>
       <c r="D357" s="0">
-        <v>1650</v>
+        <v>4440.9</v>
       </c>
     </row>
     <row r="358">
@@ -8219,7 +8225,7 @@
         <v>29</v>
       </c>
       <c r="D358" s="0">
-        <v>1908.8</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="359">
@@ -8230,10 +8236,10 @@
         <v>775</v>
       </c>
       <c r="C359" s="0" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="D359" s="0">
-        <v>450</v>
+        <v>1908.8</v>
       </c>
     </row>
     <row r="360">
@@ -8247,7 +8253,7 @@
         <v>16</v>
       </c>
       <c r="D360" s="0">
-        <v>825</v>
+        <v>450</v>
       </c>
     </row>
     <row r="361">
@@ -8272,10 +8278,10 @@
         <v>781</v>
       </c>
       <c r="C362" s="0" t="s">
-        <v>371</v>
+        <v>16</v>
       </c>
       <c r="D362" s="0">
-        <v>134775.6</v>
+        <v>825</v>
       </c>
     </row>
     <row r="363">
@@ -8289,7 +8295,7 @@
         <v>371</v>
       </c>
       <c r="D363" s="0">
-        <v>175991.55</v>
+        <v>134775.6</v>
       </c>
     </row>
     <row r="364">
@@ -8300,10 +8306,10 @@
         <v>785</v>
       </c>
       <c r="C364" s="0" t="s">
-        <v>69</v>
+        <v>371</v>
       </c>
       <c r="D364" s="0">
-        <v>3263</v>
+        <v>175991.55</v>
       </c>
     </row>
     <row r="365">
@@ -8317,7 +8323,7 @@
         <v>69</v>
       </c>
       <c r="D365" s="0">
-        <v>18027</v>
+        <v>3263</v>
       </c>
     </row>
     <row r="366">
@@ -8328,10 +8334,10 @@
         <v>789</v>
       </c>
       <c r="C366" s="0" t="s">
-        <v>276</v>
+        <v>69</v>
       </c>
       <c r="D366" s="0">
-        <v>515</v>
+        <v>18027</v>
       </c>
     </row>
     <row r="367">
@@ -8342,38 +8348,38 @@
         <v>791</v>
       </c>
       <c r="C367" s="0" t="s">
-        <v>38</v>
+        <v>276</v>
       </c>
       <c r="D367" s="0">
         <v>515</v>
       </c>
     </row>
     <row r="368">
-      <c r="A368" s="2" t="s">
+      <c r="A368" s="0" t="s">
         <v>792</v>
       </c>
-      <c r="B368" s="2" t="s">
+      <c r="B368" s="0" t="s">
         <v>793</v>
       </c>
-      <c r="C368" s="2" t="s">
+      <c r="C368" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="D368" s="0">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="2" t="s">
+        <v>794</v>
+      </c>
+      <c r="B369" s="2" t="s">
+        <v>795</v>
+      </c>
+      <c r="C369" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D368" s="2">
+      <c r="D369" s="2">
         <v>10154</v>
-      </c>
-    </row>
-    <row r="369">
-      <c r="A369" s="0" t="s">
-        <v>794</v>
-      </c>
-      <c r="B369" s="0" t="s">
-        <v>795</v>
-      </c>
-      <c r="C369" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="D369" s="0">
-        <v>9500</v>
       </c>
     </row>
     <row r="370">
@@ -8384,10 +8390,10 @@
         <v>797</v>
       </c>
       <c r="C370" s="0" t="s">
-        <v>469</v>
+        <v>51</v>
       </c>
       <c r="D370" s="0">
-        <v>207558.08</v>
+        <v>9500</v>
       </c>
     </row>
     <row r="371">
@@ -8401,7 +8407,7 @@
         <v>469</v>
       </c>
       <c r="D371" s="0">
-        <v>249069.69</v>
+        <v>207558.08</v>
       </c>
     </row>
     <row r="372">
@@ -8412,10 +8418,10 @@
         <v>801</v>
       </c>
       <c r="C372" s="0" t="s">
-        <v>69</v>
+        <v>469</v>
       </c>
       <c r="D372" s="0">
-        <v>10021.22</v>
+        <v>249069.69</v>
       </c>
     </row>
     <row r="373">
@@ -8429,7 +8435,7 @@
         <v>69</v>
       </c>
       <c r="D373" s="0">
-        <v>17710</v>
+        <v>10021.22</v>
       </c>
     </row>
     <row r="374">
@@ -8440,24 +8446,24 @@
         <v>805</v>
       </c>
       <c r="C374" s="0" t="s">
-        <v>806</v>
+        <v>69</v>
       </c>
       <c r="D374" s="0">
-        <v>1080</v>
+        <v>17710</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="0" t="s">
+        <v>806</v>
+      </c>
+      <c r="B375" s="0" t="s">
         <v>807</v>
       </c>
-      <c r="B375" s="0" t="s">
+      <c r="C375" s="0" t="s">
         <v>808</v>
       </c>
-      <c r="C375" s="0" t="s">
-        <v>19</v>
-      </c>
       <c r="D375" s="0">
-        <v>691.03</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="376">
@@ -8468,24 +8474,24 @@
         <v>810</v>
       </c>
       <c r="C376" s="0" t="s">
-        <v>811</v>
+        <v>19</v>
       </c>
       <c r="D376" s="0">
-        <v>520</v>
+        <v>691.03</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="0" t="s">
+        <v>811</v>
+      </c>
+      <c r="B377" s="0" t="s">
         <v>812</v>
       </c>
-      <c r="B377" s="0" t="s">
+      <c r="C377" s="0" t="s">
         <v>813</v>
       </c>
-      <c r="C377" s="0" t="s">
-        <v>811</v>
-      </c>
       <c r="D377" s="0">
-        <v>300</v>
+        <v>520</v>
       </c>
     </row>
     <row r="378">
@@ -8496,10 +8502,10 @@
         <v>815</v>
       </c>
       <c r="C378" s="0" t="s">
-        <v>16</v>
+        <v>813</v>
       </c>
       <c r="D378" s="0">
-        <v>2200</v>
+        <v>300</v>
       </c>
     </row>
     <row r="379">
@@ -8513,7 +8519,7 @@
         <v>16</v>
       </c>
       <c r="D379" s="0">
-        <v>2800</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="380">
@@ -8524,10 +8530,10 @@
         <v>819</v>
       </c>
       <c r="C380" s="0" t="s">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="D380" s="0">
-        <v>4791.6</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="381">
@@ -8538,10 +8544,10 @@
         <v>821</v>
       </c>
       <c r="C381" s="0" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="D381" s="0">
-        <v>2699.64</v>
+        <v>4791.6</v>
       </c>
     </row>
     <row r="382">
@@ -8552,10 +8558,10 @@
         <v>823</v>
       </c>
       <c r="C382" s="0" t="s">
-        <v>35</v>
+        <v>69</v>
       </c>
       <c r="D382" s="0">
-        <v>3800</v>
+        <v>2699.64</v>
       </c>
     </row>
     <row r="383">
@@ -8566,10 +8572,10 @@
         <v>825</v>
       </c>
       <c r="C383" s="0" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D383" s="0">
-        <v>4000</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="384">
@@ -8580,24 +8586,24 @@
         <v>827</v>
       </c>
       <c r="C384" s="0" t="s">
-        <v>828</v>
+        <v>16</v>
       </c>
       <c r="D384" s="0">
-        <v>3800</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="0" t="s">
+        <v>828</v>
+      </c>
+      <c r="B385" s="0" t="s">
         <v>829</v>
       </c>
-      <c r="B385" s="0" t="s">
+      <c r="C385" s="0" t="s">
         <v>830</v>
       </c>
-      <c r="C385" s="0" t="s">
-        <v>22</v>
-      </c>
       <c r="D385" s="0">
-        <v>353</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="386">
@@ -8608,10 +8614,10 @@
         <v>832</v>
       </c>
       <c r="C386" s="0" t="s">
-        <v>355</v>
+        <v>22</v>
       </c>
       <c r="D386" s="0">
-        <v>1800</v>
+        <v>353</v>
       </c>
     </row>
     <row r="387">
@@ -8622,10 +8628,10 @@
         <v>834</v>
       </c>
       <c r="C387" s="0" t="s">
-        <v>16</v>
+        <v>355</v>
       </c>
       <c r="D387" s="0">
-        <v>2948</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="388">
@@ -8636,10 +8642,10 @@
         <v>836</v>
       </c>
       <c r="C388" s="0" t="s">
-        <v>202</v>
+        <v>16</v>
       </c>
       <c r="D388" s="0">
-        <v>65537</v>
+        <v>2948</v>
       </c>
     </row>
     <row r="389">
@@ -8650,10 +8656,10 @@
         <v>838</v>
       </c>
       <c r="C389" s="0" t="s">
-        <v>132</v>
+        <v>202</v>
       </c>
       <c r="D389" s="0">
-        <v>3820.86</v>
+        <v>65537</v>
       </c>
     </row>
     <row r="390">
@@ -8667,7 +8673,7 @@
         <v>132</v>
       </c>
       <c r="D390" s="0">
-        <v>3962</v>
+        <v>4049.6</v>
       </c>
     </row>
     <row r="391">
@@ -8681,7 +8687,7 @@
         <v>132</v>
       </c>
       <c r="D391" s="0">
-        <v>5802.4</v>
+        <v>4199.2</v>
       </c>
     </row>
     <row r="392">
@@ -8692,10 +8698,10 @@
         <v>844</v>
       </c>
       <c r="C392" s="0" t="s">
-        <v>303</v>
+        <v>132</v>
       </c>
       <c r="D392" s="0">
-        <v>570</v>
+        <v>6397.2</v>
       </c>
     </row>
     <row r="393">
@@ -8706,10 +8712,10 @@
         <v>846</v>
       </c>
       <c r="C393" s="0" t="s">
-        <v>69</v>
+        <v>303</v>
       </c>
       <c r="D393" s="0">
-        <v>550</v>
+        <v>570</v>
       </c>
     </row>
     <row r="394">
@@ -8720,10 +8726,10 @@
         <v>848</v>
       </c>
       <c r="C394" s="0" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="D394" s="0">
-        <v>167</v>
+        <v>550</v>
       </c>
     </row>
     <row r="395">
@@ -8734,10 +8740,10 @@
         <v>850</v>
       </c>
       <c r="C395" s="0" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="D395" s="0">
-        <v>701.42</v>
+        <v>167</v>
       </c>
     </row>
     <row r="396">
@@ -8748,10 +8754,10 @@
         <v>852</v>
       </c>
       <c r="C396" s="0" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="D396" s="0">
-        <v>101000</v>
+        <v>701.42</v>
       </c>
     </row>
     <row r="397">
@@ -8762,10 +8768,10 @@
         <v>854</v>
       </c>
       <c r="C397" s="0" t="s">
-        <v>115</v>
+        <v>58</v>
       </c>
       <c r="D397" s="0">
-        <v>6251</v>
+        <v>101000</v>
       </c>
     </row>
     <row r="398">
@@ -8776,10 +8782,10 @@
         <v>856</v>
       </c>
       <c r="C398" s="0" t="s">
-        <v>368</v>
+        <v>115</v>
       </c>
       <c r="D398" s="0">
-        <v>857.67</v>
+        <v>6251</v>
       </c>
     </row>
     <row r="399">
@@ -8790,10 +8796,10 @@
         <v>858</v>
       </c>
       <c r="C399" s="0" t="s">
-        <v>89</v>
+        <v>368</v>
       </c>
       <c r="D399" s="0">
-        <v>1164.66</v>
+        <v>857.67</v>
       </c>
     </row>
     <row r="400">
@@ -8804,10 +8810,10 @@
         <v>860</v>
       </c>
       <c r="C400" s="0" t="s">
-        <v>143</v>
+        <v>89</v>
       </c>
       <c r="D400" s="0">
-        <v>360</v>
+        <v>1164.66</v>
       </c>
     </row>
     <row r="401">
@@ -8821,7 +8827,7 @@
         <v>143</v>
       </c>
       <c r="D401" s="0">
-        <v>450</v>
+        <v>360</v>
       </c>
     </row>
     <row r="402">
@@ -8835,7 +8841,7 @@
         <v>143</v>
       </c>
       <c r="D402" s="0">
-        <v>2050</v>
+        <v>450</v>
       </c>
     </row>
     <row r="403">
@@ -8846,10 +8852,10 @@
         <v>866</v>
       </c>
       <c r="C403" s="0" t="s">
-        <v>570</v>
+        <v>143</v>
       </c>
       <c r="D403" s="0">
-        <v>25192.82</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="404">
@@ -8860,10 +8866,10 @@
         <v>868</v>
       </c>
       <c r="C404" s="0" t="s">
-        <v>69</v>
+        <v>570</v>
       </c>
       <c r="D404" s="0">
-        <v>3500</v>
+        <v>25192.82</v>
       </c>
     </row>
     <row r="405">
@@ -8874,10 +8880,10 @@
         <v>870</v>
       </c>
       <c r="C405" s="0" t="s">
-        <v>170</v>
+        <v>69</v>
       </c>
       <c r="D405" s="0">
-        <v>600</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="406">
@@ -8888,24 +8894,24 @@
         <v>872</v>
       </c>
       <c r="C406" s="0" t="s">
-        <v>873</v>
+        <v>170</v>
       </c>
       <c r="D406" s="0">
-        <v>1080</v>
+        <v>600</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="0" t="s">
+        <v>873</v>
+      </c>
+      <c r="B407" s="0" t="s">
         <v>874</v>
       </c>
-      <c r="B407" s="0" t="s">
+      <c r="C407" s="0" t="s">
         <v>875</v>
       </c>
-      <c r="C407" s="0" t="s">
-        <v>331</v>
-      </c>
       <c r="D407" s="0">
-        <v>8628</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="408">
@@ -8919,7 +8925,7 @@
         <v>331</v>
       </c>
       <c r="D408" s="0">
-        <v>9125.1</v>
+        <v>8628</v>
       </c>
     </row>
     <row r="409">
@@ -8930,10 +8936,10 @@
         <v>879</v>
       </c>
       <c r="C409" s="0" t="s">
-        <v>41</v>
+        <v>331</v>
       </c>
       <c r="D409" s="0">
-        <v>27991.54</v>
+        <v>9125.1</v>
       </c>
     </row>
     <row r="410">
@@ -8944,10 +8950,10 @@
         <v>881</v>
       </c>
       <c r="C410" s="0" t="s">
-        <v>132</v>
+        <v>41</v>
       </c>
       <c r="D410" s="0">
-        <v>1080</v>
+        <v>27991.54</v>
       </c>
     </row>
     <row r="411">
@@ -8961,7 +8967,7 @@
         <v>132</v>
       </c>
       <c r="D411" s="0">
-        <v>4500</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="412">
@@ -8972,10 +8978,10 @@
         <v>885</v>
       </c>
       <c r="C412" s="0" t="s">
-        <v>44</v>
+        <v>132</v>
       </c>
       <c r="D412" s="0">
-        <v>4194.88</v>
+        <v>4012</v>
       </c>
     </row>
     <row r="413">
@@ -8989,7 +8995,7 @@
         <v>44</v>
       </c>
       <c r="D413" s="0">
-        <v>2139.28</v>
+        <v>4404.62</v>
       </c>
     </row>
     <row r="414">
@@ -9003,7 +9009,7 @@
         <v>44</v>
       </c>
       <c r="D414" s="0">
-        <v>1699.1</v>
+        <v>2246.24</v>
       </c>
     </row>
     <row r="415">
@@ -9017,7 +9023,7 @@
         <v>44</v>
       </c>
       <c r="D415" s="0">
-        <v>3427.58</v>
+        <v>1784.06</v>
       </c>
     </row>
     <row r="416">
@@ -9031,7 +9037,7 @@
         <v>44</v>
       </c>
       <c r="D416" s="0">
-        <v>19700</v>
+        <v>3598.96</v>
       </c>
     </row>
     <row r="417">
@@ -9045,7 +9051,7 @@
         <v>44</v>
       </c>
       <c r="D417" s="0">
-        <v>1839.2</v>
+        <v>20685</v>
       </c>
     </row>
     <row r="418">
@@ -9059,7 +9065,7 @@
         <v>44</v>
       </c>
       <c r="D418" s="0">
-        <v>4215.45</v>
+        <v>1931.16</v>
       </c>
     </row>
     <row r="419">
@@ -9073,7 +9079,7 @@
         <v>44</v>
       </c>
       <c r="D419" s="0">
-        <v>3395.26</v>
+        <v>4426.22</v>
       </c>
     </row>
     <row r="420">
@@ -9084,10 +9090,10 @@
         <v>901</v>
       </c>
       <c r="C420" s="0" t="s">
-        <v>478</v>
+        <v>44</v>
       </c>
       <c r="D420" s="0">
-        <v>510</v>
+        <v>3565.02</v>
       </c>
     </row>
     <row r="421">
@@ -9098,7 +9104,7 @@
         <v>903</v>
       </c>
       <c r="C421" s="0" t="s">
-        <v>38</v>
+        <v>478</v>
       </c>
       <c r="D421" s="0">
         <v>510</v>
@@ -9112,24 +9118,24 @@
         <v>905</v>
       </c>
       <c r="C422" s="0" t="s">
-        <v>906</v>
+        <v>38</v>
       </c>
       <c r="D422" s="0">
-        <v>559</v>
+        <v>510</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="0" t="s">
+        <v>906</v>
+      </c>
+      <c r="B423" s="0" t="s">
         <v>907</v>
       </c>
-      <c r="B423" s="0" t="s">
+      <c r="C423" s="0" t="s">
         <v>908</v>
       </c>
-      <c r="C423" s="0" t="s">
-        <v>906</v>
-      </c>
       <c r="D423" s="0">
-        <v>559</v>
+        <v>580</v>
       </c>
     </row>
     <row r="424">
@@ -9140,10 +9146,10 @@
         <v>910</v>
       </c>
       <c r="C424" s="0" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
       <c r="D424" s="0">
-        <v>559</v>
+        <v>580</v>
       </c>
     </row>
     <row r="425">
@@ -9154,10 +9160,10 @@
         <v>912</v>
       </c>
       <c r="C425" s="0" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
       <c r="D425" s="0">
-        <v>342</v>
+        <v>580</v>
       </c>
     </row>
     <row r="426">
@@ -9168,7 +9174,7 @@
         <v>914</v>
       </c>
       <c r="C426" s="0" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
       <c r="D426" s="0">
         <v>342</v>
@@ -9182,7 +9188,7 @@
         <v>916</v>
       </c>
       <c r="C427" s="0" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
       <c r="D427" s="0">
         <v>342</v>
@@ -9196,10 +9202,10 @@
         <v>918</v>
       </c>
       <c r="C428" s="0" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
       <c r="D428" s="0">
-        <v>0</v>
+        <v>342</v>
       </c>
     </row>
     <row r="429">
@@ -9210,7 +9216,7 @@
         <v>920</v>
       </c>
       <c r="C429" s="0" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
       <c r="D429" s="0">
         <v>0</v>
@@ -9224,10 +9230,10 @@
         <v>922</v>
       </c>
       <c r="C430" s="0" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
       <c r="D430" s="0">
-        <v>423</v>
+        <v>0</v>
       </c>
     </row>
     <row r="431">
@@ -9238,10 +9244,10 @@
         <v>924</v>
       </c>
       <c r="C431" s="0" t="s">
-        <v>69</v>
+        <v>908</v>
       </c>
       <c r="D431" s="0">
-        <v>15968</v>
+        <v>423</v>
       </c>
     </row>
     <row r="432">
@@ -9252,10 +9258,10 @@
         <v>926</v>
       </c>
       <c r="C432" s="0" t="s">
-        <v>109</v>
+        <v>69</v>
       </c>
       <c r="D432" s="0">
-        <v>14000</v>
+        <v>15968</v>
       </c>
     </row>
     <row r="433">
@@ -9266,10 +9272,10 @@
         <v>928</v>
       </c>
       <c r="C433" s="0" t="s">
-        <v>132</v>
+        <v>109</v>
       </c>
       <c r="D433" s="0">
-        <v>14001</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="434">
@@ -9280,10 +9286,10 @@
         <v>930</v>
       </c>
       <c r="C434" s="0" t="s">
-        <v>89</v>
+        <v>132</v>
       </c>
       <c r="D434" s="0">
-        <v>266200</v>
+        <v>14001</v>
       </c>
     </row>
     <row r="435">
@@ -9297,7 +9303,7 @@
         <v>89</v>
       </c>
       <c r="D435" s="0">
-        <v>194991.5</v>
+        <v>266200</v>
       </c>
     </row>
     <row r="436">
@@ -9311,7 +9317,7 @@
         <v>89</v>
       </c>
       <c r="D436" s="0">
-        <v>289492.5</v>
+        <v>194991.5</v>
       </c>
     </row>
     <row r="437">
@@ -9322,24 +9328,24 @@
         <v>936</v>
       </c>
       <c r="C437" s="0" t="s">
-        <v>937</v>
+        <v>89</v>
       </c>
       <c r="D437" s="0">
-        <v>13722.52</v>
+        <v>289492.5</v>
       </c>
     </row>
     <row r="438">
       <c r="A438" s="0" t="s">
+        <v>937</v>
+      </c>
+      <c r="B438" s="0" t="s">
         <v>938</v>
       </c>
-      <c r="B438" s="0" t="s">
+      <c r="C438" s="0" t="s">
         <v>939</v>
       </c>
-      <c r="C438" s="0" t="s">
-        <v>937</v>
-      </c>
       <c r="D438" s="0">
-        <v>15072</v>
+        <v>13722.52</v>
       </c>
     </row>
     <row r="439">
@@ -9350,10 +9356,10 @@
         <v>941</v>
       </c>
       <c r="C439" s="0" t="s">
-        <v>937</v>
+        <v>939</v>
       </c>
       <c r="D439" s="0">
-        <v>6555.64</v>
+        <v>15072</v>
       </c>
     </row>
     <row r="440">
@@ -9364,10 +9370,10 @@
         <v>943</v>
       </c>
       <c r="C440" s="0" t="s">
-        <v>937</v>
+        <v>939</v>
       </c>
       <c r="D440" s="0">
-        <v>8964.61</v>
+        <v>6555.64</v>
       </c>
     </row>
     <row r="441">
@@ -9378,10 +9384,10 @@
         <v>945</v>
       </c>
       <c r="C441" s="0" t="s">
-        <v>937</v>
+        <v>939</v>
       </c>
       <c r="D441" s="0">
-        <v>11735</v>
+        <v>8964.61</v>
       </c>
     </row>
     <row r="442">
@@ -9392,10 +9398,10 @@
         <v>947</v>
       </c>
       <c r="C442" s="0" t="s">
-        <v>69</v>
+        <v>939</v>
       </c>
       <c r="D442" s="0">
-        <v>3380</v>
+        <v>11735</v>
       </c>
     </row>
     <row r="443">
@@ -9406,10 +9412,10 @@
         <v>949</v>
       </c>
       <c r="C443" s="0" t="s">
-        <v>132</v>
+        <v>69</v>
       </c>
       <c r="D443" s="0">
-        <v>3822.39</v>
+        <v>3380</v>
       </c>
     </row>
     <row r="444">
@@ -9420,10 +9426,10 @@
         <v>951</v>
       </c>
       <c r="C444" s="0" t="s">
-        <v>89</v>
+        <v>132</v>
       </c>
       <c r="D444" s="0">
-        <v>4392.3</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="445">
@@ -9434,24 +9440,24 @@
         <v>953</v>
       </c>
       <c r="C445" s="0" t="s">
-        <v>954</v>
+        <v>89</v>
       </c>
       <c r="D445" s="0">
-        <v>5254.41</v>
+        <v>4392.3</v>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="0" t="s">
+        <v>954</v>
+      </c>
+      <c r="B446" s="0" t="s">
         <v>955</v>
       </c>
-      <c r="B446" s="0" t="s">
+      <c r="C446" s="0" t="s">
         <v>956</v>
       </c>
-      <c r="C446" s="0" t="s">
-        <v>51</v>
-      </c>
       <c r="D446" s="0">
-        <v>1200</v>
+        <v>5254.41</v>
       </c>
     </row>
     <row r="447">
@@ -9465,7 +9471,7 @@
         <v>51</v>
       </c>
       <c r="D447" s="0">
-        <v>278</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="448">
@@ -9479,7 +9485,7 @@
         <v>51</v>
       </c>
       <c r="D448" s="0">
-        <v>562</v>
+        <v>278</v>
       </c>
     </row>
     <row r="449">
@@ -9490,10 +9496,10 @@
         <v>962</v>
       </c>
       <c r="C449" s="0" t="s">
-        <v>368</v>
+        <v>51</v>
       </c>
       <c r="D449" s="0">
-        <v>65142.6</v>
+        <v>562</v>
       </c>
     </row>
     <row r="450">
@@ -9507,7 +9513,7 @@
         <v>368</v>
       </c>
       <c r="D450" s="0">
-        <v>23482.7</v>
+        <v>65142.6</v>
       </c>
     </row>
     <row r="451">
@@ -9518,10 +9524,10 @@
         <v>966</v>
       </c>
       <c r="C451" s="0" t="s">
-        <v>29</v>
+        <v>368</v>
       </c>
       <c r="D451" s="0">
-        <v>5917.17</v>
+        <v>23482.7</v>
       </c>
     </row>
     <row r="452">
@@ -9532,10 +9538,10 @@
         <v>968</v>
       </c>
       <c r="C452" s="0" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="D452" s="0">
-        <v>10985</v>
+        <v>5917.17</v>
       </c>
     </row>
     <row r="453">
@@ -9549,7 +9555,7 @@
         <v>51</v>
       </c>
       <c r="D453" s="0">
-        <v>17425</v>
+        <v>10985</v>
       </c>
     </row>
     <row r="454">
@@ -9560,24 +9566,24 @@
         <v>972</v>
       </c>
       <c r="C454" s="0" t="s">
-        <v>973</v>
+        <v>51</v>
       </c>
       <c r="D454" s="0">
-        <v>1958</v>
+        <v>17425</v>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="0" t="s">
+        <v>973</v>
+      </c>
+      <c r="B455" s="0" t="s">
         <v>974</v>
       </c>
-      <c r="B455" s="0" t="s">
+      <c r="C455" s="0" t="s">
         <v>975</v>
       </c>
-      <c r="C455" s="0" t="s">
-        <v>89</v>
-      </c>
       <c r="D455" s="0">
-        <v>249562.5</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="456">
@@ -9588,10 +9594,10 @@
         <v>977</v>
       </c>
       <c r="C456" s="0" t="s">
-        <v>570</v>
+        <v>89</v>
       </c>
       <c r="D456" s="0">
-        <v>71176.4</v>
+        <v>249562.5</v>
       </c>
     </row>
     <row r="457">
@@ -9602,10 +9608,10 @@
         <v>979</v>
       </c>
       <c r="C457" s="0" t="s">
-        <v>132</v>
+        <v>570</v>
       </c>
       <c r="D457" s="0">
-        <v>82</v>
+        <v>71176.4</v>
       </c>
     </row>
     <row r="458">
@@ -9616,10 +9622,10 @@
         <v>981</v>
       </c>
       <c r="C458" s="0" t="s">
-        <v>69</v>
+        <v>132</v>
       </c>
       <c r="D458" s="0">
-        <v>950</v>
+        <v>96</v>
       </c>
     </row>
     <row r="459">
@@ -9630,10 +9636,10 @@
         <v>983</v>
       </c>
       <c r="C459" s="0" t="s">
-        <v>469</v>
+        <v>69</v>
       </c>
       <c r="D459" s="0">
-        <v>342641</v>
+        <v>950</v>
       </c>
     </row>
     <row r="460">
@@ -9644,10 +9650,10 @@
         <v>985</v>
       </c>
       <c r="C460" s="0" t="s">
-        <v>150</v>
+        <v>469</v>
       </c>
       <c r="D460" s="0">
-        <v>2200</v>
+        <v>342641</v>
       </c>
     </row>
     <row r="461">
@@ -9658,10 +9664,10 @@
         <v>987</v>
       </c>
       <c r="C461" s="0" t="s">
-        <v>478</v>
+        <v>150</v>
       </c>
       <c r="D461" s="0">
-        <v>41000</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="462">
@@ -9672,10 +9678,10 @@
         <v>989</v>
       </c>
       <c r="C462" s="0" t="s">
-        <v>69</v>
+        <v>478</v>
       </c>
       <c r="D462" s="0">
-        <v>9299</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="463">
@@ -9686,10 +9692,10 @@
         <v>991</v>
       </c>
       <c r="C463" s="0" t="s">
-        <v>906</v>
+        <v>69</v>
       </c>
       <c r="D463" s="0">
-        <v>595</v>
+        <v>9299</v>
       </c>
     </row>
     <row r="464">
@@ -9700,10 +9706,10 @@
         <v>993</v>
       </c>
       <c r="C464" s="0" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
       <c r="D464" s="0">
-        <v>595</v>
+        <v>825</v>
       </c>
     </row>
     <row r="465">
@@ -9714,10 +9720,10 @@
         <v>995</v>
       </c>
       <c r="C465" s="0" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
       <c r="D465" s="0">
-        <v>595</v>
+        <v>825</v>
       </c>
     </row>
     <row r="466">
@@ -9728,10 +9734,10 @@
         <v>997</v>
       </c>
       <c r="C466" s="0" t="s">
-        <v>22</v>
+        <v>908</v>
       </c>
       <c r="D466" s="0">
-        <v>563.36</v>
+        <v>825</v>
       </c>
     </row>
     <row r="467">
@@ -9742,10 +9748,10 @@
         <v>999</v>
       </c>
       <c r="C467" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D467" s="0">
-        <v>3520</v>
+        <v>563.36</v>
       </c>
     </row>
     <row r="468">
@@ -9759,7 +9765,7 @@
         <v>16</v>
       </c>
       <c r="D468" s="0">
-        <v>2600</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="469">
@@ -9770,10 +9776,10 @@
         <v>1003</v>
       </c>
       <c r="C469" s="0" t="s">
-        <v>276</v>
+        <v>16</v>
       </c>
       <c r="D469" s="0">
-        <v>3700</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="470">
@@ -9787,7 +9793,7 @@
         <v>276</v>
       </c>
       <c r="D470" s="0">
-        <v>2600</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="471">
@@ -9798,10 +9804,10 @@
         <v>1007</v>
       </c>
       <c r="C471" s="0" t="s">
-        <v>16</v>
+        <v>276</v>
       </c>
       <c r="D471" s="0">
-        <v>2235</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="472">
@@ -9815,35 +9821,35 @@
         <v>16</v>
       </c>
       <c r="D472" s="0">
-        <v>3850</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="0" t="s">
-        <v>389</v>
+        <v>1010</v>
       </c>
       <c r="B473" s="0" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="C473" s="0" t="s">
-        <v>1011</v>
+        <v>16</v>
       </c>
       <c r="D473" s="0">
-        <v>1</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="474">
       <c r="A474" s="0" t="s">
+        <v>389</v>
+      </c>
+      <c r="B474" s="0" t="s">
         <v>1012</v>
       </c>
-      <c r="B474" s="0" t="s">
+      <c r="C474" s="0" t="s">
         <v>1013</v>
       </c>
-      <c r="C474" s="0" t="s">
-        <v>29</v>
-      </c>
       <c r="D474" s="0">
-        <v>13715</v>
+        <v>1</v>
       </c>
     </row>
     <row r="475">
@@ -9854,10 +9860,10 @@
         <v>1015</v>
       </c>
       <c r="C475" s="0" t="s">
-        <v>368</v>
+        <v>29</v>
       </c>
       <c r="D475" s="0">
-        <v>3859.93</v>
+        <v>13715</v>
       </c>
     </row>
     <row r="476">
@@ -9871,7 +9877,7 @@
         <v>368</v>
       </c>
       <c r="D476" s="0">
-        <v>11751.49</v>
+        <v>3859.93</v>
       </c>
     </row>
     <row r="477">
@@ -9882,10 +9888,10 @@
         <v>1019</v>
       </c>
       <c r="C477" s="0" t="s">
-        <v>331</v>
+        <v>368</v>
       </c>
       <c r="D477" s="0">
-        <v>6000</v>
+        <v>11751.49</v>
       </c>
     </row>
     <row r="478">
@@ -9899,7 +9905,7 @@
         <v>331</v>
       </c>
       <c r="D478" s="0">
-        <v>3000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="479">
@@ -9910,10 +9916,10 @@
         <v>1023</v>
       </c>
       <c r="C479" s="0" t="s">
-        <v>38</v>
+        <v>331</v>
       </c>
       <c r="D479" s="0">
-        <v>618</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="480">
@@ -9924,24 +9930,24 @@
         <v>1025</v>
       </c>
       <c r="C480" s="0" t="s">
-        <v>1026</v>
+        <v>38</v>
       </c>
       <c r="D480" s="0">
-        <v>24600</v>
+        <v>618</v>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="0" t="s">
+        <v>1026</v>
+      </c>
+      <c r="B481" s="0" t="s">
         <v>1027</v>
       </c>
-      <c r="B481" s="0" t="s">
+      <c r="C481" s="0" t="s">
         <v>1028</v>
       </c>
-      <c r="C481" s="0" t="s">
-        <v>102</v>
-      </c>
       <c r="D481" s="0">
-        <v>0</v>
+        <v>24600</v>
       </c>
     </row>
     <row r="482">
@@ -9952,10 +9958,10 @@
         <v>1030</v>
       </c>
       <c r="C482" s="0" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="D482" s="0">
-        <v>32942.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="483">
@@ -9966,10 +9972,10 @@
         <v>1032</v>
       </c>
       <c r="C483" s="0" t="s">
-        <v>368</v>
+        <v>89</v>
       </c>
       <c r="D483" s="0">
-        <v>75529.71</v>
+        <v>32942.25</v>
       </c>
     </row>
     <row r="484">
@@ -9983,7 +9989,7 @@
         <v>368</v>
       </c>
       <c r="D484" s="0">
-        <v>41613.42</v>
+        <v>75529.71</v>
       </c>
     </row>
     <row r="485">
@@ -9997,7 +10003,7 @@
         <v>368</v>
       </c>
       <c r="D485" s="0">
-        <v>87056.42</v>
+        <v>41613.42</v>
       </c>
     </row>
     <row r="486">
@@ -10011,7 +10017,7 @@
         <v>368</v>
       </c>
       <c r="D486" s="0">
-        <v>49243.16</v>
+        <v>87056.42</v>
       </c>
     </row>
     <row r="487">
@@ -10022,10 +10028,10 @@
         <v>1040</v>
       </c>
       <c r="C487" s="0" t="s">
-        <v>22</v>
+        <v>368</v>
       </c>
       <c r="D487" s="0">
-        <v>1600</v>
+        <v>49243.16</v>
       </c>
     </row>
     <row r="488">
@@ -10036,10 +10042,10 @@
         <v>1042</v>
       </c>
       <c r="C488" s="0" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D488" s="0">
-        <v>3338.9</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="489">
@@ -10053,7 +10059,7 @@
         <v>29</v>
       </c>
       <c r="D489" s="0">
-        <v>3987</v>
+        <v>3338.9</v>
       </c>
     </row>
     <row r="490">
@@ -10067,7 +10073,7 @@
         <v>29</v>
       </c>
       <c r="D490" s="0">
-        <v>4010.17</v>
+        <v>3987</v>
       </c>
     </row>
     <row r="491">
@@ -10081,35 +10087,35 @@
         <v>29</v>
       </c>
       <c r="D491" s="0">
+        <v>4010.17</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="0" t="s">
+        <v>1049</v>
+      </c>
+      <c r="B492" s="0" t="s">
+        <v>1050</v>
+      </c>
+      <c r="C492" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D492" s="0">
         <v>3382.65</v>
       </c>
     </row>
-    <row r="492">
-      <c r="A492" s="2" t="s">
-        <v>1049</v>
-      </c>
-      <c r="B492" s="2" t="s">
-        <v>1050</v>
-      </c>
-      <c r="C492" s="2" t="s">
+    <row r="493">
+      <c r="A493" s="2" t="s">
+        <v>1051</v>
+      </c>
+      <c r="B493" s="2" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C493" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D492" s="2">
+      <c r="D493" s="2">
         <v>0</v>
-      </c>
-    </row>
-    <row r="493">
-      <c r="A493" s="0" t="s">
-        <v>1051</v>
-      </c>
-      <c r="B493" s="0" t="s">
-        <v>1052</v>
-      </c>
-      <c r="C493" s="0" t="s">
-        <v>150</v>
-      </c>
-      <c r="D493" s="0">
-        <v>430</v>
       </c>
     </row>
     <row r="494">
@@ -10120,10 +10126,24 @@
         <v>1054</v>
       </c>
       <c r="C494" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="D494" s="0">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="0" t="s">
+        <v>1055</v>
+      </c>
+      <c r="B495" s="0" t="s">
+        <v>1056</v>
+      </c>
+      <c r="C495" s="0" t="s">
         <v>132</v>
       </c>
-      <c r="D494" s="0">
-        <v>435</v>
+      <c r="D495" s="0">
+        <v>462</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sync: stock y precios actualizados mié. 01/07/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -3480,7 +3480,7 @@
         <v>44</v>
       </c>
       <c r="D18" s="0">
-        <v>2675.19</v>
+        <v>3532.97</v>
       </c>
     </row>
     <row r="19">
@@ -4740,7 +4740,7 @@
         <v>44</v>
       </c>
       <c r="D108" s="0">
-        <v>4007.07</v>
+        <v>5291.87</v>
       </c>
     </row>
     <row r="109">
@@ -7862,7 +7862,7 @@
         <v>44</v>
       </c>
       <c r="D331" s="0">
-        <v>4053.7</v>
+        <v>5300</v>
       </c>
     </row>
     <row r="332">
@@ -8958,16 +8958,16 @@
       </c>
     </row>
     <row r="410">
-      <c r="A410" s="0" t="s">
+      <c r="A410" s="2" t="s">
         <v>880</v>
       </c>
-      <c r="B410" s="0" t="s">
+      <c r="B410" s="2" t="s">
         <v>881</v>
       </c>
-      <c r="C410" s="0" t="s">
+      <c r="C410" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="D410" s="0">
+      <c r="D410" s="2">
         <v>9125.1</v>
       </c>
     </row>
@@ -9024,7 +9024,7 @@
         <v>44</v>
       </c>
       <c r="D414" s="0">
-        <v>4404.62</v>
+        <v>5816.9</v>
       </c>
     </row>
     <row r="415">
@@ -9038,7 +9038,7 @@
         <v>44</v>
       </c>
       <c r="D415" s="0">
-        <v>2246.24</v>
+        <v>2624.28</v>
       </c>
     </row>
     <row r="416">
@@ -9052,20 +9052,20 @@
         <v>44</v>
       </c>
       <c r="D416" s="0">
-        <v>1784.06</v>
+        <v>1953.98</v>
       </c>
     </row>
     <row r="417">
-      <c r="A417" s="0" t="s">
+      <c r="A417" s="2" t="s">
         <v>894</v>
       </c>
-      <c r="B417" s="0" t="s">
+      <c r="B417" s="2" t="s">
         <v>895</v>
       </c>
-      <c r="C417" s="0" t="s">
+      <c r="C417" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D417" s="0">
+      <c r="D417" s="2">
         <v>3598.96</v>
       </c>
     </row>
@@ -9080,7 +9080,7 @@
         <v>44</v>
       </c>
       <c r="D418" s="0">
-        <v>20685</v>
+        <v>27318.17</v>
       </c>
     </row>
     <row r="419">
@@ -9094,7 +9094,7 @@
         <v>44</v>
       </c>
       <c r="D419" s="0">
-        <v>1931.16</v>
+        <v>2115.26</v>
       </c>
     </row>
     <row r="420">
@@ -9108,7 +9108,7 @@
         <v>44</v>
       </c>
       <c r="D420" s="0">
-        <v>4426.22</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="421">
@@ -9122,7 +9122,7 @@
         <v>44</v>
       </c>
       <c r="D421" s="0">
-        <v>3565.02</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="422">

</xml_diff>

<commit_message>
sync: stock y precios actualizados sáb. 04/07/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1062" uniqueCount="1062">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1064" uniqueCount="1064">
   <si>
     <t>Código</t>
   </si>
@@ -1461,6 +1461,12 @@
   </si>
   <si>
     <t>GRIPABEN CARAMELOS Caram. x 9 - 000016343</t>
+  </si>
+  <si>
+    <t>000024406</t>
+  </si>
+  <si>
+    <t>GUANTE DE EXAMEN DE NITRILO TALLE M X 100 - 000024406</t>
   </si>
   <si>
     <t>000023840</t>
@@ -3256,7 +3262,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A3:D497"/>
+  <dimension ref="A3:D498"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="3">
@@ -3508,7 +3514,7 @@
         <v>44</v>
       </c>
       <c r="D20" s="0">
-        <v>22133.38</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="21">
@@ -3914,7 +3920,7 @@
         <v>89</v>
       </c>
       <c r="D49" s="0">
-        <v>31944</v>
+        <v>33275</v>
       </c>
     </row>
     <row r="50">
@@ -4614,7 +4620,7 @@
         <v>89</v>
       </c>
       <c r="D99" s="0">
-        <v>3141.2</v>
+        <v>3194.4</v>
       </c>
     </row>
     <row r="100">
@@ -4628,7 +4634,7 @@
         <v>89</v>
       </c>
       <c r="D100" s="0">
-        <v>2355.84</v>
+        <v>2435.76</v>
       </c>
     </row>
     <row r="101">
@@ -4642,7 +4648,7 @@
         <v>89</v>
       </c>
       <c r="D101" s="0">
-        <v>3533.76</v>
+        <v>3653.64</v>
       </c>
     </row>
     <row r="102">
@@ -4824,7 +4830,7 @@
         <v>89</v>
       </c>
       <c r="D114" s="0">
-        <v>9649.75</v>
+        <v>9982.5</v>
       </c>
     </row>
     <row r="115">
@@ -6280,7 +6286,7 @@
         <v>51</v>
       </c>
       <c r="D218" s="0">
-        <v>4200</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="219">
@@ -6319,21 +6325,21 @@
         <v>490</v>
       </c>
       <c r="C221" s="0" t="s">
-        <v>491</v>
+        <v>51</v>
       </c>
       <c r="D221" s="0">
-        <v>265</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="0" t="s">
+        <v>491</v>
+      </c>
+      <c r="B222" s="0" t="s">
         <v>492</v>
       </c>
-      <c r="B222" s="0" t="s">
+      <c r="C222" s="0" t="s">
         <v>493</v>
-      </c>
-      <c r="C222" s="0" t="s">
-        <v>491</v>
       </c>
       <c r="D222" s="0">
         <v>265</v>
@@ -6347,7 +6353,7 @@
         <v>495</v>
       </c>
       <c r="C223" s="0" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="D223" s="0">
         <v>265</v>
@@ -6361,7 +6367,7 @@
         <v>497</v>
       </c>
       <c r="C224" s="0" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="D224" s="0">
         <v>265</v>
@@ -6375,7 +6381,7 @@
         <v>499</v>
       </c>
       <c r="C225" s="0" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="D225" s="0">
         <v>265</v>
@@ -6389,7 +6395,7 @@
         <v>501</v>
       </c>
       <c r="C226" s="0" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="D226" s="0">
         <v>265</v>
@@ -6403,21 +6409,21 @@
         <v>503</v>
       </c>
       <c r="C227" s="0" t="s">
-        <v>504</v>
+        <v>493</v>
       </c>
       <c r="D227" s="0">
-        <v>4700</v>
+        <v>265</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="0" t="s">
+        <v>504</v>
+      </c>
+      <c r="B228" s="0" t="s">
         <v>505</v>
       </c>
-      <c r="B228" s="0" t="s">
+      <c r="C228" s="0" t="s">
         <v>506</v>
-      </c>
-      <c r="C228" s="0" t="s">
-        <v>507</v>
       </c>
       <c r="D228" s="0">
         <v>4700</v>
@@ -6425,13 +6431,13 @@
     </row>
     <row r="229">
       <c r="A229" s="0" t="s">
+        <v>507</v>
+      </c>
+      <c r="B229" s="0" t="s">
         <v>508</v>
       </c>
-      <c r="B229" s="0" t="s">
+      <c r="C229" s="0" t="s">
         <v>509</v>
-      </c>
-      <c r="C229" s="0" t="s">
-        <v>504</v>
       </c>
       <c r="D229" s="0">
         <v>4700</v>
@@ -6448,7 +6454,7 @@
         <v>51</v>
       </c>
       <c r="D230" s="0">
-        <v>500</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="231">
@@ -6462,7 +6468,7 @@
         <v>51</v>
       </c>
       <c r="D231" s="0">
-        <v>210</v>
+        <v>500</v>
       </c>
     </row>
     <row r="232">
@@ -6476,7 +6482,7 @@
         <v>51</v>
       </c>
       <c r="D232" s="0">
-        <v>247</v>
+        <v>210</v>
       </c>
     </row>
     <row r="233">
@@ -6487,10 +6493,10 @@
         <v>517</v>
       </c>
       <c r="C233" s="0" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="D233" s="0">
-        <v>5600</v>
+        <v>247</v>
       </c>
     </row>
     <row r="234">
@@ -6501,10 +6507,10 @@
         <v>519</v>
       </c>
       <c r="C234" s="0" t="s">
-        <v>143</v>
+        <v>38</v>
       </c>
       <c r="D234" s="0">
-        <v>6000</v>
+        <v>5600</v>
       </c>
     </row>
     <row r="235">
@@ -6515,10 +6521,10 @@
         <v>521</v>
       </c>
       <c r="C235" s="0" t="s">
-        <v>69</v>
+        <v>143</v>
       </c>
       <c r="D235" s="0">
-        <v>80000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="236">
@@ -6532,7 +6538,7 @@
         <v>69</v>
       </c>
       <c r="D236" s="0">
-        <v>90000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="237">
@@ -6546,7 +6552,7 @@
         <v>69</v>
       </c>
       <c r="D237" s="0">
-        <v>110000</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="238">
@@ -6557,10 +6563,10 @@
         <v>527</v>
       </c>
       <c r="C238" s="0" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="D238" s="0">
-        <v>1100</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="239">
@@ -6574,7 +6580,7 @@
         <v>16</v>
       </c>
       <c r="D239" s="0">
-        <v>2500</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="240">
@@ -6585,10 +6591,10 @@
         <v>531</v>
       </c>
       <c r="C240" s="0" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="D240" s="0">
-        <v>13304.2</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="241">
@@ -6599,10 +6605,10 @@
         <v>533</v>
       </c>
       <c r="C241" s="0" t="s">
-        <v>279</v>
+        <v>29</v>
       </c>
       <c r="D241" s="0">
-        <v>450</v>
+        <v>13304.2</v>
       </c>
     </row>
     <row r="242">
@@ -6613,10 +6619,10 @@
         <v>535</v>
       </c>
       <c r="C242" s="0" t="s">
-        <v>16</v>
+        <v>279</v>
       </c>
       <c r="D242" s="0">
-        <v>555</v>
+        <v>450</v>
       </c>
     </row>
     <row r="243">
@@ -6630,7 +6636,7 @@
         <v>16</v>
       </c>
       <c r="D243" s="0">
-        <v>825</v>
+        <v>555</v>
       </c>
     </row>
     <row r="244">
@@ -6644,7 +6650,7 @@
         <v>16</v>
       </c>
       <c r="D244" s="0">
-        <v>36.3</v>
+        <v>825</v>
       </c>
     </row>
     <row r="245">
@@ -6658,7 +6664,7 @@
         <v>16</v>
       </c>
       <c r="D245" s="0">
-        <v>544.5</v>
+        <v>36.3</v>
       </c>
     </row>
     <row r="246">
@@ -6672,7 +6678,7 @@
         <v>16</v>
       </c>
       <c r="D246" s="0">
-        <v>640</v>
+        <v>544.5</v>
       </c>
     </row>
     <row r="247">
@@ -6683,10 +6689,10 @@
         <v>545</v>
       </c>
       <c r="C247" s="0" t="s">
-        <v>143</v>
+        <v>16</v>
       </c>
       <c r="D247" s="0">
-        <v>1130</v>
+        <v>640</v>
       </c>
     </row>
     <row r="248">
@@ -6697,10 +6703,10 @@
         <v>547</v>
       </c>
       <c r="C248" s="0" t="s">
-        <v>51</v>
+        <v>143</v>
       </c>
       <c r="D248" s="0">
-        <v>4510</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="249">
@@ -6753,10 +6759,10 @@
         <v>555</v>
       </c>
       <c r="C252" s="0" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="D252" s="0">
-        <v>902</v>
+        <v>4510</v>
       </c>
     </row>
     <row r="253">
@@ -6770,7 +6776,7 @@
         <v>16</v>
       </c>
       <c r="D253" s="0">
-        <v>880</v>
+        <v>902</v>
       </c>
     </row>
     <row r="254">
@@ -6781,10 +6787,10 @@
         <v>559</v>
       </c>
       <c r="C254" s="0" t="s">
-        <v>132</v>
+        <v>16</v>
       </c>
       <c r="D254" s="0">
-        <v>430</v>
+        <v>880</v>
       </c>
     </row>
     <row r="255">
@@ -6798,7 +6804,7 @@
         <v>132</v>
       </c>
       <c r="D255" s="0">
-        <v>354.54</v>
+        <v>430</v>
       </c>
     </row>
     <row r="256">
@@ -6809,10 +6815,10 @@
         <v>563</v>
       </c>
       <c r="C256" s="0" t="s">
-        <v>19</v>
+        <v>132</v>
       </c>
       <c r="D256" s="0">
-        <v>318.63</v>
+        <v>354.54</v>
       </c>
     </row>
     <row r="257">
@@ -6826,7 +6832,7 @@
         <v>19</v>
       </c>
       <c r="D257" s="0">
-        <v>415.15</v>
+        <v>318.63</v>
       </c>
     </row>
     <row r="258">
@@ -6840,7 +6846,7 @@
         <v>19</v>
       </c>
       <c r="D258" s="0">
-        <v>760</v>
+        <v>415.15</v>
       </c>
     </row>
     <row r="259">
@@ -6854,7 +6860,7 @@
         <v>19</v>
       </c>
       <c r="D259" s="0">
-        <v>820</v>
+        <v>760</v>
       </c>
     </row>
     <row r="260">
@@ -6865,24 +6871,24 @@
         <v>571</v>
       </c>
       <c r="C260" s="0" t="s">
-        <v>572</v>
+        <v>19</v>
       </c>
       <c r="D260" s="0">
-        <v>177940.1</v>
+        <v>820</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="0" t="s">
+        <v>572</v>
+      </c>
+      <c r="B261" s="0" t="s">
         <v>573</v>
       </c>
-      <c r="B261" s="0" t="s">
+      <c r="C261" s="0" t="s">
         <v>574</v>
       </c>
-      <c r="C261" s="0" t="s">
-        <v>69</v>
-      </c>
       <c r="D261" s="0">
-        <v>34000</v>
+        <v>177940.1</v>
       </c>
     </row>
     <row r="262">
@@ -6896,7 +6902,7 @@
         <v>69</v>
       </c>
       <c r="D262" s="0">
-        <v>30000</v>
+        <v>34000</v>
       </c>
     </row>
     <row r="263">
@@ -6907,10 +6913,10 @@
         <v>578</v>
       </c>
       <c r="C263" s="0" t="s">
-        <v>471</v>
+        <v>69</v>
       </c>
       <c r="D263" s="0">
-        <v>227939.52</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="264">
@@ -6924,7 +6930,7 @@
         <v>471</v>
       </c>
       <c r="D264" s="0">
-        <v>184488.7</v>
+        <v>227939.52</v>
       </c>
     </row>
     <row r="265">
@@ -6935,10 +6941,10 @@
         <v>582</v>
       </c>
       <c r="C265" s="0" t="s">
-        <v>16</v>
+        <v>471</v>
       </c>
       <c r="D265" s="0">
-        <v>1760</v>
+        <v>184488.7</v>
       </c>
     </row>
     <row r="266">
@@ -6949,24 +6955,24 @@
         <v>584</v>
       </c>
       <c r="C266" s="0" t="s">
-        <v>585</v>
+        <v>16</v>
       </c>
       <c r="D266" s="0">
-        <v>26350</v>
+        <v>1760</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="0" t="s">
+        <v>585</v>
+      </c>
+      <c r="B267" s="0" t="s">
         <v>586</v>
       </c>
-      <c r="B267" s="0" t="s">
+      <c r="C267" s="0" t="s">
         <v>587</v>
       </c>
-      <c r="C267" s="0" t="s">
-        <v>480</v>
-      </c>
       <c r="D267" s="0">
-        <v>31250</v>
+        <v>26350</v>
       </c>
     </row>
     <row r="268">
@@ -6977,10 +6983,10 @@
         <v>589</v>
       </c>
       <c r="C268" s="0" t="s">
-        <v>51</v>
+        <v>480</v>
       </c>
       <c r="D268" s="0">
-        <v>34.98</v>
+        <v>31250</v>
       </c>
     </row>
     <row r="269">
@@ -6994,7 +7000,7 @@
         <v>51</v>
       </c>
       <c r="D269" s="0">
-        <v>65</v>
+        <v>34.98</v>
       </c>
     </row>
     <row r="270">
@@ -7008,7 +7014,7 @@
         <v>51</v>
       </c>
       <c r="D270" s="0">
-        <v>92</v>
+        <v>65</v>
       </c>
     </row>
     <row r="271">
@@ -7022,7 +7028,7 @@
         <v>51</v>
       </c>
       <c r="D271" s="0">
-        <v>33</v>
+        <v>92</v>
       </c>
     </row>
     <row r="272">
@@ -7036,7 +7042,7 @@
         <v>51</v>
       </c>
       <c r="D272" s="0">
-        <v>38.22</v>
+        <v>33</v>
       </c>
     </row>
     <row r="273">
@@ -7047,10 +7053,10 @@
         <v>599</v>
       </c>
       <c r="C273" s="0" t="s">
-        <v>334</v>
+        <v>51</v>
       </c>
       <c r="D273" s="0">
-        <v>300</v>
+        <v>38.22</v>
       </c>
     </row>
     <row r="274">
@@ -7064,7 +7070,7 @@
         <v>334</v>
       </c>
       <c r="D274" s="0">
-        <v>370</v>
+        <v>300</v>
       </c>
     </row>
     <row r="275">
@@ -7075,10 +7081,10 @@
         <v>603</v>
       </c>
       <c r="C275" s="0" t="s">
-        <v>355</v>
+        <v>334</v>
       </c>
       <c r="D275" s="0">
-        <v>450</v>
+        <v>370</v>
       </c>
     </row>
     <row r="276">
@@ -7089,7 +7095,7 @@
         <v>605</v>
       </c>
       <c r="C276" s="0" t="s">
-        <v>38</v>
+        <v>355</v>
       </c>
       <c r="D276" s="0">
         <v>450</v>
@@ -7103,7 +7109,7 @@
         <v>607</v>
       </c>
       <c r="C277" s="0" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="D277" s="0">
         <v>450</v>
@@ -7120,7 +7126,7 @@
         <v>16</v>
       </c>
       <c r="D278" s="0">
-        <v>1650</v>
+        <v>450</v>
       </c>
     </row>
     <row r="279">
@@ -7134,7 +7140,7 @@
         <v>16</v>
       </c>
       <c r="D279" s="0">
-        <v>2100</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="280">
@@ -7148,7 +7154,7 @@
         <v>16</v>
       </c>
       <c r="D280" s="0">
-        <v>1980</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="281">
@@ -7162,7 +7168,7 @@
         <v>16</v>
       </c>
       <c r="D281" s="0">
-        <v>2160</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="282">
@@ -7176,7 +7182,7 @@
         <v>16</v>
       </c>
       <c r="D282" s="0">
-        <v>1100</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="283">
@@ -7190,7 +7196,7 @@
         <v>16</v>
       </c>
       <c r="D283" s="0">
-        <v>2600</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="284">
@@ -7204,7 +7210,7 @@
         <v>16</v>
       </c>
       <c r="D284" s="0">
-        <v>2000</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="285">
@@ -7218,7 +7224,7 @@
         <v>16</v>
       </c>
       <c r="D285" s="0">
-        <v>6700</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="286">
@@ -7232,7 +7238,7 @@
         <v>16</v>
       </c>
       <c r="D286" s="0">
-        <v>1650</v>
+        <v>6700</v>
       </c>
     </row>
     <row r="287">
@@ -7246,7 +7252,7 @@
         <v>16</v>
       </c>
       <c r="D287" s="0">
-        <v>1035</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="288">
@@ -7260,7 +7266,7 @@
         <v>16</v>
       </c>
       <c r="D288" s="0">
-        <v>2600</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="289">
@@ -7274,7 +7280,7 @@
         <v>16</v>
       </c>
       <c r="D289" s="0">
-        <v>2400</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="290">
@@ -7285,10 +7291,10 @@
         <v>633</v>
       </c>
       <c r="C290" s="0" t="s">
-        <v>132</v>
+        <v>16</v>
       </c>
       <c r="D290" s="0">
-        <v>4497.2</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="291">
@@ -7302,7 +7308,7 @@
         <v>132</v>
       </c>
       <c r="D291" s="0">
-        <v>2328</v>
+        <v>4497.2</v>
       </c>
     </row>
     <row r="292">
@@ -7316,7 +7322,7 @@
         <v>132</v>
       </c>
       <c r="D292" s="0">
-        <v>1138</v>
+        <v>2328</v>
       </c>
     </row>
     <row r="293">
@@ -7327,10 +7333,10 @@
         <v>639</v>
       </c>
       <c r="C293" s="0" t="s">
-        <v>29</v>
+        <v>132</v>
       </c>
       <c r="D293" s="0">
-        <v>7234.96</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="294">
@@ -7341,10 +7347,10 @@
         <v>641</v>
       </c>
       <c r="C294" s="0" t="s">
-        <v>115</v>
+        <v>29</v>
       </c>
       <c r="D294" s="0">
-        <v>1790</v>
+        <v>7234.96</v>
       </c>
     </row>
     <row r="295">
@@ -7358,7 +7364,7 @@
         <v>115</v>
       </c>
       <c r="D295" s="0">
-        <v>2859.96</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="296">
@@ -7372,7 +7378,7 @@
         <v>115</v>
       </c>
       <c r="D296" s="0">
-        <v>4800</v>
+        <v>2859.96</v>
       </c>
     </row>
     <row r="297">
@@ -7383,24 +7389,24 @@
         <v>647</v>
       </c>
       <c r="C297" s="0" t="s">
-        <v>648</v>
+        <v>115</v>
       </c>
       <c r="D297" s="0">
-        <v>0</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="0" t="s">
+        <v>648</v>
+      </c>
+      <c r="B298" s="0" t="s">
         <v>649</v>
       </c>
-      <c r="B298" s="0" t="s">
+      <c r="C298" s="0" t="s">
         <v>650</v>
       </c>
-      <c r="C298" s="0" t="s">
-        <v>29</v>
-      </c>
       <c r="D298" s="0">
-        <v>494</v>
+        <v>0</v>
       </c>
     </row>
     <row r="299">
@@ -7414,7 +7420,7 @@
         <v>29</v>
       </c>
       <c r="D299" s="0">
-        <v>665.3</v>
+        <v>494</v>
       </c>
     </row>
     <row r="300">
@@ -7425,10 +7431,10 @@
         <v>654</v>
       </c>
       <c r="C300" s="0" t="s">
-        <v>89</v>
+        <v>29</v>
       </c>
       <c r="D300" s="0">
-        <v>32609.5</v>
+        <v>665.3</v>
       </c>
     </row>
     <row r="301">
@@ -7442,7 +7448,7 @@
         <v>89</v>
       </c>
       <c r="D301" s="0">
-        <v>4525.4</v>
+        <v>33275</v>
       </c>
     </row>
     <row r="302">
@@ -7453,10 +7459,10 @@
         <v>658</v>
       </c>
       <c r="C302" s="0" t="s">
-        <v>143</v>
+        <v>89</v>
       </c>
       <c r="D302" s="0">
-        <v>896</v>
+        <v>4525.4</v>
       </c>
     </row>
     <row r="303">
@@ -7467,10 +7473,10 @@
         <v>660</v>
       </c>
       <c r="C303" s="0" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="D303" s="0">
-        <v>1250</v>
+        <v>896</v>
       </c>
     </row>
     <row r="304">
@@ -7481,10 +7487,10 @@
         <v>662</v>
       </c>
       <c r="C304" s="0" t="s">
-        <v>89</v>
+        <v>132</v>
       </c>
       <c r="D304" s="0">
-        <v>306130</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="305">
@@ -7495,10 +7501,10 @@
         <v>664</v>
       </c>
       <c r="C305" s="0" t="s">
-        <v>197</v>
+        <v>89</v>
       </c>
       <c r="D305" s="0">
-        <v>17440</v>
+        <v>312785</v>
       </c>
     </row>
     <row r="306">
@@ -7512,7 +7518,7 @@
         <v>197</v>
       </c>
       <c r="D306" s="0">
-        <v>4390</v>
+        <v>17440</v>
       </c>
     </row>
     <row r="307">
@@ -7537,10 +7543,10 @@
         <v>670</v>
       </c>
       <c r="C308" s="0" t="s">
-        <v>279</v>
+        <v>197</v>
       </c>
       <c r="D308" s="0">
-        <v>2250</v>
+        <v>4390</v>
       </c>
     </row>
     <row r="309">
@@ -7551,10 +7557,10 @@
         <v>672</v>
       </c>
       <c r="C309" s="0" t="s">
-        <v>197</v>
+        <v>279</v>
       </c>
       <c r="D309" s="0">
-        <v>3355</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="310">
@@ -7565,10 +7571,10 @@
         <v>674</v>
       </c>
       <c r="C310" s="0" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="D310" s="0">
-        <v>7500</v>
+        <v>3355</v>
       </c>
     </row>
     <row r="311">
@@ -7579,10 +7585,10 @@
         <v>676</v>
       </c>
       <c r="C311" s="0" t="s">
-        <v>89</v>
+        <v>202</v>
       </c>
       <c r="D311" s="0">
-        <v>23958</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="312">
@@ -7596,7 +7602,7 @@
         <v>89</v>
       </c>
       <c r="D312" s="0">
-        <v>239580</v>
+        <v>23958</v>
       </c>
     </row>
     <row r="313">
@@ -7607,10 +7613,10 @@
         <v>680</v>
       </c>
       <c r="C313" s="0" t="s">
-        <v>51</v>
+        <v>89</v>
       </c>
       <c r="D313" s="0">
-        <v>130</v>
+        <v>239580</v>
       </c>
     </row>
     <row r="314">
@@ -7621,10 +7627,10 @@
         <v>682</v>
       </c>
       <c r="C314" s="0" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="D314" s="0">
-        <v>285.6</v>
+        <v>130</v>
       </c>
     </row>
     <row r="315">
@@ -7638,7 +7644,7 @@
         <v>22</v>
       </c>
       <c r="D315" s="0">
-        <v>338</v>
+        <v>285.6</v>
       </c>
     </row>
     <row r="316">
@@ -7649,21 +7655,21 @@
         <v>686</v>
       </c>
       <c r="C316" s="0" t="s">
-        <v>687</v>
+        <v>22</v>
       </c>
       <c r="D316" s="0">
-        <v>770</v>
+        <v>338</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="0" t="s">
+        <v>687</v>
+      </c>
+      <c r="B317" s="0" t="s">
         <v>688</v>
       </c>
-      <c r="B317" s="0" t="s">
+      <c r="C317" s="0" t="s">
         <v>689</v>
-      </c>
-      <c r="C317" s="0" t="s">
-        <v>690</v>
       </c>
       <c r="D317" s="0">
         <v>770</v>
@@ -7671,16 +7677,16 @@
     </row>
     <row r="318">
       <c r="A318" s="0" t="s">
+        <v>690</v>
+      </c>
+      <c r="B318" s="0" t="s">
         <v>691</v>
       </c>
-      <c r="B318" s="0" t="s">
+      <c r="C318" s="0" t="s">
         <v>692</v>
       </c>
-      <c r="C318" s="0" t="s">
-        <v>16</v>
-      </c>
       <c r="D318" s="0">
-        <v>973.5</v>
+        <v>770</v>
       </c>
     </row>
     <row r="319">
@@ -7691,10 +7697,10 @@
         <v>694</v>
       </c>
       <c r="C319" s="0" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D319" s="0">
-        <v>507.08</v>
+        <v>973.5</v>
       </c>
     </row>
     <row r="320">
@@ -7705,10 +7711,10 @@
         <v>696</v>
       </c>
       <c r="C320" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D320" s="0">
-        <v>450</v>
+        <v>507.08</v>
       </c>
     </row>
     <row r="321">
@@ -7719,10 +7725,10 @@
         <v>698</v>
       </c>
       <c r="C321" s="0" t="s">
-        <v>143</v>
+        <v>16</v>
       </c>
       <c r="D321" s="0">
-        <v>760</v>
+        <v>450</v>
       </c>
     </row>
     <row r="322">
@@ -7733,10 +7739,10 @@
         <v>700</v>
       </c>
       <c r="C322" s="0" t="s">
-        <v>279</v>
+        <v>143</v>
       </c>
       <c r="D322" s="0">
-        <v>5900</v>
+        <v>760</v>
       </c>
     </row>
     <row r="323">
@@ -7750,7 +7756,7 @@
         <v>279</v>
       </c>
       <c r="D323" s="0">
-        <v>2900</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="324">
@@ -7761,10 +7767,10 @@
         <v>704</v>
       </c>
       <c r="C324" s="0" t="s">
-        <v>132</v>
+        <v>279</v>
       </c>
       <c r="D324" s="0">
-        <v>886.2</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="325">
@@ -7778,7 +7784,7 @@
         <v>132</v>
       </c>
       <c r="D325" s="0">
-        <v>589.9</v>
+        <v>886.2</v>
       </c>
     </row>
     <row r="326">
@@ -7792,7 +7798,7 @@
         <v>132</v>
       </c>
       <c r="D326" s="0">
-        <v>65</v>
+        <v>589.9</v>
       </c>
     </row>
     <row r="327">
@@ -7803,10 +7809,10 @@
         <v>710</v>
       </c>
       <c r="C327" s="0" t="s">
-        <v>89</v>
+        <v>132</v>
       </c>
       <c r="D327" s="0">
-        <v>11313.5</v>
+        <v>65</v>
       </c>
     </row>
     <row r="328">
@@ -7817,10 +7823,10 @@
         <v>712</v>
       </c>
       <c r="C328" s="0" t="s">
-        <v>35</v>
+        <v>89</v>
       </c>
       <c r="D328" s="0">
-        <v>418</v>
+        <v>11313.5</v>
       </c>
     </row>
     <row r="329">
@@ -7831,7 +7837,7 @@
         <v>714</v>
       </c>
       <c r="C329" s="0" t="s">
-        <v>355</v>
+        <v>35</v>
       </c>
       <c r="D329" s="0">
         <v>418</v>
@@ -7845,10 +7851,10 @@
         <v>716</v>
       </c>
       <c r="C330" s="0" t="s">
-        <v>22</v>
+        <v>355</v>
       </c>
       <c r="D330" s="0">
-        <v>377</v>
+        <v>418</v>
       </c>
     </row>
     <row r="331">
@@ -7859,10 +7865,10 @@
         <v>718</v>
       </c>
       <c r="C331" s="0" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="D331" s="0">
-        <v>5300</v>
+        <v>377</v>
       </c>
     </row>
     <row r="332">
@@ -7873,10 +7879,10 @@
         <v>720</v>
       </c>
       <c r="C332" s="0" t="s">
-        <v>69</v>
+        <v>44</v>
       </c>
       <c r="D332" s="0">
-        <v>898</v>
+        <v>5300</v>
       </c>
     </row>
     <row r="333">
@@ -7887,10 +7893,10 @@
         <v>722</v>
       </c>
       <c r="C333" s="0" t="s">
-        <v>115</v>
+        <v>69</v>
       </c>
       <c r="D333" s="0">
-        <v>4767</v>
+        <v>898</v>
       </c>
     </row>
     <row r="334">
@@ -7901,10 +7907,10 @@
         <v>724</v>
       </c>
       <c r="C334" s="0" t="s">
-        <v>35</v>
+        <v>115</v>
       </c>
       <c r="D334" s="0">
-        <v>650</v>
+        <v>4767</v>
       </c>
     </row>
     <row r="335">
@@ -7915,7 +7921,7 @@
         <v>726</v>
       </c>
       <c r="C335" s="0" t="s">
-        <v>69</v>
+        <v>35</v>
       </c>
       <c r="D335" s="0">
         <v>650</v>
@@ -7929,10 +7935,10 @@
         <v>728</v>
       </c>
       <c r="C336" s="0" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="D336" s="0">
-        <v>2178</v>
+        <v>650</v>
       </c>
     </row>
     <row r="337">
@@ -7943,10 +7949,10 @@
         <v>730</v>
       </c>
       <c r="C337" s="0" t="s">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="D337" s="0">
-        <v>7986</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="338">
@@ -7957,24 +7963,24 @@
         <v>732</v>
       </c>
       <c r="C338" s="0" t="s">
-        <v>733</v>
+        <v>89</v>
       </c>
       <c r="D338" s="0">
-        <v>1800</v>
+        <v>7986</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="0" t="s">
+        <v>733</v>
+      </c>
+      <c r="B339" s="0" t="s">
         <v>734</v>
       </c>
-      <c r="B339" s="0" t="s">
+      <c r="C339" s="0" t="s">
         <v>735</v>
       </c>
-      <c r="C339" s="0" t="s">
-        <v>143</v>
-      </c>
       <c r="D339" s="0">
-        <v>900</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="340">
@@ -7985,10 +7991,10 @@
         <v>737</v>
       </c>
       <c r="C340" s="0" t="s">
-        <v>22</v>
+        <v>143</v>
       </c>
       <c r="D340" s="0">
-        <v>1722</v>
+        <v>900</v>
       </c>
     </row>
     <row r="341">
@@ -7999,10 +8005,10 @@
         <v>739</v>
       </c>
       <c r="C341" s="0" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="D341" s="0">
-        <v>456</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="342">
@@ -8016,7 +8022,7 @@
         <v>35</v>
       </c>
       <c r="D342" s="0">
-        <v>45600</v>
+        <v>456</v>
       </c>
     </row>
     <row r="343">
@@ -8027,10 +8033,10 @@
         <v>743</v>
       </c>
       <c r="C343" s="0" t="s">
-        <v>143</v>
+        <v>35</v>
       </c>
       <c r="D343" s="0">
-        <v>750</v>
+        <v>45600</v>
       </c>
     </row>
     <row r="344">
@@ -8044,7 +8050,7 @@
         <v>143</v>
       </c>
       <c r="D344" s="0">
-        <v>1212</v>
+        <v>750</v>
       </c>
     </row>
     <row r="345">
@@ -8058,7 +8064,7 @@
         <v>143</v>
       </c>
       <c r="D345" s="0">
-        <v>1300</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="346">
@@ -8072,7 +8078,7 @@
         <v>143</v>
       </c>
       <c r="D346" s="0">
-        <v>1500</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="347">
@@ -8086,7 +8092,7 @@
         <v>143</v>
       </c>
       <c r="D347" s="0">
-        <v>1400</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="348">
@@ -8097,10 +8103,10 @@
         <v>753</v>
       </c>
       <c r="C348" s="0" t="s">
-        <v>255</v>
+        <v>143</v>
       </c>
       <c r="D348" s="0">
-        <v>11959</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="349">
@@ -8111,10 +8117,10 @@
         <v>755</v>
       </c>
       <c r="C349" s="0" t="s">
-        <v>132</v>
+        <v>255</v>
       </c>
       <c r="D349" s="0">
-        <v>345</v>
+        <v>11959</v>
       </c>
     </row>
     <row r="350">
@@ -8125,10 +8131,10 @@
         <v>757</v>
       </c>
       <c r="C350" s="0" t="s">
-        <v>279</v>
+        <v>132</v>
       </c>
       <c r="D350" s="0">
-        <v>1450</v>
+        <v>345</v>
       </c>
     </row>
     <row r="351">
@@ -8139,10 +8145,10 @@
         <v>759</v>
       </c>
       <c r="C351" s="0" t="s">
-        <v>89</v>
+        <v>279</v>
       </c>
       <c r="D351" s="0">
-        <v>7320.5</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="352">
@@ -8153,10 +8159,10 @@
         <v>761</v>
       </c>
       <c r="C352" s="0" t="s">
-        <v>16</v>
+        <v>89</v>
       </c>
       <c r="D352" s="0">
-        <v>900</v>
+        <v>7320.5</v>
       </c>
     </row>
     <row r="353">
@@ -8167,10 +8173,10 @@
         <v>763</v>
       </c>
       <c r="C353" s="0" t="s">
-        <v>279</v>
+        <v>16</v>
       </c>
       <c r="D353" s="0">
-        <v>520</v>
+        <v>900</v>
       </c>
     </row>
     <row r="354">
@@ -8181,10 +8187,10 @@
         <v>765</v>
       </c>
       <c r="C354" s="0" t="s">
-        <v>471</v>
+        <v>279</v>
       </c>
       <c r="D354" s="0">
-        <v>64925</v>
+        <v>520</v>
       </c>
     </row>
     <row r="355">
@@ -8195,10 +8201,10 @@
         <v>767</v>
       </c>
       <c r="C355" s="0" t="s">
-        <v>16</v>
+        <v>471</v>
       </c>
       <c r="D355" s="0">
-        <v>1100</v>
+        <v>64925</v>
       </c>
     </row>
     <row r="356">
@@ -8209,10 +8215,10 @@
         <v>769</v>
       </c>
       <c r="C356" s="0" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D356" s="0">
-        <v>1623</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="357">
@@ -8223,10 +8229,10 @@
         <v>771</v>
       </c>
       <c r="C357" s="0" t="s">
-        <v>132</v>
+        <v>22</v>
       </c>
       <c r="D357" s="0">
-        <v>1182.75</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="358">
@@ -8240,7 +8246,7 @@
         <v>132</v>
       </c>
       <c r="D358" s="0">
-        <v>4440.9</v>
+        <v>1182.75</v>
       </c>
     </row>
     <row r="359">
@@ -8251,10 +8257,10 @@
         <v>775</v>
       </c>
       <c r="C359" s="0" t="s">
-        <v>29</v>
+        <v>132</v>
       </c>
       <c r="D359" s="0">
-        <v>1650</v>
+        <v>4440.9</v>
       </c>
     </row>
     <row r="360">
@@ -8268,7 +8274,7 @@
         <v>29</v>
       </c>
       <c r="D360" s="0">
-        <v>1908.8</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="361">
@@ -8279,10 +8285,10 @@
         <v>779</v>
       </c>
       <c r="C361" s="0" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="D361" s="0">
-        <v>450</v>
+        <v>1908.8</v>
       </c>
     </row>
     <row r="362">
@@ -8296,7 +8302,7 @@
         <v>16</v>
       </c>
       <c r="D362" s="0">
-        <v>825</v>
+        <v>450</v>
       </c>
     </row>
     <row r="363">
@@ -8321,10 +8327,10 @@
         <v>785</v>
       </c>
       <c r="C364" s="0" t="s">
-        <v>373</v>
+        <v>16</v>
       </c>
       <c r="D364" s="0">
-        <v>134775.6</v>
+        <v>825</v>
       </c>
     </row>
     <row r="365">
@@ -8338,7 +8344,7 @@
         <v>373</v>
       </c>
       <c r="D365" s="0">
-        <v>175991.55</v>
+        <v>134775.6</v>
       </c>
     </row>
     <row r="366">
@@ -8349,10 +8355,10 @@
         <v>789</v>
       </c>
       <c r="C366" s="0" t="s">
-        <v>69</v>
+        <v>373</v>
       </c>
       <c r="D366" s="0">
-        <v>3263</v>
+        <v>175991.55</v>
       </c>
     </row>
     <row r="367">
@@ -8366,7 +8372,7 @@
         <v>69</v>
       </c>
       <c r="D367" s="0">
-        <v>18027</v>
+        <v>3263</v>
       </c>
     </row>
     <row r="368">
@@ -8377,10 +8383,10 @@
         <v>793</v>
       </c>
       <c r="C368" s="0" t="s">
-        <v>279</v>
+        <v>69</v>
       </c>
       <c r="D368" s="0">
-        <v>515</v>
+        <v>18027</v>
       </c>
     </row>
     <row r="369">
@@ -8391,38 +8397,38 @@
         <v>795</v>
       </c>
       <c r="C369" s="0" t="s">
-        <v>38</v>
+        <v>279</v>
       </c>
       <c r="D369" s="0">
         <v>515</v>
       </c>
     </row>
     <row r="370">
-      <c r="A370" s="2" t="s">
+      <c r="A370" s="0" t="s">
         <v>796</v>
       </c>
-      <c r="B370" s="2" t="s">
+      <c r="B370" s="0" t="s">
         <v>797</v>
       </c>
-      <c r="C370" s="2" t="s">
+      <c r="C370" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="D370" s="0">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="2" t="s">
+        <v>798</v>
+      </c>
+      <c r="B371" s="2" t="s">
+        <v>799</v>
+      </c>
+      <c r="C371" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D370" s="2">
+      <c r="D371" s="2">
         <v>10154</v>
-      </c>
-    </row>
-    <row r="371">
-      <c r="A371" s="0" t="s">
-        <v>798</v>
-      </c>
-      <c r="B371" s="0" t="s">
-        <v>799</v>
-      </c>
-      <c r="C371" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="D371" s="0">
-        <v>9500</v>
       </c>
     </row>
     <row r="372">
@@ -8433,10 +8439,10 @@
         <v>801</v>
       </c>
       <c r="C372" s="0" t="s">
-        <v>471</v>
+        <v>51</v>
       </c>
       <c r="D372" s="0">
-        <v>207558.08</v>
+        <v>9500</v>
       </c>
     </row>
     <row r="373">
@@ -8450,7 +8456,7 @@
         <v>471</v>
       </c>
       <c r="D373" s="0">
-        <v>249069.69</v>
+        <v>207558.08</v>
       </c>
     </row>
     <row r="374">
@@ -8461,10 +8467,10 @@
         <v>805</v>
       </c>
       <c r="C374" s="0" t="s">
-        <v>69</v>
+        <v>471</v>
       </c>
       <c r="D374" s="0">
-        <v>10021.22</v>
+        <v>249069.69</v>
       </c>
     </row>
     <row r="375">
@@ -8478,7 +8484,7 @@
         <v>69</v>
       </c>
       <c r="D375" s="0">
-        <v>17710</v>
+        <v>10021.22</v>
       </c>
     </row>
     <row r="376">
@@ -8489,24 +8495,24 @@
         <v>809</v>
       </c>
       <c r="C376" s="0" t="s">
-        <v>810</v>
+        <v>69</v>
       </c>
       <c r="D376" s="0">
-        <v>1080</v>
+        <v>17710</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="0" t="s">
+        <v>810</v>
+      </c>
+      <c r="B377" s="0" t="s">
         <v>811</v>
       </c>
-      <c r="B377" s="0" t="s">
+      <c r="C377" s="0" t="s">
         <v>812</v>
       </c>
-      <c r="C377" s="0" t="s">
-        <v>19</v>
-      </c>
       <c r="D377" s="0">
-        <v>691.03</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="378">
@@ -8517,24 +8523,24 @@
         <v>814</v>
       </c>
       <c r="C378" s="0" t="s">
-        <v>815</v>
+        <v>19</v>
       </c>
       <c r="D378" s="0">
-        <v>520</v>
+        <v>691.03</v>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="0" t="s">
+        <v>815</v>
+      </c>
+      <c r="B379" s="0" t="s">
         <v>816</v>
       </c>
-      <c r="B379" s="0" t="s">
+      <c r="C379" s="0" t="s">
         <v>817</v>
       </c>
-      <c r="C379" s="0" t="s">
-        <v>815</v>
-      </c>
       <c r="D379" s="0">
-        <v>300</v>
+        <v>520</v>
       </c>
     </row>
     <row r="380">
@@ -8545,10 +8551,10 @@
         <v>819</v>
       </c>
       <c r="C380" s="0" t="s">
-        <v>16</v>
+        <v>817</v>
       </c>
       <c r="D380" s="0">
-        <v>2200</v>
+        <v>300</v>
       </c>
     </row>
     <row r="381">
@@ -8562,7 +8568,7 @@
         <v>16</v>
       </c>
       <c r="D381" s="0">
-        <v>2800</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="382">
@@ -8573,10 +8579,10 @@
         <v>823</v>
       </c>
       <c r="C382" s="0" t="s">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="D382" s="0">
-        <v>4791.6</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="383">
@@ -8587,10 +8593,10 @@
         <v>825</v>
       </c>
       <c r="C383" s="0" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="D383" s="0">
-        <v>2699.64</v>
+        <v>4791.6</v>
       </c>
     </row>
     <row r="384">
@@ -8601,10 +8607,10 @@
         <v>827</v>
       </c>
       <c r="C384" s="0" t="s">
-        <v>35</v>
+        <v>69</v>
       </c>
       <c r="D384" s="0">
-        <v>3800</v>
+        <v>2699.64</v>
       </c>
     </row>
     <row r="385">
@@ -8615,10 +8621,10 @@
         <v>829</v>
       </c>
       <c r="C385" s="0" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D385" s="0">
-        <v>4000</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="386">
@@ -8629,24 +8635,24 @@
         <v>831</v>
       </c>
       <c r="C386" s="0" t="s">
-        <v>832</v>
+        <v>16</v>
       </c>
       <c r="D386" s="0">
-        <v>3800</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="387">
       <c r="A387" s="0" t="s">
+        <v>832</v>
+      </c>
+      <c r="B387" s="0" t="s">
         <v>833</v>
       </c>
-      <c r="B387" s="0" t="s">
+      <c r="C387" s="0" t="s">
         <v>834</v>
       </c>
-      <c r="C387" s="0" t="s">
-        <v>22</v>
-      </c>
       <c r="D387" s="0">
-        <v>353</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="388">
@@ -8657,10 +8663,10 @@
         <v>836</v>
       </c>
       <c r="C388" s="0" t="s">
-        <v>207</v>
+        <v>22</v>
       </c>
       <c r="D388" s="0">
-        <v>1800</v>
+        <v>353</v>
       </c>
     </row>
     <row r="389">
@@ -8671,10 +8677,10 @@
         <v>838</v>
       </c>
       <c r="C389" s="0" t="s">
-        <v>16</v>
+        <v>207</v>
       </c>
       <c r="D389" s="0">
-        <v>2948</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="390">
@@ -8685,10 +8691,10 @@
         <v>840</v>
       </c>
       <c r="C390" s="0" t="s">
-        <v>202</v>
+        <v>16</v>
       </c>
       <c r="D390" s="0">
-        <v>65537</v>
+        <v>2948</v>
       </c>
     </row>
     <row r="391">
@@ -8699,10 +8705,10 @@
         <v>842</v>
       </c>
       <c r="C391" s="0" t="s">
-        <v>132</v>
+        <v>202</v>
       </c>
       <c r="D391" s="0">
-        <v>4049.6</v>
+        <v>65537</v>
       </c>
     </row>
     <row r="392">
@@ -8716,7 +8722,7 @@
         <v>132</v>
       </c>
       <c r="D392" s="0">
-        <v>4199.2</v>
+        <v>4049.6</v>
       </c>
     </row>
     <row r="393">
@@ -8730,7 +8736,7 @@
         <v>132</v>
       </c>
       <c r="D393" s="0">
-        <v>6397.2</v>
+        <v>4199.2</v>
       </c>
     </row>
     <row r="394">
@@ -8741,10 +8747,10 @@
         <v>848</v>
       </c>
       <c r="C394" s="0" t="s">
-        <v>306</v>
+        <v>132</v>
       </c>
       <c r="D394" s="0">
-        <v>570</v>
+        <v>6397.2</v>
       </c>
     </row>
     <row r="395">
@@ -8755,10 +8761,10 @@
         <v>850</v>
       </c>
       <c r="C395" s="0" t="s">
-        <v>69</v>
+        <v>306</v>
       </c>
       <c r="D395" s="0">
-        <v>550</v>
+        <v>570</v>
       </c>
     </row>
     <row r="396">
@@ -8769,10 +8775,10 @@
         <v>852</v>
       </c>
       <c r="C396" s="0" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="D396" s="0">
-        <v>167</v>
+        <v>550</v>
       </c>
     </row>
     <row r="397">
@@ -8783,10 +8789,10 @@
         <v>854</v>
       </c>
       <c r="C397" s="0" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="D397" s="0">
-        <v>701.42</v>
+        <v>167</v>
       </c>
     </row>
     <row r="398">
@@ -8797,10 +8803,10 @@
         <v>856</v>
       </c>
       <c r="C398" s="0" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="D398" s="0">
-        <v>101000</v>
+        <v>701.42</v>
       </c>
     </row>
     <row r="399">
@@ -8811,10 +8817,10 @@
         <v>858</v>
       </c>
       <c r="C399" s="0" t="s">
-        <v>115</v>
+        <v>58</v>
       </c>
       <c r="D399" s="0">
-        <v>6251</v>
+        <v>101000</v>
       </c>
     </row>
     <row r="400">
@@ -8825,10 +8831,10 @@
         <v>860</v>
       </c>
       <c r="C400" s="0" t="s">
-        <v>370</v>
+        <v>115</v>
       </c>
       <c r="D400" s="0">
-        <v>857.67</v>
+        <v>6251</v>
       </c>
     </row>
     <row r="401">
@@ -8839,10 +8845,10 @@
         <v>862</v>
       </c>
       <c r="C401" s="0" t="s">
-        <v>89</v>
+        <v>370</v>
       </c>
       <c r="D401" s="0">
-        <v>1164.66</v>
+        <v>857.67</v>
       </c>
     </row>
     <row r="402">
@@ -8853,10 +8859,10 @@
         <v>864</v>
       </c>
       <c r="C402" s="0" t="s">
-        <v>143</v>
+        <v>89</v>
       </c>
       <c r="D402" s="0">
-        <v>360</v>
+        <v>1164.66</v>
       </c>
     </row>
     <row r="403">
@@ -8870,7 +8876,7 @@
         <v>143</v>
       </c>
       <c r="D403" s="0">
-        <v>450</v>
+        <v>360</v>
       </c>
     </row>
     <row r="404">
@@ -8884,7 +8890,7 @@
         <v>143</v>
       </c>
       <c r="D404" s="0">
-        <v>2050</v>
+        <v>450</v>
       </c>
     </row>
     <row r="405">
@@ -8895,10 +8901,10 @@
         <v>870</v>
       </c>
       <c r="C405" s="0" t="s">
-        <v>572</v>
+        <v>143</v>
       </c>
       <c r="D405" s="0">
-        <v>25192.82</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="406">
@@ -8909,10 +8915,10 @@
         <v>872</v>
       </c>
       <c r="C406" s="0" t="s">
-        <v>69</v>
+        <v>574</v>
       </c>
       <c r="D406" s="0">
-        <v>3500</v>
+        <v>25192.82</v>
       </c>
     </row>
     <row r="407">
@@ -8923,10 +8929,10 @@
         <v>874</v>
       </c>
       <c r="C407" s="0" t="s">
-        <v>170</v>
+        <v>69</v>
       </c>
       <c r="D407" s="0">
-        <v>600</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="408">
@@ -8937,52 +8943,52 @@
         <v>876</v>
       </c>
       <c r="C408" s="0" t="s">
-        <v>877</v>
+        <v>170</v>
       </c>
       <c r="D408" s="0">
-        <v>1080</v>
+        <v>600</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="0" t="s">
+        <v>877</v>
+      </c>
+      <c r="B409" s="0" t="s">
         <v>878</v>
       </c>
-      <c r="B409" s="0" t="s">
+      <c r="C409" s="0" t="s">
         <v>879</v>
       </c>
-      <c r="C409" s="0" t="s">
+      <c r="D409" s="0">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="0" t="s">
+        <v>880</v>
+      </c>
+      <c r="B410" s="0" t="s">
+        <v>881</v>
+      </c>
+      <c r="C410" s="0" t="s">
         <v>334</v>
       </c>
-      <c r="D409" s="0">
+      <c r="D410" s="0">
         <v>8628</v>
       </c>
     </row>
-    <row r="410">
-      <c r="A410" s="2" t="s">
-        <v>880</v>
-      </c>
-      <c r="B410" s="2" t="s">
-        <v>881</v>
-      </c>
-      <c r="C410" s="2" t="s">
+    <row r="411">
+      <c r="A411" s="2" t="s">
+        <v>882</v>
+      </c>
+      <c r="B411" s="2" t="s">
+        <v>883</v>
+      </c>
+      <c r="C411" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="D410" s="2">
+      <c r="D411" s="2">
         <v>9125.1</v>
-      </c>
-    </row>
-    <row r="411">
-      <c r="A411" s="0" t="s">
-        <v>882</v>
-      </c>
-      <c r="B411" s="0" t="s">
-        <v>883</v>
-      </c>
-      <c r="C411" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="D411" s="0">
-        <v>27991.54</v>
       </c>
     </row>
     <row r="412">
@@ -8993,10 +8999,10 @@
         <v>885</v>
       </c>
       <c r="C412" s="0" t="s">
-        <v>132</v>
+        <v>41</v>
       </c>
       <c r="D412" s="0">
-        <v>1080</v>
+        <v>27991.54</v>
       </c>
     </row>
     <row r="413">
@@ -9010,7 +9016,7 @@
         <v>132</v>
       </c>
       <c r="D413" s="0">
-        <v>4012</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="414">
@@ -9021,10 +9027,10 @@
         <v>889</v>
       </c>
       <c r="C414" s="0" t="s">
-        <v>44</v>
+        <v>132</v>
       </c>
       <c r="D414" s="0">
-        <v>5816.9</v>
+        <v>4012</v>
       </c>
     </row>
     <row r="415">
@@ -9038,7 +9044,7 @@
         <v>44</v>
       </c>
       <c r="D415" s="0">
-        <v>2624.28</v>
+        <v>5816.9</v>
       </c>
     </row>
     <row r="416">
@@ -9052,35 +9058,35 @@
         <v>44</v>
       </c>
       <c r="D416" s="0">
+        <v>2624.28</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="0" t="s">
+        <v>894</v>
+      </c>
+      <c r="B417" s="0" t="s">
+        <v>895</v>
+      </c>
+      <c r="C417" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="D417" s="0">
         <v>1953.98</v>
       </c>
     </row>
-    <row r="417">
-      <c r="A417" s="2" t="s">
-        <v>894</v>
-      </c>
-      <c r="B417" s="2" t="s">
-        <v>895</v>
-      </c>
-      <c r="C417" s="2" t="s">
+    <row r="418">
+      <c r="A418" s="2" t="s">
+        <v>896</v>
+      </c>
+      <c r="B418" s="2" t="s">
+        <v>897</v>
+      </c>
+      <c r="C418" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D417" s="2">
+      <c r="D418" s="2">
         <v>3598.96</v>
-      </c>
-    </row>
-    <row r="418">
-      <c r="A418" s="0" t="s">
-        <v>896</v>
-      </c>
-      <c r="B418" s="0" t="s">
-        <v>897</v>
-      </c>
-      <c r="C418" s="0" t="s">
-        <v>44</v>
-      </c>
-      <c r="D418" s="0">
-        <v>27318.17</v>
       </c>
     </row>
     <row r="419">
@@ -9094,7 +9100,7 @@
         <v>44</v>
       </c>
       <c r="D419" s="0">
-        <v>2115.26</v>
+        <v>27318.17</v>
       </c>
     </row>
     <row r="420">
@@ -9108,7 +9114,7 @@
         <v>44</v>
       </c>
       <c r="D420" s="0">
-        <v>4700</v>
+        <v>2115.26</v>
       </c>
     </row>
     <row r="421">
@@ -9122,7 +9128,7 @@
         <v>44</v>
       </c>
       <c r="D421" s="0">
-        <v>3750</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="422">
@@ -9133,10 +9139,10 @@
         <v>905</v>
       </c>
       <c r="C422" s="0" t="s">
-        <v>480</v>
+        <v>44</v>
       </c>
       <c r="D422" s="0">
-        <v>510</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="423">
@@ -9147,7 +9153,7 @@
         <v>907</v>
       </c>
       <c r="C423" s="0" t="s">
-        <v>38</v>
+        <v>480</v>
       </c>
       <c r="D423" s="0">
         <v>510</v>
@@ -9161,21 +9167,21 @@
         <v>909</v>
       </c>
       <c r="C424" s="0" t="s">
-        <v>910</v>
+        <v>38</v>
       </c>
       <c r="D424" s="0">
-        <v>580</v>
+        <v>510</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="0" t="s">
+        <v>910</v>
+      </c>
+      <c r="B425" s="0" t="s">
         <v>911</v>
       </c>
-      <c r="B425" s="0" t="s">
+      <c r="C425" s="0" t="s">
         <v>912</v>
-      </c>
-      <c r="C425" s="0" t="s">
-        <v>910</v>
       </c>
       <c r="D425" s="0">
         <v>580</v>
@@ -9189,7 +9195,7 @@
         <v>914</v>
       </c>
       <c r="C426" s="0" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
       <c r="D426" s="0">
         <v>580</v>
@@ -9203,10 +9209,10 @@
         <v>916</v>
       </c>
       <c r="C427" s="0" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
       <c r="D427" s="0">
-        <v>342</v>
+        <v>580</v>
       </c>
     </row>
     <row r="428">
@@ -9217,7 +9223,7 @@
         <v>918</v>
       </c>
       <c r="C428" s="0" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
       <c r="D428" s="0">
         <v>342</v>
@@ -9231,7 +9237,7 @@
         <v>920</v>
       </c>
       <c r="C429" s="0" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
       <c r="D429" s="0">
         <v>342</v>
@@ -9245,10 +9251,10 @@
         <v>922</v>
       </c>
       <c r="C430" s="0" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
       <c r="D430" s="0">
-        <v>0</v>
+        <v>342</v>
       </c>
     </row>
     <row r="431">
@@ -9259,7 +9265,7 @@
         <v>924</v>
       </c>
       <c r="C431" s="0" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
       <c r="D431" s="0">
         <v>0</v>
@@ -9273,10 +9279,10 @@
         <v>926</v>
       </c>
       <c r="C432" s="0" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
       <c r="D432" s="0">
-        <v>423</v>
+        <v>0</v>
       </c>
     </row>
     <row r="433">
@@ -9287,10 +9293,10 @@
         <v>928</v>
       </c>
       <c r="C433" s="0" t="s">
-        <v>69</v>
+        <v>912</v>
       </c>
       <c r="D433" s="0">
-        <v>15968</v>
+        <v>423</v>
       </c>
     </row>
     <row r="434">
@@ -9301,10 +9307,10 @@
         <v>930</v>
       </c>
       <c r="C434" s="0" t="s">
-        <v>109</v>
+        <v>69</v>
       </c>
       <c r="D434" s="0">
-        <v>14000</v>
+        <v>15968</v>
       </c>
     </row>
     <row r="435">
@@ -9315,10 +9321,10 @@
         <v>932</v>
       </c>
       <c r="C435" s="0" t="s">
-        <v>132</v>
+        <v>109</v>
       </c>
       <c r="D435" s="0">
-        <v>14001</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="436">
@@ -9329,10 +9335,10 @@
         <v>934</v>
       </c>
       <c r="C436" s="0" t="s">
-        <v>89</v>
+        <v>132</v>
       </c>
       <c r="D436" s="0">
-        <v>266200</v>
+        <v>14001</v>
       </c>
     </row>
     <row r="437">
@@ -9346,7 +9352,7 @@
         <v>89</v>
       </c>
       <c r="D437" s="0">
-        <v>194991.5</v>
+        <v>266200</v>
       </c>
     </row>
     <row r="438">
@@ -9360,7 +9366,7 @@
         <v>89</v>
       </c>
       <c r="D438" s="0">
-        <v>289492.5</v>
+        <v>194991.5</v>
       </c>
     </row>
     <row r="439">
@@ -9371,24 +9377,24 @@
         <v>940</v>
       </c>
       <c r="C439" s="0" t="s">
-        <v>941</v>
+        <v>89</v>
       </c>
       <c r="D439" s="0">
-        <v>13722.52</v>
+        <v>289492.5</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="0" t="s">
+        <v>941</v>
+      </c>
+      <c r="B440" s="0" t="s">
         <v>942</v>
       </c>
-      <c r="B440" s="0" t="s">
+      <c r="C440" s="0" t="s">
         <v>943</v>
       </c>
-      <c r="C440" s="0" t="s">
-        <v>941</v>
-      </c>
       <c r="D440" s="0">
-        <v>15072</v>
+        <v>13722.52</v>
       </c>
     </row>
     <row r="441">
@@ -9399,10 +9405,10 @@
         <v>945</v>
       </c>
       <c r="C441" s="0" t="s">
-        <v>941</v>
+        <v>943</v>
       </c>
       <c r="D441" s="0">
-        <v>6555.64</v>
+        <v>15072</v>
       </c>
     </row>
     <row r="442">
@@ -9413,10 +9419,10 @@
         <v>947</v>
       </c>
       <c r="C442" s="0" t="s">
-        <v>941</v>
+        <v>943</v>
       </c>
       <c r="D442" s="0">
-        <v>8964.61</v>
+        <v>6555.64</v>
       </c>
     </row>
     <row r="443">
@@ -9427,10 +9433,10 @@
         <v>949</v>
       </c>
       <c r="C443" s="0" t="s">
-        <v>941</v>
+        <v>943</v>
       </c>
       <c r="D443" s="0">
-        <v>11735</v>
+        <v>8964.61</v>
       </c>
     </row>
     <row r="444">
@@ -9441,10 +9447,10 @@
         <v>951</v>
       </c>
       <c r="C444" s="0" t="s">
-        <v>69</v>
+        <v>943</v>
       </c>
       <c r="D444" s="0">
-        <v>3380</v>
+        <v>11735</v>
       </c>
     </row>
     <row r="445">
@@ -9455,10 +9461,10 @@
         <v>953</v>
       </c>
       <c r="C445" s="0" t="s">
-        <v>132</v>
+        <v>69</v>
       </c>
       <c r="D445" s="0">
-        <v>3750</v>
+        <v>3380</v>
       </c>
     </row>
     <row r="446">
@@ -9469,10 +9475,10 @@
         <v>955</v>
       </c>
       <c r="C446" s="0" t="s">
-        <v>89</v>
+        <v>132</v>
       </c>
       <c r="D446" s="0">
-        <v>4392.3</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="447">
@@ -9483,24 +9489,24 @@
         <v>957</v>
       </c>
       <c r="C447" s="0" t="s">
-        <v>958</v>
+        <v>89</v>
       </c>
       <c r="D447" s="0">
-        <v>5254.41</v>
+        <v>4392.3</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="0" t="s">
+        <v>958</v>
+      </c>
+      <c r="B448" s="0" t="s">
         <v>959</v>
       </c>
-      <c r="B448" s="0" t="s">
+      <c r="C448" s="0" t="s">
         <v>960</v>
       </c>
-      <c r="C448" s="0" t="s">
-        <v>51</v>
-      </c>
       <c r="D448" s="0">
-        <v>1200</v>
+        <v>5254.41</v>
       </c>
     </row>
     <row r="449">
@@ -9514,7 +9520,7 @@
         <v>51</v>
       </c>
       <c r="D449" s="0">
-        <v>278</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="450">
@@ -9528,7 +9534,7 @@
         <v>51</v>
       </c>
       <c r="D450" s="0">
-        <v>562</v>
+        <v>278</v>
       </c>
     </row>
     <row r="451">
@@ -9539,10 +9545,10 @@
         <v>966</v>
       </c>
       <c r="C451" s="0" t="s">
-        <v>370</v>
+        <v>51</v>
       </c>
       <c r="D451" s="0">
-        <v>65142.6</v>
+        <v>562</v>
       </c>
     </row>
     <row r="452">
@@ -9556,7 +9562,7 @@
         <v>370</v>
       </c>
       <c r="D452" s="0">
-        <v>23482.7</v>
+        <v>65142.6</v>
       </c>
     </row>
     <row r="453">
@@ -9567,10 +9573,10 @@
         <v>970</v>
       </c>
       <c r="C453" s="0" t="s">
-        <v>29</v>
+        <v>370</v>
       </c>
       <c r="D453" s="0">
-        <v>5917.17</v>
+        <v>23482.7</v>
       </c>
     </row>
     <row r="454">
@@ -9581,10 +9587,10 @@
         <v>972</v>
       </c>
       <c r="C454" s="0" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="D454" s="0">
-        <v>10985</v>
+        <v>5917.17</v>
       </c>
     </row>
     <row r="455">
@@ -9598,7 +9604,7 @@
         <v>51</v>
       </c>
       <c r="D455" s="0">
-        <v>17425</v>
+        <v>10985</v>
       </c>
     </row>
     <row r="456">
@@ -9609,38 +9615,38 @@
         <v>976</v>
       </c>
       <c r="C456" s="0" t="s">
-        <v>977</v>
+        <v>51</v>
       </c>
       <c r="D456" s="0">
-        <v>1958</v>
+        <v>17425</v>
       </c>
     </row>
     <row r="457">
       <c r="A457" s="0" t="s">
+        <v>977</v>
+      </c>
+      <c r="B457" s="0" t="s">
         <v>978</v>
       </c>
-      <c r="B457" s="0" t="s">
+      <c r="C457" s="0" t="s">
         <v>979</v>
       </c>
-      <c r="C457" s="0" t="s">
-        <v>980</v>
-      </c>
       <c r="D457" s="0">
-        <v>385.4</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="0" t="s">
+        <v>980</v>
+      </c>
+      <c r="B458" s="0" t="s">
         <v>981</v>
       </c>
-      <c r="B458" s="0" t="s">
+      <c r="C458" s="0" t="s">
         <v>982</v>
       </c>
-      <c r="C458" s="0" t="s">
-        <v>89</v>
-      </c>
       <c r="D458" s="0">
-        <v>249562.5</v>
+        <v>385.4</v>
       </c>
     </row>
     <row r="459">
@@ -9651,10 +9657,10 @@
         <v>984</v>
       </c>
       <c r="C459" s="0" t="s">
-        <v>572</v>
+        <v>89</v>
       </c>
       <c r="D459" s="0">
-        <v>71176.4</v>
+        <v>296147.5</v>
       </c>
     </row>
     <row r="460">
@@ -9665,10 +9671,10 @@
         <v>986</v>
       </c>
       <c r="C460" s="0" t="s">
-        <v>132</v>
+        <v>574</v>
       </c>
       <c r="D460" s="0">
-        <v>96</v>
+        <v>71176.4</v>
       </c>
     </row>
     <row r="461">
@@ -9679,10 +9685,10 @@
         <v>988</v>
       </c>
       <c r="C461" s="0" t="s">
-        <v>69</v>
+        <v>132</v>
       </c>
       <c r="D461" s="0">
-        <v>950</v>
+        <v>96</v>
       </c>
     </row>
     <row r="462">
@@ -9693,10 +9699,10 @@
         <v>990</v>
       </c>
       <c r="C462" s="0" t="s">
-        <v>471</v>
+        <v>69</v>
       </c>
       <c r="D462" s="0">
-        <v>342641</v>
+        <v>950</v>
       </c>
     </row>
     <row r="463">
@@ -9707,10 +9713,10 @@
         <v>992</v>
       </c>
       <c r="C463" s="0" t="s">
-        <v>150</v>
+        <v>471</v>
       </c>
       <c r="D463" s="0">
-        <v>2200</v>
+        <v>342641</v>
       </c>
     </row>
     <row r="464">
@@ -9721,10 +9727,10 @@
         <v>994</v>
       </c>
       <c r="C464" s="0" t="s">
-        <v>480</v>
+        <v>150</v>
       </c>
       <c r="D464" s="0">
-        <v>41000</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="465">
@@ -9735,10 +9741,10 @@
         <v>996</v>
       </c>
       <c r="C465" s="0" t="s">
-        <v>69</v>
+        <v>480</v>
       </c>
       <c r="D465" s="0">
-        <v>9299</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="466">
@@ -9749,10 +9755,10 @@
         <v>998</v>
       </c>
       <c r="C466" s="0" t="s">
-        <v>910</v>
+        <v>69</v>
       </c>
       <c r="D466" s="0">
-        <v>825</v>
+        <v>9299</v>
       </c>
     </row>
     <row r="467">
@@ -9763,7 +9769,7 @@
         <v>1000</v>
       </c>
       <c r="C467" s="0" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
       <c r="D467" s="0">
         <v>825</v>
@@ -9777,7 +9783,7 @@
         <v>1002</v>
       </c>
       <c r="C468" s="0" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
       <c r="D468" s="0">
         <v>825</v>
@@ -9791,10 +9797,10 @@
         <v>1004</v>
       </c>
       <c r="C469" s="0" t="s">
-        <v>22</v>
+        <v>912</v>
       </c>
       <c r="D469" s="0">
-        <v>563.36</v>
+        <v>825</v>
       </c>
     </row>
     <row r="470">
@@ -9805,10 +9811,10 @@
         <v>1006</v>
       </c>
       <c r="C470" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D470" s="0">
-        <v>3520</v>
+        <v>563.36</v>
       </c>
     </row>
     <row r="471">
@@ -9822,7 +9828,7 @@
         <v>16</v>
       </c>
       <c r="D471" s="0">
-        <v>2600</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="472">
@@ -9833,10 +9839,10 @@
         <v>1010</v>
       </c>
       <c r="C472" s="0" t="s">
-        <v>279</v>
+        <v>16</v>
       </c>
       <c r="D472" s="0">
-        <v>3700</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="473">
@@ -9850,7 +9856,7 @@
         <v>279</v>
       </c>
       <c r="D473" s="0">
-        <v>2600</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="474">
@@ -9861,10 +9867,10 @@
         <v>1014</v>
       </c>
       <c r="C474" s="0" t="s">
-        <v>16</v>
+        <v>279</v>
       </c>
       <c r="D474" s="0">
-        <v>2235</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="475">
@@ -9878,35 +9884,35 @@
         <v>16</v>
       </c>
       <c r="D475" s="0">
-        <v>3850</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="476">
       <c r="A476" s="0" t="s">
-        <v>391</v>
+        <v>1017</v>
       </c>
       <c r="B476" s="0" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="C476" s="0" t="s">
-        <v>1018</v>
+        <v>16</v>
       </c>
       <c r="D476" s="0">
-        <v>1</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="477">
       <c r="A477" s="0" t="s">
+        <v>391</v>
+      </c>
+      <c r="B477" s="0" t="s">
         <v>1019</v>
       </c>
-      <c r="B477" s="0" t="s">
+      <c r="C477" s="0" t="s">
         <v>1020</v>
       </c>
-      <c r="C477" s="0" t="s">
-        <v>29</v>
-      </c>
       <c r="D477" s="0">
-        <v>13715</v>
+        <v>1</v>
       </c>
     </row>
     <row r="478">
@@ -9917,10 +9923,10 @@
         <v>1022</v>
       </c>
       <c r="C478" s="0" t="s">
-        <v>370</v>
+        <v>29</v>
       </c>
       <c r="D478" s="0">
-        <v>3859.93</v>
+        <v>13715</v>
       </c>
     </row>
     <row r="479">
@@ -9934,7 +9940,7 @@
         <v>370</v>
       </c>
       <c r="D479" s="0">
-        <v>11751.49</v>
+        <v>3859.93</v>
       </c>
     </row>
     <row r="480">
@@ -9945,10 +9951,10 @@
         <v>1026</v>
       </c>
       <c r="C480" s="0" t="s">
-        <v>334</v>
+        <v>370</v>
       </c>
       <c r="D480" s="0">
-        <v>6000</v>
+        <v>11751.49</v>
       </c>
     </row>
     <row r="481">
@@ -9962,7 +9968,7 @@
         <v>334</v>
       </c>
       <c r="D481" s="0">
-        <v>3000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="482">
@@ -9973,10 +9979,10 @@
         <v>1030</v>
       </c>
       <c r="C482" s="0" t="s">
-        <v>38</v>
+        <v>334</v>
       </c>
       <c r="D482" s="0">
-        <v>618</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="483">
@@ -9987,24 +9993,24 @@
         <v>1032</v>
       </c>
       <c r="C483" s="0" t="s">
-        <v>1033</v>
+        <v>38</v>
       </c>
       <c r="D483" s="0">
-        <v>24600</v>
+        <v>618</v>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="0" t="s">
+        <v>1033</v>
+      </c>
+      <c r="B484" s="0" t="s">
         <v>1034</v>
       </c>
-      <c r="B484" s="0" t="s">
+      <c r="C484" s="0" t="s">
         <v>1035</v>
       </c>
-      <c r="C484" s="0" t="s">
-        <v>102</v>
-      </c>
       <c r="D484" s="0">
-        <v>0</v>
+        <v>24600</v>
       </c>
     </row>
     <row r="485">
@@ -10015,10 +10021,10 @@
         <v>1037</v>
       </c>
       <c r="C485" s="0" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="D485" s="0">
-        <v>32942.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="486">
@@ -10029,10 +10035,10 @@
         <v>1039</v>
       </c>
       <c r="C486" s="0" t="s">
-        <v>370</v>
+        <v>89</v>
       </c>
       <c r="D486" s="0">
-        <v>75529.71</v>
+        <v>40928.25</v>
       </c>
     </row>
     <row r="487">
@@ -10046,7 +10052,7 @@
         <v>370</v>
       </c>
       <c r="D487" s="0">
-        <v>41613.42</v>
+        <v>75529.71</v>
       </c>
     </row>
     <row r="488">
@@ -10060,7 +10066,7 @@
         <v>370</v>
       </c>
       <c r="D488" s="0">
-        <v>87056.42</v>
+        <v>41613.42</v>
       </c>
     </row>
     <row r="489">
@@ -10074,7 +10080,7 @@
         <v>370</v>
       </c>
       <c r="D489" s="0">
-        <v>49243.16</v>
+        <v>87056.42</v>
       </c>
     </row>
     <row r="490">
@@ -10085,10 +10091,10 @@
         <v>1047</v>
       </c>
       <c r="C490" s="0" t="s">
-        <v>22</v>
+        <v>370</v>
       </c>
       <c r="D490" s="0">
-        <v>1600</v>
+        <v>49243.16</v>
       </c>
     </row>
     <row r="491">
@@ -10099,10 +10105,10 @@
         <v>1049</v>
       </c>
       <c r="C491" s="0" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D491" s="0">
-        <v>3338.9</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="492">
@@ -10116,7 +10122,7 @@
         <v>29</v>
       </c>
       <c r="D492" s="0">
-        <v>3987</v>
+        <v>3338.9</v>
       </c>
     </row>
     <row r="493">
@@ -10130,7 +10136,7 @@
         <v>29</v>
       </c>
       <c r="D493" s="0">
-        <v>4010.17</v>
+        <v>3987</v>
       </c>
     </row>
     <row r="494">
@@ -10144,35 +10150,35 @@
         <v>29</v>
       </c>
       <c r="D494" s="0">
+        <v>4010.17</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="0" t="s">
+        <v>1056</v>
+      </c>
+      <c r="B495" s="0" t="s">
+        <v>1057</v>
+      </c>
+      <c r="C495" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D495" s="0">
         <v>3382.65</v>
       </c>
     </row>
-    <row r="495">
-      <c r="A495" s="2" t="s">
-        <v>1056</v>
-      </c>
-      <c r="B495" s="2" t="s">
-        <v>1057</v>
-      </c>
-      <c r="C495" s="2" t="s">
+    <row r="496">
+      <c r="A496" s="2" t="s">
+        <v>1058</v>
+      </c>
+      <c r="B496" s="2" t="s">
+        <v>1059</v>
+      </c>
+      <c r="C496" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D495" s="2">
+      <c r="D496" s="2">
         <v>0</v>
-      </c>
-    </row>
-    <row r="496">
-      <c r="A496" s="0" t="s">
-        <v>1058</v>
-      </c>
-      <c r="B496" s="0" t="s">
-        <v>1059</v>
-      </c>
-      <c r="C496" s="0" t="s">
-        <v>150</v>
-      </c>
-      <c r="D496" s="0">
-        <v>430</v>
       </c>
     </row>
     <row r="497">
@@ -10183,9 +10189,23 @@
         <v>1061</v>
       </c>
       <c r="C497" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="D497" s="0">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="0" t="s">
+        <v>1062</v>
+      </c>
+      <c r="B498" s="0" t="s">
+        <v>1063</v>
+      </c>
+      <c r="C498" s="0" t="s">
         <v>132</v>
       </c>
-      <c r="D497" s="0">
+      <c r="D498" s="0">
         <v>462</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: stock y precios actualizados mar. 21/07/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1072" uniqueCount="1072">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="1074">
   <si>
     <t>Código</t>
   </si>
@@ -1473,6 +1473,12 @@
   </si>
   <si>
     <t>GRIPABEN CARAMELOS Caram. x 9 - 000016343</t>
+  </si>
+  <si>
+    <t>000024189</t>
+  </si>
+  <si>
+    <t>GRIPABEN T DESC. LIMON Y MIEL SOBRES X 5 X 5G - 000024189</t>
   </si>
   <si>
     <t>000024406</t>
@@ -3286,7 +3292,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A3:D502"/>
+  <dimension ref="A3:D503"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="3">
@@ -3440,7 +3446,7 @@
         <v>29</v>
       </c>
       <c r="D13" s="0">
-        <v>132.08</v>
+        <v>134.59</v>
       </c>
     </row>
     <row r="14">
@@ -3622,7 +3628,7 @@
         <v>29</v>
       </c>
       <c r="D26" s="0">
-        <v>157.16</v>
+        <v>160.14</v>
       </c>
     </row>
     <row r="27">
@@ -3720,7 +3726,7 @@
         <v>19</v>
       </c>
       <c r="D33" s="0">
-        <v>12456.52</v>
+        <v>10856.33</v>
       </c>
     </row>
     <row r="34">
@@ -5050,7 +5056,7 @@
         <v>29</v>
       </c>
       <c r="D128" s="0">
-        <v>6986.2</v>
+        <v>7118.9</v>
       </c>
     </row>
     <row r="129">
@@ -5442,7 +5448,7 @@
         <v>29</v>
       </c>
       <c r="D156" s="0">
-        <v>97734</v>
+        <v>103000</v>
       </c>
     </row>
     <row r="157">
@@ -5456,7 +5462,7 @@
         <v>29</v>
       </c>
       <c r="D157" s="0">
-        <v>105490.7</v>
+        <v>114000</v>
       </c>
     </row>
     <row r="158">
@@ -5470,7 +5476,7 @@
         <v>29</v>
       </c>
       <c r="D158" s="0">
-        <v>131863.3</v>
+        <v>135000</v>
       </c>
     </row>
     <row r="159">
@@ -5638,7 +5644,7 @@
         <v>29</v>
       </c>
       <c r="D170" s="0">
-        <v>950</v>
+        <v>954.8</v>
       </c>
     </row>
     <row r="171">
@@ -5652,7 +5658,7 @@
         <v>29</v>
       </c>
       <c r="D171" s="0">
-        <v>265.3</v>
+        <v>744.2</v>
       </c>
     </row>
     <row r="172">
@@ -5806,7 +5812,7 @@
         <v>78</v>
       </c>
       <c r="D182" s="0">
-        <v>2687.98</v>
+        <v>2850</v>
       </c>
     </row>
     <row r="183">
@@ -5876,7 +5882,7 @@
         <v>19</v>
       </c>
       <c r="D187" s="0">
-        <v>330</v>
+        <v>405</v>
       </c>
     </row>
     <row r="188">
@@ -6324,7 +6330,7 @@
         <v>19</v>
       </c>
       <c r="D219" s="0">
-        <v>1547.86</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="220">
@@ -6335,10 +6341,10 @@
         <v>488</v>
       </c>
       <c r="C220" s="0" t="s">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="D220" s="0">
-        <v>4700</v>
+        <v>4391.8</v>
       </c>
     </row>
     <row r="221">
@@ -6352,7 +6358,7 @@
         <v>53</v>
       </c>
       <c r="D221" s="0">
-        <v>4200</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="222">
@@ -6391,21 +6397,21 @@
         <v>496</v>
       </c>
       <c r="C224" s="0" t="s">
-        <v>497</v>
+        <v>53</v>
       </c>
       <c r="D224" s="0">
-        <v>265</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="0" t="s">
+        <v>497</v>
+      </c>
+      <c r="B225" s="0" t="s">
         <v>498</v>
       </c>
-      <c r="B225" s="0" t="s">
+      <c r="C225" s="0" t="s">
         <v>499</v>
-      </c>
-      <c r="C225" s="0" t="s">
-        <v>497</v>
       </c>
       <c r="D225" s="0">
         <v>265</v>
@@ -6419,7 +6425,7 @@
         <v>501</v>
       </c>
       <c r="C226" s="0" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="D226" s="0">
         <v>265</v>
@@ -6433,7 +6439,7 @@
         <v>503</v>
       </c>
       <c r="C227" s="0" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="D227" s="0">
         <v>265</v>
@@ -6447,7 +6453,7 @@
         <v>505</v>
       </c>
       <c r="C228" s="0" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="D228" s="0">
         <v>265</v>
@@ -6461,7 +6467,7 @@
         <v>507</v>
       </c>
       <c r="C229" s="0" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="D229" s="0">
         <v>265</v>
@@ -6475,21 +6481,21 @@
         <v>509</v>
       </c>
       <c r="C230" s="0" t="s">
-        <v>510</v>
+        <v>499</v>
       </c>
       <c r="D230" s="0">
-        <v>4700</v>
+        <v>265</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="0" t="s">
+        <v>510</v>
+      </c>
+      <c r="B231" s="0" t="s">
         <v>511</v>
       </c>
-      <c r="B231" s="0" t="s">
+      <c r="C231" s="0" t="s">
         <v>512</v>
-      </c>
-      <c r="C231" s="0" t="s">
-        <v>513</v>
       </c>
       <c r="D231" s="0">
         <v>4700</v>
@@ -6497,13 +6503,13 @@
     </row>
     <row r="232">
       <c r="A232" s="0" t="s">
+        <v>513</v>
+      </c>
+      <c r="B232" s="0" t="s">
         <v>514</v>
       </c>
-      <c r="B232" s="0" t="s">
+      <c r="C232" s="0" t="s">
         <v>515</v>
-      </c>
-      <c r="C232" s="0" t="s">
-        <v>53</v>
       </c>
       <c r="D232" s="0">
         <v>4700</v>
@@ -6520,7 +6526,7 @@
         <v>53</v>
       </c>
       <c r="D233" s="0">
-        <v>500</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="234">
@@ -6534,7 +6540,7 @@
         <v>53</v>
       </c>
       <c r="D234" s="0">
-        <v>210</v>
+        <v>500</v>
       </c>
     </row>
     <row r="235">
@@ -6548,7 +6554,7 @@
         <v>53</v>
       </c>
       <c r="D235" s="0">
-        <v>247</v>
+        <v>210</v>
       </c>
     </row>
     <row r="236">
@@ -6559,10 +6565,10 @@
         <v>523</v>
       </c>
       <c r="C236" s="0" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="D236" s="0">
-        <v>5600</v>
+        <v>247</v>
       </c>
     </row>
     <row r="237">
@@ -6573,10 +6579,10 @@
         <v>525</v>
       </c>
       <c r="C237" s="0" t="s">
-        <v>148</v>
+        <v>38</v>
       </c>
       <c r="D237" s="0">
-        <v>6000</v>
+        <v>5600</v>
       </c>
     </row>
     <row r="238">
@@ -6587,10 +6593,10 @@
         <v>527</v>
       </c>
       <c r="C238" s="0" t="s">
-        <v>71</v>
+        <v>148</v>
       </c>
       <c r="D238" s="0">
-        <v>80000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="239">
@@ -6604,7 +6610,7 @@
         <v>71</v>
       </c>
       <c r="D239" s="0">
-        <v>90000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="240">
@@ -6618,7 +6624,7 @@
         <v>71</v>
       </c>
       <c r="D240" s="0">
-        <v>110000</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="241">
@@ -6629,10 +6635,10 @@
         <v>533</v>
       </c>
       <c r="C241" s="0" t="s">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="D241" s="0">
-        <v>1100</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="242">
@@ -6646,7 +6652,7 @@
         <v>16</v>
       </c>
       <c r="D242" s="0">
-        <v>2500</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="243">
@@ -6657,10 +6663,10 @@
         <v>537</v>
       </c>
       <c r="C243" s="0" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="D243" s="0">
-        <v>13304.2</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="244">
@@ -6671,10 +6677,10 @@
         <v>539</v>
       </c>
       <c r="C244" s="0" t="s">
-        <v>283</v>
+        <v>29</v>
       </c>
       <c r="D244" s="0">
-        <v>450</v>
+        <v>13636.84</v>
       </c>
     </row>
     <row r="245">
@@ -6685,10 +6691,10 @@
         <v>541</v>
       </c>
       <c r="C245" s="0" t="s">
-        <v>16</v>
+        <v>283</v>
       </c>
       <c r="D245" s="0">
-        <v>555</v>
+        <v>450</v>
       </c>
     </row>
     <row r="246">
@@ -6702,7 +6708,7 @@
         <v>16</v>
       </c>
       <c r="D246" s="0">
-        <v>825</v>
+        <v>555</v>
       </c>
     </row>
     <row r="247">
@@ -6716,7 +6722,7 @@
         <v>16</v>
       </c>
       <c r="D247" s="0">
-        <v>36.3</v>
+        <v>825</v>
       </c>
     </row>
     <row r="248">
@@ -6730,7 +6736,7 @@
         <v>16</v>
       </c>
       <c r="D248" s="0">
-        <v>544.5</v>
+        <v>36.3</v>
       </c>
     </row>
     <row r="249">
@@ -6744,7 +6750,7 @@
         <v>16</v>
       </c>
       <c r="D249" s="0">
-        <v>750</v>
+        <v>544.5</v>
       </c>
     </row>
     <row r="250">
@@ -6755,10 +6761,10 @@
         <v>551</v>
       </c>
       <c r="C250" s="0" t="s">
-        <v>148</v>
+        <v>16</v>
       </c>
       <c r="D250" s="0">
-        <v>1130</v>
+        <v>750</v>
       </c>
     </row>
     <row r="251">
@@ -6769,10 +6775,10 @@
         <v>553</v>
       </c>
       <c r="C251" s="0" t="s">
-        <v>53</v>
+        <v>148</v>
       </c>
       <c r="D251" s="0">
-        <v>4510</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="252">
@@ -6825,10 +6831,10 @@
         <v>561</v>
       </c>
       <c r="C255" s="0" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="D255" s="0">
-        <v>902</v>
+        <v>4510</v>
       </c>
     </row>
     <row r="256">
@@ -6842,7 +6848,7 @@
         <v>16</v>
       </c>
       <c r="D256" s="0">
-        <v>880</v>
+        <v>902</v>
       </c>
     </row>
     <row r="257">
@@ -6853,10 +6859,10 @@
         <v>565</v>
       </c>
       <c r="C257" s="0" t="s">
-        <v>137</v>
+        <v>16</v>
       </c>
       <c r="D257" s="0">
-        <v>430</v>
+        <v>880</v>
       </c>
     </row>
     <row r="258">
@@ -6870,7 +6876,7 @@
         <v>137</v>
       </c>
       <c r="D258" s="0">
-        <v>354.54</v>
+        <v>430</v>
       </c>
     </row>
     <row r="259">
@@ -6881,10 +6887,10 @@
         <v>569</v>
       </c>
       <c r="C259" s="0" t="s">
-        <v>19</v>
+        <v>137</v>
       </c>
       <c r="D259" s="0">
-        <v>318.63</v>
+        <v>354.54</v>
       </c>
     </row>
     <row r="260">
@@ -6898,7 +6904,7 @@
         <v>19</v>
       </c>
       <c r="D260" s="0">
-        <v>415.15</v>
+        <v>318.63</v>
       </c>
     </row>
     <row r="261">
@@ -6912,7 +6918,7 @@
         <v>19</v>
       </c>
       <c r="D261" s="0">
-        <v>760</v>
+        <v>415.15</v>
       </c>
     </row>
     <row r="262">
@@ -6926,7 +6932,7 @@
         <v>19</v>
       </c>
       <c r="D262" s="0">
-        <v>820</v>
+        <v>760</v>
       </c>
     </row>
     <row r="263">
@@ -6937,24 +6943,24 @@
         <v>577</v>
       </c>
       <c r="C263" s="0" t="s">
-        <v>578</v>
+        <v>19</v>
       </c>
       <c r="D263" s="0">
-        <v>177940.1</v>
+        <v>820</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="0" t="s">
+        <v>578</v>
+      </c>
+      <c r="B264" s="0" t="s">
         <v>579</v>
       </c>
-      <c r="B264" s="0" t="s">
+      <c r="C264" s="0" t="s">
         <v>580</v>
       </c>
-      <c r="C264" s="0" t="s">
-        <v>71</v>
-      </c>
       <c r="D264" s="0">
-        <v>34000</v>
+        <v>177940.1</v>
       </c>
     </row>
     <row r="265">
@@ -6968,7 +6974,7 @@
         <v>71</v>
       </c>
       <c r="D265" s="0">
-        <v>30000</v>
+        <v>34000</v>
       </c>
     </row>
     <row r="266">
@@ -6979,10 +6985,10 @@
         <v>584</v>
       </c>
       <c r="C266" s="0" t="s">
-        <v>475</v>
+        <v>71</v>
       </c>
       <c r="D266" s="0">
-        <v>227939.52</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="267">
@@ -6996,7 +7002,7 @@
         <v>475</v>
       </c>
       <c r="D267" s="0">
-        <v>184488.7</v>
+        <v>227939.52</v>
       </c>
     </row>
     <row r="268">
@@ -7007,10 +7013,10 @@
         <v>588</v>
       </c>
       <c r="C268" s="0" t="s">
-        <v>16</v>
+        <v>475</v>
       </c>
       <c r="D268" s="0">
-        <v>1760</v>
+        <v>184488.7</v>
       </c>
     </row>
     <row r="269">
@@ -7021,24 +7027,24 @@
         <v>590</v>
       </c>
       <c r="C269" s="0" t="s">
-        <v>591</v>
+        <v>16</v>
       </c>
       <c r="D269" s="0">
-        <v>26350</v>
+        <v>1760</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="0" t="s">
+        <v>591</v>
+      </c>
+      <c r="B270" s="0" t="s">
         <v>592</v>
       </c>
-      <c r="B270" s="0" t="s">
+      <c r="C270" s="0" t="s">
         <v>593</v>
       </c>
-      <c r="C270" s="0" t="s">
-        <v>484</v>
-      </c>
       <c r="D270" s="0">
-        <v>31250</v>
+        <v>26350</v>
       </c>
     </row>
     <row r="271">
@@ -7049,10 +7055,10 @@
         <v>595</v>
       </c>
       <c r="C271" s="0" t="s">
-        <v>53</v>
+        <v>484</v>
       </c>
       <c r="D271" s="0">
-        <v>34.98</v>
+        <v>31250</v>
       </c>
     </row>
     <row r="272">
@@ -7066,7 +7072,7 @@
         <v>53</v>
       </c>
       <c r="D272" s="0">
-        <v>65</v>
+        <v>34.98</v>
       </c>
     </row>
     <row r="273">
@@ -7080,7 +7086,7 @@
         <v>53</v>
       </c>
       <c r="D273" s="0">
-        <v>92</v>
+        <v>65</v>
       </c>
     </row>
     <row r="274">
@@ -7094,7 +7100,7 @@
         <v>53</v>
       </c>
       <c r="D274" s="0">
-        <v>33</v>
+        <v>92</v>
       </c>
     </row>
     <row r="275">
@@ -7108,7 +7114,7 @@
         <v>53</v>
       </c>
       <c r="D275" s="0">
-        <v>38.22</v>
+        <v>33</v>
       </c>
     </row>
     <row r="276">
@@ -7119,10 +7125,10 @@
         <v>605</v>
       </c>
       <c r="C276" s="0" t="s">
-        <v>338</v>
+        <v>53</v>
       </c>
       <c r="D276" s="0">
-        <v>300</v>
+        <v>38.22</v>
       </c>
     </row>
     <row r="277">
@@ -7136,7 +7142,7 @@
         <v>338</v>
       </c>
       <c r="D277" s="0">
-        <v>370</v>
+        <v>300</v>
       </c>
     </row>
     <row r="278">
@@ -7147,10 +7153,10 @@
         <v>609</v>
       </c>
       <c r="C278" s="0" t="s">
-        <v>359</v>
+        <v>338</v>
       </c>
       <c r="D278" s="0">
-        <v>450</v>
+        <v>370</v>
       </c>
     </row>
     <row r="279">
@@ -7161,7 +7167,7 @@
         <v>611</v>
       </c>
       <c r="C279" s="0" t="s">
-        <v>38</v>
+        <v>359</v>
       </c>
       <c r="D279" s="0">
         <v>450</v>
@@ -7175,7 +7181,7 @@
         <v>613</v>
       </c>
       <c r="C280" s="0" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="D280" s="0">
         <v>450</v>
@@ -7192,7 +7198,7 @@
         <v>16</v>
       </c>
       <c r="D281" s="0">
-        <v>1650</v>
+        <v>450</v>
       </c>
     </row>
     <row r="282">
@@ -7206,7 +7212,7 @@
         <v>16</v>
       </c>
       <c r="D282" s="0">
-        <v>2100</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="283">
@@ -7220,7 +7226,7 @@
         <v>16</v>
       </c>
       <c r="D283" s="0">
-        <v>1980</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="284">
@@ -7234,7 +7240,7 @@
         <v>16</v>
       </c>
       <c r="D284" s="0">
-        <v>2160</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="285">
@@ -7248,7 +7254,7 @@
         <v>16</v>
       </c>
       <c r="D285" s="0">
-        <v>1100</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="286">
@@ -7262,7 +7268,7 @@
         <v>16</v>
       </c>
       <c r="D286" s="0">
-        <v>2600</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="287">
@@ -7276,7 +7282,7 @@
         <v>16</v>
       </c>
       <c r="D287" s="0">
-        <v>2000</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="288">
@@ -7290,7 +7296,7 @@
         <v>16</v>
       </c>
       <c r="D288" s="0">
-        <v>6700</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="289">
@@ -7304,7 +7310,7 @@
         <v>16</v>
       </c>
       <c r="D289" s="0">
-        <v>1650</v>
+        <v>6700</v>
       </c>
     </row>
     <row r="290">
@@ -7318,7 +7324,7 @@
         <v>16</v>
       </c>
       <c r="D290" s="0">
-        <v>1035</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="291">
@@ -7332,7 +7338,7 @@
         <v>16</v>
       </c>
       <c r="D291" s="0">
-        <v>2600</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="292">
@@ -7346,7 +7352,7 @@
         <v>16</v>
       </c>
       <c r="D292" s="0">
-        <v>2400</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="293">
@@ -7357,10 +7363,10 @@
         <v>639</v>
       </c>
       <c r="C293" s="0" t="s">
-        <v>137</v>
+        <v>16</v>
       </c>
       <c r="D293" s="0">
-        <v>4497.2</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="294">
@@ -7374,7 +7380,7 @@
         <v>137</v>
       </c>
       <c r="D294" s="0">
-        <v>2328</v>
+        <v>4497.2</v>
       </c>
     </row>
     <row r="295">
@@ -7388,7 +7394,7 @@
         <v>137</v>
       </c>
       <c r="D295" s="0">
-        <v>1138</v>
+        <v>2328</v>
       </c>
     </row>
     <row r="296">
@@ -7399,10 +7405,10 @@
         <v>645</v>
       </c>
       <c r="C296" s="0" t="s">
-        <v>29</v>
+        <v>137</v>
       </c>
       <c r="D296" s="0">
-        <v>7234.96</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="297">
@@ -7413,10 +7419,10 @@
         <v>647</v>
       </c>
       <c r="C297" s="0" t="s">
-        <v>120</v>
+        <v>29</v>
       </c>
       <c r="D297" s="0">
-        <v>1790</v>
+        <v>7372.42</v>
       </c>
     </row>
     <row r="298">
@@ -7430,7 +7436,7 @@
         <v>120</v>
       </c>
       <c r="D298" s="0">
-        <v>2859.96</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="299">
@@ -7444,7 +7450,7 @@
         <v>120</v>
       </c>
       <c r="D299" s="0">
-        <v>4800</v>
+        <v>2859.96</v>
       </c>
     </row>
     <row r="300">
@@ -7455,24 +7461,24 @@
         <v>653</v>
       </c>
       <c r="C300" s="0" t="s">
-        <v>654</v>
+        <v>120</v>
       </c>
       <c r="D300" s="0">
-        <v>0</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="0" t="s">
+        <v>654</v>
+      </c>
+      <c r="B301" s="0" t="s">
         <v>655</v>
       </c>
-      <c r="B301" s="0" t="s">
+      <c r="C301" s="0" t="s">
         <v>656</v>
       </c>
-      <c r="C301" s="0" t="s">
-        <v>29</v>
-      </c>
       <c r="D301" s="0">
-        <v>494</v>
+        <v>0</v>
       </c>
     </row>
     <row r="302">
@@ -7486,7 +7492,7 @@
         <v>29</v>
       </c>
       <c r="D302" s="0">
-        <v>665.3</v>
+        <v>494</v>
       </c>
     </row>
     <row r="303">
@@ -7497,10 +7503,10 @@
         <v>660</v>
       </c>
       <c r="C303" s="0" t="s">
-        <v>91</v>
+        <v>29</v>
       </c>
       <c r="D303" s="0">
-        <v>33275</v>
+        <v>665.3</v>
       </c>
     </row>
     <row r="304">
@@ -7514,7 +7520,7 @@
         <v>91</v>
       </c>
       <c r="D304" s="0">
-        <v>4525.4</v>
+        <v>33275</v>
       </c>
     </row>
     <row r="305">
@@ -7525,10 +7531,10 @@
         <v>664</v>
       </c>
       <c r="C305" s="0" t="s">
-        <v>148</v>
+        <v>91</v>
       </c>
       <c r="D305" s="0">
-        <v>896</v>
+        <v>4525.4</v>
       </c>
     </row>
     <row r="306">
@@ -7539,10 +7545,10 @@
         <v>666</v>
       </c>
       <c r="C306" s="0" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="D306" s="0">
-        <v>1250</v>
+        <v>896</v>
       </c>
     </row>
     <row r="307">
@@ -7553,10 +7559,10 @@
         <v>668</v>
       </c>
       <c r="C307" s="0" t="s">
-        <v>91</v>
+        <v>137</v>
       </c>
       <c r="D307" s="0">
-        <v>312785</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="308">
@@ -7567,10 +7573,10 @@
         <v>670</v>
       </c>
       <c r="C308" s="0" t="s">
-        <v>202</v>
+        <v>91</v>
       </c>
       <c r="D308" s="0">
-        <v>17440</v>
+        <v>312785</v>
       </c>
     </row>
     <row r="309">
@@ -7584,7 +7590,7 @@
         <v>202</v>
       </c>
       <c r="D309" s="0">
-        <v>4390</v>
+        <v>17440</v>
       </c>
     </row>
     <row r="310">
@@ -7609,10 +7615,10 @@
         <v>676</v>
       </c>
       <c r="C311" s="0" t="s">
-        <v>283</v>
+        <v>202</v>
       </c>
       <c r="D311" s="0">
-        <v>2250</v>
+        <v>4390</v>
       </c>
     </row>
     <row r="312">
@@ -7623,10 +7629,10 @@
         <v>678</v>
       </c>
       <c r="C312" s="0" t="s">
-        <v>202</v>
+        <v>283</v>
       </c>
       <c r="D312" s="0">
-        <v>3355</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="313">
@@ -7637,10 +7643,10 @@
         <v>680</v>
       </c>
       <c r="C313" s="0" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="D313" s="0">
-        <v>7500</v>
+        <v>3355</v>
       </c>
     </row>
     <row r="314">
@@ -7651,10 +7657,10 @@
         <v>682</v>
       </c>
       <c r="C314" s="0" t="s">
-        <v>91</v>
+        <v>207</v>
       </c>
       <c r="D314" s="0">
-        <v>23958</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="315">
@@ -7668,7 +7674,7 @@
         <v>91</v>
       </c>
       <c r="D315" s="0">
-        <v>239580</v>
+        <v>23958</v>
       </c>
     </row>
     <row r="316">
@@ -7679,10 +7685,10 @@
         <v>686</v>
       </c>
       <c r="C316" s="0" t="s">
-        <v>53</v>
+        <v>91</v>
       </c>
       <c r="D316" s="0">
-        <v>130</v>
+        <v>239580</v>
       </c>
     </row>
     <row r="317">
@@ -7693,10 +7699,10 @@
         <v>688</v>
       </c>
       <c r="C317" s="0" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="D317" s="0">
-        <v>285.6</v>
+        <v>130</v>
       </c>
     </row>
     <row r="318">
@@ -7710,7 +7716,7 @@
         <v>22</v>
       </c>
       <c r="D318" s="0">
-        <v>338</v>
+        <v>285.6</v>
       </c>
     </row>
     <row r="319">
@@ -7721,21 +7727,21 @@
         <v>692</v>
       </c>
       <c r="C319" s="0" t="s">
-        <v>693</v>
+        <v>22</v>
       </c>
       <c r="D319" s="0">
-        <v>770</v>
+        <v>338</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="0" t="s">
+        <v>693</v>
+      </c>
+      <c r="B320" s="0" t="s">
         <v>694</v>
       </c>
-      <c r="B320" s="0" t="s">
+      <c r="C320" s="0" t="s">
         <v>695</v>
-      </c>
-      <c r="C320" s="0" t="s">
-        <v>696</v>
       </c>
       <c r="D320" s="0">
         <v>770</v>
@@ -7743,16 +7749,16 @@
     </row>
     <row r="321">
       <c r="A321" s="0" t="s">
+        <v>696</v>
+      </c>
+      <c r="B321" s="0" t="s">
         <v>697</v>
       </c>
-      <c r="B321" s="0" t="s">
+      <c r="C321" s="0" t="s">
         <v>698</v>
       </c>
-      <c r="C321" s="0" t="s">
-        <v>16</v>
-      </c>
       <c r="D321" s="0">
-        <v>973.5</v>
+        <v>770</v>
       </c>
     </row>
     <row r="322">
@@ -7763,10 +7769,10 @@
         <v>700</v>
       </c>
       <c r="C322" s="0" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D322" s="0">
-        <v>507.08</v>
+        <v>973.5</v>
       </c>
     </row>
     <row r="323">
@@ -7777,10 +7783,10 @@
         <v>702</v>
       </c>
       <c r="C323" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D323" s="0">
-        <v>450</v>
+        <v>507.08</v>
       </c>
     </row>
     <row r="324">
@@ -7791,10 +7797,10 @@
         <v>704</v>
       </c>
       <c r="C324" s="0" t="s">
-        <v>148</v>
+        <v>16</v>
       </c>
       <c r="D324" s="0">
-        <v>760</v>
+        <v>450</v>
       </c>
     </row>
     <row r="325">
@@ -7805,10 +7811,10 @@
         <v>706</v>
       </c>
       <c r="C325" s="0" t="s">
-        <v>283</v>
+        <v>148</v>
       </c>
       <c r="D325" s="0">
-        <v>5900</v>
+        <v>760</v>
       </c>
     </row>
     <row r="326">
@@ -7822,7 +7828,7 @@
         <v>283</v>
       </c>
       <c r="D326" s="0">
-        <v>2900</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="327">
@@ -7833,10 +7839,10 @@
         <v>710</v>
       </c>
       <c r="C327" s="0" t="s">
-        <v>137</v>
+        <v>283</v>
       </c>
       <c r="D327" s="0">
-        <v>886.2</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="328">
@@ -7850,7 +7856,7 @@
         <v>137</v>
       </c>
       <c r="D328" s="0">
-        <v>589.9</v>
+        <v>886.2</v>
       </c>
     </row>
     <row r="329">
@@ -7864,7 +7870,7 @@
         <v>137</v>
       </c>
       <c r="D329" s="0">
-        <v>65</v>
+        <v>589.9</v>
       </c>
     </row>
     <row r="330">
@@ -7875,10 +7881,10 @@
         <v>716</v>
       </c>
       <c r="C330" s="0" t="s">
-        <v>91</v>
+        <v>137</v>
       </c>
       <c r="D330" s="0">
-        <v>11313.5</v>
+        <v>65</v>
       </c>
     </row>
     <row r="331">
@@ -7889,10 +7895,10 @@
         <v>718</v>
       </c>
       <c r="C331" s="0" t="s">
-        <v>35</v>
+        <v>91</v>
       </c>
       <c r="D331" s="0">
-        <v>420</v>
+        <v>11313.5</v>
       </c>
     </row>
     <row r="332">
@@ -7903,10 +7909,10 @@
         <v>720</v>
       </c>
       <c r="C332" s="0" t="s">
-        <v>359</v>
+        <v>35</v>
       </c>
       <c r="D332" s="0">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="333">
@@ -7917,10 +7923,10 @@
         <v>722</v>
       </c>
       <c r="C333" s="0" t="s">
-        <v>22</v>
+        <v>359</v>
       </c>
       <c r="D333" s="0">
-        <v>377</v>
+        <v>418</v>
       </c>
     </row>
     <row r="334">
@@ -7931,10 +7937,10 @@
         <v>724</v>
       </c>
       <c r="C334" s="0" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="D334" s="0">
-        <v>5300</v>
+        <v>377</v>
       </c>
     </row>
     <row r="335">
@@ -7945,10 +7951,10 @@
         <v>726</v>
       </c>
       <c r="C335" s="0" t="s">
-        <v>71</v>
+        <v>46</v>
       </c>
       <c r="D335" s="0">
-        <v>898</v>
+        <v>5300</v>
       </c>
     </row>
     <row r="336">
@@ -7959,10 +7965,10 @@
         <v>728</v>
       </c>
       <c r="C336" s="0" t="s">
-        <v>120</v>
+        <v>71</v>
       </c>
       <c r="D336" s="0">
-        <v>4767</v>
+        <v>898</v>
       </c>
     </row>
     <row r="337">
@@ -7973,10 +7979,10 @@
         <v>730</v>
       </c>
       <c r="C337" s="0" t="s">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="D337" s="0">
-        <v>650</v>
+        <v>4767</v>
       </c>
     </row>
     <row r="338">
@@ -7987,7 +7993,7 @@
         <v>732</v>
       </c>
       <c r="C338" s="0" t="s">
-        <v>71</v>
+        <v>35</v>
       </c>
       <c r="D338" s="0">
         <v>650</v>
@@ -8001,10 +8007,10 @@
         <v>734</v>
       </c>
       <c r="C339" s="0" t="s">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="D339" s="0">
-        <v>2178</v>
+        <v>650</v>
       </c>
     </row>
     <row r="340">
@@ -8015,10 +8021,10 @@
         <v>736</v>
       </c>
       <c r="C340" s="0" t="s">
-        <v>91</v>
+        <v>16</v>
       </c>
       <c r="D340" s="0">
-        <v>7986</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="341">
@@ -8029,24 +8035,24 @@
         <v>738</v>
       </c>
       <c r="C341" s="0" t="s">
-        <v>739</v>
+        <v>91</v>
       </c>
       <c r="D341" s="0">
-        <v>1910</v>
+        <v>7986</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="0" t="s">
+        <v>739</v>
+      </c>
+      <c r="B342" s="0" t="s">
         <v>740</v>
       </c>
-      <c r="B342" s="0" t="s">
+      <c r="C342" s="0" t="s">
         <v>741</v>
       </c>
-      <c r="C342" s="0" t="s">
-        <v>148</v>
-      </c>
       <c r="D342" s="0">
-        <v>900</v>
+        <v>1910</v>
       </c>
     </row>
     <row r="343">
@@ -8057,10 +8063,10 @@
         <v>743</v>
       </c>
       <c r="C343" s="0" t="s">
-        <v>22</v>
+        <v>148</v>
       </c>
       <c r="D343" s="0">
-        <v>1722</v>
+        <v>900</v>
       </c>
     </row>
     <row r="344">
@@ -8071,10 +8077,10 @@
         <v>745</v>
       </c>
       <c r="C344" s="0" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="D344" s="0">
-        <v>456</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="345">
@@ -8088,7 +8094,7 @@
         <v>35</v>
       </c>
       <c r="D345" s="0">
-        <v>59000</v>
+        <v>456</v>
       </c>
     </row>
     <row r="346">
@@ -8099,10 +8105,10 @@
         <v>749</v>
       </c>
       <c r="C346" s="0" t="s">
-        <v>148</v>
+        <v>35</v>
       </c>
       <c r="D346" s="0">
-        <v>750</v>
+        <v>59000</v>
       </c>
     </row>
     <row r="347">
@@ -8116,7 +8122,7 @@
         <v>148</v>
       </c>
       <c r="D347" s="0">
-        <v>1212</v>
+        <v>750</v>
       </c>
     </row>
     <row r="348">
@@ -8130,7 +8136,7 @@
         <v>148</v>
       </c>
       <c r="D348" s="0">
-        <v>1300</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="349">
@@ -8144,7 +8150,7 @@
         <v>148</v>
       </c>
       <c r="D349" s="0">
-        <v>1500</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="350">
@@ -8158,7 +8164,7 @@
         <v>148</v>
       </c>
       <c r="D350" s="0">
-        <v>1400</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="351">
@@ -8169,10 +8175,10 @@
         <v>759</v>
       </c>
       <c r="C351" s="0" t="s">
-        <v>259</v>
+        <v>148</v>
       </c>
       <c r="D351" s="0">
-        <v>11959</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="352">
@@ -8183,10 +8189,10 @@
         <v>761</v>
       </c>
       <c r="C352" s="0" t="s">
-        <v>137</v>
+        <v>259</v>
       </c>
       <c r="D352" s="0">
-        <v>345</v>
+        <v>11959</v>
       </c>
     </row>
     <row r="353">
@@ -8197,10 +8203,10 @@
         <v>763</v>
       </c>
       <c r="C353" s="0" t="s">
-        <v>283</v>
+        <v>137</v>
       </c>
       <c r="D353" s="0">
-        <v>1450</v>
+        <v>345</v>
       </c>
     </row>
     <row r="354">
@@ -8211,10 +8217,10 @@
         <v>765</v>
       </c>
       <c r="C354" s="0" t="s">
-        <v>91</v>
+        <v>283</v>
       </c>
       <c r="D354" s="0">
-        <v>7320.5</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="355">
@@ -8225,10 +8231,10 @@
         <v>767</v>
       </c>
       <c r="C355" s="0" t="s">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="D355" s="0">
-        <v>900</v>
+        <v>7320.5</v>
       </c>
     </row>
     <row r="356">
@@ -8239,10 +8245,10 @@
         <v>769</v>
       </c>
       <c r="C356" s="0" t="s">
-        <v>283</v>
+        <v>16</v>
       </c>
       <c r="D356" s="0">
-        <v>520</v>
+        <v>900</v>
       </c>
     </row>
     <row r="357">
@@ -8253,10 +8259,10 @@
         <v>771</v>
       </c>
       <c r="C357" s="0" t="s">
-        <v>475</v>
+        <v>283</v>
       </c>
       <c r="D357" s="0">
-        <v>64925</v>
+        <v>520</v>
       </c>
     </row>
     <row r="358">
@@ -8267,10 +8273,10 @@
         <v>773</v>
       </c>
       <c r="C358" s="0" t="s">
-        <v>16</v>
+        <v>475</v>
       </c>
       <c r="D358" s="0">
-        <v>1100</v>
+        <v>64925</v>
       </c>
     </row>
     <row r="359">
@@ -8281,10 +8287,10 @@
         <v>775</v>
       </c>
       <c r="C359" s="0" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D359" s="0">
-        <v>1623</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="360">
@@ -8295,10 +8301,10 @@
         <v>777</v>
       </c>
       <c r="C360" s="0" t="s">
-        <v>137</v>
+        <v>22</v>
       </c>
       <c r="D360" s="0">
-        <v>1182.75</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="361">
@@ -8312,7 +8318,7 @@
         <v>137</v>
       </c>
       <c r="D361" s="0">
-        <v>4440.9</v>
+        <v>1182.75</v>
       </c>
     </row>
     <row r="362">
@@ -8323,10 +8329,10 @@
         <v>781</v>
       </c>
       <c r="C362" s="0" t="s">
-        <v>29</v>
+        <v>137</v>
       </c>
       <c r="D362" s="0">
-        <v>1650</v>
+        <v>4440.9</v>
       </c>
     </row>
     <row r="363">
@@ -8340,7 +8346,7 @@
         <v>29</v>
       </c>
       <c r="D363" s="0">
-        <v>1908.8</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="364">
@@ -8351,10 +8357,10 @@
         <v>785</v>
       </c>
       <c r="C364" s="0" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="D364" s="0">
-        <v>450</v>
+        <v>1945.1</v>
       </c>
     </row>
     <row r="365">
@@ -8368,7 +8374,7 @@
         <v>16</v>
       </c>
       <c r="D365" s="0">
-        <v>825</v>
+        <v>450</v>
       </c>
     </row>
     <row r="366">
@@ -8393,10 +8399,10 @@
         <v>791</v>
       </c>
       <c r="C367" s="0" t="s">
-        <v>377</v>
+        <v>16</v>
       </c>
       <c r="D367" s="0">
-        <v>134775.6</v>
+        <v>825</v>
       </c>
     </row>
     <row r="368">
@@ -8410,7 +8416,7 @@
         <v>377</v>
       </c>
       <c r="D368" s="0">
-        <v>175991.55</v>
+        <v>134775.6</v>
       </c>
     </row>
     <row r="369">
@@ -8421,10 +8427,10 @@
         <v>795</v>
       </c>
       <c r="C369" s="0" t="s">
-        <v>71</v>
+        <v>377</v>
       </c>
       <c r="D369" s="0">
-        <v>3263</v>
+        <v>175991.55</v>
       </c>
     </row>
     <row r="370">
@@ -8438,7 +8444,7 @@
         <v>71</v>
       </c>
       <c r="D370" s="0">
-        <v>18027</v>
+        <v>3263</v>
       </c>
     </row>
     <row r="371">
@@ -8449,10 +8455,10 @@
         <v>799</v>
       </c>
       <c r="C371" s="0" t="s">
-        <v>283</v>
+        <v>71</v>
       </c>
       <c r="D371" s="0">
-        <v>515</v>
+        <v>18027</v>
       </c>
     </row>
     <row r="372">
@@ -8463,38 +8469,38 @@
         <v>801</v>
       </c>
       <c r="C372" s="0" t="s">
-        <v>38</v>
+        <v>283</v>
       </c>
       <c r="D372" s="0">
         <v>515</v>
       </c>
     </row>
     <row r="373">
-      <c r="A373" s="2" t="s">
+      <c r="A373" s="0" t="s">
         <v>802</v>
       </c>
-      <c r="B373" s="2" t="s">
+      <c r="B373" s="0" t="s">
         <v>803</v>
       </c>
-      <c r="C373" s="2" t="s">
+      <c r="C373" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="D373" s="0">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="2" t="s">
+        <v>804</v>
+      </c>
+      <c r="B374" s="2" t="s">
+        <v>805</v>
+      </c>
+      <c r="C374" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D373" s="2">
+      <c r="D374" s="2">
         <v>10154</v>
-      </c>
-    </row>
-    <row r="374">
-      <c r="A374" s="0" t="s">
-        <v>804</v>
-      </c>
-      <c r="B374" s="0" t="s">
-        <v>805</v>
-      </c>
-      <c r="C374" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="D374" s="0">
-        <v>9500</v>
       </c>
     </row>
     <row r="375">
@@ -8505,10 +8511,10 @@
         <v>807</v>
       </c>
       <c r="C375" s="0" t="s">
-        <v>475</v>
+        <v>53</v>
       </c>
       <c r="D375" s="0">
-        <v>207558.08</v>
+        <v>9500</v>
       </c>
     </row>
     <row r="376">
@@ -8522,7 +8528,7 @@
         <v>475</v>
       </c>
       <c r="D376" s="0">
-        <v>249069.69</v>
+        <v>207558.08</v>
       </c>
     </row>
     <row r="377">
@@ -8533,10 +8539,10 @@
         <v>811</v>
       </c>
       <c r="C377" s="0" t="s">
-        <v>71</v>
+        <v>475</v>
       </c>
       <c r="D377" s="0">
-        <v>10021.22</v>
+        <v>249069.69</v>
       </c>
     </row>
     <row r="378">
@@ -8550,7 +8556,7 @@
         <v>71</v>
       </c>
       <c r="D378" s="0">
-        <v>17710</v>
+        <v>10021.22</v>
       </c>
     </row>
     <row r="379">
@@ -8561,24 +8567,24 @@
         <v>815</v>
       </c>
       <c r="C379" s="0" t="s">
-        <v>816</v>
+        <v>71</v>
       </c>
       <c r="D379" s="0">
-        <v>1080</v>
+        <v>17710</v>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="0" t="s">
+        <v>816</v>
+      </c>
+      <c r="B380" s="0" t="s">
         <v>817</v>
       </c>
-      <c r="B380" s="0" t="s">
+      <c r="C380" s="0" t="s">
         <v>818</v>
       </c>
-      <c r="C380" s="0" t="s">
-        <v>19</v>
-      </c>
       <c r="D380" s="0">
-        <v>570</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="381">
@@ -8589,24 +8595,24 @@
         <v>820</v>
       </c>
       <c r="C381" s="0" t="s">
-        <v>821</v>
+        <v>19</v>
       </c>
       <c r="D381" s="0">
-        <v>520</v>
+        <v>570</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="0" t="s">
+        <v>821</v>
+      </c>
+      <c r="B382" s="0" t="s">
         <v>822</v>
       </c>
-      <c r="B382" s="0" t="s">
+      <c r="C382" s="0" t="s">
         <v>823</v>
       </c>
-      <c r="C382" s="0" t="s">
-        <v>821</v>
-      </c>
       <c r="D382" s="0">
-        <v>300</v>
+        <v>520</v>
       </c>
     </row>
     <row r="383">
@@ -8617,10 +8623,10 @@
         <v>825</v>
       </c>
       <c r="C383" s="0" t="s">
-        <v>16</v>
+        <v>823</v>
       </c>
       <c r="D383" s="0">
-        <v>2200</v>
+        <v>300</v>
       </c>
     </row>
     <row r="384">
@@ -8634,7 +8640,7 @@
         <v>16</v>
       </c>
       <c r="D384" s="0">
-        <v>2800</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="385">
@@ -8645,10 +8651,10 @@
         <v>829</v>
       </c>
       <c r="C385" s="0" t="s">
-        <v>91</v>
+        <v>16</v>
       </c>
       <c r="D385" s="0">
-        <v>4791.6</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="386">
@@ -8659,10 +8665,10 @@
         <v>831</v>
       </c>
       <c r="C386" s="0" t="s">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="D386" s="0">
-        <v>2699.64</v>
+        <v>4791.6</v>
       </c>
     </row>
     <row r="387">
@@ -8673,10 +8679,10 @@
         <v>833</v>
       </c>
       <c r="C387" s="0" t="s">
-        <v>35</v>
+        <v>71</v>
       </c>
       <c r="D387" s="0">
-        <v>3800</v>
+        <v>2699.64</v>
       </c>
     </row>
     <row r="388">
@@ -8687,10 +8693,10 @@
         <v>835</v>
       </c>
       <c r="C388" s="0" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D388" s="0">
-        <v>4000</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="389">
@@ -8701,24 +8707,24 @@
         <v>837</v>
       </c>
       <c r="C389" s="0" t="s">
-        <v>838</v>
+        <v>16</v>
       </c>
       <c r="D389" s="0">
-        <v>3800</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="0" t="s">
+        <v>838</v>
+      </c>
+      <c r="B390" s="0" t="s">
         <v>839</v>
       </c>
-      <c r="B390" s="0" t="s">
+      <c r="C390" s="0" t="s">
         <v>840</v>
       </c>
-      <c r="C390" s="0" t="s">
-        <v>22</v>
-      </c>
       <c r="D390" s="0">
-        <v>353</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="391">
@@ -8729,10 +8735,10 @@
         <v>842</v>
       </c>
       <c r="C391" s="0" t="s">
-        <v>109</v>
+        <v>22</v>
       </c>
       <c r="D391" s="0">
-        <v>1800</v>
+        <v>353</v>
       </c>
     </row>
     <row r="392">
@@ -8743,10 +8749,10 @@
         <v>844</v>
       </c>
       <c r="C392" s="0" t="s">
-        <v>16</v>
+        <v>109</v>
       </c>
       <c r="D392" s="0">
-        <v>2948</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="393">
@@ -8757,10 +8763,10 @@
         <v>846</v>
       </c>
       <c r="C393" s="0" t="s">
-        <v>207</v>
+        <v>16</v>
       </c>
       <c r="D393" s="0">
-        <v>65537</v>
+        <v>2948</v>
       </c>
     </row>
     <row r="394">
@@ -8771,10 +8777,10 @@
         <v>848</v>
       </c>
       <c r="C394" s="0" t="s">
-        <v>137</v>
+        <v>207</v>
       </c>
       <c r="D394" s="0">
-        <v>4049.6</v>
+        <v>65537</v>
       </c>
     </row>
     <row r="395">
@@ -8788,7 +8794,7 @@
         <v>137</v>
       </c>
       <c r="D395" s="0">
-        <v>4199.2</v>
+        <v>4049.6</v>
       </c>
     </row>
     <row r="396">
@@ -8802,7 +8808,7 @@
         <v>137</v>
       </c>
       <c r="D396" s="0">
-        <v>6397.2</v>
+        <v>4199.2</v>
       </c>
     </row>
     <row r="397">
@@ -8813,10 +8819,10 @@
         <v>854</v>
       </c>
       <c r="C397" s="0" t="s">
-        <v>310</v>
+        <v>137</v>
       </c>
       <c r="D397" s="0">
-        <v>570</v>
+        <v>6397.2</v>
       </c>
     </row>
     <row r="398">
@@ -8827,10 +8833,10 @@
         <v>856</v>
       </c>
       <c r="C398" s="0" t="s">
-        <v>71</v>
+        <v>310</v>
       </c>
       <c r="D398" s="0">
-        <v>550</v>
+        <v>570</v>
       </c>
     </row>
     <row r="399">
@@ -8841,10 +8847,10 @@
         <v>858</v>
       </c>
       <c r="C399" s="0" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="D399" s="0">
-        <v>167</v>
+        <v>550</v>
       </c>
     </row>
     <row r="400">
@@ -8855,10 +8861,10 @@
         <v>860</v>
       </c>
       <c r="C400" s="0" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="D400" s="0">
-        <v>701.42</v>
+        <v>167</v>
       </c>
     </row>
     <row r="401">
@@ -8869,10 +8875,10 @@
         <v>862</v>
       </c>
       <c r="C401" s="0" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="D401" s="0">
-        <v>101000</v>
+        <v>714.74</v>
       </c>
     </row>
     <row r="402">
@@ -8883,10 +8889,10 @@
         <v>864</v>
       </c>
       <c r="C402" s="0" t="s">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="D402" s="0">
-        <v>6251</v>
+        <v>101000</v>
       </c>
     </row>
     <row r="403">
@@ -8897,10 +8903,10 @@
         <v>866</v>
       </c>
       <c r="C403" s="0" t="s">
-        <v>374</v>
+        <v>120</v>
       </c>
       <c r="D403" s="0">
-        <v>857.67</v>
+        <v>6251</v>
       </c>
     </row>
     <row r="404">
@@ -8911,10 +8917,10 @@
         <v>868</v>
       </c>
       <c r="C404" s="0" t="s">
-        <v>91</v>
+        <v>374</v>
       </c>
       <c r="D404" s="0">
-        <v>1164.66</v>
+        <v>857.67</v>
       </c>
     </row>
     <row r="405">
@@ -8925,10 +8931,10 @@
         <v>870</v>
       </c>
       <c r="C405" s="0" t="s">
-        <v>148</v>
+        <v>91</v>
       </c>
       <c r="D405" s="0">
-        <v>360</v>
+        <v>1164.66</v>
       </c>
     </row>
     <row r="406">
@@ -8942,7 +8948,7 @@
         <v>148</v>
       </c>
       <c r="D406" s="0">
-        <v>450</v>
+        <v>360</v>
       </c>
     </row>
     <row r="407">
@@ -8956,7 +8962,7 @@
         <v>148</v>
       </c>
       <c r="D407" s="0">
-        <v>2050</v>
+        <v>450</v>
       </c>
     </row>
     <row r="408">
@@ -8967,10 +8973,10 @@
         <v>876</v>
       </c>
       <c r="C408" s="0" t="s">
-        <v>578</v>
+        <v>148</v>
       </c>
       <c r="D408" s="0">
-        <v>25192.82</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="409">
@@ -8981,10 +8987,10 @@
         <v>878</v>
       </c>
       <c r="C409" s="0" t="s">
-        <v>71</v>
+        <v>580</v>
       </c>
       <c r="D409" s="0">
-        <v>3500</v>
+        <v>25192.82</v>
       </c>
     </row>
     <row r="410">
@@ -8995,10 +9001,10 @@
         <v>880</v>
       </c>
       <c r="C410" s="0" t="s">
-        <v>175</v>
+        <v>71</v>
       </c>
       <c r="D410" s="0">
-        <v>600</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="411">
@@ -9009,52 +9015,52 @@
         <v>882</v>
       </c>
       <c r="C411" s="0" t="s">
-        <v>883</v>
+        <v>175</v>
       </c>
       <c r="D411" s="0">
-        <v>1080</v>
+        <v>600</v>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="0" t="s">
+        <v>883</v>
+      </c>
+      <c r="B412" s="0" t="s">
         <v>884</v>
       </c>
-      <c r="B412" s="0" t="s">
+      <c r="C412" s="0" t="s">
         <v>885</v>
       </c>
-      <c r="C412" s="0" t="s">
+      <c r="D412" s="0">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="0" t="s">
+        <v>886</v>
+      </c>
+      <c r="B413" s="0" t="s">
+        <v>887</v>
+      </c>
+      <c r="C413" s="0" t="s">
         <v>338</v>
       </c>
-      <c r="D412" s="0">
+      <c r="D413" s="0">
         <v>8628</v>
       </c>
     </row>
-    <row r="413">
-      <c r="A413" s="2" t="s">
-        <v>886</v>
-      </c>
-      <c r="B413" s="2" t="s">
-        <v>887</v>
-      </c>
-      <c r="C413" s="2" t="s">
+    <row r="414">
+      <c r="A414" s="2" t="s">
+        <v>888</v>
+      </c>
+      <c r="B414" s="2" t="s">
+        <v>889</v>
+      </c>
+      <c r="C414" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="D413" s="2">
+      <c r="D414" s="2">
         <v>9125.1</v>
-      </c>
-    </row>
-    <row r="414">
-      <c r="A414" s="0" t="s">
-        <v>888</v>
-      </c>
-      <c r="B414" s="0" t="s">
-        <v>889</v>
-      </c>
-      <c r="C414" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="D414" s="0">
-        <v>27991.54</v>
       </c>
     </row>
     <row r="415">
@@ -9065,10 +9071,10 @@
         <v>891</v>
       </c>
       <c r="C415" s="0" t="s">
-        <v>137</v>
+        <v>41</v>
       </c>
       <c r="D415" s="0">
-        <v>1080</v>
+        <v>27991.54</v>
       </c>
     </row>
     <row r="416">
@@ -9082,7 +9088,7 @@
         <v>137</v>
       </c>
       <c r="D416" s="0">
-        <v>4012</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="417">
@@ -9093,10 +9099,10 @@
         <v>895</v>
       </c>
       <c r="C417" s="0" t="s">
-        <v>46</v>
+        <v>137</v>
       </c>
       <c r="D417" s="0">
-        <v>5816.9</v>
+        <v>4012</v>
       </c>
     </row>
     <row r="418">
@@ -9110,7 +9116,7 @@
         <v>46</v>
       </c>
       <c r="D418" s="0">
-        <v>2624.28</v>
+        <v>5816.9</v>
       </c>
     </row>
     <row r="419">
@@ -9124,35 +9130,35 @@
         <v>46</v>
       </c>
       <c r="D419" s="0">
+        <v>2624.28</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="0" t="s">
+        <v>900</v>
+      </c>
+      <c r="B420" s="0" t="s">
+        <v>901</v>
+      </c>
+      <c r="C420" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="D420" s="0">
         <v>1953.98</v>
       </c>
     </row>
-    <row r="420">
-      <c r="A420" s="2" t="s">
-        <v>900</v>
-      </c>
-      <c r="B420" s="2" t="s">
-        <v>901</v>
-      </c>
-      <c r="C420" s="2" t="s">
+    <row r="421">
+      <c r="A421" s="2" t="s">
+        <v>902</v>
+      </c>
+      <c r="B421" s="2" t="s">
+        <v>903</v>
+      </c>
+      <c r="C421" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D420" s="2">
+      <c r="D421" s="2">
         <v>3598.96</v>
-      </c>
-    </row>
-    <row r="421">
-      <c r="A421" s="0" t="s">
-        <v>902</v>
-      </c>
-      <c r="B421" s="0" t="s">
-        <v>903</v>
-      </c>
-      <c r="C421" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="D421" s="0">
-        <v>27318.17</v>
       </c>
     </row>
     <row r="422">
@@ -9166,7 +9172,7 @@
         <v>46</v>
       </c>
       <c r="D422" s="0">
-        <v>2115.26</v>
+        <v>27318.17</v>
       </c>
     </row>
     <row r="423">
@@ -9180,7 +9186,7 @@
         <v>46</v>
       </c>
       <c r="D423" s="0">
-        <v>4700</v>
+        <v>2115.26</v>
       </c>
     </row>
     <row r="424">
@@ -9194,7 +9200,7 @@
         <v>46</v>
       </c>
       <c r="D424" s="0">
-        <v>3750</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="425">
@@ -9205,10 +9211,10 @@
         <v>911</v>
       </c>
       <c r="C425" s="0" t="s">
-        <v>484</v>
+        <v>46</v>
       </c>
       <c r="D425" s="0">
-        <v>510</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="426">
@@ -9219,7 +9225,7 @@
         <v>913</v>
       </c>
       <c r="C426" s="0" t="s">
-        <v>38</v>
+        <v>484</v>
       </c>
       <c r="D426" s="0">
         <v>510</v>
@@ -9233,21 +9239,21 @@
         <v>915</v>
       </c>
       <c r="C427" s="0" t="s">
-        <v>916</v>
+        <v>38</v>
       </c>
       <c r="D427" s="0">
-        <v>580</v>
+        <v>510</v>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="0" t="s">
+        <v>916</v>
+      </c>
+      <c r="B428" s="0" t="s">
         <v>917</v>
       </c>
-      <c r="B428" s="0" t="s">
+      <c r="C428" s="0" t="s">
         <v>918</v>
-      </c>
-      <c r="C428" s="0" t="s">
-        <v>916</v>
       </c>
       <c r="D428" s="0">
         <v>580</v>
@@ -9261,7 +9267,7 @@
         <v>920</v>
       </c>
       <c r="C429" s="0" t="s">
-        <v>916</v>
+        <v>918</v>
       </c>
       <c r="D429" s="0">
         <v>580</v>
@@ -9275,10 +9281,10 @@
         <v>922</v>
       </c>
       <c r="C430" s="0" t="s">
-        <v>916</v>
+        <v>918</v>
       </c>
       <c r="D430" s="0">
-        <v>342</v>
+        <v>580</v>
       </c>
     </row>
     <row r="431">
@@ -9289,7 +9295,7 @@
         <v>924</v>
       </c>
       <c r="C431" s="0" t="s">
-        <v>916</v>
+        <v>918</v>
       </c>
       <c r="D431" s="0">
         <v>342</v>
@@ -9303,7 +9309,7 @@
         <v>926</v>
       </c>
       <c r="C432" s="0" t="s">
-        <v>916</v>
+        <v>918</v>
       </c>
       <c r="D432" s="0">
         <v>342</v>
@@ -9317,10 +9323,10 @@
         <v>928</v>
       </c>
       <c r="C433" s="0" t="s">
-        <v>916</v>
+        <v>918</v>
       </c>
       <c r="D433" s="0">
-        <v>0</v>
+        <v>342</v>
       </c>
     </row>
     <row r="434">
@@ -9331,7 +9337,7 @@
         <v>930</v>
       </c>
       <c r="C434" s="0" t="s">
-        <v>916</v>
+        <v>918</v>
       </c>
       <c r="D434" s="0">
         <v>0</v>
@@ -9345,10 +9351,10 @@
         <v>932</v>
       </c>
       <c r="C435" s="0" t="s">
-        <v>916</v>
+        <v>918</v>
       </c>
       <c r="D435" s="0">
-        <v>423</v>
+        <v>0</v>
       </c>
     </row>
     <row r="436">
@@ -9359,10 +9365,10 @@
         <v>934</v>
       </c>
       <c r="C436" s="0" t="s">
-        <v>71</v>
+        <v>918</v>
       </c>
       <c r="D436" s="0">
-        <v>15968</v>
+        <v>423</v>
       </c>
     </row>
     <row r="437">
@@ -9373,10 +9379,10 @@
         <v>936</v>
       </c>
       <c r="C437" s="0" t="s">
-        <v>35</v>
+        <v>71</v>
       </c>
       <c r="D437" s="0">
-        <v>430</v>
+        <v>15968</v>
       </c>
     </row>
     <row r="438">
@@ -9387,7 +9393,7 @@
         <v>938</v>
       </c>
       <c r="C438" s="0" t="s">
-        <v>283</v>
+        <v>35</v>
       </c>
       <c r="D438" s="0">
         <v>430</v>
@@ -9401,10 +9407,10 @@
         <v>940</v>
       </c>
       <c r="C439" s="0" t="s">
-        <v>114</v>
+        <v>283</v>
       </c>
       <c r="D439" s="0">
-        <v>14000</v>
+        <v>430</v>
       </c>
     </row>
     <row r="440">
@@ -9415,10 +9421,10 @@
         <v>942</v>
       </c>
       <c r="C440" s="0" t="s">
-        <v>137</v>
+        <v>114</v>
       </c>
       <c r="D440" s="0">
-        <v>14001</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="441">
@@ -9429,10 +9435,10 @@
         <v>944</v>
       </c>
       <c r="C441" s="0" t="s">
-        <v>91</v>
+        <v>137</v>
       </c>
       <c r="D441" s="0">
-        <v>266200</v>
+        <v>14001</v>
       </c>
     </row>
     <row r="442">
@@ -9446,7 +9452,7 @@
         <v>91</v>
       </c>
       <c r="D442" s="0">
-        <v>194991.5</v>
+        <v>266200</v>
       </c>
     </row>
     <row r="443">
@@ -9460,7 +9466,7 @@
         <v>91</v>
       </c>
       <c r="D443" s="0">
-        <v>289492.5</v>
+        <v>194991.5</v>
       </c>
     </row>
     <row r="444">
@@ -9471,24 +9477,24 @@
         <v>950</v>
       </c>
       <c r="C444" s="0" t="s">
-        <v>951</v>
+        <v>91</v>
       </c>
       <c r="D444" s="0">
-        <v>13722.52</v>
+        <v>289492.5</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="0" t="s">
+        <v>951</v>
+      </c>
+      <c r="B445" s="0" t="s">
         <v>952</v>
       </c>
-      <c r="B445" s="0" t="s">
+      <c r="C445" s="0" t="s">
         <v>953</v>
       </c>
-      <c r="C445" s="0" t="s">
-        <v>951</v>
-      </c>
       <c r="D445" s="0">
-        <v>15072</v>
+        <v>13722.52</v>
       </c>
     </row>
     <row r="446">
@@ -9499,10 +9505,10 @@
         <v>955</v>
       </c>
       <c r="C446" s="0" t="s">
-        <v>951</v>
+        <v>953</v>
       </c>
       <c r="D446" s="0">
-        <v>6555.64</v>
+        <v>15072</v>
       </c>
     </row>
     <row r="447">
@@ -9513,10 +9519,10 @@
         <v>957</v>
       </c>
       <c r="C447" s="0" t="s">
-        <v>951</v>
+        <v>953</v>
       </c>
       <c r="D447" s="0">
-        <v>8964.61</v>
+        <v>6555.64</v>
       </c>
     </row>
     <row r="448">
@@ -9527,10 +9533,10 @@
         <v>959</v>
       </c>
       <c r="C448" s="0" t="s">
-        <v>951</v>
+        <v>953</v>
       </c>
       <c r="D448" s="0">
-        <v>11735</v>
+        <v>8964.61</v>
       </c>
     </row>
     <row r="449">
@@ -9541,10 +9547,10 @@
         <v>961</v>
       </c>
       <c r="C449" s="0" t="s">
-        <v>71</v>
+        <v>953</v>
       </c>
       <c r="D449" s="0">
-        <v>3380</v>
+        <v>11735</v>
       </c>
     </row>
     <row r="450">
@@ -9555,10 +9561,10 @@
         <v>963</v>
       </c>
       <c r="C450" s="0" t="s">
-        <v>137</v>
+        <v>71</v>
       </c>
       <c r="D450" s="0">
-        <v>3750</v>
+        <v>3380</v>
       </c>
     </row>
     <row r="451">
@@ -9569,10 +9575,10 @@
         <v>965</v>
       </c>
       <c r="C451" s="0" t="s">
-        <v>91</v>
+        <v>137</v>
       </c>
       <c r="D451" s="0">
-        <v>4392.3</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="452">
@@ -9583,24 +9589,24 @@
         <v>967</v>
       </c>
       <c r="C452" s="0" t="s">
-        <v>968</v>
+        <v>91</v>
       </c>
       <c r="D452" s="0">
-        <v>5254.41</v>
+        <v>4392.3</v>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="0" t="s">
+        <v>968</v>
+      </c>
+      <c r="B453" s="0" t="s">
         <v>969</v>
       </c>
-      <c r="B453" s="0" t="s">
+      <c r="C453" s="0" t="s">
         <v>970</v>
       </c>
-      <c r="C453" s="0" t="s">
-        <v>53</v>
-      </c>
       <c r="D453" s="0">
-        <v>1200</v>
+        <v>5254.41</v>
       </c>
     </row>
     <row r="454">
@@ -9614,7 +9620,7 @@
         <v>53</v>
       </c>
       <c r="D454" s="0">
-        <v>278</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="455">
@@ -9628,7 +9634,7 @@
         <v>53</v>
       </c>
       <c r="D455" s="0">
-        <v>562</v>
+        <v>278</v>
       </c>
     </row>
     <row r="456">
@@ -9639,10 +9645,10 @@
         <v>976</v>
       </c>
       <c r="C456" s="0" t="s">
-        <v>374</v>
+        <v>53</v>
       </c>
       <c r="D456" s="0">
-        <v>65142.6</v>
+        <v>562</v>
       </c>
     </row>
     <row r="457">
@@ -9656,7 +9662,7 @@
         <v>374</v>
       </c>
       <c r="D457" s="0">
-        <v>23482.7</v>
+        <v>65142.6</v>
       </c>
     </row>
     <row r="458">
@@ -9667,10 +9673,10 @@
         <v>980</v>
       </c>
       <c r="C458" s="0" t="s">
-        <v>29</v>
+        <v>374</v>
       </c>
       <c r="D458" s="0">
-        <v>5917.17</v>
+        <v>23482.7</v>
       </c>
     </row>
     <row r="459">
@@ -9681,10 +9687,10 @@
         <v>982</v>
       </c>
       <c r="C459" s="0" t="s">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="D459" s="0">
-        <v>10985</v>
+        <v>6029.59</v>
       </c>
     </row>
     <row r="460">
@@ -9698,7 +9704,7 @@
         <v>53</v>
       </c>
       <c r="D460" s="0">
-        <v>17425</v>
+        <v>10985</v>
       </c>
     </row>
     <row r="461">
@@ -9709,38 +9715,38 @@
         <v>986</v>
       </c>
       <c r="C461" s="0" t="s">
-        <v>987</v>
+        <v>53</v>
       </c>
       <c r="D461" s="0">
-        <v>1958</v>
+        <v>17425</v>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="0" t="s">
+        <v>987</v>
+      </c>
+      <c r="B462" s="0" t="s">
         <v>988</v>
       </c>
-      <c r="B462" s="0" t="s">
+      <c r="C462" s="0" t="s">
         <v>989</v>
       </c>
-      <c r="C462" s="0" t="s">
-        <v>990</v>
-      </c>
       <c r="D462" s="0">
-        <v>385.4</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="0" t="s">
+        <v>990</v>
+      </c>
+      <c r="B463" s="0" t="s">
         <v>991</v>
       </c>
-      <c r="B463" s="0" t="s">
+      <c r="C463" s="0" t="s">
         <v>992</v>
       </c>
-      <c r="C463" s="0" t="s">
-        <v>91</v>
-      </c>
       <c r="D463" s="0">
-        <v>296147.5</v>
+        <v>385.4</v>
       </c>
     </row>
     <row r="464">
@@ -9751,10 +9757,10 @@
         <v>994</v>
       </c>
       <c r="C464" s="0" t="s">
-        <v>578</v>
+        <v>91</v>
       </c>
       <c r="D464" s="0">
-        <v>71176.4</v>
+        <v>296147.5</v>
       </c>
     </row>
     <row r="465">
@@ -9765,10 +9771,10 @@
         <v>996</v>
       </c>
       <c r="C465" s="0" t="s">
-        <v>137</v>
+        <v>580</v>
       </c>
       <c r="D465" s="0">
-        <v>96</v>
+        <v>71176.4</v>
       </c>
     </row>
     <row r="466">
@@ -9779,10 +9785,10 @@
         <v>998</v>
       </c>
       <c r="C466" s="0" t="s">
-        <v>71</v>
+        <v>137</v>
       </c>
       <c r="D466" s="0">
-        <v>950</v>
+        <v>96</v>
       </c>
     </row>
     <row r="467">
@@ -9793,10 +9799,10 @@
         <v>1000</v>
       </c>
       <c r="C467" s="0" t="s">
-        <v>475</v>
+        <v>71</v>
       </c>
       <c r="D467" s="0">
-        <v>342641</v>
+        <v>950</v>
       </c>
     </row>
     <row r="468">
@@ -9807,10 +9813,10 @@
         <v>1002</v>
       </c>
       <c r="C468" s="0" t="s">
-        <v>155</v>
+        <v>475</v>
       </c>
       <c r="D468" s="0">
-        <v>2200</v>
+        <v>342641</v>
       </c>
     </row>
     <row r="469">
@@ -9821,10 +9827,10 @@
         <v>1004</v>
       </c>
       <c r="C469" s="0" t="s">
-        <v>484</v>
+        <v>155</v>
       </c>
       <c r="D469" s="0">
-        <v>41000</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="470">
@@ -9835,10 +9841,10 @@
         <v>1006</v>
       </c>
       <c r="C470" s="0" t="s">
-        <v>71</v>
+        <v>484</v>
       </c>
       <c r="D470" s="0">
-        <v>9299</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="471">
@@ -9849,10 +9855,10 @@
         <v>1008</v>
       </c>
       <c r="C471" s="0" t="s">
-        <v>916</v>
+        <v>71</v>
       </c>
       <c r="D471" s="0">
-        <v>825</v>
+        <v>9299</v>
       </c>
     </row>
     <row r="472">
@@ -9863,7 +9869,7 @@
         <v>1010</v>
       </c>
       <c r="C472" s="0" t="s">
-        <v>916</v>
+        <v>918</v>
       </c>
       <c r="D472" s="0">
         <v>825</v>
@@ -9877,7 +9883,7 @@
         <v>1012</v>
       </c>
       <c r="C473" s="0" t="s">
-        <v>916</v>
+        <v>918</v>
       </c>
       <c r="D473" s="0">
         <v>825</v>
@@ -9891,10 +9897,10 @@
         <v>1014</v>
       </c>
       <c r="C474" s="0" t="s">
-        <v>22</v>
+        <v>918</v>
       </c>
       <c r="D474" s="0">
-        <v>563.36</v>
+        <v>825</v>
       </c>
     </row>
     <row r="475">
@@ -9905,10 +9911,10 @@
         <v>1016</v>
       </c>
       <c r="C475" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D475" s="0">
-        <v>3520</v>
+        <v>563.36</v>
       </c>
     </row>
     <row r="476">
@@ -9922,7 +9928,7 @@
         <v>16</v>
       </c>
       <c r="D476" s="0">
-        <v>2600</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="477">
@@ -9933,10 +9939,10 @@
         <v>1020</v>
       </c>
       <c r="C477" s="0" t="s">
-        <v>283</v>
+        <v>16</v>
       </c>
       <c r="D477" s="0">
-        <v>3700</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="478">
@@ -9950,7 +9956,7 @@
         <v>283</v>
       </c>
       <c r="D478" s="0">
-        <v>2600</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="479">
@@ -9961,10 +9967,10 @@
         <v>1024</v>
       </c>
       <c r="C479" s="0" t="s">
-        <v>16</v>
+        <v>283</v>
       </c>
       <c r="D479" s="0">
-        <v>2235</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="480">
@@ -9978,35 +9984,35 @@
         <v>16</v>
       </c>
       <c r="D480" s="0">
-        <v>3850</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="0" t="s">
-        <v>395</v>
+        <v>1027</v>
       </c>
       <c r="B481" s="0" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="C481" s="0" t="s">
-        <v>1028</v>
+        <v>16</v>
       </c>
       <c r="D481" s="0">
-        <v>1</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="0" t="s">
+        <v>395</v>
+      </c>
+      <c r="B482" s="0" t="s">
         <v>1029</v>
       </c>
-      <c r="B482" s="0" t="s">
+      <c r="C482" s="0" t="s">
         <v>1030</v>
       </c>
-      <c r="C482" s="0" t="s">
-        <v>29</v>
-      </c>
       <c r="D482" s="0">
-        <v>13715</v>
+        <v>1</v>
       </c>
     </row>
     <row r="483">
@@ -10017,10 +10023,10 @@
         <v>1032</v>
       </c>
       <c r="C483" s="0" t="s">
-        <v>374</v>
+        <v>29</v>
       </c>
       <c r="D483" s="0">
-        <v>3859.93</v>
+        <v>14819</v>
       </c>
     </row>
     <row r="484">
@@ -10034,7 +10040,7 @@
         <v>374</v>
       </c>
       <c r="D484" s="0">
-        <v>11751.49</v>
+        <v>3859.93</v>
       </c>
     </row>
     <row r="485">
@@ -10045,10 +10051,10 @@
         <v>1036</v>
       </c>
       <c r="C485" s="0" t="s">
-        <v>338</v>
+        <v>374</v>
       </c>
       <c r="D485" s="0">
-        <v>6000</v>
+        <v>11751.49</v>
       </c>
     </row>
     <row r="486">
@@ -10062,7 +10068,7 @@
         <v>338</v>
       </c>
       <c r="D486" s="0">
-        <v>3000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="487">
@@ -10073,10 +10079,10 @@
         <v>1040</v>
       </c>
       <c r="C487" s="0" t="s">
-        <v>38</v>
+        <v>338</v>
       </c>
       <c r="D487" s="0">
-        <v>618</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="488">
@@ -10087,24 +10093,24 @@
         <v>1042</v>
       </c>
       <c r="C488" s="0" t="s">
-        <v>1043</v>
+        <v>38</v>
       </c>
       <c r="D488" s="0">
-        <v>24600</v>
+        <v>618</v>
       </c>
     </row>
     <row r="489">
       <c r="A489" s="0" t="s">
+        <v>1043</v>
+      </c>
+      <c r="B489" s="0" t="s">
         <v>1044</v>
       </c>
-      <c r="B489" s="0" t="s">
+      <c r="C489" s="0" t="s">
         <v>1045</v>
       </c>
-      <c r="C489" s="0" t="s">
-        <v>104</v>
-      </c>
       <c r="D489" s="0">
-        <v>0</v>
+        <v>24600</v>
       </c>
     </row>
     <row r="490">
@@ -10115,10 +10121,10 @@
         <v>1047</v>
       </c>
       <c r="C490" s="0" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="D490" s="0">
-        <v>40928.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="491">
@@ -10129,10 +10135,10 @@
         <v>1049</v>
       </c>
       <c r="C491" s="0" t="s">
-        <v>374</v>
+        <v>91</v>
       </c>
       <c r="D491" s="0">
-        <v>75529.71</v>
+        <v>40928.25</v>
       </c>
     </row>
     <row r="492">
@@ -10146,7 +10152,7 @@
         <v>374</v>
       </c>
       <c r="D492" s="0">
-        <v>41613.42</v>
+        <v>75529.71</v>
       </c>
     </row>
     <row r="493">
@@ -10160,7 +10166,7 @@
         <v>374</v>
       </c>
       <c r="D493" s="0">
-        <v>87056.42</v>
+        <v>41613.42</v>
       </c>
     </row>
     <row r="494">
@@ -10174,7 +10180,7 @@
         <v>374</v>
       </c>
       <c r="D494" s="0">
-        <v>49243.16</v>
+        <v>87056.42</v>
       </c>
     </row>
     <row r="495">
@@ -10185,10 +10191,10 @@
         <v>1057</v>
       </c>
       <c r="C495" s="0" t="s">
-        <v>22</v>
+        <v>374</v>
       </c>
       <c r="D495" s="0">
-        <v>1600</v>
+        <v>49243.16</v>
       </c>
     </row>
     <row r="496">
@@ -10199,10 +10205,10 @@
         <v>1059</v>
       </c>
       <c r="C496" s="0" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D496" s="0">
-        <v>3338.9</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="497">
@@ -10216,7 +10222,7 @@
         <v>29</v>
       </c>
       <c r="D497" s="0">
-        <v>3987</v>
+        <v>3455.8</v>
       </c>
     </row>
     <row r="498">
@@ -10230,7 +10236,7 @@
         <v>29</v>
       </c>
       <c r="D498" s="0">
-        <v>4010.17</v>
+        <v>3987</v>
       </c>
     </row>
     <row r="499">
@@ -10244,35 +10250,35 @@
         <v>29</v>
       </c>
       <c r="D499" s="0">
+        <v>4010.17</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="0" t="s">
+        <v>1066</v>
+      </c>
+      <c r="B500" s="0" t="s">
+        <v>1067</v>
+      </c>
+      <c r="C500" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D500" s="0">
         <v>3382.65</v>
       </c>
     </row>
-    <row r="500">
-      <c r="A500" s="2" t="s">
-        <v>1066</v>
-      </c>
-      <c r="B500" s="2" t="s">
-        <v>1067</v>
-      </c>
-      <c r="C500" s="2" t="s">
+    <row r="501">
+      <c r="A501" s="2" t="s">
+        <v>1068</v>
+      </c>
+      <c r="B501" s="2" t="s">
+        <v>1069</v>
+      </c>
+      <c r="C501" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D500" s="2">
+      <c r="D501" s="2">
         <v>0</v>
-      </c>
-    </row>
-    <row r="501">
-      <c r="A501" s="0" t="s">
-        <v>1068</v>
-      </c>
-      <c r="B501" s="0" t="s">
-        <v>1069</v>
-      </c>
-      <c r="C501" s="0" t="s">
-        <v>155</v>
-      </c>
-      <c r="D501" s="0">
-        <v>430</v>
       </c>
     </row>
     <row r="502">
@@ -10283,9 +10289,23 @@
         <v>1071</v>
       </c>
       <c r="C502" s="0" t="s">
+        <v>155</v>
+      </c>
+      <c r="D502" s="0">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="0" t="s">
+        <v>1072</v>
+      </c>
+      <c r="B503" s="0" t="s">
+        <v>1073</v>
+      </c>
+      <c r="C503" s="0" t="s">
         <v>137</v>
       </c>
-      <c r="D502" s="0">
+      <c r="D503" s="0">
         <v>462</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: stock y precios actualizados jue. 23/07/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="1074">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1080" uniqueCount="1080">
   <si>
     <t>Código</t>
   </si>
@@ -1808,6 +1808,15 @@
     <t>JERINGA 1 ML EUROMIX - 000024331</t>
   </si>
   <si>
+    <t>000024702</t>
+  </si>
+  <si>
+    <t>JERINGA 10 ML - KANGJIN - 000024702</t>
+  </si>
+  <si>
+    <t>KANGJIN</t>
+  </si>
+  <si>
     <t>000023732</t>
   </si>
   <si>
@@ -2811,6 +2820,15 @@
   </si>
   <si>
     <t>SONDA T/K 97 PVC EST NELATON Nº 10 WELL LEAD - 000023933</t>
+  </si>
+  <si>
+    <t>000024703</t>
+  </si>
+  <si>
+    <t>SONDA T/K PVC EST BIGOTERA ADULTO - KANGYUAN - 000024703</t>
+  </si>
+  <si>
+    <t>KANGYUAN</t>
   </si>
   <si>
     <t>000023832</t>
@@ -3292,7 +3310,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A3:D503"/>
+  <dimension ref="A3:D505"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="3">
@@ -3530,7 +3548,7 @@
         <v>46</v>
       </c>
       <c r="D19" s="0">
-        <v>3532.97</v>
+        <v>3853.77</v>
       </c>
     </row>
     <row r="20">
@@ -3558,7 +3576,7 @@
         <v>46</v>
       </c>
       <c r="D21" s="0">
-        <v>28000</v>
+        <v>32000</v>
       </c>
     </row>
     <row r="22">
@@ -4804,7 +4822,7 @@
         <v>46</v>
       </c>
       <c r="D110" s="0">
-        <v>5291.87</v>
+        <v>5772.37</v>
       </c>
     </row>
     <row r="111">
@@ -6078,7 +6096,7 @@
         <v>46</v>
       </c>
       <c r="D201" s="0">
-        <v>4336.22</v>
+        <v>4729.95</v>
       </c>
     </row>
     <row r="202">
@@ -7083,7 +7101,7 @@
         <v>599</v>
       </c>
       <c r="C273" s="0" t="s">
-        <v>53</v>
+        <v>600</v>
       </c>
       <c r="D273" s="0">
         <v>65</v>
@@ -7091,97 +7109,97 @@
     </row>
     <row r="274">
       <c r="A274" s="0" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="B274" s="0" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="C274" s="0" t="s">
         <v>53</v>
       </c>
       <c r="D274" s="0">
-        <v>92</v>
+        <v>65</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="0" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B275" s="0" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="C275" s="0" t="s">
         <v>53</v>
       </c>
       <c r="D275" s="0">
-        <v>33</v>
+        <v>92</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="0" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="B276" s="0" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="C276" s="0" t="s">
         <v>53</v>
       </c>
       <c r="D276" s="0">
-        <v>38.22</v>
+        <v>33</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="0" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="B277" s="0" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="C277" s="0" t="s">
-        <v>338</v>
+        <v>53</v>
       </c>
       <c r="D277" s="0">
-        <v>300</v>
+        <v>38.22</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="0" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="B278" s="0" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="C278" s="0" t="s">
         <v>338</v>
       </c>
       <c r="D278" s="0">
-        <v>370</v>
+        <v>300</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="0" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B279" s="0" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="C279" s="0" t="s">
-        <v>359</v>
+        <v>338</v>
       </c>
       <c r="D279" s="0">
-        <v>450</v>
+        <v>370</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="0" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="B280" s="0" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="C280" s="0" t="s">
-        <v>38</v>
+        <v>359</v>
       </c>
       <c r="D280" s="0">
         <v>450</v>
@@ -7189,13 +7207,13 @@
     </row>
     <row r="281">
       <c r="A281" s="0" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="B281" s="0" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="C281" s="0" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="D281" s="0">
         <v>450</v>
@@ -7203,282 +7221,282 @@
     </row>
     <row r="282">
       <c r="A282" s="0" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="B282" s="0" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="C282" s="0" t="s">
         <v>16</v>
       </c>
       <c r="D282" s="0">
-        <v>1650</v>
+        <v>450</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="0" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="B283" s="0" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="C283" s="0" t="s">
         <v>16</v>
       </c>
       <c r="D283" s="0">
-        <v>2100</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="0" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B284" s="0" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="C284" s="0" t="s">
         <v>16</v>
       </c>
       <c r="D284" s="0">
-        <v>1980</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="0" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B285" s="0" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="C285" s="0" t="s">
         <v>16</v>
       </c>
       <c r="D285" s="0">
-        <v>2160</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="0" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B286" s="0" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="C286" s="0" t="s">
         <v>16</v>
       </c>
       <c r="D286" s="0">
-        <v>1100</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="0" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="B287" s="0" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="C287" s="0" t="s">
         <v>16</v>
       </c>
       <c r="D287" s="0">
-        <v>2600</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="0" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="B288" s="0" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="C288" s="0" t="s">
         <v>16</v>
       </c>
       <c r="D288" s="0">
-        <v>2000</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="0" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="B289" s="0" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="C289" s="0" t="s">
         <v>16</v>
       </c>
       <c r="D289" s="0">
-        <v>6700</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="0" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="B290" s="0" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="C290" s="0" t="s">
         <v>16</v>
       </c>
       <c r="D290" s="0">
-        <v>1650</v>
+        <v>6700</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="0" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="B291" s="0" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="C291" s="0" t="s">
         <v>16</v>
       </c>
       <c r="D291" s="0">
-        <v>1035</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="0" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B292" s="0" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="C292" s="0" t="s">
         <v>16</v>
       </c>
       <c r="D292" s="0">
-        <v>2600</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="0" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B293" s="0" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C293" s="0" t="s">
         <v>16</v>
       </c>
       <c r="D293" s="0">
-        <v>2400</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="0" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="B294" s="0" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="C294" s="0" t="s">
-        <v>137</v>
+        <v>16</v>
       </c>
       <c r="D294" s="0">
-        <v>4497.2</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="0" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="B295" s="0" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="C295" s="0" t="s">
         <v>137</v>
       </c>
       <c r="D295" s="0">
-        <v>2328</v>
+        <v>4497.2</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="0" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B296" s="0" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="C296" s="0" t="s">
         <v>137</v>
       </c>
       <c r="D296" s="0">
-        <v>1138</v>
+        <v>2328</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="0" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B297" s="0" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C297" s="0" t="s">
-        <v>29</v>
+        <v>137</v>
       </c>
       <c r="D297" s="0">
-        <v>7372.42</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="0" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B298" s="0" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="C298" s="0" t="s">
-        <v>120</v>
+        <v>29</v>
       </c>
       <c r="D298" s="0">
-        <v>1790</v>
+        <v>7372.42</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="0" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B299" s="0" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="C299" s="0" t="s">
         <v>120</v>
       </c>
       <c r="D299" s="0">
-        <v>2859.96</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="0" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B300" s="0" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="C300" s="0" t="s">
         <v>120</v>
       </c>
       <c r="D300" s="0">
-        <v>4800</v>
+        <v>2859.96</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="0" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="B301" s="0" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C301" s="0" t="s">
-        <v>656</v>
+        <v>120</v>
       </c>
       <c r="D301" s="0">
-        <v>0</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="302">
@@ -7489,130 +7507,130 @@
         <v>658</v>
       </c>
       <c r="C302" s="0" t="s">
-        <v>29</v>
+        <v>659</v>
       </c>
       <c r="D302" s="0">
-        <v>494</v>
+        <v>0</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="0" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B303" s="0" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="C303" s="0" t="s">
         <v>29</v>
       </c>
       <c r="D303" s="0">
-        <v>665.3</v>
+        <v>494</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="0" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B304" s="0" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="C304" s="0" t="s">
-        <v>91</v>
+        <v>29</v>
       </c>
       <c r="D304" s="0">
-        <v>33275</v>
+        <v>665.3</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="0" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="B305" s="0" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="C305" s="0" t="s">
         <v>91</v>
       </c>
       <c r="D305" s="0">
-        <v>4525.4</v>
+        <v>33275</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="0" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B306" s="0" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="C306" s="0" t="s">
-        <v>148</v>
+        <v>91</v>
       </c>
       <c r="D306" s="0">
-        <v>896</v>
+        <v>4525.4</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="0" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B307" s="0" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="C307" s="0" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="D307" s="0">
-        <v>1250</v>
+        <v>896</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="0" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="B308" s="0" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="C308" s="0" t="s">
-        <v>91</v>
+        <v>137</v>
       </c>
       <c r="D308" s="0">
-        <v>312785</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="0" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B309" s="0" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="C309" s="0" t="s">
-        <v>202</v>
+        <v>91</v>
       </c>
       <c r="D309" s="0">
-        <v>17440</v>
+        <v>312785</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="0" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B310" s="0" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="C310" s="0" t="s">
         <v>202</v>
       </c>
       <c r="D310" s="0">
-        <v>4390</v>
+        <v>17440</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="0" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="B311" s="0" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="C311" s="0" t="s">
         <v>202</v>
@@ -7623,128 +7641,128 @@
     </row>
     <row r="312">
       <c r="A312" s="0" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="B312" s="0" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="C312" s="0" t="s">
-        <v>283</v>
+        <v>202</v>
       </c>
       <c r="D312" s="0">
-        <v>2250</v>
+        <v>4390</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="0" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B313" s="0" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="C313" s="0" t="s">
-        <v>202</v>
+        <v>283</v>
       </c>
       <c r="D313" s="0">
-        <v>3355</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="0" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="B314" s="0" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="C314" s="0" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="D314" s="0">
-        <v>7500</v>
+        <v>3355</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="0" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B315" s="0" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C315" s="0" t="s">
-        <v>91</v>
+        <v>207</v>
       </c>
       <c r="D315" s="0">
-        <v>23958</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="0" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="B316" s="0" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="C316" s="0" t="s">
         <v>91</v>
       </c>
       <c r="D316" s="0">
-        <v>239580</v>
+        <v>23958</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="0" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B317" s="0" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="C317" s="0" t="s">
-        <v>53</v>
+        <v>91</v>
       </c>
       <c r="D317" s="0">
-        <v>130</v>
+        <v>239580</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="0" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="B318" s="0" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="C318" s="0" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="D318" s="0">
-        <v>285.6</v>
+        <v>130</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="0" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B319" s="0" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="C319" s="0" t="s">
         <v>22</v>
       </c>
       <c r="D319" s="0">
-        <v>338</v>
+        <v>285.6</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="0" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B320" s="0" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="C320" s="0" t="s">
-        <v>695</v>
+        <v>22</v>
       </c>
       <c r="D320" s="0">
-        <v>770</v>
+        <v>338</v>
       </c>
     </row>
     <row r="321">
@@ -7769,245 +7787,245 @@
         <v>700</v>
       </c>
       <c r="C322" s="0" t="s">
-        <v>16</v>
+        <v>701</v>
       </c>
       <c r="D322" s="0">
-        <v>973.5</v>
+        <v>770</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="0" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B323" s="0" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="C323" s="0" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D323" s="0">
-        <v>507.08</v>
+        <v>973.5</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="0" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B324" s="0" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="C324" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D324" s="0">
-        <v>450</v>
+        <v>507.08</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="0" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="B325" s="0" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="C325" s="0" t="s">
-        <v>148</v>
+        <v>16</v>
       </c>
       <c r="D325" s="0">
-        <v>760</v>
+        <v>450</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="0" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B326" s="0" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="C326" s="0" t="s">
-        <v>283</v>
+        <v>148</v>
       </c>
       <c r="D326" s="0">
-        <v>5900</v>
+        <v>760</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="0" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B327" s="0" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="C327" s="0" t="s">
         <v>283</v>
       </c>
       <c r="D327" s="0">
-        <v>2900</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="0" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B328" s="0" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="C328" s="0" t="s">
-        <v>137</v>
+        <v>283</v>
       </c>
       <c r="D328" s="0">
-        <v>886.2</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="0" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B329" s="0" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="C329" s="0" t="s">
         <v>137</v>
       </c>
       <c r="D329" s="0">
-        <v>589.9</v>
+        <v>886.2</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="0" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B330" s="0" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="C330" s="0" t="s">
         <v>137</v>
       </c>
       <c r="D330" s="0">
-        <v>65</v>
+        <v>589.9</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="0" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B331" s="0" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="C331" s="0" t="s">
-        <v>91</v>
+        <v>137</v>
       </c>
       <c r="D331" s="0">
-        <v>11313.5</v>
+        <v>65</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="0" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B332" s="0" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="C332" s="0" t="s">
-        <v>35</v>
+        <v>91</v>
       </c>
       <c r="D332" s="0">
-        <v>420</v>
+        <v>11313.5</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="0" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B333" s="0" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="C333" s="0" t="s">
-        <v>359</v>
+        <v>35</v>
       </c>
       <c r="D333" s="0">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="0" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B334" s="0" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="C334" s="0" t="s">
-        <v>22</v>
+        <v>359</v>
       </c>
       <c r="D334" s="0">
-        <v>377</v>
+        <v>418</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="0" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B335" s="0" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="C335" s="0" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="D335" s="0">
-        <v>5300</v>
+        <v>377</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="0" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B336" s="0" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="C336" s="0" t="s">
-        <v>71</v>
+        <v>46</v>
       </c>
       <c r="D336" s="0">
-        <v>898</v>
+        <v>5781.24</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="0" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B337" s="0" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="C337" s="0" t="s">
-        <v>120</v>
+        <v>71</v>
       </c>
       <c r="D337" s="0">
-        <v>4767</v>
+        <v>898</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="0" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="B338" s="0" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="C338" s="0" t="s">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="D338" s="0">
-        <v>650</v>
+        <v>4767</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="0" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B339" s="0" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="C339" s="0" t="s">
-        <v>71</v>
+        <v>35</v>
       </c>
       <c r="D339" s="0">
         <v>650</v>
@@ -8015,44 +8033,44 @@
     </row>
     <row r="340">
       <c r="A340" s="0" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B340" s="0" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="C340" s="0" t="s">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="D340" s="0">
-        <v>2178</v>
+        <v>650</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="0" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B341" s="0" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="C341" s="0" t="s">
-        <v>91</v>
+        <v>16</v>
       </c>
       <c r="D341" s="0">
-        <v>7986</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="0" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B342" s="0" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="C342" s="0" t="s">
-        <v>741</v>
+        <v>91</v>
       </c>
       <c r="D342" s="0">
-        <v>1910</v>
+        <v>7986</v>
       </c>
     </row>
     <row r="343">
@@ -8063,340 +8081,340 @@
         <v>743</v>
       </c>
       <c r="C343" s="0" t="s">
-        <v>148</v>
+        <v>744</v>
       </c>
       <c r="D343" s="0">
-        <v>900</v>
+        <v>1910</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="0" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B344" s="0" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="C344" s="0" t="s">
-        <v>22</v>
+        <v>148</v>
       </c>
       <c r="D344" s="0">
-        <v>1722</v>
+        <v>900</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="0" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B345" s="0" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="C345" s="0" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="D345" s="0">
-        <v>456</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" s="0" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B346" s="0" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="C346" s="0" t="s">
         <v>35</v>
       </c>
       <c r="D346" s="0">
-        <v>59000</v>
+        <v>456</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" s="0" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B347" s="0" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="C347" s="0" t="s">
-        <v>148</v>
+        <v>35</v>
       </c>
       <c r="D347" s="0">
-        <v>750</v>
+        <v>59000</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" s="0" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B348" s="0" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="C348" s="0" t="s">
         <v>148</v>
       </c>
       <c r="D348" s="0">
-        <v>1212</v>
+        <v>750</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="0" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B349" s="0" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="C349" s="0" t="s">
         <v>148</v>
       </c>
       <c r="D349" s="0">
-        <v>1300</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" s="0" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B350" s="0" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="C350" s="0" t="s">
         <v>148</v>
       </c>
       <c r="D350" s="0">
-        <v>1500</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="0" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B351" s="0" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="C351" s="0" t="s">
         <v>148</v>
       </c>
       <c r="D351" s="0">
-        <v>1400</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" s="0" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="B352" s="0" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="C352" s="0" t="s">
-        <v>259</v>
+        <v>148</v>
       </c>
       <c r="D352" s="0">
-        <v>11959</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="0" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B353" s="0" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="C353" s="0" t="s">
-        <v>137</v>
+        <v>259</v>
       </c>
       <c r="D353" s="0">
-        <v>345</v>
+        <v>11959</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="0" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="B354" s="0" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="C354" s="0" t="s">
-        <v>283</v>
+        <v>137</v>
       </c>
       <c r="D354" s="0">
-        <v>1450</v>
+        <v>345</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="0" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="B355" s="0" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="C355" s="0" t="s">
-        <v>91</v>
+        <v>283</v>
       </c>
       <c r="D355" s="0">
-        <v>7320.5</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" s="0" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="B356" s="0" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="C356" s="0" t="s">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="D356" s="0">
-        <v>900</v>
+        <v>7320.5</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="0" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="B357" s="0" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="C357" s="0" t="s">
-        <v>283</v>
+        <v>16</v>
       </c>
       <c r="D357" s="0">
-        <v>520</v>
+        <v>900</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="0" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="B358" s="0" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="C358" s="0" t="s">
-        <v>475</v>
+        <v>283</v>
       </c>
       <c r="D358" s="0">
-        <v>64925</v>
+        <v>520</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="0" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="B359" s="0" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="C359" s="0" t="s">
-        <v>16</v>
+        <v>475</v>
       </c>
       <c r="D359" s="0">
-        <v>1100</v>
+        <v>64925</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="0" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="B360" s="0" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="C360" s="0" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D360" s="0">
-        <v>1623</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="0" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="B361" s="0" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="C361" s="0" t="s">
-        <v>137</v>
+        <v>22</v>
       </c>
       <c r="D361" s="0">
-        <v>1182.75</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="0" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="B362" s="0" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="C362" s="0" t="s">
         <v>137</v>
       </c>
       <c r="D362" s="0">
-        <v>4440.9</v>
+        <v>1182.75</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="0" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="B363" s="0" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="C363" s="0" t="s">
-        <v>29</v>
+        <v>137</v>
       </c>
       <c r="D363" s="0">
-        <v>1250</v>
+        <v>4440.9</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="0" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="B364" s="0" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="C364" s="0" t="s">
         <v>29</v>
       </c>
       <c r="D364" s="0">
-        <v>1945.1</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="0" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="B365" s="0" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="C365" s="0" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="D365" s="0">
-        <v>450</v>
+        <v>1945.1</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="0" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="B366" s="0" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="C366" s="0" t="s">
         <v>16</v>
       </c>
       <c r="D366" s="0">
-        <v>825</v>
+        <v>450</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="0" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="B367" s="0" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="C367" s="0" t="s">
         <v>16</v>
@@ -8407,184 +8425,184 @@
     </row>
     <row r="368">
       <c r="A368" s="0" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="B368" s="0" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="C368" s="0" t="s">
-        <v>377</v>
+        <v>16</v>
       </c>
       <c r="D368" s="0">
-        <v>134775.6</v>
+        <v>825</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="0" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="B369" s="0" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="C369" s="0" t="s">
         <v>377</v>
       </c>
       <c r="D369" s="0">
-        <v>175991.55</v>
+        <v>134775.6</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" s="0" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="B370" s="0" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="C370" s="0" t="s">
-        <v>71</v>
+        <v>377</v>
       </c>
       <c r="D370" s="0">
-        <v>3263</v>
+        <v>175991.55</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="0" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="B371" s="0" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="C371" s="0" t="s">
         <v>71</v>
       </c>
       <c r="D371" s="0">
-        <v>18027</v>
+        <v>3263</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="0" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="B372" s="0" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="C372" s="0" t="s">
-        <v>283</v>
+        <v>71</v>
       </c>
       <c r="D372" s="0">
-        <v>515</v>
+        <v>18027</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="0" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="B373" s="0" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="C373" s="0" t="s">
-        <v>38</v>
+        <v>283</v>
       </c>
       <c r="D373" s="0">
         <v>515</v>
       </c>
     </row>
     <row r="374">
-      <c r="A374" s="2" t="s">
-        <v>804</v>
-      </c>
-      <c r="B374" s="2" t="s">
+      <c r="A374" s="0" t="s">
         <v>805</v>
       </c>
-      <c r="C374" s="2" t="s">
+      <c r="B374" s="0" t="s">
+        <v>806</v>
+      </c>
+      <c r="C374" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="D374" s="0">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="2" t="s">
+        <v>807</v>
+      </c>
+      <c r="B375" s="2" t="s">
+        <v>808</v>
+      </c>
+      <c r="C375" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D374" s="2">
+      <c r="D375" s="2">
         <v>10154</v>
-      </c>
-    </row>
-    <row r="375">
-      <c r="A375" s="0" t="s">
-        <v>806</v>
-      </c>
-      <c r="B375" s="0" t="s">
-        <v>807</v>
-      </c>
-      <c r="C375" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="D375" s="0">
-        <v>9500</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="0" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="B376" s="0" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="C376" s="0" t="s">
-        <v>475</v>
+        <v>53</v>
       </c>
       <c r="D376" s="0">
-        <v>207558.08</v>
+        <v>9500</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="0" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="B377" s="0" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="C377" s="0" t="s">
         <v>475</v>
       </c>
       <c r="D377" s="0">
-        <v>249069.69</v>
+        <v>207558.08</v>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="0" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="B378" s="0" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="C378" s="0" t="s">
-        <v>71</v>
+        <v>475</v>
       </c>
       <c r="D378" s="0">
-        <v>10021.22</v>
+        <v>249069.69</v>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="0" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="B379" s="0" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="C379" s="0" t="s">
         <v>71</v>
       </c>
       <c r="D379" s="0">
-        <v>17710</v>
+        <v>10021.22</v>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="0" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="B380" s="0" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="C380" s="0" t="s">
-        <v>818</v>
+        <v>71</v>
       </c>
       <c r="D380" s="0">
-        <v>1080</v>
+        <v>17710</v>
       </c>
     </row>
     <row r="381">
@@ -8595,24 +8613,24 @@
         <v>820</v>
       </c>
       <c r="C381" s="0" t="s">
-        <v>19</v>
+        <v>821</v>
       </c>
       <c r="D381" s="0">
-        <v>570</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="0" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="B382" s="0" t="s">
-        <v>822</v>
+        <v>823</v>
       </c>
       <c r="C382" s="0" t="s">
-        <v>823</v>
+        <v>19</v>
       </c>
       <c r="D382" s="0">
-        <v>520</v>
+        <v>570</v>
       </c>
     </row>
     <row r="383">
@@ -8623,108 +8641,108 @@
         <v>825</v>
       </c>
       <c r="C383" s="0" t="s">
-        <v>823</v>
+        <v>826</v>
       </c>
       <c r="D383" s="0">
-        <v>300</v>
+        <v>520</v>
       </c>
     </row>
     <row r="384">
       <c r="A384" s="0" t="s">
+        <v>827</v>
+      </c>
+      <c r="B384" s="0" t="s">
+        <v>828</v>
+      </c>
+      <c r="C384" s="0" t="s">
         <v>826</v>
       </c>
-      <c r="B384" s="0" t="s">
-        <v>827</v>
-      </c>
-      <c r="C384" s="0" t="s">
-        <v>16</v>
-      </c>
       <c r="D384" s="0">
-        <v>2200</v>
+        <v>300</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="0" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="B385" s="0" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="C385" s="0" t="s">
         <v>16</v>
       </c>
       <c r="D385" s="0">
-        <v>2800</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="386">
       <c r="A386" s="0" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="B386" s="0" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="C386" s="0" t="s">
-        <v>91</v>
+        <v>16</v>
       </c>
       <c r="D386" s="0">
-        <v>4791.6</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="387">
       <c r="A387" s="0" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="B387" s="0" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="C387" s="0" t="s">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="D387" s="0">
-        <v>2699.64</v>
+        <v>4791.6</v>
       </c>
     </row>
     <row r="388">
       <c r="A388" s="0" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="B388" s="0" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="C388" s="0" t="s">
-        <v>35</v>
+        <v>71</v>
       </c>
       <c r="D388" s="0">
-        <v>3800</v>
+        <v>2699.64</v>
       </c>
     </row>
     <row r="389">
       <c r="A389" s="0" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="B389" s="0" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="C389" s="0" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D389" s="0">
-        <v>4000</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="0" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="B390" s="0" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="C390" s="0" t="s">
-        <v>840</v>
+        <v>16</v>
       </c>
       <c r="D390" s="0">
-        <v>3800</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="391">
@@ -8735,304 +8753,304 @@
         <v>842</v>
       </c>
       <c r="C391" s="0" t="s">
-        <v>22</v>
+        <v>843</v>
       </c>
       <c r="D391" s="0">
-        <v>353</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="392">
       <c r="A392" s="0" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="B392" s="0" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="C392" s="0" t="s">
-        <v>109</v>
+        <v>22</v>
       </c>
       <c r="D392" s="0">
-        <v>1800</v>
+        <v>353</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="0" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="B393" s="0" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="C393" s="0" t="s">
-        <v>16</v>
+        <v>109</v>
       </c>
       <c r="D393" s="0">
-        <v>2948</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="0" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="B394" s="0" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="C394" s="0" t="s">
-        <v>207</v>
+        <v>16</v>
       </c>
       <c r="D394" s="0">
-        <v>65537</v>
+        <v>2948</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="0" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="B395" s="0" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="C395" s="0" t="s">
-        <v>137</v>
+        <v>207</v>
       </c>
       <c r="D395" s="0">
-        <v>4049.6</v>
+        <v>65537</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="0" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="B396" s="0" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="C396" s="0" t="s">
         <v>137</v>
       </c>
       <c r="D396" s="0">
-        <v>4199.2</v>
+        <v>4049.6</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="0" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="B397" s="0" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="C397" s="0" t="s">
         <v>137</v>
       </c>
       <c r="D397" s="0">
-        <v>6397.2</v>
+        <v>4199.2</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="0" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="B398" s="0" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="C398" s="0" t="s">
-        <v>310</v>
+        <v>137</v>
       </c>
       <c r="D398" s="0">
-        <v>570</v>
+        <v>6397.2</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="0" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="B399" s="0" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="C399" s="0" t="s">
-        <v>71</v>
+        <v>310</v>
       </c>
       <c r="D399" s="0">
-        <v>550</v>
+        <v>570</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="0" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="B400" s="0" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="C400" s="0" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="D400" s="0">
-        <v>167</v>
+        <v>550</v>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="0" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="B401" s="0" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="C401" s="0" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="D401" s="0">
-        <v>714.74</v>
+        <v>167</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" s="0" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="B402" s="0" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="C402" s="0" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="D402" s="0">
-        <v>101000</v>
+        <v>714.74</v>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="0" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="B403" s="0" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="C403" s="0" t="s">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="D403" s="0">
-        <v>6251</v>
+        <v>101000</v>
       </c>
     </row>
     <row r="404">
       <c r="A404" s="0" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="B404" s="0" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="C404" s="0" t="s">
-        <v>374</v>
+        <v>120</v>
       </c>
       <c r="D404" s="0">
-        <v>857.67</v>
+        <v>6251</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="0" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="B405" s="0" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="C405" s="0" t="s">
-        <v>91</v>
+        <v>374</v>
       </c>
       <c r="D405" s="0">
-        <v>1164.66</v>
+        <v>857.67</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="0" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="B406" s="0" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="C406" s="0" t="s">
-        <v>148</v>
+        <v>91</v>
       </c>
       <c r="D406" s="0">
-        <v>360</v>
+        <v>1164.66</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="0" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="B407" s="0" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="C407" s="0" t="s">
         <v>148</v>
       </c>
       <c r="D407" s="0">
-        <v>450</v>
+        <v>360</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="0" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="B408" s="0" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="C408" s="0" t="s">
         <v>148</v>
       </c>
       <c r="D408" s="0">
-        <v>2050</v>
+        <v>450</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="0" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="B409" s="0" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="C409" s="0" t="s">
-        <v>580</v>
+        <v>148</v>
       </c>
       <c r="D409" s="0">
-        <v>25192.82</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="410">
       <c r="A410" s="0" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="B410" s="0" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="C410" s="0" t="s">
-        <v>71</v>
+        <v>580</v>
       </c>
       <c r="D410" s="0">
-        <v>3500</v>
+        <v>25192.82</v>
       </c>
     </row>
     <row r="411">
       <c r="A411" s="0" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="B411" s="0" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="C411" s="0" t="s">
-        <v>175</v>
+        <v>71</v>
       </c>
       <c r="D411" s="0">
-        <v>600</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="0" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="B412" s="0" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="C412" s="0" t="s">
-        <v>885</v>
+        <v>175</v>
       </c>
       <c r="D412" s="0">
-        <v>1080</v>
+        <v>600</v>
       </c>
     </row>
     <row r="413">
@@ -9043,203 +9061,203 @@
         <v>887</v>
       </c>
       <c r="C413" s="0" t="s">
+        <v>888</v>
+      </c>
+      <c r="D413" s="0">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="0" t="s">
+        <v>889</v>
+      </c>
+      <c r="B414" s="0" t="s">
+        <v>890</v>
+      </c>
+      <c r="C414" s="0" t="s">
         <v>338</v>
       </c>
-      <c r="D413" s="0">
+      <c r="D414" s="0">
         <v>8628</v>
       </c>
     </row>
-    <row r="414">
-      <c r="A414" s="2" t="s">
-        <v>888</v>
-      </c>
-      <c r="B414" s="2" t="s">
-        <v>889</v>
-      </c>
-      <c r="C414" s="2" t="s">
+    <row r="415">
+      <c r="A415" s="2" t="s">
+        <v>891</v>
+      </c>
+      <c r="B415" s="2" t="s">
+        <v>892</v>
+      </c>
+      <c r="C415" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="D414" s="2">
+      <c r="D415" s="2">
         <v>9125.1</v>
-      </c>
-    </row>
-    <row r="415">
-      <c r="A415" s="0" t="s">
-        <v>890</v>
-      </c>
-      <c r="B415" s="0" t="s">
-        <v>891</v>
-      </c>
-      <c r="C415" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="D415" s="0">
-        <v>27991.54</v>
       </c>
     </row>
     <row r="416">
       <c r="A416" s="0" t="s">
-        <v>892</v>
+        <v>893</v>
       </c>
       <c r="B416" s="0" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
       <c r="C416" s="0" t="s">
-        <v>137</v>
+        <v>41</v>
       </c>
       <c r="D416" s="0">
-        <v>1080</v>
+        <v>27991.54</v>
       </c>
     </row>
     <row r="417">
       <c r="A417" s="0" t="s">
-        <v>894</v>
+        <v>895</v>
       </c>
       <c r="B417" s="0" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
       <c r="C417" s="0" t="s">
         <v>137</v>
       </c>
       <c r="D417" s="0">
-        <v>4012</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="0" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="B418" s="0" t="s">
-        <v>897</v>
+        <v>898</v>
       </c>
       <c r="C418" s="0" t="s">
-        <v>46</v>
+        <v>137</v>
       </c>
       <c r="D418" s="0">
-        <v>5816.9</v>
+        <v>4012</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" s="0" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
       <c r="B419" s="0" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="C419" s="0" t="s">
         <v>46</v>
       </c>
       <c r="D419" s="0">
-        <v>2624.28</v>
+        <v>6345.07</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" s="0" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
       <c r="B420" s="0" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="C420" s="0" t="s">
         <v>46</v>
       </c>
       <c r="D420" s="0">
-        <v>1953.98</v>
+        <v>2862.56</v>
       </c>
     </row>
     <row r="421">
-      <c r="A421" s="2" t="s">
-        <v>902</v>
-      </c>
-      <c r="B421" s="2" t="s">
+      <c r="A421" s="0" t="s">
         <v>903</v>
       </c>
-      <c r="C421" s="2" t="s">
+      <c r="B421" s="0" t="s">
+        <v>904</v>
+      </c>
+      <c r="C421" s="0" t="s">
         <v>46</v>
       </c>
-      <c r="D421" s="2">
-        <v>3598.96</v>
+      <c r="D421" s="0">
+        <v>2131.4</v>
       </c>
     </row>
     <row r="422">
-      <c r="A422" s="0" t="s">
-        <v>904</v>
-      </c>
-      <c r="B422" s="0" t="s">
+      <c r="A422" s="2" t="s">
         <v>905</v>
       </c>
-      <c r="C422" s="0" t="s">
+      <c r="B422" s="2" t="s">
+        <v>906</v>
+      </c>
+      <c r="C422" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D422" s="0">
-        <v>27318.17</v>
+      <c r="D422" s="2">
+        <v>3925.75</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="0" t="s">
-        <v>906</v>
+        <v>907</v>
       </c>
       <c r="B423" s="0" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="C423" s="0" t="s">
         <v>46</v>
       </c>
       <c r="D423" s="0">
-        <v>2115.26</v>
+        <v>29798.66</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="0" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="B424" s="0" t="s">
-        <v>909</v>
+        <v>910</v>
       </c>
       <c r="C424" s="0" t="s">
         <v>46</v>
       </c>
       <c r="D424" s="0">
-        <v>4700</v>
+        <v>2307.32</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="0" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="B425" s="0" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
       <c r="C425" s="0" t="s">
         <v>46</v>
       </c>
       <c r="D425" s="0">
-        <v>3750</v>
+        <v>5250</v>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="0" t="s">
-        <v>912</v>
+        <v>913</v>
       </c>
       <c r="B426" s="0" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="C426" s="0" t="s">
-        <v>484</v>
+        <v>46</v>
       </c>
       <c r="D426" s="0">
-        <v>510</v>
+        <v>4400</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="0" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="B427" s="0" t="s">
-        <v>915</v>
+        <v>916</v>
       </c>
       <c r="C427" s="0" t="s">
-        <v>38</v>
+        <v>484</v>
       </c>
       <c r="D427" s="0">
         <v>510</v>
@@ -9247,16 +9265,16 @@
     </row>
     <row r="428">
       <c r="A428" s="0" t="s">
-        <v>916</v>
+        <v>917</v>
       </c>
       <c r="B428" s="0" t="s">
-        <v>917</v>
+        <v>918</v>
       </c>
       <c r="C428" s="0" t="s">
-        <v>918</v>
+        <v>38</v>
       </c>
       <c r="D428" s="0">
-        <v>580</v>
+        <v>510</v>
       </c>
     </row>
     <row r="429">
@@ -9267,7 +9285,7 @@
         <v>920</v>
       </c>
       <c r="C429" s="0" t="s">
-        <v>918</v>
+        <v>921</v>
       </c>
       <c r="D429" s="0">
         <v>580</v>
@@ -9275,13 +9293,13 @@
     </row>
     <row r="430">
       <c r="A430" s="0" t="s">
+        <v>922</v>
+      </c>
+      <c r="B430" s="0" t="s">
+        <v>923</v>
+      </c>
+      <c r="C430" s="0" t="s">
         <v>921</v>
-      </c>
-      <c r="B430" s="0" t="s">
-        <v>922</v>
-      </c>
-      <c r="C430" s="0" t="s">
-        <v>918</v>
       </c>
       <c r="D430" s="0">
         <v>580</v>
@@ -9289,27 +9307,27 @@
     </row>
     <row r="431">
       <c r="A431" s="0" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
       <c r="B431" s="0" t="s">
-        <v>924</v>
+        <v>925</v>
       </c>
       <c r="C431" s="0" t="s">
-        <v>918</v>
+        <v>921</v>
       </c>
       <c r="D431" s="0">
-        <v>342</v>
+        <v>580</v>
       </c>
     </row>
     <row r="432">
       <c r="A432" s="0" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="B432" s="0" t="s">
-        <v>926</v>
+        <v>927</v>
       </c>
       <c r="C432" s="0" t="s">
-        <v>918</v>
+        <v>921</v>
       </c>
       <c r="D432" s="0">
         <v>342</v>
@@ -9317,13 +9335,13 @@
     </row>
     <row r="433">
       <c r="A433" s="0" t="s">
-        <v>927</v>
+        <v>928</v>
       </c>
       <c r="B433" s="0" t="s">
-        <v>928</v>
+        <v>929</v>
       </c>
       <c r="C433" s="0" t="s">
-        <v>918</v>
+        <v>921</v>
       </c>
       <c r="D433" s="0">
         <v>342</v>
@@ -9331,27 +9349,27 @@
     </row>
     <row r="434">
       <c r="A434" s="0" t="s">
-        <v>929</v>
+        <v>930</v>
       </c>
       <c r="B434" s="0" t="s">
-        <v>930</v>
+        <v>931</v>
       </c>
       <c r="C434" s="0" t="s">
-        <v>918</v>
+        <v>921</v>
       </c>
       <c r="D434" s="0">
-        <v>0</v>
+        <v>342</v>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="0" t="s">
-        <v>931</v>
+        <v>932</v>
       </c>
       <c r="B435" s="0" t="s">
-        <v>932</v>
+        <v>933</v>
       </c>
       <c r="C435" s="0" t="s">
-        <v>918</v>
+        <v>921</v>
       </c>
       <c r="D435" s="0">
         <v>0</v>
@@ -9359,394 +9377,394 @@
     </row>
     <row r="436">
       <c r="A436" s="0" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
       <c r="B436" s="0" t="s">
-        <v>934</v>
+        <v>935</v>
       </c>
       <c r="C436" s="0" t="s">
-        <v>918</v>
+        <v>921</v>
       </c>
       <c r="D436" s="0">
-        <v>423</v>
+        <v>0</v>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="0" t="s">
-        <v>935</v>
+        <v>936</v>
       </c>
       <c r="B437" s="0" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="C437" s="0" t="s">
-        <v>71</v>
+        <v>938</v>
       </c>
       <c r="D437" s="0">
-        <v>15968</v>
+        <v>453</v>
       </c>
     </row>
     <row r="438">
       <c r="A438" s="0" t="s">
-        <v>937</v>
+        <v>939</v>
       </c>
       <c r="B438" s="0" t="s">
-        <v>938</v>
+        <v>940</v>
       </c>
       <c r="C438" s="0" t="s">
-        <v>35</v>
+        <v>921</v>
       </c>
       <c r="D438" s="0">
-        <v>430</v>
+        <v>453</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="0" t="s">
-        <v>939</v>
+        <v>941</v>
       </c>
       <c r="B439" s="0" t="s">
-        <v>940</v>
+        <v>942</v>
       </c>
       <c r="C439" s="0" t="s">
-        <v>283</v>
+        <v>71</v>
       </c>
       <c r="D439" s="0">
-        <v>430</v>
+        <v>15968</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="0" t="s">
-        <v>941</v>
+        <v>943</v>
       </c>
       <c r="B440" s="0" t="s">
-        <v>942</v>
+        <v>944</v>
       </c>
       <c r="C440" s="0" t="s">
-        <v>114</v>
+        <v>35</v>
       </c>
       <c r="D440" s="0">
-        <v>14000</v>
+        <v>430</v>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="0" t="s">
-        <v>943</v>
+        <v>945</v>
       </c>
       <c r="B441" s="0" t="s">
-        <v>944</v>
+        <v>946</v>
       </c>
       <c r="C441" s="0" t="s">
-        <v>137</v>
+        <v>283</v>
       </c>
       <c r="D441" s="0">
-        <v>14001</v>
+        <v>430</v>
       </c>
     </row>
     <row r="442">
       <c r="A442" s="0" t="s">
-        <v>945</v>
+        <v>947</v>
       </c>
       <c r="B442" s="0" t="s">
-        <v>946</v>
+        <v>948</v>
       </c>
       <c r="C442" s="0" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="D442" s="0">
-        <v>266200</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="0" t="s">
-        <v>947</v>
+        <v>949</v>
       </c>
       <c r="B443" s="0" t="s">
-        <v>948</v>
+        <v>950</v>
       </c>
       <c r="C443" s="0" t="s">
-        <v>91</v>
+        <v>137</v>
       </c>
       <c r="D443" s="0">
-        <v>194991.5</v>
+        <v>14001</v>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="0" t="s">
-        <v>949</v>
+        <v>951</v>
       </c>
       <c r="B444" s="0" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
       <c r="C444" s="0" t="s">
         <v>91</v>
       </c>
       <c r="D444" s="0">
-        <v>289492.5</v>
+        <v>266200</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="0" t="s">
-        <v>951</v>
+        <v>953</v>
       </c>
       <c r="B445" s="0" t="s">
-        <v>952</v>
+        <v>954</v>
       </c>
       <c r="C445" s="0" t="s">
-        <v>953</v>
+        <v>91</v>
       </c>
       <c r="D445" s="0">
-        <v>13722.52</v>
+        <v>194991.5</v>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="0" t="s">
-        <v>954</v>
+        <v>955</v>
       </c>
       <c r="B446" s="0" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="C446" s="0" t="s">
-        <v>953</v>
+        <v>91</v>
       </c>
       <c r="D446" s="0">
-        <v>15072</v>
+        <v>289492.5</v>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="0" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
       <c r="B447" s="0" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="C447" s="0" t="s">
-        <v>953</v>
+        <v>959</v>
       </c>
       <c r="D447" s="0">
-        <v>6555.64</v>
+        <v>13722.52</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="0" t="s">
-        <v>958</v>
+        <v>960</v>
       </c>
       <c r="B448" s="0" t="s">
+        <v>961</v>
+      </c>
+      <c r="C448" s="0" t="s">
         <v>959</v>
       </c>
-      <c r="C448" s="0" t="s">
-        <v>953</v>
-      </c>
       <c r="D448" s="0">
-        <v>8964.61</v>
+        <v>15072</v>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="0" t="s">
-        <v>960</v>
+        <v>962</v>
       </c>
       <c r="B449" s="0" t="s">
-        <v>961</v>
+        <v>963</v>
       </c>
       <c r="C449" s="0" t="s">
-        <v>953</v>
+        <v>959</v>
       </c>
       <c r="D449" s="0">
-        <v>11735</v>
+        <v>6555.64</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="0" t="s">
-        <v>962</v>
+        <v>964</v>
       </c>
       <c r="B450" s="0" t="s">
-        <v>963</v>
+        <v>965</v>
       </c>
       <c r="C450" s="0" t="s">
-        <v>71</v>
+        <v>959</v>
       </c>
       <c r="D450" s="0">
-        <v>3380</v>
+        <v>8964.61</v>
       </c>
     </row>
     <row r="451">
       <c r="A451" s="0" t="s">
-        <v>964</v>
+        <v>966</v>
       </c>
       <c r="B451" s="0" t="s">
-        <v>965</v>
+        <v>967</v>
       </c>
       <c r="C451" s="0" t="s">
-        <v>137</v>
+        <v>959</v>
       </c>
       <c r="D451" s="0">
-        <v>3750</v>
+        <v>11735</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="0" t="s">
-        <v>966</v>
+        <v>968</v>
       </c>
       <c r="B452" s="0" t="s">
-        <v>967</v>
+        <v>969</v>
       </c>
       <c r="C452" s="0" t="s">
-        <v>91</v>
+        <v>71</v>
       </c>
       <c r="D452" s="0">
-        <v>4392.3</v>
+        <v>3380</v>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="0" t="s">
-        <v>968</v>
+        <v>970</v>
       </c>
       <c r="B453" s="0" t="s">
-        <v>969</v>
+        <v>971</v>
       </c>
       <c r="C453" s="0" t="s">
-        <v>970</v>
+        <v>137</v>
       </c>
       <c r="D453" s="0">
-        <v>5254.41</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="0" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="B454" s="0" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
       <c r="C454" s="0" t="s">
-        <v>53</v>
+        <v>91</v>
       </c>
       <c r="D454" s="0">
-        <v>1200</v>
+        <v>4392.3</v>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="0" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="B455" s="0" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
       <c r="C455" s="0" t="s">
-        <v>53</v>
+        <v>976</v>
       </c>
       <c r="D455" s="0">
-        <v>278</v>
+        <v>5254.41</v>
       </c>
     </row>
     <row r="456">
       <c r="A456" s="0" t="s">
-        <v>975</v>
+        <v>977</v>
       </c>
       <c r="B456" s="0" t="s">
-        <v>976</v>
+        <v>978</v>
       </c>
       <c r="C456" s="0" t="s">
         <v>53</v>
       </c>
       <c r="D456" s="0">
-        <v>562</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="457">
       <c r="A457" s="0" t="s">
-        <v>977</v>
+        <v>979</v>
       </c>
       <c r="B457" s="0" t="s">
-        <v>978</v>
+        <v>980</v>
       </c>
       <c r="C457" s="0" t="s">
-        <v>374</v>
+        <v>53</v>
       </c>
       <c r="D457" s="0">
-        <v>65142.6</v>
+        <v>278</v>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="0" t="s">
-        <v>979</v>
+        <v>981</v>
       </c>
       <c r="B458" s="0" t="s">
-        <v>980</v>
+        <v>982</v>
       </c>
       <c r="C458" s="0" t="s">
-        <v>374</v>
+        <v>53</v>
       </c>
       <c r="D458" s="0">
-        <v>23482.7</v>
+        <v>562</v>
       </c>
     </row>
     <row r="459">
       <c r="A459" s="0" t="s">
-        <v>981</v>
+        <v>983</v>
       </c>
       <c r="B459" s="0" t="s">
-        <v>982</v>
+        <v>984</v>
       </c>
       <c r="C459" s="0" t="s">
-        <v>29</v>
+        <v>374</v>
       </c>
       <c r="D459" s="0">
-        <v>6029.59</v>
+        <v>65142.6</v>
       </c>
     </row>
     <row r="460">
       <c r="A460" s="0" t="s">
-        <v>983</v>
+        <v>985</v>
       </c>
       <c r="B460" s="0" t="s">
-        <v>984</v>
+        <v>986</v>
       </c>
       <c r="C460" s="0" t="s">
-        <v>53</v>
+        <v>374</v>
       </c>
       <c r="D460" s="0">
-        <v>10985</v>
+        <v>23482.7</v>
       </c>
     </row>
     <row r="461">
       <c r="A461" s="0" t="s">
-        <v>985</v>
+        <v>987</v>
       </c>
       <c r="B461" s="0" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
       <c r="C461" s="0" t="s">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="D461" s="0">
-        <v>17425</v>
+        <v>6029.59</v>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="0" t="s">
-        <v>987</v>
+        <v>989</v>
       </c>
       <c r="B462" s="0" t="s">
-        <v>988</v>
+        <v>990</v>
       </c>
       <c r="C462" s="0" t="s">
-        <v>989</v>
+        <v>53</v>
       </c>
       <c r="D462" s="0">
-        <v>1958</v>
+        <v>10985</v>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="0" t="s">
-        <v>990</v>
+        <v>991</v>
       </c>
       <c r="B463" s="0" t="s">
-        <v>991</v>
+        <v>992</v>
       </c>
       <c r="C463" s="0" t="s">
-        <v>992</v>
+        <v>53</v>
       </c>
       <c r="D463" s="0">
-        <v>385.4</v>
+        <v>17425</v>
       </c>
     </row>
     <row r="464">
@@ -9757,147 +9775,147 @@
         <v>994</v>
       </c>
       <c r="C464" s="0" t="s">
-        <v>91</v>
+        <v>995</v>
       </c>
       <c r="D464" s="0">
-        <v>296147.5</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="0" t="s">
-        <v>995</v>
+        <v>996</v>
       </c>
       <c r="B465" s="0" t="s">
-        <v>996</v>
+        <v>997</v>
       </c>
       <c r="C465" s="0" t="s">
-        <v>580</v>
+        <v>998</v>
       </c>
       <c r="D465" s="0">
-        <v>71176.4</v>
+        <v>385.4</v>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="0" t="s">
-        <v>997</v>
+        <v>999</v>
       </c>
       <c r="B466" s="0" t="s">
-        <v>998</v>
+        <v>1000</v>
       </c>
       <c r="C466" s="0" t="s">
-        <v>137</v>
+        <v>91</v>
       </c>
       <c r="D466" s="0">
-        <v>96</v>
+        <v>296147.5</v>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="0" t="s">
-        <v>999</v>
+        <v>1001</v>
       </c>
       <c r="B467" s="0" t="s">
-        <v>1000</v>
+        <v>1002</v>
       </c>
       <c r="C467" s="0" t="s">
-        <v>71</v>
+        <v>580</v>
       </c>
       <c r="D467" s="0">
-        <v>950</v>
+        <v>71176.4</v>
       </c>
     </row>
     <row r="468">
       <c r="A468" s="0" t="s">
-        <v>1001</v>
+        <v>1003</v>
       </c>
       <c r="B468" s="0" t="s">
-        <v>1002</v>
+        <v>1004</v>
       </c>
       <c r="C468" s="0" t="s">
-        <v>475</v>
+        <v>137</v>
       </c>
       <c r="D468" s="0">
-        <v>342641</v>
+        <v>96</v>
       </c>
     </row>
     <row r="469">
       <c r="A469" s="0" t="s">
-        <v>1003</v>
+        <v>1005</v>
       </c>
       <c r="B469" s="0" t="s">
-        <v>1004</v>
+        <v>1006</v>
       </c>
       <c r="C469" s="0" t="s">
-        <v>155</v>
+        <v>71</v>
       </c>
       <c r="D469" s="0">
-        <v>2200</v>
+        <v>950</v>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="0" t="s">
-        <v>1005</v>
+        <v>1007</v>
       </c>
       <c r="B470" s="0" t="s">
-        <v>1006</v>
+        <v>1008</v>
       </c>
       <c r="C470" s="0" t="s">
-        <v>484</v>
+        <v>475</v>
       </c>
       <c r="D470" s="0">
-        <v>41000</v>
+        <v>342641</v>
       </c>
     </row>
     <row r="471">
       <c r="A471" s="0" t="s">
-        <v>1007</v>
+        <v>1009</v>
       </c>
       <c r="B471" s="0" t="s">
-        <v>1008</v>
+        <v>1010</v>
       </c>
       <c r="C471" s="0" t="s">
-        <v>71</v>
+        <v>155</v>
       </c>
       <c r="D471" s="0">
-        <v>9299</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="0" t="s">
-        <v>1009</v>
+        <v>1011</v>
       </c>
       <c r="B472" s="0" t="s">
-        <v>1010</v>
+        <v>1012</v>
       </c>
       <c r="C472" s="0" t="s">
-        <v>918</v>
+        <v>484</v>
       </c>
       <c r="D472" s="0">
-        <v>825</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="0" t="s">
-        <v>1011</v>
+        <v>1013</v>
       </c>
       <c r="B473" s="0" t="s">
-        <v>1012</v>
+        <v>1014</v>
       </c>
       <c r="C473" s="0" t="s">
-        <v>918</v>
+        <v>71</v>
       </c>
       <c r="D473" s="0">
-        <v>825</v>
+        <v>9299</v>
       </c>
     </row>
     <row r="474">
       <c r="A474" s="0" t="s">
-        <v>1013</v>
+        <v>1015</v>
       </c>
       <c r="B474" s="0" t="s">
-        <v>1014</v>
+        <v>1016</v>
       </c>
       <c r="C474" s="0" t="s">
-        <v>918</v>
+        <v>921</v>
       </c>
       <c r="D474" s="0">
         <v>825</v>
@@ -9905,69 +9923,69 @@
     </row>
     <row r="475">
       <c r="A475" s="0" t="s">
-        <v>1015</v>
+        <v>1017</v>
       </c>
       <c r="B475" s="0" t="s">
-        <v>1016</v>
+        <v>1018</v>
       </c>
       <c r="C475" s="0" t="s">
-        <v>22</v>
+        <v>921</v>
       </c>
       <c r="D475" s="0">
-        <v>563.36</v>
+        <v>825</v>
       </c>
     </row>
     <row r="476">
       <c r="A476" s="0" t="s">
-        <v>1017</v>
+        <v>1019</v>
       </c>
       <c r="B476" s="0" t="s">
-        <v>1018</v>
+        <v>1020</v>
       </c>
       <c r="C476" s="0" t="s">
-        <v>16</v>
+        <v>921</v>
       </c>
       <c r="D476" s="0">
-        <v>3520</v>
+        <v>825</v>
       </c>
     </row>
     <row r="477">
       <c r="A477" s="0" t="s">
-        <v>1019</v>
+        <v>1021</v>
       </c>
       <c r="B477" s="0" t="s">
-        <v>1020</v>
+        <v>1022</v>
       </c>
       <c r="C477" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D477" s="0">
-        <v>2600</v>
+        <v>563.36</v>
       </c>
     </row>
     <row r="478">
       <c r="A478" s="0" t="s">
-        <v>1021</v>
+        <v>1023</v>
       </c>
       <c r="B478" s="0" t="s">
-        <v>1022</v>
+        <v>1024</v>
       </c>
       <c r="C478" s="0" t="s">
-        <v>283</v>
+        <v>16</v>
       </c>
       <c r="D478" s="0">
-        <v>3700</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="479">
       <c r="A479" s="0" t="s">
-        <v>1023</v>
+        <v>1025</v>
       </c>
       <c r="B479" s="0" t="s">
-        <v>1024</v>
+        <v>1026</v>
       </c>
       <c r="C479" s="0" t="s">
-        <v>283</v>
+        <v>16</v>
       </c>
       <c r="D479" s="0">
         <v>2600</v>
@@ -9975,337 +9993,365 @@
     </row>
     <row r="480">
       <c r="A480" s="0" t="s">
-        <v>1025</v>
+        <v>1027</v>
       </c>
       <c r="B480" s="0" t="s">
-        <v>1026</v>
+        <v>1028</v>
       </c>
       <c r="C480" s="0" t="s">
-        <v>16</v>
+        <v>283</v>
       </c>
       <c r="D480" s="0">
-        <v>2235</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="0" t="s">
-        <v>1027</v>
+        <v>1029</v>
       </c>
       <c r="B481" s="0" t="s">
-        <v>1028</v>
+        <v>1030</v>
       </c>
       <c r="C481" s="0" t="s">
-        <v>16</v>
+        <v>283</v>
       </c>
       <c r="D481" s="0">
-        <v>3850</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="0" t="s">
-        <v>395</v>
+        <v>1031</v>
       </c>
       <c r="B482" s="0" t="s">
-        <v>1029</v>
+        <v>1032</v>
       </c>
       <c r="C482" s="0" t="s">
-        <v>1030</v>
+        <v>16</v>
       </c>
       <c r="D482" s="0">
-        <v>1</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="0" t="s">
-        <v>1031</v>
+        <v>1033</v>
       </c>
       <c r="B483" s="0" t="s">
-        <v>1032</v>
+        <v>1034</v>
       </c>
       <c r="C483" s="0" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="D483" s="0">
-        <v>14819</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="0" t="s">
-        <v>1033</v>
+        <v>395</v>
       </c>
       <c r="B484" s="0" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="C484" s="0" t="s">
-        <v>374</v>
+        <v>1036</v>
       </c>
       <c r="D484" s="0">
-        <v>3859.93</v>
+        <v>1</v>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="0" t="s">
-        <v>1035</v>
+        <v>1037</v>
       </c>
       <c r="B485" s="0" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
       <c r="C485" s="0" t="s">
-        <v>374</v>
+        <v>29</v>
       </c>
       <c r="D485" s="0">
-        <v>11751.49</v>
+        <v>14819</v>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="0" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
       <c r="B486" s="0" t="s">
-        <v>1038</v>
+        <v>1040</v>
       </c>
       <c r="C486" s="0" t="s">
-        <v>338</v>
+        <v>374</v>
       </c>
       <c r="D486" s="0">
-        <v>6000</v>
+        <v>3859.93</v>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="0" t="s">
-        <v>1039</v>
+        <v>1041</v>
       </c>
       <c r="B487" s="0" t="s">
-        <v>1040</v>
+        <v>1042</v>
       </c>
       <c r="C487" s="0" t="s">
-        <v>338</v>
+        <v>374</v>
       </c>
       <c r="D487" s="0">
-        <v>3000</v>
+        <v>11751.49</v>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="0" t="s">
-        <v>1041</v>
+        <v>1043</v>
       </c>
       <c r="B488" s="0" t="s">
-        <v>1042</v>
+        <v>1044</v>
       </c>
       <c r="C488" s="0" t="s">
-        <v>38</v>
+        <v>338</v>
       </c>
       <c r="D488" s="0">
-        <v>618</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="489">
       <c r="A489" s="0" t="s">
-        <v>1043</v>
+        <v>1045</v>
       </c>
       <c r="B489" s="0" t="s">
-        <v>1044</v>
+        <v>1046</v>
       </c>
       <c r="C489" s="0" t="s">
-        <v>1045</v>
+        <v>338</v>
       </c>
       <c r="D489" s="0">
-        <v>24600</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="490">
       <c r="A490" s="0" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="B490" s="0" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="C490" s="0" t="s">
-        <v>104</v>
+        <v>38</v>
       </c>
       <c r="D490" s="0">
-        <v>0</v>
+        <v>618</v>
       </c>
     </row>
     <row r="491">
       <c r="A491" s="0" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="B491" s="0" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="C491" s="0" t="s">
-        <v>91</v>
+        <v>1051</v>
       </c>
       <c r="D491" s="0">
-        <v>40928.25</v>
+        <v>24600</v>
       </c>
     </row>
     <row r="492">
       <c r="A492" s="0" t="s">
-        <v>1050</v>
+        <v>1052</v>
       </c>
       <c r="B492" s="0" t="s">
-        <v>1051</v>
+        <v>1053</v>
       </c>
       <c r="C492" s="0" t="s">
-        <v>374</v>
+        <v>104</v>
       </c>
       <c r="D492" s="0">
-        <v>75529.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="0" t="s">
-        <v>1052</v>
+        <v>1054</v>
       </c>
       <c r="B493" s="0" t="s">
-        <v>1053</v>
+        <v>1055</v>
       </c>
       <c r="C493" s="0" t="s">
-        <v>374</v>
+        <v>91</v>
       </c>
       <c r="D493" s="0">
-        <v>41613.42</v>
+        <v>40928.25</v>
       </c>
     </row>
     <row r="494">
       <c r="A494" s="0" t="s">
-        <v>1054</v>
+        <v>1056</v>
       </c>
       <c r="B494" s="0" t="s">
-        <v>1055</v>
+        <v>1057</v>
       </c>
       <c r="C494" s="0" t="s">
         <v>374</v>
       </c>
       <c r="D494" s="0">
-        <v>87056.42</v>
+        <v>75529.71</v>
       </c>
     </row>
     <row r="495">
       <c r="A495" s="0" t="s">
-        <v>1056</v>
+        <v>1058</v>
       </c>
       <c r="B495" s="0" t="s">
-        <v>1057</v>
+        <v>1059</v>
       </c>
       <c r="C495" s="0" t="s">
         <v>374</v>
       </c>
       <c r="D495" s="0">
-        <v>49243.16</v>
+        <v>41613.42</v>
       </c>
     </row>
     <row r="496">
       <c r="A496" s="0" t="s">
-        <v>1058</v>
+        <v>1060</v>
       </c>
       <c r="B496" s="0" t="s">
-        <v>1059</v>
+        <v>1061</v>
       </c>
       <c r="C496" s="0" t="s">
-        <v>22</v>
+        <v>374</v>
       </c>
       <c r="D496" s="0">
-        <v>1600</v>
+        <v>87056.42</v>
       </c>
     </row>
     <row r="497">
       <c r="A497" s="0" t="s">
-        <v>1060</v>
+        <v>1062</v>
       </c>
       <c r="B497" s="0" t="s">
-        <v>1061</v>
+        <v>1063</v>
       </c>
       <c r="C497" s="0" t="s">
-        <v>29</v>
+        <v>374</v>
       </c>
       <c r="D497" s="0">
-        <v>3455.8</v>
+        <v>49243.16</v>
       </c>
     </row>
     <row r="498">
       <c r="A498" s="0" t="s">
-        <v>1062</v>
+        <v>1064</v>
       </c>
       <c r="B498" s="0" t="s">
-        <v>1063</v>
+        <v>1065</v>
       </c>
       <c r="C498" s="0" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D498" s="0">
-        <v>3987</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="499">
       <c r="A499" s="0" t="s">
-        <v>1064</v>
+        <v>1066</v>
       </c>
       <c r="B499" s="0" t="s">
-        <v>1065</v>
+        <v>1067</v>
       </c>
       <c r="C499" s="0" t="s">
         <v>29</v>
       </c>
       <c r="D499" s="0">
-        <v>4010.17</v>
+        <v>3455.8</v>
       </c>
     </row>
     <row r="500">
       <c r="A500" s="0" t="s">
-        <v>1066</v>
+        <v>1068</v>
       </c>
       <c r="B500" s="0" t="s">
-        <v>1067</v>
+        <v>1069</v>
       </c>
       <c r="C500" s="0" t="s">
         <v>29</v>
       </c>
       <c r="D500" s="0">
-        <v>3382.65</v>
+        <v>3987</v>
       </c>
     </row>
     <row r="501">
-      <c r="A501" s="2" t="s">
-        <v>1068</v>
-      </c>
-      <c r="B501" s="2" t="s">
-        <v>1069</v>
-      </c>
-      <c r="C501" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D501" s="2">
-        <v>0</v>
+      <c r="A501" s="0" t="s">
+        <v>1070</v>
+      </c>
+      <c r="B501" s="0" t="s">
+        <v>1071</v>
+      </c>
+      <c r="C501" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D501" s="0">
+        <v>4010.17</v>
       </c>
     </row>
     <row r="502">
       <c r="A502" s="0" t="s">
-        <v>1070</v>
+        <v>1072</v>
       </c>
       <c r="B502" s="0" t="s">
-        <v>1071</v>
+        <v>1073</v>
       </c>
       <c r="C502" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D502" s="0">
+        <v>3382.65</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="2" t="s">
+        <v>1074</v>
+      </c>
+      <c r="B503" s="2" t="s">
+        <v>1075</v>
+      </c>
+      <c r="C503" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D503" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="0" t="s">
+        <v>1076</v>
+      </c>
+      <c r="B504" s="0" t="s">
+        <v>1077</v>
+      </c>
+      <c r="C504" s="0" t="s">
         <v>155</v>
       </c>
-      <c r="D502" s="0">
+      <c r="D504" s="0">
         <v>430</v>
       </c>
     </row>
-    <row r="503">
-      <c r="A503" s="0" t="s">
-        <v>1072</v>
-      </c>
-      <c r="B503" s="0" t="s">
-        <v>1073</v>
-      </c>
-      <c r="C503" s="0" t="s">
+    <row r="505">
+      <c r="A505" s="0" t="s">
+        <v>1078</v>
+      </c>
+      <c r="B505" s="0" t="s">
+        <v>1079</v>
+      </c>
+      <c r="C505" s="0" t="s">
         <v>137</v>
       </c>
-      <c r="D503" s="0">
+      <c r="D505" s="0">
         <v>462</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: stock y precios actualizados sáb. 25/07/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1082" uniqueCount="1082">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="1084">
   <si>
     <t>Código</t>
   </si>
@@ -1104,6 +1104,12 @@
   </si>
   <si>
     <t>DIPIRONA 50 MG X 100 ML JBE - BIOSINTEX - 000024668</t>
+  </si>
+  <si>
+    <t>000023390</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIPIRONA DRAWER 1G INY. AMP. X  1 X 2ML - 000023390</t>
   </si>
   <si>
     <t>000023431</t>
@@ -3316,7 +3322,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A3:D506"/>
+  <dimension ref="A3:D507"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="3">
@@ -3554,7 +3560,7 @@
         <v>46</v>
       </c>
       <c r="D19" s="0">
-        <v>3853.77</v>
+        <v>3853.39</v>
       </c>
     </row>
     <row r="20">
@@ -3582,7 +3588,7 @@
         <v>46</v>
       </c>
       <c r="D21" s="0">
-        <v>32000</v>
+        <v>31996.8</v>
       </c>
     </row>
     <row r="22">
@@ -4842,7 +4848,7 @@
         <v>46</v>
       </c>
       <c r="D111" s="0">
-        <v>5772.37</v>
+        <v>5771.79</v>
       </c>
     </row>
     <row r="112">
@@ -5553,7 +5559,7 @@
         <v>365</v>
       </c>
       <c r="C162" s="0" t="s">
-        <v>148</v>
+        <v>35</v>
       </c>
       <c r="D162" s="0">
         <v>650</v>
@@ -5567,7 +5573,7 @@
         <v>367</v>
       </c>
       <c r="C163" s="0" t="s">
-        <v>16</v>
+        <v>148</v>
       </c>
       <c r="D163" s="0">
         <v>650</v>
@@ -5584,7 +5590,7 @@
         <v>16</v>
       </c>
       <c r="D164" s="0">
-        <v>1700</v>
+        <v>650</v>
       </c>
     </row>
     <row r="165">
@@ -5598,7 +5604,7 @@
         <v>16</v>
       </c>
       <c r="D165" s="0">
-        <v>0</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="166">
@@ -5609,10 +5615,10 @@
         <v>373</v>
       </c>
       <c r="C166" s="0" t="s">
-        <v>114</v>
+        <v>16</v>
       </c>
       <c r="D166" s="0">
-        <v>1290</v>
+        <v>0</v>
       </c>
     </row>
     <row r="167">
@@ -5623,38 +5629,38 @@
         <v>375</v>
       </c>
       <c r="C167" s="0" t="s">
-        <v>376</v>
+        <v>114</v>
       </c>
       <c r="D167" s="0">
-        <v>52972.83</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="0" t="s">
+        <v>376</v>
+      </c>
+      <c r="B168" s="0" t="s">
         <v>377</v>
       </c>
-      <c r="B168" s="0" t="s">
+      <c r="C168" s="0" t="s">
         <v>378</v>
       </c>
-      <c r="C168" s="0" t="s">
-        <v>379</v>
-      </c>
       <c r="D168" s="0">
-        <v>104695.98</v>
+        <v>52972.83</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="0" t="s">
+        <v>379</v>
+      </c>
+      <c r="B169" s="0" t="s">
         <v>380</v>
       </c>
-      <c r="B169" s="0" t="s">
+      <c r="C169" s="0" t="s">
         <v>381</v>
       </c>
-      <c r="C169" s="0" t="s">
-        <v>379</v>
-      </c>
       <c r="D169" s="0">
-        <v>80478.92</v>
+        <v>104695.98</v>
       </c>
     </row>
     <row r="170">
@@ -5665,10 +5671,10 @@
         <v>383</v>
       </c>
       <c r="C170" s="0" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="D170" s="0">
-        <v>92546.68</v>
+        <v>80478.92</v>
       </c>
     </row>
     <row r="171">
@@ -5679,10 +5685,10 @@
         <v>385</v>
       </c>
       <c r="C171" s="0" t="s">
-        <v>29</v>
+        <v>381</v>
       </c>
       <c r="D171" s="0">
-        <v>954.8</v>
+        <v>92546.68</v>
       </c>
     </row>
     <row r="172">
@@ -5696,7 +5702,7 @@
         <v>29</v>
       </c>
       <c r="D172" s="0">
-        <v>744.2</v>
+        <v>954.8</v>
       </c>
     </row>
     <row r="173">
@@ -5710,7 +5716,7 @@
         <v>29</v>
       </c>
       <c r="D173" s="0">
-        <v>2743.71</v>
+        <v>265.3</v>
       </c>
     </row>
     <row r="174">
@@ -5721,24 +5727,24 @@
         <v>391</v>
       </c>
       <c r="C174" s="0" t="s">
-        <v>392</v>
+        <v>29</v>
       </c>
       <c r="D174" s="0">
-        <v>81</v>
+        <v>2743.71</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="0" t="s">
+        <v>392</v>
+      </c>
+      <c r="B175" s="0" t="s">
         <v>393</v>
       </c>
-      <c r="B175" s="0" t="s">
+      <c r="C175" s="0" t="s">
         <v>394</v>
       </c>
-      <c r="C175" s="0" t="s">
-        <v>19</v>
-      </c>
       <c r="D175" s="0">
-        <v>270</v>
+        <v>81</v>
       </c>
     </row>
     <row r="176">
@@ -5749,38 +5755,38 @@
         <v>396</v>
       </c>
       <c r="C176" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D176" s="0">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="0" t="s">
+        <v>397</v>
+      </c>
+      <c r="B177" s="0" t="s">
+        <v>398</v>
+      </c>
+      <c r="C177" s="0" t="s">
         <v>148</v>
       </c>
-      <c r="D176" s="0">
+      <c r="D177" s="0">
         <v>257</v>
       </c>
     </row>
-    <row r="177">
-      <c r="A177" s="2" t="s">
-        <v>397</v>
-      </c>
-      <c r="B177" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="C177" s="2" t="s">
+    <row r="178">
+      <c r="A178" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="B178" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="C178" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="D177" s="2">
+      <c r="D178" s="2">
         <v>1</v>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="0" t="s">
-        <v>399</v>
-      </c>
-      <c r="B178" s="0" t="s">
-        <v>400</v>
-      </c>
-      <c r="C178" s="0" t="s">
-        <v>137</v>
-      </c>
-      <c r="D178" s="0">
-        <v>2762.43</v>
       </c>
     </row>
     <row r="179">
@@ -5794,7 +5800,7 @@
         <v>137</v>
       </c>
       <c r="D179" s="0">
-        <v>3573.45</v>
+        <v>2762.43</v>
       </c>
     </row>
     <row r="180">
@@ -5805,10 +5811,10 @@
         <v>404</v>
       </c>
       <c r="C180" s="0" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
       <c r="D180" s="0">
-        <v>5100</v>
+        <v>3573.45</v>
       </c>
     </row>
     <row r="181">
@@ -5819,10 +5825,10 @@
         <v>406</v>
       </c>
       <c r="C181" s="0" t="s">
-        <v>376</v>
+        <v>120</v>
       </c>
       <c r="D181" s="0">
-        <v>36105.51</v>
+        <v>5100</v>
       </c>
     </row>
     <row r="182">
@@ -5833,10 +5839,10 @@
         <v>408</v>
       </c>
       <c r="C182" s="0" t="s">
-        <v>78</v>
+        <v>378</v>
       </c>
       <c r="D182" s="0">
-        <v>783.93</v>
+        <v>36105.51</v>
       </c>
     </row>
     <row r="183">
@@ -5850,7 +5856,7 @@
         <v>78</v>
       </c>
       <c r="D183" s="0">
-        <v>2850</v>
+        <v>783.93</v>
       </c>
     </row>
     <row r="184">
@@ -5861,10 +5867,10 @@
         <v>412</v>
       </c>
       <c r="C184" s="0" t="s">
-        <v>19</v>
+        <v>78</v>
       </c>
       <c r="D184" s="0">
-        <v>6599.67</v>
+        <v>2850</v>
       </c>
     </row>
     <row r="185">
@@ -5878,7 +5884,7 @@
         <v>19</v>
       </c>
       <c r="D185" s="0">
-        <v>343.2</v>
+        <v>6599.67</v>
       </c>
     </row>
     <row r="186">
@@ -5889,10 +5895,10 @@
         <v>416</v>
       </c>
       <c r="C186" s="0" t="s">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="D186" s="0">
-        <v>10007.57</v>
+        <v>343.2</v>
       </c>
     </row>
     <row r="187">
@@ -5903,10 +5909,10 @@
         <v>418</v>
       </c>
       <c r="C187" s="0" t="s">
-        <v>19</v>
+        <v>78</v>
       </c>
       <c r="D187" s="0">
-        <v>3479.75</v>
+        <v>10007.57</v>
       </c>
     </row>
     <row r="188">
@@ -5920,7 +5926,7 @@
         <v>19</v>
       </c>
       <c r="D188" s="0">
-        <v>405</v>
+        <v>3479.75</v>
       </c>
     </row>
     <row r="189">
@@ -5934,7 +5940,7 @@
         <v>19</v>
       </c>
       <c r="D189" s="0">
-        <v>2015.51</v>
+        <v>405</v>
       </c>
     </row>
     <row r="190">
@@ -5945,10 +5951,10 @@
         <v>424</v>
       </c>
       <c r="C190" s="0" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="D190" s="0">
-        <v>9041.55</v>
+        <v>2015.51</v>
       </c>
     </row>
     <row r="191">
@@ -5959,10 +5965,10 @@
         <v>426</v>
       </c>
       <c r="C191" s="0" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="D191" s="0">
-        <v>430</v>
+        <v>9041.55</v>
       </c>
     </row>
     <row r="192">
@@ -5976,7 +5982,7 @@
         <v>71</v>
       </c>
       <c r="D192" s="0">
-        <v>800</v>
+        <v>430</v>
       </c>
     </row>
     <row r="193">
@@ -5987,10 +5993,10 @@
         <v>430</v>
       </c>
       <c r="C193" s="0" t="s">
-        <v>244</v>
+        <v>71</v>
       </c>
       <c r="D193" s="0">
-        <v>2280</v>
+        <v>800</v>
       </c>
     </row>
     <row r="194">
@@ -6004,7 +6010,7 @@
         <v>244</v>
       </c>
       <c r="D194" s="0">
-        <v>1620</v>
+        <v>2280</v>
       </c>
     </row>
     <row r="195">
@@ -6015,10 +6021,10 @@
         <v>434</v>
       </c>
       <c r="C195" s="0" t="s">
-        <v>376</v>
+        <v>244</v>
       </c>
       <c r="D195" s="0">
-        <v>236458.17</v>
+        <v>1620</v>
       </c>
     </row>
     <row r="196">
@@ -6029,38 +6035,38 @@
         <v>436</v>
       </c>
       <c r="C196" s="0" t="s">
+        <v>378</v>
+      </c>
+      <c r="D196" s="0">
+        <v>236458.17</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="0" t="s">
+        <v>437</v>
+      </c>
+      <c r="B197" s="0" t="s">
+        <v>438</v>
+      </c>
+      <c r="C197" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="D196" s="0">
+      <c r="D197" s="0">
         <v>691</v>
       </c>
     </row>
-    <row r="197">
-      <c r="A197" s="2" t="s">
-        <v>437</v>
-      </c>
-      <c r="B197" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="C197" s="2" t="s">
+    <row r="198">
+      <c r="A198" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="B198" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="C198" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D197" s="2">
+      <c r="D198" s="2">
         <v>2015</v>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" s="0" t="s">
-        <v>439</v>
-      </c>
-      <c r="B198" s="0" t="s">
-        <v>440</v>
-      </c>
-      <c r="C198" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="D198" s="0">
-        <v>300</v>
       </c>
     </row>
     <row r="199">
@@ -6071,10 +6077,10 @@
         <v>442</v>
       </c>
       <c r="C199" s="0" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="D199" s="0">
-        <v>317.2</v>
+        <v>300</v>
       </c>
     </row>
     <row r="200">
@@ -6085,10 +6091,10 @@
         <v>444</v>
       </c>
       <c r="C200" s="0" t="s">
-        <v>376</v>
+        <v>29</v>
       </c>
       <c r="D200" s="0">
-        <v>25100</v>
+        <v>317.2</v>
       </c>
     </row>
     <row r="201">
@@ -6099,24 +6105,24 @@
         <v>446</v>
       </c>
       <c r="C201" s="0" t="s">
-        <v>447</v>
+        <v>378</v>
       </c>
       <c r="D201" s="0">
-        <v>20900</v>
+        <v>25100</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="0" t="s">
+        <v>447</v>
+      </c>
+      <c r="B202" s="0" t="s">
         <v>448</v>
       </c>
-      <c r="B202" s="0" t="s">
+      <c r="C202" s="0" t="s">
         <v>449</v>
       </c>
-      <c r="C202" s="0" t="s">
-        <v>46</v>
-      </c>
       <c r="D202" s="0">
-        <v>4729.95</v>
+        <v>20900</v>
       </c>
     </row>
     <row r="203">
@@ -6127,10 +6133,10 @@
         <v>451</v>
       </c>
       <c r="C203" s="0" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="D203" s="0">
-        <v>1104.46</v>
+        <v>4729.48</v>
       </c>
     </row>
     <row r="204">
@@ -6141,10 +6147,10 @@
         <v>453</v>
       </c>
       <c r="C204" s="0" t="s">
-        <v>91</v>
+        <v>22</v>
       </c>
       <c r="D204" s="0">
-        <v>11646.25</v>
+        <v>1104.46</v>
       </c>
     </row>
     <row r="205">
@@ -6155,10 +6161,10 @@
         <v>455</v>
       </c>
       <c r="C205" s="0" t="s">
-        <v>120</v>
+        <v>91</v>
       </c>
       <c r="D205" s="0">
-        <v>6072</v>
+        <v>11646.25</v>
       </c>
     </row>
     <row r="206">
@@ -6169,10 +6175,10 @@
         <v>457</v>
       </c>
       <c r="C206" s="0" t="s">
-        <v>71</v>
+        <v>120</v>
       </c>
       <c r="D206" s="0">
-        <v>400</v>
+        <v>6072</v>
       </c>
     </row>
     <row r="207">
@@ -6183,10 +6189,10 @@
         <v>459</v>
       </c>
       <c r="C207" s="0" t="s">
-        <v>22</v>
+        <v>71</v>
       </c>
       <c r="D207" s="0">
-        <v>409</v>
+        <v>400</v>
       </c>
     </row>
     <row r="208">
@@ -6197,10 +6203,10 @@
         <v>461</v>
       </c>
       <c r="C208" s="0" t="s">
-        <v>65</v>
+        <v>22</v>
       </c>
       <c r="D208" s="0">
-        <v>10537</v>
+        <v>409</v>
       </c>
     </row>
     <row r="209">
@@ -6214,7 +6220,7 @@
         <v>65</v>
       </c>
       <c r="D209" s="0">
-        <v>12198</v>
+        <v>10537</v>
       </c>
     </row>
     <row r="210">
@@ -6225,10 +6231,10 @@
         <v>465</v>
       </c>
       <c r="C210" s="0" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="D210" s="0">
-        <v>2000</v>
+        <v>12198</v>
       </c>
     </row>
     <row r="211">
@@ -6239,24 +6245,24 @@
         <v>467</v>
       </c>
       <c r="C211" s="0" t="s">
-        <v>468</v>
+        <v>53</v>
       </c>
       <c r="D211" s="0">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="0" t="s">
+        <v>468</v>
+      </c>
+      <c r="B212" s="0" t="s">
         <v>469</v>
       </c>
-      <c r="B212" s="0" t="s">
+      <c r="C212" s="0" t="s">
         <v>470</v>
       </c>
-      <c r="C212" s="0" t="s">
-        <v>16</v>
-      </c>
       <c r="D212" s="0">
-        <v>490</v>
+        <v>0</v>
       </c>
     </row>
     <row r="213">
@@ -6267,10 +6273,10 @@
         <v>472</v>
       </c>
       <c r="C213" s="0" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="D213" s="0">
-        <v>0</v>
+        <v>490</v>
       </c>
     </row>
     <row r="214">
@@ -6281,10 +6287,10 @@
         <v>474</v>
       </c>
       <c r="C214" s="0" t="s">
-        <v>157</v>
+        <v>35</v>
       </c>
       <c r="D214" s="0">
-        <v>25171.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="215">
@@ -6295,24 +6301,24 @@
         <v>476</v>
       </c>
       <c r="C215" s="0" t="s">
-        <v>477</v>
+        <v>157</v>
       </c>
       <c r="D215" s="0">
-        <v>60630</v>
+        <v>25171.1</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="0" t="s">
+        <v>477</v>
+      </c>
+      <c r="B216" s="0" t="s">
         <v>478</v>
       </c>
-      <c r="B216" s="0" t="s">
+      <c r="C216" s="0" t="s">
         <v>479</v>
       </c>
-      <c r="C216" s="0" t="s">
-        <v>148</v>
-      </c>
       <c r="D216" s="0">
-        <v>1800</v>
+        <v>60630</v>
       </c>
     </row>
     <row r="217">
@@ -6323,10 +6329,10 @@
         <v>481</v>
       </c>
       <c r="C217" s="0" t="s">
-        <v>35</v>
+        <v>148</v>
       </c>
       <c r="D217" s="0">
-        <v>0</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="218">
@@ -6337,10 +6343,10 @@
         <v>483</v>
       </c>
       <c r="C218" s="0" t="s">
-        <v>137</v>
+        <v>35</v>
       </c>
       <c r="D218" s="0">
-        <v>492.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="219">
@@ -6351,24 +6357,24 @@
         <v>485</v>
       </c>
       <c r="C219" s="0" t="s">
-        <v>486</v>
+        <v>137</v>
       </c>
       <c r="D219" s="0">
-        <v>495</v>
+        <v>492.2</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="0" t="s">
+        <v>486</v>
+      </c>
+      <c r="B220" s="0" t="s">
         <v>487</v>
       </c>
-      <c r="B220" s="0" t="s">
+      <c r="C220" s="0" t="s">
         <v>488</v>
       </c>
-      <c r="C220" s="0" t="s">
-        <v>19</v>
-      </c>
       <c r="D220" s="0">
-        <v>1786</v>
+        <v>495</v>
       </c>
     </row>
     <row r="221">
@@ -6382,7 +6388,7 @@
         <v>19</v>
       </c>
       <c r="D221" s="0">
-        <v>4391.8</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="222">
@@ -6393,10 +6399,10 @@
         <v>492</v>
       </c>
       <c r="C222" s="0" t="s">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="D222" s="0">
-        <v>4700</v>
+        <v>4391.8</v>
       </c>
     </row>
     <row r="223">
@@ -6410,7 +6416,7 @@
         <v>53</v>
       </c>
       <c r="D223" s="0">
-        <v>4200</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="224">
@@ -6449,21 +6455,21 @@
         <v>500</v>
       </c>
       <c r="C226" s="0" t="s">
-        <v>501</v>
+        <v>53</v>
       </c>
       <c r="D226" s="0">
-        <v>265</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="0" t="s">
+        <v>501</v>
+      </c>
+      <c r="B227" s="0" t="s">
         <v>502</v>
       </c>
-      <c r="B227" s="0" t="s">
+      <c r="C227" s="0" t="s">
         <v>503</v>
-      </c>
-      <c r="C227" s="0" t="s">
-        <v>501</v>
       </c>
       <c r="D227" s="0">
         <v>265</v>
@@ -6477,7 +6483,7 @@
         <v>505</v>
       </c>
       <c r="C228" s="0" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="D228" s="0">
         <v>265</v>
@@ -6491,7 +6497,7 @@
         <v>507</v>
       </c>
       <c r="C229" s="0" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="D229" s="0">
         <v>265</v>
@@ -6505,7 +6511,7 @@
         <v>509</v>
       </c>
       <c r="C230" s="0" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="D230" s="0">
         <v>265</v>
@@ -6519,7 +6525,7 @@
         <v>511</v>
       </c>
       <c r="C231" s="0" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="D231" s="0">
         <v>265</v>
@@ -6533,21 +6539,21 @@
         <v>513</v>
       </c>
       <c r="C232" s="0" t="s">
-        <v>514</v>
+        <v>503</v>
       </c>
       <c r="D232" s="0">
-        <v>4700</v>
+        <v>265</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="0" t="s">
+        <v>514</v>
+      </c>
+      <c r="B233" s="0" t="s">
         <v>515</v>
       </c>
-      <c r="B233" s="0" t="s">
+      <c r="C233" s="0" t="s">
         <v>516</v>
-      </c>
-      <c r="C233" s="0" t="s">
-        <v>517</v>
       </c>
       <c r="D233" s="0">
         <v>4700</v>
@@ -6555,13 +6561,13 @@
     </row>
     <row r="234">
       <c r="A234" s="0" t="s">
+        <v>517</v>
+      </c>
+      <c r="B234" s="0" t="s">
         <v>518</v>
       </c>
-      <c r="B234" s="0" t="s">
+      <c r="C234" s="0" t="s">
         <v>519</v>
-      </c>
-      <c r="C234" s="0" t="s">
-        <v>53</v>
       </c>
       <c r="D234" s="0">
         <v>4700</v>
@@ -6578,7 +6584,7 @@
         <v>53</v>
       </c>
       <c r="D235" s="0">
-        <v>500</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="236">
@@ -6592,7 +6598,7 @@
         <v>53</v>
       </c>
       <c r="D236" s="0">
-        <v>210</v>
+        <v>500</v>
       </c>
     </row>
     <row r="237">
@@ -6606,7 +6612,7 @@
         <v>53</v>
       </c>
       <c r="D237" s="0">
-        <v>247</v>
+        <v>210</v>
       </c>
     </row>
     <row r="238">
@@ -6617,10 +6623,10 @@
         <v>527</v>
       </c>
       <c r="C238" s="0" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="D238" s="0">
-        <v>5600</v>
+        <v>247</v>
       </c>
     </row>
     <row r="239">
@@ -6631,10 +6637,10 @@
         <v>529</v>
       </c>
       <c r="C239" s="0" t="s">
-        <v>148</v>
+        <v>38</v>
       </c>
       <c r="D239" s="0">
-        <v>6000</v>
+        <v>5600</v>
       </c>
     </row>
     <row r="240">
@@ -6645,10 +6651,10 @@
         <v>531</v>
       </c>
       <c r="C240" s="0" t="s">
-        <v>71</v>
+        <v>148</v>
       </c>
       <c r="D240" s="0">
-        <v>80000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="241">
@@ -6662,7 +6668,7 @@
         <v>71</v>
       </c>
       <c r="D241" s="0">
-        <v>90000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="242">
@@ -6676,7 +6682,7 @@
         <v>71</v>
       </c>
       <c r="D242" s="0">
-        <v>110000</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="243">
@@ -6687,10 +6693,10 @@
         <v>537</v>
       </c>
       <c r="C243" s="0" t="s">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="D243" s="0">
-        <v>1100</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="244">
@@ -6704,7 +6710,7 @@
         <v>16</v>
       </c>
       <c r="D244" s="0">
-        <v>2500</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="245">
@@ -6715,10 +6721,10 @@
         <v>541</v>
       </c>
       <c r="C245" s="0" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="D245" s="0">
-        <v>13636.84</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="246">
@@ -6729,10 +6735,10 @@
         <v>543</v>
       </c>
       <c r="C246" s="0" t="s">
-        <v>285</v>
+        <v>29</v>
       </c>
       <c r="D246" s="0">
-        <v>450</v>
+        <v>13636.84</v>
       </c>
     </row>
     <row r="247">
@@ -6743,10 +6749,10 @@
         <v>545</v>
       </c>
       <c r="C247" s="0" t="s">
-        <v>16</v>
+        <v>285</v>
       </c>
       <c r="D247" s="0">
-        <v>555</v>
+        <v>450</v>
       </c>
     </row>
     <row r="248">
@@ -6760,7 +6766,7 @@
         <v>16</v>
       </c>
       <c r="D248" s="0">
-        <v>825</v>
+        <v>555</v>
       </c>
     </row>
     <row r="249">
@@ -6774,7 +6780,7 @@
         <v>16</v>
       </c>
       <c r="D249" s="0">
-        <v>36.3</v>
+        <v>825</v>
       </c>
     </row>
     <row r="250">
@@ -6788,7 +6794,7 @@
         <v>16</v>
       </c>
       <c r="D250" s="0">
-        <v>544.5</v>
+        <v>36.3</v>
       </c>
     </row>
     <row r="251">
@@ -6802,7 +6808,7 @@
         <v>16</v>
       </c>
       <c r="D251" s="0">
-        <v>750</v>
+        <v>544.5</v>
       </c>
     </row>
     <row r="252">
@@ -6813,10 +6819,10 @@
         <v>555</v>
       </c>
       <c r="C252" s="0" t="s">
-        <v>148</v>
+        <v>16</v>
       </c>
       <c r="D252" s="0">
-        <v>1130</v>
+        <v>750</v>
       </c>
     </row>
     <row r="253">
@@ -6827,10 +6833,10 @@
         <v>557</v>
       </c>
       <c r="C253" s="0" t="s">
-        <v>53</v>
+        <v>148</v>
       </c>
       <c r="D253" s="0">
-        <v>4510</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="254">
@@ -6883,10 +6889,10 @@
         <v>565</v>
       </c>
       <c r="C257" s="0" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="D257" s="0">
-        <v>902</v>
+        <v>4510</v>
       </c>
     </row>
     <row r="258">
@@ -6900,7 +6906,7 @@
         <v>16</v>
       </c>
       <c r="D258" s="0">
-        <v>880</v>
+        <v>902</v>
       </c>
     </row>
     <row r="259">
@@ -6911,10 +6917,10 @@
         <v>569</v>
       </c>
       <c r="C259" s="0" t="s">
-        <v>137</v>
+        <v>16</v>
       </c>
       <c r="D259" s="0">
-        <v>430</v>
+        <v>880</v>
       </c>
     </row>
     <row r="260">
@@ -6928,7 +6934,7 @@
         <v>137</v>
       </c>
       <c r="D260" s="0">
-        <v>354.54</v>
+        <v>430</v>
       </c>
     </row>
     <row r="261">
@@ -6939,10 +6945,10 @@
         <v>573</v>
       </c>
       <c r="C261" s="0" t="s">
-        <v>19</v>
+        <v>137</v>
       </c>
       <c r="D261" s="0">
-        <v>318.63</v>
+        <v>354.54</v>
       </c>
     </row>
     <row r="262">
@@ -6956,7 +6962,7 @@
         <v>19</v>
       </c>
       <c r="D262" s="0">
-        <v>415.15</v>
+        <v>318.63</v>
       </c>
     </row>
     <row r="263">
@@ -6970,7 +6976,7 @@
         <v>19</v>
       </c>
       <c r="D263" s="0">
-        <v>760</v>
+        <v>415.15</v>
       </c>
     </row>
     <row r="264">
@@ -6984,7 +6990,7 @@
         <v>19</v>
       </c>
       <c r="D264" s="0">
-        <v>820</v>
+        <v>760</v>
       </c>
     </row>
     <row r="265">
@@ -6995,24 +7001,24 @@
         <v>581</v>
       </c>
       <c r="C265" s="0" t="s">
-        <v>582</v>
+        <v>19</v>
       </c>
       <c r="D265" s="0">
-        <v>177940.1</v>
+        <v>820</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="0" t="s">
+        <v>582</v>
+      </c>
+      <c r="B266" s="0" t="s">
         <v>583</v>
       </c>
-      <c r="B266" s="0" t="s">
+      <c r="C266" s="0" t="s">
         <v>584</v>
       </c>
-      <c r="C266" s="0" t="s">
-        <v>71</v>
-      </c>
       <c r="D266" s="0">
-        <v>34000</v>
+        <v>177940.1</v>
       </c>
     </row>
     <row r="267">
@@ -7026,7 +7032,7 @@
         <v>71</v>
       </c>
       <c r="D267" s="0">
-        <v>30000</v>
+        <v>34000</v>
       </c>
     </row>
     <row r="268">
@@ -7037,10 +7043,10 @@
         <v>588</v>
       </c>
       <c r="C268" s="0" t="s">
-        <v>477</v>
+        <v>71</v>
       </c>
       <c r="D268" s="0">
-        <v>227939.52</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="269">
@@ -7051,10 +7057,10 @@
         <v>590</v>
       </c>
       <c r="C269" s="0" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="D269" s="0">
-        <v>184488.7</v>
+        <v>227939.52</v>
       </c>
     </row>
     <row r="270">
@@ -7065,10 +7071,10 @@
         <v>592</v>
       </c>
       <c r="C270" s="0" t="s">
-        <v>16</v>
+        <v>479</v>
       </c>
       <c r="D270" s="0">
-        <v>1760</v>
+        <v>184488.7</v>
       </c>
     </row>
     <row r="271">
@@ -7079,24 +7085,24 @@
         <v>594</v>
       </c>
       <c r="C271" s="0" t="s">
-        <v>595</v>
+        <v>16</v>
       </c>
       <c r="D271" s="0">
-        <v>26350</v>
+        <v>1760</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="0" t="s">
+        <v>595</v>
+      </c>
+      <c r="B272" s="0" t="s">
         <v>596</v>
       </c>
-      <c r="B272" s="0" t="s">
+      <c r="C272" s="0" t="s">
         <v>597</v>
       </c>
-      <c r="C272" s="0" t="s">
-        <v>486</v>
-      </c>
       <c r="D272" s="0">
-        <v>31250</v>
+        <v>26350</v>
       </c>
     </row>
     <row r="273">
@@ -7107,10 +7113,10 @@
         <v>599</v>
       </c>
       <c r="C273" s="0" t="s">
-        <v>53</v>
+        <v>488</v>
       </c>
       <c r="D273" s="0">
-        <v>34.98</v>
+        <v>31250</v>
       </c>
     </row>
     <row r="274">
@@ -7121,21 +7127,21 @@
         <v>601</v>
       </c>
       <c r="C274" s="0" t="s">
-        <v>602</v>
+        <v>53</v>
       </c>
       <c r="D274" s="0">
-        <v>65</v>
+        <v>34.98</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="0" t="s">
+        <v>602</v>
+      </c>
+      <c r="B275" s="0" t="s">
         <v>603</v>
       </c>
-      <c r="B275" s="0" t="s">
+      <c r="C275" s="0" t="s">
         <v>604</v>
-      </c>
-      <c r="C275" s="0" t="s">
-        <v>53</v>
       </c>
       <c r="D275" s="0">
         <v>65</v>
@@ -7152,7 +7158,7 @@
         <v>53</v>
       </c>
       <c r="D276" s="0">
-        <v>92</v>
+        <v>65</v>
       </c>
     </row>
     <row r="277">
@@ -7166,7 +7172,7 @@
         <v>53</v>
       </c>
       <c r="D277" s="0">
-        <v>33</v>
+        <v>92</v>
       </c>
     </row>
     <row r="278">
@@ -7180,7 +7186,7 @@
         <v>53</v>
       </c>
       <c r="D278" s="0">
-        <v>38.22</v>
+        <v>33</v>
       </c>
     </row>
     <row r="279">
@@ -7191,10 +7197,10 @@
         <v>612</v>
       </c>
       <c r="C279" s="0" t="s">
-        <v>340</v>
+        <v>53</v>
       </c>
       <c r="D279" s="0">
-        <v>300</v>
+        <v>38.22</v>
       </c>
     </row>
     <row r="280">
@@ -7208,7 +7214,7 @@
         <v>340</v>
       </c>
       <c r="D280" s="0">
-        <v>370</v>
+        <v>300</v>
       </c>
     </row>
     <row r="281">
@@ -7219,10 +7225,10 @@
         <v>616</v>
       </c>
       <c r="C281" s="0" t="s">
-        <v>361</v>
+        <v>340</v>
       </c>
       <c r="D281" s="0">
-        <v>450</v>
+        <v>370</v>
       </c>
     </row>
     <row r="282">
@@ -7233,7 +7239,7 @@
         <v>618</v>
       </c>
       <c r="C282" s="0" t="s">
-        <v>38</v>
+        <v>361</v>
       </c>
       <c r="D282" s="0">
         <v>450</v>
@@ -7247,7 +7253,7 @@
         <v>620</v>
       </c>
       <c r="C283" s="0" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="D283" s="0">
         <v>450</v>
@@ -7264,7 +7270,7 @@
         <v>16</v>
       </c>
       <c r="D284" s="0">
-        <v>1650</v>
+        <v>450</v>
       </c>
     </row>
     <row r="285">
@@ -7278,7 +7284,7 @@
         <v>16</v>
       </c>
       <c r="D285" s="0">
-        <v>2100</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="286">
@@ -7292,7 +7298,7 @@
         <v>16</v>
       </c>
       <c r="D286" s="0">
-        <v>1980</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="287">
@@ -7306,7 +7312,7 @@
         <v>16</v>
       </c>
       <c r="D287" s="0">
-        <v>2160</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="288">
@@ -7320,7 +7326,7 @@
         <v>16</v>
       </c>
       <c r="D288" s="0">
-        <v>1100</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="289">
@@ -7334,7 +7340,7 @@
         <v>16</v>
       </c>
       <c r="D289" s="0">
-        <v>2600</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="290">
@@ -7348,7 +7354,7 @@
         <v>16</v>
       </c>
       <c r="D290" s="0">
-        <v>2000</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="291">
@@ -7362,7 +7368,7 @@
         <v>16</v>
       </c>
       <c r="D291" s="0">
-        <v>6700</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="292">
@@ -7376,7 +7382,7 @@
         <v>16</v>
       </c>
       <c r="D292" s="0">
-        <v>1650</v>
+        <v>6700</v>
       </c>
     </row>
     <row r="293">
@@ -7390,7 +7396,7 @@
         <v>16</v>
       </c>
       <c r="D293" s="0">
-        <v>1035</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="294">
@@ -7404,7 +7410,7 @@
         <v>16</v>
       </c>
       <c r="D294" s="0">
-        <v>2600</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="295">
@@ -7418,7 +7424,7 @@
         <v>16</v>
       </c>
       <c r="D295" s="0">
-        <v>2400</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="296">
@@ -7429,10 +7435,10 @@
         <v>646</v>
       </c>
       <c r="C296" s="0" t="s">
-        <v>137</v>
+        <v>16</v>
       </c>
       <c r="D296" s="0">
-        <v>4497.2</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="297">
@@ -7446,7 +7452,7 @@
         <v>137</v>
       </c>
       <c r="D297" s="0">
-        <v>2328</v>
+        <v>4497.2</v>
       </c>
     </row>
     <row r="298">
@@ -7460,7 +7466,7 @@
         <v>137</v>
       </c>
       <c r="D298" s="0">
-        <v>1138</v>
+        <v>2328</v>
       </c>
     </row>
     <row r="299">
@@ -7471,10 +7477,10 @@
         <v>652</v>
       </c>
       <c r="C299" s="0" t="s">
-        <v>29</v>
+        <v>137</v>
       </c>
       <c r="D299" s="0">
-        <v>7372.42</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="300">
@@ -7485,10 +7491,10 @@
         <v>654</v>
       </c>
       <c r="C300" s="0" t="s">
-        <v>120</v>
+        <v>29</v>
       </c>
       <c r="D300" s="0">
-        <v>1790</v>
+        <v>7372.42</v>
       </c>
     </row>
     <row r="301">
@@ -7502,7 +7508,7 @@
         <v>120</v>
       </c>
       <c r="D301" s="0">
-        <v>2859.96</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="302">
@@ -7516,7 +7522,7 @@
         <v>120</v>
       </c>
       <c r="D302" s="0">
-        <v>4800</v>
+        <v>2859.96</v>
       </c>
     </row>
     <row r="303">
@@ -7527,24 +7533,24 @@
         <v>660</v>
       </c>
       <c r="C303" s="0" t="s">
-        <v>661</v>
+        <v>120</v>
       </c>
       <c r="D303" s="0">
-        <v>0</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="0" t="s">
+        <v>661</v>
+      </c>
+      <c r="B304" s="0" t="s">
         <v>662</v>
       </c>
-      <c r="B304" s="0" t="s">
+      <c r="C304" s="0" t="s">
         <v>663</v>
       </c>
-      <c r="C304" s="0" t="s">
-        <v>29</v>
-      </c>
       <c r="D304" s="0">
-        <v>494</v>
+        <v>0</v>
       </c>
     </row>
     <row r="305">
@@ -7558,7 +7564,7 @@
         <v>29</v>
       </c>
       <c r="D305" s="0">
-        <v>665.3</v>
+        <v>494</v>
       </c>
     </row>
     <row r="306">
@@ -7569,10 +7575,10 @@
         <v>667</v>
       </c>
       <c r="C306" s="0" t="s">
-        <v>91</v>
+        <v>29</v>
       </c>
       <c r="D306" s="0">
-        <v>33275</v>
+        <v>665.3</v>
       </c>
     </row>
     <row r="307">
@@ -7586,7 +7592,7 @@
         <v>91</v>
       </c>
       <c r="D307" s="0">
-        <v>4525.4</v>
+        <v>33275</v>
       </c>
     </row>
     <row r="308">
@@ -7597,10 +7603,10 @@
         <v>671</v>
       </c>
       <c r="C308" s="0" t="s">
-        <v>148</v>
+        <v>91</v>
       </c>
       <c r="D308" s="0">
-        <v>896</v>
+        <v>4525.4</v>
       </c>
     </row>
     <row r="309">
@@ -7611,10 +7617,10 @@
         <v>673</v>
       </c>
       <c r="C309" s="0" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="D309" s="0">
-        <v>1250</v>
+        <v>896</v>
       </c>
     </row>
     <row r="310">
@@ -7625,10 +7631,10 @@
         <v>675</v>
       </c>
       <c r="C310" s="0" t="s">
-        <v>91</v>
+        <v>137</v>
       </c>
       <c r="D310" s="0">
-        <v>312785</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="311">
@@ -7639,10 +7645,10 @@
         <v>677</v>
       </c>
       <c r="C311" s="0" t="s">
-        <v>204</v>
+        <v>91</v>
       </c>
       <c r="D311" s="0">
-        <v>17440</v>
+        <v>312785</v>
       </c>
     </row>
     <row r="312">
@@ -7656,7 +7662,7 @@
         <v>204</v>
       </c>
       <c r="D312" s="0">
-        <v>4390</v>
+        <v>17440</v>
       </c>
     </row>
     <row r="313">
@@ -7681,10 +7687,10 @@
         <v>683</v>
       </c>
       <c r="C314" s="0" t="s">
-        <v>285</v>
+        <v>204</v>
       </c>
       <c r="D314" s="0">
-        <v>2250</v>
+        <v>4390</v>
       </c>
     </row>
     <row r="315">
@@ -7695,10 +7701,10 @@
         <v>685</v>
       </c>
       <c r="C315" s="0" t="s">
-        <v>204</v>
+        <v>285</v>
       </c>
       <c r="D315" s="0">
-        <v>3355</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="316">
@@ -7709,10 +7715,10 @@
         <v>687</v>
       </c>
       <c r="C316" s="0" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="D316" s="0">
-        <v>7500</v>
+        <v>3355</v>
       </c>
     </row>
     <row r="317">
@@ -7723,10 +7729,10 @@
         <v>689</v>
       </c>
       <c r="C317" s="0" t="s">
-        <v>91</v>
+        <v>209</v>
       </c>
       <c r="D317" s="0">
-        <v>23958</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="318">
@@ -7740,7 +7746,7 @@
         <v>91</v>
       </c>
       <c r="D318" s="0">
-        <v>239580</v>
+        <v>23958</v>
       </c>
     </row>
     <row r="319">
@@ -7751,10 +7757,10 @@
         <v>693</v>
       </c>
       <c r="C319" s="0" t="s">
-        <v>53</v>
+        <v>91</v>
       </c>
       <c r="D319" s="0">
-        <v>130</v>
+        <v>239580</v>
       </c>
     </row>
     <row r="320">
@@ -7765,10 +7771,10 @@
         <v>695</v>
       </c>
       <c r="C320" s="0" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="D320" s="0">
-        <v>285.6</v>
+        <v>130</v>
       </c>
     </row>
     <row r="321">
@@ -7782,7 +7788,7 @@
         <v>22</v>
       </c>
       <c r="D321" s="0">
-        <v>338</v>
+        <v>285.6</v>
       </c>
     </row>
     <row r="322">
@@ -7793,21 +7799,21 @@
         <v>699</v>
       </c>
       <c r="C322" s="0" t="s">
-        <v>700</v>
+        <v>22</v>
       </c>
       <c r="D322" s="0">
-        <v>770</v>
+        <v>338</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="0" t="s">
+        <v>700</v>
+      </c>
+      <c r="B323" s="0" t="s">
         <v>701</v>
       </c>
-      <c r="B323" s="0" t="s">
+      <c r="C323" s="0" t="s">
         <v>702</v>
-      </c>
-      <c r="C323" s="0" t="s">
-        <v>703</v>
       </c>
       <c r="D323" s="0">
         <v>770</v>
@@ -7815,16 +7821,16 @@
     </row>
     <row r="324">
       <c r="A324" s="0" t="s">
+        <v>703</v>
+      </c>
+      <c r="B324" s="0" t="s">
         <v>704</v>
       </c>
-      <c r="B324" s="0" t="s">
+      <c r="C324" s="0" t="s">
         <v>705</v>
       </c>
-      <c r="C324" s="0" t="s">
-        <v>16</v>
-      </c>
       <c r="D324" s="0">
-        <v>973.5</v>
+        <v>770</v>
       </c>
     </row>
     <row r="325">
@@ -7835,10 +7841,10 @@
         <v>707</v>
       </c>
       <c r="C325" s="0" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D325" s="0">
-        <v>507.08</v>
+        <v>973.5</v>
       </c>
     </row>
     <row r="326">
@@ -7849,10 +7855,10 @@
         <v>709</v>
       </c>
       <c r="C326" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D326" s="0">
-        <v>450</v>
+        <v>507.08</v>
       </c>
     </row>
     <row r="327">
@@ -7863,10 +7869,10 @@
         <v>711</v>
       </c>
       <c r="C327" s="0" t="s">
-        <v>148</v>
+        <v>16</v>
       </c>
       <c r="D327" s="0">
-        <v>760</v>
+        <v>450</v>
       </c>
     </row>
     <row r="328">
@@ -7877,10 +7883,10 @@
         <v>713</v>
       </c>
       <c r="C328" s="0" t="s">
-        <v>285</v>
+        <v>148</v>
       </c>
       <c r="D328" s="0">
-        <v>5900</v>
+        <v>760</v>
       </c>
     </row>
     <row r="329">
@@ -7894,7 +7900,7 @@
         <v>285</v>
       </c>
       <c r="D329" s="0">
-        <v>2900</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="330">
@@ -7905,10 +7911,10 @@
         <v>717</v>
       </c>
       <c r="C330" s="0" t="s">
-        <v>137</v>
+        <v>285</v>
       </c>
       <c r="D330" s="0">
-        <v>886.2</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="331">
@@ -7922,7 +7928,7 @@
         <v>137</v>
       </c>
       <c r="D331" s="0">
-        <v>589.9</v>
+        <v>886.2</v>
       </c>
     </row>
     <row r="332">
@@ -7936,7 +7942,7 @@
         <v>137</v>
       </c>
       <c r="D332" s="0">
-        <v>65</v>
+        <v>589.9</v>
       </c>
     </row>
     <row r="333">
@@ -7947,10 +7953,10 @@
         <v>723</v>
       </c>
       <c r="C333" s="0" t="s">
-        <v>91</v>
+        <v>137</v>
       </c>
       <c r="D333" s="0">
-        <v>11313.5</v>
+        <v>65</v>
       </c>
     </row>
     <row r="334">
@@ -7961,10 +7967,10 @@
         <v>725</v>
       </c>
       <c r="C334" s="0" t="s">
-        <v>35</v>
+        <v>91</v>
       </c>
       <c r="D334" s="0">
-        <v>420</v>
+        <v>11313.5</v>
       </c>
     </row>
     <row r="335">
@@ -7975,10 +7981,10 @@
         <v>727</v>
       </c>
       <c r="C335" s="0" t="s">
-        <v>361</v>
+        <v>35</v>
       </c>
       <c r="D335" s="0">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="336">
@@ -7989,10 +7995,10 @@
         <v>729</v>
       </c>
       <c r="C336" s="0" t="s">
-        <v>22</v>
+        <v>361</v>
       </c>
       <c r="D336" s="0">
-        <v>377</v>
+        <v>418</v>
       </c>
     </row>
     <row r="337">
@@ -8003,10 +8009,10 @@
         <v>731</v>
       </c>
       <c r="C337" s="0" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="D337" s="0">
-        <v>5781.24</v>
+        <v>377</v>
       </c>
     </row>
     <row r="338">
@@ -8017,10 +8023,10 @@
         <v>733</v>
       </c>
       <c r="C338" s="0" t="s">
-        <v>71</v>
+        <v>46</v>
       </c>
       <c r="D338" s="0">
-        <v>898</v>
+        <v>5780.66</v>
       </c>
     </row>
     <row r="339">
@@ -8031,10 +8037,10 @@
         <v>735</v>
       </c>
       <c r="C339" s="0" t="s">
-        <v>120</v>
+        <v>71</v>
       </c>
       <c r="D339" s="0">
-        <v>4767</v>
+        <v>898</v>
       </c>
     </row>
     <row r="340">
@@ -8045,10 +8051,10 @@
         <v>737</v>
       </c>
       <c r="C340" s="0" t="s">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="D340" s="0">
-        <v>650</v>
+        <v>4767</v>
       </c>
     </row>
     <row r="341">
@@ -8059,7 +8065,7 @@
         <v>739</v>
       </c>
       <c r="C341" s="0" t="s">
-        <v>71</v>
+        <v>35</v>
       </c>
       <c r="D341" s="0">
         <v>650</v>
@@ -8073,10 +8079,10 @@
         <v>741</v>
       </c>
       <c r="C342" s="0" t="s">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="D342" s="0">
-        <v>2178</v>
+        <v>650</v>
       </c>
     </row>
     <row r="343">
@@ -8087,10 +8093,10 @@
         <v>743</v>
       </c>
       <c r="C343" s="0" t="s">
-        <v>91</v>
+        <v>16</v>
       </c>
       <c r="D343" s="0">
-        <v>7986</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="344">
@@ -8101,24 +8107,24 @@
         <v>745</v>
       </c>
       <c r="C344" s="0" t="s">
-        <v>746</v>
+        <v>91</v>
       </c>
       <c r="D344" s="0">
-        <v>1910</v>
+        <v>7986</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="0" t="s">
+        <v>746</v>
+      </c>
+      <c r="B345" s="0" t="s">
         <v>747</v>
       </c>
-      <c r="B345" s="0" t="s">
+      <c r="C345" s="0" t="s">
         <v>748</v>
       </c>
-      <c r="C345" s="0" t="s">
-        <v>148</v>
-      </c>
       <c r="D345" s="0">
-        <v>900</v>
+        <v>1910</v>
       </c>
     </row>
     <row r="346">
@@ -8129,10 +8135,10 @@
         <v>750</v>
       </c>
       <c r="C346" s="0" t="s">
-        <v>22</v>
+        <v>148</v>
       </c>
       <c r="D346" s="0">
-        <v>1722</v>
+        <v>900</v>
       </c>
     </row>
     <row r="347">
@@ -8143,10 +8149,10 @@
         <v>752</v>
       </c>
       <c r="C347" s="0" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="D347" s="0">
-        <v>456</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="348">
@@ -8160,7 +8166,7 @@
         <v>35</v>
       </c>
       <c r="D348" s="0">
-        <v>59000</v>
+        <v>456</v>
       </c>
     </row>
     <row r="349">
@@ -8171,10 +8177,10 @@
         <v>756</v>
       </c>
       <c r="C349" s="0" t="s">
-        <v>148</v>
+        <v>35</v>
       </c>
       <c r="D349" s="0">
-        <v>750</v>
+        <v>59000</v>
       </c>
     </row>
     <row r="350">
@@ -8188,7 +8194,7 @@
         <v>148</v>
       </c>
       <c r="D350" s="0">
-        <v>1212</v>
+        <v>750</v>
       </c>
     </row>
     <row r="351">
@@ -8202,7 +8208,7 @@
         <v>148</v>
       </c>
       <c r="D351" s="0">
-        <v>1300</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="352">
@@ -8216,7 +8222,7 @@
         <v>148</v>
       </c>
       <c r="D352" s="0">
-        <v>1500</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="353">
@@ -8230,7 +8236,7 @@
         <v>148</v>
       </c>
       <c r="D353" s="0">
-        <v>1400</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="354">
@@ -8241,10 +8247,10 @@
         <v>766</v>
       </c>
       <c r="C354" s="0" t="s">
-        <v>261</v>
+        <v>148</v>
       </c>
       <c r="D354" s="0">
-        <v>11959</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="355">
@@ -8255,10 +8261,10 @@
         <v>768</v>
       </c>
       <c r="C355" s="0" t="s">
-        <v>137</v>
+        <v>261</v>
       </c>
       <c r="D355" s="0">
-        <v>345</v>
+        <v>11959</v>
       </c>
     </row>
     <row r="356">
@@ -8269,10 +8275,10 @@
         <v>770</v>
       </c>
       <c r="C356" s="0" t="s">
-        <v>285</v>
+        <v>137</v>
       </c>
       <c r="D356" s="0">
-        <v>1450</v>
+        <v>345</v>
       </c>
     </row>
     <row r="357">
@@ -8283,10 +8289,10 @@
         <v>772</v>
       </c>
       <c r="C357" s="0" t="s">
-        <v>91</v>
+        <v>285</v>
       </c>
       <c r="D357" s="0">
-        <v>7320.5</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="358">
@@ -8297,10 +8303,10 @@
         <v>774</v>
       </c>
       <c r="C358" s="0" t="s">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="D358" s="0">
-        <v>900</v>
+        <v>7320.5</v>
       </c>
     </row>
     <row r="359">
@@ -8311,10 +8317,10 @@
         <v>776</v>
       </c>
       <c r="C359" s="0" t="s">
-        <v>285</v>
+        <v>16</v>
       </c>
       <c r="D359" s="0">
-        <v>520</v>
+        <v>900</v>
       </c>
     </row>
     <row r="360">
@@ -8325,10 +8331,10 @@
         <v>778</v>
       </c>
       <c r="C360" s="0" t="s">
-        <v>477</v>
+        <v>285</v>
       </c>
       <c r="D360" s="0">
-        <v>64925</v>
+        <v>520</v>
       </c>
     </row>
     <row r="361">
@@ -8339,10 +8345,10 @@
         <v>780</v>
       </c>
       <c r="C361" s="0" t="s">
-        <v>16</v>
+        <v>479</v>
       </c>
       <c r="D361" s="0">
-        <v>1100</v>
+        <v>64925</v>
       </c>
     </row>
     <row r="362">
@@ -8353,10 +8359,10 @@
         <v>782</v>
       </c>
       <c r="C362" s="0" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D362" s="0">
-        <v>1623</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="363">
@@ -8367,10 +8373,10 @@
         <v>784</v>
       </c>
       <c r="C363" s="0" t="s">
-        <v>137</v>
+        <v>22</v>
       </c>
       <c r="D363" s="0">
-        <v>1182.75</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="364">
@@ -8384,7 +8390,7 @@
         <v>137</v>
       </c>
       <c r="D364" s="0">
-        <v>4440.9</v>
+        <v>1182.75</v>
       </c>
     </row>
     <row r="365">
@@ -8395,10 +8401,10 @@
         <v>788</v>
       </c>
       <c r="C365" s="0" t="s">
-        <v>29</v>
+        <v>137</v>
       </c>
       <c r="D365" s="0">
-        <v>1250</v>
+        <v>4440.9</v>
       </c>
     </row>
     <row r="366">
@@ -8412,7 +8418,7 @@
         <v>29</v>
       </c>
       <c r="D366" s="0">
-        <v>1945.1</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="367">
@@ -8423,10 +8429,10 @@
         <v>792</v>
       </c>
       <c r="C367" s="0" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="D367" s="0">
-        <v>450</v>
+        <v>1945.1</v>
       </c>
     </row>
     <row r="368">
@@ -8440,7 +8446,7 @@
         <v>16</v>
       </c>
       <c r="D368" s="0">
-        <v>825</v>
+        <v>450</v>
       </c>
     </row>
     <row r="369">
@@ -8465,10 +8471,10 @@
         <v>798</v>
       </c>
       <c r="C370" s="0" t="s">
-        <v>379</v>
+        <v>16</v>
       </c>
       <c r="D370" s="0">
-        <v>134775.6</v>
+        <v>825</v>
       </c>
     </row>
     <row r="371">
@@ -8479,10 +8485,10 @@
         <v>800</v>
       </c>
       <c r="C371" s="0" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="D371" s="0">
-        <v>175991.55</v>
+        <v>134775.6</v>
       </c>
     </row>
     <row r="372">
@@ -8493,10 +8499,10 @@
         <v>802</v>
       </c>
       <c r="C372" s="0" t="s">
-        <v>71</v>
+        <v>381</v>
       </c>
       <c r="D372" s="0">
-        <v>3263</v>
+        <v>175991.55</v>
       </c>
     </row>
     <row r="373">
@@ -8510,7 +8516,7 @@
         <v>71</v>
       </c>
       <c r="D373" s="0">
-        <v>18027</v>
+        <v>3263</v>
       </c>
     </row>
     <row r="374">
@@ -8521,10 +8527,10 @@
         <v>806</v>
       </c>
       <c r="C374" s="0" t="s">
-        <v>285</v>
+        <v>71</v>
       </c>
       <c r="D374" s="0">
-        <v>515</v>
+        <v>18027</v>
       </c>
     </row>
     <row r="375">
@@ -8535,38 +8541,38 @@
         <v>808</v>
       </c>
       <c r="C375" s="0" t="s">
-        <v>38</v>
+        <v>285</v>
       </c>
       <c r="D375" s="0">
         <v>515</v>
       </c>
     </row>
     <row r="376">
-      <c r="A376" s="2" t="s">
+      <c r="A376" s="0" t="s">
         <v>809</v>
       </c>
-      <c r="B376" s="2" t="s">
+      <c r="B376" s="0" t="s">
         <v>810</v>
       </c>
-      <c r="C376" s="2" t="s">
+      <c r="C376" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="D376" s="0">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="2" t="s">
+        <v>811</v>
+      </c>
+      <c r="B377" s="2" t="s">
+        <v>812</v>
+      </c>
+      <c r="C377" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D376" s="2">
+      <c r="D377" s="2">
         <v>10154</v>
-      </c>
-    </row>
-    <row r="377">
-      <c r="A377" s="0" t="s">
-        <v>811</v>
-      </c>
-      <c r="B377" s="0" t="s">
-        <v>812</v>
-      </c>
-      <c r="C377" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="D377" s="0">
-        <v>9500</v>
       </c>
     </row>
     <row r="378">
@@ -8577,10 +8583,10 @@
         <v>814</v>
       </c>
       <c r="C378" s="0" t="s">
-        <v>477</v>
+        <v>53</v>
       </c>
       <c r="D378" s="0">
-        <v>207558.08</v>
+        <v>9500</v>
       </c>
     </row>
     <row r="379">
@@ -8591,10 +8597,10 @@
         <v>816</v>
       </c>
       <c r="C379" s="0" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="D379" s="0">
-        <v>249069.69</v>
+        <v>207558.08</v>
       </c>
     </row>
     <row r="380">
@@ -8605,10 +8611,10 @@
         <v>818</v>
       </c>
       <c r="C380" s="0" t="s">
-        <v>71</v>
+        <v>479</v>
       </c>
       <c r="D380" s="0">
-        <v>10021.22</v>
+        <v>249069.69</v>
       </c>
     </row>
     <row r="381">
@@ -8622,7 +8628,7 @@
         <v>71</v>
       </c>
       <c r="D381" s="0">
-        <v>17710</v>
+        <v>10021.22</v>
       </c>
     </row>
     <row r="382">
@@ -8633,24 +8639,24 @@
         <v>822</v>
       </c>
       <c r="C382" s="0" t="s">
-        <v>823</v>
+        <v>71</v>
       </c>
       <c r="D382" s="0">
-        <v>1080</v>
+        <v>17710</v>
       </c>
     </row>
     <row r="383">
       <c r="A383" s="0" t="s">
+        <v>823</v>
+      </c>
+      <c r="B383" s="0" t="s">
         <v>824</v>
       </c>
-      <c r="B383" s="0" t="s">
+      <c r="C383" s="0" t="s">
         <v>825</v>
       </c>
-      <c r="C383" s="0" t="s">
-        <v>19</v>
-      </c>
       <c r="D383" s="0">
-        <v>570</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="384">
@@ -8661,24 +8667,24 @@
         <v>827</v>
       </c>
       <c r="C384" s="0" t="s">
-        <v>828</v>
+        <v>19</v>
       </c>
       <c r="D384" s="0">
-        <v>520</v>
+        <v>570</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="0" t="s">
+        <v>828</v>
+      </c>
+      <c r="B385" s="0" t="s">
         <v>829</v>
       </c>
-      <c r="B385" s="0" t="s">
+      <c r="C385" s="0" t="s">
         <v>830</v>
       </c>
-      <c r="C385" s="0" t="s">
-        <v>828</v>
-      </c>
       <c r="D385" s="0">
-        <v>300</v>
+        <v>520</v>
       </c>
     </row>
     <row r="386">
@@ -8689,10 +8695,10 @@
         <v>832</v>
       </c>
       <c r="C386" s="0" t="s">
-        <v>16</v>
+        <v>830</v>
       </c>
       <c r="D386" s="0">
-        <v>2200</v>
+        <v>300</v>
       </c>
     </row>
     <row r="387">
@@ -8706,7 +8712,7 @@
         <v>16</v>
       </c>
       <c r="D387" s="0">
-        <v>2800</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="388">
@@ -8717,10 +8723,10 @@
         <v>836</v>
       </c>
       <c r="C388" s="0" t="s">
-        <v>91</v>
+        <v>16</v>
       </c>
       <c r="D388" s="0">
-        <v>4791.6</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="389">
@@ -8731,10 +8737,10 @@
         <v>838</v>
       </c>
       <c r="C389" s="0" t="s">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="D389" s="0">
-        <v>2699.64</v>
+        <v>4791.6</v>
       </c>
     </row>
     <row r="390">
@@ -8745,10 +8751,10 @@
         <v>840</v>
       </c>
       <c r="C390" s="0" t="s">
-        <v>35</v>
+        <v>71</v>
       </c>
       <c r="D390" s="0">
-        <v>3800</v>
+        <v>2699.64</v>
       </c>
     </row>
     <row r="391">
@@ -8759,10 +8765,10 @@
         <v>842</v>
       </c>
       <c r="C391" s="0" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D391" s="0">
-        <v>4000</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="392">
@@ -8773,24 +8779,24 @@
         <v>844</v>
       </c>
       <c r="C392" s="0" t="s">
-        <v>845</v>
+        <v>16</v>
       </c>
       <c r="D392" s="0">
-        <v>3800</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="0" t="s">
+        <v>845</v>
+      </c>
+      <c r="B393" s="0" t="s">
         <v>846</v>
       </c>
-      <c r="B393" s="0" t="s">
+      <c r="C393" s="0" t="s">
         <v>847</v>
       </c>
-      <c r="C393" s="0" t="s">
-        <v>22</v>
-      </c>
       <c r="D393" s="0">
-        <v>353</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="394">
@@ -8801,10 +8807,10 @@
         <v>849</v>
       </c>
       <c r="C394" s="0" t="s">
-        <v>109</v>
+        <v>22</v>
       </c>
       <c r="D394" s="0">
-        <v>1800</v>
+        <v>353</v>
       </c>
     </row>
     <row r="395">
@@ -8815,10 +8821,10 @@
         <v>851</v>
       </c>
       <c r="C395" s="0" t="s">
-        <v>16</v>
+        <v>109</v>
       </c>
       <c r="D395" s="0">
-        <v>2948</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="396">
@@ -8829,10 +8835,10 @@
         <v>853</v>
       </c>
       <c r="C396" s="0" t="s">
-        <v>209</v>
+        <v>16</v>
       </c>
       <c r="D396" s="0">
-        <v>65537</v>
+        <v>2948</v>
       </c>
     </row>
     <row r="397">
@@ -8843,10 +8849,10 @@
         <v>855</v>
       </c>
       <c r="C397" s="0" t="s">
-        <v>137</v>
+        <v>209</v>
       </c>
       <c r="D397" s="0">
-        <v>4049.6</v>
+        <v>65537</v>
       </c>
     </row>
     <row r="398">
@@ -8860,7 +8866,7 @@
         <v>137</v>
       </c>
       <c r="D398" s="0">
-        <v>4199.2</v>
+        <v>4049.6</v>
       </c>
     </row>
     <row r="399">
@@ -8874,7 +8880,7 @@
         <v>137</v>
       </c>
       <c r="D399" s="0">
-        <v>6397.2</v>
+        <v>4199.2</v>
       </c>
     </row>
     <row r="400">
@@ -8885,10 +8891,10 @@
         <v>861</v>
       </c>
       <c r="C400" s="0" t="s">
-        <v>312</v>
+        <v>137</v>
       </c>
       <c r="D400" s="0">
-        <v>570</v>
+        <v>6397.2</v>
       </c>
     </row>
     <row r="401">
@@ -8899,10 +8905,10 @@
         <v>863</v>
       </c>
       <c r="C401" s="0" t="s">
-        <v>71</v>
+        <v>312</v>
       </c>
       <c r="D401" s="0">
-        <v>550</v>
+        <v>570</v>
       </c>
     </row>
     <row r="402">
@@ -8913,10 +8919,10 @@
         <v>865</v>
       </c>
       <c r="C402" s="0" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="D402" s="0">
-        <v>167</v>
+        <v>550</v>
       </c>
     </row>
     <row r="403">
@@ -8927,10 +8933,10 @@
         <v>867</v>
       </c>
       <c r="C403" s="0" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="D403" s="0">
-        <v>714.74</v>
+        <v>167</v>
       </c>
     </row>
     <row r="404">
@@ -8941,10 +8947,10 @@
         <v>869</v>
       </c>
       <c r="C404" s="0" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="D404" s="0">
-        <v>101000</v>
+        <v>714.74</v>
       </c>
     </row>
     <row r="405">
@@ -8955,10 +8961,10 @@
         <v>871</v>
       </c>
       <c r="C405" s="0" t="s">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="D405" s="0">
-        <v>6251</v>
+        <v>101000</v>
       </c>
     </row>
     <row r="406">
@@ -8969,10 +8975,10 @@
         <v>873</v>
       </c>
       <c r="C406" s="0" t="s">
-        <v>376</v>
+        <v>120</v>
       </c>
       <c r="D406" s="0">
-        <v>857.67</v>
+        <v>6251</v>
       </c>
     </row>
     <row r="407">
@@ -8983,10 +8989,10 @@
         <v>875</v>
       </c>
       <c r="C407" s="0" t="s">
-        <v>91</v>
+        <v>378</v>
       </c>
       <c r="D407" s="0">
-        <v>1164.66</v>
+        <v>857.67</v>
       </c>
     </row>
     <row r="408">
@@ -8997,10 +9003,10 @@
         <v>877</v>
       </c>
       <c r="C408" s="0" t="s">
-        <v>148</v>
+        <v>91</v>
       </c>
       <c r="D408" s="0">
-        <v>360</v>
+        <v>1164.66</v>
       </c>
     </row>
     <row r="409">
@@ -9014,7 +9020,7 @@
         <v>148</v>
       </c>
       <c r="D409" s="0">
-        <v>450</v>
+        <v>360</v>
       </c>
     </row>
     <row r="410">
@@ -9028,7 +9034,7 @@
         <v>148</v>
       </c>
       <c r="D410" s="0">
-        <v>2050</v>
+        <v>450</v>
       </c>
     </row>
     <row r="411">
@@ -9039,10 +9045,10 @@
         <v>883</v>
       </c>
       <c r="C411" s="0" t="s">
-        <v>582</v>
+        <v>148</v>
       </c>
       <c r="D411" s="0">
-        <v>25192.82</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="412">
@@ -9053,10 +9059,10 @@
         <v>885</v>
       </c>
       <c r="C412" s="0" t="s">
-        <v>71</v>
+        <v>584</v>
       </c>
       <c r="D412" s="0">
-        <v>3500</v>
+        <v>25192.82</v>
       </c>
     </row>
     <row r="413">
@@ -9067,10 +9073,10 @@
         <v>887</v>
       </c>
       <c r="C413" s="0" t="s">
-        <v>177</v>
+        <v>71</v>
       </c>
       <c r="D413" s="0">
-        <v>600</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="414">
@@ -9081,52 +9087,52 @@
         <v>889</v>
       </c>
       <c r="C414" s="0" t="s">
-        <v>890</v>
+        <v>177</v>
       </c>
       <c r="D414" s="0">
-        <v>1080</v>
+        <v>600</v>
       </c>
     </row>
     <row r="415">
       <c r="A415" s="0" t="s">
+        <v>890</v>
+      </c>
+      <c r="B415" s="0" t="s">
         <v>891</v>
       </c>
-      <c r="B415" s="0" t="s">
+      <c r="C415" s="0" t="s">
         <v>892</v>
       </c>
-      <c r="C415" s="0" t="s">
+      <c r="D415" s="0">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="0" t="s">
+        <v>893</v>
+      </c>
+      <c r="B416" s="0" t="s">
+        <v>894</v>
+      </c>
+      <c r="C416" s="0" t="s">
         <v>340</v>
       </c>
-      <c r="D415" s="0">
+      <c r="D416" s="0">
         <v>8628</v>
       </c>
     </row>
-    <row r="416">
-      <c r="A416" s="2" t="s">
-        <v>893</v>
-      </c>
-      <c r="B416" s="2" t="s">
-        <v>894</v>
-      </c>
-      <c r="C416" s="2" t="s">
+    <row r="417">
+      <c r="A417" s="2" t="s">
+        <v>895</v>
+      </c>
+      <c r="B417" s="2" t="s">
+        <v>896</v>
+      </c>
+      <c r="C417" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="D416" s="2">
+      <c r="D417" s="2">
         <v>9125.1</v>
-      </c>
-    </row>
-    <row r="417">
-      <c r="A417" s="0" t="s">
-        <v>895</v>
-      </c>
-      <c r="B417" s="0" t="s">
-        <v>896</v>
-      </c>
-      <c r="C417" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="D417" s="0">
-        <v>27991.54</v>
       </c>
     </row>
     <row r="418">
@@ -9137,10 +9143,10 @@
         <v>898</v>
       </c>
       <c r="C418" s="0" t="s">
-        <v>137</v>
+        <v>41</v>
       </c>
       <c r="D418" s="0">
-        <v>1080</v>
+        <v>27991.54</v>
       </c>
     </row>
     <row r="419">
@@ -9154,7 +9160,7 @@
         <v>137</v>
       </c>
       <c r="D419" s="0">
-        <v>4012</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="420">
@@ -9165,10 +9171,10 @@
         <v>902</v>
       </c>
       <c r="C420" s="0" t="s">
-        <v>46</v>
+        <v>137</v>
       </c>
       <c r="D420" s="0">
-        <v>6345.07</v>
+        <v>4012</v>
       </c>
     </row>
     <row r="421">
@@ -9182,7 +9188,7 @@
         <v>46</v>
       </c>
       <c r="D421" s="0">
-        <v>2862.56</v>
+        <v>6344.43</v>
       </c>
     </row>
     <row r="422">
@@ -9196,35 +9202,35 @@
         <v>46</v>
       </c>
       <c r="D422" s="0">
-        <v>2131.4</v>
+        <v>2862.28</v>
       </c>
     </row>
     <row r="423">
-      <c r="A423" s="2" t="s">
+      <c r="A423" s="0" t="s">
         <v>907</v>
       </c>
-      <c r="B423" s="2" t="s">
+      <c r="B423" s="0" t="s">
         <v>908</v>
       </c>
-      <c r="C423" s="2" t="s">
+      <c r="C423" s="0" t="s">
         <v>46</v>
       </c>
-      <c r="D423" s="2">
-        <v>3925.75</v>
+      <c r="D423" s="0">
+        <v>2131.18</v>
       </c>
     </row>
     <row r="424">
-      <c r="A424" s="0" t="s">
+      <c r="A424" s="2" t="s">
         <v>909</v>
       </c>
-      <c r="B424" s="0" t="s">
+      <c r="B424" s="2" t="s">
         <v>910</v>
       </c>
-      <c r="C424" s="0" t="s">
+      <c r="C424" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D424" s="0">
-        <v>29798.66</v>
+      <c r="D424" s="2">
+        <v>3925.36</v>
       </c>
     </row>
     <row r="425">
@@ -9238,7 +9244,7 @@
         <v>46</v>
       </c>
       <c r="D425" s="0">
-        <v>2307.32</v>
+        <v>29795.68</v>
       </c>
     </row>
     <row r="426">
@@ -9252,7 +9258,7 @@
         <v>46</v>
       </c>
       <c r="D426" s="0">
-        <v>5250</v>
+        <v>2307.09</v>
       </c>
     </row>
     <row r="427">
@@ -9266,7 +9272,7 @@
         <v>46</v>
       </c>
       <c r="D427" s="0">
-        <v>4400</v>
+        <v>5249.48</v>
       </c>
     </row>
     <row r="428">
@@ -9277,10 +9283,10 @@
         <v>918</v>
       </c>
       <c r="C428" s="0" t="s">
-        <v>486</v>
+        <v>46</v>
       </c>
       <c r="D428" s="0">
-        <v>510</v>
+        <v>4399.56</v>
       </c>
     </row>
     <row r="429">
@@ -9291,7 +9297,7 @@
         <v>920</v>
       </c>
       <c r="C429" s="0" t="s">
-        <v>38</v>
+        <v>488</v>
       </c>
       <c r="D429" s="0">
         <v>510</v>
@@ -9305,21 +9311,21 @@
         <v>922</v>
       </c>
       <c r="C430" s="0" t="s">
-        <v>923</v>
+        <v>38</v>
       </c>
       <c r="D430" s="0">
-        <v>580</v>
+        <v>510</v>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="0" t="s">
+        <v>923</v>
+      </c>
+      <c r="B431" s="0" t="s">
         <v>924</v>
       </c>
-      <c r="B431" s="0" t="s">
+      <c r="C431" s="0" t="s">
         <v>925</v>
-      </c>
-      <c r="C431" s="0" t="s">
-        <v>923</v>
       </c>
       <c r="D431" s="0">
         <v>580</v>
@@ -9333,7 +9339,7 @@
         <v>927</v>
       </c>
       <c r="C432" s="0" t="s">
-        <v>923</v>
+        <v>925</v>
       </c>
       <c r="D432" s="0">
         <v>580</v>
@@ -9347,10 +9353,10 @@
         <v>929</v>
       </c>
       <c r="C433" s="0" t="s">
-        <v>923</v>
+        <v>925</v>
       </c>
       <c r="D433" s="0">
-        <v>342</v>
+        <v>580</v>
       </c>
     </row>
     <row r="434">
@@ -9361,7 +9367,7 @@
         <v>931</v>
       </c>
       <c r="C434" s="0" t="s">
-        <v>923</v>
+        <v>925</v>
       </c>
       <c r="D434" s="0">
         <v>342</v>
@@ -9375,7 +9381,7 @@
         <v>933</v>
       </c>
       <c r="C435" s="0" t="s">
-        <v>923</v>
+        <v>925</v>
       </c>
       <c r="D435" s="0">
         <v>342</v>
@@ -9389,10 +9395,10 @@
         <v>935</v>
       </c>
       <c r="C436" s="0" t="s">
-        <v>923</v>
+        <v>925</v>
       </c>
       <c r="D436" s="0">
-        <v>0</v>
+        <v>342</v>
       </c>
     </row>
     <row r="437">
@@ -9403,7 +9409,7 @@
         <v>937</v>
       </c>
       <c r="C437" s="0" t="s">
-        <v>923</v>
+        <v>925</v>
       </c>
       <c r="D437" s="0">
         <v>0</v>
@@ -9417,21 +9423,21 @@
         <v>939</v>
       </c>
       <c r="C438" s="0" t="s">
-        <v>940</v>
+        <v>925</v>
       </c>
       <c r="D438" s="0">
-        <v>453</v>
+        <v>0</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="0" t="s">
+        <v>940</v>
+      </c>
+      <c r="B439" s="0" t="s">
         <v>941</v>
       </c>
-      <c r="B439" s="0" t="s">
+      <c r="C439" s="0" t="s">
         <v>942</v>
-      </c>
-      <c r="C439" s="0" t="s">
-        <v>923</v>
       </c>
       <c r="D439" s="0">
         <v>453</v>
@@ -9445,10 +9451,10 @@
         <v>944</v>
       </c>
       <c r="C440" s="0" t="s">
-        <v>71</v>
+        <v>925</v>
       </c>
       <c r="D440" s="0">
-        <v>15968</v>
+        <v>453</v>
       </c>
     </row>
     <row r="441">
@@ -9459,10 +9465,10 @@
         <v>946</v>
       </c>
       <c r="C441" s="0" t="s">
-        <v>35</v>
+        <v>71</v>
       </c>
       <c r="D441" s="0">
-        <v>430</v>
+        <v>15968</v>
       </c>
     </row>
     <row r="442">
@@ -9473,7 +9479,7 @@
         <v>948</v>
       </c>
       <c r="C442" s="0" t="s">
-        <v>285</v>
+        <v>35</v>
       </c>
       <c r="D442" s="0">
         <v>430</v>
@@ -9487,10 +9493,10 @@
         <v>950</v>
       </c>
       <c r="C443" s="0" t="s">
-        <v>114</v>
+        <v>285</v>
       </c>
       <c r="D443" s="0">
-        <v>14000</v>
+        <v>430</v>
       </c>
     </row>
     <row r="444">
@@ -9501,10 +9507,10 @@
         <v>952</v>
       </c>
       <c r="C444" s="0" t="s">
-        <v>137</v>
+        <v>114</v>
       </c>
       <c r="D444" s="0">
-        <v>14001</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="445">
@@ -9515,10 +9521,10 @@
         <v>954</v>
       </c>
       <c r="C445" s="0" t="s">
-        <v>91</v>
+        <v>137</v>
       </c>
       <c r="D445" s="0">
-        <v>266200</v>
+        <v>14001</v>
       </c>
     </row>
     <row r="446">
@@ -9532,7 +9538,7 @@
         <v>91</v>
       </c>
       <c r="D446" s="0">
-        <v>194991.5</v>
+        <v>266200</v>
       </c>
     </row>
     <row r="447">
@@ -9546,7 +9552,7 @@
         <v>91</v>
       </c>
       <c r="D447" s="0">
-        <v>289492.5</v>
+        <v>194991.5</v>
       </c>
     </row>
     <row r="448">
@@ -9557,24 +9563,24 @@
         <v>960</v>
       </c>
       <c r="C448" s="0" t="s">
-        <v>961</v>
+        <v>91</v>
       </c>
       <c r="D448" s="0">
-        <v>13722.52</v>
+        <v>289492.5</v>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="0" t="s">
+        <v>961</v>
+      </c>
+      <c r="B449" s="0" t="s">
         <v>962</v>
       </c>
-      <c r="B449" s="0" t="s">
+      <c r="C449" s="0" t="s">
         <v>963</v>
       </c>
-      <c r="C449" s="0" t="s">
-        <v>961</v>
-      </c>
       <c r="D449" s="0">
-        <v>15072</v>
+        <v>13722.52</v>
       </c>
     </row>
     <row r="450">
@@ -9585,10 +9591,10 @@
         <v>965</v>
       </c>
       <c r="C450" s="0" t="s">
-        <v>961</v>
+        <v>963</v>
       </c>
       <c r="D450" s="0">
-        <v>6555.64</v>
+        <v>15072</v>
       </c>
     </row>
     <row r="451">
@@ -9599,10 +9605,10 @@
         <v>967</v>
       </c>
       <c r="C451" s="0" t="s">
-        <v>961</v>
+        <v>963</v>
       </c>
       <c r="D451" s="0">
-        <v>8964.61</v>
+        <v>6555.64</v>
       </c>
     </row>
     <row r="452">
@@ -9613,10 +9619,10 @@
         <v>969</v>
       </c>
       <c r="C452" s="0" t="s">
-        <v>961</v>
+        <v>963</v>
       </c>
       <c r="D452" s="0">
-        <v>11735</v>
+        <v>8964.61</v>
       </c>
     </row>
     <row r="453">
@@ -9627,10 +9633,10 @@
         <v>971</v>
       </c>
       <c r="C453" s="0" t="s">
-        <v>71</v>
+        <v>963</v>
       </c>
       <c r="D453" s="0">
-        <v>3380</v>
+        <v>11735</v>
       </c>
     </row>
     <row r="454">
@@ -9641,10 +9647,10 @@
         <v>973</v>
       </c>
       <c r="C454" s="0" t="s">
-        <v>137</v>
+        <v>71</v>
       </c>
       <c r="D454" s="0">
-        <v>3750</v>
+        <v>3380</v>
       </c>
     </row>
     <row r="455">
@@ -9655,10 +9661,10 @@
         <v>975</v>
       </c>
       <c r="C455" s="0" t="s">
-        <v>91</v>
+        <v>137</v>
       </c>
       <c r="D455" s="0">
-        <v>4392.3</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="456">
@@ -9669,24 +9675,24 @@
         <v>977</v>
       </c>
       <c r="C456" s="0" t="s">
-        <v>978</v>
+        <v>91</v>
       </c>
       <c r="D456" s="0">
-        <v>5254.41</v>
+        <v>4392.3</v>
       </c>
     </row>
     <row r="457">
       <c r="A457" s="0" t="s">
+        <v>978</v>
+      </c>
+      <c r="B457" s="0" t="s">
         <v>979</v>
       </c>
-      <c r="B457" s="0" t="s">
+      <c r="C457" s="0" t="s">
         <v>980</v>
       </c>
-      <c r="C457" s="0" t="s">
-        <v>53</v>
-      </c>
       <c r="D457" s="0">
-        <v>1200</v>
+        <v>5254.41</v>
       </c>
     </row>
     <row r="458">
@@ -9700,7 +9706,7 @@
         <v>53</v>
       </c>
       <c r="D458" s="0">
-        <v>278</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="459">
@@ -9714,7 +9720,7 @@
         <v>53</v>
       </c>
       <c r="D459" s="0">
-        <v>562</v>
+        <v>278</v>
       </c>
     </row>
     <row r="460">
@@ -9725,10 +9731,10 @@
         <v>986</v>
       </c>
       <c r="C460" s="0" t="s">
-        <v>376</v>
+        <v>53</v>
       </c>
       <c r="D460" s="0">
-        <v>65142.6</v>
+        <v>562</v>
       </c>
     </row>
     <row r="461">
@@ -9739,10 +9745,10 @@
         <v>988</v>
       </c>
       <c r="C461" s="0" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="D461" s="0">
-        <v>23482.7</v>
+        <v>65142.6</v>
       </c>
     </row>
     <row r="462">
@@ -9753,10 +9759,10 @@
         <v>990</v>
       </c>
       <c r="C462" s="0" t="s">
-        <v>29</v>
+        <v>378</v>
       </c>
       <c r="D462" s="0">
-        <v>6029.59</v>
+        <v>23482.7</v>
       </c>
     </row>
     <row r="463">
@@ -9767,10 +9773,10 @@
         <v>992</v>
       </c>
       <c r="C463" s="0" t="s">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="D463" s="0">
-        <v>10985</v>
+        <v>6029.59</v>
       </c>
     </row>
     <row r="464">
@@ -9784,7 +9790,7 @@
         <v>53</v>
       </c>
       <c r="D464" s="0">
-        <v>17425</v>
+        <v>10985</v>
       </c>
     </row>
     <row r="465">
@@ -9795,38 +9801,38 @@
         <v>996</v>
       </c>
       <c r="C465" s="0" t="s">
-        <v>997</v>
+        <v>53</v>
       </c>
       <c r="D465" s="0">
-        <v>1958</v>
+        <v>17425</v>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="0" t="s">
+        <v>997</v>
+      </c>
+      <c r="B466" s="0" t="s">
         <v>998</v>
       </c>
-      <c r="B466" s="0" t="s">
+      <c r="C466" s="0" t="s">
         <v>999</v>
       </c>
-      <c r="C466" s="0" t="s">
-        <v>1000</v>
-      </c>
       <c r="D466" s="0">
-        <v>385.4</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="0" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B467" s="0" t="s">
         <v>1001</v>
       </c>
-      <c r="B467" s="0" t="s">
+      <c r="C467" s="0" t="s">
         <v>1002</v>
       </c>
-      <c r="C467" s="0" t="s">
-        <v>91</v>
-      </c>
       <c r="D467" s="0">
-        <v>296147.5</v>
+        <v>385.4</v>
       </c>
     </row>
     <row r="468">
@@ -9837,10 +9843,10 @@
         <v>1004</v>
       </c>
       <c r="C468" s="0" t="s">
-        <v>582</v>
+        <v>91</v>
       </c>
       <c r="D468" s="0">
-        <v>71176.4</v>
+        <v>296147.5</v>
       </c>
     </row>
     <row r="469">
@@ -9851,10 +9857,10 @@
         <v>1006</v>
       </c>
       <c r="C469" s="0" t="s">
-        <v>137</v>
+        <v>584</v>
       </c>
       <c r="D469" s="0">
-        <v>96</v>
+        <v>71176.4</v>
       </c>
     </row>
     <row r="470">
@@ -9865,10 +9871,10 @@
         <v>1008</v>
       </c>
       <c r="C470" s="0" t="s">
-        <v>71</v>
+        <v>137</v>
       </c>
       <c r="D470" s="0">
-        <v>950</v>
+        <v>96</v>
       </c>
     </row>
     <row r="471">
@@ -9879,10 +9885,10 @@
         <v>1010</v>
       </c>
       <c r="C471" s="0" t="s">
-        <v>477</v>
+        <v>71</v>
       </c>
       <c r="D471" s="0">
-        <v>342641</v>
+        <v>950</v>
       </c>
     </row>
     <row r="472">
@@ -9893,10 +9899,10 @@
         <v>1012</v>
       </c>
       <c r="C472" s="0" t="s">
-        <v>157</v>
+        <v>479</v>
       </c>
       <c r="D472" s="0">
-        <v>2200</v>
+        <v>342641</v>
       </c>
     </row>
     <row r="473">
@@ -9907,10 +9913,10 @@
         <v>1014</v>
       </c>
       <c r="C473" s="0" t="s">
-        <v>486</v>
+        <v>157</v>
       </c>
       <c r="D473" s="0">
-        <v>41000</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="474">
@@ -9921,10 +9927,10 @@
         <v>1016</v>
       </c>
       <c r="C474" s="0" t="s">
-        <v>71</v>
+        <v>488</v>
       </c>
       <c r="D474" s="0">
-        <v>9299</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="475">
@@ -9935,10 +9941,10 @@
         <v>1018</v>
       </c>
       <c r="C475" s="0" t="s">
-        <v>923</v>
+        <v>71</v>
       </c>
       <c r="D475" s="0">
-        <v>825</v>
+        <v>9299</v>
       </c>
     </row>
     <row r="476">
@@ -9949,7 +9955,7 @@
         <v>1020</v>
       </c>
       <c r="C476" s="0" t="s">
-        <v>923</v>
+        <v>925</v>
       </c>
       <c r="D476" s="0">
         <v>825</v>
@@ -9963,7 +9969,7 @@
         <v>1022</v>
       </c>
       <c r="C477" s="0" t="s">
-        <v>923</v>
+        <v>925</v>
       </c>
       <c r="D477" s="0">
         <v>825</v>
@@ -9977,10 +9983,10 @@
         <v>1024</v>
       </c>
       <c r="C478" s="0" t="s">
-        <v>22</v>
+        <v>925</v>
       </c>
       <c r="D478" s="0">
-        <v>563.36</v>
+        <v>825</v>
       </c>
     </row>
     <row r="479">
@@ -9991,10 +9997,10 @@
         <v>1026</v>
       </c>
       <c r="C479" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D479" s="0">
-        <v>3520</v>
+        <v>563.36</v>
       </c>
     </row>
     <row r="480">
@@ -10008,7 +10014,7 @@
         <v>16</v>
       </c>
       <c r="D480" s="0">
-        <v>2600</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="481">
@@ -10019,10 +10025,10 @@
         <v>1030</v>
       </c>
       <c r="C481" s="0" t="s">
-        <v>285</v>
+        <v>16</v>
       </c>
       <c r="D481" s="0">
-        <v>3700</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="482">
@@ -10036,7 +10042,7 @@
         <v>285</v>
       </c>
       <c r="D482" s="0">
-        <v>2600</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="483">
@@ -10047,10 +10053,10 @@
         <v>1034</v>
       </c>
       <c r="C483" s="0" t="s">
-        <v>16</v>
+        <v>285</v>
       </c>
       <c r="D483" s="0">
-        <v>2235</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="484">
@@ -10064,35 +10070,35 @@
         <v>16</v>
       </c>
       <c r="D484" s="0">
-        <v>3850</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="0" t="s">
-        <v>397</v>
+        <v>1037</v>
       </c>
       <c r="B485" s="0" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
       <c r="C485" s="0" t="s">
-        <v>1038</v>
+        <v>16</v>
       </c>
       <c r="D485" s="0">
-        <v>1</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="0" t="s">
+        <v>399</v>
+      </c>
+      <c r="B486" s="0" t="s">
         <v>1039</v>
       </c>
-      <c r="B486" s="0" t="s">
+      <c r="C486" s="0" t="s">
         <v>1040</v>
       </c>
-      <c r="C486" s="0" t="s">
-        <v>29</v>
-      </c>
       <c r="D486" s="0">
-        <v>14819</v>
+        <v>1</v>
       </c>
     </row>
     <row r="487">
@@ -10103,10 +10109,10 @@
         <v>1042</v>
       </c>
       <c r="C487" s="0" t="s">
-        <v>376</v>
+        <v>29</v>
       </c>
       <c r="D487" s="0">
-        <v>3859.93</v>
+        <v>14819</v>
       </c>
     </row>
     <row r="488">
@@ -10117,10 +10123,10 @@
         <v>1044</v>
       </c>
       <c r="C488" s="0" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="D488" s="0">
-        <v>11751.49</v>
+        <v>3859.93</v>
       </c>
     </row>
     <row r="489">
@@ -10131,10 +10137,10 @@
         <v>1046</v>
       </c>
       <c r="C489" s="0" t="s">
-        <v>340</v>
+        <v>378</v>
       </c>
       <c r="D489" s="0">
-        <v>6000</v>
+        <v>11751.49</v>
       </c>
     </row>
     <row r="490">
@@ -10148,7 +10154,7 @@
         <v>340</v>
       </c>
       <c r="D490" s="0">
-        <v>3000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="491">
@@ -10159,10 +10165,10 @@
         <v>1050</v>
       </c>
       <c r="C491" s="0" t="s">
-        <v>38</v>
+        <v>340</v>
       </c>
       <c r="D491" s="0">
-        <v>618</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="492">
@@ -10173,24 +10179,24 @@
         <v>1052</v>
       </c>
       <c r="C492" s="0" t="s">
-        <v>1053</v>
+        <v>38</v>
       </c>
       <c r="D492" s="0">
-        <v>24600</v>
+        <v>618</v>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="0" t="s">
+        <v>1053</v>
+      </c>
+      <c r="B493" s="0" t="s">
         <v>1054</v>
       </c>
-      <c r="B493" s="0" t="s">
+      <c r="C493" s="0" t="s">
         <v>1055</v>
       </c>
-      <c r="C493" s="0" t="s">
-        <v>104</v>
-      </c>
       <c r="D493" s="0">
-        <v>0</v>
+        <v>24600</v>
       </c>
     </row>
     <row r="494">
@@ -10201,10 +10207,10 @@
         <v>1057</v>
       </c>
       <c r="C494" s="0" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="D494" s="0">
-        <v>40928.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="495">
@@ -10215,10 +10221,10 @@
         <v>1059</v>
       </c>
       <c r="C495" s="0" t="s">
-        <v>376</v>
+        <v>91</v>
       </c>
       <c r="D495" s="0">
-        <v>75529.71</v>
+        <v>40928.25</v>
       </c>
     </row>
     <row r="496">
@@ -10229,10 +10235,10 @@
         <v>1061</v>
       </c>
       <c r="C496" s="0" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="D496" s="0">
-        <v>41613.42</v>
+        <v>75529.71</v>
       </c>
     </row>
     <row r="497">
@@ -10243,10 +10249,10 @@
         <v>1063</v>
       </c>
       <c r="C497" s="0" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="D497" s="0">
-        <v>87056.42</v>
+        <v>41613.42</v>
       </c>
     </row>
     <row r="498">
@@ -10257,10 +10263,10 @@
         <v>1065</v>
       </c>
       <c r="C498" s="0" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="D498" s="0">
-        <v>49243.16</v>
+        <v>87056.42</v>
       </c>
     </row>
     <row r="499">
@@ -10271,10 +10277,10 @@
         <v>1067</v>
       </c>
       <c r="C499" s="0" t="s">
-        <v>22</v>
+        <v>378</v>
       </c>
       <c r="D499" s="0">
-        <v>1600</v>
+        <v>49243.16</v>
       </c>
     </row>
     <row r="500">
@@ -10285,10 +10291,10 @@
         <v>1069</v>
       </c>
       <c r="C500" s="0" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D500" s="0">
-        <v>3455.8</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="501">
@@ -10302,7 +10308,7 @@
         <v>29</v>
       </c>
       <c r="D501" s="0">
-        <v>3987</v>
+        <v>3455.8</v>
       </c>
     </row>
     <row r="502">
@@ -10316,7 +10322,7 @@
         <v>29</v>
       </c>
       <c r="D502" s="0">
-        <v>4010.17</v>
+        <v>3987</v>
       </c>
     </row>
     <row r="503">
@@ -10330,35 +10336,35 @@
         <v>29</v>
       </c>
       <c r="D503" s="0">
+        <v>4010.17</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="0" t="s">
+        <v>1076</v>
+      </c>
+      <c r="B504" s="0" t="s">
+        <v>1077</v>
+      </c>
+      <c r="C504" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D504" s="0">
         <v>3382.65</v>
       </c>
     </row>
-    <row r="504">
-      <c r="A504" s="2" t="s">
-        <v>1076</v>
-      </c>
-      <c r="B504" s="2" t="s">
-        <v>1077</v>
-      </c>
-      <c r="C504" s="2" t="s">
+    <row r="505">
+      <c r="A505" s="2" t="s">
+        <v>1078</v>
+      </c>
+      <c r="B505" s="2" t="s">
+        <v>1079</v>
+      </c>
+      <c r="C505" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D504" s="2">
+      <c r="D505" s="2">
         <v>0</v>
-      </c>
-    </row>
-    <row r="505">
-      <c r="A505" s="0" t="s">
-        <v>1078</v>
-      </c>
-      <c r="B505" s="0" t="s">
-        <v>1079</v>
-      </c>
-      <c r="C505" s="0" t="s">
-        <v>157</v>
-      </c>
-      <c r="D505" s="0">
-        <v>430</v>
       </c>
     </row>
     <row r="506">
@@ -10369,9 +10375,23 @@
         <v>1081</v>
       </c>
       <c r="C506" s="0" t="s">
+        <v>157</v>
+      </c>
+      <c r="D506" s="0">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="0" t="s">
+        <v>1082</v>
+      </c>
+      <c r="B507" s="0" t="s">
+        <v>1083</v>
+      </c>
+      <c r="C507" s="0" t="s">
         <v>137</v>
       </c>
-      <c r="D506" s="0">
+      <c r="D507" s="0">
         <v>462</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: stock y precios actualizados mié. 29/07/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="1084">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="1087">
   <si>
     <t>Código</t>
   </si>
@@ -248,21 +248,21 @@
     <t>ALMAXIMO 100MG COMP. X 20 - 000024128</t>
   </si>
   <si>
+    <t>000024363</t>
+  </si>
+  <si>
+    <t>ALMAXIMO 36 20 MG COMP. X 8 - 000024363</t>
+  </si>
+  <si>
+    <t>000024023</t>
+  </si>
+  <si>
+    <t>ALMAXIMO 36 5MG COMP. X 30 COMPR - 000024023</t>
+  </si>
+  <si>
     <t>FABOP</t>
   </si>
   <si>
-    <t>000024363</t>
-  </si>
-  <si>
-    <t>ALMAXIMO 36 20 MG COMP. X 8 - 000024363</t>
-  </si>
-  <si>
-    <t>000024023</t>
-  </si>
-  <si>
-    <t>ALMAXIMO 36 5MG COMP. X 30 COMPR - 000024023</t>
-  </si>
-  <si>
     <t>000024129</t>
   </si>
   <si>
@@ -3012,6 +3012,15 @@
   </si>
   <si>
     <t>ETEMP</t>
+  </si>
+  <si>
+    <t>000024705</t>
+  </si>
+  <si>
+    <t>TERMOMETRO DIGITAL PUNTA FLEXIBLE - 000024705</t>
+  </si>
+  <si>
+    <t>MICROLIFE</t>
   </si>
   <si>
     <t>000024688</t>
@@ -3322,7 +3331,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A3:D507"/>
+  <dimension ref="A3:D508"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="3">
@@ -3739,7 +3748,7 @@
         <v>77</v>
       </c>
       <c r="C32" s="0" t="s">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="D32" s="0">
         <v>9395.8</v>
@@ -3747,10 +3756,10 @@
     </row>
     <row r="33">
       <c r="A33" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="B33" s="0" t="s">
         <v>79</v>
-      </c>
-      <c r="B33" s="0" t="s">
-        <v>80</v>
       </c>
       <c r="C33" s="0" t="s">
         <v>19</v>
@@ -3761,13 +3770,13 @@
     </row>
     <row r="34">
       <c r="A34" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="B34" s="0" t="s">
         <v>81</v>
       </c>
-      <c r="B34" s="0" t="s">
+      <c r="C34" s="0" t="s">
         <v>82</v>
-      </c>
-      <c r="C34" s="0" t="s">
-        <v>78</v>
       </c>
       <c r="D34" s="0">
         <v>10520</v>
@@ -3781,7 +3790,7 @@
         <v>84</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="D35" s="0">
         <v>7173.6</v>
@@ -3795,7 +3804,7 @@
         <v>86</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="D36" s="0">
         <v>10440</v>
@@ -3809,7 +3818,7 @@
         <v>88</v>
       </c>
       <c r="C37" s="0" t="s">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="D37" s="0">
         <v>7173.6</v>
@@ -4075,7 +4084,7 @@
         <v>134</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D56" s="2">
         <v>0</v>
@@ -5853,7 +5862,7 @@
         <v>410</v>
       </c>
       <c r="C183" s="0" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D183" s="0">
         <v>783.93</v>
@@ -5867,7 +5876,7 @@
         <v>412</v>
       </c>
       <c r="C184" s="0" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D184" s="0">
         <v>2850</v>
@@ -5909,7 +5918,7 @@
         <v>418</v>
       </c>
       <c r="C187" s="0" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D187" s="0">
         <v>10007.57</v>
@@ -5940,7 +5949,7 @@
         <v>19</v>
       </c>
       <c r="D189" s="0">
-        <v>405</v>
+        <v>412.8</v>
       </c>
     </row>
     <row r="190">
@@ -6042,16 +6051,16 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="0" t="s">
+      <c r="A197" s="2" t="s">
         <v>437</v>
       </c>
-      <c r="B197" s="0" t="s">
+      <c r="B197" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="C197" s="0" t="s">
+      <c r="C197" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D197" s="0">
+      <c r="D197" s="2">
         <v>691</v>
       </c>
     </row>
@@ -6070,16 +6079,16 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="0" t="s">
+      <c r="A199" s="2" t="s">
         <v>441</v>
       </c>
-      <c r="B199" s="0" t="s">
+      <c r="B199" s="2" t="s">
         <v>442</v>
       </c>
-      <c r="C199" s="0" t="s">
+      <c r="C199" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D199" s="0">
+      <c r="D199" s="2">
         <v>300</v>
       </c>
     </row>
@@ -7340,7 +7349,7 @@
         <v>16</v>
       </c>
       <c r="D289" s="0">
-        <v>1100</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="290">
@@ -9832,7 +9841,7 @@
         <v>1002</v>
       </c>
       <c r="D467" s="0">
-        <v>385.4</v>
+        <v>2282.3</v>
       </c>
     </row>
     <row r="468">
@@ -9843,360 +9852,360 @@
         <v>1004</v>
       </c>
       <c r="C468" s="0" t="s">
-        <v>91</v>
+        <v>1005</v>
       </c>
       <c r="D468" s="0">
-        <v>296147.5</v>
+        <v>385.4</v>
       </c>
     </row>
     <row r="469">
       <c r="A469" s="0" t="s">
-        <v>1005</v>
+        <v>1006</v>
       </c>
       <c r="B469" s="0" t="s">
-        <v>1006</v>
+        <v>1007</v>
       </c>
       <c r="C469" s="0" t="s">
-        <v>584</v>
+        <v>91</v>
       </c>
       <c r="D469" s="0">
-        <v>71176.4</v>
+        <v>296147.5</v>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="0" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="B470" s="0" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="C470" s="0" t="s">
-        <v>137</v>
+        <v>584</v>
       </c>
       <c r="D470" s="0">
-        <v>96</v>
+        <v>71176.4</v>
       </c>
     </row>
     <row r="471">
       <c r="A471" s="0" t="s">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="B471" s="0" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="C471" s="0" t="s">
-        <v>71</v>
+        <v>137</v>
       </c>
       <c r="D471" s="0">
-        <v>950</v>
+        <v>96</v>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="0" t="s">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="B472" s="0" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="C472" s="0" t="s">
-        <v>479</v>
+        <v>71</v>
       </c>
       <c r="D472" s="0">
-        <v>342641</v>
+        <v>950</v>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="0" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="B473" s="0" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="C473" s="0" t="s">
-        <v>157</v>
+        <v>479</v>
       </c>
       <c r="D473" s="0">
-        <v>2200</v>
+        <v>342641</v>
       </c>
     </row>
     <row r="474">
       <c r="A474" s="0" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="B474" s="0" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="C474" s="0" t="s">
-        <v>488</v>
+        <v>157</v>
       </c>
       <c r="D474" s="0">
-        <v>41000</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="475">
       <c r="A475" s="0" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="B475" s="0" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="C475" s="0" t="s">
-        <v>71</v>
+        <v>488</v>
       </c>
       <c r="D475" s="0">
-        <v>9299</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="476">
       <c r="A476" s="0" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="B476" s="0" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
       <c r="C476" s="0" t="s">
-        <v>925</v>
+        <v>71</v>
       </c>
       <c r="D476" s="0">
-        <v>825</v>
+        <v>9299</v>
       </c>
     </row>
     <row r="477">
       <c r="A477" s="0" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
       <c r="B477" s="0" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="C477" s="0" t="s">
         <v>925</v>
       </c>
       <c r="D477" s="0">
-        <v>825</v>
+        <v>880</v>
       </c>
     </row>
     <row r="478">
       <c r="A478" s="0" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
       <c r="B478" s="0" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="C478" s="0" t="s">
         <v>925</v>
       </c>
       <c r="D478" s="0">
-        <v>825</v>
+        <v>880</v>
       </c>
     </row>
     <row r="479">
       <c r="A479" s="0" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
       <c r="B479" s="0" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="C479" s="0" t="s">
-        <v>22</v>
+        <v>925</v>
       </c>
       <c r="D479" s="0">
-        <v>563.36</v>
+        <v>880</v>
       </c>
     </row>
     <row r="480">
       <c r="A480" s="0" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="B480" s="0" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="C480" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D480" s="0">
-        <v>3520</v>
+        <v>563.36</v>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="0" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="B481" s="0" t="s">
-        <v>1030</v>
+        <v>1031</v>
       </c>
       <c r="C481" s="0" t="s">
         <v>16</v>
       </c>
       <c r="D481" s="0">
-        <v>2600</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="0" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="B482" s="0" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="C482" s="0" t="s">
-        <v>285</v>
+        <v>16</v>
       </c>
       <c r="D482" s="0">
-        <v>3700</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="0" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="B483" s="0" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="C483" s="0" t="s">
         <v>285</v>
       </c>
       <c r="D483" s="0">
-        <v>2600</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="0" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="B484" s="0" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="C484" s="0" t="s">
-        <v>16</v>
+        <v>285</v>
       </c>
       <c r="D484" s="0">
-        <v>2235</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="0" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
       <c r="B485" s="0" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="C485" s="0" t="s">
         <v>16</v>
       </c>
       <c r="D485" s="0">
-        <v>3850</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="0" t="s">
-        <v>399</v>
+        <v>1040</v>
       </c>
       <c r="B486" s="0" t="s">
-        <v>1039</v>
+        <v>1041</v>
       </c>
       <c r="C486" s="0" t="s">
-        <v>1040</v>
+        <v>16</v>
       </c>
       <c r="D486" s="0">
-        <v>1</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="0" t="s">
-        <v>1041</v>
+        <v>399</v>
       </c>
       <c r="B487" s="0" t="s">
         <v>1042</v>
       </c>
       <c r="C487" s="0" t="s">
-        <v>29</v>
+        <v>1043</v>
       </c>
       <c r="D487" s="0">
-        <v>14819</v>
+        <v>1</v>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="0" t="s">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="B488" s="0" t="s">
-        <v>1044</v>
+        <v>1045</v>
       </c>
       <c r="C488" s="0" t="s">
-        <v>378</v>
+        <v>29</v>
       </c>
       <c r="D488" s="0">
-        <v>3859.93</v>
+        <v>14819</v>
       </c>
     </row>
     <row r="489">
       <c r="A489" s="0" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
       <c r="B489" s="0" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="C489" s="0" t="s">
         <v>378</v>
       </c>
       <c r="D489" s="0">
-        <v>11751.49</v>
+        <v>3859.93</v>
       </c>
     </row>
     <row r="490">
       <c r="A490" s="0" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="B490" s="0" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="C490" s="0" t="s">
-        <v>340</v>
+        <v>378</v>
       </c>
       <c r="D490" s="0">
-        <v>6000</v>
+        <v>11751.49</v>
       </c>
     </row>
     <row r="491">
       <c r="A491" s="0" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="B491" s="0" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="C491" s="0" t="s">
         <v>340</v>
       </c>
       <c r="D491" s="0">
-        <v>3000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="492">
       <c r="A492" s="0" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="B492" s="0" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
       <c r="C492" s="0" t="s">
-        <v>38</v>
+        <v>340</v>
       </c>
       <c r="D492" s="0">
-        <v>618</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="0" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="B493" s="0" t="s">
-        <v>1054</v>
+        <v>1055</v>
       </c>
       <c r="C493" s="0" t="s">
-        <v>1055</v>
+        <v>38</v>
       </c>
       <c r="D493" s="0">
-        <v>24600</v>
+        <v>618</v>
       </c>
     </row>
     <row r="494">
@@ -10207,191 +10216,205 @@
         <v>1057</v>
       </c>
       <c r="C494" s="0" t="s">
-        <v>104</v>
+        <v>1058</v>
       </c>
       <c r="D494" s="0">
-        <v>0</v>
+        <v>24600</v>
       </c>
     </row>
     <row r="495">
       <c r="A495" s="0" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
       <c r="B495" s="0" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="C495" s="0" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="D495" s="0">
-        <v>40928.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="496">
       <c r="A496" s="0" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
       <c r="B496" s="0" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="C496" s="0" t="s">
-        <v>378</v>
+        <v>91</v>
       </c>
       <c r="D496" s="0">
-        <v>75529.71</v>
+        <v>40928.25</v>
       </c>
     </row>
     <row r="497">
       <c r="A497" s="0" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="B497" s="0" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="C497" s="0" t="s">
         <v>378</v>
       </c>
       <c r="D497" s="0">
-        <v>41613.42</v>
+        <v>75529.71</v>
       </c>
     </row>
     <row r="498">
       <c r="A498" s="0" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="B498" s="0" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="C498" s="0" t="s">
         <v>378</v>
       </c>
       <c r="D498" s="0">
-        <v>87056.42</v>
+        <v>41613.42</v>
       </c>
     </row>
     <row r="499">
       <c r="A499" s="0" t="s">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="B499" s="0" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="C499" s="0" t="s">
         <v>378</v>
       </c>
       <c r="D499" s="0">
-        <v>49243.16</v>
+        <v>87056.42</v>
       </c>
     </row>
     <row r="500">
       <c r="A500" s="0" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="B500" s="0" t="s">
-        <v>1069</v>
+        <v>1070</v>
       </c>
       <c r="C500" s="0" t="s">
-        <v>22</v>
+        <v>378</v>
       </c>
       <c r="D500" s="0">
-        <v>1600</v>
+        <v>49243.16</v>
       </c>
     </row>
     <row r="501">
       <c r="A501" s="0" t="s">
-        <v>1070</v>
+        <v>1071</v>
       </c>
       <c r="B501" s="0" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="C501" s="0" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D501" s="0">
-        <v>3455.8</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="502">
       <c r="A502" s="0" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="B502" s="0" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
       <c r="C502" s="0" t="s">
         <v>29</v>
       </c>
       <c r="D502" s="0">
-        <v>3987</v>
+        <v>3455.8</v>
       </c>
     </row>
     <row r="503">
       <c r="A503" s="0" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
       <c r="B503" s="0" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C503" s="0" t="s">
         <v>29</v>
       </c>
       <c r="D503" s="0">
-        <v>4010.17</v>
+        <v>3987</v>
       </c>
     </row>
     <row r="504">
       <c r="A504" s="0" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="B504" s="0" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="C504" s="0" t="s">
         <v>29</v>
       </c>
       <c r="D504" s="0">
+        <v>4010.17</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="0" t="s">
+        <v>1079</v>
+      </c>
+      <c r="B505" s="0" t="s">
+        <v>1080</v>
+      </c>
+      <c r="C505" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D505" s="0">
         <v>3382.65</v>
       </c>
     </row>
-    <row r="505">
-      <c r="A505" s="2" t="s">
-        <v>1078</v>
-      </c>
-      <c r="B505" s="2" t="s">
-        <v>1079</v>
-      </c>
-      <c r="C505" s="2" t="s">
+    <row r="506">
+      <c r="A506" s="2" t="s">
+        <v>1081</v>
+      </c>
+      <c r="B506" s="2" t="s">
+        <v>1082</v>
+      </c>
+      <c r="C506" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D505" s="2">
+      <c r="D506" s="2">
         <v>0</v>
-      </c>
-    </row>
-    <row r="506">
-      <c r="A506" s="0" t="s">
-        <v>1080</v>
-      </c>
-      <c r="B506" s="0" t="s">
-        <v>1081</v>
-      </c>
-      <c r="C506" s="0" t="s">
-        <v>157</v>
-      </c>
-      <c r="D506" s="0">
-        <v>430</v>
       </c>
     </row>
     <row r="507">
       <c r="A507" s="0" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
       <c r="B507" s="0" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
       <c r="C507" s="0" t="s">
+        <v>157</v>
+      </c>
+      <c r="D507" s="0">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="0" t="s">
+        <v>1085</v>
+      </c>
+      <c r="B508" s="0" t="s">
+        <v>1086</v>
+      </c>
+      <c r="C508" s="0" t="s">
         <v>137</v>
       </c>
-      <c r="D507" s="0">
+      <c r="D508" s="0">
         <v>462</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: stock y precios actualizados vie. 31/07/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -1268,7 +1268,7 @@
     <t>000024046</t>
   </si>
   <si>
-    <t xml:space="preserve">FABOGESIC 600 RAPIDA ACCION  CAPS X 50  - 000024046</t>
+    <t xml:space="preserve">FABOGESIC 600 RAPIDA ACCION  CAPS X 50 - 000024046</t>
   </si>
   <si>
     <t>000024648</t>
@@ -3751,7 +3751,7 @@
         <v>19</v>
       </c>
       <c r="D32" s="0">
-        <v>9395.8</v>
+        <v>9122.1</v>
       </c>
     </row>
     <row r="33">
@@ -3765,7 +3765,7 @@
         <v>19</v>
       </c>
       <c r="D33" s="0">
-        <v>10856.33</v>
+        <v>10540.09</v>
       </c>
     </row>
     <row r="34">
@@ -3793,7 +3793,7 @@
         <v>19</v>
       </c>
       <c r="D35" s="0">
-        <v>7173.6</v>
+        <v>6964.6</v>
       </c>
     </row>
     <row r="36">
@@ -3807,7 +3807,7 @@
         <v>19</v>
       </c>
       <c r="D36" s="0">
-        <v>10440</v>
+        <v>10135.7</v>
       </c>
     </row>
     <row r="37">
@@ -3821,7 +3821,7 @@
         <v>19</v>
       </c>
       <c r="D37" s="0">
-        <v>7173.6</v>
+        <v>6964.6</v>
       </c>
     </row>
     <row r="38">
@@ -4717,7 +4717,7 @@
         <v>19</v>
       </c>
       <c r="D101" s="0">
-        <v>1137.36</v>
+        <v>1117.4</v>
       </c>
     </row>
     <row r="102">
@@ -5862,10 +5862,10 @@
         <v>410</v>
       </c>
       <c r="C183" s="0" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="D183" s="0">
-        <v>783.93</v>
+        <v>825.18</v>
       </c>
     </row>
     <row r="184">
@@ -5876,7 +5876,7 @@
         <v>412</v>
       </c>
       <c r="C184" s="0" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="D184" s="0">
         <v>2850</v>
@@ -5893,7 +5893,7 @@
         <v>19</v>
       </c>
       <c r="D185" s="0">
-        <v>6599.67</v>
+        <v>6384.84</v>
       </c>
     </row>
     <row r="186">
@@ -5907,7 +5907,7 @@
         <v>19</v>
       </c>
       <c r="D186" s="0">
-        <v>343.2</v>
+        <v>333.17</v>
       </c>
     </row>
     <row r="187">
@@ -5918,10 +5918,10 @@
         <v>418</v>
       </c>
       <c r="C187" s="0" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="D187" s="0">
-        <v>10007.57</v>
+        <v>9669.15</v>
       </c>
     </row>
     <row r="188">
@@ -5935,7 +5935,7 @@
         <v>19</v>
       </c>
       <c r="D188" s="0">
-        <v>3479.75</v>
+        <v>3599.84</v>
       </c>
     </row>
     <row r="189">
@@ -5963,7 +5963,7 @@
         <v>19</v>
       </c>
       <c r="D190" s="0">
-        <v>2015.51</v>
+        <v>2015.52</v>
       </c>
     </row>
     <row r="191">
@@ -8679,7 +8679,7 @@
         <v>19</v>
       </c>
       <c r="D384" s="0">
-        <v>570</v>
+        <v>569.39</v>
       </c>
     </row>
     <row r="385">

</xml_diff>

<commit_message>
sync: stock y precios actualizados mar. 11/08/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -410,6 +410,12 @@
     <t>APOSITO T/ TEGADERM 6X7CMS EUROMIX - 000024395</t>
   </si>
   <si>
+    <t>000008848</t>
+  </si>
+  <si>
+    <t>ARZOMICIN 200mg /5ml Susp. x 15ml - 000008848</t>
+  </si>
+  <si>
     <t>000009286</t>
   </si>
   <si>
@@ -992,10 +998,10 @@
     <t>DEXAMETASONA DRAWER 8MG INY. AMP. X 1 X 2ML - 000023387</t>
   </si>
   <si>
-    <t>000024493</t>
-  </si>
-  <si>
-    <t>DEXMEDETOMIDINA RICHET 200MCG/2ML X 5 FA - 000024493</t>
+    <t>000023955</t>
+  </si>
+  <si>
+    <t>DEXMEDETOMIDINA RICHET FCO. AMP. X 2 ML - 000023955</t>
   </si>
   <si>
     <t>01720000</t>
@@ -2217,12 +2223,6 @@
   </si>
   <si>
     <t>NAPROXENO VANNIER 500mg Comp. x 10 - 000010079</t>
-  </si>
-  <si>
-    <t>000023401</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NEOSTIGMINA DRAWER 0.5MG AMP. X   1 X 1ML - 000023401</t>
   </si>
   <si>
     <t>000010058</t>
@@ -4016,24 +4016,24 @@
         <v>133</v>
       </c>
       <c r="C56" s="0" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="D56" s="0">
-        <v>473.6</v>
+        <v>3550</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="B57" s="0" t="s">
         <v>135</v>
       </c>
-      <c r="B57" s="0" t="s">
+      <c r="C57" s="0" t="s">
         <v>136</v>
       </c>
-      <c r="C57" s="0" t="s">
-        <v>134</v>
-      </c>
       <c r="D57" s="0">
-        <v>584.3</v>
+        <v>473.6</v>
       </c>
     </row>
     <row r="58">
@@ -4044,10 +4044,10 @@
         <v>138</v>
       </c>
       <c r="C58" s="0" t="s">
-        <v>18</v>
+        <v>136</v>
       </c>
       <c r="D58" s="0">
-        <v>436.1</v>
+        <v>584.3</v>
       </c>
     </row>
     <row r="59">
@@ -4061,7 +4061,7 @@
         <v>18</v>
       </c>
       <c r="D59" s="0">
-        <v>508.5</v>
+        <v>436.1</v>
       </c>
     </row>
     <row r="60">
@@ -4072,10 +4072,10 @@
         <v>142</v>
       </c>
       <c r="C60" s="0" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D60" s="0">
-        <v>484</v>
+        <v>508.5</v>
       </c>
     </row>
     <row r="61">
@@ -4086,24 +4086,24 @@
         <v>144</v>
       </c>
       <c r="C61" s="0" t="s">
-        <v>145</v>
+        <v>15</v>
       </c>
       <c r="D61" s="0">
-        <v>410</v>
+        <v>484</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="0" t="s">
+        <v>145</v>
+      </c>
+      <c r="B62" s="0" t="s">
         <v>146</v>
       </c>
-      <c r="B62" s="0" t="s">
+      <c r="C62" s="0" t="s">
         <v>147</v>
       </c>
-      <c r="C62" s="0" t="s">
-        <v>113</v>
-      </c>
       <c r="D62" s="0">
-        <v>1080</v>
+        <v>410</v>
       </c>
     </row>
     <row r="63">
@@ -4114,7 +4114,7 @@
         <v>149</v>
       </c>
       <c r="C63" s="0" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="D63" s="0">
         <v>1080</v>
@@ -4128,10 +4128,10 @@
         <v>151</v>
       </c>
       <c r="C64" s="0" t="s">
-        <v>15</v>
+        <v>119</v>
       </c>
       <c r="D64" s="0">
-        <v>3200</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="65">
@@ -4142,24 +4142,24 @@
         <v>153</v>
       </c>
       <c r="C65" s="0" t="s">
-        <v>154</v>
+        <v>15</v>
       </c>
       <c r="D65" s="0">
-        <v>3800</v>
+        <v>3200</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="B66" s="0" t="s">
         <v>155</v>
       </c>
-      <c r="B66" s="0" t="s">
+      <c r="C66" s="0" t="s">
         <v>156</v>
       </c>
-      <c r="C66" s="0" t="s">
-        <v>52</v>
-      </c>
       <c r="D66" s="0">
-        <v>9</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="67">
@@ -4187,7 +4187,7 @@
         <v>52</v>
       </c>
       <c r="D68" s="0">
-        <v>1075</v>
+        <v>9</v>
       </c>
     </row>
     <row r="69">
@@ -4198,10 +4198,10 @@
         <v>162</v>
       </c>
       <c r="C69" s="0" t="s">
-        <v>134</v>
+        <v>52</v>
       </c>
       <c r="D69" s="0">
-        <v>537</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="70">
@@ -4212,10 +4212,10 @@
         <v>164</v>
       </c>
       <c r="C70" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D70" s="0">
-        <v>705</v>
+        <v>537</v>
       </c>
     </row>
     <row r="71">
@@ -4226,10 +4226,10 @@
         <v>166</v>
       </c>
       <c r="C71" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D71" s="0">
-        <v>6700</v>
+        <v>705</v>
       </c>
     </row>
     <row r="72">
@@ -4240,24 +4240,24 @@
         <v>168</v>
       </c>
       <c r="C72" s="0" t="s">
-        <v>169</v>
+        <v>136</v>
       </c>
       <c r="D72" s="0">
-        <v>600</v>
+        <v>6700</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="B73" s="0" t="s">
         <v>170</v>
       </c>
-      <c r="B73" s="0" t="s">
+      <c r="C73" s="0" t="s">
         <v>171</v>
       </c>
-      <c r="C73" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="D73" s="0">
-        <v>1782</v>
+        <v>600</v>
       </c>
     </row>
     <row r="74">
@@ -4271,7 +4271,7 @@
         <v>15</v>
       </c>
       <c r="D74" s="0">
-        <v>1400</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="75">
@@ -4285,7 +4285,7 @@
         <v>15</v>
       </c>
       <c r="D75" s="0">
-        <v>680</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="76">
@@ -4299,7 +4299,7 @@
         <v>15</v>
       </c>
       <c r="D76" s="0">
-        <v>780</v>
+        <v>680</v>
       </c>
     </row>
     <row r="77">
@@ -4313,7 +4313,7 @@
         <v>15</v>
       </c>
       <c r="D77" s="0">
-        <v>2580</v>
+        <v>780</v>
       </c>
     </row>
     <row r="78">
@@ -4327,7 +4327,7 @@
         <v>15</v>
       </c>
       <c r="D78" s="0">
-        <v>1100</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="79">
@@ -4338,24 +4338,24 @@
         <v>183</v>
       </c>
       <c r="C79" s="0" t="s">
-        <v>184</v>
+        <v>15</v>
       </c>
       <c r="D79" s="0">
-        <v>2450</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="0" t="s">
+        <v>184</v>
+      </c>
+      <c r="B80" s="0" t="s">
         <v>185</v>
       </c>
-      <c r="B80" s="0" t="s">
+      <c r="C80" s="0" t="s">
         <v>186</v>
       </c>
-      <c r="C80" s="0" t="s">
-        <v>52</v>
-      </c>
       <c r="D80" s="0">
-        <v>330</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="81">
@@ -4366,10 +4366,10 @@
         <v>188</v>
       </c>
       <c r="C81" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="D81" s="0">
-        <v>33.7</v>
+        <v>330</v>
       </c>
     </row>
     <row r="82">
@@ -4380,10 +4380,10 @@
         <v>190</v>
       </c>
       <c r="C82" s="0" t="s">
-        <v>119</v>
+        <v>21</v>
       </c>
       <c r="D82" s="0">
-        <v>1080</v>
+        <v>33.7</v>
       </c>
     </row>
     <row r="83">
@@ -4394,38 +4394,38 @@
         <v>192</v>
       </c>
       <c r="C83" s="0" t="s">
-        <v>193</v>
+        <v>119</v>
       </c>
       <c r="D83" s="0">
-        <v>0</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="0" t="s">
+        <v>193</v>
+      </c>
+      <c r="B84" s="0" t="s">
         <v>194</v>
       </c>
-      <c r="B84" s="0" t="s">
+      <c r="C84" s="0" t="s">
         <v>195</v>
       </c>
-      <c r="C84" s="0" t="s">
-        <v>196</v>
-      </c>
       <c r="D84" s="0">
-        <v>5650</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="0" t="s">
+        <v>196</v>
+      </c>
+      <c r="B85" s="0" t="s">
         <v>197</v>
       </c>
-      <c r="B85" s="0" t="s">
+      <c r="C85" s="0" t="s">
         <v>198</v>
       </c>
-      <c r="C85" s="0" t="s">
-        <v>196</v>
-      </c>
       <c r="D85" s="0">
-        <v>2590</v>
+        <v>5650</v>
       </c>
     </row>
     <row r="86">
@@ -4436,21 +4436,21 @@
         <v>200</v>
       </c>
       <c r="C86" s="0" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D86" s="0">
-        <v>3000</v>
+        <v>2590</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="B87" s="0" t="s">
         <v>202</v>
       </c>
-      <c r="B87" s="0" t="s">
+      <c r="C87" s="0" t="s">
         <v>203</v>
-      </c>
-      <c r="C87" s="0" t="s">
-        <v>201</v>
       </c>
       <c r="D87" s="0">
         <v>3000</v>
@@ -4464,10 +4464,10 @@
         <v>205</v>
       </c>
       <c r="C88" s="0" t="s">
-        <v>108</v>
+        <v>203</v>
       </c>
       <c r="D88" s="0">
-        <v>1770</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="89">
@@ -4478,10 +4478,10 @@
         <v>207</v>
       </c>
       <c r="C89" s="0" t="s">
-        <v>70</v>
+        <v>108</v>
       </c>
       <c r="D89" s="0">
-        <v>900</v>
+        <v>1770</v>
       </c>
     </row>
     <row r="90">
@@ -4492,10 +4492,10 @@
         <v>209</v>
       </c>
       <c r="C90" s="0" t="s">
-        <v>134</v>
+        <v>70</v>
       </c>
       <c r="D90" s="0">
-        <v>636.16</v>
+        <v>900</v>
       </c>
     </row>
     <row r="91">
@@ -4506,10 +4506,10 @@
         <v>211</v>
       </c>
       <c r="C91" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D91" s="0">
-        <v>543.06</v>
+        <v>636.16</v>
       </c>
     </row>
     <row r="92">
@@ -4520,10 +4520,10 @@
         <v>213</v>
       </c>
       <c r="C92" s="0" t="s">
-        <v>52</v>
+        <v>136</v>
       </c>
       <c r="D92" s="0">
-        <v>190</v>
+        <v>543.06</v>
       </c>
     </row>
     <row r="93">
@@ -4537,7 +4537,7 @@
         <v>52</v>
       </c>
       <c r="D93" s="0">
-        <v>180</v>
+        <v>190</v>
       </c>
     </row>
     <row r="94">
@@ -4579,7 +4579,7 @@
         <v>52</v>
       </c>
       <c r="D96" s="0">
-        <v>190</v>
+        <v>180</v>
       </c>
     </row>
     <row r="97">
@@ -4590,10 +4590,10 @@
         <v>223</v>
       </c>
       <c r="C97" s="0" t="s">
-        <v>15</v>
+        <v>52</v>
       </c>
       <c r="D97" s="0">
-        <v>1760</v>
+        <v>190</v>
       </c>
     </row>
     <row r="98">
@@ -4604,10 +4604,10 @@
         <v>225</v>
       </c>
       <c r="C98" s="0" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D98" s="0">
-        <v>1117.4</v>
+        <v>1760</v>
       </c>
     </row>
     <row r="99">
@@ -4618,10 +4618,10 @@
         <v>227</v>
       </c>
       <c r="C99" s="0" t="s">
-        <v>90</v>
+        <v>18</v>
       </c>
       <c r="D99" s="0">
-        <v>3194.4</v>
+        <v>1117.4</v>
       </c>
     </row>
     <row r="100">
@@ -4635,7 +4635,7 @@
         <v>90</v>
       </c>
       <c r="D100" s="0">
-        <v>2435.76</v>
+        <v>3194.4</v>
       </c>
     </row>
     <row r="101">
@@ -4649,7 +4649,7 @@
         <v>90</v>
       </c>
       <c r="D101" s="0">
-        <v>3653.64</v>
+        <v>2435.76</v>
       </c>
     </row>
     <row r="102">
@@ -4660,10 +4660,10 @@
         <v>233</v>
       </c>
       <c r="C102" s="0" t="s">
-        <v>116</v>
+        <v>90</v>
       </c>
       <c r="D102" s="0">
-        <v>1810</v>
+        <v>3653.64</v>
       </c>
     </row>
     <row r="103">
@@ -4674,24 +4674,24 @@
         <v>235</v>
       </c>
       <c r="C103" s="0" t="s">
-        <v>236</v>
+        <v>116</v>
       </c>
       <c r="D103" s="0">
-        <v>1800</v>
+        <v>1810</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="0" t="s">
+        <v>236</v>
+      </c>
+      <c r="B104" s="0" t="s">
         <v>237</v>
       </c>
-      <c r="B104" s="0" t="s">
+      <c r="C104" s="0" t="s">
         <v>238</v>
       </c>
-      <c r="C104" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="D104" s="0">
-        <v>1600</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="105">
@@ -4705,7 +4705,7 @@
         <v>15</v>
       </c>
       <c r="D105" s="0">
-        <v>1800</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="106">
@@ -4716,10 +4716,10 @@
         <v>242</v>
       </c>
       <c r="C106" s="0" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D106" s="0">
-        <v>1600</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="107">
@@ -4730,10 +4730,10 @@
         <v>244</v>
       </c>
       <c r="C107" s="0" t="s">
-        <v>116</v>
+        <v>34</v>
       </c>
       <c r="D107" s="0">
-        <v>1900</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="108">
@@ -4744,10 +4744,10 @@
         <v>246</v>
       </c>
       <c r="C108" s="0" t="s">
-        <v>15</v>
+        <v>116</v>
       </c>
       <c r="D108" s="0">
-        <v>1600</v>
+        <v>1900</v>
       </c>
     </row>
     <row r="109">
@@ -4758,10 +4758,10 @@
         <v>248</v>
       </c>
       <c r="C109" s="0" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="D109" s="0">
-        <v>5771.79</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="110">
@@ -4772,10 +4772,10 @@
         <v>250</v>
       </c>
       <c r="C110" s="0" t="s">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="D110" s="0">
-        <v>975</v>
+        <v>5771.79</v>
       </c>
     </row>
     <row r="111">
@@ -4786,10 +4786,10 @@
         <v>252</v>
       </c>
       <c r="C111" s="0" t="s">
-        <v>134</v>
+        <v>18</v>
       </c>
       <c r="D111" s="0">
-        <v>980</v>
+        <v>975</v>
       </c>
     </row>
     <row r="112">
@@ -4800,24 +4800,24 @@
         <v>254</v>
       </c>
       <c r="C112" s="0" t="s">
-        <v>255</v>
+        <v>136</v>
       </c>
       <c r="D112" s="0">
-        <v>2800</v>
+        <v>980</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="0" t="s">
+        <v>255</v>
+      </c>
+      <c r="B113" s="0" t="s">
         <v>256</v>
       </c>
-      <c r="B113" s="0" t="s">
+      <c r="C113" s="0" t="s">
         <v>257</v>
       </c>
-      <c r="C113" s="0" t="s">
-        <v>255</v>
-      </c>
       <c r="D113" s="0">
-        <v>4525.4</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="114">
@@ -4828,10 +4828,10 @@
         <v>259</v>
       </c>
       <c r="C114" s="0" t="s">
-        <v>21</v>
+        <v>257</v>
       </c>
       <c r="D114" s="0">
-        <v>2954</v>
+        <v>4525.4</v>
       </c>
     </row>
     <row r="115">
@@ -4842,10 +4842,10 @@
         <v>261</v>
       </c>
       <c r="C115" s="0" t="s">
-        <v>90</v>
+        <v>21</v>
       </c>
       <c r="D115" s="0">
-        <v>9982.5</v>
+        <v>2954</v>
       </c>
     </row>
     <row r="116">
@@ -4856,10 +4856,10 @@
         <v>263</v>
       </c>
       <c r="C116" s="0" t="s">
-        <v>34</v>
+        <v>90</v>
       </c>
       <c r="D116" s="0">
-        <v>2400</v>
+        <v>9982.5</v>
       </c>
     </row>
     <row r="117">
@@ -4870,7 +4870,7 @@
         <v>265</v>
       </c>
       <c r="C117" s="0" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D117" s="0">
         <v>2400</v>
@@ -4884,10 +4884,10 @@
         <v>267</v>
       </c>
       <c r="C118" s="0" t="s">
-        <v>90</v>
+        <v>37</v>
       </c>
       <c r="D118" s="0">
-        <v>212.96</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="119">
@@ -4898,21 +4898,21 @@
         <v>269</v>
       </c>
       <c r="C119" s="0" t="s">
-        <v>270</v>
+        <v>90</v>
       </c>
       <c r="D119" s="0">
-        <v>0</v>
+        <v>212.96</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="0" t="s">
+        <v>270</v>
+      </c>
+      <c r="B120" s="0" t="s">
         <v>271</v>
       </c>
-      <c r="B120" s="0" t="s">
+      <c r="C120" s="0" t="s">
         <v>272</v>
-      </c>
-      <c r="C120" s="0" t="s">
-        <v>270</v>
       </c>
       <c r="D120" s="0">
         <v>0</v>
@@ -4926,21 +4926,21 @@
         <v>274</v>
       </c>
       <c r="C121" s="0" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="D121" s="0">
-        <v>520</v>
+        <v>0</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="0" t="s">
+        <v>275</v>
+      </c>
+      <c r="B122" s="0" t="s">
         <v>276</v>
       </c>
-      <c r="B122" s="0" t="s">
+      <c r="C122" s="0" t="s">
         <v>277</v>
-      </c>
-      <c r="C122" s="0" t="s">
-        <v>34</v>
       </c>
       <c r="D122" s="0">
         <v>520</v>
@@ -4954,10 +4954,10 @@
         <v>279</v>
       </c>
       <c r="C123" s="0" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="D123" s="0">
-        <v>22</v>
+        <v>520</v>
       </c>
     </row>
     <row r="124">
@@ -4968,10 +4968,10 @@
         <v>281</v>
       </c>
       <c r="C124" s="0" t="s">
-        <v>15</v>
+        <v>52</v>
       </c>
       <c r="D124" s="0">
-        <v>3200</v>
+        <v>22</v>
       </c>
     </row>
     <row r="125">
@@ -4982,10 +4982,10 @@
         <v>283</v>
       </c>
       <c r="C125" s="0" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="D125" s="0">
-        <v>7118.9</v>
+        <v>3200</v>
       </c>
     </row>
     <row r="126">
@@ -4996,24 +4996,24 @@
         <v>285</v>
       </c>
       <c r="C126" s="0" t="s">
-        <v>286</v>
+        <v>28</v>
       </c>
       <c r="D126" s="0">
-        <v>16095</v>
+        <v>7118.9</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="0" t="s">
+        <v>286</v>
+      </c>
+      <c r="B127" s="0" t="s">
         <v>287</v>
       </c>
-      <c r="B127" s="0" t="s">
+      <c r="C127" s="0" t="s">
         <v>288</v>
       </c>
-      <c r="C127" s="0" t="s">
-        <v>134</v>
-      </c>
       <c r="D127" s="0">
-        <v>2800</v>
+        <v>16095</v>
       </c>
     </row>
     <row r="128">
@@ -5024,10 +5024,10 @@
         <v>290</v>
       </c>
       <c r="C128" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D128" s="0">
-        <v>6375</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="129">
@@ -5038,10 +5038,10 @@
         <v>292</v>
       </c>
       <c r="C129" s="0" t="s">
-        <v>15</v>
+        <v>136</v>
       </c>
       <c r="D129" s="0">
-        <v>4200</v>
+        <v>6375</v>
       </c>
     </row>
     <row r="130">
@@ -5055,7 +5055,7 @@
         <v>15</v>
       </c>
       <c r="D130" s="0">
-        <v>1050</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="131">
@@ -5066,21 +5066,21 @@
         <v>296</v>
       </c>
       <c r="C131" s="0" t="s">
-        <v>297</v>
+        <v>15</v>
       </c>
       <c r="D131" s="0">
-        <v>3350</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="0" t="s">
+        <v>297</v>
+      </c>
+      <c r="B132" s="0" t="s">
         <v>298</v>
       </c>
-      <c r="B132" s="0" t="s">
+      <c r="C132" s="0" t="s">
         <v>299</v>
-      </c>
-      <c r="C132" s="0" t="s">
-        <v>119</v>
       </c>
       <c r="D132" s="0">
         <v>3350</v>
@@ -5094,24 +5094,24 @@
         <v>301</v>
       </c>
       <c r="C133" s="0" t="s">
-        <v>302</v>
+        <v>119</v>
       </c>
       <c r="D133" s="0">
-        <v>0</v>
+        <v>3350</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="0" t="s">
+        <v>302</v>
+      </c>
+      <c r="B134" s="0" t="s">
         <v>303</v>
       </c>
-      <c r="B134" s="0" t="s">
+      <c r="C134" s="0" t="s">
         <v>304</v>
       </c>
-      <c r="C134" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="D134" s="0">
-        <v>1600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="135">
@@ -5125,7 +5125,7 @@
         <v>15</v>
       </c>
       <c r="D135" s="0">
-        <v>2000</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="136">
@@ -5136,24 +5136,24 @@
         <v>308</v>
       </c>
       <c r="C136" s="0" t="s">
-        <v>309</v>
+        <v>15</v>
       </c>
       <c r="D136" s="0">
-        <v>2728</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="0" t="s">
+        <v>309</v>
+      </c>
+      <c r="B137" s="0" t="s">
         <v>310</v>
       </c>
-      <c r="B137" s="0" t="s">
+      <c r="C137" s="0" t="s">
         <v>311</v>
       </c>
-      <c r="C137" s="0" t="s">
-        <v>70</v>
-      </c>
       <c r="D137" s="0">
-        <v>0</v>
+        <v>2728</v>
       </c>
     </row>
     <row r="138">
@@ -5167,7 +5167,7 @@
         <v>70</v>
       </c>
       <c r="D138" s="0">
-        <v>88248.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139">
@@ -5178,10 +5178,10 @@
         <v>315</v>
       </c>
       <c r="C139" s="0" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="D139" s="0">
-        <v>1800</v>
+        <v>88248.3</v>
       </c>
     </row>
     <row r="140">
@@ -5195,7 +5195,7 @@
         <v>52</v>
       </c>
       <c r="D140" s="0">
-        <v>2060</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="141">
@@ -5206,10 +5206,10 @@
         <v>319</v>
       </c>
       <c r="C141" s="0" t="s">
-        <v>15</v>
+        <v>52</v>
       </c>
       <c r="D141" s="0">
-        <v>1270</v>
+        <v>2060</v>
       </c>
     </row>
     <row r="142">
@@ -5220,10 +5220,10 @@
         <v>321</v>
       </c>
       <c r="C142" s="0" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="D142" s="0">
-        <v>700</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="143">
@@ -5234,7 +5234,7 @@
         <v>323</v>
       </c>
       <c r="C143" s="0" t="s">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="D143" s="0">
         <v>700</v>
@@ -5248,7 +5248,7 @@
         <v>325</v>
       </c>
       <c r="C144" s="0" t="s">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="D144" s="0">
         <v>700</v>
@@ -5262,10 +5262,10 @@
         <v>327</v>
       </c>
       <c r="C145" s="0" t="s">
-        <v>90</v>
+        <v>34</v>
       </c>
       <c r="D145" s="0">
-        <v>8318.75</v>
+        <v>700</v>
       </c>
     </row>
     <row r="146">
@@ -5276,24 +5276,24 @@
         <v>329</v>
       </c>
       <c r="C146" s="0" t="s">
-        <v>330</v>
+        <v>90</v>
       </c>
       <c r="D146" s="0">
-        <v>4500</v>
+        <v>1663.75</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="0" t="s">
+        <v>330</v>
+      </c>
+      <c r="B147" s="0" t="s">
         <v>331</v>
       </c>
-      <c r="B147" s="0" t="s">
+      <c r="C147" s="0" t="s">
         <v>332</v>
       </c>
-      <c r="C147" s="0" t="s">
-        <v>34</v>
-      </c>
       <c r="D147" s="0">
-        <v>390</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="148">
@@ -5304,10 +5304,10 @@
         <v>334</v>
       </c>
       <c r="C148" s="0" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="D148" s="0">
-        <v>500</v>
+        <v>390</v>
       </c>
     </row>
     <row r="149">
@@ -5318,10 +5318,10 @@
         <v>336</v>
       </c>
       <c r="C149" s="0" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D149" s="0">
-        <v>400</v>
+        <v>500</v>
       </c>
     </row>
     <row r="150">
@@ -5332,10 +5332,10 @@
         <v>338</v>
       </c>
       <c r="C150" s="0" t="s">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="D150" s="0">
-        <v>410</v>
+        <v>400</v>
       </c>
     </row>
     <row r="151">
@@ -5349,7 +5349,7 @@
         <v>70</v>
       </c>
       <c r="D151" s="0">
-        <v>580</v>
+        <v>410</v>
       </c>
     </row>
     <row r="152">
@@ -5360,10 +5360,10 @@
         <v>342</v>
       </c>
       <c r="C152" s="0" t="s">
-        <v>15</v>
+        <v>70</v>
       </c>
       <c r="D152" s="0">
-        <v>572</v>
+        <v>580</v>
       </c>
     </row>
     <row r="153">
@@ -5374,10 +5374,10 @@
         <v>344</v>
       </c>
       <c r="C153" s="0" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="D153" s="0">
-        <v>103000</v>
+        <v>572</v>
       </c>
     </row>
     <row r="154">
@@ -5391,7 +5391,7 @@
         <v>28</v>
       </c>
       <c r="D154" s="0">
-        <v>114000</v>
+        <v>103000</v>
       </c>
     </row>
     <row r="155">
@@ -5405,7 +5405,7 @@
         <v>28</v>
       </c>
       <c r="D155" s="0">
-        <v>135000</v>
+        <v>114000</v>
       </c>
     </row>
     <row r="156">
@@ -5416,24 +5416,24 @@
         <v>350</v>
       </c>
       <c r="C156" s="0" t="s">
-        <v>351</v>
+        <v>28</v>
       </c>
       <c r="D156" s="0">
-        <v>650</v>
+        <v>135000</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="0" t="s">
+        <v>351</v>
+      </c>
+      <c r="B157" s="0" t="s">
         <v>352</v>
       </c>
-      <c r="B157" s="0" t="s">
+      <c r="C157" s="0" t="s">
         <v>353</v>
       </c>
-      <c r="C157" s="0" t="s">
-        <v>108</v>
-      </c>
       <c r="D157" s="0">
-        <v>1590</v>
+        <v>650</v>
       </c>
     </row>
     <row r="158">
@@ -5444,10 +5444,10 @@
         <v>355</v>
       </c>
       <c r="C158" s="0" t="s">
-        <v>34</v>
+        <v>108</v>
       </c>
       <c r="D158" s="0">
-        <v>650</v>
+        <v>1590</v>
       </c>
     </row>
     <row r="159">
@@ -5458,7 +5458,7 @@
         <v>357</v>
       </c>
       <c r="C159" s="0" t="s">
-        <v>145</v>
+        <v>34</v>
       </c>
       <c r="D159" s="0">
         <v>650</v>
@@ -5472,7 +5472,7 @@
         <v>359</v>
       </c>
       <c r="C160" s="0" t="s">
-        <v>15</v>
+        <v>147</v>
       </c>
       <c r="D160" s="0">
         <v>650</v>
@@ -5489,7 +5489,7 @@
         <v>15</v>
       </c>
       <c r="D161" s="0">
-        <v>1700</v>
+        <v>650</v>
       </c>
     </row>
     <row r="162">
@@ -5503,7 +5503,7 @@
         <v>15</v>
       </c>
       <c r="D162" s="0">
-        <v>0</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="163">
@@ -5514,10 +5514,10 @@
         <v>365</v>
       </c>
       <c r="C163" s="0" t="s">
-        <v>113</v>
+        <v>15</v>
       </c>
       <c r="D163" s="0">
-        <v>1290</v>
+        <v>0</v>
       </c>
     </row>
     <row r="164">
@@ -5528,38 +5528,38 @@
         <v>367</v>
       </c>
       <c r="C164" s="0" t="s">
-        <v>368</v>
+        <v>113</v>
       </c>
       <c r="D164" s="0">
-        <v>55058.9</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="0" t="s">
+        <v>368</v>
+      </c>
+      <c r="B165" s="0" t="s">
         <v>369</v>
       </c>
-      <c r="B165" s="0" t="s">
+      <c r="C165" s="0" t="s">
         <v>370</v>
       </c>
-      <c r="C165" s="0" t="s">
-        <v>371</v>
-      </c>
       <c r="D165" s="0">
-        <v>104695.98</v>
+        <v>55058.9</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="0" t="s">
+        <v>371</v>
+      </c>
+      <c r="B166" s="0" t="s">
         <v>372</v>
       </c>
-      <c r="B166" s="0" t="s">
+      <c r="C166" s="0" t="s">
         <v>373</v>
       </c>
-      <c r="C166" s="0" t="s">
-        <v>371</v>
-      </c>
       <c r="D166" s="0">
-        <v>80478.92</v>
+        <v>104695.98</v>
       </c>
     </row>
     <row r="167">
@@ -5570,10 +5570,10 @@
         <v>375</v>
       </c>
       <c r="C167" s="0" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="D167" s="0">
-        <v>92546.68</v>
+        <v>80478.92</v>
       </c>
     </row>
     <row r="168">
@@ -5584,10 +5584,10 @@
         <v>377</v>
       </c>
       <c r="C168" s="0" t="s">
-        <v>28</v>
+        <v>373</v>
       </c>
       <c r="D168" s="0">
-        <v>954.8</v>
+        <v>92546.68</v>
       </c>
     </row>
     <row r="169">
@@ -5601,7 +5601,7 @@
         <v>28</v>
       </c>
       <c r="D169" s="0">
-        <v>265.3</v>
+        <v>954.8</v>
       </c>
     </row>
     <row r="170">
@@ -5615,7 +5615,7 @@
         <v>28</v>
       </c>
       <c r="D170" s="0">
-        <v>2743.71</v>
+        <v>265.3</v>
       </c>
     </row>
     <row r="171">
@@ -5626,24 +5626,24 @@
         <v>383</v>
       </c>
       <c r="C171" s="0" t="s">
-        <v>384</v>
+        <v>28</v>
       </c>
       <c r="D171" s="0">
-        <v>81</v>
+        <v>2743.71</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="0" t="s">
+        <v>384</v>
+      </c>
+      <c r="B172" s="0" t="s">
         <v>385</v>
       </c>
-      <c r="B172" s="0" t="s">
+      <c r="C172" s="0" t="s">
         <v>386</v>
       </c>
-      <c r="C172" s="0" t="s">
-        <v>18</v>
-      </c>
       <c r="D172" s="0">
-        <v>270</v>
+        <v>81</v>
       </c>
     </row>
     <row r="173">
@@ -5654,10 +5654,10 @@
         <v>388</v>
       </c>
       <c r="C173" s="0" t="s">
-        <v>145</v>
+        <v>18</v>
       </c>
       <c r="D173" s="0">
-        <v>257</v>
+        <v>270</v>
       </c>
     </row>
     <row r="174">
@@ -5668,10 +5668,10 @@
         <v>390</v>
       </c>
       <c r="C174" s="0" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="D174" s="0">
-        <v>2762.43</v>
+        <v>257</v>
       </c>
     </row>
     <row r="175">
@@ -5682,10 +5682,10 @@
         <v>392</v>
       </c>
       <c r="C175" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D175" s="0">
-        <v>3573.45</v>
+        <v>2762.43</v>
       </c>
     </row>
     <row r="176">
@@ -5696,10 +5696,10 @@
         <v>394</v>
       </c>
       <c r="C176" s="0" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
       <c r="D176" s="0">
-        <v>5100</v>
+        <v>3573.45</v>
       </c>
     </row>
     <row r="177">
@@ -5710,10 +5710,10 @@
         <v>396</v>
       </c>
       <c r="C177" s="0" t="s">
-        <v>368</v>
+        <v>119</v>
       </c>
       <c r="D177" s="0">
-        <v>37527.35</v>
+        <v>5100</v>
       </c>
     </row>
     <row r="178">
@@ -5724,10 +5724,10 @@
         <v>398</v>
       </c>
       <c r="C178" s="0" t="s">
-        <v>18</v>
+        <v>370</v>
       </c>
       <c r="D178" s="0">
-        <v>825.18</v>
+        <v>37527.35</v>
       </c>
     </row>
     <row r="179">
@@ -5741,7 +5741,7 @@
         <v>18</v>
       </c>
       <c r="D179" s="0">
-        <v>2850</v>
+        <v>825.18</v>
       </c>
     </row>
     <row r="180">
@@ -5755,7 +5755,7 @@
         <v>18</v>
       </c>
       <c r="D180" s="0">
-        <v>6384.84</v>
+        <v>2850</v>
       </c>
     </row>
     <row r="181">
@@ -5769,7 +5769,7 @@
         <v>18</v>
       </c>
       <c r="D181" s="0">
-        <v>333.17</v>
+        <v>6384.84</v>
       </c>
     </row>
     <row r="182">
@@ -5783,7 +5783,7 @@
         <v>18</v>
       </c>
       <c r="D182" s="0">
-        <v>9669.15</v>
+        <v>333.17</v>
       </c>
     </row>
     <row r="183">
@@ -5797,7 +5797,7 @@
         <v>18</v>
       </c>
       <c r="D183" s="0">
-        <v>3599.84</v>
+        <v>9669.15</v>
       </c>
     </row>
     <row r="184">
@@ -5811,7 +5811,7 @@
         <v>18</v>
       </c>
       <c r="D184" s="0">
-        <v>412.8</v>
+        <v>3599.84</v>
       </c>
     </row>
     <row r="185">
@@ -5825,7 +5825,7 @@
         <v>18</v>
       </c>
       <c r="D185" s="0">
-        <v>2015.52</v>
+        <v>412.8</v>
       </c>
     </row>
     <row r="186">
@@ -5836,10 +5836,10 @@
         <v>414</v>
       </c>
       <c r="C186" s="0" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="D186" s="0">
-        <v>9041.55</v>
+        <v>2015.52</v>
       </c>
     </row>
     <row r="187">
@@ -5850,10 +5850,10 @@
         <v>416</v>
       </c>
       <c r="C187" s="0" t="s">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="D187" s="0">
-        <v>430</v>
+        <v>9041.55</v>
       </c>
     </row>
     <row r="188">
@@ -5867,7 +5867,7 @@
         <v>70</v>
       </c>
       <c r="D188" s="0">
-        <v>800</v>
+        <v>430</v>
       </c>
     </row>
     <row r="189">
@@ -5878,10 +5878,10 @@
         <v>420</v>
       </c>
       <c r="C189" s="0" t="s">
-        <v>236</v>
+        <v>70</v>
       </c>
       <c r="D189" s="0">
-        <v>2280</v>
+        <v>800</v>
       </c>
     </row>
     <row r="190">
@@ -5892,10 +5892,10 @@
         <v>422</v>
       </c>
       <c r="C190" s="0" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D190" s="0">
-        <v>1620</v>
+        <v>2280</v>
       </c>
     </row>
     <row r="191">
@@ -5906,10 +5906,10 @@
         <v>424</v>
       </c>
       <c r="C191" s="0" t="s">
-        <v>368</v>
+        <v>238</v>
       </c>
       <c r="D191" s="0">
-        <v>236458.17</v>
+        <v>1620</v>
       </c>
     </row>
     <row r="192">
@@ -5920,10 +5920,10 @@
         <v>426</v>
       </c>
       <c r="C192" s="0" t="s">
-        <v>28</v>
+        <v>370</v>
       </c>
       <c r="D192" s="0">
-        <v>317.2</v>
+        <v>236458.17</v>
       </c>
     </row>
     <row r="193">
@@ -5934,10 +5934,10 @@
         <v>428</v>
       </c>
       <c r="C193" s="0" t="s">
-        <v>368</v>
+        <v>28</v>
       </c>
       <c r="D193" s="0">
-        <v>25100</v>
+        <v>317.2</v>
       </c>
     </row>
     <row r="194">
@@ -5948,24 +5948,24 @@
         <v>430</v>
       </c>
       <c r="C194" s="0" t="s">
-        <v>431</v>
+        <v>370</v>
       </c>
       <c r="D194" s="0">
-        <v>20900</v>
+        <v>25100</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="0" t="s">
+        <v>431</v>
+      </c>
+      <c r="B195" s="0" t="s">
         <v>432</v>
       </c>
-      <c r="B195" s="0" t="s">
+      <c r="C195" s="0" t="s">
         <v>433</v>
       </c>
-      <c r="C195" s="0" t="s">
-        <v>45</v>
-      </c>
       <c r="D195" s="0">
-        <v>4729.48</v>
+        <v>20900</v>
       </c>
     </row>
     <row r="196">
@@ -5976,10 +5976,10 @@
         <v>435</v>
       </c>
       <c r="C196" s="0" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="D196" s="0">
-        <v>1104.46</v>
+        <v>4729.48</v>
       </c>
     </row>
     <row r="197">
@@ -5990,10 +5990,10 @@
         <v>437</v>
       </c>
       <c r="C197" s="0" t="s">
-        <v>90</v>
+        <v>21</v>
       </c>
       <c r="D197" s="0">
-        <v>11646.25</v>
+        <v>1104.46</v>
       </c>
     </row>
     <row r="198">
@@ -6004,10 +6004,10 @@
         <v>439</v>
       </c>
       <c r="C198" s="0" t="s">
-        <v>119</v>
+        <v>90</v>
       </c>
       <c r="D198" s="0">
-        <v>6072</v>
+        <v>11646.25</v>
       </c>
     </row>
     <row r="199">
@@ -6018,10 +6018,10 @@
         <v>441</v>
       </c>
       <c r="C199" s="0" t="s">
-        <v>70</v>
+        <v>119</v>
       </c>
       <c r="D199" s="0">
-        <v>400</v>
+        <v>6072</v>
       </c>
     </row>
     <row r="200">
@@ -6032,10 +6032,10 @@
         <v>443</v>
       </c>
       <c r="C200" s="0" t="s">
-        <v>21</v>
+        <v>70</v>
       </c>
       <c r="D200" s="0">
-        <v>409</v>
+        <v>400</v>
       </c>
     </row>
     <row r="201">
@@ -6046,10 +6046,10 @@
         <v>445</v>
       </c>
       <c r="C201" s="0" t="s">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="D201" s="0">
-        <v>10748</v>
+        <v>409</v>
       </c>
     </row>
     <row r="202">
@@ -6063,7 +6063,7 @@
         <v>64</v>
       </c>
       <c r="D202" s="0">
-        <v>12898</v>
+        <v>10748</v>
       </c>
     </row>
     <row r="203">
@@ -6074,10 +6074,10 @@
         <v>449</v>
       </c>
       <c r="C203" s="0" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="D203" s="0">
-        <v>2000</v>
+        <v>12898</v>
       </c>
     </row>
     <row r="204">
@@ -6088,24 +6088,24 @@
         <v>451</v>
       </c>
       <c r="C204" s="0" t="s">
-        <v>452</v>
+        <v>52</v>
       </c>
       <c r="D204" s="0">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="0" t="s">
+        <v>452</v>
+      </c>
+      <c r="B205" s="0" t="s">
         <v>453</v>
       </c>
-      <c r="B205" s="0" t="s">
+      <c r="C205" s="0" t="s">
         <v>454</v>
       </c>
-      <c r="C205" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="D205" s="0">
-        <v>490</v>
+        <v>0</v>
       </c>
     </row>
     <row r="206">
@@ -6116,10 +6116,10 @@
         <v>456</v>
       </c>
       <c r="C206" s="0" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D206" s="0">
-        <v>0</v>
+        <v>490</v>
       </c>
     </row>
     <row r="207">
@@ -6130,10 +6130,10 @@
         <v>458</v>
       </c>
       <c r="C207" s="0" t="s">
-        <v>154</v>
+        <v>34</v>
       </c>
       <c r="D207" s="0">
-        <v>25171.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="208">
@@ -6144,24 +6144,24 @@
         <v>460</v>
       </c>
       <c r="C208" s="0" t="s">
-        <v>461</v>
+        <v>156</v>
       </c>
       <c r="D208" s="0">
-        <v>60630</v>
+        <v>25171.1</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="0" t="s">
+        <v>461</v>
+      </c>
+      <c r="B209" s="0" t="s">
         <v>462</v>
       </c>
-      <c r="B209" s="0" t="s">
+      <c r="C209" s="0" t="s">
         <v>463</v>
       </c>
-      <c r="C209" s="0" t="s">
-        <v>145</v>
-      </c>
       <c r="D209" s="0">
-        <v>1800</v>
+        <v>60630</v>
       </c>
     </row>
     <row r="210">
@@ -6172,10 +6172,10 @@
         <v>465</v>
       </c>
       <c r="C210" s="0" t="s">
-        <v>34</v>
+        <v>147</v>
       </c>
       <c r="D210" s="0">
-        <v>0</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="211">
@@ -6186,10 +6186,10 @@
         <v>467</v>
       </c>
       <c r="C211" s="0" t="s">
-        <v>134</v>
+        <v>34</v>
       </c>
       <c r="D211" s="0">
-        <v>492.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="212">
@@ -6200,24 +6200,24 @@
         <v>469</v>
       </c>
       <c r="C212" s="0" t="s">
-        <v>470</v>
+        <v>136</v>
       </c>
       <c r="D212" s="0">
-        <v>495</v>
+        <v>492.2</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="0" t="s">
+        <v>470</v>
+      </c>
+      <c r="B213" s="0" t="s">
         <v>471</v>
       </c>
-      <c r="B213" s="0" t="s">
+      <c r="C213" s="0" t="s">
         <v>472</v>
       </c>
-      <c r="C213" s="0" t="s">
-        <v>18</v>
-      </c>
       <c r="D213" s="0">
-        <v>1786</v>
+        <v>495</v>
       </c>
     </row>
     <row r="214">
@@ -6231,7 +6231,7 @@
         <v>18</v>
       </c>
       <c r="D214" s="0">
-        <v>4391.8</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="215">
@@ -6242,10 +6242,10 @@
         <v>476</v>
       </c>
       <c r="C215" s="0" t="s">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="D215" s="0">
-        <v>4700</v>
+        <v>4391.8</v>
       </c>
     </row>
     <row r="216">
@@ -6259,7 +6259,7 @@
         <v>52</v>
       </c>
       <c r="D216" s="0">
-        <v>4200</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="217">
@@ -6298,21 +6298,21 @@
         <v>484</v>
       </c>
       <c r="C219" s="0" t="s">
-        <v>485</v>
+        <v>52</v>
       </c>
       <c r="D219" s="0">
-        <v>265</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="0" t="s">
+        <v>485</v>
+      </c>
+      <c r="B220" s="0" t="s">
         <v>486</v>
       </c>
-      <c r="B220" s="0" t="s">
+      <c r="C220" s="0" t="s">
         <v>487</v>
-      </c>
-      <c r="C220" s="0" t="s">
-        <v>485</v>
       </c>
       <c r="D220" s="0">
         <v>265</v>
@@ -6326,7 +6326,7 @@
         <v>489</v>
       </c>
       <c r="C221" s="0" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="D221" s="0">
         <v>265</v>
@@ -6340,7 +6340,7 @@
         <v>491</v>
       </c>
       <c r="C222" s="0" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="D222" s="0">
         <v>265</v>
@@ -6354,7 +6354,7 @@
         <v>493</v>
       </c>
       <c r="C223" s="0" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="D223" s="0">
         <v>265</v>
@@ -6368,7 +6368,7 @@
         <v>495</v>
       </c>
       <c r="C224" s="0" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="D224" s="0">
         <v>265</v>
@@ -6382,21 +6382,21 @@
         <v>497</v>
       </c>
       <c r="C225" s="0" t="s">
-        <v>498</v>
+        <v>487</v>
       </c>
       <c r="D225" s="0">
-        <v>4700</v>
+        <v>265</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="0" t="s">
+        <v>498</v>
+      </c>
+      <c r="B226" s="0" t="s">
         <v>499</v>
       </c>
-      <c r="B226" s="0" t="s">
+      <c r="C226" s="0" t="s">
         <v>500</v>
-      </c>
-      <c r="C226" s="0" t="s">
-        <v>501</v>
       </c>
       <c r="D226" s="0">
         <v>4700</v>
@@ -6404,13 +6404,13 @@
     </row>
     <row r="227">
       <c r="A227" s="0" t="s">
+        <v>501</v>
+      </c>
+      <c r="B227" s="0" t="s">
         <v>502</v>
       </c>
-      <c r="B227" s="0" t="s">
+      <c r="C227" s="0" t="s">
         <v>503</v>
-      </c>
-      <c r="C227" s="0" t="s">
-        <v>52</v>
       </c>
       <c r="D227" s="0">
         <v>4700</v>
@@ -6427,7 +6427,7 @@
         <v>52</v>
       </c>
       <c r="D228" s="0">
-        <v>500</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="229">
@@ -6441,7 +6441,7 @@
         <v>52</v>
       </c>
       <c r="D229" s="0">
-        <v>210</v>
+        <v>500</v>
       </c>
     </row>
     <row r="230">
@@ -6455,7 +6455,7 @@
         <v>52</v>
       </c>
       <c r="D230" s="0">
-        <v>247</v>
+        <v>210</v>
       </c>
     </row>
     <row r="231">
@@ -6466,10 +6466,10 @@
         <v>511</v>
       </c>
       <c r="C231" s="0" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="D231" s="0">
-        <v>5600</v>
+        <v>247</v>
       </c>
     </row>
     <row r="232">
@@ -6480,10 +6480,10 @@
         <v>513</v>
       </c>
       <c r="C232" s="0" t="s">
-        <v>145</v>
+        <v>37</v>
       </c>
       <c r="D232" s="0">
-        <v>6000</v>
+        <v>5600</v>
       </c>
     </row>
     <row r="233">
@@ -6494,10 +6494,10 @@
         <v>515</v>
       </c>
       <c r="C233" s="0" t="s">
-        <v>70</v>
+        <v>147</v>
       </c>
       <c r="D233" s="0">
-        <v>80000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="234">
@@ -6511,7 +6511,7 @@
         <v>70</v>
       </c>
       <c r="D234" s="0">
-        <v>90000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="235">
@@ -6525,7 +6525,7 @@
         <v>70</v>
       </c>
       <c r="D235" s="0">
-        <v>110000</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="236">
@@ -6536,10 +6536,10 @@
         <v>521</v>
       </c>
       <c r="C236" s="0" t="s">
-        <v>15</v>
+        <v>70</v>
       </c>
       <c r="D236" s="0">
-        <v>1100</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="237">
@@ -6553,7 +6553,7 @@
         <v>15</v>
       </c>
       <c r="D237" s="0">
-        <v>2500</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="238">
@@ -6564,10 +6564,10 @@
         <v>525</v>
       </c>
       <c r="C238" s="0" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="D238" s="0">
-        <v>13636.84</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="239">
@@ -6578,10 +6578,10 @@
         <v>527</v>
       </c>
       <c r="C239" s="0" t="s">
-        <v>275</v>
+        <v>28</v>
       </c>
       <c r="D239" s="0">
-        <v>450</v>
+        <v>13636.84</v>
       </c>
     </row>
     <row r="240">
@@ -6592,10 +6592,10 @@
         <v>529</v>
       </c>
       <c r="C240" s="0" t="s">
-        <v>15</v>
+        <v>277</v>
       </c>
       <c r="D240" s="0">
-        <v>555</v>
+        <v>450</v>
       </c>
     </row>
     <row r="241">
@@ -6609,7 +6609,7 @@
         <v>15</v>
       </c>
       <c r="D241" s="0">
-        <v>825</v>
+        <v>555</v>
       </c>
     </row>
     <row r="242">
@@ -6623,7 +6623,7 @@
         <v>15</v>
       </c>
       <c r="D242" s="0">
-        <v>36.3</v>
+        <v>825</v>
       </c>
     </row>
     <row r="243">
@@ -6637,7 +6637,7 @@
         <v>15</v>
       </c>
       <c r="D243" s="0">
-        <v>544.5</v>
+        <v>36.3</v>
       </c>
     </row>
     <row r="244">
@@ -6651,7 +6651,7 @@
         <v>15</v>
       </c>
       <c r="D244" s="0">
-        <v>750</v>
+        <v>544.5</v>
       </c>
     </row>
     <row r="245">
@@ -6662,10 +6662,10 @@
         <v>539</v>
       </c>
       <c r="C245" s="0" t="s">
-        <v>145</v>
+        <v>15</v>
       </c>
       <c r="D245" s="0">
-        <v>1130</v>
+        <v>750</v>
       </c>
     </row>
     <row r="246">
@@ -6676,10 +6676,10 @@
         <v>541</v>
       </c>
       <c r="C246" s="0" t="s">
-        <v>52</v>
+        <v>147</v>
       </c>
       <c r="D246" s="0">
-        <v>4510</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="247">
@@ -6732,10 +6732,10 @@
         <v>549</v>
       </c>
       <c r="C250" s="0" t="s">
-        <v>15</v>
+        <v>52</v>
       </c>
       <c r="D250" s="0">
-        <v>902</v>
+        <v>4510</v>
       </c>
     </row>
     <row r="251">
@@ -6749,7 +6749,7 @@
         <v>15</v>
       </c>
       <c r="D251" s="0">
-        <v>880</v>
+        <v>902</v>
       </c>
     </row>
     <row r="252">
@@ -6760,10 +6760,10 @@
         <v>553</v>
       </c>
       <c r="C252" s="0" t="s">
-        <v>134</v>
+        <v>15</v>
       </c>
       <c r="D252" s="0">
-        <v>430</v>
+        <v>880</v>
       </c>
     </row>
     <row r="253">
@@ -6774,10 +6774,10 @@
         <v>555</v>
       </c>
       <c r="C253" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D253" s="0">
-        <v>354.54</v>
+        <v>430</v>
       </c>
     </row>
     <row r="254">
@@ -6788,10 +6788,10 @@
         <v>557</v>
       </c>
       <c r="C254" s="0" t="s">
-        <v>18</v>
+        <v>136</v>
       </c>
       <c r="D254" s="0">
-        <v>318.63</v>
+        <v>354.54</v>
       </c>
     </row>
     <row r="255">
@@ -6805,7 +6805,7 @@
         <v>18</v>
       </c>
       <c r="D255" s="0">
-        <v>415.15</v>
+        <v>318.63</v>
       </c>
     </row>
     <row r="256">
@@ -6819,7 +6819,7 @@
         <v>18</v>
       </c>
       <c r="D256" s="0">
-        <v>760</v>
+        <v>415.15</v>
       </c>
     </row>
     <row r="257">
@@ -6833,7 +6833,7 @@
         <v>18</v>
       </c>
       <c r="D257" s="0">
-        <v>820</v>
+        <v>760</v>
       </c>
     </row>
     <row r="258">
@@ -6844,24 +6844,24 @@
         <v>565</v>
       </c>
       <c r="C258" s="0" t="s">
-        <v>566</v>
+        <v>18</v>
       </c>
       <c r="D258" s="0">
-        <v>177940.1</v>
+        <v>820</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="0" t="s">
+        <v>566</v>
+      </c>
+      <c r="B259" s="0" t="s">
         <v>567</v>
       </c>
-      <c r="B259" s="0" t="s">
+      <c r="C259" s="0" t="s">
         <v>568</v>
       </c>
-      <c r="C259" s="0" t="s">
-        <v>70</v>
-      </c>
       <c r="D259" s="0">
-        <v>34000</v>
+        <v>177940.1</v>
       </c>
     </row>
     <row r="260">
@@ -6875,7 +6875,7 @@
         <v>70</v>
       </c>
       <c r="D260" s="0">
-        <v>30000</v>
+        <v>34000</v>
       </c>
     </row>
     <row r="261">
@@ -6886,10 +6886,10 @@
         <v>572</v>
       </c>
       <c r="C261" s="0" t="s">
-        <v>461</v>
+        <v>70</v>
       </c>
       <c r="D261" s="0">
-        <v>227939.52</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="262">
@@ -6900,10 +6900,10 @@
         <v>574</v>
       </c>
       <c r="C262" s="0" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="D262" s="0">
-        <v>184488.7</v>
+        <v>227939.52</v>
       </c>
     </row>
     <row r="263">
@@ -6914,10 +6914,10 @@
         <v>576</v>
       </c>
       <c r="C263" s="0" t="s">
-        <v>15</v>
+        <v>463</v>
       </c>
       <c r="D263" s="0">
-        <v>1760</v>
+        <v>184488.7</v>
       </c>
     </row>
     <row r="264">
@@ -6928,24 +6928,24 @@
         <v>578</v>
       </c>
       <c r="C264" s="0" t="s">
-        <v>579</v>
+        <v>15</v>
       </c>
       <c r="D264" s="0">
-        <v>26350</v>
+        <v>1760</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="0" t="s">
+        <v>579</v>
+      </c>
+      <c r="B265" s="0" t="s">
         <v>580</v>
       </c>
-      <c r="B265" s="0" t="s">
+      <c r="C265" s="0" t="s">
         <v>581</v>
       </c>
-      <c r="C265" s="0" t="s">
-        <v>470</v>
-      </c>
       <c r="D265" s="0">
-        <v>31250</v>
+        <v>26350</v>
       </c>
     </row>
     <row r="266">
@@ -6956,10 +6956,10 @@
         <v>583</v>
       </c>
       <c r="C266" s="0" t="s">
-        <v>52</v>
+        <v>472</v>
       </c>
       <c r="D266" s="0">
-        <v>34.98</v>
+        <v>31250</v>
       </c>
     </row>
     <row r="267">
@@ -6970,21 +6970,21 @@
         <v>585</v>
       </c>
       <c r="C267" s="0" t="s">
-        <v>586</v>
+        <v>52</v>
       </c>
       <c r="D267" s="0">
-        <v>65</v>
+        <v>34.98</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="0" t="s">
+        <v>586</v>
+      </c>
+      <c r="B268" s="0" t="s">
         <v>587</v>
       </c>
-      <c r="B268" s="0" t="s">
+      <c r="C268" s="0" t="s">
         <v>588</v>
-      </c>
-      <c r="C268" s="0" t="s">
-        <v>52</v>
       </c>
       <c r="D268" s="0">
         <v>65</v>
@@ -7001,7 +7001,7 @@
         <v>52</v>
       </c>
       <c r="D269" s="0">
-        <v>92</v>
+        <v>65</v>
       </c>
     </row>
     <row r="270">
@@ -7015,7 +7015,7 @@
         <v>52</v>
       </c>
       <c r="D270" s="0">
-        <v>33</v>
+        <v>92</v>
       </c>
     </row>
     <row r="271">
@@ -7029,7 +7029,7 @@
         <v>52</v>
       </c>
       <c r="D271" s="0">
-        <v>38.22</v>
+        <v>33</v>
       </c>
     </row>
     <row r="272">
@@ -7040,10 +7040,10 @@
         <v>596</v>
       </c>
       <c r="C272" s="0" t="s">
-        <v>330</v>
+        <v>52</v>
       </c>
       <c r="D272" s="0">
-        <v>300</v>
+        <v>38.22</v>
       </c>
     </row>
     <row r="273">
@@ -7054,10 +7054,10 @@
         <v>598</v>
       </c>
       <c r="C273" s="0" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="D273" s="0">
-        <v>370</v>
+        <v>300</v>
       </c>
     </row>
     <row r="274">
@@ -7068,10 +7068,10 @@
         <v>600</v>
       </c>
       <c r="C274" s="0" t="s">
-        <v>351</v>
+        <v>332</v>
       </c>
       <c r="D274" s="0">
-        <v>450</v>
+        <v>370</v>
       </c>
     </row>
     <row r="275">
@@ -7082,7 +7082,7 @@
         <v>602</v>
       </c>
       <c r="C275" s="0" t="s">
-        <v>37</v>
+        <v>353</v>
       </c>
       <c r="D275" s="0">
         <v>450</v>
@@ -7096,7 +7096,7 @@
         <v>604</v>
       </c>
       <c r="C276" s="0" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="D276" s="0">
         <v>450</v>
@@ -7113,7 +7113,7 @@
         <v>15</v>
       </c>
       <c r="D277" s="0">
-        <v>1650</v>
+        <v>450</v>
       </c>
     </row>
     <row r="278">
@@ -7127,7 +7127,7 @@
         <v>15</v>
       </c>
       <c r="D278" s="0">
-        <v>2100</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="279">
@@ -7141,7 +7141,7 @@
         <v>15</v>
       </c>
       <c r="D279" s="0">
-        <v>1980</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="280">
@@ -7155,7 +7155,7 @@
         <v>15</v>
       </c>
       <c r="D280" s="0">
-        <v>2160</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="281">
@@ -7169,7 +7169,7 @@
         <v>15</v>
       </c>
       <c r="D281" s="0">
-        <v>1500</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="282">
@@ -7183,7 +7183,7 @@
         <v>15</v>
       </c>
       <c r="D282" s="0">
-        <v>2600</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="283">
@@ -7197,7 +7197,7 @@
         <v>15</v>
       </c>
       <c r="D283" s="0">
-        <v>2000</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="284">
@@ -7211,7 +7211,7 @@
         <v>15</v>
       </c>
       <c r="D284" s="0">
-        <v>6700</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="285">
@@ -7225,7 +7225,7 @@
         <v>15</v>
       </c>
       <c r="D285" s="0">
-        <v>1650</v>
+        <v>6700</v>
       </c>
     </row>
     <row r="286">
@@ -7239,7 +7239,7 @@
         <v>15</v>
       </c>
       <c r="D286" s="0">
-        <v>1035</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="287">
@@ -7253,7 +7253,7 @@
         <v>15</v>
       </c>
       <c r="D287" s="0">
-        <v>2600</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="288">
@@ -7267,7 +7267,7 @@
         <v>15</v>
       </c>
       <c r="D288" s="0">
-        <v>2400</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="289">
@@ -7278,10 +7278,10 @@
         <v>630</v>
       </c>
       <c r="C289" s="0" t="s">
-        <v>134</v>
+        <v>15</v>
       </c>
       <c r="D289" s="0">
-        <v>4497.2</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="290">
@@ -7292,10 +7292,10 @@
         <v>632</v>
       </c>
       <c r="C290" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D290" s="0">
-        <v>2328</v>
+        <v>4497.2</v>
       </c>
     </row>
     <row r="291">
@@ -7306,10 +7306,10 @@
         <v>634</v>
       </c>
       <c r="C291" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D291" s="0">
-        <v>1138</v>
+        <v>2328</v>
       </c>
     </row>
     <row r="292">
@@ -7320,10 +7320,10 @@
         <v>636</v>
       </c>
       <c r="C292" s="0" t="s">
-        <v>28</v>
+        <v>136</v>
       </c>
       <c r="D292" s="0">
-        <v>7372.42</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="293">
@@ -7334,10 +7334,10 @@
         <v>638</v>
       </c>
       <c r="C293" s="0" t="s">
-        <v>119</v>
+        <v>28</v>
       </c>
       <c r="D293" s="0">
-        <v>1790</v>
+        <v>7372.42</v>
       </c>
     </row>
     <row r="294">
@@ -7351,7 +7351,7 @@
         <v>119</v>
       </c>
       <c r="D294" s="0">
-        <v>2859.96</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="295">
@@ -7365,7 +7365,7 @@
         <v>119</v>
       </c>
       <c r="D295" s="0">
-        <v>4800</v>
+        <v>2859.96</v>
       </c>
     </row>
     <row r="296">
@@ -7376,24 +7376,24 @@
         <v>644</v>
       </c>
       <c r="C296" s="0" t="s">
-        <v>645</v>
+        <v>119</v>
       </c>
       <c r="D296" s="0">
-        <v>0</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="0" t="s">
+        <v>645</v>
+      </c>
+      <c r="B297" s="0" t="s">
         <v>646</v>
       </c>
-      <c r="B297" s="0" t="s">
+      <c r="C297" s="0" t="s">
         <v>647</v>
       </c>
-      <c r="C297" s="0" t="s">
-        <v>28</v>
-      </c>
       <c r="D297" s="0">
-        <v>494</v>
+        <v>0</v>
       </c>
     </row>
     <row r="298">
@@ -7407,7 +7407,7 @@
         <v>28</v>
       </c>
       <c r="D298" s="0">
-        <v>665.3</v>
+        <v>494</v>
       </c>
     </row>
     <row r="299">
@@ -7418,10 +7418,10 @@
         <v>651</v>
       </c>
       <c r="C299" s="0" t="s">
-        <v>90</v>
+        <v>28</v>
       </c>
       <c r="D299" s="0">
-        <v>33275</v>
+        <v>665.3</v>
       </c>
     </row>
     <row r="300">
@@ -7435,7 +7435,7 @@
         <v>90</v>
       </c>
       <c r="D300" s="0">
-        <v>4525.4</v>
+        <v>33275</v>
       </c>
     </row>
     <row r="301">
@@ -7446,10 +7446,10 @@
         <v>655</v>
       </c>
       <c r="C301" s="0" t="s">
-        <v>145</v>
+        <v>90</v>
       </c>
       <c r="D301" s="0">
-        <v>896</v>
+        <v>4525.4</v>
       </c>
     </row>
     <row r="302">
@@ -7460,10 +7460,10 @@
         <v>657</v>
       </c>
       <c r="C302" s="0" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="D302" s="0">
-        <v>1250</v>
+        <v>896</v>
       </c>
     </row>
     <row r="303">
@@ -7474,10 +7474,10 @@
         <v>659</v>
       </c>
       <c r="C303" s="0" t="s">
-        <v>90</v>
+        <v>136</v>
       </c>
       <c r="D303" s="0">
-        <v>312785</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="304">
@@ -7488,10 +7488,10 @@
         <v>661</v>
       </c>
       <c r="C304" s="0" t="s">
-        <v>196</v>
+        <v>90</v>
       </c>
       <c r="D304" s="0">
-        <v>17440</v>
+        <v>312785</v>
       </c>
     </row>
     <row r="305">
@@ -7502,10 +7502,10 @@
         <v>663</v>
       </c>
       <c r="C305" s="0" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D305" s="0">
-        <v>4390</v>
+        <v>17440</v>
       </c>
     </row>
     <row r="306">
@@ -7516,7 +7516,7 @@
         <v>665</v>
       </c>
       <c r="C306" s="0" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D306" s="0">
         <v>4390</v>
@@ -7530,10 +7530,10 @@
         <v>667</v>
       </c>
       <c r="C307" s="0" t="s">
-        <v>275</v>
+        <v>198</v>
       </c>
       <c r="D307" s="0">
-        <v>2250</v>
+        <v>4390</v>
       </c>
     </row>
     <row r="308">
@@ -7544,10 +7544,10 @@
         <v>669</v>
       </c>
       <c r="C308" s="0" t="s">
-        <v>196</v>
+        <v>277</v>
       </c>
       <c r="D308" s="0">
-        <v>3355</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="309">
@@ -7558,10 +7558,10 @@
         <v>671</v>
       </c>
       <c r="C309" s="0" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D309" s="0">
-        <v>7500</v>
+        <v>3355</v>
       </c>
     </row>
     <row r="310">
@@ -7572,10 +7572,10 @@
         <v>673</v>
       </c>
       <c r="C310" s="0" t="s">
-        <v>90</v>
+        <v>203</v>
       </c>
       <c r="D310" s="0">
-        <v>23958</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="311">
@@ -7589,7 +7589,7 @@
         <v>90</v>
       </c>
       <c r="D311" s="0">
-        <v>239580</v>
+        <v>23958</v>
       </c>
     </row>
     <row r="312">
@@ -7600,10 +7600,10 @@
         <v>677</v>
       </c>
       <c r="C312" s="0" t="s">
-        <v>52</v>
+        <v>90</v>
       </c>
       <c r="D312" s="0">
-        <v>130</v>
+        <v>239580</v>
       </c>
     </row>
     <row r="313">
@@ -7614,10 +7614,10 @@
         <v>679</v>
       </c>
       <c r="C313" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="D313" s="0">
-        <v>285.6</v>
+        <v>130</v>
       </c>
     </row>
     <row r="314">
@@ -7631,7 +7631,7 @@
         <v>21</v>
       </c>
       <c r="D314" s="0">
-        <v>338</v>
+        <v>285.6</v>
       </c>
     </row>
     <row r="315">
@@ -7642,21 +7642,21 @@
         <v>683</v>
       </c>
       <c r="C315" s="0" t="s">
-        <v>684</v>
+        <v>21</v>
       </c>
       <c r="D315" s="0">
-        <v>770</v>
+        <v>338</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="0" t="s">
+        <v>684</v>
+      </c>
+      <c r="B316" s="0" t="s">
         <v>685</v>
       </c>
-      <c r="B316" s="0" t="s">
+      <c r="C316" s="0" t="s">
         <v>686</v>
-      </c>
-      <c r="C316" s="0" t="s">
-        <v>687</v>
       </c>
       <c r="D316" s="0">
         <v>770</v>
@@ -7664,16 +7664,16 @@
     </row>
     <row r="317">
       <c r="A317" s="0" t="s">
+        <v>687</v>
+      </c>
+      <c r="B317" s="0" t="s">
         <v>688</v>
       </c>
-      <c r="B317" s="0" t="s">
+      <c r="C317" s="0" t="s">
         <v>689</v>
       </c>
-      <c r="C317" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="D317" s="0">
-        <v>973.5</v>
+        <v>770</v>
       </c>
     </row>
     <row r="318">
@@ -7684,10 +7684,10 @@
         <v>691</v>
       </c>
       <c r="C318" s="0" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D318" s="0">
-        <v>507.08</v>
+        <v>973.5</v>
       </c>
     </row>
     <row r="319">
@@ -7698,10 +7698,10 @@
         <v>693</v>
       </c>
       <c r="C319" s="0" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D319" s="0">
-        <v>450</v>
+        <v>507.08</v>
       </c>
     </row>
     <row r="320">
@@ -7712,10 +7712,10 @@
         <v>695</v>
       </c>
       <c r="C320" s="0" t="s">
-        <v>145</v>
+        <v>15</v>
       </c>
       <c r="D320" s="0">
-        <v>760</v>
+        <v>450</v>
       </c>
     </row>
     <row r="321">
@@ -7726,10 +7726,10 @@
         <v>697</v>
       </c>
       <c r="C321" s="0" t="s">
-        <v>275</v>
+        <v>147</v>
       </c>
       <c r="D321" s="0">
-        <v>5900</v>
+        <v>760</v>
       </c>
     </row>
     <row r="322">
@@ -7740,10 +7740,10 @@
         <v>699</v>
       </c>
       <c r="C322" s="0" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D322" s="0">
-        <v>2900</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="323">
@@ -7754,10 +7754,10 @@
         <v>701</v>
       </c>
       <c r="C323" s="0" t="s">
-        <v>134</v>
+        <v>277</v>
       </c>
       <c r="D323" s="0">
-        <v>886.2</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="324">
@@ -7768,10 +7768,10 @@
         <v>703</v>
       </c>
       <c r="C324" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D324" s="0">
-        <v>589.9</v>
+        <v>886.2</v>
       </c>
     </row>
     <row r="325">
@@ -7782,10 +7782,10 @@
         <v>705</v>
       </c>
       <c r="C325" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D325" s="0">
-        <v>65</v>
+        <v>589.9</v>
       </c>
     </row>
     <row r="326">
@@ -7796,10 +7796,10 @@
         <v>707</v>
       </c>
       <c r="C326" s="0" t="s">
-        <v>90</v>
+        <v>136</v>
       </c>
       <c r="D326" s="0">
-        <v>11313.5</v>
+        <v>65</v>
       </c>
     </row>
     <row r="327">
@@ -7810,10 +7810,10 @@
         <v>709</v>
       </c>
       <c r="C327" s="0" t="s">
-        <v>34</v>
+        <v>90</v>
       </c>
       <c r="D327" s="0">
-        <v>420</v>
+        <v>11313.5</v>
       </c>
     </row>
     <row r="328">
@@ -7824,10 +7824,10 @@
         <v>711</v>
       </c>
       <c r="C328" s="0" t="s">
-        <v>351</v>
+        <v>34</v>
       </c>
       <c r="D328" s="0">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="329">
@@ -7838,10 +7838,10 @@
         <v>713</v>
       </c>
       <c r="C329" s="0" t="s">
-        <v>21</v>
+        <v>353</v>
       </c>
       <c r="D329" s="0">
-        <v>377</v>
+        <v>418</v>
       </c>
     </row>
     <row r="330">
@@ -7852,10 +7852,10 @@
         <v>715</v>
       </c>
       <c r="C330" s="0" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="D330" s="0">
-        <v>5780.66</v>
+        <v>377</v>
       </c>
     </row>
     <row r="331">
@@ -7866,10 +7866,10 @@
         <v>717</v>
       </c>
       <c r="C331" s="0" t="s">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="D331" s="0">
-        <v>898</v>
+        <v>5780.66</v>
       </c>
     </row>
     <row r="332">
@@ -7880,10 +7880,10 @@
         <v>719</v>
       </c>
       <c r="C332" s="0" t="s">
-        <v>119</v>
+        <v>70</v>
       </c>
       <c r="D332" s="0">
-        <v>4767</v>
+        <v>898</v>
       </c>
     </row>
     <row r="333">
@@ -7894,10 +7894,10 @@
         <v>721</v>
       </c>
       <c r="C333" s="0" t="s">
-        <v>34</v>
+        <v>119</v>
       </c>
       <c r="D333" s="0">
-        <v>650</v>
+        <v>4767</v>
       </c>
     </row>
     <row r="334">
@@ -7908,7 +7908,7 @@
         <v>723</v>
       </c>
       <c r="C334" s="0" t="s">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="D334" s="0">
         <v>650</v>
@@ -7922,10 +7922,10 @@
         <v>725</v>
       </c>
       <c r="C335" s="0" t="s">
-        <v>15</v>
+        <v>70</v>
       </c>
       <c r="D335" s="0">
-        <v>2178</v>
+        <v>650</v>
       </c>
     </row>
     <row r="336">
@@ -7936,10 +7936,10 @@
         <v>727</v>
       </c>
       <c r="C336" s="0" t="s">
-        <v>90</v>
+        <v>15</v>
       </c>
       <c r="D336" s="0">
-        <v>7986</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="337">
@@ -7950,24 +7950,24 @@
         <v>729</v>
       </c>
       <c r="C337" s="0" t="s">
-        <v>730</v>
+        <v>90</v>
       </c>
       <c r="D337" s="0">
-        <v>1910</v>
+        <v>7986</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="0" t="s">
+        <v>730</v>
+      </c>
+      <c r="B338" s="0" t="s">
         <v>731</v>
       </c>
-      <c r="B338" s="0" t="s">
+      <c r="C338" s="0" t="s">
         <v>732</v>
       </c>
-      <c r="C338" s="0" t="s">
-        <v>145</v>
-      </c>
       <c r="D338" s="0">
-        <v>900</v>
+        <v>1910</v>
       </c>
     </row>
     <row r="339">
@@ -7978,10 +7978,10 @@
         <v>734</v>
       </c>
       <c r="C339" s="0" t="s">
-        <v>21</v>
+        <v>147</v>
       </c>
       <c r="D339" s="0">
-        <v>1722</v>
+        <v>900</v>
       </c>
     </row>
     <row r="340">
@@ -7992,10 +7992,10 @@
         <v>736</v>
       </c>
       <c r="C340" s="0" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="D340" s="0">
-        <v>456</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="341">
@@ -8020,7 +8020,7 @@
         <v>740</v>
       </c>
       <c r="C342" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D342" s="0">
         <v>750</v>
@@ -8034,7 +8034,7 @@
         <v>742</v>
       </c>
       <c r="C343" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D343" s="0">
         <v>1212</v>
@@ -8048,7 +8048,7 @@
         <v>744</v>
       </c>
       <c r="C344" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D344" s="0">
         <v>1300</v>
@@ -8062,7 +8062,7 @@
         <v>746</v>
       </c>
       <c r="C345" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D345" s="0">
         <v>1500</v>
@@ -8076,7 +8076,7 @@
         <v>748</v>
       </c>
       <c r="C346" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D346" s="0">
         <v>1400</v>
@@ -8090,7 +8090,7 @@
         <v>750</v>
       </c>
       <c r="C347" s="0" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D347" s="0">
         <v>11959</v>
@@ -8104,7 +8104,7 @@
         <v>752</v>
       </c>
       <c r="C348" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D348" s="0">
         <v>345</v>
@@ -8118,7 +8118,7 @@
         <v>754</v>
       </c>
       <c r="C349" s="0" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D349" s="0">
         <v>1450</v>
@@ -8160,7 +8160,7 @@
         <v>760</v>
       </c>
       <c r="C352" s="0" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D352" s="0">
         <v>566</v>
@@ -8174,7 +8174,7 @@
         <v>762</v>
       </c>
       <c r="C353" s="0" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="D353" s="0">
         <v>64925</v>
@@ -8216,7 +8216,7 @@
         <v>768</v>
       </c>
       <c r="C356" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D356" s="0">
         <v>1182.75</v>
@@ -8230,7 +8230,7 @@
         <v>770</v>
       </c>
       <c r="C357" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D357" s="0">
         <v>4440.9</v>
@@ -8314,7 +8314,7 @@
         <v>782</v>
       </c>
       <c r="C363" s="0" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="D363" s="0">
         <v>134775.6</v>
@@ -8328,7 +8328,7 @@
         <v>784</v>
       </c>
       <c r="C364" s="0" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="D364" s="0">
         <v>175991.55</v>
@@ -8370,7 +8370,7 @@
         <v>790</v>
       </c>
       <c r="C367" s="0" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D367" s="0">
         <v>515</v>
@@ -8412,7 +8412,7 @@
         <v>796</v>
       </c>
       <c r="C370" s="0" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="D370" s="0">
         <v>207558.08</v>
@@ -8426,7 +8426,7 @@
         <v>798</v>
       </c>
       <c r="C371" s="0" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="D371" s="0">
         <v>249069.69</v>
@@ -8664,7 +8664,7 @@
         <v>835</v>
       </c>
       <c r="C388" s="0" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D388" s="0">
         <v>65537</v>
@@ -8678,7 +8678,7 @@
         <v>837</v>
       </c>
       <c r="C389" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D389" s="0">
         <v>4049.6</v>
@@ -8692,7 +8692,7 @@
         <v>839</v>
       </c>
       <c r="C390" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D390" s="0">
         <v>4199.2</v>
@@ -8706,7 +8706,7 @@
         <v>841</v>
       </c>
       <c r="C391" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D391" s="0">
         <v>6397.2</v>
@@ -8720,7 +8720,7 @@
         <v>843</v>
       </c>
       <c r="C392" s="0" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D392" s="0">
         <v>570</v>
@@ -8804,7 +8804,7 @@
         <v>855</v>
       </c>
       <c r="C398" s="0" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D398" s="0">
         <v>857.67</v>
@@ -8832,7 +8832,7 @@
         <v>859</v>
       </c>
       <c r="C400" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D400" s="0">
         <v>360</v>
@@ -8846,7 +8846,7 @@
         <v>861</v>
       </c>
       <c r="C401" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D401" s="0">
         <v>450</v>
@@ -8860,10 +8860,10 @@
         <v>863</v>
       </c>
       <c r="C402" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D402" s="0">
-        <v>2050</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="403">
@@ -8874,7 +8874,7 @@
         <v>865</v>
       </c>
       <c r="C403" s="0" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="D403" s="0">
         <v>25192.82</v>
@@ -8902,7 +8902,7 @@
         <v>869</v>
       </c>
       <c r="C405" s="0" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D405" s="0">
         <v>600</v>
@@ -8930,7 +8930,7 @@
         <v>874</v>
       </c>
       <c r="C407" s="0" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="D407" s="0">
         <v>8628</v>
@@ -8958,7 +8958,7 @@
         <v>878</v>
       </c>
       <c r="C409" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D409" s="0">
         <v>1080</v>
@@ -8972,7 +8972,7 @@
         <v>880</v>
       </c>
       <c r="C410" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D410" s="0">
         <v>4012</v>
@@ -9084,7 +9084,7 @@
         <v>896</v>
       </c>
       <c r="C418" s="0" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="D418" s="0">
         <v>510</v>
@@ -9280,7 +9280,7 @@
         <v>926</v>
       </c>
       <c r="C432" s="0" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D432" s="0">
         <v>430</v>
@@ -9308,7 +9308,7 @@
         <v>930</v>
       </c>
       <c r="C434" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D434" s="0">
         <v>14001</v>
@@ -9448,7 +9448,7 @@
         <v>951</v>
       </c>
       <c r="C444" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D444" s="0">
         <v>3750</v>
@@ -9532,7 +9532,7 @@
         <v>964</v>
       </c>
       <c r="C450" s="0" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D450" s="0">
         <v>65142.6</v>
@@ -9546,7 +9546,7 @@
         <v>966</v>
       </c>
       <c r="C451" s="0" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D451" s="0">
         <v>23482.7</v>
@@ -9658,7 +9658,7 @@
         <v>985</v>
       </c>
       <c r="C459" s="0" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="D459" s="0">
         <v>71176.4</v>
@@ -9672,7 +9672,7 @@
         <v>987</v>
       </c>
       <c r="C460" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D460" s="0">
         <v>96</v>
@@ -9700,7 +9700,7 @@
         <v>991</v>
       </c>
       <c r="C462" s="0" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="D462" s="0">
         <v>342641</v>
@@ -9714,7 +9714,7 @@
         <v>993</v>
       </c>
       <c r="C463" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D463" s="0">
         <v>2200</v>
@@ -9728,7 +9728,7 @@
         <v>995</v>
       </c>
       <c r="C464" s="0" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="D464" s="0">
         <v>41000</v>
@@ -9840,7 +9840,7 @@
         <v>1011</v>
       </c>
       <c r="C472" s="0" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D472" s="0">
         <v>3700</v>
@@ -9854,7 +9854,7 @@
         <v>1013</v>
       </c>
       <c r="C473" s="0" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D473" s="0">
         <v>2600</v>
@@ -9924,7 +9924,7 @@
         <v>1024</v>
       </c>
       <c r="C478" s="0" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D478" s="0">
         <v>3859.93</v>
@@ -9938,7 +9938,7 @@
         <v>1026</v>
       </c>
       <c r="C479" s="0" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D479" s="0">
         <v>11751.49</v>
@@ -9952,7 +9952,7 @@
         <v>1028</v>
       </c>
       <c r="C480" s="0" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="D480" s="0">
         <v>6000</v>
@@ -9966,7 +9966,7 @@
         <v>1030</v>
       </c>
       <c r="C481" s="0" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="D481" s="0">
         <v>3000</v>
@@ -10036,7 +10036,7 @@
         <v>1041</v>
       </c>
       <c r="C486" s="0" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="D486" s="0">
         <v>207558.07</v>
@@ -10050,7 +10050,7 @@
         <v>1043</v>
       </c>
       <c r="C487" s="0" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D487" s="0">
         <v>77429.29</v>
@@ -10064,7 +10064,7 @@
         <v>1045</v>
       </c>
       <c r="C488" s="0" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D488" s="0">
         <v>42913.42</v>
@@ -10078,7 +10078,7 @@
         <v>1047</v>
       </c>
       <c r="C489" s="0" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D489" s="0">
         <v>88806.25</v>
@@ -10092,7 +10092,7 @@
         <v>1049</v>
       </c>
       <c r="C490" s="0" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D490" s="0">
         <v>50781.52</v>
@@ -10176,7 +10176,7 @@
         <v>1061</v>
       </c>
       <c r="C496" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D496" s="0">
         <v>430</v>
@@ -10190,7 +10190,7 @@
         <v>1063</v>
       </c>
       <c r="C497" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D497" s="0">
         <v>462</v>

</xml_diff>

<commit_message>
sync: stock y precios actualizados sáb. 15/08/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1066" uniqueCount="1066">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="1068">
   <si>
     <t>Solo Activos</t>
   </si>
@@ -933,6 +933,12 @@
   </si>
   <si>
     <t>KRATEC</t>
+  </si>
+  <si>
+    <t>000024401</t>
+  </si>
+  <si>
+    <t>DAZOMET METFORMINA 500MG X 10 - SAVANT - 000024401</t>
   </si>
   <si>
     <t>000023860</t>
@@ -3275,7 +3281,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:D498"/>
+  <dimension ref="A2:D499"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -5142,10 +5148,10 @@
         <v>308</v>
       </c>
       <c r="C136" s="0" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D136" s="0">
-        <v>1600</v>
+        <v>589.9</v>
       </c>
     </row>
     <row r="137">
@@ -5159,7 +5165,7 @@
         <v>15</v>
       </c>
       <c r="D137" s="0">
-        <v>2000</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="138">
@@ -5170,24 +5176,24 @@
         <v>312</v>
       </c>
       <c r="C138" s="0" t="s">
-        <v>313</v>
+        <v>15</v>
       </c>
       <c r="D138" s="0">
-        <v>2728</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="0" t="s">
+        <v>313</v>
+      </c>
+      <c r="B139" s="0" t="s">
         <v>314</v>
       </c>
-      <c r="B139" s="0" t="s">
+      <c r="C139" s="0" t="s">
         <v>315</v>
       </c>
-      <c r="C139" s="0" t="s">
-        <v>70</v>
-      </c>
       <c r="D139" s="0">
-        <v>0</v>
+        <v>2728</v>
       </c>
     </row>
     <row r="140">
@@ -5201,7 +5207,7 @@
         <v>70</v>
       </c>
       <c r="D140" s="0">
-        <v>88248.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="141">
@@ -5212,10 +5218,10 @@
         <v>319</v>
       </c>
       <c r="C141" s="0" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="D141" s="0">
-        <v>1800</v>
+        <v>88248.3</v>
       </c>
     </row>
     <row r="142">
@@ -5229,7 +5235,7 @@
         <v>52</v>
       </c>
       <c r="D142" s="0">
-        <v>2060</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="143">
@@ -5240,10 +5246,10 @@
         <v>323</v>
       </c>
       <c r="C143" s="0" t="s">
-        <v>15</v>
+        <v>52</v>
       </c>
       <c r="D143" s="0">
-        <v>1270</v>
+        <v>2060</v>
       </c>
     </row>
     <row r="144">
@@ -5254,10 +5260,10 @@
         <v>325</v>
       </c>
       <c r="C144" s="0" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="D144" s="0">
-        <v>700</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="145">
@@ -5268,7 +5274,7 @@
         <v>327</v>
       </c>
       <c r="C145" s="0" t="s">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="D145" s="0">
         <v>700</v>
@@ -5282,7 +5288,7 @@
         <v>329</v>
       </c>
       <c r="C146" s="0" t="s">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="D146" s="0">
         <v>700</v>
@@ -5296,10 +5302,10 @@
         <v>331</v>
       </c>
       <c r="C147" s="0" t="s">
-        <v>92</v>
+        <v>34</v>
       </c>
       <c r="D147" s="0">
-        <v>1663.75</v>
+        <v>700</v>
       </c>
     </row>
     <row r="148">
@@ -5310,24 +5316,24 @@
         <v>333</v>
       </c>
       <c r="C148" s="0" t="s">
-        <v>334</v>
+        <v>92</v>
       </c>
       <c r="D148" s="0">
-        <v>4500</v>
+        <v>1663.75</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="0" t="s">
+        <v>334</v>
+      </c>
+      <c r="B149" s="0" t="s">
         <v>335</v>
       </c>
-      <c r="B149" s="0" t="s">
+      <c r="C149" s="0" t="s">
         <v>336</v>
       </c>
-      <c r="C149" s="0" t="s">
-        <v>34</v>
-      </c>
       <c r="D149" s="0">
-        <v>390</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="150">
@@ -5338,10 +5344,10 @@
         <v>338</v>
       </c>
       <c r="C150" s="0" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="D150" s="0">
-        <v>500</v>
+        <v>390</v>
       </c>
     </row>
     <row r="151">
@@ -5352,10 +5358,10 @@
         <v>340</v>
       </c>
       <c r="C151" s="0" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D151" s="0">
-        <v>400</v>
+        <v>500</v>
       </c>
     </row>
     <row r="152">
@@ -5366,10 +5372,10 @@
         <v>342</v>
       </c>
       <c r="C152" s="0" t="s">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="D152" s="0">
-        <v>410</v>
+        <v>400</v>
       </c>
     </row>
     <row r="153">
@@ -5383,7 +5389,7 @@
         <v>70</v>
       </c>
       <c r="D153" s="0">
-        <v>580</v>
+        <v>410</v>
       </c>
     </row>
     <row r="154">
@@ -5394,10 +5400,10 @@
         <v>346</v>
       </c>
       <c r="C154" s="0" t="s">
-        <v>15</v>
+        <v>70</v>
       </c>
       <c r="D154" s="0">
-        <v>572</v>
+        <v>580</v>
       </c>
     </row>
     <row r="155">
@@ -5408,10 +5414,10 @@
         <v>348</v>
       </c>
       <c r="C155" s="0" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="D155" s="0">
-        <v>103000</v>
+        <v>572</v>
       </c>
     </row>
     <row r="156">
@@ -5425,7 +5431,7 @@
         <v>28</v>
       </c>
       <c r="D156" s="0">
-        <v>114000</v>
+        <v>103000</v>
       </c>
     </row>
     <row r="157">
@@ -5439,7 +5445,7 @@
         <v>28</v>
       </c>
       <c r="D157" s="0">
-        <v>135000</v>
+        <v>114000</v>
       </c>
     </row>
     <row r="158">
@@ -5450,24 +5456,24 @@
         <v>354</v>
       </c>
       <c r="C158" s="0" t="s">
-        <v>355</v>
+        <v>28</v>
       </c>
       <c r="D158" s="0">
-        <v>650</v>
+        <v>135000</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="0" t="s">
+        <v>355</v>
+      </c>
+      <c r="B159" s="0" t="s">
         <v>356</v>
       </c>
-      <c r="B159" s="0" t="s">
+      <c r="C159" s="0" t="s">
         <v>357</v>
       </c>
-      <c r="C159" s="0" t="s">
-        <v>110</v>
-      </c>
       <c r="D159" s="0">
-        <v>1590</v>
+        <v>650</v>
       </c>
     </row>
     <row r="160">
@@ -5478,10 +5484,10 @@
         <v>359</v>
       </c>
       <c r="C160" s="0" t="s">
-        <v>34</v>
+        <v>110</v>
       </c>
       <c r="D160" s="0">
-        <v>650</v>
+        <v>1590</v>
       </c>
     </row>
     <row r="161">
@@ -5492,7 +5498,7 @@
         <v>361</v>
       </c>
       <c r="C161" s="0" t="s">
-        <v>149</v>
+        <v>34</v>
       </c>
       <c r="D161" s="0">
         <v>650</v>
@@ -5506,7 +5512,7 @@
         <v>363</v>
       </c>
       <c r="C162" s="0" t="s">
-        <v>15</v>
+        <v>149</v>
       </c>
       <c r="D162" s="0">
         <v>650</v>
@@ -5523,7 +5529,7 @@
         <v>15</v>
       </c>
       <c r="D163" s="0">
-        <v>1700</v>
+        <v>650</v>
       </c>
     </row>
     <row r="164">
@@ -5537,7 +5543,7 @@
         <v>15</v>
       </c>
       <c r="D164" s="0">
-        <v>0</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="165">
@@ -5548,10 +5554,10 @@
         <v>369</v>
       </c>
       <c r="C165" s="0" t="s">
-        <v>115</v>
+        <v>15</v>
       </c>
       <c r="D165" s="0">
-        <v>1290</v>
+        <v>0</v>
       </c>
     </row>
     <row r="166">
@@ -5562,38 +5568,38 @@
         <v>371</v>
       </c>
       <c r="C166" s="0" t="s">
-        <v>372</v>
+        <v>115</v>
       </c>
       <c r="D166" s="0">
-        <v>55058.9</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="0" t="s">
+        <v>372</v>
+      </c>
+      <c r="B167" s="0" t="s">
         <v>373</v>
       </c>
-      <c r="B167" s="0" t="s">
+      <c r="C167" s="0" t="s">
         <v>374</v>
       </c>
-      <c r="C167" s="0" t="s">
-        <v>375</v>
-      </c>
       <c r="D167" s="0">
-        <v>104695.98</v>
+        <v>55058.9</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="B168" s="0" t="s">
         <v>376</v>
       </c>
-      <c r="B168" s="0" t="s">
+      <c r="C168" s="0" t="s">
         <v>377</v>
       </c>
-      <c r="C168" s="0" t="s">
-        <v>375</v>
-      </c>
       <c r="D168" s="0">
-        <v>80478.92</v>
+        <v>104695.98</v>
       </c>
     </row>
     <row r="169">
@@ -5604,10 +5610,10 @@
         <v>379</v>
       </c>
       <c r="C169" s="0" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="D169" s="0">
-        <v>92546.68</v>
+        <v>80478.92</v>
       </c>
     </row>
     <row r="170">
@@ -5618,10 +5624,10 @@
         <v>381</v>
       </c>
       <c r="C170" s="0" t="s">
-        <v>28</v>
+        <v>377</v>
       </c>
       <c r="D170" s="0">
-        <v>954.8</v>
+        <v>92546.68</v>
       </c>
     </row>
     <row r="171">
@@ -5635,7 +5641,7 @@
         <v>28</v>
       </c>
       <c r="D171" s="0">
-        <v>265.3</v>
+        <v>954.8</v>
       </c>
     </row>
     <row r="172">
@@ -5649,7 +5655,7 @@
         <v>28</v>
       </c>
       <c r="D172" s="0">
-        <v>2743.71</v>
+        <v>265.3</v>
       </c>
     </row>
     <row r="173">
@@ -5660,24 +5666,24 @@
         <v>387</v>
       </c>
       <c r="C173" s="0" t="s">
-        <v>388</v>
+        <v>28</v>
       </c>
       <c r="D173" s="0">
-        <v>81</v>
+        <v>2743.71</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="0" t="s">
+        <v>388</v>
+      </c>
+      <c r="B174" s="0" t="s">
         <v>389</v>
       </c>
-      <c r="B174" s="0" t="s">
+      <c r="C174" s="0" t="s">
         <v>390</v>
       </c>
-      <c r="C174" s="0" t="s">
-        <v>18</v>
-      </c>
       <c r="D174" s="0">
-        <v>270</v>
+        <v>81</v>
       </c>
     </row>
     <row r="175">
@@ -5688,10 +5694,10 @@
         <v>392</v>
       </c>
       <c r="C175" s="0" t="s">
-        <v>149</v>
+        <v>18</v>
       </c>
       <c r="D175" s="0">
-        <v>257</v>
+        <v>270</v>
       </c>
     </row>
     <row r="176">
@@ -5702,10 +5708,10 @@
         <v>394</v>
       </c>
       <c r="C176" s="0" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="D176" s="0">
-        <v>2762.43</v>
+        <v>257</v>
       </c>
     </row>
     <row r="177">
@@ -5719,7 +5725,7 @@
         <v>138</v>
       </c>
       <c r="D177" s="0">
-        <v>3573.45</v>
+        <v>2762.43</v>
       </c>
     </row>
     <row r="178">
@@ -5730,10 +5736,10 @@
         <v>398</v>
       </c>
       <c r="C178" s="0" t="s">
-        <v>121</v>
+        <v>138</v>
       </c>
       <c r="D178" s="0">
-        <v>5100</v>
+        <v>3573.45</v>
       </c>
     </row>
     <row r="179">
@@ -5744,10 +5750,10 @@
         <v>400</v>
       </c>
       <c r="C179" s="0" t="s">
-        <v>372</v>
+        <v>121</v>
       </c>
       <c r="D179" s="0">
-        <v>37527.35</v>
+        <v>5100</v>
       </c>
     </row>
     <row r="180">
@@ -5758,10 +5764,10 @@
         <v>402</v>
       </c>
       <c r="C180" s="0" t="s">
-        <v>18</v>
+        <v>374</v>
       </c>
       <c r="D180" s="0">
-        <v>825.18</v>
+        <v>37527.35</v>
       </c>
     </row>
     <row r="181">
@@ -5775,7 +5781,7 @@
         <v>18</v>
       </c>
       <c r="D181" s="0">
-        <v>2850</v>
+        <v>825.18</v>
       </c>
     </row>
     <row r="182">
@@ -5789,7 +5795,7 @@
         <v>18</v>
       </c>
       <c r="D182" s="0">
-        <v>6384.84</v>
+        <v>2850</v>
       </c>
     </row>
     <row r="183">
@@ -5803,7 +5809,7 @@
         <v>18</v>
       </c>
       <c r="D183" s="0">
-        <v>333.17</v>
+        <v>6384.84</v>
       </c>
     </row>
     <row r="184">
@@ -5817,7 +5823,7 @@
         <v>18</v>
       </c>
       <c r="D184" s="0">
-        <v>9669.15</v>
+        <v>333.17</v>
       </c>
     </row>
     <row r="185">
@@ -5831,7 +5837,7 @@
         <v>18</v>
       </c>
       <c r="D185" s="0">
-        <v>3599.84</v>
+        <v>9669.15</v>
       </c>
     </row>
     <row r="186">
@@ -5845,7 +5851,7 @@
         <v>18</v>
       </c>
       <c r="D186" s="0">
-        <v>412.8</v>
+        <v>3599.84</v>
       </c>
     </row>
     <row r="187">
@@ -5859,7 +5865,7 @@
         <v>18</v>
       </c>
       <c r="D187" s="0">
-        <v>2015.52</v>
+        <v>412.8</v>
       </c>
     </row>
     <row r="188">
@@ -5870,10 +5876,10 @@
         <v>418</v>
       </c>
       <c r="C188" s="0" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="D188" s="0">
-        <v>9041.55</v>
+        <v>2015.52</v>
       </c>
     </row>
     <row r="189">
@@ -5884,10 +5890,10 @@
         <v>420</v>
       </c>
       <c r="C189" s="0" t="s">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="D189" s="0">
-        <v>430</v>
+        <v>9041.55</v>
       </c>
     </row>
     <row r="190">
@@ -5901,7 +5907,7 @@
         <v>70</v>
       </c>
       <c r="D190" s="0">
-        <v>800</v>
+        <v>430</v>
       </c>
     </row>
     <row r="191">
@@ -5912,10 +5918,10 @@
         <v>424</v>
       </c>
       <c r="C191" s="0" t="s">
-        <v>240</v>
+        <v>70</v>
       </c>
       <c r="D191" s="0">
-        <v>2280</v>
+        <v>800</v>
       </c>
     </row>
     <row r="192">
@@ -5929,7 +5935,7 @@
         <v>240</v>
       </c>
       <c r="D192" s="0">
-        <v>1620</v>
+        <v>2280</v>
       </c>
     </row>
     <row r="193">
@@ -5940,10 +5946,10 @@
         <v>428</v>
       </c>
       <c r="C193" s="0" t="s">
-        <v>372</v>
+        <v>240</v>
       </c>
       <c r="D193" s="0">
-        <v>236458.17</v>
+        <v>1620</v>
       </c>
     </row>
     <row r="194">
@@ -5954,10 +5960,10 @@
         <v>430</v>
       </c>
       <c r="C194" s="0" t="s">
-        <v>28</v>
+        <v>374</v>
       </c>
       <c r="D194" s="0">
-        <v>317.2</v>
+        <v>236458.17</v>
       </c>
     </row>
     <row r="195">
@@ -5968,10 +5974,10 @@
         <v>432</v>
       </c>
       <c r="C195" s="0" t="s">
-        <v>372</v>
+        <v>28</v>
       </c>
       <c r="D195" s="0">
-        <v>25100</v>
+        <v>317.2</v>
       </c>
     </row>
     <row r="196">
@@ -5982,24 +5988,24 @@
         <v>434</v>
       </c>
       <c r="C196" s="0" t="s">
-        <v>435</v>
+        <v>374</v>
       </c>
       <c r="D196" s="0">
-        <v>20900</v>
+        <v>25100</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="0" t="s">
+        <v>435</v>
+      </c>
+      <c r="B197" s="0" t="s">
         <v>436</v>
       </c>
-      <c r="B197" s="0" t="s">
+      <c r="C197" s="0" t="s">
         <v>437</v>
       </c>
-      <c r="C197" s="0" t="s">
-        <v>45</v>
-      </c>
       <c r="D197" s="0">
-        <v>4729.48</v>
+        <v>20900</v>
       </c>
     </row>
     <row r="198">
@@ -6010,10 +6016,10 @@
         <v>439</v>
       </c>
       <c r="C198" s="0" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="D198" s="0">
-        <v>1104.46</v>
+        <v>4729.48</v>
       </c>
     </row>
     <row r="199">
@@ -6024,10 +6030,10 @@
         <v>441</v>
       </c>
       <c r="C199" s="0" t="s">
-        <v>92</v>
+        <v>21</v>
       </c>
       <c r="D199" s="0">
-        <v>11646.25</v>
+        <v>1104.46</v>
       </c>
     </row>
     <row r="200">
@@ -6038,10 +6044,10 @@
         <v>443</v>
       </c>
       <c r="C200" s="0" t="s">
-        <v>121</v>
+        <v>92</v>
       </c>
       <c r="D200" s="0">
-        <v>6072</v>
+        <v>11646.25</v>
       </c>
     </row>
     <row r="201">
@@ -6052,10 +6058,10 @@
         <v>445</v>
       </c>
       <c r="C201" s="0" t="s">
-        <v>70</v>
+        <v>121</v>
       </c>
       <c r="D201" s="0">
-        <v>400</v>
+        <v>6072</v>
       </c>
     </row>
     <row r="202">
@@ -6066,10 +6072,10 @@
         <v>447</v>
       </c>
       <c r="C202" s="0" t="s">
-        <v>21</v>
+        <v>70</v>
       </c>
       <c r="D202" s="0">
-        <v>409</v>
+        <v>400</v>
       </c>
     </row>
     <row r="203">
@@ -6080,10 +6086,10 @@
         <v>449</v>
       </c>
       <c r="C203" s="0" t="s">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="D203" s="0">
-        <v>10748</v>
+        <v>409</v>
       </c>
     </row>
     <row r="204">
@@ -6097,7 +6103,7 @@
         <v>64</v>
       </c>
       <c r="D204" s="0">
-        <v>12898</v>
+        <v>10748</v>
       </c>
     </row>
     <row r="205">
@@ -6108,10 +6114,10 @@
         <v>453</v>
       </c>
       <c r="C205" s="0" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="D205" s="0">
-        <v>2000</v>
+        <v>12898</v>
       </c>
     </row>
     <row r="206">
@@ -6122,24 +6128,24 @@
         <v>455</v>
       </c>
       <c r="C206" s="0" t="s">
-        <v>456</v>
+        <v>52</v>
       </c>
       <c r="D206" s="0">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="0" t="s">
+        <v>456</v>
+      </c>
+      <c r="B207" s="0" t="s">
         <v>457</v>
       </c>
-      <c r="B207" s="0" t="s">
+      <c r="C207" s="0" t="s">
         <v>458</v>
       </c>
-      <c r="C207" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="D207" s="0">
-        <v>490</v>
+        <v>0</v>
       </c>
     </row>
     <row r="208">
@@ -6150,10 +6156,10 @@
         <v>460</v>
       </c>
       <c r="C208" s="0" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D208" s="0">
-        <v>0</v>
+        <v>490</v>
       </c>
     </row>
     <row r="209">
@@ -6164,10 +6170,10 @@
         <v>462</v>
       </c>
       <c r="C209" s="0" t="s">
-        <v>158</v>
+        <v>34</v>
       </c>
       <c r="D209" s="0">
-        <v>25171.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="210">
@@ -6178,24 +6184,24 @@
         <v>464</v>
       </c>
       <c r="C210" s="0" t="s">
-        <v>465</v>
+        <v>158</v>
       </c>
       <c r="D210" s="0">
-        <v>60630</v>
+        <v>25171.1</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="0" t="s">
+        <v>465</v>
+      </c>
+      <c r="B211" s="0" t="s">
         <v>466</v>
       </c>
-      <c r="B211" s="0" t="s">
+      <c r="C211" s="0" t="s">
         <v>467</v>
       </c>
-      <c r="C211" s="0" t="s">
-        <v>149</v>
-      </c>
       <c r="D211" s="0">
-        <v>1800</v>
+        <v>60630</v>
       </c>
     </row>
     <row r="212">
@@ -6206,10 +6212,10 @@
         <v>469</v>
       </c>
       <c r="C212" s="0" t="s">
-        <v>34</v>
+        <v>149</v>
       </c>
       <c r="D212" s="0">
-        <v>0</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="213">
@@ -6220,10 +6226,10 @@
         <v>471</v>
       </c>
       <c r="C213" s="0" t="s">
-        <v>138</v>
+        <v>34</v>
       </c>
       <c r="D213" s="0">
-        <v>492.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="214">
@@ -6234,24 +6240,24 @@
         <v>473</v>
       </c>
       <c r="C214" s="0" t="s">
-        <v>474</v>
+        <v>138</v>
       </c>
       <c r="D214" s="0">
-        <v>495</v>
+        <v>492.2</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="0" t="s">
+        <v>474</v>
+      </c>
+      <c r="B215" s="0" t="s">
         <v>475</v>
       </c>
-      <c r="B215" s="0" t="s">
+      <c r="C215" s="0" t="s">
         <v>476</v>
       </c>
-      <c r="C215" s="0" t="s">
-        <v>18</v>
-      </c>
       <c r="D215" s="0">
-        <v>1786</v>
+        <v>495</v>
       </c>
     </row>
     <row r="216">
@@ -6265,7 +6271,7 @@
         <v>18</v>
       </c>
       <c r="D216" s="0">
-        <v>4391.8</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="217">
@@ -6276,10 +6282,10 @@
         <v>480</v>
       </c>
       <c r="C217" s="0" t="s">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="D217" s="0">
-        <v>4700</v>
+        <v>4391.8</v>
       </c>
     </row>
     <row r="218">
@@ -6293,7 +6299,7 @@
         <v>52</v>
       </c>
       <c r="D218" s="0">
-        <v>4200</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="219">
@@ -6332,21 +6338,21 @@
         <v>488</v>
       </c>
       <c r="C221" s="0" t="s">
-        <v>489</v>
+        <v>52</v>
       </c>
       <c r="D221" s="0">
-        <v>265</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="0" t="s">
+        <v>489</v>
+      </c>
+      <c r="B222" s="0" t="s">
         <v>490</v>
       </c>
-      <c r="B222" s="0" t="s">
+      <c r="C222" s="0" t="s">
         <v>491</v>
-      </c>
-      <c r="C222" s="0" t="s">
-        <v>489</v>
       </c>
       <c r="D222" s="0">
         <v>265</v>
@@ -6360,7 +6366,7 @@
         <v>493</v>
       </c>
       <c r="C223" s="0" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="D223" s="0">
         <v>265</v>
@@ -6374,7 +6380,7 @@
         <v>495</v>
       </c>
       <c r="C224" s="0" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="D224" s="0">
         <v>265</v>
@@ -6388,7 +6394,7 @@
         <v>497</v>
       </c>
       <c r="C225" s="0" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="D225" s="0">
         <v>265</v>
@@ -6402,7 +6408,7 @@
         <v>499</v>
       </c>
       <c r="C226" s="0" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="D226" s="0">
         <v>265</v>
@@ -6416,21 +6422,21 @@
         <v>501</v>
       </c>
       <c r="C227" s="0" t="s">
-        <v>502</v>
+        <v>491</v>
       </c>
       <c r="D227" s="0">
-        <v>4700</v>
+        <v>265</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="0" t="s">
+        <v>502</v>
+      </c>
+      <c r="B228" s="0" t="s">
         <v>503</v>
       </c>
-      <c r="B228" s="0" t="s">
+      <c r="C228" s="0" t="s">
         <v>504</v>
-      </c>
-      <c r="C228" s="0" t="s">
-        <v>505</v>
       </c>
       <c r="D228" s="0">
         <v>4700</v>
@@ -6438,13 +6444,13 @@
     </row>
     <row r="229">
       <c r="A229" s="0" t="s">
+        <v>505</v>
+      </c>
+      <c r="B229" s="0" t="s">
         <v>506</v>
       </c>
-      <c r="B229" s="0" t="s">
+      <c r="C229" s="0" t="s">
         <v>507</v>
-      </c>
-      <c r="C229" s="0" t="s">
-        <v>52</v>
       </c>
       <c r="D229" s="0">
         <v>4700</v>
@@ -6461,7 +6467,7 @@
         <v>52</v>
       </c>
       <c r="D230" s="0">
-        <v>500</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="231">
@@ -6475,7 +6481,7 @@
         <v>52</v>
       </c>
       <c r="D231" s="0">
-        <v>210</v>
+        <v>500</v>
       </c>
     </row>
     <row r="232">
@@ -6489,7 +6495,7 @@
         <v>52</v>
       </c>
       <c r="D232" s="0">
-        <v>247</v>
+        <v>210</v>
       </c>
     </row>
     <row r="233">
@@ -6500,10 +6506,10 @@
         <v>515</v>
       </c>
       <c r="C233" s="0" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="D233" s="0">
-        <v>5600</v>
+        <v>247</v>
       </c>
     </row>
     <row r="234">
@@ -6514,10 +6520,10 @@
         <v>517</v>
       </c>
       <c r="C234" s="0" t="s">
-        <v>149</v>
+        <v>37</v>
       </c>
       <c r="D234" s="0">
-        <v>6000</v>
+        <v>5600</v>
       </c>
     </row>
     <row r="235">
@@ -6528,10 +6534,10 @@
         <v>519</v>
       </c>
       <c r="C235" s="0" t="s">
-        <v>70</v>
+        <v>149</v>
       </c>
       <c r="D235" s="0">
-        <v>80000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="236">
@@ -6545,7 +6551,7 @@
         <v>70</v>
       </c>
       <c r="D236" s="0">
-        <v>90000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="237">
@@ -6559,7 +6565,7 @@
         <v>70</v>
       </c>
       <c r="D237" s="0">
-        <v>110000</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="238">
@@ -6570,10 +6576,10 @@
         <v>525</v>
       </c>
       <c r="C238" s="0" t="s">
-        <v>15</v>
+        <v>70</v>
       </c>
       <c r="D238" s="0">
-        <v>1100</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="239">
@@ -6587,7 +6593,7 @@
         <v>15</v>
       </c>
       <c r="D239" s="0">
-        <v>2500</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="240">
@@ -6598,10 +6604,10 @@
         <v>529</v>
       </c>
       <c r="C240" s="0" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="D240" s="0">
-        <v>13636.84</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="241">
@@ -6612,10 +6618,10 @@
         <v>531</v>
       </c>
       <c r="C241" s="0" t="s">
-        <v>279</v>
+        <v>28</v>
       </c>
       <c r="D241" s="0">
-        <v>450</v>
+        <v>13636.84</v>
       </c>
     </row>
     <row r="242">
@@ -6626,10 +6632,10 @@
         <v>533</v>
       </c>
       <c r="C242" s="0" t="s">
-        <v>15</v>
+        <v>279</v>
       </c>
       <c r="D242" s="0">
-        <v>555</v>
+        <v>450</v>
       </c>
     </row>
     <row r="243">
@@ -6643,7 +6649,7 @@
         <v>15</v>
       </c>
       <c r="D243" s="0">
-        <v>825</v>
+        <v>555</v>
       </c>
     </row>
     <row r="244">
@@ -6657,7 +6663,7 @@
         <v>15</v>
       </c>
       <c r="D244" s="0">
-        <v>36.3</v>
+        <v>825</v>
       </c>
     </row>
     <row r="245">
@@ -6671,7 +6677,7 @@
         <v>15</v>
       </c>
       <c r="D245" s="0">
-        <v>544.5</v>
+        <v>36.3</v>
       </c>
     </row>
     <row r="246">
@@ -6685,7 +6691,7 @@
         <v>15</v>
       </c>
       <c r="D246" s="0">
-        <v>750</v>
+        <v>544.5</v>
       </c>
     </row>
     <row r="247">
@@ -6696,10 +6702,10 @@
         <v>543</v>
       </c>
       <c r="C247" s="0" t="s">
-        <v>149</v>
+        <v>15</v>
       </c>
       <c r="D247" s="0">
-        <v>1130</v>
+        <v>750</v>
       </c>
     </row>
     <row r="248">
@@ -6710,10 +6716,10 @@
         <v>545</v>
       </c>
       <c r="C248" s="0" t="s">
-        <v>52</v>
+        <v>149</v>
       </c>
       <c r="D248" s="0">
-        <v>4510</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="249">
@@ -6766,10 +6772,10 @@
         <v>553</v>
       </c>
       <c r="C252" s="0" t="s">
-        <v>15</v>
+        <v>52</v>
       </c>
       <c r="D252" s="0">
-        <v>902</v>
+        <v>4510</v>
       </c>
     </row>
     <row r="253">
@@ -6783,7 +6789,7 @@
         <v>15</v>
       </c>
       <c r="D253" s="0">
-        <v>880</v>
+        <v>902</v>
       </c>
     </row>
     <row r="254">
@@ -6794,10 +6800,10 @@
         <v>557</v>
       </c>
       <c r="C254" s="0" t="s">
-        <v>138</v>
+        <v>15</v>
       </c>
       <c r="D254" s="0">
-        <v>430</v>
+        <v>880</v>
       </c>
     </row>
     <row r="255">
@@ -6811,7 +6817,7 @@
         <v>138</v>
       </c>
       <c r="D255" s="0">
-        <v>354.54</v>
+        <v>430</v>
       </c>
     </row>
     <row r="256">
@@ -6822,10 +6828,10 @@
         <v>561</v>
       </c>
       <c r="C256" s="0" t="s">
-        <v>18</v>
+        <v>138</v>
       </c>
       <c r="D256" s="0">
-        <v>318.63</v>
+        <v>354.54</v>
       </c>
     </row>
     <row r="257">
@@ -6839,7 +6845,7 @@
         <v>18</v>
       </c>
       <c r="D257" s="0">
-        <v>415.15</v>
+        <v>318.63</v>
       </c>
     </row>
     <row r="258">
@@ -6853,7 +6859,7 @@
         <v>18</v>
       </c>
       <c r="D258" s="0">
-        <v>760</v>
+        <v>415.15</v>
       </c>
     </row>
     <row r="259">
@@ -6867,7 +6873,7 @@
         <v>18</v>
       </c>
       <c r="D259" s="0">
-        <v>820</v>
+        <v>760</v>
       </c>
     </row>
     <row r="260">
@@ -6878,24 +6884,24 @@
         <v>569</v>
       </c>
       <c r="C260" s="0" t="s">
-        <v>570</v>
+        <v>18</v>
       </c>
       <c r="D260" s="0">
-        <v>177940.1</v>
+        <v>820</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="0" t="s">
+        <v>570</v>
+      </c>
+      <c r="B261" s="0" t="s">
         <v>571</v>
       </c>
-      <c r="B261" s="0" t="s">
+      <c r="C261" s="0" t="s">
         <v>572</v>
       </c>
-      <c r="C261" s="0" t="s">
-        <v>70</v>
-      </c>
       <c r="D261" s="0">
-        <v>34000</v>
+        <v>177940.1</v>
       </c>
     </row>
     <row r="262">
@@ -6909,7 +6915,7 @@
         <v>70</v>
       </c>
       <c r="D262" s="0">
-        <v>30000</v>
+        <v>34000</v>
       </c>
     </row>
     <row r="263">
@@ -6920,10 +6926,10 @@
         <v>576</v>
       </c>
       <c r="C263" s="0" t="s">
-        <v>465</v>
+        <v>70</v>
       </c>
       <c r="D263" s="0">
-        <v>227939.52</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="264">
@@ -6934,10 +6940,10 @@
         <v>578</v>
       </c>
       <c r="C264" s="0" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="D264" s="0">
-        <v>184488.7</v>
+        <v>227939.52</v>
       </c>
     </row>
     <row r="265">
@@ -6948,10 +6954,10 @@
         <v>580</v>
       </c>
       <c r="C265" s="0" t="s">
-        <v>15</v>
+        <v>467</v>
       </c>
       <c r="D265" s="0">
-        <v>1760</v>
+        <v>184488.7</v>
       </c>
     </row>
     <row r="266">
@@ -6962,24 +6968,24 @@
         <v>582</v>
       </c>
       <c r="C266" s="0" t="s">
-        <v>583</v>
+        <v>15</v>
       </c>
       <c r="D266" s="0">
-        <v>26350</v>
+        <v>1760</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="0" t="s">
+        <v>583</v>
+      </c>
+      <c r="B267" s="0" t="s">
         <v>584</v>
       </c>
-      <c r="B267" s="0" t="s">
+      <c r="C267" s="0" t="s">
         <v>585</v>
       </c>
-      <c r="C267" s="0" t="s">
-        <v>474</v>
-      </c>
       <c r="D267" s="0">
-        <v>31250</v>
+        <v>26350</v>
       </c>
     </row>
     <row r="268">
@@ -6990,10 +6996,10 @@
         <v>587</v>
       </c>
       <c r="C268" s="0" t="s">
-        <v>52</v>
+        <v>476</v>
       </c>
       <c r="D268" s="0">
-        <v>34.98</v>
+        <v>31250</v>
       </c>
     </row>
     <row r="269">
@@ -7004,21 +7010,21 @@
         <v>589</v>
       </c>
       <c r="C269" s="0" t="s">
-        <v>590</v>
+        <v>52</v>
       </c>
       <c r="D269" s="0">
-        <v>65</v>
+        <v>34.98</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="0" t="s">
+        <v>590</v>
+      </c>
+      <c r="B270" s="0" t="s">
         <v>591</v>
       </c>
-      <c r="B270" s="0" t="s">
+      <c r="C270" s="0" t="s">
         <v>592</v>
-      </c>
-      <c r="C270" s="0" t="s">
-        <v>52</v>
       </c>
       <c r="D270" s="0">
         <v>65</v>
@@ -7035,7 +7041,7 @@
         <v>52</v>
       </c>
       <c r="D271" s="0">
-        <v>92</v>
+        <v>65</v>
       </c>
     </row>
     <row r="272">
@@ -7049,7 +7055,7 @@
         <v>52</v>
       </c>
       <c r="D272" s="0">
-        <v>33</v>
+        <v>92</v>
       </c>
     </row>
     <row r="273">
@@ -7063,7 +7069,7 @@
         <v>52</v>
       </c>
       <c r="D273" s="0">
-        <v>38.22</v>
+        <v>33</v>
       </c>
     </row>
     <row r="274">
@@ -7074,10 +7080,10 @@
         <v>600</v>
       </c>
       <c r="C274" s="0" t="s">
-        <v>334</v>
+        <v>52</v>
       </c>
       <c r="D274" s="0">
-        <v>300</v>
+        <v>38.22</v>
       </c>
     </row>
     <row r="275">
@@ -7088,10 +7094,10 @@
         <v>602</v>
       </c>
       <c r="C275" s="0" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="D275" s="0">
-        <v>370</v>
+        <v>300</v>
       </c>
     </row>
     <row r="276">
@@ -7102,10 +7108,10 @@
         <v>604</v>
       </c>
       <c r="C276" s="0" t="s">
-        <v>355</v>
+        <v>336</v>
       </c>
       <c r="D276" s="0">
-        <v>450</v>
+        <v>370</v>
       </c>
     </row>
     <row r="277">
@@ -7116,7 +7122,7 @@
         <v>606</v>
       </c>
       <c r="C277" s="0" t="s">
-        <v>37</v>
+        <v>357</v>
       </c>
       <c r="D277" s="0">
         <v>450</v>
@@ -7130,7 +7136,7 @@
         <v>608</v>
       </c>
       <c r="C278" s="0" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="D278" s="0">
         <v>450</v>
@@ -7147,7 +7153,7 @@
         <v>15</v>
       </c>
       <c r="D279" s="0">
-        <v>1650</v>
+        <v>450</v>
       </c>
     </row>
     <row r="280">
@@ -7161,7 +7167,7 @@
         <v>15</v>
       </c>
       <c r="D280" s="0">
-        <v>2100</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="281">
@@ -7175,7 +7181,7 @@
         <v>15</v>
       </c>
       <c r="D281" s="0">
-        <v>1980</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="282">
@@ -7189,7 +7195,7 @@
         <v>15</v>
       </c>
       <c r="D282" s="0">
-        <v>2160</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="283">
@@ -7203,7 +7209,7 @@
         <v>15</v>
       </c>
       <c r="D283" s="0">
-        <v>1500</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="284">
@@ -7217,7 +7223,7 @@
         <v>15</v>
       </c>
       <c r="D284" s="0">
-        <v>2600</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="285">
@@ -7231,7 +7237,7 @@
         <v>15</v>
       </c>
       <c r="D285" s="0">
-        <v>2000</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="286">
@@ -7245,7 +7251,7 @@
         <v>15</v>
       </c>
       <c r="D286" s="0">
-        <v>6700</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="287">
@@ -7259,7 +7265,7 @@
         <v>15</v>
       </c>
       <c r="D287" s="0">
-        <v>1650</v>
+        <v>6700</v>
       </c>
     </row>
     <row r="288">
@@ -7273,7 +7279,7 @@
         <v>15</v>
       </c>
       <c r="D288" s="0">
-        <v>1035</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="289">
@@ -7287,7 +7293,7 @@
         <v>15</v>
       </c>
       <c r="D289" s="0">
-        <v>2600</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="290">
@@ -7301,7 +7307,7 @@
         <v>15</v>
       </c>
       <c r="D290" s="0">
-        <v>2400</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="291">
@@ -7312,10 +7318,10 @@
         <v>634</v>
       </c>
       <c r="C291" s="0" t="s">
-        <v>138</v>
+        <v>15</v>
       </c>
       <c r="D291" s="0">
-        <v>4497.2</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="292">
@@ -7329,7 +7335,7 @@
         <v>138</v>
       </c>
       <c r="D292" s="0">
-        <v>2328</v>
+        <v>4497.2</v>
       </c>
     </row>
     <row r="293">
@@ -7343,7 +7349,7 @@
         <v>138</v>
       </c>
       <c r="D293" s="0">
-        <v>1138</v>
+        <v>2328</v>
       </c>
     </row>
     <row r="294">
@@ -7354,10 +7360,10 @@
         <v>640</v>
       </c>
       <c r="C294" s="0" t="s">
-        <v>28</v>
+        <v>138</v>
       </c>
       <c r="D294" s="0">
-        <v>7372.42</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="295">
@@ -7368,10 +7374,10 @@
         <v>642</v>
       </c>
       <c r="C295" s="0" t="s">
-        <v>121</v>
+        <v>28</v>
       </c>
       <c r="D295" s="0">
-        <v>1790</v>
+        <v>7372.42</v>
       </c>
     </row>
     <row r="296">
@@ -7385,7 +7391,7 @@
         <v>121</v>
       </c>
       <c r="D296" s="0">
-        <v>2859.96</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="297">
@@ -7399,7 +7405,7 @@
         <v>121</v>
       </c>
       <c r="D297" s="0">
-        <v>4800</v>
+        <v>2859.96</v>
       </c>
     </row>
     <row r="298">
@@ -7410,24 +7416,24 @@
         <v>648</v>
       </c>
       <c r="C298" s="0" t="s">
-        <v>649</v>
+        <v>121</v>
       </c>
       <c r="D298" s="0">
-        <v>0</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="0" t="s">
+        <v>649</v>
+      </c>
+      <c r="B299" s="0" t="s">
         <v>650</v>
       </c>
-      <c r="B299" s="0" t="s">
+      <c r="C299" s="0" t="s">
         <v>651</v>
       </c>
-      <c r="C299" s="0" t="s">
-        <v>28</v>
-      </c>
       <c r="D299" s="0">
-        <v>494</v>
+        <v>0</v>
       </c>
     </row>
     <row r="300">
@@ -7441,7 +7447,7 @@
         <v>28</v>
       </c>
       <c r="D300" s="0">
-        <v>665.3</v>
+        <v>494</v>
       </c>
     </row>
     <row r="301">
@@ -7452,10 +7458,10 @@
         <v>655</v>
       </c>
       <c r="C301" s="0" t="s">
-        <v>92</v>
+        <v>28</v>
       </c>
       <c r="D301" s="0">
-        <v>33940.5</v>
+        <v>665.3</v>
       </c>
     </row>
     <row r="302">
@@ -7469,7 +7475,7 @@
         <v>92</v>
       </c>
       <c r="D302" s="0">
-        <v>4525.4</v>
+        <v>33940.5</v>
       </c>
     </row>
     <row r="303">
@@ -7480,10 +7486,10 @@
         <v>659</v>
       </c>
       <c r="C303" s="0" t="s">
-        <v>149</v>
+        <v>92</v>
       </c>
       <c r="D303" s="0">
-        <v>896</v>
+        <v>4525.4</v>
       </c>
     </row>
     <row r="304">
@@ -7494,10 +7500,10 @@
         <v>661</v>
       </c>
       <c r="C304" s="0" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="D304" s="0">
-        <v>1250</v>
+        <v>896</v>
       </c>
     </row>
     <row r="305">
@@ -7508,10 +7514,10 @@
         <v>663</v>
       </c>
       <c r="C305" s="0" t="s">
-        <v>92</v>
+        <v>138</v>
       </c>
       <c r="D305" s="0">
-        <v>319440</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="306">
@@ -7522,10 +7528,10 @@
         <v>665</v>
       </c>
       <c r="C306" s="0" t="s">
-        <v>200</v>
+        <v>92</v>
       </c>
       <c r="D306" s="0">
-        <v>17440</v>
+        <v>319440</v>
       </c>
     </row>
     <row r="307">
@@ -7539,7 +7545,7 @@
         <v>200</v>
       </c>
       <c r="D307" s="0">
-        <v>4390</v>
+        <v>17440</v>
       </c>
     </row>
     <row r="308">
@@ -7564,10 +7570,10 @@
         <v>671</v>
       </c>
       <c r="C309" s="0" t="s">
-        <v>279</v>
+        <v>200</v>
       </c>
       <c r="D309" s="0">
-        <v>2250</v>
+        <v>4390</v>
       </c>
     </row>
     <row r="310">
@@ -7578,10 +7584,10 @@
         <v>673</v>
       </c>
       <c r="C310" s="0" t="s">
-        <v>200</v>
+        <v>279</v>
       </c>
       <c r="D310" s="0">
-        <v>3355</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="311">
@@ -7592,10 +7598,10 @@
         <v>675</v>
       </c>
       <c r="C311" s="0" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="D311" s="0">
-        <v>7500</v>
+        <v>3355</v>
       </c>
     </row>
     <row r="312">
@@ -7606,10 +7612,10 @@
         <v>677</v>
       </c>
       <c r="C312" s="0" t="s">
-        <v>92</v>
+        <v>205</v>
       </c>
       <c r="D312" s="0">
-        <v>25289</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="313">
@@ -7623,7 +7629,7 @@
         <v>92</v>
       </c>
       <c r="D313" s="0">
-        <v>252890</v>
+        <v>25289</v>
       </c>
     </row>
     <row r="314">
@@ -7634,10 +7640,10 @@
         <v>681</v>
       </c>
       <c r="C314" s="0" t="s">
-        <v>52</v>
+        <v>92</v>
       </c>
       <c r="D314" s="0">
-        <v>130</v>
+        <v>252890</v>
       </c>
     </row>
     <row r="315">
@@ -7648,10 +7654,10 @@
         <v>683</v>
       </c>
       <c r="C315" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="D315" s="0">
-        <v>285.6</v>
+        <v>130</v>
       </c>
     </row>
     <row r="316">
@@ -7665,7 +7671,7 @@
         <v>21</v>
       </c>
       <c r="D316" s="0">
-        <v>338</v>
+        <v>285.6</v>
       </c>
     </row>
     <row r="317">
@@ -7676,21 +7682,21 @@
         <v>687</v>
       </c>
       <c r="C317" s="0" t="s">
-        <v>688</v>
+        <v>21</v>
       </c>
       <c r="D317" s="0">
-        <v>770</v>
+        <v>338</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="0" t="s">
+        <v>688</v>
+      </c>
+      <c r="B318" s="0" t="s">
         <v>689</v>
       </c>
-      <c r="B318" s="0" t="s">
+      <c r="C318" s="0" t="s">
         <v>690</v>
-      </c>
-      <c r="C318" s="0" t="s">
-        <v>691</v>
       </c>
       <c r="D318" s="0">
         <v>770</v>
@@ -7698,16 +7704,16 @@
     </row>
     <row r="319">
       <c r="A319" s="0" t="s">
+        <v>691</v>
+      </c>
+      <c r="B319" s="0" t="s">
         <v>692</v>
       </c>
-      <c r="B319" s="0" t="s">
+      <c r="C319" s="0" t="s">
         <v>693</v>
       </c>
-      <c r="C319" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="D319" s="0">
-        <v>973.5</v>
+        <v>770</v>
       </c>
     </row>
     <row r="320">
@@ -7718,10 +7724,10 @@
         <v>695</v>
       </c>
       <c r="C320" s="0" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D320" s="0">
-        <v>507.08</v>
+        <v>973.5</v>
       </c>
     </row>
     <row r="321">
@@ -7732,10 +7738,10 @@
         <v>697</v>
       </c>
       <c r="C321" s="0" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D321" s="0">
-        <v>450</v>
+        <v>507.08</v>
       </c>
     </row>
     <row r="322">
@@ -7746,10 +7752,10 @@
         <v>699</v>
       </c>
       <c r="C322" s="0" t="s">
-        <v>149</v>
+        <v>15</v>
       </c>
       <c r="D322" s="0">
-        <v>760</v>
+        <v>450</v>
       </c>
     </row>
     <row r="323">
@@ -7760,10 +7766,10 @@
         <v>701</v>
       </c>
       <c r="C323" s="0" t="s">
-        <v>279</v>
+        <v>149</v>
       </c>
       <c r="D323" s="0">
-        <v>5900</v>
+        <v>760</v>
       </c>
     </row>
     <row r="324">
@@ -7777,7 +7783,7 @@
         <v>279</v>
       </c>
       <c r="D324" s="0">
-        <v>2900</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="325">
@@ -7788,10 +7794,10 @@
         <v>705</v>
       </c>
       <c r="C325" s="0" t="s">
-        <v>138</v>
+        <v>279</v>
       </c>
       <c r="D325" s="0">
-        <v>886.2</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="326">
@@ -7805,7 +7811,7 @@
         <v>138</v>
       </c>
       <c r="D326" s="0">
-        <v>589.9</v>
+        <v>886.2</v>
       </c>
     </row>
     <row r="327">
@@ -7819,7 +7825,7 @@
         <v>138</v>
       </c>
       <c r="D327" s="0">
-        <v>65</v>
+        <v>589.9</v>
       </c>
     </row>
     <row r="328">
@@ -7830,10 +7836,10 @@
         <v>711</v>
       </c>
       <c r="C328" s="0" t="s">
-        <v>92</v>
+        <v>138</v>
       </c>
       <c r="D328" s="0">
-        <v>11313.5</v>
+        <v>65</v>
       </c>
     </row>
     <row r="329">
@@ -7844,10 +7850,10 @@
         <v>713</v>
       </c>
       <c r="C329" s="0" t="s">
-        <v>34</v>
+        <v>92</v>
       </c>
       <c r="D329" s="0">
-        <v>420</v>
+        <v>11313.5</v>
       </c>
     </row>
     <row r="330">
@@ -7858,10 +7864,10 @@
         <v>715</v>
       </c>
       <c r="C330" s="0" t="s">
-        <v>355</v>
+        <v>34</v>
       </c>
       <c r="D330" s="0">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="331">
@@ -7872,10 +7878,10 @@
         <v>717</v>
       </c>
       <c r="C331" s="0" t="s">
-        <v>21</v>
+        <v>357</v>
       </c>
       <c r="D331" s="0">
-        <v>377</v>
+        <v>418</v>
       </c>
     </row>
     <row r="332">
@@ -7886,10 +7892,10 @@
         <v>719</v>
       </c>
       <c r="C332" s="0" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="D332" s="0">
-        <v>5780.66</v>
+        <v>377</v>
       </c>
     </row>
     <row r="333">
@@ -7900,10 +7906,10 @@
         <v>721</v>
       </c>
       <c r="C333" s="0" t="s">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="D333" s="0">
-        <v>898</v>
+        <v>5780.66</v>
       </c>
     </row>
     <row r="334">
@@ -7914,10 +7920,10 @@
         <v>723</v>
       </c>
       <c r="C334" s="0" t="s">
-        <v>121</v>
+        <v>70</v>
       </c>
       <c r="D334" s="0">
-        <v>4767</v>
+        <v>898</v>
       </c>
     </row>
     <row r="335">
@@ -7928,10 +7934,10 @@
         <v>725</v>
       </c>
       <c r="C335" s="0" t="s">
-        <v>34</v>
+        <v>121</v>
       </c>
       <c r="D335" s="0">
-        <v>650</v>
+        <v>4767</v>
       </c>
     </row>
     <row r="336">
@@ -7942,7 +7948,7 @@
         <v>727</v>
       </c>
       <c r="C336" s="0" t="s">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="D336" s="0">
         <v>650</v>
@@ -7956,10 +7962,10 @@
         <v>729</v>
       </c>
       <c r="C337" s="0" t="s">
-        <v>15</v>
+        <v>70</v>
       </c>
       <c r="D337" s="0">
-        <v>2178</v>
+        <v>650</v>
       </c>
     </row>
     <row r="338">
@@ -7970,10 +7976,10 @@
         <v>731</v>
       </c>
       <c r="C338" s="0" t="s">
-        <v>92</v>
+        <v>15</v>
       </c>
       <c r="D338" s="0">
-        <v>7986</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="339">
@@ -7984,24 +7990,24 @@
         <v>733</v>
       </c>
       <c r="C339" s="0" t="s">
-        <v>734</v>
+        <v>92</v>
       </c>
       <c r="D339" s="0">
-        <v>1910</v>
+        <v>7986</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="0" t="s">
+        <v>734</v>
+      </c>
+      <c r="B340" s="0" t="s">
         <v>735</v>
       </c>
-      <c r="B340" s="0" t="s">
+      <c r="C340" s="0" t="s">
         <v>736</v>
       </c>
-      <c r="C340" s="0" t="s">
-        <v>149</v>
-      </c>
       <c r="D340" s="0">
-        <v>900</v>
+        <v>1910</v>
       </c>
     </row>
     <row r="341">
@@ -8012,10 +8018,10 @@
         <v>738</v>
       </c>
       <c r="C341" s="0" t="s">
-        <v>21</v>
+        <v>149</v>
       </c>
       <c r="D341" s="0">
-        <v>1722</v>
+        <v>900</v>
       </c>
     </row>
     <row r="342">
@@ -8026,10 +8032,10 @@
         <v>740</v>
       </c>
       <c r="C342" s="0" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="D342" s="0">
-        <v>59000</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="343">
@@ -8040,10 +8046,10 @@
         <v>742</v>
       </c>
       <c r="C343" s="0" t="s">
-        <v>149</v>
+        <v>34</v>
       </c>
       <c r="D343" s="0">
-        <v>750</v>
+        <v>59000</v>
       </c>
     </row>
     <row r="344">
@@ -8057,7 +8063,7 @@
         <v>149</v>
       </c>
       <c r="D344" s="0">
-        <v>1212</v>
+        <v>750</v>
       </c>
     </row>
     <row r="345">
@@ -8071,7 +8077,7 @@
         <v>149</v>
       </c>
       <c r="D345" s="0">
-        <v>1300</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="346">
@@ -8085,7 +8091,7 @@
         <v>149</v>
       </c>
       <c r="D346" s="0">
-        <v>1500</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="347">
@@ -8099,7 +8105,7 @@
         <v>149</v>
       </c>
       <c r="D347" s="0">
-        <v>1400</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="348">
@@ -8110,10 +8116,10 @@
         <v>752</v>
       </c>
       <c r="C348" s="0" t="s">
-        <v>259</v>
+        <v>149</v>
       </c>
       <c r="D348" s="0">
-        <v>11959</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="349">
@@ -8124,10 +8130,10 @@
         <v>754</v>
       </c>
       <c r="C349" s="0" t="s">
-        <v>138</v>
+        <v>259</v>
       </c>
       <c r="D349" s="0">
-        <v>345</v>
+        <v>11959</v>
       </c>
     </row>
     <row r="350">
@@ -8138,10 +8144,10 @@
         <v>756</v>
       </c>
       <c r="C350" s="0" t="s">
-        <v>279</v>
+        <v>138</v>
       </c>
       <c r="D350" s="0">
-        <v>1450</v>
+        <v>345</v>
       </c>
     </row>
     <row r="351">
@@ -8152,10 +8158,10 @@
         <v>758</v>
       </c>
       <c r="C351" s="0" t="s">
-        <v>92</v>
+        <v>279</v>
       </c>
       <c r="D351" s="0">
-        <v>7320.5</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="352">
@@ -8166,10 +8172,10 @@
         <v>760</v>
       </c>
       <c r="C352" s="0" t="s">
-        <v>15</v>
+        <v>92</v>
       </c>
       <c r="D352" s="0">
-        <v>900</v>
+        <v>7320.5</v>
       </c>
     </row>
     <row r="353">
@@ -8180,10 +8186,10 @@
         <v>762</v>
       </c>
       <c r="C353" s="0" t="s">
-        <v>279</v>
+        <v>15</v>
       </c>
       <c r="D353" s="0">
-        <v>566</v>
+        <v>900</v>
       </c>
     </row>
     <row r="354">
@@ -8194,10 +8200,10 @@
         <v>764</v>
       </c>
       <c r="C354" s="0" t="s">
-        <v>465</v>
+        <v>279</v>
       </c>
       <c r="D354" s="0">
-        <v>64925</v>
+        <v>566</v>
       </c>
     </row>
     <row r="355">
@@ -8208,10 +8214,10 @@
         <v>766</v>
       </c>
       <c r="C355" s="0" t="s">
-        <v>15</v>
+        <v>467</v>
       </c>
       <c r="D355" s="0">
-        <v>1100</v>
+        <v>64925</v>
       </c>
     </row>
     <row r="356">
@@ -8222,10 +8228,10 @@
         <v>768</v>
       </c>
       <c r="C356" s="0" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D356" s="0">
-        <v>1623</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="357">
@@ -8236,10 +8242,10 @@
         <v>770</v>
       </c>
       <c r="C357" s="0" t="s">
-        <v>138</v>
+        <v>21</v>
       </c>
       <c r="D357" s="0">
-        <v>1182.75</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="358">
@@ -8253,7 +8259,7 @@
         <v>138</v>
       </c>
       <c r="D358" s="0">
-        <v>4440.9</v>
+        <v>1182.75</v>
       </c>
     </row>
     <row r="359">
@@ -8264,10 +8270,10 @@
         <v>774</v>
       </c>
       <c r="C359" s="0" t="s">
-        <v>28</v>
+        <v>138</v>
       </c>
       <c r="D359" s="0">
-        <v>1250</v>
+        <v>4440.9</v>
       </c>
     </row>
     <row r="360">
@@ -8281,7 +8287,7 @@
         <v>28</v>
       </c>
       <c r="D360" s="0">
-        <v>1945.1</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="361">
@@ -8292,10 +8298,10 @@
         <v>778</v>
       </c>
       <c r="C361" s="0" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="D361" s="0">
-        <v>450</v>
+        <v>1945.1</v>
       </c>
     </row>
     <row r="362">
@@ -8309,7 +8315,7 @@
         <v>15</v>
       </c>
       <c r="D362" s="0">
-        <v>825</v>
+        <v>450</v>
       </c>
     </row>
     <row r="363">
@@ -8334,10 +8340,10 @@
         <v>784</v>
       </c>
       <c r="C364" s="0" t="s">
-        <v>375</v>
+        <v>15</v>
       </c>
       <c r="D364" s="0">
-        <v>134775.6</v>
+        <v>825</v>
       </c>
     </row>
     <row r="365">
@@ -8348,10 +8354,10 @@
         <v>786</v>
       </c>
       <c r="C365" s="0" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="D365" s="0">
-        <v>175991.55</v>
+        <v>134775.6</v>
       </c>
     </row>
     <row r="366">
@@ -8362,10 +8368,10 @@
         <v>788</v>
       </c>
       <c r="C366" s="0" t="s">
-        <v>70</v>
+        <v>377</v>
       </c>
       <c r="D366" s="0">
-        <v>3263</v>
+        <v>175991.55</v>
       </c>
     </row>
     <row r="367">
@@ -8379,7 +8385,7 @@
         <v>70</v>
       </c>
       <c r="D367" s="0">
-        <v>18027</v>
+        <v>3263</v>
       </c>
     </row>
     <row r="368">
@@ -8390,10 +8396,10 @@
         <v>792</v>
       </c>
       <c r="C368" s="0" t="s">
-        <v>279</v>
+        <v>70</v>
       </c>
       <c r="D368" s="0">
-        <v>515</v>
+        <v>18027</v>
       </c>
     </row>
     <row r="369">
@@ -8404,7 +8410,7 @@
         <v>794</v>
       </c>
       <c r="C369" s="0" t="s">
-        <v>37</v>
+        <v>279</v>
       </c>
       <c r="D369" s="0">
         <v>515</v>
@@ -8418,10 +8424,10 @@
         <v>796</v>
       </c>
       <c r="C370" s="0" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="D370" s="0">
-        <v>9500</v>
+        <v>515</v>
       </c>
     </row>
     <row r="371">
@@ -8432,10 +8438,10 @@
         <v>798</v>
       </c>
       <c r="C371" s="0" t="s">
-        <v>465</v>
+        <v>52</v>
       </c>
       <c r="D371" s="0">
-        <v>207558.08</v>
+        <v>9500</v>
       </c>
     </row>
     <row r="372">
@@ -8446,10 +8452,10 @@
         <v>800</v>
       </c>
       <c r="C372" s="0" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="D372" s="0">
-        <v>249069.69</v>
+        <v>207558.08</v>
       </c>
     </row>
     <row r="373">
@@ -8460,10 +8466,10 @@
         <v>802</v>
       </c>
       <c r="C373" s="0" t="s">
-        <v>70</v>
+        <v>467</v>
       </c>
       <c r="D373" s="0">
-        <v>10021.22</v>
+        <v>249069.69</v>
       </c>
     </row>
     <row r="374">
@@ -8477,7 +8483,7 @@
         <v>70</v>
       </c>
       <c r="D374" s="0">
-        <v>17710</v>
+        <v>10021.22</v>
       </c>
     </row>
     <row r="375">
@@ -8488,24 +8494,24 @@
         <v>806</v>
       </c>
       <c r="C375" s="0" t="s">
-        <v>807</v>
+        <v>70</v>
       </c>
       <c r="D375" s="0">
-        <v>1080</v>
+        <v>17710</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="0" t="s">
+        <v>807</v>
+      </c>
+      <c r="B376" s="0" t="s">
         <v>808</v>
       </c>
-      <c r="B376" s="0" t="s">
+      <c r="C376" s="0" t="s">
         <v>809</v>
       </c>
-      <c r="C376" s="0" t="s">
-        <v>18</v>
-      </c>
       <c r="D376" s="0">
-        <v>569.39</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="377">
@@ -8516,24 +8522,24 @@
         <v>811</v>
       </c>
       <c r="C377" s="0" t="s">
-        <v>812</v>
+        <v>18</v>
       </c>
       <c r="D377" s="0">
-        <v>520</v>
+        <v>569.39</v>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="0" t="s">
+        <v>812</v>
+      </c>
+      <c r="B378" s="0" t="s">
         <v>813</v>
       </c>
-      <c r="B378" s="0" t="s">
+      <c r="C378" s="0" t="s">
         <v>814</v>
       </c>
-      <c r="C378" s="0" t="s">
-        <v>812</v>
-      </c>
       <c r="D378" s="0">
-        <v>300</v>
+        <v>520</v>
       </c>
     </row>
     <row r="379">
@@ -8544,10 +8550,10 @@
         <v>816</v>
       </c>
       <c r="C379" s="0" t="s">
-        <v>15</v>
+        <v>814</v>
       </c>
       <c r="D379" s="0">
-        <v>2200</v>
+        <v>300</v>
       </c>
     </row>
     <row r="380">
@@ -8561,7 +8567,7 @@
         <v>15</v>
       </c>
       <c r="D380" s="0">
-        <v>2800</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="381">
@@ -8572,10 +8578,10 @@
         <v>820</v>
       </c>
       <c r="C381" s="0" t="s">
-        <v>92</v>
+        <v>15</v>
       </c>
       <c r="D381" s="0">
-        <v>4924.7</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="382">
@@ -8586,10 +8592,10 @@
         <v>822</v>
       </c>
       <c r="C382" s="0" t="s">
-        <v>70</v>
+        <v>92</v>
       </c>
       <c r="D382" s="0">
-        <v>2699.64</v>
+        <v>4924.7</v>
       </c>
     </row>
     <row r="383">
@@ -8600,10 +8606,10 @@
         <v>824</v>
       </c>
       <c r="C383" s="0" t="s">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="D383" s="0">
-        <v>3800</v>
+        <v>2699.64</v>
       </c>
     </row>
     <row r="384">
@@ -8614,10 +8620,10 @@
         <v>826</v>
       </c>
       <c r="C384" s="0" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="D384" s="0">
-        <v>4000</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="385">
@@ -8628,24 +8634,24 @@
         <v>828</v>
       </c>
       <c r="C385" s="0" t="s">
-        <v>829</v>
+        <v>15</v>
       </c>
       <c r="D385" s="0">
-        <v>3800</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="386">
       <c r="A386" s="0" t="s">
+        <v>829</v>
+      </c>
+      <c r="B386" s="0" t="s">
         <v>830</v>
       </c>
-      <c r="B386" s="0" t="s">
+      <c r="C386" s="0" t="s">
         <v>831</v>
       </c>
-      <c r="C386" s="0" t="s">
-        <v>21</v>
-      </c>
       <c r="D386" s="0">
-        <v>353</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="387">
@@ -8656,10 +8662,10 @@
         <v>833</v>
       </c>
       <c r="C387" s="0" t="s">
-        <v>110</v>
+        <v>21</v>
       </c>
       <c r="D387" s="0">
-        <v>1800</v>
+        <v>353</v>
       </c>
     </row>
     <row r="388">
@@ -8670,10 +8676,10 @@
         <v>835</v>
       </c>
       <c r="C388" s="0" t="s">
-        <v>15</v>
+        <v>110</v>
       </c>
       <c r="D388" s="0">
-        <v>2948</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="389">
@@ -8684,10 +8690,10 @@
         <v>837</v>
       </c>
       <c r="C389" s="0" t="s">
-        <v>205</v>
+        <v>15</v>
       </c>
       <c r="D389" s="0">
-        <v>65537</v>
+        <v>2948</v>
       </c>
     </row>
     <row r="390">
@@ -8698,10 +8704,10 @@
         <v>839</v>
       </c>
       <c r="C390" s="0" t="s">
-        <v>138</v>
+        <v>205</v>
       </c>
       <c r="D390" s="0">
-        <v>4049.6</v>
+        <v>65537</v>
       </c>
     </row>
     <row r="391">
@@ -8715,7 +8721,7 @@
         <v>138</v>
       </c>
       <c r="D391" s="0">
-        <v>4199.2</v>
+        <v>4049.6</v>
       </c>
     </row>
     <row r="392">
@@ -8729,7 +8735,7 @@
         <v>138</v>
       </c>
       <c r="D392" s="0">
-        <v>6397.2</v>
+        <v>4199.2</v>
       </c>
     </row>
     <row r="393">
@@ -8740,10 +8746,10 @@
         <v>845</v>
       </c>
       <c r="C393" s="0" t="s">
-        <v>306</v>
+        <v>138</v>
       </c>
       <c r="D393" s="0">
-        <v>570</v>
+        <v>6397.2</v>
       </c>
     </row>
     <row r="394">
@@ -8754,10 +8760,10 @@
         <v>847</v>
       </c>
       <c r="C394" s="0" t="s">
-        <v>70</v>
+        <v>306</v>
       </c>
       <c r="D394" s="0">
-        <v>550</v>
+        <v>570</v>
       </c>
     </row>
     <row r="395">
@@ -8768,10 +8774,10 @@
         <v>849</v>
       </c>
       <c r="C395" s="0" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="D395" s="0">
-        <v>167</v>
+        <v>550</v>
       </c>
     </row>
     <row r="396">
@@ -8782,10 +8788,10 @@
         <v>851</v>
       </c>
       <c r="C396" s="0" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="D396" s="0">
-        <v>714.74</v>
+        <v>167</v>
       </c>
     </row>
     <row r="397">
@@ -8796,10 +8802,10 @@
         <v>853</v>
       </c>
       <c r="C397" s="0" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="D397" s="0">
-        <v>101000</v>
+        <v>714.74</v>
       </c>
     </row>
     <row r="398">
@@ -8810,10 +8816,10 @@
         <v>855</v>
       </c>
       <c r="C398" s="0" t="s">
-        <v>121</v>
+        <v>59</v>
       </c>
       <c r="D398" s="0">
-        <v>6251</v>
+        <v>101000</v>
       </c>
     </row>
     <row r="399">
@@ -8824,10 +8830,10 @@
         <v>857</v>
       </c>
       <c r="C399" s="0" t="s">
-        <v>372</v>
+        <v>121</v>
       </c>
       <c r="D399" s="0">
-        <v>857.67</v>
+        <v>6251</v>
       </c>
     </row>
     <row r="400">
@@ -8838,10 +8844,10 @@
         <v>859</v>
       </c>
       <c r="C400" s="0" t="s">
-        <v>92</v>
+        <v>374</v>
       </c>
       <c r="D400" s="0">
-        <v>1164.66</v>
+        <v>857.67</v>
       </c>
     </row>
     <row r="401">
@@ -8852,10 +8858,10 @@
         <v>861</v>
       </c>
       <c r="C401" s="0" t="s">
-        <v>149</v>
+        <v>92</v>
       </c>
       <c r="D401" s="0">
-        <v>360</v>
+        <v>1164.66</v>
       </c>
     </row>
     <row r="402">
@@ -8869,7 +8875,7 @@
         <v>149</v>
       </c>
       <c r="D402" s="0">
-        <v>450</v>
+        <v>360</v>
       </c>
     </row>
     <row r="403">
@@ -8883,7 +8889,7 @@
         <v>149</v>
       </c>
       <c r="D403" s="0">
-        <v>2150</v>
+        <v>450</v>
       </c>
     </row>
     <row r="404">
@@ -8894,10 +8900,10 @@
         <v>867</v>
       </c>
       <c r="C404" s="0" t="s">
-        <v>570</v>
+        <v>149</v>
       </c>
       <c r="D404" s="0">
-        <v>25192.82</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="405">
@@ -8908,10 +8914,10 @@
         <v>869</v>
       </c>
       <c r="C405" s="0" t="s">
-        <v>70</v>
+        <v>572</v>
       </c>
       <c r="D405" s="0">
-        <v>3500</v>
+        <v>25192.82</v>
       </c>
     </row>
     <row r="406">
@@ -8922,10 +8928,10 @@
         <v>871</v>
       </c>
       <c r="C406" s="0" t="s">
-        <v>173</v>
+        <v>70</v>
       </c>
       <c r="D406" s="0">
-        <v>600</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="407">
@@ -8936,24 +8942,24 @@
         <v>873</v>
       </c>
       <c r="C407" s="0" t="s">
-        <v>874</v>
+        <v>173</v>
       </c>
       <c r="D407" s="0">
-        <v>1080</v>
+        <v>600</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="0" t="s">
+        <v>874</v>
+      </c>
+      <c r="B408" s="0" t="s">
         <v>875</v>
       </c>
-      <c r="B408" s="0" t="s">
+      <c r="C408" s="0" t="s">
         <v>876</v>
       </c>
-      <c r="C408" s="0" t="s">
-        <v>334</v>
-      </c>
       <c r="D408" s="0">
-        <v>8628</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="409">
@@ -8964,10 +8970,10 @@
         <v>878</v>
       </c>
       <c r="C409" s="0" t="s">
-        <v>40</v>
+        <v>336</v>
       </c>
       <c r="D409" s="0">
-        <v>27991.54</v>
+        <v>8628</v>
       </c>
     </row>
     <row r="410">
@@ -8978,10 +8984,10 @@
         <v>880</v>
       </c>
       <c r="C410" s="0" t="s">
-        <v>138</v>
+        <v>40</v>
       </c>
       <c r="D410" s="0">
-        <v>1080</v>
+        <v>27991.54</v>
       </c>
     </row>
     <row r="411">
@@ -8995,7 +9001,7 @@
         <v>138</v>
       </c>
       <c r="D411" s="0">
-        <v>4012</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="412">
@@ -9006,10 +9012,10 @@
         <v>884</v>
       </c>
       <c r="C412" s="0" t="s">
-        <v>45</v>
+        <v>138</v>
       </c>
       <c r="D412" s="0">
-        <v>6344.43</v>
+        <v>4012</v>
       </c>
     </row>
     <row r="413">
@@ -9023,7 +9029,7 @@
         <v>45</v>
       </c>
       <c r="D413" s="0">
-        <v>2862.28</v>
+        <v>6344.43</v>
       </c>
     </row>
     <row r="414">
@@ -9037,7 +9043,7 @@
         <v>45</v>
       </c>
       <c r="D414" s="0">
-        <v>2131.18</v>
+        <v>2862.28</v>
       </c>
     </row>
     <row r="415">
@@ -9051,7 +9057,7 @@
         <v>45</v>
       </c>
       <c r="D415" s="0">
-        <v>29795.68</v>
+        <v>2131.18</v>
       </c>
     </row>
     <row r="416">
@@ -9065,7 +9071,7 @@
         <v>45</v>
       </c>
       <c r="D416" s="0">
-        <v>2307.09</v>
+        <v>29795.68</v>
       </c>
     </row>
     <row r="417">
@@ -9079,7 +9085,7 @@
         <v>45</v>
       </c>
       <c r="D417" s="0">
-        <v>5249.48</v>
+        <v>2307.09</v>
       </c>
     </row>
     <row r="418">
@@ -9093,7 +9099,7 @@
         <v>45</v>
       </c>
       <c r="D418" s="0">
-        <v>4399.56</v>
+        <v>5249.48</v>
       </c>
     </row>
     <row r="419">
@@ -9104,10 +9110,10 @@
         <v>898</v>
       </c>
       <c r="C419" s="0" t="s">
-        <v>474</v>
+        <v>45</v>
       </c>
       <c r="D419" s="0">
-        <v>510</v>
+        <v>4399.56</v>
       </c>
     </row>
     <row r="420">
@@ -9118,7 +9124,7 @@
         <v>900</v>
       </c>
       <c r="C420" s="0" t="s">
-        <v>37</v>
+        <v>476</v>
       </c>
       <c r="D420" s="0">
         <v>510</v>
@@ -9132,21 +9138,21 @@
         <v>902</v>
       </c>
       <c r="C421" s="0" t="s">
-        <v>903</v>
+        <v>37</v>
       </c>
       <c r="D421" s="0">
-        <v>580</v>
+        <v>510</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="0" t="s">
+        <v>903</v>
+      </c>
+      <c r="B422" s="0" t="s">
         <v>904</v>
       </c>
-      <c r="B422" s="0" t="s">
+      <c r="C422" s="0" t="s">
         <v>905</v>
-      </c>
-      <c r="C422" s="0" t="s">
-        <v>903</v>
       </c>
       <c r="D422" s="0">
         <v>580</v>
@@ -9160,7 +9166,7 @@
         <v>907</v>
       </c>
       <c r="C423" s="0" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="D423" s="0">
         <v>580</v>
@@ -9174,10 +9180,10 @@
         <v>909</v>
       </c>
       <c r="C424" s="0" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="D424" s="0">
-        <v>342</v>
+        <v>580</v>
       </c>
     </row>
     <row r="425">
@@ -9188,7 +9194,7 @@
         <v>911</v>
       </c>
       <c r="C425" s="0" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="D425" s="0">
         <v>342</v>
@@ -9202,7 +9208,7 @@
         <v>913</v>
       </c>
       <c r="C426" s="0" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="D426" s="0">
         <v>342</v>
@@ -9216,10 +9222,10 @@
         <v>915</v>
       </c>
       <c r="C427" s="0" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="D427" s="0">
-        <v>0</v>
+        <v>342</v>
       </c>
     </row>
     <row r="428">
@@ -9230,7 +9236,7 @@
         <v>917</v>
       </c>
       <c r="C428" s="0" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="D428" s="0">
         <v>0</v>
@@ -9244,21 +9250,21 @@
         <v>919</v>
       </c>
       <c r="C429" s="0" t="s">
-        <v>920</v>
+        <v>905</v>
       </c>
       <c r="D429" s="0">
-        <v>453</v>
+        <v>0</v>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="0" t="s">
+        <v>920</v>
+      </c>
+      <c r="B430" s="0" t="s">
         <v>921</v>
       </c>
-      <c r="B430" s="0" t="s">
+      <c r="C430" s="0" t="s">
         <v>922</v>
-      </c>
-      <c r="C430" s="0" t="s">
-        <v>903</v>
       </c>
       <c r="D430" s="0">
         <v>453</v>
@@ -9272,10 +9278,10 @@
         <v>924</v>
       </c>
       <c r="C431" s="0" t="s">
-        <v>70</v>
+        <v>905</v>
       </c>
       <c r="D431" s="0">
-        <v>15968</v>
+        <v>453</v>
       </c>
     </row>
     <row r="432">
@@ -9286,10 +9292,10 @@
         <v>926</v>
       </c>
       <c r="C432" s="0" t="s">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="D432" s="0">
-        <v>430</v>
+        <v>15968</v>
       </c>
     </row>
     <row r="433">
@@ -9300,7 +9306,7 @@
         <v>928</v>
       </c>
       <c r="C433" s="0" t="s">
-        <v>279</v>
+        <v>34</v>
       </c>
       <c r="D433" s="0">
         <v>430</v>
@@ -9314,10 +9320,10 @@
         <v>930</v>
       </c>
       <c r="C434" s="0" t="s">
-        <v>115</v>
+        <v>279</v>
       </c>
       <c r="D434" s="0">
-        <v>14000</v>
+        <v>430</v>
       </c>
     </row>
     <row r="435">
@@ -9328,10 +9334,10 @@
         <v>932</v>
       </c>
       <c r="C435" s="0" t="s">
-        <v>138</v>
+        <v>115</v>
       </c>
       <c r="D435" s="0">
-        <v>14001</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="436">
@@ -9342,10 +9348,10 @@
         <v>934</v>
       </c>
       <c r="C436" s="0" t="s">
-        <v>92</v>
+        <v>138</v>
       </c>
       <c r="D436" s="0">
-        <v>266200</v>
+        <v>14001</v>
       </c>
     </row>
     <row r="437">
@@ -9359,7 +9365,7 @@
         <v>92</v>
       </c>
       <c r="D437" s="0">
-        <v>194991.5</v>
+        <v>266200</v>
       </c>
     </row>
     <row r="438">
@@ -9373,7 +9379,7 @@
         <v>92</v>
       </c>
       <c r="D438" s="0">
-        <v>289492.5</v>
+        <v>194991.5</v>
       </c>
     </row>
     <row r="439">
@@ -9384,24 +9390,24 @@
         <v>940</v>
       </c>
       <c r="C439" s="0" t="s">
-        <v>941</v>
+        <v>92</v>
       </c>
       <c r="D439" s="0">
-        <v>13722.52</v>
+        <v>289492.5</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="0" t="s">
+        <v>941</v>
+      </c>
+      <c r="B440" s="0" t="s">
         <v>942</v>
       </c>
-      <c r="B440" s="0" t="s">
+      <c r="C440" s="0" t="s">
         <v>943</v>
       </c>
-      <c r="C440" s="0" t="s">
-        <v>941</v>
-      </c>
       <c r="D440" s="0">
-        <v>15072</v>
+        <v>13722.52</v>
       </c>
     </row>
     <row r="441">
@@ -9412,10 +9418,10 @@
         <v>945</v>
       </c>
       <c r="C441" s="0" t="s">
-        <v>941</v>
+        <v>943</v>
       </c>
       <c r="D441" s="0">
-        <v>6555.64</v>
+        <v>15072</v>
       </c>
     </row>
     <row r="442">
@@ -9426,10 +9432,10 @@
         <v>947</v>
       </c>
       <c r="C442" s="0" t="s">
-        <v>941</v>
+        <v>943</v>
       </c>
       <c r="D442" s="0">
-        <v>8964.61</v>
+        <v>6555.64</v>
       </c>
     </row>
     <row r="443">
@@ -9440,10 +9446,10 @@
         <v>949</v>
       </c>
       <c r="C443" s="0" t="s">
-        <v>941</v>
+        <v>943</v>
       </c>
       <c r="D443" s="0">
-        <v>11735</v>
+        <v>8964.61</v>
       </c>
     </row>
     <row r="444">
@@ -9454,10 +9460,10 @@
         <v>951</v>
       </c>
       <c r="C444" s="0" t="s">
-        <v>70</v>
+        <v>943</v>
       </c>
       <c r="D444" s="0">
-        <v>3380</v>
+        <v>11735</v>
       </c>
     </row>
     <row r="445">
@@ -9468,10 +9474,10 @@
         <v>953</v>
       </c>
       <c r="C445" s="0" t="s">
-        <v>138</v>
+        <v>70</v>
       </c>
       <c r="D445" s="0">
-        <v>3750</v>
+        <v>3380</v>
       </c>
     </row>
     <row r="446">
@@ -9482,10 +9488,10 @@
         <v>955</v>
       </c>
       <c r="C446" s="0" t="s">
-        <v>92</v>
+        <v>138</v>
       </c>
       <c r="D446" s="0">
-        <v>4392.3</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="447">
@@ -9496,24 +9502,24 @@
         <v>957</v>
       </c>
       <c r="C447" s="0" t="s">
-        <v>958</v>
+        <v>92</v>
       </c>
       <c r="D447" s="0">
-        <v>5254.41</v>
+        <v>4392.3</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="0" t="s">
+        <v>958</v>
+      </c>
+      <c r="B448" s="0" t="s">
         <v>959</v>
       </c>
-      <c r="B448" s="0" t="s">
+      <c r="C448" s="0" t="s">
         <v>960</v>
       </c>
-      <c r="C448" s="0" t="s">
-        <v>52</v>
-      </c>
       <c r="D448" s="0">
-        <v>1200</v>
+        <v>5254.41</v>
       </c>
     </row>
     <row r="449">
@@ -9527,7 +9533,7 @@
         <v>52</v>
       </c>
       <c r="D449" s="0">
-        <v>278</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="450">
@@ -9541,7 +9547,7 @@
         <v>52</v>
       </c>
       <c r="D450" s="0">
-        <v>562</v>
+        <v>278</v>
       </c>
     </row>
     <row r="451">
@@ -9552,10 +9558,10 @@
         <v>966</v>
       </c>
       <c r="C451" s="0" t="s">
-        <v>372</v>
+        <v>52</v>
       </c>
       <c r="D451" s="0">
-        <v>65142.6</v>
+        <v>562</v>
       </c>
     </row>
     <row r="452">
@@ -9566,10 +9572,10 @@
         <v>968</v>
       </c>
       <c r="C452" s="0" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="D452" s="0">
-        <v>23482.7</v>
+        <v>65142.6</v>
       </c>
     </row>
     <row r="453">
@@ -9580,10 +9586,10 @@
         <v>970</v>
       </c>
       <c r="C453" s="0" t="s">
-        <v>28</v>
+        <v>374</v>
       </c>
       <c r="D453" s="0">
-        <v>6029.59</v>
+        <v>23482.7</v>
       </c>
     </row>
     <row r="454">
@@ -9594,10 +9600,10 @@
         <v>972</v>
       </c>
       <c r="C454" s="0" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="D454" s="0">
-        <v>10985</v>
+        <v>6029.59</v>
       </c>
     </row>
     <row r="455">
@@ -9611,7 +9617,7 @@
         <v>52</v>
       </c>
       <c r="D455" s="0">
-        <v>17425</v>
+        <v>10985</v>
       </c>
     </row>
     <row r="456">
@@ -9622,52 +9628,52 @@
         <v>976</v>
       </c>
       <c r="C456" s="0" t="s">
-        <v>977</v>
+        <v>52</v>
       </c>
       <c r="D456" s="0">
-        <v>1958</v>
+        <v>17425</v>
       </c>
     </row>
     <row r="457">
       <c r="A457" s="0" t="s">
+        <v>977</v>
+      </c>
+      <c r="B457" s="0" t="s">
         <v>978</v>
       </c>
-      <c r="B457" s="0" t="s">
+      <c r="C457" s="0" t="s">
         <v>979</v>
       </c>
-      <c r="C457" s="0" t="s">
-        <v>980</v>
-      </c>
       <c r="D457" s="0">
-        <v>2282.3</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="0" t="s">
+        <v>980</v>
+      </c>
+      <c r="B458" s="0" t="s">
         <v>981</v>
       </c>
-      <c r="B458" s="0" t="s">
+      <c r="C458" s="0" t="s">
         <v>982</v>
       </c>
-      <c r="C458" s="0" t="s">
-        <v>983</v>
-      </c>
       <c r="D458" s="0">
-        <v>385.4</v>
+        <v>2282.3</v>
       </c>
     </row>
     <row r="459">
       <c r="A459" s="0" t="s">
+        <v>983</v>
+      </c>
+      <c r="B459" s="0" t="s">
         <v>984</v>
       </c>
-      <c r="B459" s="0" t="s">
+      <c r="C459" s="0" t="s">
         <v>985</v>
       </c>
-      <c r="C459" s="0" t="s">
-        <v>92</v>
-      </c>
       <c r="D459" s="0">
-        <v>296147.5</v>
+        <v>385.4</v>
       </c>
     </row>
     <row r="460">
@@ -9678,10 +9684,10 @@
         <v>987</v>
       </c>
       <c r="C460" s="0" t="s">
-        <v>570</v>
+        <v>92</v>
       </c>
       <c r="D460" s="0">
-        <v>71176.4</v>
+        <v>296147.5</v>
       </c>
     </row>
     <row r="461">
@@ -9692,10 +9698,10 @@
         <v>989</v>
       </c>
       <c r="C461" s="0" t="s">
-        <v>138</v>
+        <v>572</v>
       </c>
       <c r="D461" s="0">
-        <v>96</v>
+        <v>71176.4</v>
       </c>
     </row>
     <row r="462">
@@ -9706,10 +9712,10 @@
         <v>991</v>
       </c>
       <c r="C462" s="0" t="s">
-        <v>70</v>
+        <v>138</v>
       </c>
       <c r="D462" s="0">
-        <v>950</v>
+        <v>96</v>
       </c>
     </row>
     <row r="463">
@@ -9720,10 +9726,10 @@
         <v>993</v>
       </c>
       <c r="C463" s="0" t="s">
-        <v>465</v>
+        <v>70</v>
       </c>
       <c r="D463" s="0">
-        <v>342641</v>
+        <v>950</v>
       </c>
     </row>
     <row r="464">
@@ -9734,10 +9740,10 @@
         <v>995</v>
       </c>
       <c r="C464" s="0" t="s">
-        <v>158</v>
+        <v>467</v>
       </c>
       <c r="D464" s="0">
-        <v>2200</v>
+        <v>342641</v>
       </c>
     </row>
     <row r="465">
@@ -9748,10 +9754,10 @@
         <v>997</v>
       </c>
       <c r="C465" s="0" t="s">
-        <v>474</v>
+        <v>158</v>
       </c>
       <c r="D465" s="0">
-        <v>41000</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="466">
@@ -9762,10 +9768,10 @@
         <v>999</v>
       </c>
       <c r="C466" s="0" t="s">
-        <v>70</v>
+        <v>476</v>
       </c>
       <c r="D466" s="0">
-        <v>9299</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="467">
@@ -9776,10 +9782,10 @@
         <v>1001</v>
       </c>
       <c r="C467" s="0" t="s">
-        <v>903</v>
+        <v>70</v>
       </c>
       <c r="D467" s="0">
-        <v>880</v>
+        <v>9299</v>
       </c>
     </row>
     <row r="468">
@@ -9790,7 +9796,7 @@
         <v>1003</v>
       </c>
       <c r="C468" s="0" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="D468" s="0">
         <v>880</v>
@@ -9804,7 +9810,7 @@
         <v>1005</v>
       </c>
       <c r="C469" s="0" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="D469" s="0">
         <v>880</v>
@@ -9818,10 +9824,10 @@
         <v>1007</v>
       </c>
       <c r="C470" s="0" t="s">
-        <v>21</v>
+        <v>905</v>
       </c>
       <c r="D470" s="0">
-        <v>563.36</v>
+        <v>880</v>
       </c>
     </row>
     <row r="471">
@@ -9832,10 +9838,10 @@
         <v>1009</v>
       </c>
       <c r="C471" s="0" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D471" s="0">
-        <v>3520</v>
+        <v>563.36</v>
       </c>
     </row>
     <row r="472">
@@ -9849,7 +9855,7 @@
         <v>15</v>
       </c>
       <c r="D472" s="0">
-        <v>2600</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="473">
@@ -9860,10 +9866,10 @@
         <v>1013</v>
       </c>
       <c r="C473" s="0" t="s">
-        <v>279</v>
+        <v>15</v>
       </c>
       <c r="D473" s="0">
-        <v>3700</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="474">
@@ -9877,7 +9883,7 @@
         <v>279</v>
       </c>
       <c r="D474" s="0">
-        <v>2600</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="475">
@@ -9888,10 +9894,10 @@
         <v>1017</v>
       </c>
       <c r="C475" s="0" t="s">
-        <v>15</v>
+        <v>279</v>
       </c>
       <c r="D475" s="0">
-        <v>2235</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="476">
@@ -9905,7 +9911,7 @@
         <v>15</v>
       </c>
       <c r="D476" s="0">
-        <v>3850</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="477">
@@ -9916,24 +9922,24 @@
         <v>1021</v>
       </c>
       <c r="C477" s="0" t="s">
-        <v>1022</v>
+        <v>15</v>
       </c>
       <c r="D477" s="0">
-        <v>1</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="478">
       <c r="A478" s="0" t="s">
+        <v>1022</v>
+      </c>
+      <c r="B478" s="0" t="s">
         <v>1023</v>
       </c>
-      <c r="B478" s="0" t="s">
+      <c r="C478" s="0" t="s">
         <v>1024</v>
       </c>
-      <c r="C478" s="0" t="s">
-        <v>28</v>
-      </c>
       <c r="D478" s="0">
-        <v>14819</v>
+        <v>1</v>
       </c>
     </row>
     <row r="479">
@@ -9944,10 +9950,10 @@
         <v>1026</v>
       </c>
       <c r="C479" s="0" t="s">
-        <v>372</v>
+        <v>28</v>
       </c>
       <c r="D479" s="0">
-        <v>3859.93</v>
+        <v>14819</v>
       </c>
     </row>
     <row r="480">
@@ -9958,10 +9964,10 @@
         <v>1028</v>
       </c>
       <c r="C480" s="0" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="D480" s="0">
-        <v>11751.49</v>
+        <v>3859.93</v>
       </c>
     </row>
     <row r="481">
@@ -9972,10 +9978,10 @@
         <v>1030</v>
       </c>
       <c r="C481" s="0" t="s">
-        <v>334</v>
+        <v>374</v>
       </c>
       <c r="D481" s="0">
-        <v>6000</v>
+        <v>11751.49</v>
       </c>
     </row>
     <row r="482">
@@ -9986,10 +9992,10 @@
         <v>1032</v>
       </c>
       <c r="C482" s="0" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="D482" s="0">
-        <v>3000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="483">
@@ -10000,10 +10006,10 @@
         <v>1034</v>
       </c>
       <c r="C483" s="0" t="s">
-        <v>37</v>
+        <v>336</v>
       </c>
       <c r="D483" s="0">
-        <v>618</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="484">
@@ -10014,24 +10020,24 @@
         <v>1036</v>
       </c>
       <c r="C484" s="0" t="s">
-        <v>1037</v>
+        <v>37</v>
       </c>
       <c r="D484" s="0">
-        <v>24600</v>
+        <v>618</v>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="0" t="s">
+        <v>1037</v>
+      </c>
+      <c r="B485" s="0" t="s">
         <v>1038</v>
       </c>
-      <c r="B485" s="0" t="s">
+      <c r="C485" s="0" t="s">
         <v>1039</v>
       </c>
-      <c r="C485" s="0" t="s">
-        <v>105</v>
-      </c>
       <c r="D485" s="0">
-        <v>0</v>
+        <v>24600</v>
       </c>
     </row>
     <row r="486">
@@ -10042,10 +10048,10 @@
         <v>1041</v>
       </c>
       <c r="C486" s="0" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="D486" s="0">
-        <v>41593.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="487">
@@ -10056,10 +10062,10 @@
         <v>1043</v>
       </c>
       <c r="C487" s="0" t="s">
-        <v>465</v>
+        <v>92</v>
       </c>
       <c r="D487" s="0">
-        <v>207558.07</v>
+        <v>41593.75</v>
       </c>
     </row>
     <row r="488">
@@ -10070,10 +10076,10 @@
         <v>1045</v>
       </c>
       <c r="C488" s="0" t="s">
-        <v>372</v>
+        <v>467</v>
       </c>
       <c r="D488" s="0">
-        <v>77429.29</v>
+        <v>207558.07</v>
       </c>
     </row>
     <row r="489">
@@ -10084,10 +10090,10 @@
         <v>1047</v>
       </c>
       <c r="C489" s="0" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="D489" s="0">
-        <v>42913.42</v>
+        <v>77429.29</v>
       </c>
     </row>
     <row r="490">
@@ -10098,10 +10104,10 @@
         <v>1049</v>
       </c>
       <c r="C490" s="0" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="D490" s="0">
-        <v>88806.25</v>
+        <v>42913.42</v>
       </c>
     </row>
     <row r="491">
@@ -10112,10 +10118,10 @@
         <v>1051</v>
       </c>
       <c r="C491" s="0" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="D491" s="0">
-        <v>50781.52</v>
+        <v>88806.25</v>
       </c>
     </row>
     <row r="492">
@@ -10126,10 +10132,10 @@
         <v>1053</v>
       </c>
       <c r="C492" s="0" t="s">
-        <v>21</v>
+        <v>374</v>
       </c>
       <c r="D492" s="0">
-        <v>1600</v>
+        <v>50781.52</v>
       </c>
     </row>
     <row r="493">
@@ -10140,10 +10146,10 @@
         <v>1055</v>
       </c>
       <c r="C493" s="0" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D493" s="0">
-        <v>3455.8</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="494">
@@ -10157,7 +10163,7 @@
         <v>28</v>
       </c>
       <c r="D494" s="0">
-        <v>3987</v>
+        <v>3455.8</v>
       </c>
     </row>
     <row r="495">
@@ -10171,7 +10177,7 @@
         <v>28</v>
       </c>
       <c r="D495" s="0">
-        <v>4010.17</v>
+        <v>3987</v>
       </c>
     </row>
     <row r="496">
@@ -10185,7 +10191,7 @@
         <v>28</v>
       </c>
       <c r="D496" s="0">
-        <v>3382.65</v>
+        <v>4010.17</v>
       </c>
     </row>
     <row r="497">
@@ -10196,10 +10202,10 @@
         <v>1063</v>
       </c>
       <c r="C497" s="0" t="s">
-        <v>158</v>
+        <v>28</v>
       </c>
       <c r="D497" s="0">
-        <v>430</v>
+        <v>3382.65</v>
       </c>
     </row>
     <row r="498">
@@ -10210,9 +10216,23 @@
         <v>1065</v>
       </c>
       <c r="C498" s="0" t="s">
+        <v>158</v>
+      </c>
+      <c r="D498" s="0">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="0" t="s">
+        <v>1066</v>
+      </c>
+      <c r="B499" s="0" t="s">
+        <v>1067</v>
+      </c>
+      <c r="C499" s="0" t="s">
         <v>138</v>
       </c>
-      <c r="D498" s="0">
+      <c r="D499" s="0">
         <v>462</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: lista de precios actualizada (test de embarazo ALL-TEST Iraola)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="1074">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1077" uniqueCount="1077">
   <si>
     <t>Solo Activos</t>
   </si>
@@ -2979,6 +2979,15 @@
   </si>
   <si>
     <t>MICROLIFE</t>
+  </si>
+  <si>
+    <t>000024697</t>
+  </si>
+  <si>
+    <t>TEST DE EMBARAZO ALL-TEST IRAOLA X 1 - - 000024697</t>
+  </si>
+  <si>
+    <t>IRAOLA</t>
   </si>
   <si>
     <t>000024688</t>
@@ -3299,7 +3308,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:D502"/>
+  <dimension ref="A2:D503"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -9733,7 +9742,7 @@
         <v>991</v>
       </c>
       <c r="D462" s="0">
-        <v>385.4</v>
+        <v>386</v>
       </c>
     </row>
     <row r="463">
@@ -9744,130 +9753,130 @@
         <v>993</v>
       </c>
       <c r="C463" s="0" t="s">
-        <v>92</v>
+        <v>994</v>
       </c>
       <c r="D463" s="0">
-        <v>296147.5</v>
+        <v>385.4</v>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="0" t="s">
-        <v>994</v>
+        <v>995</v>
       </c>
       <c r="B464" s="0" t="s">
-        <v>995</v>
+        <v>996</v>
       </c>
       <c r="C464" s="0" t="s">
-        <v>576</v>
+        <v>92</v>
       </c>
       <c r="D464" s="0">
-        <v>71176.4</v>
+        <v>296147.5</v>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="0" t="s">
-        <v>996</v>
+        <v>997</v>
       </c>
       <c r="B465" s="0" t="s">
-        <v>997</v>
+        <v>998</v>
       </c>
       <c r="C465" s="0" t="s">
-        <v>140</v>
+        <v>576</v>
       </c>
       <c r="D465" s="0">
-        <v>87</v>
+        <v>71176.4</v>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="0" t="s">
-        <v>998</v>
+        <v>999</v>
       </c>
       <c r="B466" s="0" t="s">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="C466" s="0" t="s">
-        <v>70</v>
+        <v>140</v>
       </c>
       <c r="D466" s="0">
-        <v>950</v>
+        <v>87</v>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="0" t="s">
-        <v>1000</v>
+        <v>1001</v>
       </c>
       <c r="B467" s="0" t="s">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="C467" s="0" t="s">
-        <v>469</v>
+        <v>70</v>
       </c>
       <c r="D467" s="0">
-        <v>342641</v>
+        <v>950</v>
       </c>
     </row>
     <row r="468">
       <c r="A468" s="0" t="s">
-        <v>1002</v>
+        <v>1003</v>
       </c>
       <c r="B468" s="0" t="s">
-        <v>1003</v>
+        <v>1004</v>
       </c>
       <c r="C468" s="0" t="s">
-        <v>160</v>
+        <v>469</v>
       </c>
       <c r="D468" s="0">
-        <v>2200</v>
+        <v>342641</v>
       </c>
     </row>
     <row r="469">
       <c r="A469" s="0" t="s">
-        <v>1004</v>
+        <v>1005</v>
       </c>
       <c r="B469" s="0" t="s">
-        <v>1005</v>
+        <v>1006</v>
       </c>
       <c r="C469" s="0" t="s">
-        <v>478</v>
+        <v>160</v>
       </c>
       <c r="D469" s="0">
-        <v>41000</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="0" t="s">
-        <v>1006</v>
+        <v>1007</v>
       </c>
       <c r="B470" s="0" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="C470" s="0" t="s">
-        <v>70</v>
+        <v>478</v>
       </c>
       <c r="D470" s="0">
-        <v>9299</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="471">
       <c r="A471" s="0" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="B471" s="0" t="s">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="C471" s="0" t="s">
-        <v>911</v>
+        <v>70</v>
       </c>
       <c r="D471" s="0">
-        <v>880</v>
+        <v>9299</v>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="0" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="B472" s="0" t="s">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="C472" s="0" t="s">
         <v>911</v>
@@ -9878,10 +9887,10 @@
     </row>
     <row r="473">
       <c r="A473" s="0" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="B473" s="0" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="C473" s="0" t="s">
         <v>911</v>
@@ -9892,114 +9901,114 @@
     </row>
     <row r="474">
       <c r="A474" s="0" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="B474" s="0" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="C474" s="0" t="s">
-        <v>21</v>
+        <v>911</v>
       </c>
       <c r="D474" s="0">
-        <v>563.36</v>
+        <v>880</v>
       </c>
     </row>
     <row r="475">
       <c r="A475" s="0" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="B475" s="0" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="C475" s="0" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D475" s="0">
-        <v>3520</v>
+        <v>563.36</v>
       </c>
     </row>
     <row r="476">
       <c r="A476" s="0" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="B476" s="0" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="C476" s="0" t="s">
         <v>15</v>
       </c>
       <c r="D476" s="0">
-        <v>2600</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="477">
       <c r="A477" s="0" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
       <c r="B477" s="0" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
       <c r="C477" s="0" t="s">
-        <v>281</v>
+        <v>15</v>
       </c>
       <c r="D477" s="0">
-        <v>3700</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="478">
       <c r="A478" s="0" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="B478" s="0" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
       <c r="C478" s="0" t="s">
         <v>281</v>
       </c>
       <c r="D478" s="0">
-        <v>2600</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="479">
       <c r="A479" s="0" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="B479" s="0" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
       <c r="C479" s="0" t="s">
-        <v>15</v>
+        <v>281</v>
       </c>
       <c r="D479" s="0">
-        <v>2235</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="480">
       <c r="A480" s="0" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="B480" s="0" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="C480" s="0" t="s">
         <v>15</v>
       </c>
       <c r="D480" s="0">
-        <v>3850</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="0" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="B481" s="0" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="C481" s="0" t="s">
-        <v>1030</v>
+        <v>15</v>
       </c>
       <c r="D481" s="0">
-        <v>1</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="482">
@@ -10010,94 +10019,94 @@
         <v>1032</v>
       </c>
       <c r="C482" s="0" t="s">
-        <v>28</v>
+        <v>1033</v>
       </c>
       <c r="D482" s="0">
-        <v>14819</v>
+        <v>1</v>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="0" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="B483" s="0" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="C483" s="0" t="s">
-        <v>376</v>
+        <v>28</v>
       </c>
       <c r="D483" s="0">
-        <v>3859.93</v>
+        <v>14819</v>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="0" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="B484" s="0" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="C484" s="0" t="s">
         <v>376</v>
       </c>
       <c r="D484" s="0">
-        <v>11751.49</v>
+        <v>3859.93</v>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="0" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
       <c r="B485" s="0" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="C485" s="0" t="s">
-        <v>338</v>
+        <v>376</v>
       </c>
       <c r="D485" s="0">
-        <v>6000</v>
+        <v>11751.49</v>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="0" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="B486" s="0" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="C486" s="0" t="s">
         <v>338</v>
       </c>
       <c r="D486" s="0">
-        <v>3000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="0" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="B487" s="0" t="s">
-        <v>1042</v>
+        <v>1043</v>
       </c>
       <c r="C487" s="0" t="s">
-        <v>37</v>
+        <v>338</v>
       </c>
       <c r="D487" s="0">
-        <v>618</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="0" t="s">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="B488" s="0" t="s">
-        <v>1044</v>
+        <v>1045</v>
       </c>
       <c r="C488" s="0" t="s">
-        <v>1045</v>
+        <v>37</v>
       </c>
       <c r="D488" s="0">
-        <v>24600</v>
+        <v>618</v>
       </c>
     </row>
     <row r="489">
@@ -10108,191 +10117,205 @@
         <v>1047</v>
       </c>
       <c r="C489" s="0" t="s">
-        <v>105</v>
+        <v>1048</v>
       </c>
       <c r="D489" s="0">
-        <v>0</v>
+        <v>24600</v>
       </c>
     </row>
     <row r="490">
       <c r="A490" s="0" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="B490" s="0" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="C490" s="0" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="D490" s="0">
-        <v>41593.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="491">
       <c r="A491" s="0" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="B491" s="0" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="C491" s="0" t="s">
-        <v>469</v>
+        <v>92</v>
       </c>
       <c r="D491" s="0">
-        <v>207558.07</v>
+        <v>41593.75</v>
       </c>
     </row>
     <row r="492">
       <c r="A492" s="0" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
       <c r="B492" s="0" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="C492" s="0" t="s">
-        <v>376</v>
+        <v>469</v>
       </c>
       <c r="D492" s="0">
-        <v>77429.29</v>
+        <v>207558.07</v>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="0" t="s">
-        <v>1054</v>
+        <v>1055</v>
       </c>
       <c r="B493" s="0" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
       <c r="C493" s="0" t="s">
         <v>376</v>
       </c>
       <c r="D493" s="0">
-        <v>42913.42</v>
+        <v>77429.29</v>
       </c>
     </row>
     <row r="494">
       <c r="A494" s="0" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
       <c r="B494" s="0" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="C494" s="0" t="s">
         <v>376</v>
       </c>
       <c r="D494" s="0">
-        <v>88806.25</v>
+        <v>42913.42</v>
       </c>
     </row>
     <row r="495">
       <c r="A495" s="0" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
       <c r="B495" s="0" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="C495" s="0" t="s">
         <v>376</v>
       </c>
       <c r="D495" s="0">
-        <v>50781.52</v>
+        <v>88806.25</v>
       </c>
     </row>
     <row r="496">
       <c r="A496" s="0" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
       <c r="B496" s="0" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="C496" s="0" t="s">
-        <v>21</v>
+        <v>376</v>
       </c>
       <c r="D496" s="0">
-        <v>1600</v>
+        <v>50781.52</v>
       </c>
     </row>
     <row r="497">
       <c r="A497" s="0" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="B497" s="0" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="C497" s="0" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D497" s="0">
-        <v>3455.8</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="498">
       <c r="A498" s="0" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="B498" s="0" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="C498" s="0" t="s">
         <v>28</v>
       </c>
       <c r="D498" s="0">
-        <v>3987</v>
+        <v>3455.8</v>
       </c>
     </row>
     <row r="499">
       <c r="A499" s="0" t="s">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="B499" s="0" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="C499" s="0" t="s">
         <v>28</v>
       </c>
       <c r="D499" s="0">
-        <v>4010.17</v>
+        <v>3987</v>
       </c>
     </row>
     <row r="500">
       <c r="A500" s="0" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="B500" s="0" t="s">
-        <v>1069</v>
+        <v>1070</v>
       </c>
       <c r="C500" s="0" t="s">
         <v>28</v>
       </c>
       <c r="D500" s="0">
-        <v>3382.65</v>
+        <v>4010.17</v>
       </c>
     </row>
     <row r="501">
       <c r="A501" s="0" t="s">
-        <v>1070</v>
+        <v>1071</v>
       </c>
       <c r="B501" s="0" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="C501" s="0" t="s">
-        <v>160</v>
+        <v>28</v>
       </c>
       <c r="D501" s="0">
-        <v>430</v>
+        <v>3382.65</v>
       </c>
     </row>
     <row r="502">
       <c r="A502" s="0" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="B502" s="0" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
       <c r="C502" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="D502" s="0">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="0" t="s">
+        <v>1075</v>
+      </c>
+      <c r="B503" s="0" t="s">
+        <v>1076</v>
+      </c>
+      <c r="C503" s="0" t="s">
         <v>140</v>
       </c>
-      <c r="D502" s="0">
+      <c r="D503" s="0">
         <v>465</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: stock y precios actualizados jue. 20/08/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -3680,7 +3680,7 @@
         <v>70</v>
       </c>
       <c r="D29" s="0">
-        <v>5152</v>
+        <v>5126</v>
       </c>
     </row>
     <row r="30">
@@ -3694,7 +3694,7 @@
         <v>70</v>
       </c>
       <c r="D30" s="0">
-        <v>12825</v>
+        <v>14813</v>
       </c>
     </row>
     <row r="31">
@@ -3708,7 +3708,7 @@
         <v>70</v>
       </c>
       <c r="D31" s="0">
-        <v>4048</v>
+        <v>4454</v>
       </c>
     </row>
     <row r="32">
@@ -4044,7 +4044,7 @@
         <v>70</v>
       </c>
       <c r="D55" s="0">
-        <v>3916</v>
+        <v>3795</v>
       </c>
     </row>
     <row r="56">
@@ -6970,7 +6970,7 @@
         <v>70</v>
       </c>
       <c r="D264" s="0">
-        <v>34000</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="265">
@@ -6984,7 +6984,7 @@
         <v>70</v>
       </c>
       <c r="D265" s="0">
-        <v>30000</v>
+        <v>34000</v>
       </c>
     </row>
     <row r="266">
@@ -8440,7 +8440,7 @@
         <v>70</v>
       </c>
       <c r="D369" s="0">
-        <v>3263</v>
+        <v>3427</v>
       </c>
     </row>
     <row r="370">
@@ -8454,7 +8454,7 @@
         <v>70</v>
       </c>
       <c r="D370" s="0">
-        <v>18027</v>
+        <v>10618</v>
       </c>
     </row>
     <row r="371">
@@ -8538,7 +8538,7 @@
         <v>70</v>
       </c>
       <c r="D376" s="0">
-        <v>10021.22</v>
+        <v>10522</v>
       </c>
     </row>
     <row r="377">
@@ -8552,7 +8552,7 @@
         <v>70</v>
       </c>
       <c r="D377" s="0">
-        <v>17710</v>
+        <v>19481</v>
       </c>
     </row>
     <row r="378">
@@ -8664,7 +8664,7 @@
         <v>70</v>
       </c>
       <c r="D385" s="0">
-        <v>2699.64</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="386">
@@ -9364,7 +9364,7 @@
         <v>70</v>
       </c>
       <c r="D435" s="0">
-        <v>15968</v>
+        <v>19322</v>
       </c>
     </row>
     <row r="436">
@@ -9546,7 +9546,7 @@
         <v>70</v>
       </c>
       <c r="D448" s="0">
-        <v>3380</v>
+        <v>4276</v>
       </c>
     </row>
     <row r="449">
@@ -9868,7 +9868,7 @@
         <v>70</v>
       </c>
       <c r="D471" s="0">
-        <v>9299</v>
+        <v>5790</v>
       </c>
     </row>
     <row r="472">

</xml_diff>

<commit_message>
sync: stock y precios actualizados sáb. 29/08/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1077" uniqueCount="1077">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="1081">
   <si>
     <t>Solo Activos</t>
   </si>
@@ -1620,6 +1620,18 @@
   </si>
   <si>
     <t>HIGLUCEM 30MG COMP. X 28 - 000014951</t>
+  </si>
+  <si>
+    <t>000024696</t>
+  </si>
+  <si>
+    <t>HIOSCINA + DIPIRONA DUNCAN AMP X 1 - N-BUTIL BROMURO - 000024696</t>
+  </si>
+  <si>
+    <t>000024135</t>
+  </si>
+  <si>
+    <t>HIOSCINA + DIPIRONA LARJAN X 5 ML - 000024135</t>
   </si>
   <si>
     <t>1973456</t>
@@ -3308,7 +3320,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:D503"/>
+  <dimension ref="A2:D505"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -6687,10 +6699,10 @@
         <v>537</v>
       </c>
       <c r="C244" s="0" t="s">
-        <v>281</v>
+        <v>151</v>
       </c>
       <c r="D244" s="0">
-        <v>450</v>
+        <v>700</v>
       </c>
     </row>
     <row r="245">
@@ -6701,10 +6713,10 @@
         <v>539</v>
       </c>
       <c r="C245" s="0" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="D245" s="0">
-        <v>555</v>
+        <v>700</v>
       </c>
     </row>
     <row r="246">
@@ -6715,10 +6727,10 @@
         <v>541</v>
       </c>
       <c r="C246" s="0" t="s">
-        <v>15</v>
+        <v>281</v>
       </c>
       <c r="D246" s="0">
-        <v>825</v>
+        <v>450</v>
       </c>
     </row>
     <row r="247">
@@ -6732,7 +6744,7 @@
         <v>15</v>
       </c>
       <c r="D247" s="0">
-        <v>36.3</v>
+        <v>555</v>
       </c>
     </row>
     <row r="248">
@@ -6746,7 +6758,7 @@
         <v>15</v>
       </c>
       <c r="D248" s="0">
-        <v>544.5</v>
+        <v>825</v>
       </c>
     </row>
     <row r="249">
@@ -6760,7 +6772,7 @@
         <v>15</v>
       </c>
       <c r="D249" s="0">
-        <v>750</v>
+        <v>36.3</v>
       </c>
     </row>
     <row r="250">
@@ -6771,10 +6783,10 @@
         <v>549</v>
       </c>
       <c r="C250" s="0" t="s">
-        <v>151</v>
+        <v>15</v>
       </c>
       <c r="D250" s="0">
-        <v>1130</v>
+        <v>544.5</v>
       </c>
     </row>
     <row r="251">
@@ -6785,10 +6797,10 @@
         <v>551</v>
       </c>
       <c r="C251" s="0" t="s">
-        <v>52</v>
+        <v>15</v>
       </c>
       <c r="D251" s="0">
-        <v>4510</v>
+        <v>750</v>
       </c>
     </row>
     <row r="252">
@@ -6799,10 +6811,10 @@
         <v>553</v>
       </c>
       <c r="C252" s="0" t="s">
-        <v>52</v>
+        <v>151</v>
       </c>
       <c r="D252" s="0">
-        <v>4510</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="253">
@@ -6841,10 +6853,10 @@
         <v>559</v>
       </c>
       <c r="C255" s="0" t="s">
-        <v>15</v>
+        <v>52</v>
       </c>
       <c r="D255" s="0">
-        <v>902</v>
+        <v>4510</v>
       </c>
     </row>
     <row r="256">
@@ -6855,10 +6867,10 @@
         <v>561</v>
       </c>
       <c r="C256" s="0" t="s">
-        <v>15</v>
+        <v>52</v>
       </c>
       <c r="D256" s="0">
-        <v>880</v>
+        <v>4510</v>
       </c>
     </row>
     <row r="257">
@@ -6869,10 +6881,10 @@
         <v>563</v>
       </c>
       <c r="C257" s="0" t="s">
-        <v>140</v>
+        <v>15</v>
       </c>
       <c r="D257" s="0">
-        <v>430</v>
+        <v>902</v>
       </c>
     </row>
     <row r="258">
@@ -6883,10 +6895,10 @@
         <v>565</v>
       </c>
       <c r="C258" s="0" t="s">
-        <v>140</v>
+        <v>15</v>
       </c>
       <c r="D258" s="0">
-        <v>373</v>
+        <v>880</v>
       </c>
     </row>
     <row r="259">
@@ -6897,10 +6909,10 @@
         <v>567</v>
       </c>
       <c r="C259" s="0" t="s">
-        <v>18</v>
+        <v>140</v>
       </c>
       <c r="D259" s="0">
-        <v>318.63</v>
+        <v>430</v>
       </c>
     </row>
     <row r="260">
@@ -6911,10 +6923,10 @@
         <v>569</v>
       </c>
       <c r="C260" s="0" t="s">
-        <v>18</v>
+        <v>140</v>
       </c>
       <c r="D260" s="0">
-        <v>415.15</v>
+        <v>373</v>
       </c>
     </row>
     <row r="261">
@@ -6928,7 +6940,7 @@
         <v>18</v>
       </c>
       <c r="D261" s="0">
-        <v>760</v>
+        <v>318.63</v>
       </c>
     </row>
     <row r="262">
@@ -6942,7 +6954,7 @@
         <v>18</v>
       </c>
       <c r="D262" s="0">
-        <v>820</v>
+        <v>415.15</v>
       </c>
     </row>
     <row r="263">
@@ -6953,38 +6965,38 @@
         <v>575</v>
       </c>
       <c r="C263" s="0" t="s">
-        <v>576</v>
+        <v>18</v>
       </c>
       <c r="D263" s="0">
-        <v>177940.1</v>
+        <v>760</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="0" t="s">
+        <v>576</v>
+      </c>
+      <c r="B264" s="0" t="s">
         <v>577</v>
       </c>
-      <c r="B264" s="0" t="s">
-        <v>578</v>
-      </c>
       <c r="C264" s="0" t="s">
-        <v>70</v>
+        <v>18</v>
       </c>
       <c r="D264" s="0">
-        <v>28000</v>
+        <v>820</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="0" t="s">
+        <v>578</v>
+      </c>
+      <c r="B265" s="0" t="s">
         <v>579</v>
       </c>
-      <c r="B265" s="0" t="s">
+      <c r="C265" s="0" t="s">
         <v>580</v>
       </c>
-      <c r="C265" s="0" t="s">
-        <v>70</v>
-      </c>
       <c r="D265" s="0">
-        <v>34000</v>
+        <v>177940.1</v>
       </c>
     </row>
     <row r="266">
@@ -6995,10 +7007,10 @@
         <v>582</v>
       </c>
       <c r="C266" s="0" t="s">
-        <v>469</v>
+        <v>70</v>
       </c>
       <c r="D266" s="0">
-        <v>227939.52</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="267">
@@ -7009,10 +7021,10 @@
         <v>584</v>
       </c>
       <c r="C267" s="0" t="s">
-        <v>469</v>
+        <v>70</v>
       </c>
       <c r="D267" s="0">
-        <v>184488.7</v>
+        <v>34000</v>
       </c>
     </row>
     <row r="268">
@@ -7023,10 +7035,10 @@
         <v>586</v>
       </c>
       <c r="C268" s="0" t="s">
-        <v>15</v>
+        <v>469</v>
       </c>
       <c r="D268" s="0">
-        <v>1760</v>
+        <v>227939.52</v>
       </c>
     </row>
     <row r="269">
@@ -7037,38 +7049,38 @@
         <v>588</v>
       </c>
       <c r="C269" s="0" t="s">
-        <v>589</v>
+        <v>469</v>
       </c>
       <c r="D269" s="0">
-        <v>26350</v>
+        <v>184488.7</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="0" t="s">
+        <v>589</v>
+      </c>
+      <c r="B270" s="0" t="s">
         <v>590</v>
       </c>
-      <c r="B270" s="0" t="s">
-        <v>591</v>
-      </c>
       <c r="C270" s="0" t="s">
-        <v>478</v>
+        <v>15</v>
       </c>
       <c r="D270" s="0">
-        <v>31250</v>
+        <v>1760</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="0" t="s">
+        <v>591</v>
+      </c>
+      <c r="B271" s="0" t="s">
         <v>592</v>
       </c>
-      <c r="B271" s="0" t="s">
+      <c r="C271" s="0" t="s">
         <v>593</v>
       </c>
-      <c r="C271" s="0" t="s">
-        <v>52</v>
-      </c>
       <c r="D271" s="0">
-        <v>34.98</v>
+        <v>26350</v>
       </c>
     </row>
     <row r="272">
@@ -7079,38 +7091,38 @@
         <v>595</v>
       </c>
       <c r="C272" s="0" t="s">
-        <v>596</v>
+        <v>478</v>
       </c>
       <c r="D272" s="0">
-        <v>65</v>
+        <v>31250</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="0" t="s">
+        <v>596</v>
+      </c>
+      <c r="B273" s="0" t="s">
         <v>597</v>
-      </c>
-      <c r="B273" s="0" t="s">
-        <v>598</v>
       </c>
       <c r="C273" s="0" t="s">
         <v>52</v>
       </c>
       <c r="D273" s="0">
-        <v>65</v>
+        <v>34.98</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="0" t="s">
+        <v>598</v>
+      </c>
+      <c r="B274" s="0" t="s">
         <v>599</v>
       </c>
-      <c r="B274" s="0" t="s">
+      <c r="C274" s="0" t="s">
         <v>600</v>
       </c>
-      <c r="C274" s="0" t="s">
-        <v>52</v>
-      </c>
       <c r="D274" s="0">
-        <v>92</v>
+        <v>65</v>
       </c>
     </row>
     <row r="275">
@@ -7124,7 +7136,7 @@
         <v>52</v>
       </c>
       <c r="D275" s="0">
-        <v>33</v>
+        <v>65</v>
       </c>
     </row>
     <row r="276">
@@ -7138,7 +7150,7 @@
         <v>52</v>
       </c>
       <c r="D276" s="0">
-        <v>38.22</v>
+        <v>92</v>
       </c>
     </row>
     <row r="277">
@@ -7149,10 +7161,10 @@
         <v>606</v>
       </c>
       <c r="C277" s="0" t="s">
-        <v>338</v>
+        <v>52</v>
       </c>
       <c r="D277" s="0">
-        <v>300</v>
+        <v>33</v>
       </c>
     </row>
     <row r="278">
@@ -7163,10 +7175,10 @@
         <v>608</v>
       </c>
       <c r="C278" s="0" t="s">
-        <v>338</v>
+        <v>52</v>
       </c>
       <c r="D278" s="0">
-        <v>370</v>
+        <v>38.22</v>
       </c>
     </row>
     <row r="279">
@@ -7177,10 +7189,10 @@
         <v>610</v>
       </c>
       <c r="C279" s="0" t="s">
-        <v>359</v>
+        <v>338</v>
       </c>
       <c r="D279" s="0">
-        <v>450</v>
+        <v>300</v>
       </c>
     </row>
     <row r="280">
@@ -7191,10 +7203,10 @@
         <v>612</v>
       </c>
       <c r="C280" s="0" t="s">
-        <v>37</v>
+        <v>338</v>
       </c>
       <c r="D280" s="0">
-        <v>450</v>
+        <v>370</v>
       </c>
     </row>
     <row r="281">
@@ -7205,7 +7217,7 @@
         <v>614</v>
       </c>
       <c r="C281" s="0" t="s">
-        <v>15</v>
+        <v>359</v>
       </c>
       <c r="D281" s="0">
         <v>450</v>
@@ -7219,10 +7231,10 @@
         <v>616</v>
       </c>
       <c r="C282" s="0" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="D282" s="0">
-        <v>1650</v>
+        <v>450</v>
       </c>
     </row>
     <row r="283">
@@ -7236,7 +7248,7 @@
         <v>15</v>
       </c>
       <c r="D283" s="0">
-        <v>2100</v>
+        <v>450</v>
       </c>
     </row>
     <row r="284">
@@ -7250,7 +7262,7 @@
         <v>15</v>
       </c>
       <c r="D284" s="0">
-        <v>1980</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="285">
@@ -7264,7 +7276,7 @@
         <v>15</v>
       </c>
       <c r="D285" s="0">
-        <v>2160</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="286">
@@ -7278,7 +7290,7 @@
         <v>15</v>
       </c>
       <c r="D286" s="0">
-        <v>1500</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="287">
@@ -7292,7 +7304,7 @@
         <v>15</v>
       </c>
       <c r="D287" s="0">
-        <v>2600</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="288">
@@ -7306,7 +7318,7 @@
         <v>15</v>
       </c>
       <c r="D288" s="0">
-        <v>2000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="289">
@@ -7320,7 +7332,7 @@
         <v>15</v>
       </c>
       <c r="D289" s="0">
-        <v>6700</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="290">
@@ -7334,7 +7346,7 @@
         <v>15</v>
       </c>
       <c r="D290" s="0">
-        <v>1650</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="291">
@@ -7348,7 +7360,7 @@
         <v>15</v>
       </c>
       <c r="D291" s="0">
-        <v>1035</v>
+        <v>6700</v>
       </c>
     </row>
     <row r="292">
@@ -7362,7 +7374,7 @@
         <v>15</v>
       </c>
       <c r="D292" s="0">
-        <v>2600</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="293">
@@ -7376,7 +7388,7 @@
         <v>15</v>
       </c>
       <c r="D293" s="0">
-        <v>2400</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="294">
@@ -7387,10 +7399,10 @@
         <v>640</v>
       </c>
       <c r="C294" s="0" t="s">
-        <v>140</v>
+        <v>15</v>
       </c>
       <c r="D294" s="0">
-        <v>4590</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="295">
@@ -7401,10 +7413,10 @@
         <v>642</v>
       </c>
       <c r="C295" s="0" t="s">
-        <v>140</v>
+        <v>15</v>
       </c>
       <c r="D295" s="0">
-        <v>2300</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="296">
@@ -7418,7 +7430,7 @@
         <v>140</v>
       </c>
       <c r="D296" s="0">
-        <v>1150</v>
+        <v>4590</v>
       </c>
     </row>
     <row r="297">
@@ -7429,10 +7441,10 @@
         <v>646</v>
       </c>
       <c r="C297" s="0" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="D297" s="0">
-        <v>7372.42</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="298">
@@ -7443,10 +7455,10 @@
         <v>648</v>
       </c>
       <c r="C298" s="0" t="s">
-        <v>123</v>
+        <v>140</v>
       </c>
       <c r="D298" s="0">
-        <v>1790</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="299">
@@ -7457,10 +7469,10 @@
         <v>650</v>
       </c>
       <c r="C299" s="0" t="s">
-        <v>123</v>
+        <v>28</v>
       </c>
       <c r="D299" s="0">
-        <v>2859.96</v>
+        <v>7372.42</v>
       </c>
     </row>
     <row r="300">
@@ -7474,7 +7486,7 @@
         <v>123</v>
       </c>
       <c r="D300" s="0">
-        <v>4800</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="301">
@@ -7485,38 +7497,38 @@
         <v>654</v>
       </c>
       <c r="C301" s="0" t="s">
-        <v>655</v>
+        <v>123</v>
       </c>
       <c r="D301" s="0">
-        <v>0</v>
+        <v>2859.96</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="0" t="s">
+        <v>655</v>
+      </c>
+      <c r="B302" s="0" t="s">
         <v>656</v>
       </c>
-      <c r="B302" s="0" t="s">
-        <v>657</v>
-      </c>
       <c r="C302" s="0" t="s">
-        <v>28</v>
+        <v>123</v>
       </c>
       <c r="D302" s="0">
-        <v>494</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="0" t="s">
+        <v>657</v>
+      </c>
+      <c r="B303" s="0" t="s">
         <v>658</v>
       </c>
-      <c r="B303" s="0" t="s">
+      <c r="C303" s="0" t="s">
         <v>659</v>
       </c>
-      <c r="C303" s="0" t="s">
-        <v>28</v>
-      </c>
       <c r="D303" s="0">
-        <v>665.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="304">
@@ -7527,10 +7539,10 @@
         <v>661</v>
       </c>
       <c r="C304" s="0" t="s">
-        <v>92</v>
+        <v>28</v>
       </c>
       <c r="D304" s="0">
-        <v>33940.5</v>
+        <v>494</v>
       </c>
     </row>
     <row r="305">
@@ -7541,10 +7553,10 @@
         <v>663</v>
       </c>
       <c r="C305" s="0" t="s">
-        <v>92</v>
+        <v>28</v>
       </c>
       <c r="D305" s="0">
-        <v>4525.4</v>
+        <v>665.3</v>
       </c>
     </row>
     <row r="306">
@@ -7555,10 +7567,10 @@
         <v>665</v>
       </c>
       <c r="C306" s="0" t="s">
-        <v>151</v>
+        <v>92</v>
       </c>
       <c r="D306" s="0">
-        <v>896</v>
+        <v>33940.5</v>
       </c>
     </row>
     <row r="307">
@@ -7569,10 +7581,10 @@
         <v>667</v>
       </c>
       <c r="C307" s="0" t="s">
-        <v>140</v>
+        <v>92</v>
       </c>
       <c r="D307" s="0">
-        <v>1250</v>
+        <v>4525.4</v>
       </c>
     </row>
     <row r="308">
@@ -7583,10 +7595,10 @@
         <v>669</v>
       </c>
       <c r="C308" s="0" t="s">
-        <v>92</v>
+        <v>151</v>
       </c>
       <c r="D308" s="0">
-        <v>319440</v>
+        <v>896</v>
       </c>
     </row>
     <row r="309">
@@ -7597,10 +7609,10 @@
         <v>671</v>
       </c>
       <c r="C309" s="0" t="s">
-        <v>202</v>
+        <v>140</v>
       </c>
       <c r="D309" s="0">
-        <v>17440</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="310">
@@ -7611,10 +7623,10 @@
         <v>673</v>
       </c>
       <c r="C310" s="0" t="s">
-        <v>202</v>
+        <v>92</v>
       </c>
       <c r="D310" s="0">
-        <v>4390</v>
+        <v>319440</v>
       </c>
     </row>
     <row r="311">
@@ -7628,7 +7640,7 @@
         <v>202</v>
       </c>
       <c r="D311" s="0">
-        <v>4390</v>
+        <v>17440</v>
       </c>
     </row>
     <row r="312">
@@ -7639,10 +7651,10 @@
         <v>677</v>
       </c>
       <c r="C312" s="0" t="s">
-        <v>281</v>
+        <v>202</v>
       </c>
       <c r="D312" s="0">
-        <v>2250</v>
+        <v>4390</v>
       </c>
     </row>
     <row r="313">
@@ -7656,7 +7668,7 @@
         <v>202</v>
       </c>
       <c r="D313" s="0">
-        <v>3355</v>
+        <v>4390</v>
       </c>
     </row>
     <row r="314">
@@ -7667,10 +7679,10 @@
         <v>681</v>
       </c>
       <c r="C314" s="0" t="s">
-        <v>207</v>
+        <v>281</v>
       </c>
       <c r="D314" s="0">
-        <v>7500</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="315">
@@ -7681,10 +7693,10 @@
         <v>683</v>
       </c>
       <c r="C315" s="0" t="s">
-        <v>92</v>
+        <v>202</v>
       </c>
       <c r="D315" s="0">
-        <v>25289</v>
+        <v>3355</v>
       </c>
     </row>
     <row r="316">
@@ -7695,10 +7707,10 @@
         <v>685</v>
       </c>
       <c r="C316" s="0" t="s">
-        <v>92</v>
+        <v>207</v>
       </c>
       <c r="D316" s="0">
-        <v>252890</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="317">
@@ -7709,10 +7721,10 @@
         <v>687</v>
       </c>
       <c r="C317" s="0" t="s">
-        <v>52</v>
+        <v>92</v>
       </c>
       <c r="D317" s="0">
-        <v>130</v>
+        <v>25289</v>
       </c>
     </row>
     <row r="318">
@@ -7723,10 +7735,10 @@
         <v>689</v>
       </c>
       <c r="C318" s="0" t="s">
-        <v>21</v>
+        <v>92</v>
       </c>
       <c r="D318" s="0">
-        <v>285.6</v>
+        <v>252890</v>
       </c>
     </row>
     <row r="319">
@@ -7737,10 +7749,10 @@
         <v>691</v>
       </c>
       <c r="C319" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="D319" s="0">
-        <v>338</v>
+        <v>130</v>
       </c>
     </row>
     <row r="320">
@@ -7751,52 +7763,52 @@
         <v>693</v>
       </c>
       <c r="C320" s="0" t="s">
-        <v>694</v>
+        <v>21</v>
       </c>
       <c r="D320" s="0">
-        <v>770</v>
+        <v>285.6</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="0" t="s">
+        <v>694</v>
+      </c>
+      <c r="B321" s="0" t="s">
         <v>695</v>
       </c>
-      <c r="B321" s="0" t="s">
-        <v>696</v>
-      </c>
       <c r="C321" s="0" t="s">
-        <v>697</v>
+        <v>21</v>
       </c>
       <c r="D321" s="0">
-        <v>770</v>
+        <v>338</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="0" t="s">
+        <v>696</v>
+      </c>
+      <c r="B322" s="0" t="s">
+        <v>697</v>
+      </c>
+      <c r="C322" s="0" t="s">
         <v>698</v>
       </c>
-      <c r="B322" s="0" t="s">
-        <v>699</v>
-      </c>
-      <c r="C322" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="D322" s="0">
-        <v>973.5</v>
+        <v>770</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="0" t="s">
+        <v>699</v>
+      </c>
+      <c r="B323" s="0" t="s">
         <v>700</v>
       </c>
-      <c r="B323" s="0" t="s">
+      <c r="C323" s="0" t="s">
         <v>701</v>
       </c>
-      <c r="C323" s="0" t="s">
-        <v>21</v>
-      </c>
       <c r="D323" s="0">
-        <v>507.08</v>
+        <v>770</v>
       </c>
     </row>
     <row r="324">
@@ -7810,7 +7822,7 @@
         <v>15</v>
       </c>
       <c r="D324" s="0">
-        <v>450</v>
+        <v>973.5</v>
       </c>
     </row>
     <row r="325">
@@ -7821,10 +7833,10 @@
         <v>705</v>
       </c>
       <c r="C325" s="0" t="s">
-        <v>151</v>
+        <v>21</v>
       </c>
       <c r="D325" s="0">
-        <v>760</v>
+        <v>507.08</v>
       </c>
     </row>
     <row r="326">
@@ -7835,10 +7847,10 @@
         <v>707</v>
       </c>
       <c r="C326" s="0" t="s">
-        <v>281</v>
+        <v>15</v>
       </c>
       <c r="D326" s="0">
-        <v>5900</v>
+        <v>450</v>
       </c>
     </row>
     <row r="327">
@@ -7849,10 +7861,10 @@
         <v>709</v>
       </c>
       <c r="C327" s="0" t="s">
-        <v>281</v>
+        <v>151</v>
       </c>
       <c r="D327" s="0">
-        <v>2900</v>
+        <v>760</v>
       </c>
     </row>
     <row r="328">
@@ -7863,10 +7875,10 @@
         <v>711</v>
       </c>
       <c r="C328" s="0" t="s">
-        <v>140</v>
+        <v>281</v>
       </c>
       <c r="D328" s="0">
-        <v>890</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="329">
@@ -7877,10 +7889,10 @@
         <v>713</v>
       </c>
       <c r="C329" s="0" t="s">
-        <v>140</v>
+        <v>281</v>
       </c>
       <c r="D329" s="0">
-        <v>594</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="330">
@@ -7894,7 +7906,7 @@
         <v>140</v>
       </c>
       <c r="D330" s="0">
-        <v>65</v>
+        <v>890</v>
       </c>
     </row>
     <row r="331">
@@ -7905,10 +7917,10 @@
         <v>717</v>
       </c>
       <c r="C331" s="0" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="D331" s="0">
-        <v>11313.5</v>
+        <v>594</v>
       </c>
     </row>
     <row r="332">
@@ -7919,10 +7931,10 @@
         <v>719</v>
       </c>
       <c r="C332" s="0" t="s">
-        <v>34</v>
+        <v>140</v>
       </c>
       <c r="D332" s="0">
-        <v>420</v>
+        <v>65</v>
       </c>
     </row>
     <row r="333">
@@ -7933,10 +7945,10 @@
         <v>721</v>
       </c>
       <c r="C333" s="0" t="s">
-        <v>359</v>
+        <v>92</v>
       </c>
       <c r="D333" s="0">
-        <v>418</v>
+        <v>11313.5</v>
       </c>
     </row>
     <row r="334">
@@ -7947,10 +7959,10 @@
         <v>723</v>
       </c>
       <c r="C334" s="0" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="D334" s="0">
-        <v>377</v>
+        <v>420</v>
       </c>
     </row>
     <row r="335">
@@ -7961,10 +7973,10 @@
         <v>725</v>
       </c>
       <c r="C335" s="0" t="s">
-        <v>45</v>
+        <v>359</v>
       </c>
       <c r="D335" s="0">
-        <v>5780.66</v>
+        <v>418</v>
       </c>
     </row>
     <row r="336">
@@ -7975,10 +7987,10 @@
         <v>727</v>
       </c>
       <c r="C336" s="0" t="s">
-        <v>70</v>
+        <v>21</v>
       </c>
       <c r="D336" s="0">
-        <v>898</v>
+        <v>377</v>
       </c>
     </row>
     <row r="337">
@@ -7989,10 +8001,10 @@
         <v>729</v>
       </c>
       <c r="C337" s="0" t="s">
-        <v>123</v>
+        <v>45</v>
       </c>
       <c r="D337" s="0">
-        <v>4767</v>
+        <v>5780.66</v>
       </c>
     </row>
     <row r="338">
@@ -8003,10 +8015,10 @@
         <v>731</v>
       </c>
       <c r="C338" s="0" t="s">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="D338" s="0">
-        <v>650</v>
+        <v>898</v>
       </c>
     </row>
     <row r="339">
@@ -8017,10 +8029,10 @@
         <v>733</v>
       </c>
       <c r="C339" s="0" t="s">
-        <v>70</v>
+        <v>123</v>
       </c>
       <c r="D339" s="0">
-        <v>650</v>
+        <v>4767</v>
       </c>
     </row>
     <row r="340">
@@ -8031,10 +8043,10 @@
         <v>735</v>
       </c>
       <c r="C340" s="0" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="D340" s="0">
-        <v>2178</v>
+        <v>650</v>
       </c>
     </row>
     <row r="341">
@@ -8045,10 +8057,10 @@
         <v>737</v>
       </c>
       <c r="C341" s="0" t="s">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="D341" s="0">
-        <v>7986</v>
+        <v>650</v>
       </c>
     </row>
     <row r="342">
@@ -8059,38 +8071,38 @@
         <v>739</v>
       </c>
       <c r="C342" s="0" t="s">
-        <v>740</v>
+        <v>15</v>
       </c>
       <c r="D342" s="0">
-        <v>1910</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" s="0" t="s">
+        <v>740</v>
+      </c>
+      <c r="B343" s="0" t="s">
         <v>741</v>
       </c>
-      <c r="B343" s="0" t="s">
-        <v>742</v>
-      </c>
       <c r="C343" s="0" t="s">
-        <v>151</v>
+        <v>92</v>
       </c>
       <c r="D343" s="0">
-        <v>900</v>
+        <v>7986</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="0" t="s">
+        <v>742</v>
+      </c>
+      <c r="B344" s="0" t="s">
         <v>743</v>
       </c>
-      <c r="B344" s="0" t="s">
+      <c r="C344" s="0" t="s">
         <v>744</v>
       </c>
-      <c r="C344" s="0" t="s">
-        <v>21</v>
-      </c>
       <c r="D344" s="0">
-        <v>1722</v>
+        <v>1910</v>
       </c>
     </row>
     <row r="345">
@@ -8101,10 +8113,10 @@
         <v>746</v>
       </c>
       <c r="C345" s="0" t="s">
-        <v>34</v>
+        <v>151</v>
       </c>
       <c r="D345" s="0">
-        <v>59000</v>
+        <v>900</v>
       </c>
     </row>
     <row r="346">
@@ -8115,10 +8127,10 @@
         <v>748</v>
       </c>
       <c r="C346" s="0" t="s">
-        <v>151</v>
+        <v>21</v>
       </c>
       <c r="D346" s="0">
-        <v>750</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="347">
@@ -8129,10 +8141,10 @@
         <v>750</v>
       </c>
       <c r="C347" s="0" t="s">
-        <v>151</v>
+        <v>34</v>
       </c>
       <c r="D347" s="0">
-        <v>1212</v>
+        <v>59000</v>
       </c>
     </row>
     <row r="348">
@@ -8146,7 +8158,7 @@
         <v>151</v>
       </c>
       <c r="D348" s="0">
-        <v>1300</v>
+        <v>750</v>
       </c>
     </row>
     <row r="349">
@@ -8160,7 +8172,7 @@
         <v>151</v>
       </c>
       <c r="D349" s="0">
-        <v>1500</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="350">
@@ -8174,7 +8186,7 @@
         <v>151</v>
       </c>
       <c r="D350" s="0">
-        <v>1400</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="351">
@@ -8185,10 +8197,10 @@
         <v>758</v>
       </c>
       <c r="C351" s="0" t="s">
-        <v>261</v>
+        <v>151</v>
       </c>
       <c r="D351" s="0">
-        <v>11959</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="352">
@@ -8199,10 +8211,10 @@
         <v>760</v>
       </c>
       <c r="C352" s="0" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="D352" s="0">
-        <v>350</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="353">
@@ -8213,10 +8225,10 @@
         <v>762</v>
       </c>
       <c r="C353" s="0" t="s">
-        <v>281</v>
+        <v>261</v>
       </c>
       <c r="D353" s="0">
-        <v>1450</v>
+        <v>11959</v>
       </c>
     </row>
     <row r="354">
@@ -8227,10 +8239,10 @@
         <v>764</v>
       </c>
       <c r="C354" s="0" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="D354" s="0">
-        <v>7320.5</v>
+        <v>350</v>
       </c>
     </row>
     <row r="355">
@@ -8241,10 +8253,10 @@
         <v>766</v>
       </c>
       <c r="C355" s="0" t="s">
-        <v>15</v>
+        <v>281</v>
       </c>
       <c r="D355" s="0">
-        <v>900</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="356">
@@ -8255,10 +8267,10 @@
         <v>768</v>
       </c>
       <c r="C356" s="0" t="s">
-        <v>281</v>
+        <v>92</v>
       </c>
       <c r="D356" s="0">
-        <v>566</v>
+        <v>7320.5</v>
       </c>
     </row>
     <row r="357">
@@ -8269,10 +8281,10 @@
         <v>770</v>
       </c>
       <c r="C357" s="0" t="s">
-        <v>469</v>
+        <v>15</v>
       </c>
       <c r="D357" s="0">
-        <v>64925</v>
+        <v>900</v>
       </c>
     </row>
     <row r="358">
@@ -8283,10 +8295,10 @@
         <v>772</v>
       </c>
       <c r="C358" s="0" t="s">
-        <v>15</v>
+        <v>281</v>
       </c>
       <c r="D358" s="0">
-        <v>1100</v>
+        <v>566</v>
       </c>
     </row>
     <row r="359">
@@ -8297,10 +8309,10 @@
         <v>774</v>
       </c>
       <c r="C359" s="0" t="s">
-        <v>21</v>
+        <v>469</v>
       </c>
       <c r="D359" s="0">
-        <v>1623</v>
+        <v>64925</v>
       </c>
     </row>
     <row r="360">
@@ -8311,10 +8323,10 @@
         <v>776</v>
       </c>
       <c r="C360" s="0" t="s">
-        <v>140</v>
+        <v>15</v>
       </c>
       <c r="D360" s="0">
-        <v>1229</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="361">
@@ -8325,10 +8337,10 @@
         <v>778</v>
       </c>
       <c r="C361" s="0" t="s">
-        <v>140</v>
+        <v>21</v>
       </c>
       <c r="D361" s="0">
-        <v>4500</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="362">
@@ -8339,10 +8351,10 @@
         <v>780</v>
       </c>
       <c r="C362" s="0" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="D362" s="0">
-        <v>1250</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="363">
@@ -8353,10 +8365,10 @@
         <v>782</v>
       </c>
       <c r="C363" s="0" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="D363" s="0">
-        <v>1945.1</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="364">
@@ -8367,10 +8379,10 @@
         <v>784</v>
       </c>
       <c r="C364" s="0" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="D364" s="0">
-        <v>450</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="365">
@@ -8381,10 +8393,10 @@
         <v>786</v>
       </c>
       <c r="C365" s="0" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="D365" s="0">
-        <v>825</v>
+        <v>1945.1</v>
       </c>
     </row>
     <row r="366">
@@ -8398,7 +8410,7 @@
         <v>15</v>
       </c>
       <c r="D366" s="0">
-        <v>825</v>
+        <v>450</v>
       </c>
     </row>
     <row r="367">
@@ -8409,10 +8421,10 @@
         <v>790</v>
       </c>
       <c r="C367" s="0" t="s">
-        <v>379</v>
+        <v>15</v>
       </c>
       <c r="D367" s="0">
-        <v>134775.6</v>
+        <v>825</v>
       </c>
     </row>
     <row r="368">
@@ -8423,10 +8435,10 @@
         <v>792</v>
       </c>
       <c r="C368" s="0" t="s">
-        <v>379</v>
+        <v>15</v>
       </c>
       <c r="D368" s="0">
-        <v>175991.55</v>
+        <v>825</v>
       </c>
     </row>
     <row r="369">
@@ -8437,10 +8449,10 @@
         <v>794</v>
       </c>
       <c r="C369" s="0" t="s">
-        <v>70</v>
+        <v>379</v>
       </c>
       <c r="D369" s="0">
-        <v>3427</v>
+        <v>134775.6</v>
       </c>
     </row>
     <row r="370">
@@ -8451,10 +8463,10 @@
         <v>796</v>
       </c>
       <c r="C370" s="0" t="s">
-        <v>70</v>
+        <v>379</v>
       </c>
       <c r="D370" s="0">
-        <v>10618</v>
+        <v>175991.55</v>
       </c>
     </row>
     <row r="371">
@@ -8465,10 +8477,10 @@
         <v>798</v>
       </c>
       <c r="C371" s="0" t="s">
-        <v>281</v>
+        <v>70</v>
       </c>
       <c r="D371" s="0">
-        <v>515</v>
+        <v>3427</v>
       </c>
     </row>
     <row r="372">
@@ -8479,10 +8491,10 @@
         <v>800</v>
       </c>
       <c r="C372" s="0" t="s">
-        <v>37</v>
+        <v>70</v>
       </c>
       <c r="D372" s="0">
-        <v>515</v>
+        <v>10618</v>
       </c>
     </row>
     <row r="373">
@@ -8493,10 +8505,10 @@
         <v>802</v>
       </c>
       <c r="C373" s="0" t="s">
-        <v>52</v>
+        <v>281</v>
       </c>
       <c r="D373" s="0">
-        <v>9500</v>
+        <v>515</v>
       </c>
     </row>
     <row r="374">
@@ -8507,10 +8519,10 @@
         <v>804</v>
       </c>
       <c r="C374" s="0" t="s">
-        <v>469</v>
+        <v>37</v>
       </c>
       <c r="D374" s="0">
-        <v>207558.08</v>
+        <v>515</v>
       </c>
     </row>
     <row r="375">
@@ -8521,10 +8533,10 @@
         <v>806</v>
       </c>
       <c r="C375" s="0" t="s">
-        <v>469</v>
+        <v>52</v>
       </c>
       <c r="D375" s="0">
-        <v>249069.69</v>
+        <v>9500</v>
       </c>
     </row>
     <row r="376">
@@ -8535,10 +8547,10 @@
         <v>808</v>
       </c>
       <c r="C376" s="0" t="s">
-        <v>70</v>
+        <v>469</v>
       </c>
       <c r="D376" s="0">
-        <v>10522</v>
+        <v>207558.08</v>
       </c>
     </row>
     <row r="377">
@@ -8549,10 +8561,10 @@
         <v>810</v>
       </c>
       <c r="C377" s="0" t="s">
-        <v>70</v>
+        <v>469</v>
       </c>
       <c r="D377" s="0">
-        <v>19481</v>
+        <v>249069.69</v>
       </c>
     </row>
     <row r="378">
@@ -8563,66 +8575,66 @@
         <v>812</v>
       </c>
       <c r="C378" s="0" t="s">
-        <v>813</v>
+        <v>70</v>
       </c>
       <c r="D378" s="0">
-        <v>1080</v>
+        <v>10522</v>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="0" t="s">
+        <v>813</v>
+      </c>
+      <c r="B379" s="0" t="s">
         <v>814</v>
       </c>
-      <c r="B379" s="0" t="s">
-        <v>815</v>
-      </c>
       <c r="C379" s="0" t="s">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="D379" s="0">
-        <v>586.49</v>
+        <v>19481</v>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="0" t="s">
+        <v>815</v>
+      </c>
+      <c r="B380" s="0" t="s">
         <v>816</v>
       </c>
-      <c r="B380" s="0" t="s">
+      <c r="C380" s="0" t="s">
         <v>817</v>
       </c>
-      <c r="C380" s="0" t="s">
-        <v>818</v>
-      </c>
       <c r="D380" s="0">
-        <v>520</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="0" t="s">
+        <v>818</v>
+      </c>
+      <c r="B381" s="0" t="s">
         <v>819</v>
       </c>
-      <c r="B381" s="0" t="s">
-        <v>820</v>
-      </c>
       <c r="C381" s="0" t="s">
-        <v>818</v>
+        <v>18</v>
       </c>
       <c r="D381" s="0">
-        <v>300</v>
+        <v>586.49</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="0" t="s">
+        <v>820</v>
+      </c>
+      <c r="B382" s="0" t="s">
         <v>821</v>
       </c>
-      <c r="B382" s="0" t="s">
+      <c r="C382" s="0" t="s">
         <v>822</v>
       </c>
-      <c r="C382" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="D382" s="0">
-        <v>2200</v>
+        <v>520</v>
       </c>
     </row>
     <row r="383">
@@ -8633,10 +8645,10 @@
         <v>824</v>
       </c>
       <c r="C383" s="0" t="s">
-        <v>15</v>
+        <v>822</v>
       </c>
       <c r="D383" s="0">
-        <v>2800</v>
+        <v>300</v>
       </c>
     </row>
     <row r="384">
@@ -8647,10 +8659,10 @@
         <v>826</v>
       </c>
       <c r="C384" s="0" t="s">
-        <v>92</v>
+        <v>15</v>
       </c>
       <c r="D384" s="0">
-        <v>4924.7</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="385">
@@ -8661,10 +8673,10 @@
         <v>828</v>
       </c>
       <c r="C385" s="0" t="s">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="D385" s="0">
-        <v>2969</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="386">
@@ -8675,10 +8687,10 @@
         <v>830</v>
       </c>
       <c r="C386" s="0" t="s">
-        <v>34</v>
+        <v>92</v>
       </c>
       <c r="D386" s="0">
-        <v>3800</v>
+        <v>4924.7</v>
       </c>
     </row>
     <row r="387">
@@ -8689,10 +8701,10 @@
         <v>832</v>
       </c>
       <c r="C387" s="0" t="s">
-        <v>15</v>
+        <v>70</v>
       </c>
       <c r="D387" s="0">
-        <v>4000</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="388">
@@ -8703,7 +8715,7 @@
         <v>834</v>
       </c>
       <c r="C388" s="0" t="s">
-        <v>835</v>
+        <v>34</v>
       </c>
       <c r="D388" s="0">
         <v>3800</v>
@@ -8711,30 +8723,30 @@
     </row>
     <row r="389">
       <c r="A389" s="0" t="s">
+        <v>835</v>
+      </c>
+      <c r="B389" s="0" t="s">
         <v>836</v>
       </c>
-      <c r="B389" s="0" t="s">
-        <v>837</v>
-      </c>
       <c r="C389" s="0" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D389" s="0">
-        <v>353</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="0" t="s">
+        <v>837</v>
+      </c>
+      <c r="B390" s="0" t="s">
         <v>838</v>
       </c>
-      <c r="B390" s="0" t="s">
+      <c r="C390" s="0" t="s">
         <v>839</v>
       </c>
-      <c r="C390" s="0" t="s">
-        <v>110</v>
-      </c>
       <c r="D390" s="0">
-        <v>1800</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="391">
@@ -8745,10 +8757,10 @@
         <v>841</v>
       </c>
       <c r="C391" s="0" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D391" s="0">
-        <v>2948</v>
+        <v>353</v>
       </c>
     </row>
     <row r="392">
@@ -8759,10 +8771,10 @@
         <v>843</v>
       </c>
       <c r="C392" s="0" t="s">
-        <v>92</v>
+        <v>110</v>
       </c>
       <c r="D392" s="0">
-        <v>146</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="393">
@@ -8773,10 +8785,10 @@
         <v>845</v>
       </c>
       <c r="C393" s="0" t="s">
-        <v>207</v>
+        <v>15</v>
       </c>
       <c r="D393" s="0">
-        <v>65537</v>
+        <v>2948</v>
       </c>
     </row>
     <row r="394">
@@ -8787,10 +8799,10 @@
         <v>847</v>
       </c>
       <c r="C394" s="0" t="s">
-        <v>140</v>
+        <v>92</v>
       </c>
       <c r="D394" s="0">
-        <v>4130.4</v>
+        <v>146</v>
       </c>
     </row>
     <row r="395">
@@ -8801,10 +8813,10 @@
         <v>849</v>
       </c>
       <c r="C395" s="0" t="s">
-        <v>140</v>
+        <v>207</v>
       </c>
       <c r="D395" s="0">
-        <v>4283</v>
+        <v>65537</v>
       </c>
     </row>
     <row r="396">
@@ -8818,7 +8830,7 @@
         <v>140</v>
       </c>
       <c r="D396" s="0">
-        <v>6524.8</v>
+        <v>4130.4</v>
       </c>
     </row>
     <row r="397">
@@ -8829,10 +8841,10 @@
         <v>853</v>
       </c>
       <c r="C397" s="0" t="s">
-        <v>308</v>
+        <v>140</v>
       </c>
       <c r="D397" s="0">
-        <v>570</v>
+        <v>4283</v>
       </c>
     </row>
     <row r="398">
@@ -8843,10 +8855,10 @@
         <v>855</v>
       </c>
       <c r="C398" s="0" t="s">
-        <v>70</v>
+        <v>140</v>
       </c>
       <c r="D398" s="0">
-        <v>550</v>
+        <v>6524.8</v>
       </c>
     </row>
     <row r="399">
@@ -8857,10 +8869,10 @@
         <v>857</v>
       </c>
       <c r="C399" s="0" t="s">
-        <v>52</v>
+        <v>308</v>
       </c>
       <c r="D399" s="0">
-        <v>167</v>
+        <v>570</v>
       </c>
     </row>
     <row r="400">
@@ -8871,10 +8883,10 @@
         <v>859</v>
       </c>
       <c r="C400" s="0" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="D400" s="0">
-        <v>714.74</v>
+        <v>550</v>
       </c>
     </row>
     <row r="401">
@@ -8885,10 +8897,10 @@
         <v>861</v>
       </c>
       <c r="C401" s="0" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="D401" s="0">
-        <v>101000</v>
+        <v>167</v>
       </c>
     </row>
     <row r="402">
@@ -8899,10 +8911,10 @@
         <v>863</v>
       </c>
       <c r="C402" s="0" t="s">
-        <v>123</v>
+        <v>28</v>
       </c>
       <c r="D402" s="0">
-        <v>6251</v>
+        <v>714.74</v>
       </c>
     </row>
     <row r="403">
@@ -8913,10 +8925,10 @@
         <v>865</v>
       </c>
       <c r="C403" s="0" t="s">
-        <v>376</v>
+        <v>59</v>
       </c>
       <c r="D403" s="0">
-        <v>857.67</v>
+        <v>101000</v>
       </c>
     </row>
     <row r="404">
@@ -8927,10 +8939,10 @@
         <v>867</v>
       </c>
       <c r="C404" s="0" t="s">
-        <v>92</v>
+        <v>123</v>
       </c>
       <c r="D404" s="0">
-        <v>1164.66</v>
+        <v>6251</v>
       </c>
     </row>
     <row r="405">
@@ -8941,10 +8953,10 @@
         <v>869</v>
       </c>
       <c r="C405" s="0" t="s">
-        <v>151</v>
+        <v>376</v>
       </c>
       <c r="D405" s="0">
-        <v>360</v>
+        <v>857.67</v>
       </c>
     </row>
     <row r="406">
@@ -8955,10 +8967,10 @@
         <v>871</v>
       </c>
       <c r="C406" s="0" t="s">
-        <v>151</v>
+        <v>92</v>
       </c>
       <c r="D406" s="0">
-        <v>450</v>
+        <v>1164.66</v>
       </c>
     </row>
     <row r="407">
@@ -8972,7 +8984,7 @@
         <v>151</v>
       </c>
       <c r="D407" s="0">
-        <v>2150</v>
+        <v>360</v>
       </c>
     </row>
     <row r="408">
@@ -8983,10 +8995,10 @@
         <v>875</v>
       </c>
       <c r="C408" s="0" t="s">
-        <v>576</v>
+        <v>151</v>
       </c>
       <c r="D408" s="0">
-        <v>25192.82</v>
+        <v>450</v>
       </c>
     </row>
     <row r="409">
@@ -8997,10 +9009,10 @@
         <v>877</v>
       </c>
       <c r="C409" s="0" t="s">
-        <v>70</v>
+        <v>151</v>
       </c>
       <c r="D409" s="0">
-        <v>3500</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="410">
@@ -9011,10 +9023,10 @@
         <v>879</v>
       </c>
       <c r="C410" s="0" t="s">
-        <v>175</v>
+        <v>580</v>
       </c>
       <c r="D410" s="0">
-        <v>600</v>
+        <v>25192.82</v>
       </c>
     </row>
     <row r="411">
@@ -9025,38 +9037,38 @@
         <v>881</v>
       </c>
       <c r="C411" s="0" t="s">
-        <v>882</v>
+        <v>70</v>
       </c>
       <c r="D411" s="0">
-        <v>1080</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="0" t="s">
+        <v>882</v>
+      </c>
+      <c r="B412" s="0" t="s">
         <v>883</v>
       </c>
-      <c r="B412" s="0" t="s">
-        <v>884</v>
-      </c>
       <c r="C412" s="0" t="s">
-        <v>338</v>
+        <v>175</v>
       </c>
       <c r="D412" s="0">
-        <v>8628</v>
+        <v>600</v>
       </c>
     </row>
     <row r="413">
       <c r="A413" s="0" t="s">
+        <v>884</v>
+      </c>
+      <c r="B413" s="0" t="s">
         <v>885</v>
       </c>
-      <c r="B413" s="0" t="s">
+      <c r="C413" s="0" t="s">
         <v>886</v>
       </c>
-      <c r="C413" s="0" t="s">
-        <v>40</v>
-      </c>
       <c r="D413" s="0">
-        <v>27991.54</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="414">
@@ -9067,10 +9079,10 @@
         <v>888</v>
       </c>
       <c r="C414" s="0" t="s">
-        <v>140</v>
+        <v>338</v>
       </c>
       <c r="D414" s="0">
-        <v>1020</v>
+        <v>8628</v>
       </c>
     </row>
     <row r="415">
@@ -9081,10 +9093,10 @@
         <v>890</v>
       </c>
       <c r="C415" s="0" t="s">
-        <v>140</v>
+        <v>40</v>
       </c>
       <c r="D415" s="0">
-        <v>4106</v>
+        <v>27991.54</v>
       </c>
     </row>
     <row r="416">
@@ -9095,10 +9107,10 @@
         <v>892</v>
       </c>
       <c r="C416" s="0" t="s">
-        <v>45</v>
+        <v>140</v>
       </c>
       <c r="D416" s="0">
-        <v>6344.43</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="417">
@@ -9109,10 +9121,10 @@
         <v>894</v>
       </c>
       <c r="C417" s="0" t="s">
-        <v>45</v>
+        <v>140</v>
       </c>
       <c r="D417" s="0">
-        <v>2862.28</v>
+        <v>4106</v>
       </c>
     </row>
     <row r="418">
@@ -9126,7 +9138,7 @@
         <v>45</v>
       </c>
       <c r="D418" s="0">
-        <v>2131.18</v>
+        <v>6344.43</v>
       </c>
     </row>
     <row r="419">
@@ -9140,7 +9152,7 @@
         <v>45</v>
       </c>
       <c r="D419" s="0">
-        <v>29795.68</v>
+        <v>2862.28</v>
       </c>
     </row>
     <row r="420">
@@ -9154,7 +9166,7 @@
         <v>45</v>
       </c>
       <c r="D420" s="0">
-        <v>2307.09</v>
+        <v>2131.18</v>
       </c>
     </row>
     <row r="421">
@@ -9168,7 +9180,7 @@
         <v>45</v>
       </c>
       <c r="D421" s="0">
-        <v>5249.48</v>
+        <v>29795.68</v>
       </c>
     </row>
     <row r="422">
@@ -9182,7 +9194,7 @@
         <v>45</v>
       </c>
       <c r="D422" s="0">
-        <v>4399.56</v>
+        <v>2307.09</v>
       </c>
     </row>
     <row r="423">
@@ -9193,10 +9205,10 @@
         <v>906</v>
       </c>
       <c r="C423" s="0" t="s">
-        <v>478</v>
+        <v>45</v>
       </c>
       <c r="D423" s="0">
-        <v>510</v>
+        <v>5249.48</v>
       </c>
     </row>
     <row r="424">
@@ -9207,10 +9219,10 @@
         <v>908</v>
       </c>
       <c r="C424" s="0" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="D424" s="0">
-        <v>510</v>
+        <v>4399.56</v>
       </c>
     </row>
     <row r="425">
@@ -9221,35 +9233,35 @@
         <v>910</v>
       </c>
       <c r="C425" s="0" t="s">
-        <v>911</v>
+        <v>478</v>
       </c>
       <c r="D425" s="0">
-        <v>580</v>
+        <v>510</v>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="0" t="s">
+        <v>911</v>
+      </c>
+      <c r="B426" s="0" t="s">
         <v>912</v>
       </c>
-      <c r="B426" s="0" t="s">
-        <v>913</v>
-      </c>
       <c r="C426" s="0" t="s">
-        <v>911</v>
+        <v>37</v>
       </c>
       <c r="D426" s="0">
-        <v>580</v>
+        <v>510</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="0" t="s">
+        <v>913</v>
+      </c>
+      <c r="B427" s="0" t="s">
         <v>914</v>
       </c>
-      <c r="B427" s="0" t="s">
+      <c r="C427" s="0" t="s">
         <v>915</v>
-      </c>
-      <c r="C427" s="0" t="s">
-        <v>911</v>
       </c>
       <c r="D427" s="0">
         <v>580</v>
@@ -9263,10 +9275,10 @@
         <v>917</v>
       </c>
       <c r="C428" s="0" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
       <c r="D428" s="0">
-        <v>342</v>
+        <v>580</v>
       </c>
     </row>
     <row r="429">
@@ -9277,10 +9289,10 @@
         <v>919</v>
       </c>
       <c r="C429" s="0" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
       <c r="D429" s="0">
-        <v>342</v>
+        <v>580</v>
       </c>
     </row>
     <row r="430">
@@ -9291,7 +9303,7 @@
         <v>921</v>
       </c>
       <c r="C430" s="0" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
       <c r="D430" s="0">
         <v>342</v>
@@ -9305,10 +9317,10 @@
         <v>923</v>
       </c>
       <c r="C431" s="0" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
       <c r="D431" s="0">
-        <v>0</v>
+        <v>342</v>
       </c>
     </row>
     <row r="432">
@@ -9319,10 +9331,10 @@
         <v>925</v>
       </c>
       <c r="C432" s="0" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
       <c r="D432" s="0">
-        <v>0</v>
+        <v>342</v>
       </c>
     </row>
     <row r="433">
@@ -9333,38 +9345,38 @@
         <v>927</v>
       </c>
       <c r="C433" s="0" t="s">
-        <v>928</v>
+        <v>915</v>
       </c>
       <c r="D433" s="0">
-        <v>453</v>
+        <v>0</v>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="0" t="s">
+        <v>928</v>
+      </c>
+      <c r="B434" s="0" t="s">
         <v>929</v>
       </c>
-      <c r="B434" s="0" t="s">
-        <v>930</v>
-      </c>
       <c r="C434" s="0" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
       <c r="D434" s="0">
-        <v>453</v>
+        <v>0</v>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="0" t="s">
+        <v>930</v>
+      </c>
+      <c r="B435" s="0" t="s">
         <v>931</v>
       </c>
-      <c r="B435" s="0" t="s">
+      <c r="C435" s="0" t="s">
         <v>932</v>
       </c>
-      <c r="C435" s="0" t="s">
-        <v>70</v>
-      </c>
       <c r="D435" s="0">
-        <v>19322</v>
+        <v>453</v>
       </c>
     </row>
     <row r="436">
@@ -9375,10 +9387,10 @@
         <v>934</v>
       </c>
       <c r="C436" s="0" t="s">
-        <v>34</v>
+        <v>915</v>
       </c>
       <c r="D436" s="0">
-        <v>430</v>
+        <v>453</v>
       </c>
     </row>
     <row r="437">
@@ -9389,10 +9401,10 @@
         <v>936</v>
       </c>
       <c r="C437" s="0" t="s">
-        <v>281</v>
+        <v>70</v>
       </c>
       <c r="D437" s="0">
-        <v>430</v>
+        <v>19322</v>
       </c>
     </row>
     <row r="438">
@@ -9403,10 +9415,10 @@
         <v>938</v>
       </c>
       <c r="C438" s="0" t="s">
-        <v>115</v>
+        <v>34</v>
       </c>
       <c r="D438" s="0">
-        <v>14000</v>
+        <v>430</v>
       </c>
     </row>
     <row r="439">
@@ -9417,10 +9429,10 @@
         <v>940</v>
       </c>
       <c r="C439" s="0" t="s">
-        <v>140</v>
+        <v>281</v>
       </c>
       <c r="D439" s="0">
-        <v>15400</v>
+        <v>430</v>
       </c>
     </row>
     <row r="440">
@@ -9431,10 +9443,10 @@
         <v>942</v>
       </c>
       <c r="C440" s="0" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="D440" s="0">
-        <v>266200</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="441">
@@ -9445,10 +9457,10 @@
         <v>944</v>
       </c>
       <c r="C441" s="0" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="D441" s="0">
-        <v>194991.5</v>
+        <v>15400</v>
       </c>
     </row>
     <row r="442">
@@ -9462,7 +9474,7 @@
         <v>92</v>
       </c>
       <c r="D442" s="0">
-        <v>289492.5</v>
+        <v>266200</v>
       </c>
     </row>
     <row r="443">
@@ -9473,38 +9485,38 @@
         <v>948</v>
       </c>
       <c r="C443" s="0" t="s">
-        <v>949</v>
+        <v>92</v>
       </c>
       <c r="D443" s="0">
-        <v>13722.52</v>
+        <v>194991.5</v>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="0" t="s">
+        <v>949</v>
+      </c>
+      <c r="B444" s="0" t="s">
         <v>950</v>
       </c>
-      <c r="B444" s="0" t="s">
-        <v>951</v>
-      </c>
       <c r="C444" s="0" t="s">
-        <v>949</v>
+        <v>92</v>
       </c>
       <c r="D444" s="0">
-        <v>15072</v>
+        <v>289492.5</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="0" t="s">
+        <v>951</v>
+      </c>
+      <c r="B445" s="0" t="s">
         <v>952</v>
       </c>
-      <c r="B445" s="0" t="s">
+      <c r="C445" s="0" t="s">
         <v>953</v>
       </c>
-      <c r="C445" s="0" t="s">
-        <v>949</v>
-      </c>
       <c r="D445" s="0">
-        <v>6555.64</v>
+        <v>13722.52</v>
       </c>
     </row>
     <row r="446">
@@ -9515,10 +9527,10 @@
         <v>955</v>
       </c>
       <c r="C446" s="0" t="s">
-        <v>949</v>
+        <v>953</v>
       </c>
       <c r="D446" s="0">
-        <v>8964.61</v>
+        <v>15072</v>
       </c>
     </row>
     <row r="447">
@@ -9529,10 +9541,10 @@
         <v>957</v>
       </c>
       <c r="C447" s="0" t="s">
-        <v>949</v>
+        <v>953</v>
       </c>
       <c r="D447" s="0">
-        <v>11735</v>
+        <v>6555.64</v>
       </c>
     </row>
     <row r="448">
@@ -9543,10 +9555,10 @@
         <v>959</v>
       </c>
       <c r="C448" s="0" t="s">
-        <v>70</v>
+        <v>953</v>
       </c>
       <c r="D448" s="0">
-        <v>4276</v>
+        <v>8964.61</v>
       </c>
     </row>
     <row r="449">
@@ -9557,10 +9569,10 @@
         <v>961</v>
       </c>
       <c r="C449" s="0" t="s">
-        <v>140</v>
+        <v>953</v>
       </c>
       <c r="D449" s="0">
-        <v>3930</v>
+        <v>11735</v>
       </c>
     </row>
     <row r="450">
@@ -9571,10 +9583,10 @@
         <v>963</v>
       </c>
       <c r="C450" s="0" t="s">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="D450" s="0">
-        <v>4392.3</v>
+        <v>4276</v>
       </c>
     </row>
     <row r="451">
@@ -9585,38 +9597,38 @@
         <v>965</v>
       </c>
       <c r="C451" s="0" t="s">
-        <v>966</v>
+        <v>140</v>
       </c>
       <c r="D451" s="0">
-        <v>5254.41</v>
+        <v>3930</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="0" t="s">
+        <v>966</v>
+      </c>
+      <c r="B452" s="0" t="s">
         <v>967</v>
       </c>
-      <c r="B452" s="0" t="s">
-        <v>968</v>
-      </c>
       <c r="C452" s="0" t="s">
-        <v>52</v>
+        <v>92</v>
       </c>
       <c r="D452" s="0">
-        <v>1200</v>
+        <v>4392.3</v>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="0" t="s">
+        <v>968</v>
+      </c>
+      <c r="B453" s="0" t="s">
         <v>969</v>
       </c>
-      <c r="B453" s="0" t="s">
+      <c r="C453" s="0" t="s">
         <v>970</v>
       </c>
-      <c r="C453" s="0" t="s">
-        <v>52</v>
-      </c>
       <c r="D453" s="0">
-        <v>278</v>
+        <v>5254.41</v>
       </c>
     </row>
     <row r="454">
@@ -9630,7 +9642,7 @@
         <v>52</v>
       </c>
       <c r="D454" s="0">
-        <v>562</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="455">
@@ -9641,10 +9653,10 @@
         <v>974</v>
       </c>
       <c r="C455" s="0" t="s">
-        <v>376</v>
+        <v>52</v>
       </c>
       <c r="D455" s="0">
-        <v>65142.6</v>
+        <v>278</v>
       </c>
     </row>
     <row r="456">
@@ -9655,10 +9667,10 @@
         <v>976</v>
       </c>
       <c r="C456" s="0" t="s">
-        <v>376</v>
+        <v>52</v>
       </c>
       <c r="D456" s="0">
-        <v>23482.7</v>
+        <v>562</v>
       </c>
     </row>
     <row r="457">
@@ -9669,10 +9681,10 @@
         <v>978</v>
       </c>
       <c r="C457" s="0" t="s">
-        <v>28</v>
+        <v>376</v>
       </c>
       <c r="D457" s="0">
-        <v>6029.59</v>
+        <v>65142.6</v>
       </c>
     </row>
     <row r="458">
@@ -9683,10 +9695,10 @@
         <v>980</v>
       </c>
       <c r="C458" s="0" t="s">
-        <v>52</v>
+        <v>376</v>
       </c>
       <c r="D458" s="0">
-        <v>10985</v>
+        <v>23482.7</v>
       </c>
     </row>
     <row r="459">
@@ -9697,10 +9709,10 @@
         <v>982</v>
       </c>
       <c r="C459" s="0" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="D459" s="0">
-        <v>17425</v>
+        <v>6029.59</v>
       </c>
     </row>
     <row r="460">
@@ -9711,80 +9723,80 @@
         <v>984</v>
       </c>
       <c r="C460" s="0" t="s">
-        <v>985</v>
+        <v>52</v>
       </c>
       <c r="D460" s="0">
-        <v>1958</v>
+        <v>10985</v>
       </c>
     </row>
     <row r="461">
       <c r="A461" s="0" t="s">
+        <v>985</v>
+      </c>
+      <c r="B461" s="0" t="s">
         <v>986</v>
       </c>
-      <c r="B461" s="0" t="s">
-        <v>987</v>
-      </c>
       <c r="C461" s="0" t="s">
-        <v>988</v>
+        <v>52</v>
       </c>
       <c r="D461" s="0">
-        <v>2282.3</v>
+        <v>17425</v>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="0" t="s">
+        <v>987</v>
+      </c>
+      <c r="B462" s="0" t="s">
+        <v>988</v>
+      </c>
+      <c r="C462" s="0" t="s">
         <v>989</v>
       </c>
-      <c r="B462" s="0" t="s">
-        <v>990</v>
-      </c>
-      <c r="C462" s="0" t="s">
-        <v>991</v>
-      </c>
       <c r="D462" s="0">
-        <v>386</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="0" t="s">
+        <v>990</v>
+      </c>
+      <c r="B463" s="0" t="s">
+        <v>991</v>
+      </c>
+      <c r="C463" s="0" t="s">
         <v>992</v>
       </c>
-      <c r="B463" s="0" t="s">
-        <v>993</v>
-      </c>
-      <c r="C463" s="0" t="s">
-        <v>994</v>
-      </c>
       <c r="D463" s="0">
-        <v>385.4</v>
+        <v>2282.3</v>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="0" t="s">
+        <v>993</v>
+      </c>
+      <c r="B464" s="0" t="s">
+        <v>994</v>
+      </c>
+      <c r="C464" s="0" t="s">
         <v>995</v>
       </c>
-      <c r="B464" s="0" t="s">
-        <v>996</v>
-      </c>
-      <c r="C464" s="0" t="s">
-        <v>92</v>
-      </c>
       <c r="D464" s="0">
-        <v>296147.5</v>
+        <v>386</v>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="0" t="s">
+        <v>996</v>
+      </c>
+      <c r="B465" s="0" t="s">
         <v>997</v>
       </c>
-      <c r="B465" s="0" t="s">
+      <c r="C465" s="0" t="s">
         <v>998</v>
       </c>
-      <c r="C465" s="0" t="s">
-        <v>576</v>
-      </c>
       <c r="D465" s="0">
-        <v>71176.4</v>
+        <v>385.4</v>
       </c>
     </row>
     <row r="466">
@@ -9795,10 +9807,10 @@
         <v>1000</v>
       </c>
       <c r="C466" s="0" t="s">
-        <v>140</v>
+        <v>92</v>
       </c>
       <c r="D466" s="0">
-        <v>87</v>
+        <v>296147.5</v>
       </c>
     </row>
     <row r="467">
@@ -9809,10 +9821,10 @@
         <v>1002</v>
       </c>
       <c r="C467" s="0" t="s">
-        <v>70</v>
+        <v>580</v>
       </c>
       <c r="D467" s="0">
-        <v>950</v>
+        <v>71176.4</v>
       </c>
     </row>
     <row r="468">
@@ -9823,10 +9835,10 @@
         <v>1004</v>
       </c>
       <c r="C468" s="0" t="s">
-        <v>469</v>
+        <v>140</v>
       </c>
       <c r="D468" s="0">
-        <v>342641</v>
+        <v>87</v>
       </c>
     </row>
     <row r="469">
@@ -9837,10 +9849,10 @@
         <v>1006</v>
       </c>
       <c r="C469" s="0" t="s">
-        <v>160</v>
+        <v>70</v>
       </c>
       <c r="D469" s="0">
-        <v>2200</v>
+        <v>950</v>
       </c>
     </row>
     <row r="470">
@@ -9851,10 +9863,10 @@
         <v>1008</v>
       </c>
       <c r="C470" s="0" t="s">
-        <v>478</v>
+        <v>469</v>
       </c>
       <c r="D470" s="0">
-        <v>41000</v>
+        <v>342641</v>
       </c>
     </row>
     <row r="471">
@@ -9865,10 +9877,10 @@
         <v>1010</v>
       </c>
       <c r="C471" s="0" t="s">
-        <v>70</v>
+        <v>160</v>
       </c>
       <c r="D471" s="0">
-        <v>5790</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="472">
@@ -9879,10 +9891,10 @@
         <v>1012</v>
       </c>
       <c r="C472" s="0" t="s">
-        <v>911</v>
+        <v>478</v>
       </c>
       <c r="D472" s="0">
-        <v>880</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="473">
@@ -9893,10 +9905,10 @@
         <v>1014</v>
       </c>
       <c r="C473" s="0" t="s">
-        <v>911</v>
+        <v>70</v>
       </c>
       <c r="D473" s="0">
-        <v>880</v>
+        <v>5790</v>
       </c>
     </row>
     <row r="474">
@@ -9907,7 +9919,7 @@
         <v>1016</v>
       </c>
       <c r="C474" s="0" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
       <c r="D474" s="0">
         <v>880</v>
@@ -9921,10 +9933,10 @@
         <v>1018</v>
       </c>
       <c r="C475" s="0" t="s">
-        <v>21</v>
+        <v>915</v>
       </c>
       <c r="D475" s="0">
-        <v>563.36</v>
+        <v>880</v>
       </c>
     </row>
     <row r="476">
@@ -9935,10 +9947,10 @@
         <v>1020</v>
       </c>
       <c r="C476" s="0" t="s">
-        <v>15</v>
+        <v>915</v>
       </c>
       <c r="D476" s="0">
-        <v>3520</v>
+        <v>880</v>
       </c>
     </row>
     <row r="477">
@@ -9949,10 +9961,10 @@
         <v>1022</v>
       </c>
       <c r="C477" s="0" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D477" s="0">
-        <v>2600</v>
+        <v>563.36</v>
       </c>
     </row>
     <row r="478">
@@ -9963,10 +9975,10 @@
         <v>1024</v>
       </c>
       <c r="C478" s="0" t="s">
-        <v>281</v>
+        <v>15</v>
       </c>
       <c r="D478" s="0">
-        <v>3700</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="479">
@@ -9977,7 +9989,7 @@
         <v>1026</v>
       </c>
       <c r="C479" s="0" t="s">
-        <v>281</v>
+        <v>15</v>
       </c>
       <c r="D479" s="0">
         <v>2600</v>
@@ -9991,10 +10003,10 @@
         <v>1028</v>
       </c>
       <c r="C480" s="0" t="s">
-        <v>15</v>
+        <v>281</v>
       </c>
       <c r="D480" s="0">
-        <v>2235</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="481">
@@ -10005,10 +10017,10 @@
         <v>1030</v>
       </c>
       <c r="C481" s="0" t="s">
-        <v>15</v>
+        <v>281</v>
       </c>
       <c r="D481" s="0">
-        <v>3850</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="482">
@@ -10019,38 +10031,38 @@
         <v>1032</v>
       </c>
       <c r="C482" s="0" t="s">
-        <v>1033</v>
+        <v>15</v>
       </c>
       <c r="D482" s="0">
-        <v>1</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="0" t="s">
+        <v>1033</v>
+      </c>
+      <c r="B483" s="0" t="s">
         <v>1034</v>
       </c>
-      <c r="B483" s="0" t="s">
-        <v>1035</v>
-      </c>
       <c r="C483" s="0" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="D483" s="0">
-        <v>14819</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="0" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B484" s="0" t="s">
         <v>1036</v>
       </c>
-      <c r="B484" s="0" t="s">
+      <c r="C484" s="0" t="s">
         <v>1037</v>
       </c>
-      <c r="C484" s="0" t="s">
-        <v>376</v>
-      </c>
       <c r="D484" s="0">
-        <v>3859.93</v>
+        <v>1</v>
       </c>
     </row>
     <row r="485">
@@ -10061,10 +10073,10 @@
         <v>1039</v>
       </c>
       <c r="C485" s="0" t="s">
-        <v>376</v>
+        <v>28</v>
       </c>
       <c r="D485" s="0">
-        <v>11751.49</v>
+        <v>14819</v>
       </c>
     </row>
     <row r="486">
@@ -10075,10 +10087,10 @@
         <v>1041</v>
       </c>
       <c r="C486" s="0" t="s">
-        <v>338</v>
+        <v>376</v>
       </c>
       <c r="D486" s="0">
-        <v>6000</v>
+        <v>3859.93</v>
       </c>
     </row>
     <row r="487">
@@ -10089,10 +10101,10 @@
         <v>1043</v>
       </c>
       <c r="C487" s="0" t="s">
-        <v>338</v>
+        <v>376</v>
       </c>
       <c r="D487" s="0">
-        <v>3000</v>
+        <v>11751.49</v>
       </c>
     </row>
     <row r="488">
@@ -10103,10 +10115,10 @@
         <v>1045</v>
       </c>
       <c r="C488" s="0" t="s">
-        <v>37</v>
+        <v>338</v>
       </c>
       <c r="D488" s="0">
-        <v>618</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="489">
@@ -10117,38 +10129,38 @@
         <v>1047</v>
       </c>
       <c r="C489" s="0" t="s">
-        <v>1048</v>
+        <v>338</v>
       </c>
       <c r="D489" s="0">
-        <v>24600</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="490">
       <c r="A490" s="0" t="s">
+        <v>1048</v>
+      </c>
+      <c r="B490" s="0" t="s">
         <v>1049</v>
       </c>
-      <c r="B490" s="0" t="s">
-        <v>1050</v>
-      </c>
       <c r="C490" s="0" t="s">
-        <v>105</v>
+        <v>37</v>
       </c>
       <c r="D490" s="0">
-        <v>0</v>
+        <v>618</v>
       </c>
     </row>
     <row r="491">
       <c r="A491" s="0" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B491" s="0" t="s">
         <v>1051</v>
       </c>
-      <c r="B491" s="0" t="s">
+      <c r="C491" s="0" t="s">
         <v>1052</v>
       </c>
-      <c r="C491" s="0" t="s">
-        <v>92</v>
-      </c>
       <c r="D491" s="0">
-        <v>41593.75</v>
+        <v>24600</v>
       </c>
     </row>
     <row r="492">
@@ -10159,10 +10171,10 @@
         <v>1054</v>
       </c>
       <c r="C492" s="0" t="s">
-        <v>469</v>
+        <v>105</v>
       </c>
       <c r="D492" s="0">
-        <v>207558.07</v>
+        <v>0</v>
       </c>
     </row>
     <row r="493">
@@ -10173,10 +10185,10 @@
         <v>1056</v>
       </c>
       <c r="C493" s="0" t="s">
-        <v>376</v>
+        <v>92</v>
       </c>
       <c r="D493" s="0">
-        <v>77429.29</v>
+        <v>41593.75</v>
       </c>
     </row>
     <row r="494">
@@ -10187,10 +10199,10 @@
         <v>1058</v>
       </c>
       <c r="C494" s="0" t="s">
-        <v>376</v>
+        <v>469</v>
       </c>
       <c r="D494" s="0">
-        <v>42913.42</v>
+        <v>207558.07</v>
       </c>
     </row>
     <row r="495">
@@ -10204,7 +10216,7 @@
         <v>376</v>
       </c>
       <c r="D495" s="0">
-        <v>88806.25</v>
+        <v>77429.29</v>
       </c>
     </row>
     <row r="496">
@@ -10218,7 +10230,7 @@
         <v>376</v>
       </c>
       <c r="D496" s="0">
-        <v>50781.52</v>
+        <v>42913.42</v>
       </c>
     </row>
     <row r="497">
@@ -10229,10 +10241,10 @@
         <v>1064</v>
       </c>
       <c r="C497" s="0" t="s">
-        <v>21</v>
+        <v>376</v>
       </c>
       <c r="D497" s="0">
-        <v>1600</v>
+        <v>88806.25</v>
       </c>
     </row>
     <row r="498">
@@ -10243,10 +10255,10 @@
         <v>1066</v>
       </c>
       <c r="C498" s="0" t="s">
-        <v>28</v>
+        <v>376</v>
       </c>
       <c r="D498" s="0">
-        <v>3455.8</v>
+        <v>50781.52</v>
       </c>
     </row>
     <row r="499">
@@ -10257,10 +10269,10 @@
         <v>1068</v>
       </c>
       <c r="C499" s="0" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D499" s="0">
-        <v>3987</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="500">
@@ -10274,7 +10286,7 @@
         <v>28</v>
       </c>
       <c r="D500" s="0">
-        <v>4010.17</v>
+        <v>3455.8</v>
       </c>
     </row>
     <row r="501">
@@ -10288,7 +10300,7 @@
         <v>28</v>
       </c>
       <c r="D501" s="0">
-        <v>3382.65</v>
+        <v>3987</v>
       </c>
     </row>
     <row r="502">
@@ -10299,10 +10311,10 @@
         <v>1074</v>
       </c>
       <c r="C502" s="0" t="s">
-        <v>160</v>
+        <v>28</v>
       </c>
       <c r="D502" s="0">
-        <v>430</v>
+        <v>4010.17</v>
       </c>
     </row>
     <row r="503">
@@ -10313,9 +10325,37 @@
         <v>1076</v>
       </c>
       <c r="C503" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="D503" s="0">
+        <v>3382.65</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="0" t="s">
+        <v>1077</v>
+      </c>
+      <c r="B504" s="0" t="s">
+        <v>1078</v>
+      </c>
+      <c r="C504" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="D504" s="0">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="0" t="s">
+        <v>1079</v>
+      </c>
+      <c r="B505" s="0" t="s">
+        <v>1080</v>
+      </c>
+      <c r="C505" s="0" t="s">
         <v>140</v>
       </c>
-      <c r="D503" s="0">
+      <c r="D505" s="0">
         <v>465</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: stock y precios actualizados jue 03/09/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -3832,7 +3832,7 @@
         <v>92</v>
       </c>
       <c r="D39" s="0">
-        <v>21961.5</v>
+        <v>22627</v>
       </c>
     </row>
     <row r="40">
@@ -4028,7 +4028,7 @@
         <v>92</v>
       </c>
       <c r="D53" s="0">
-        <v>34606</v>
+        <v>35271.5</v>
       </c>
     </row>
     <row r="54">
@@ -4938,7 +4938,7 @@
         <v>92</v>
       </c>
       <c r="D118" s="0">
-        <v>10648</v>
+        <v>11313.5</v>
       </c>
     </row>
     <row r="119">
@@ -7626,7 +7626,7 @@
         <v>92</v>
       </c>
       <c r="D310" s="0">
-        <v>319440</v>
+        <v>332750</v>
       </c>
     </row>
     <row r="311">
@@ -8690,7 +8690,7 @@
         <v>92</v>
       </c>
       <c r="D386" s="0">
-        <v>4924.7</v>
+        <v>5190.9</v>
       </c>
     </row>
     <row r="387">
@@ -8802,7 +8802,7 @@
         <v>92</v>
       </c>
       <c r="D394" s="0">
-        <v>146</v>
+        <v>146.41</v>
       </c>
     </row>
     <row r="395">
@@ -10188,7 +10188,7 @@
         <v>92</v>
       </c>
       <c r="D493" s="0">
-        <v>41593.75</v>
+        <v>43590.25</v>
       </c>
     </row>
     <row r="494">

</xml_diff>

<commit_message>
sync: lista de precios actualizada - agrega SOL.FISIOLOGICA CELTYC
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="1081">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="1083">
   <si>
     <t>Solo Activos</t>
   </si>
@@ -2697,6 +2697,12 @@
   </si>
   <si>
     <t>SITROX Ext. 200mg /5ml Oral Polvo p/ Susp. x 15ml - 000010613</t>
+  </si>
+  <si>
+    <t>990100364</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOL.FISIOLOGICA AMP.X  5 ML  - CELTYC - 990100364</t>
   </si>
   <si>
     <t>456458987</t>
@@ -3320,7 +3326,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:D505"/>
+  <dimension ref="A2:D506"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -9135,10 +9141,10 @@
         <v>896</v>
       </c>
       <c r="C418" s="0" t="s">
-        <v>45</v>
+        <v>281</v>
       </c>
       <c r="D418" s="0">
-        <v>6344.43</v>
+        <v>450</v>
       </c>
     </row>
     <row r="419">
@@ -9152,7 +9158,7 @@
         <v>45</v>
       </c>
       <c r="D419" s="0">
-        <v>2862.28</v>
+        <v>6344.43</v>
       </c>
     </row>
     <row r="420">
@@ -9166,7 +9172,7 @@
         <v>45</v>
       </c>
       <c r="D420" s="0">
-        <v>2131.18</v>
+        <v>2862.28</v>
       </c>
     </row>
     <row r="421">
@@ -9180,7 +9186,7 @@
         <v>45</v>
       </c>
       <c r="D421" s="0">
-        <v>29795.68</v>
+        <v>2131.18</v>
       </c>
     </row>
     <row r="422">
@@ -9194,7 +9200,7 @@
         <v>45</v>
       </c>
       <c r="D422" s="0">
-        <v>2307.09</v>
+        <v>29795.68</v>
       </c>
     </row>
     <row r="423">
@@ -9208,7 +9214,7 @@
         <v>45</v>
       </c>
       <c r="D423" s="0">
-        <v>5249.48</v>
+        <v>2307.09</v>
       </c>
     </row>
     <row r="424">
@@ -9222,7 +9228,7 @@
         <v>45</v>
       </c>
       <c r="D424" s="0">
-        <v>4399.56</v>
+        <v>5249.48</v>
       </c>
     </row>
     <row r="425">
@@ -9233,10 +9239,10 @@
         <v>910</v>
       </c>
       <c r="C425" s="0" t="s">
-        <v>478</v>
+        <v>45</v>
       </c>
       <c r="D425" s="0">
-        <v>510</v>
+        <v>4399.56</v>
       </c>
     </row>
     <row r="426">
@@ -9247,7 +9253,7 @@
         <v>912</v>
       </c>
       <c r="C426" s="0" t="s">
-        <v>37</v>
+        <v>478</v>
       </c>
       <c r="D426" s="0">
         <v>510</v>
@@ -9261,21 +9267,21 @@
         <v>914</v>
       </c>
       <c r="C427" s="0" t="s">
-        <v>915</v>
+        <v>37</v>
       </c>
       <c r="D427" s="0">
-        <v>580</v>
+        <v>510</v>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="0" t="s">
+        <v>915</v>
+      </c>
+      <c r="B428" s="0" t="s">
         <v>916</v>
       </c>
-      <c r="B428" s="0" t="s">
+      <c r="C428" s="0" t="s">
         <v>917</v>
-      </c>
-      <c r="C428" s="0" t="s">
-        <v>915</v>
       </c>
       <c r="D428" s="0">
         <v>580</v>
@@ -9289,7 +9295,7 @@
         <v>919</v>
       </c>
       <c r="C429" s="0" t="s">
-        <v>915</v>
+        <v>917</v>
       </c>
       <c r="D429" s="0">
         <v>580</v>
@@ -9303,10 +9309,10 @@
         <v>921</v>
       </c>
       <c r="C430" s="0" t="s">
-        <v>915</v>
+        <v>917</v>
       </c>
       <c r="D430" s="0">
-        <v>342</v>
+        <v>580</v>
       </c>
     </row>
     <row r="431">
@@ -9317,7 +9323,7 @@
         <v>923</v>
       </c>
       <c r="C431" s="0" t="s">
-        <v>915</v>
+        <v>917</v>
       </c>
       <c r="D431" s="0">
         <v>342</v>
@@ -9331,7 +9337,7 @@
         <v>925</v>
       </c>
       <c r="C432" s="0" t="s">
-        <v>915</v>
+        <v>917</v>
       </c>
       <c r="D432" s="0">
         <v>342</v>
@@ -9345,10 +9351,10 @@
         <v>927</v>
       </c>
       <c r="C433" s="0" t="s">
-        <v>915</v>
+        <v>917</v>
       </c>
       <c r="D433" s="0">
-        <v>0</v>
+        <v>342</v>
       </c>
     </row>
     <row r="434">
@@ -9359,7 +9365,7 @@
         <v>929</v>
       </c>
       <c r="C434" s="0" t="s">
-        <v>915</v>
+        <v>917</v>
       </c>
       <c r="D434" s="0">
         <v>0</v>
@@ -9373,21 +9379,21 @@
         <v>931</v>
       </c>
       <c r="C435" s="0" t="s">
-        <v>932</v>
+        <v>917</v>
       </c>
       <c r="D435" s="0">
-        <v>453</v>
+        <v>0</v>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="0" t="s">
+        <v>932</v>
+      </c>
+      <c r="B436" s="0" t="s">
         <v>933</v>
       </c>
-      <c r="B436" s="0" t="s">
+      <c r="C436" s="0" t="s">
         <v>934</v>
-      </c>
-      <c r="C436" s="0" t="s">
-        <v>915</v>
       </c>
       <c r="D436" s="0">
         <v>453</v>
@@ -9401,10 +9407,10 @@
         <v>936</v>
       </c>
       <c r="C437" s="0" t="s">
-        <v>70</v>
+        <v>917</v>
       </c>
       <c r="D437" s="0">
-        <v>19322</v>
+        <v>453</v>
       </c>
     </row>
     <row r="438">
@@ -9415,10 +9421,10 @@
         <v>938</v>
       </c>
       <c r="C438" s="0" t="s">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="D438" s="0">
-        <v>430</v>
+        <v>19322</v>
       </c>
     </row>
     <row r="439">
@@ -9429,7 +9435,7 @@
         <v>940</v>
       </c>
       <c r="C439" s="0" t="s">
-        <v>281</v>
+        <v>34</v>
       </c>
       <c r="D439" s="0">
         <v>430</v>
@@ -9443,10 +9449,10 @@
         <v>942</v>
       </c>
       <c r="C440" s="0" t="s">
-        <v>115</v>
+        <v>281</v>
       </c>
       <c r="D440" s="0">
-        <v>14000</v>
+        <v>430</v>
       </c>
     </row>
     <row r="441">
@@ -9457,10 +9463,10 @@
         <v>944</v>
       </c>
       <c r="C441" s="0" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="D441" s="0">
-        <v>15400</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="442">
@@ -9471,10 +9477,10 @@
         <v>946</v>
       </c>
       <c r="C442" s="0" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="D442" s="0">
-        <v>266200</v>
+        <v>15400</v>
       </c>
     </row>
     <row r="443">
@@ -9488,7 +9494,7 @@
         <v>92</v>
       </c>
       <c r="D443" s="0">
-        <v>194991.5</v>
+        <v>266200</v>
       </c>
     </row>
     <row r="444">
@@ -9502,7 +9508,7 @@
         <v>92</v>
       </c>
       <c r="D444" s="0">
-        <v>289492.5</v>
+        <v>194991.5</v>
       </c>
     </row>
     <row r="445">
@@ -9513,24 +9519,24 @@
         <v>952</v>
       </c>
       <c r="C445" s="0" t="s">
-        <v>953</v>
+        <v>92</v>
       </c>
       <c r="D445" s="0">
-        <v>13722.52</v>
+        <v>289492.5</v>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="0" t="s">
+        <v>953</v>
+      </c>
+      <c r="B446" s="0" t="s">
         <v>954</v>
       </c>
-      <c r="B446" s="0" t="s">
+      <c r="C446" s="0" t="s">
         <v>955</v>
       </c>
-      <c r="C446" s="0" t="s">
-        <v>953</v>
-      </c>
       <c r="D446" s="0">
-        <v>15072</v>
+        <v>13722.52</v>
       </c>
     </row>
     <row r="447">
@@ -9541,10 +9547,10 @@
         <v>957</v>
       </c>
       <c r="C447" s="0" t="s">
-        <v>953</v>
+        <v>955</v>
       </c>
       <c r="D447" s="0">
-        <v>6555.64</v>
+        <v>15072</v>
       </c>
     </row>
     <row r="448">
@@ -9555,10 +9561,10 @@
         <v>959</v>
       </c>
       <c r="C448" s="0" t="s">
-        <v>953</v>
+        <v>955</v>
       </c>
       <c r="D448" s="0">
-        <v>8964.61</v>
+        <v>6555.64</v>
       </c>
     </row>
     <row r="449">
@@ -9569,10 +9575,10 @@
         <v>961</v>
       </c>
       <c r="C449" s="0" t="s">
-        <v>953</v>
+        <v>955</v>
       </c>
       <c r="D449" s="0">
-        <v>11735</v>
+        <v>8964.61</v>
       </c>
     </row>
     <row r="450">
@@ -9583,10 +9589,10 @@
         <v>963</v>
       </c>
       <c r="C450" s="0" t="s">
-        <v>70</v>
+        <v>955</v>
       </c>
       <c r="D450" s="0">
-        <v>4276</v>
+        <v>11735</v>
       </c>
     </row>
     <row r="451">
@@ -9597,10 +9603,10 @@
         <v>965</v>
       </c>
       <c r="C451" s="0" t="s">
-        <v>140</v>
+        <v>70</v>
       </c>
       <c r="D451" s="0">
-        <v>3930</v>
+        <v>4276</v>
       </c>
     </row>
     <row r="452">
@@ -9611,10 +9617,10 @@
         <v>967</v>
       </c>
       <c r="C452" s="0" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="D452" s="0">
-        <v>4392.3</v>
+        <v>3930</v>
       </c>
     </row>
     <row r="453">
@@ -9625,24 +9631,24 @@
         <v>969</v>
       </c>
       <c r="C453" s="0" t="s">
-        <v>970</v>
+        <v>92</v>
       </c>
       <c r="D453" s="0">
-        <v>5254.41</v>
+        <v>4392.3</v>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="0" t="s">
+        <v>970</v>
+      </c>
+      <c r="B454" s="0" t="s">
         <v>971</v>
       </c>
-      <c r="B454" s="0" t="s">
+      <c r="C454" s="0" t="s">
         <v>972</v>
       </c>
-      <c r="C454" s="0" t="s">
-        <v>52</v>
-      </c>
       <c r="D454" s="0">
-        <v>1200</v>
+        <v>5254.41</v>
       </c>
     </row>
     <row r="455">
@@ -9656,7 +9662,7 @@
         <v>52</v>
       </c>
       <c r="D455" s="0">
-        <v>278</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="456">
@@ -9670,7 +9676,7 @@
         <v>52</v>
       </c>
       <c r="D456" s="0">
-        <v>562</v>
+        <v>278</v>
       </c>
     </row>
     <row r="457">
@@ -9681,10 +9687,10 @@
         <v>978</v>
       </c>
       <c r="C457" s="0" t="s">
-        <v>376</v>
+        <v>52</v>
       </c>
       <c r="D457" s="0">
-        <v>65142.6</v>
+        <v>562</v>
       </c>
     </row>
     <row r="458">
@@ -9698,7 +9704,7 @@
         <v>376</v>
       </c>
       <c r="D458" s="0">
-        <v>23482.7</v>
+        <v>65142.6</v>
       </c>
     </row>
     <row r="459">
@@ -9709,10 +9715,10 @@
         <v>982</v>
       </c>
       <c r="C459" s="0" t="s">
-        <v>28</v>
+        <v>376</v>
       </c>
       <c r="D459" s="0">
-        <v>6029.59</v>
+        <v>23482.7</v>
       </c>
     </row>
     <row r="460">
@@ -9723,10 +9729,10 @@
         <v>984</v>
       </c>
       <c r="C460" s="0" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="D460" s="0">
-        <v>10985</v>
+        <v>6029.59</v>
       </c>
     </row>
     <row r="461">
@@ -9740,7 +9746,7 @@
         <v>52</v>
       </c>
       <c r="D461" s="0">
-        <v>17425</v>
+        <v>10985</v>
       </c>
     </row>
     <row r="462">
@@ -9751,66 +9757,66 @@
         <v>988</v>
       </c>
       <c r="C462" s="0" t="s">
-        <v>989</v>
+        <v>52</v>
       </c>
       <c r="D462" s="0">
-        <v>1958</v>
+        <v>17425</v>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="0" t="s">
+        <v>989</v>
+      </c>
+      <c r="B463" s="0" t="s">
         <v>990</v>
       </c>
-      <c r="B463" s="0" t="s">
+      <c r="C463" s="0" t="s">
         <v>991</v>
       </c>
-      <c r="C463" s="0" t="s">
-        <v>992</v>
-      </c>
       <c r="D463" s="0">
-        <v>2282.3</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="0" t="s">
+        <v>992</v>
+      </c>
+      <c r="B464" s="0" t="s">
         <v>993</v>
       </c>
-      <c r="B464" s="0" t="s">
+      <c r="C464" s="0" t="s">
         <v>994</v>
       </c>
-      <c r="C464" s="0" t="s">
-        <v>995</v>
-      </c>
       <c r="D464" s="0">
-        <v>386</v>
+        <v>2282.3</v>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="0" t="s">
+        <v>995</v>
+      </c>
+      <c r="B465" s="0" t="s">
         <v>996</v>
       </c>
-      <c r="B465" s="0" t="s">
+      <c r="C465" s="0" t="s">
         <v>997</v>
       </c>
-      <c r="C465" s="0" t="s">
-        <v>998</v>
-      </c>
       <c r="D465" s="0">
-        <v>385.4</v>
+        <v>386</v>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="0" t="s">
+        <v>998</v>
+      </c>
+      <c r="B466" s="0" t="s">
         <v>999</v>
       </c>
-      <c r="B466" s="0" t="s">
+      <c r="C466" s="0" t="s">
         <v>1000</v>
       </c>
-      <c r="C466" s="0" t="s">
-        <v>92</v>
-      </c>
       <c r="D466" s="0">
-        <v>296147.5</v>
+        <v>385.4</v>
       </c>
     </row>
     <row r="467">
@@ -9821,10 +9827,10 @@
         <v>1002</v>
       </c>
       <c r="C467" s="0" t="s">
-        <v>580</v>
+        <v>92</v>
       </c>
       <c r="D467" s="0">
-        <v>71176.4</v>
+        <v>296147.5</v>
       </c>
     </row>
     <row r="468">
@@ -9835,10 +9841,10 @@
         <v>1004</v>
       </c>
       <c r="C468" s="0" t="s">
-        <v>140</v>
+        <v>580</v>
       </c>
       <c r="D468" s="0">
-        <v>87</v>
+        <v>71176.4</v>
       </c>
     </row>
     <row r="469">
@@ -9849,10 +9855,10 @@
         <v>1006</v>
       </c>
       <c r="C469" s="0" t="s">
-        <v>70</v>
+        <v>140</v>
       </c>
       <c r="D469" s="0">
-        <v>950</v>
+        <v>87</v>
       </c>
     </row>
     <row r="470">
@@ -9863,10 +9869,10 @@
         <v>1008</v>
       </c>
       <c r="C470" s="0" t="s">
-        <v>469</v>
+        <v>70</v>
       </c>
       <c r="D470" s="0">
-        <v>342641</v>
+        <v>950</v>
       </c>
     </row>
     <row r="471">
@@ -9877,10 +9883,10 @@
         <v>1010</v>
       </c>
       <c r="C471" s="0" t="s">
-        <v>160</v>
+        <v>469</v>
       </c>
       <c r="D471" s="0">
-        <v>2200</v>
+        <v>342641</v>
       </c>
     </row>
     <row r="472">
@@ -9891,10 +9897,10 @@
         <v>1012</v>
       </c>
       <c r="C472" s="0" t="s">
-        <v>478</v>
+        <v>160</v>
       </c>
       <c r="D472" s="0">
-        <v>41000</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="473">
@@ -9905,10 +9911,10 @@
         <v>1014</v>
       </c>
       <c r="C473" s="0" t="s">
-        <v>70</v>
+        <v>478</v>
       </c>
       <c r="D473" s="0">
-        <v>5790</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="474">
@@ -9919,10 +9925,10 @@
         <v>1016</v>
       </c>
       <c r="C474" s="0" t="s">
-        <v>915</v>
+        <v>70</v>
       </c>
       <c r="D474" s="0">
-        <v>880</v>
+        <v>5790</v>
       </c>
     </row>
     <row r="475">
@@ -9933,7 +9939,7 @@
         <v>1018</v>
       </c>
       <c r="C475" s="0" t="s">
-        <v>915</v>
+        <v>917</v>
       </c>
       <c r="D475" s="0">
         <v>880</v>
@@ -9947,7 +9953,7 @@
         <v>1020</v>
       </c>
       <c r="C476" s="0" t="s">
-        <v>915</v>
+        <v>917</v>
       </c>
       <c r="D476" s="0">
         <v>880</v>
@@ -9961,10 +9967,10 @@
         <v>1022</v>
       </c>
       <c r="C477" s="0" t="s">
-        <v>21</v>
+        <v>917</v>
       </c>
       <c r="D477" s="0">
-        <v>563.36</v>
+        <v>880</v>
       </c>
     </row>
     <row r="478">
@@ -9975,10 +9981,10 @@
         <v>1024</v>
       </c>
       <c r="C478" s="0" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D478" s="0">
-        <v>3520</v>
+        <v>563.36</v>
       </c>
     </row>
     <row r="479">
@@ -9992,7 +9998,7 @@
         <v>15</v>
       </c>
       <c r="D479" s="0">
-        <v>2600</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="480">
@@ -10003,10 +10009,10 @@
         <v>1028</v>
       </c>
       <c r="C480" s="0" t="s">
-        <v>281</v>
+        <v>15</v>
       </c>
       <c r="D480" s="0">
-        <v>3700</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="481">
@@ -10020,7 +10026,7 @@
         <v>281</v>
       </c>
       <c r="D481" s="0">
-        <v>2600</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="482">
@@ -10031,10 +10037,10 @@
         <v>1032</v>
       </c>
       <c r="C482" s="0" t="s">
-        <v>15</v>
+        <v>281</v>
       </c>
       <c r="D482" s="0">
-        <v>2235</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="483">
@@ -10048,7 +10054,7 @@
         <v>15</v>
       </c>
       <c r="D483" s="0">
-        <v>3850</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="484">
@@ -10059,24 +10065,24 @@
         <v>1036</v>
       </c>
       <c r="C484" s="0" t="s">
-        <v>1037</v>
+        <v>15</v>
       </c>
       <c r="D484" s="0">
-        <v>1</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="0" t="s">
+        <v>1037</v>
+      </c>
+      <c r="B485" s="0" t="s">
         <v>1038</v>
       </c>
-      <c r="B485" s="0" t="s">
+      <c r="C485" s="0" t="s">
         <v>1039</v>
       </c>
-      <c r="C485" s="0" t="s">
-        <v>28</v>
-      </c>
       <c r="D485" s="0">
-        <v>14819</v>
+        <v>1</v>
       </c>
     </row>
     <row r="486">
@@ -10087,10 +10093,10 @@
         <v>1041</v>
       </c>
       <c r="C486" s="0" t="s">
-        <v>376</v>
+        <v>28</v>
       </c>
       <c r="D486" s="0">
-        <v>3859.93</v>
+        <v>14819</v>
       </c>
     </row>
     <row r="487">
@@ -10104,7 +10110,7 @@
         <v>376</v>
       </c>
       <c r="D487" s="0">
-        <v>11751.49</v>
+        <v>3859.93</v>
       </c>
     </row>
     <row r="488">
@@ -10115,10 +10121,10 @@
         <v>1045</v>
       </c>
       <c r="C488" s="0" t="s">
-        <v>338</v>
+        <v>376</v>
       </c>
       <c r="D488" s="0">
-        <v>6000</v>
+        <v>11751.49</v>
       </c>
     </row>
     <row r="489">
@@ -10132,7 +10138,7 @@
         <v>338</v>
       </c>
       <c r="D489" s="0">
-        <v>3000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="490">
@@ -10143,10 +10149,10 @@
         <v>1049</v>
       </c>
       <c r="C490" s="0" t="s">
-        <v>37</v>
+        <v>338</v>
       </c>
       <c r="D490" s="0">
-        <v>618</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="491">
@@ -10157,24 +10163,24 @@
         <v>1051</v>
       </c>
       <c r="C491" s="0" t="s">
-        <v>1052</v>
+        <v>37</v>
       </c>
       <c r="D491" s="0">
-        <v>24600</v>
+        <v>618</v>
       </c>
     </row>
     <row r="492">
       <c r="A492" s="0" t="s">
+        <v>1052</v>
+      </c>
+      <c r="B492" s="0" t="s">
         <v>1053</v>
       </c>
-      <c r="B492" s="0" t="s">
+      <c r="C492" s="0" t="s">
         <v>1054</v>
       </c>
-      <c r="C492" s="0" t="s">
-        <v>105</v>
-      </c>
       <c r="D492" s="0">
-        <v>0</v>
+        <v>24600</v>
       </c>
     </row>
     <row r="493">
@@ -10185,10 +10191,10 @@
         <v>1056</v>
       </c>
       <c r="C493" s="0" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="D493" s="0">
-        <v>43590.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="494">
@@ -10199,10 +10205,10 @@
         <v>1058</v>
       </c>
       <c r="C494" s="0" t="s">
-        <v>469</v>
+        <v>92</v>
       </c>
       <c r="D494" s="0">
-        <v>207558.07</v>
+        <v>43590.25</v>
       </c>
     </row>
     <row r="495">
@@ -10213,10 +10219,10 @@
         <v>1060</v>
       </c>
       <c r="C495" s="0" t="s">
-        <v>376</v>
+        <v>469</v>
       </c>
       <c r="D495" s="0">
-        <v>77429.29</v>
+        <v>207558.07</v>
       </c>
     </row>
     <row r="496">
@@ -10230,7 +10236,7 @@
         <v>376</v>
       </c>
       <c r="D496" s="0">
-        <v>42913.42</v>
+        <v>77429.29</v>
       </c>
     </row>
     <row r="497">
@@ -10244,7 +10250,7 @@
         <v>376</v>
       </c>
       <c r="D497" s="0">
-        <v>88806.25</v>
+        <v>42913.42</v>
       </c>
     </row>
     <row r="498">
@@ -10258,7 +10264,7 @@
         <v>376</v>
       </c>
       <c r="D498" s="0">
-        <v>50781.52</v>
+        <v>88806.25</v>
       </c>
     </row>
     <row r="499">
@@ -10269,10 +10275,10 @@
         <v>1068</v>
       </c>
       <c r="C499" s="0" t="s">
-        <v>21</v>
+        <v>376</v>
       </c>
       <c r="D499" s="0">
-        <v>1600</v>
+        <v>50781.52</v>
       </c>
     </row>
     <row r="500">
@@ -10283,10 +10289,10 @@
         <v>1070</v>
       </c>
       <c r="C500" s="0" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D500" s="0">
-        <v>3455.8</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="501">
@@ -10300,7 +10306,7 @@
         <v>28</v>
       </c>
       <c r="D501" s="0">
-        <v>3987</v>
+        <v>3455.8</v>
       </c>
     </row>
     <row r="502">
@@ -10314,7 +10320,7 @@
         <v>28</v>
       </c>
       <c r="D502" s="0">
-        <v>4010.17</v>
+        <v>3987</v>
       </c>
     </row>
     <row r="503">
@@ -10328,7 +10334,7 @@
         <v>28</v>
       </c>
       <c r="D503" s="0">
-        <v>3382.65</v>
+        <v>4010.17</v>
       </c>
     </row>
     <row r="504">
@@ -10339,10 +10345,10 @@
         <v>1078</v>
       </c>
       <c r="C504" s="0" t="s">
-        <v>160</v>
+        <v>28</v>
       </c>
       <c r="D504" s="0">
-        <v>430</v>
+        <v>3382.65</v>
       </c>
     </row>
     <row r="505">
@@ -10353,9 +10359,23 @@
         <v>1080</v>
       </c>
       <c r="C505" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="D505" s="0">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="0" t="s">
+        <v>1081</v>
+      </c>
+      <c r="B506" s="0" t="s">
+        <v>1082</v>
+      </c>
+      <c r="C506" s="0" t="s">
         <v>140</v>
       </c>
-      <c r="D505" s="0">
+      <c r="D506" s="0">
         <v>465</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: stock y precios actualizados sáb 05/09/2026
</commit_message>
<xml_diff>
--- a/price_list.xlsx
+++ b/price_list.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="1083">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="1087">
   <si>
     <t>Solo Activos</t>
   </si>
@@ -1538,7 +1538,7 @@
     <t>000023861</t>
   </si>
   <si>
-    <t xml:space="preserve">GUANTE DE NITRILO M -CJX100- S/POLVO NEGRO TOP GLOVE  - 000023861</t>
+    <t>GUANTE DE NITRILO M -CJX100- S/POLVO NEGRO TOP GLOVE - 000023861</t>
   </si>
   <si>
     <t>TOP GLOVE</t>
@@ -1985,6 +1985,12 @@
     <t>LAFELAX Jbe. x 120ml - 000013033</t>
   </si>
   <si>
+    <t>000024714</t>
+  </si>
+  <si>
+    <t>LAFEVIR 800mg Comp. x 10 - ACICLOVIR - LAFEDAR - 000024714</t>
+  </si>
+  <si>
     <t>000002001</t>
   </si>
   <si>
@@ -3021,6 +3027,12 @@
   </si>
   <si>
     <t>TIGECICLINA 50 MG INY. F. AMP. X 10 - 000023596</t>
+  </si>
+  <si>
+    <t>000024045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOFLAM OFT. SUSP. X   5 ML - 000024045</t>
   </si>
   <si>
     <t>000023618</t>
@@ -3326,7 +3338,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:D506"/>
+  <dimension ref="A2:D508"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -3600,7 +3612,7 @@
         <v>52</v>
       </c>
       <c r="D22" s="0">
-        <v>11</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="23">
@@ -3614,7 +3626,7 @@
         <v>52</v>
       </c>
       <c r="D23" s="0">
-        <v>11</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="24">
@@ -3628,7 +3640,7 @@
         <v>52</v>
       </c>
       <c r="D24" s="0">
-        <v>11</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="25">
@@ -4090,7 +4102,7 @@
         <v>52</v>
       </c>
       <c r="D57" s="0">
-        <v>102</v>
+        <v>110</v>
       </c>
     </row>
     <row r="58">
@@ -5812,7 +5824,7 @@
         <v>123</v>
       </c>
       <c r="D180" s="0">
-        <v>5100</v>
+        <v>5218</v>
       </c>
     </row>
     <row r="181">
@@ -6372,7 +6384,7 @@
         <v>52</v>
       </c>
       <c r="D220" s="0">
-        <v>4200</v>
+        <v>4670</v>
       </c>
     </row>
     <row r="221">
@@ -6386,7 +6398,7 @@
         <v>52</v>
       </c>
       <c r="D221" s="0">
-        <v>4200</v>
+        <v>4670</v>
       </c>
     </row>
     <row r="222">
@@ -6400,7 +6412,7 @@
         <v>52</v>
       </c>
       <c r="D222" s="0">
-        <v>4200</v>
+        <v>4670</v>
       </c>
     </row>
     <row r="223">
@@ -7184,7 +7196,7 @@
         <v>52</v>
       </c>
       <c r="D278" s="0">
-        <v>38.22</v>
+        <v>54.8</v>
       </c>
     </row>
     <row r="279">
@@ -7506,7 +7518,7 @@
         <v>123</v>
       </c>
       <c r="D301" s="0">
-        <v>2859.96</v>
+        <v>3016.53</v>
       </c>
     </row>
     <row r="302">
@@ -7531,24 +7543,24 @@
         <v>658</v>
       </c>
       <c r="C303" s="0" t="s">
-        <v>659</v>
+        <v>123</v>
       </c>
       <c r="D303" s="0">
-        <v>0</v>
+        <v>4450</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="0" t="s">
+        <v>659</v>
+      </c>
+      <c r="B304" s="0" t="s">
         <v>660</v>
       </c>
-      <c r="B304" s="0" t="s">
+      <c r="C304" s="0" t="s">
         <v>661</v>
       </c>
-      <c r="C304" s="0" t="s">
-        <v>28</v>
-      </c>
       <c r="D304" s="0">
-        <v>494</v>
+        <v>0</v>
       </c>
     </row>
     <row r="305">
@@ -7562,7 +7574,7 @@
         <v>28</v>
       </c>
       <c r="D305" s="0">
-        <v>665.3</v>
+        <v>494</v>
       </c>
     </row>
     <row r="306">
@@ -7573,10 +7585,10 @@
         <v>665</v>
       </c>
       <c r="C306" s="0" t="s">
-        <v>92</v>
+        <v>28</v>
       </c>
       <c r="D306" s="0">
-        <v>33940.5</v>
+        <v>665.3</v>
       </c>
     </row>
     <row r="307">
@@ -7590,7 +7602,7 @@
         <v>92</v>
       </c>
       <c r="D307" s="0">
-        <v>4525.4</v>
+        <v>33940.5</v>
       </c>
     </row>
     <row r="308">
@@ -7601,10 +7613,10 @@
         <v>669</v>
       </c>
       <c r="C308" s="0" t="s">
-        <v>151</v>
+        <v>92</v>
       </c>
       <c r="D308" s="0">
-        <v>896</v>
+        <v>4525.4</v>
       </c>
     </row>
     <row r="309">
@@ -7615,10 +7627,10 @@
         <v>671</v>
       </c>
       <c r="C309" s="0" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="D309" s="0">
-        <v>1250</v>
+        <v>896</v>
       </c>
     </row>
     <row r="310">
@@ -7629,10 +7641,10 @@
         <v>673</v>
       </c>
       <c r="C310" s="0" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="D310" s="0">
-        <v>332750</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="311">
@@ -7643,10 +7655,10 @@
         <v>675</v>
       </c>
       <c r="C311" s="0" t="s">
-        <v>202</v>
+        <v>92</v>
       </c>
       <c r="D311" s="0">
-        <v>17440</v>
+        <v>332750</v>
       </c>
     </row>
     <row r="312">
@@ -7660,7 +7672,7 @@
         <v>202</v>
       </c>
       <c r="D312" s="0">
-        <v>4390</v>
+        <v>17440</v>
       </c>
     </row>
     <row r="313">
@@ -7685,10 +7697,10 @@
         <v>681</v>
       </c>
       <c r="C314" s="0" t="s">
-        <v>281</v>
+        <v>202</v>
       </c>
       <c r="D314" s="0">
-        <v>2250</v>
+        <v>4390</v>
       </c>
     </row>
     <row r="315">
@@ -7699,10 +7711,10 @@
         <v>683</v>
       </c>
       <c r="C315" s="0" t="s">
-        <v>202</v>
+        <v>281</v>
       </c>
       <c r="D315" s="0">
-        <v>3355</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="316">
@@ -7713,10 +7725,10 @@
         <v>685</v>
       </c>
       <c r="C316" s="0" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="D316" s="0">
-        <v>7500</v>
+        <v>3355</v>
       </c>
     </row>
     <row r="317">
@@ -7727,10 +7739,10 @@
         <v>687</v>
       </c>
       <c r="C317" s="0" t="s">
-        <v>92</v>
+        <v>207</v>
       </c>
       <c r="D317" s="0">
-        <v>25289</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="318">
@@ -7744,7 +7756,7 @@
         <v>92</v>
       </c>
       <c r="D318" s="0">
-        <v>252890</v>
+        <v>25289</v>
       </c>
     </row>
     <row r="319">
@@ -7755,10 +7767,10 @@
         <v>691</v>
       </c>
       <c r="C319" s="0" t="s">
-        <v>52</v>
+        <v>92</v>
       </c>
       <c r="D319" s="0">
-        <v>130</v>
+        <v>252890</v>
       </c>
     </row>
     <row r="320">
@@ -7769,10 +7781,10 @@
         <v>693</v>
       </c>
       <c r="C320" s="0" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="D320" s="0">
-        <v>285.6</v>
+        <v>160</v>
       </c>
     </row>
     <row r="321">
@@ -7786,7 +7798,7 @@
         <v>21</v>
       </c>
       <c r="D321" s="0">
-        <v>338</v>
+        <v>285.6</v>
       </c>
     </row>
     <row r="322">
@@ -7797,21 +7809,21 @@
         <v>697</v>
       </c>
       <c r="C322" s="0" t="s">
-        <v>698</v>
+        <v>21</v>
       </c>
       <c r="D322" s="0">
-        <v>770</v>
+        <v>338</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="0" t="s">
+        <v>698</v>
+      </c>
+      <c r="B323" s="0" t="s">
         <v>699</v>
       </c>
-      <c r="B323" s="0" t="s">
+      <c r="C323" s="0" t="s">
         <v>700</v>
-      </c>
-      <c r="C323" s="0" t="s">
-        <v>701</v>
       </c>
       <c r="D323" s="0">
         <v>770</v>
@@ -7819,16 +7831,16 @@
     </row>
     <row r="324">
       <c r="A324" s="0" t="s">
+        <v>701</v>
+      </c>
+      <c r="B324" s="0" t="s">
         <v>702</v>
       </c>
-      <c r="B324" s="0" t="s">
+      <c r="C324" s="0" t="s">
         <v>703</v>
       </c>
-      <c r="C324" s="0" t="s">
-        <v>15</v>
-      </c>
       <c r="D324" s="0">
-        <v>973.5</v>
+        <v>770</v>
       </c>
     </row>
     <row r="325">
@@ -7839,10 +7851,10 @@
         <v>705</v>
       </c>
       <c r="C325" s="0" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D325" s="0">
-        <v>507.08</v>
+        <v>973.5</v>
       </c>
     </row>
     <row r="326">
@@ -7853,10 +7865,10 @@
         <v>707</v>
       </c>
       <c r="C326" s="0" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D326" s="0">
-        <v>450</v>
+        <v>507.08</v>
       </c>
     </row>
     <row r="327">
@@ -7867,10 +7879,10 @@
         <v>709</v>
       </c>
       <c r="C327" s="0" t="s">
-        <v>151</v>
+        <v>15</v>
       </c>
       <c r="D327" s="0">
-        <v>760</v>
+        <v>450</v>
       </c>
     </row>
     <row r="328">
@@ -7881,10 +7893,10 @@
         <v>711</v>
       </c>
       <c r="C328" s="0" t="s">
-        <v>281</v>
+        <v>151</v>
       </c>
       <c r="D328" s="0">
-        <v>5900</v>
+        <v>760</v>
       </c>
     </row>
     <row r="329">
@@ -7898,7 +7910,7 @@
         <v>281</v>
       </c>
       <c r="D329" s="0">
-        <v>2900</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="330">
@@ -7909,10 +7921,10 @@
         <v>715</v>
       </c>
       <c r="C330" s="0" t="s">
-        <v>140</v>
+        <v>281</v>
       </c>
       <c r="D330" s="0">
-        <v>890</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="331">
@@ -7926,7 +7938,7 @@
         <v>140</v>
       </c>
       <c r="D331" s="0">
-        <v>594</v>
+        <v>890</v>
       </c>
     </row>
     <row r="332">
@@ -7940,7 +7952,7 @@
         <v>140</v>
       </c>
       <c r="D332" s="0">
-        <v>65</v>
+        <v>594</v>
       </c>
     </row>
     <row r="333">
@@ -7951,10 +7963,10 @@
         <v>721</v>
       </c>
       <c r="C333" s="0" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="D333" s="0">
-        <v>11313.5</v>
+        <v>65</v>
       </c>
     </row>
     <row r="334">
@@ -7965,10 +7977,10 @@
         <v>723</v>
       </c>
       <c r="C334" s="0" t="s">
-        <v>34</v>
+        <v>92</v>
       </c>
       <c r="D334" s="0">
-        <v>420</v>
+        <v>11313.5</v>
       </c>
     </row>
     <row r="335">
@@ -7979,10 +7991,10 @@
         <v>725</v>
       </c>
       <c r="C335" s="0" t="s">
-        <v>359</v>
+        <v>34</v>
       </c>
       <c r="D335" s="0">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="336">
@@ -7993,10 +8005,10 @@
         <v>727</v>
       </c>
       <c r="C336" s="0" t="s">
-        <v>21</v>
+        <v>359</v>
       </c>
       <c r="D336" s="0">
-        <v>377</v>
+        <v>418</v>
       </c>
     </row>
     <row r="337">
@@ -8007,10 +8019,10 @@
         <v>729</v>
       </c>
       <c r="C337" s="0" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="D337" s="0">
-        <v>5780.66</v>
+        <v>377</v>
       </c>
     </row>
     <row r="338">
@@ -8021,10 +8033,10 @@
         <v>731</v>
       </c>
       <c r="C338" s="0" t="s">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="D338" s="0">
-        <v>898</v>
+        <v>5780.66</v>
       </c>
     </row>
     <row r="339">
@@ -8035,10 +8047,10 @@
         <v>733</v>
       </c>
       <c r="C339" s="0" t="s">
-        <v>123</v>
+        <v>70</v>
       </c>
       <c r="D339" s="0">
-        <v>4767</v>
+        <v>898</v>
       </c>
     </row>
     <row r="340">
@@ -8049,10 +8061,10 @@
         <v>735</v>
       </c>
       <c r="C340" s="0" t="s">
-        <v>34</v>
+        <v>123</v>
       </c>
       <c r="D340" s="0">
-        <v>650</v>
+        <v>4767</v>
       </c>
     </row>
     <row r="341">
@@ -8063,7 +8075,7 @@
         <v>737</v>
       </c>
       <c r="C341" s="0" t="s">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="D341" s="0">
         <v>650</v>
@@ -8077,10 +8089,10 @@
         <v>739</v>
       </c>
       <c r="C342" s="0" t="s">
-        <v>15</v>
+        <v>70</v>
       </c>
       <c r="D342" s="0">
-        <v>2178</v>
+        <v>650</v>
       </c>
     </row>
     <row r="343">
@@ -8091,10 +8103,10 @@
         <v>741</v>
       </c>
       <c r="C343" s="0" t="s">
-        <v>92</v>
+        <v>15</v>
       </c>
       <c r="D343" s="0">
-        <v>7986</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="344">
@@ -8105,24 +8117,24 @@
         <v>743</v>
       </c>
       <c r="C344" s="0" t="s">
-        <v>744</v>
+        <v>92</v>
       </c>
       <c r="D344" s="0">
-        <v>1910</v>
+        <v>7986</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="0" t="s">
+        <v>744</v>
+      </c>
+      <c r="B345" s="0" t="s">
         <v>745</v>
       </c>
-      <c r="B345" s="0" t="s">
+      <c r="C345" s="0" t="s">
         <v>746</v>
       </c>
-      <c r="C345" s="0" t="s">
-        <v>151</v>
-      </c>
       <c r="D345" s="0">
-        <v>900</v>
+        <v>1910</v>
       </c>
     </row>
     <row r="346">
@@ -8133,10 +8145,10 @@
         <v>748</v>
       </c>
       <c r="C346" s="0" t="s">
-        <v>21</v>
+        <v>151</v>
       </c>
       <c r="D346" s="0">
-        <v>1722</v>
+        <v>900</v>
       </c>
     </row>
     <row r="347">
@@ -8147,10 +8159,10 @@
         <v>750</v>
       </c>
       <c r="C347" s="0" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="D347" s="0">
-        <v>59000</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="348">
@@ -8161,10 +8173,10 @@
         <v>752</v>
       </c>
       <c r="C348" s="0" t="s">
-        <v>151</v>
+        <v>34</v>
       </c>
       <c r="D348" s="0">
-        <v>750</v>
+        <v>59000</v>
       </c>
     </row>
     <row r="349">
@@ -8178,7 +8190,7 @@
         <v>151</v>
       </c>
       <c r="D349" s="0">
-        <v>1212</v>
+        <v>750</v>
       </c>
     </row>
     <row r="350">
@@ -8192,7 +8204,7 @@
         <v>151</v>
       </c>
       <c r="D350" s="0">
-        <v>1300</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="351">
@@ -8206,7 +8218,7 @@
         <v>151</v>
       </c>
       <c r="D351" s="0">
-        <v>1500</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="352">
@@ -8220,7 +8232,7 @@
         <v>151</v>
       </c>
       <c r="D352" s="0">
-        <v>1400</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="353">
@@ -8231,10 +8243,10 @@
         <v>762</v>
       </c>
       <c r="C353" s="0" t="s">
-        <v>261</v>
+        <v>151</v>
       </c>
       <c r="D353" s="0">
-        <v>11959</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="354">
@@ -8245,10 +8257,10 @@
         <v>764</v>
       </c>
       <c r="C354" s="0" t="s">
-        <v>140</v>
+        <v>261</v>
       </c>
       <c r="D354" s="0">
-        <v>350</v>
+        <v>11959</v>
       </c>
     </row>
     <row r="355">
@@ -8259,10 +8271,10 @@
         <v>766</v>
       </c>
       <c r="C355" s="0" t="s">
-        <v>281</v>
+        <v>140</v>
       </c>
       <c r="D355" s="0">
-        <v>1450</v>
+        <v>350</v>
       </c>
     </row>
     <row r="356">
@@ -8273,10 +8285,10 @@
         <v>768</v>
       </c>
       <c r="C356" s="0" t="s">
-        <v>92</v>
+        <v>281</v>
       </c>
       <c r="D356" s="0">
-        <v>7320.5</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="357">
@@ -8287,10 +8299,10 @@
         <v>770</v>
       </c>
       <c r="C357" s="0" t="s">
-        <v>15</v>
+        <v>92</v>
       </c>
       <c r="D357" s="0">
-        <v>900</v>
+        <v>7320.5</v>
       </c>
     </row>
     <row r="358">
@@ -8301,10 +8313,10 @@
         <v>772</v>
       </c>
       <c r="C358" s="0" t="s">
-        <v>281</v>
+        <v>15</v>
       </c>
       <c r="D358" s="0">
-        <v>566</v>
+        <v>900</v>
       </c>
     </row>
     <row r="359">
@@ -8315,10 +8327,10 @@
         <v>774</v>
       </c>
       <c r="C359" s="0" t="s">
-        <v>469</v>
+        <v>281</v>
       </c>
       <c r="D359" s="0">
-        <v>64925</v>
+        <v>566</v>
       </c>
     </row>
     <row r="360">
@@ -8329,10 +8341,10 @@
         <v>776</v>
       </c>
       <c r="C360" s="0" t="s">
-        <v>15</v>
+        <v>469</v>
       </c>
       <c r="D360" s="0">
-        <v>1100</v>
+        <v>64925</v>
       </c>
     </row>
     <row r="361">
@@ -8343,10 +8355,10 @@
         <v>778</v>
       </c>
       <c r="C361" s="0" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D361" s="0">
-        <v>1623</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="362">
@@ -8357,10 +8369,10 @@
         <v>780</v>
       </c>
       <c r="C362" s="0" t="s">
-        <v>140</v>
+        <v>21</v>
       </c>
       <c r="D362" s="0">
-        <v>1229</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="363">
@@ -8374,7 +8386,7 @@
         <v>140</v>
       </c>
       <c r="D363" s="0">
-        <v>4500</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="364">
@@ -8385,10 +8397,10 @@
         <v>784</v>
       </c>
       <c r="C364" s="0" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="D364" s="0">
-        <v>1250</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="365">
@@ -8402,7 +8414,7 @@
         <v>28</v>
       </c>
       <c r="D365" s="0">
-        <v>1945.1</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="366">
@@ -8413,10 +8425,10 @@
         <v>788</v>
       </c>
       <c r="C366" s="0" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="D366" s="0">
-        <v>450</v>
+        <v>1945.1</v>
       </c>
     </row>
     <row r="367">
@@ -8430,7 +8442,7 @@
         <v>15</v>
       </c>
       <c r="D367" s="0">
-        <v>825</v>
+        <v>450</v>
       </c>
     </row>
     <row r="368">
@@ -8455,10 +8467,10 @@
         <v>794</v>
       </c>
       <c r="C369" s="0" t="s">
-        <v>379</v>
+        <v>15</v>
       </c>
       <c r="D369" s="0">
-        <v>134775.6</v>
+        <v>825</v>
       </c>
     </row>
     <row r="370">
@@ -8472,7 +8484,7 @@
         <v>379</v>
       </c>
       <c r="D370" s="0">
-        <v>175991.55</v>
+        <v>134775.6</v>
       </c>
     </row>
     <row r="371">
@@ -8483,10 +8495,10 @@
         <v>798</v>
       </c>
       <c r="C371" s="0" t="s">
-        <v>70</v>
+        <v>379</v>
       </c>
       <c r="D371" s="0">
-        <v>3427</v>
+        <v>175991.55</v>
       </c>
     </row>
     <row r="372">
@@ -8500,7 +8512,7 @@
         <v>70</v>
       </c>
       <c r="D372" s="0">
-        <v>10618</v>
+        <v>3427</v>
       </c>
     </row>
     <row r="373">
@@ -8511,10 +8523,10 @@
         <v>802</v>
       </c>
       <c r="C373" s="0" t="s">
-        <v>281</v>
+        <v>70</v>
       </c>
       <c r="D373" s="0">
-        <v>515</v>
+        <v>10618</v>
       </c>
     </row>
     <row r="374">
@@ -8525,7 +8537,7 @@
         <v>804</v>
       </c>
       <c r="C374" s="0" t="s">
-        <v>37</v>
+        <v>281</v>
       </c>
       <c r="D374" s="0">
         <v>515</v>
@@ -8539,10 +8551,10 @@
         <v>806</v>
       </c>
       <c r="C375" s="0" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="D375" s="0">
-        <v>9500</v>
+        <v>515</v>
       </c>
     </row>
     <row r="376">
@@ -8553,10 +8565,10 @@
         <v>808</v>
       </c>
       <c r="C376" s="0" t="s">
-        <v>469</v>
+        <v>52</v>
       </c>
       <c r="D376" s="0">
-        <v>207558.08</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="377">
@@ -8570,7 +8582,7 @@
         <v>469</v>
       </c>
       <c r="D377" s="0">
-        <v>249069.69</v>
+        <v>207558.08</v>
       </c>
     </row>
     <row r="378">
@@ -8581,10 +8593,10 @@
         <v>812</v>
       </c>
       <c r="C378" s="0" t="s">
-        <v>70</v>
+        <v>469</v>
       </c>
       <c r="D378" s="0">
-        <v>10522</v>
+        <v>249069.69</v>
       </c>
     </row>
     <row r="379">
@@ -8598,7 +8610,7 @@
         <v>70</v>
       </c>
       <c r="D379" s="0">
-        <v>19481</v>
+        <v>10522</v>
       </c>
     </row>
     <row r="380">
@@ -8609,24 +8621,24 @@
         <v>816</v>
       </c>
       <c r="C380" s="0" t="s">
-        <v>817</v>
+        <v>70</v>
       </c>
       <c r="D380" s="0">
-        <v>1080</v>
+        <v>19481</v>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="0" t="s">
+        <v>817</v>
+      </c>
+      <c r="B381" s="0" t="s">
         <v>818</v>
       </c>
-      <c r="B381" s="0" t="s">
+      <c r="C381" s="0" t="s">
         <v>819</v>
       </c>
-      <c r="C381" s="0" t="s">
-        <v>18</v>
-      </c>
       <c r="D381" s="0">
-        <v>586.49</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="382">
@@ -8637,24 +8649,24 @@
         <v>821</v>
       </c>
       <c r="C382" s="0" t="s">
-        <v>822</v>
+        <v>18</v>
       </c>
       <c r="D382" s="0">
-        <v>520</v>
+        <v>586.49</v>
       </c>
     </row>
     <row r="383">
       <c r="A383" s="0" t="s">
+        <v>822</v>
+      </c>
+      <c r="B383" s="0" t="s">
         <v>823</v>
       </c>
-      <c r="B383" s="0" t="s">
+      <c r="C383" s="0" t="s">
         <v>824</v>
       </c>
-      <c r="C383" s="0" t="s">
-        <v>822</v>
-      </c>
       <c r="D383" s="0">
-        <v>300</v>
+        <v>520</v>
       </c>
     </row>
     <row r="384">
@@ -8665,10 +8677,10 @@
         <v>826</v>
       </c>
       <c r="C384" s="0" t="s">
-        <v>15</v>
+        <v>824</v>
       </c>
       <c r="D384" s="0">
-        <v>2200</v>
+        <v>300</v>
       </c>
     </row>
     <row r="385">
@@ -8682,7 +8694,7 @@
         <v>15</v>
       </c>
       <c r="D385" s="0">
-        <v>2800</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="386">
@@ -8693,10 +8705,10 @@
         <v>830</v>
       </c>
       <c r="C386" s="0" t="s">
-        <v>92</v>
+        <v>15</v>
       </c>
       <c r="D386" s="0">
-        <v>5190.9</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="387">
@@ -8707,10 +8719,10 @@
         <v>832</v>
       </c>
       <c r="C387" s="0" t="s">
-        <v>70</v>
+        <v>92</v>
       </c>
       <c r="D387" s="0">
-        <v>2969</v>
+        <v>5190.9</v>
       </c>
     </row>
     <row r="388">
@@ -8721,10 +8733,10 @@
         <v>834</v>
       </c>
       <c r="C388" s="0" t="s">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="D388" s="0">
-        <v>3800</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="389">
@@ -8735,10 +8747,10 @@
         <v>836</v>
       </c>
       <c r="C389" s="0" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="D389" s="0">
-        <v>4000</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="390">
@@ -8749,24 +8761,24 @@
         <v>838</v>
       </c>
       <c r="C390" s="0" t="s">
-        <v>839</v>
+        <v>15</v>
       </c>
       <c r="D390" s="0">
-        <v>3800</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="0" t="s">
+        <v>839</v>
+      </c>
+      <c r="B391" s="0" t="s">
         <v>840</v>
       </c>
-      <c r="B391" s="0" t="s">
+      <c r="C391" s="0" t="s">
         <v>841</v>
       </c>
-      <c r="C391" s="0" t="s">
-        <v>21</v>
-      </c>
       <c r="D391" s="0">
-        <v>353</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="392">
@@ -8777,10 +8789,10 @@
         <v>843</v>
       </c>
       <c r="C392" s="0" t="s">
-        <v>110</v>
+        <v>21</v>
       </c>
       <c r="D392" s="0">
-        <v>1800</v>
+        <v>353</v>
       </c>
     </row>
     <row r="393">
@@ -8791,10 +8803,10 @@
         <v>845</v>
       </c>
       <c r="C393" s="0" t="s">
-        <v>15</v>
+        <v>110</v>
       </c>
       <c r="D393" s="0">
-        <v>2948</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="394">
@@ -8805,10 +8817,10 @@
         <v>847</v>
       </c>
       <c r="C394" s="0" t="s">
-        <v>92</v>
+        <v>15</v>
       </c>
       <c r="D394" s="0">
-        <v>146.41</v>
+        <v>2948</v>
       </c>
     </row>
     <row r="395">
@@ -8819,10 +8831,10 @@
         <v>849</v>
       </c>
       <c r="C395" s="0" t="s">
-        <v>207</v>
+        <v>92</v>
       </c>
       <c r="D395" s="0">
-        <v>65537</v>
+        <v>146.41</v>
       </c>
     </row>
     <row r="396">
@@ -8833,10 +8845,10 @@
         <v>851</v>
       </c>
       <c r="C396" s="0" t="s">
-        <v>140</v>
+        <v>207</v>
       </c>
       <c r="D396" s="0">
-        <v>4130.4</v>
+        <v>65537</v>
       </c>
     </row>
     <row r="397">
@@ -8850,7 +8862,7 @@
         <v>140</v>
       </c>
       <c r="D397" s="0">
-        <v>4283</v>
+        <v>4130.4</v>
       </c>
     </row>
     <row r="398">
@@ -8864,7 +8876,7 @@
         <v>140</v>
       </c>
       <c r="D398" s="0">
-        <v>6524.8</v>
+        <v>4283</v>
       </c>
     </row>
     <row r="399">
@@ -8875,10 +8887,10 @@
         <v>857</v>
       </c>
       <c r="C399" s="0" t="s">
-        <v>308</v>
+        <v>140</v>
       </c>
       <c r="D399" s="0">
-        <v>570</v>
+        <v>6524.8</v>
       </c>
     </row>
     <row r="400">
@@ -8889,10 +8901,10 @@
         <v>859</v>
       </c>
       <c r="C400" s="0" t="s">
-        <v>70</v>
+        <v>308</v>
       </c>
       <c r="D400" s="0">
-        <v>550</v>
+        <v>570</v>
       </c>
     </row>
     <row r="401">
@@ -8903,10 +8915,10 @@
         <v>861</v>
       </c>
       <c r="C401" s="0" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="D401" s="0">
-        <v>167</v>
+        <v>550</v>
       </c>
     </row>
     <row r="402">
@@ -8917,10 +8929,10 @@
         <v>863</v>
       </c>
       <c r="C402" s="0" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="D402" s="0">
-        <v>714.74</v>
+        <v>158</v>
       </c>
     </row>
     <row r="403">
@@ -8931,10 +8943,10 @@
         <v>865</v>
       </c>
       <c r="C403" s="0" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="D403" s="0">
-        <v>101000</v>
+        <v>714.74</v>
       </c>
     </row>
     <row r="404">
@@ -8945,10 +8957,10 @@
         <v>867</v>
       </c>
       <c r="C404" s="0" t="s">
-        <v>123</v>
+        <v>59</v>
       </c>
       <c r="D404" s="0">
-        <v>6251</v>
+        <v>101000</v>
       </c>
     </row>
     <row r="405">
@@ -8959,10 +8971,10 @@
         <v>869</v>
       </c>
       <c r="C405" s="0" t="s">
-        <v>376</v>
+        <v>123</v>
       </c>
       <c r="D405" s="0">
-        <v>857.67</v>
+        <v>6251</v>
       </c>
     </row>
     <row r="406">
@@ -8973,10 +8985,10 @@
         <v>871</v>
       </c>
       <c r="C406" s="0" t="s">
-        <v>92</v>
+        <v>376</v>
       </c>
       <c r="D406" s="0">
-        <v>1164.66</v>
+        <v>857.67</v>
       </c>
     </row>
     <row r="407">
@@ -8987,10 +8999,10 @@
         <v>873</v>
       </c>
       <c r="C407" s="0" t="s">
-        <v>151</v>
+        <v>92</v>
       </c>
       <c r="D407" s="0">
-        <v>360</v>
+        <v>1164.66</v>
       </c>
     </row>
     <row r="408">
@@ -9004,7 +9016,7 @@
         <v>151</v>
       </c>
       <c r="D408" s="0">
-        <v>450</v>
+        <v>360</v>
       </c>
     </row>
     <row r="409">
@@ -9018,7 +9030,7 @@
         <v>151</v>
       </c>
       <c r="D409" s="0">
-        <v>2150</v>
+        <v>450</v>
       </c>
     </row>
     <row r="410">
@@ -9029,10 +9041,10 @@
         <v>879</v>
       </c>
       <c r="C410" s="0" t="s">
-        <v>580</v>
+        <v>151</v>
       </c>
       <c r="D410" s="0">
-        <v>25192.82</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="411">
@@ -9043,10 +9055,10 @@
         <v>881</v>
       </c>
       <c r="C411" s="0" t="s">
-        <v>70</v>
+        <v>580</v>
       </c>
       <c r="D411" s="0">
-        <v>3500</v>
+        <v>25192.82</v>
       </c>
     </row>
     <row r="412">
@@ -9057,10 +9069,10 @@
         <v>883</v>
       </c>
       <c r="C412" s="0" t="s">
-        <v>175</v>
+        <v>70</v>
       </c>
       <c r="D412" s="0">
-        <v>600</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="413">
@@ -9071,24 +9083,24 @@
         <v>885</v>
       </c>
       <c r="C413" s="0" t="s">
-        <v>886</v>
+        <v>175</v>
       </c>
       <c r="D413" s="0">
-        <v>1080</v>
+        <v>600</v>
       </c>
     </row>
     <row r="414">
       <c r="A414" s="0" t="s">
+        <v>886</v>
+      </c>
+      <c r="B414" s="0" t="s">
         <v>887</v>
       </c>
-      <c r="B414" s="0" t="s">
+      <c r="C414" s="0" t="s">
         <v>888</v>
       </c>
-      <c r="C414" s="0" t="s">
-        <v>338</v>
-      </c>
       <c r="D414" s="0">
-        <v>8628</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="415">
@@ -9099,10 +9111,10 @@
         <v>890</v>
       </c>
       <c r="C415" s="0" t="s">
-        <v>40</v>
+        <v>338</v>
       </c>
       <c r="D415" s="0">
-        <v>27991.54</v>
+        <v>8628</v>
       </c>
     </row>
     <row r="416">
@@ -9113,10 +9125,10 @@
         <v>892</v>
       </c>
       <c r="C416" s="0" t="s">
-        <v>140</v>
+        <v>40</v>
       </c>
       <c r="D416" s="0">
-        <v>1020</v>
+        <v>27991.54</v>
       </c>
     </row>
     <row r="417">
@@ -9130,7 +9142,7 @@
         <v>140</v>
       </c>
       <c r="D417" s="0">
-        <v>4106</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="418">
@@ -9141,10 +9153,10 @@
         <v>896</v>
       </c>
       <c r="C418" s="0" t="s">
-        <v>281</v>
+        <v>140</v>
       </c>
       <c r="D418" s="0">
-        <v>450</v>
+        <v>4106</v>
       </c>
     </row>
     <row r="419">
@@ -9155,10 +9167,10 @@
         <v>898</v>
       </c>
       <c r="C419" s="0" t="s">
-        <v>45</v>
+        <v>281</v>
       </c>
       <c r="D419" s="0">
-        <v>6344.43</v>
+        <v>450</v>
       </c>
     </row>
     <row r="420">
@@ -9172,7 +9184,7 @@
         <v>45</v>
       </c>
       <c r="D420" s="0">
-        <v>2862.28</v>
+        <v>6344.43</v>
       </c>
     </row>
     <row r="421">
@@ -9186,7 +9198,7 @@
         <v>45</v>
       </c>
       <c r="D421" s="0">
-        <v>2131.18</v>
+        <v>2862.28</v>
       </c>
     </row>
     <row r="422">
@@ -9200,7 +9212,7 @@
         <v>45</v>
       </c>
       <c r="D422" s="0">
-        <v>29795.68</v>
+        <v>2131.18</v>
       </c>
     </row>
     <row r="423">
@@ -9214,7 +9226,7 @@
         <v>45</v>
       </c>
       <c r="D423" s="0">
-        <v>2307.09</v>
+        <v>29795.68</v>
       </c>
     </row>
     <row r="424">
@@ -9228,7 +9240,7 @@
         <v>45</v>
       </c>
       <c r="D424" s="0">
-        <v>5249.48</v>
+        <v>2307.09</v>
       </c>
     </row>
     <row r="425">
@@ -9242,7 +9254,7 @@
         <v>45</v>
       </c>
       <c r="D425" s="0">
-        <v>4399.56</v>
+        <v>5249.48</v>
       </c>
     </row>
     <row r="426">
@@ -9253,10 +9265,10 @@
         <v>912</v>
       </c>
       <c r="C426" s="0" t="s">
-        <v>478</v>
+        <v>45</v>
       </c>
       <c r="D426" s="0">
-        <v>510</v>
+        <v>4399.56</v>
       </c>
     </row>
     <row r="427">
@@ -9267,7 +9279,7 @@
         <v>914</v>
       </c>
       <c r="C427" s="0" t="s">
-        <v>37</v>
+        <v>478</v>
       </c>
       <c r="D427" s="0">
         <v>510</v>
@@ -9281,21 +9293,21 @@
         <v>916</v>
       </c>
       <c r="C428" s="0" t="s">
-        <v>917</v>
+        <v>37</v>
       </c>
       <c r="D428" s="0">
-        <v>580</v>
+        <v>510</v>
       </c>
     </row>
     <row r="429">
       <c r="A429" s="0" t="s">
+        <v>917</v>
+      </c>
+      <c r="B429" s="0" t="s">
         <v>918</v>
       </c>
-      <c r="B429" s="0" t="s">
+      <c r="C429" s="0" t="s">
         <v>919</v>
-      </c>
-      <c r="C429" s="0" t="s">
-        <v>917</v>
       </c>
       <c r="D429" s="0">
         <v>580</v>
@@ -9309,7 +9321,7 @@
         <v>921</v>
       </c>
       <c r="C430" s="0" t="s">
-        <v>917</v>
+        <v>919</v>
       </c>
       <c r="D430" s="0">
         <v>580</v>
@@ -9323,10 +9335,10 @@
         <v>923</v>
       </c>
       <c r="C431" s="0" t="s">
-        <v>917</v>
+        <v>919</v>
       </c>
       <c r="D431" s="0">
-        <v>342</v>
+        <v>580</v>
       </c>
     </row>
     <row r="432">
@@ -9337,7 +9349,7 @@
         <v>925</v>
       </c>
       <c r="C432" s="0" t="s">
-        <v>917</v>
+        <v>919</v>
       </c>
       <c r="D432" s="0">
         <v>342</v>
@@ -9351,7 +9363,7 @@
         <v>927</v>
       </c>
       <c r="C433" s="0" t="s">
-        <v>917</v>
+        <v>919</v>
       </c>
       <c r="D433" s="0">
         <v>342</v>
@@ -9365,10 +9377,10 @@
         <v>929</v>
       </c>
       <c r="C434" s="0" t="s">
-        <v>917</v>
+        <v>919</v>
       </c>
       <c r="D434" s="0">
-        <v>0</v>
+        <v>342</v>
       </c>
     </row>
     <row r="435">
@@ -9379,7 +9391,7 @@
         <v>931</v>
       </c>
       <c r="C435" s="0" t="s">
-        <v>917</v>
+        <v>919</v>
       </c>
       <c r="D435" s="0">
         <v>0</v>
@@ -9393,21 +9405,21 @@
         <v>933</v>
       </c>
       <c r="C436" s="0" t="s">
-        <v>934</v>
+        <v>919</v>
       </c>
       <c r="D436" s="0">
-        <v>453</v>
+        <v>0</v>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="0" t="s">
+        <v>934</v>
+      </c>
+      <c r="B437" s="0" t="s">
         <v>935</v>
       </c>
-      <c r="B437" s="0" t="s">
+      <c r="C437" s="0" t="s">
         <v>936</v>
-      </c>
-      <c r="C437" s="0" t="s">
-        <v>917</v>
       </c>
       <c r="D437" s="0">
         <v>453</v>
@@ -9421,10 +9433,10 @@
         <v>938</v>
       </c>
       <c r="C438" s="0" t="s">
-        <v>70</v>
+        <v>919</v>
       </c>
       <c r="D438" s="0">
-        <v>19322</v>
+        <v>453</v>
       </c>
     </row>
     <row r="439">
@@ -9435,10 +9447,10 @@
         <v>940</v>
       </c>
       <c r="C439" s="0" t="s">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="D439" s="0">
-        <v>430</v>
+        <v>19322</v>
       </c>
     </row>
     <row r="440">
@@ -9449,7 +9461,7 @@
         <v>942</v>
       </c>
       <c r="C440" s="0" t="s">
-        <v>281</v>
+        <v>34</v>
       </c>
       <c r="D440" s="0">
         <v>430</v>
@@ -9463,10 +9475,10 @@
         <v>944</v>
       </c>
       <c r="C441" s="0" t="s">
-        <v>115</v>
+        <v>281</v>
       </c>
       <c r="D441" s="0">
-        <v>14000</v>
+        <v>430</v>
       </c>
     </row>
     <row r="442">
@@ -9477,10 +9489,10 @@
         <v>946</v>
       </c>
       <c r="C442" s="0" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="D442" s="0">
-        <v>15400</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="443">
@@ -9491,10 +9503,10 @@
         <v>948</v>
       </c>
       <c r="C443" s="0" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="D443" s="0">
-        <v>266200</v>
+        <v>15400</v>
       </c>
     </row>
     <row r="444">
@@ -9508,7 +9520,7 @@
         <v>92</v>
       </c>
       <c r="D444" s="0">
-        <v>194991.5</v>
+        <v>266200</v>
       </c>
     </row>
     <row r="445">
@@ -9522,7 +9534,7 @@
         <v>92</v>
       </c>
       <c r="D445" s="0">
-        <v>289492.5</v>
+        <v>194991.5</v>
       </c>
     </row>
     <row r="446">
@@ -9533,24 +9545,24 @@
         <v>954</v>
       </c>
       <c r="C446" s="0" t="s">
-        <v>955</v>
+        <v>92</v>
       </c>
       <c r="D446" s="0">
-        <v>13722.52</v>
+        <v>289492.5</v>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="0" t="s">
+        <v>955</v>
+      </c>
+      <c r="B447" s="0" t="s">
         <v>956</v>
       </c>
-      <c r="B447" s="0" t="s">
+      <c r="C447" s="0" t="s">
         <v>957</v>
       </c>
-      <c r="C447" s="0" t="s">
-        <v>955</v>
-      </c>
       <c r="D447" s="0">
-        <v>15072</v>
+        <v>13722.52</v>
       </c>
     </row>
     <row r="448">
@@ -9561,10 +9573,10 @@
         <v>959</v>
       </c>
       <c r="C448" s="0" t="s">
-        <v>955</v>
+        <v>957</v>
       </c>
       <c r="D448" s="0">
-        <v>6555.64</v>
+        <v>15072</v>
       </c>
     </row>
     <row r="449">
@@ -9575,10 +9587,10 @@
         <v>961</v>
       </c>
       <c r="C449" s="0" t="s">
-        <v>955</v>
+        <v>957</v>
       </c>
       <c r="D449" s="0">
-        <v>8964.61</v>
+        <v>6555.64</v>
       </c>
     </row>
     <row r="450">
@@ -9589,10 +9601,10 @@
         <v>963</v>
       </c>
       <c r="C450" s="0" t="s">
-        <v>955</v>
+        <v>957</v>
       </c>
       <c r="D450" s="0">
-        <v>11735</v>
+        <v>8964.61</v>
       </c>
     </row>
     <row r="451">
@@ -9603,10 +9615,10 @@
         <v>965</v>
       </c>
       <c r="C451" s="0" t="s">
-        <v>70</v>
+        <v>957</v>
       </c>
       <c r="D451" s="0">
-        <v>4276</v>
+        <v>11735</v>
       </c>
     </row>
     <row r="452">
@@ -9617,10 +9629,10 @@
         <v>967</v>
       </c>
       <c r="C452" s="0" t="s">
-        <v>140</v>
+        <v>70</v>
       </c>
       <c r="D452" s="0">
-        <v>3930</v>
+        <v>4276</v>
       </c>
     </row>
     <row r="453">
@@ -9631,10 +9643,10 @@
         <v>969</v>
       </c>
       <c r="C453" s="0" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="D453" s="0">
-        <v>4392.3</v>
+        <v>3930</v>
       </c>
     </row>
     <row r="454">
@@ -9645,24 +9657,24 @@
         <v>971</v>
       </c>
       <c r="C454" s="0" t="s">
-        <v>972</v>
+        <v>92</v>
       </c>
       <c r="D454" s="0">
-        <v>5254.41</v>
+        <v>4392.3</v>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="0" t="s">
+        <v>972</v>
+      </c>
+      <c r="B455" s="0" t="s">
         <v>973</v>
       </c>
-      <c r="B455" s="0" t="s">
+      <c r="C455" s="0" t="s">
         <v>974</v>
       </c>
-      <c r="C455" s="0" t="s">
-        <v>52</v>
-      </c>
       <c r="D455" s="0">
-        <v>1200</v>
+        <v>5254.41</v>
       </c>
     </row>
     <row r="456">
@@ -9676,7 +9688,7 @@
         <v>52</v>
       </c>
       <c r="D456" s="0">
-        <v>278</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="457">
@@ -9690,7 +9702,7 @@
         <v>52</v>
       </c>
       <c r="D457" s="0">
-        <v>562</v>
+        <v>278</v>
       </c>
     </row>
     <row r="458">
@@ -9701,10 +9713,10 @@
         <v>980</v>
       </c>
       <c r="C458" s="0" t="s">
-        <v>376</v>
+        <v>52</v>
       </c>
       <c r="D458" s="0">
-        <v>65142.6</v>
+        <v>562</v>
       </c>
     </row>
     <row r="459">
@@ -9718,7 +9730,7 @@
         <v>376</v>
       </c>
       <c r="D459" s="0">
-        <v>23482.7</v>
+        <v>65142.6</v>
       </c>
     </row>
     <row r="460">
@@ -9729,10 +9741,10 @@
         <v>984</v>
       </c>
       <c r="C460" s="0" t="s">
-        <v>28</v>
+        <v>376</v>
       </c>
       <c r="D460" s="0">
-        <v>6029.59</v>
+        <v>23482.7</v>
       </c>
     </row>
     <row r="461">
@@ -9743,10 +9755,10 @@
         <v>986</v>
       </c>
       <c r="C461" s="0" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="D461" s="0">
-        <v>10985</v>
+        <v>6029.59</v>
       </c>
     </row>
     <row r="462">
@@ -9760,7 +9772,7 @@
         <v>52</v>
       </c>
       <c r="D462" s="0">
-        <v>17425</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="463">
@@ -9771,66 +9783,66 @@
         <v>990</v>
       </c>
       <c r="C463" s="0" t="s">
-        <v>991</v>
+        <v>52</v>
       </c>
       <c r="D463" s="0">
-        <v>1958</v>
+        <v>17425</v>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="0" t="s">
+        <v>991</v>
+      </c>
+      <c r="B464" s="0" t="s">
         <v>992</v>
       </c>
-      <c r="B464" s="0" t="s">
+      <c r="C464" s="0" t="s">
         <v>993</v>
       </c>
-      <c r="C464" s="0" t="s">
-        <v>994</v>
-      </c>
       <c r="D464" s="0">
-        <v>2282.3</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="0" t="s">
+        <v>994</v>
+      </c>
+      <c r="B465" s="0" t="s">
         <v>995</v>
       </c>
-      <c r="B465" s="0" t="s">
+      <c r="C465" s="0" t="s">
         <v>996</v>
       </c>
-      <c r="C465" s="0" t="s">
-        <v>997</v>
-      </c>
       <c r="D465" s="0">
-        <v>386</v>
+        <v>2282.3</v>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="0" t="s">
+        <v>997</v>
+      </c>
+      <c r="B466" s="0" t="s">
         <v>998</v>
       </c>
-      <c r="B466" s="0" t="s">
+      <c r="C466" s="0" t="s">
         <v>999</v>
       </c>
-      <c r="C466" s="0" t="s">
-        <v>1000</v>
-      </c>
       <c r="D466" s="0">
-        <v>385.4</v>
+        <v>386</v>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="0" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B467" s="0" t="s">
         <v>1001</v>
       </c>
-      <c r="B467" s="0" t="s">
+      <c r="C467" s="0" t="s">
         <v>1002</v>
       </c>
-      <c r="C467" s="0" t="s">
-        <v>92</v>
-      </c>
       <c r="D467" s="0">
-        <v>296147.5</v>
+        <v>385.4</v>
       </c>
     </row>
     <row r="468">
@@ -9841,10 +9853,10 @@
         <v>1004</v>
       </c>
       <c r="C468" s="0" t="s">
-        <v>580</v>
+        <v>92</v>
       </c>
       <c r="D468" s="0">
-        <v>71176.4</v>
+        <v>296147.5</v>
       </c>
     </row>
     <row r="469">
@@ -9855,10 +9867,10 @@
         <v>1006</v>
       </c>
       <c r="C469" s="0" t="s">
-        <v>140</v>
+        <v>123</v>
       </c>
       <c r="D469" s="0">
-        <v>87</v>
+        <v>1890</v>
       </c>
     </row>
     <row r="470">
@@ -9869,10 +9881,10 @@
         <v>1008</v>
       </c>
       <c r="C470" s="0" t="s">
-        <v>70</v>
+        <v>580</v>
       </c>
       <c r="D470" s="0">
-        <v>950</v>
+        <v>71176.4</v>
       </c>
     </row>
     <row r="471">
@@ -9883,10 +9895,10 @@
         <v>1010</v>
       </c>
       <c r="C471" s="0" t="s">
-        <v>469</v>
+        <v>140</v>
       </c>
       <c r="D471" s="0">
-        <v>342641</v>
+        <v>87</v>
       </c>
     </row>
     <row r="472">
@@ -9897,10 +9909,10 @@
         <v>1012</v>
       </c>
       <c r="C472" s="0" t="s">
-        <v>160</v>
+        <v>70</v>
       </c>
       <c r="D472" s="0">
-        <v>2200</v>
+        <v>950</v>
       </c>
     </row>
     <row r="473">
@@ -9911,10 +9923,10 @@
         <v>1014</v>
       </c>
       <c r="C473" s="0" t="s">
-        <v>478</v>
+        <v>469</v>
       </c>
       <c r="D473" s="0">
-        <v>41000</v>
+        <v>342641</v>
       </c>
     </row>
     <row r="474">
@@ -9925,10 +9937,10 @@
         <v>1016</v>
       </c>
       <c r="C474" s="0" t="s">
-        <v>70</v>
+        <v>160</v>
       </c>
       <c r="D474" s="0">
-        <v>5790</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="475">
@@ -9939,10 +9951,10 @@
         <v>1018</v>
       </c>
       <c r="C475" s="0" t="s">
-        <v>917</v>
+        <v>478</v>
       </c>
       <c r="D475" s="0">
-        <v>880</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="476">
@@ -9953,10 +9965,10 @@
         <v>1020</v>
       </c>
       <c r="C476" s="0" t="s">
-        <v>917</v>
+        <v>70</v>
       </c>
       <c r="D476" s="0">
-        <v>880</v>
+        <v>5790</v>
       </c>
     </row>
     <row r="477">
@@ -9967,7 +9979,7 @@
         <v>1022</v>
       </c>
       <c r="C477" s="0" t="s">
-        <v>917</v>
+        <v>919</v>
       </c>
       <c r="D477" s="0">
         <v>880</v>
@@ -9981,10 +9993,10 @@
         <v>1024</v>
       </c>
       <c r="C478" s="0" t="s">
-        <v>21</v>
+        <v>919</v>
       </c>
       <c r="D478" s="0">
-        <v>563.36</v>
+        <v>880</v>
       </c>
     </row>
     <row r="479">
@@ -9995,10 +10007,10 @@
         <v>1026</v>
       </c>
       <c r="C479" s="0" t="s">
-        <v>15</v>
+        <v>919</v>
       </c>
       <c r="D479" s="0">
-        <v>3520</v>
+        <v>880</v>
       </c>
     </row>
     <row r="480">
@@ -10009,10 +10021,10 @@
         <v>1028</v>
       </c>
       <c r="C480" s="0" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D480" s="0">
-        <v>2600</v>
+        <v>563.36</v>
       </c>
     </row>
     <row r="481">
@@ -10023,10 +10035,10 @@
         <v>1030</v>
       </c>
       <c r="C481" s="0" t="s">
-        <v>281</v>
+        <v>15</v>
       </c>
       <c r="D481" s="0">
-        <v>3700</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="482">
@@ -10037,7 +10049,7 @@
         <v>1032</v>
       </c>
       <c r="C482" s="0" t="s">
-        <v>281</v>
+        <v>15</v>
       </c>
       <c r="D482" s="0">
         <v>2600</v>
@@ -10051,10 +10063,10 @@
         <v>1034</v>
       </c>
       <c r="C483" s="0" t="s">
-        <v>15</v>
+        <v>281</v>
       </c>
       <c r="D483" s="0">
-        <v>2235</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="484">
@@ -10065,10 +10077,10 @@
         <v>1036</v>
       </c>
       <c r="C484" s="0" t="s">
-        <v>15</v>
+        <v>281</v>
       </c>
       <c r="D484" s="0">
-        <v>3850</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="485">
@@ -10079,38 +10091,38 @@
         <v>1038</v>
       </c>
       <c r="C485" s="0" t="s">
-        <v>1039</v>
+        <v>15</v>
       </c>
       <c r="D485" s="0">
-        <v>1</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="0" t="s">
+        <v>1039</v>
+      </c>
+      <c r="B486" s="0" t="s">
         <v>1040</v>
       </c>
-      <c r="B486" s="0" t="s">
-        <v>1041</v>
-      </c>
       <c r="C486" s="0" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="D486" s="0">
-        <v>14819</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="0" t="s">
+        <v>1041</v>
+      </c>
+      <c r="B487" s="0" t="s">
         <v>1042</v>
       </c>
-      <c r="B487" s="0" t="s">
+      <c r="C487" s="0" t="s">
         <v>1043</v>
       </c>
-      <c r="C487" s="0" t="s">
-        <v>376</v>
-      </c>
       <c r="D487" s="0">
-        <v>3859.93</v>
+        <v>1</v>
       </c>
     </row>
     <row r="488">
@@ -10121,10 +10133,10 @@
         <v>1045</v>
       </c>
       <c r="C488" s="0" t="s">
-        <v>376</v>
+        <v>28</v>
       </c>
       <c r="D488" s="0">
-        <v>11751.49</v>
+        <v>14819</v>
       </c>
     </row>
     <row r="489">
@@ -10135,10 +10147,10 @@
         <v>1047</v>
       </c>
       <c r="C489" s="0" t="s">
-        <v>338</v>
+        <v>376</v>
       </c>
       <c r="D489" s="0">
-        <v>6000</v>
+        <v>3859.93</v>
       </c>
     </row>
     <row r="490">
@@ -10149,10 +10161,10 @@
         <v>1049</v>
       </c>
       <c r="C490" s="0" t="s">
-        <v>338</v>
+        <v>376</v>
       </c>
       <c r="D490" s="0">
-        <v>3000</v>
+        <v>11751.49</v>
       </c>
     </row>
     <row r="491">
@@ -10163,10 +10175,10 @@
         <v>1051</v>
       </c>
       <c r="C491" s="0" t="s">
-        <v>37</v>
+        <v>338</v>
       </c>
       <c r="D491" s="0">
-        <v>618</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="492">
@@ -10177,38 +10189,38 @@
         <v>1053</v>
       </c>
       <c r="C492" s="0" t="s">
-        <v>1054</v>
+        <v>338</v>
       </c>
       <c r="D492" s="0">
-        <v>24600</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="0" t="s">
+        <v>1054</v>
+      </c>
+      <c r="B493" s="0" t="s">
         <v>1055</v>
       </c>
-      <c r="B493" s="0" t="s">
-        <v>1056</v>
-      </c>
       <c r="C493" s="0" t="s">
-        <v>105</v>
+        <v>37</v>
       </c>
       <c r="D493" s="0">
-        <v>0</v>
+        <v>618</v>
       </c>
     </row>
     <row r="494">
       <c r="A494" s="0" t="s">
+        <v>1056</v>
+      </c>
+      <c r="B494" s="0" t="s">
         <v>1057</v>
       </c>
-      <c r="B494" s="0" t="s">
+      <c r="C494" s="0" t="s">
         <v>1058</v>
       </c>
-      <c r="C494" s="0" t="s">
-        <v>92</v>
-      </c>
       <c r="D494" s="0">
-        <v>43590.25</v>
+        <v>24600</v>
       </c>
     </row>
     <row r="495">
@@ -10219,10 +10231,10 @@
         <v>1060</v>
       </c>
       <c r="C495" s="0" t="s">
-        <v>469</v>
+        <v>105</v>
       </c>
       <c r="D495" s="0">
-        <v>207558.07</v>
+        <v>0</v>
       </c>
     </row>
     <row r="496">
@@ -10233,10 +10245,10 @@
         <v>1062</v>
       </c>
       <c r="C496" s="0" t="s">
-        <v>376</v>
+        <v>92</v>
       </c>
       <c r="D496" s="0">
-        <v>77429.29</v>
+        <v>43590.25</v>
       </c>
     </row>
     <row r="497">
@@ -10247,10 +10259,10 @@
         <v>1064</v>
       </c>
       <c r="C497" s="0" t="s">
-        <v>376</v>
+        <v>469</v>
       </c>
       <c r="D497" s="0">
-        <v>42913.42</v>
+        <v>207558.07</v>
       </c>
     </row>
     <row r="498">
@@ -10264,7 +10276,7 @@
         <v>376</v>
       </c>
       <c r="D498" s="0">
-        <v>88806.25</v>
+        <v>77429.29</v>
       </c>
     </row>
     <row r="499">
@@ -10278,7 +10290,7 @@
         <v>376</v>
       </c>
       <c r="D499" s="0">
-        <v>50781.52</v>
+        <v>42913.42</v>
       </c>
     </row>
     <row r="500">
@@ -10289,10 +10301,10 @@
         <v>1070</v>
       </c>
       <c r="C500" s="0" t="s">
-        <v>21</v>
+        <v>376</v>
       </c>
       <c r="D500" s="0">
-        <v>1600</v>
+        <v>88806.25</v>
       </c>
     </row>
     <row r="501">
@@ -10303,10 +10315,10 @@
         <v>1072</v>
       </c>
       <c r="C501" s="0" t="s">
-        <v>28</v>
+        <v>376</v>
       </c>
       <c r="D501" s="0">
-        <v>3455.8</v>
+        <v>50781.52</v>
       </c>
     </row>
     <row r="502">
@@ -10317,10 +10329,10 @@
         <v>1074</v>
       </c>
       <c r="C502" s="0" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D502" s="0">
-        <v>3987</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="503">
@@ -10334,7 +10346,7 @@
         <v>28</v>
       </c>
       <c r="D503" s="0">
-        <v>4010.17</v>
+        <v>3455.8</v>
       </c>
     </row>
     <row r="504">
@@ -10348,7 +10360,7 @@
         <v>28</v>
       </c>
       <c r="D504" s="0">
-        <v>3382.65</v>
+        <v>3987</v>
       </c>
     </row>
     <row r="505">
@@ -10359,10 +10371,10 @@
         <v>1080</v>
       </c>
       <c r="C505" s="0" t="s">
-        <v>160</v>
+        <v>28</v>
       </c>
       <c r="D505" s="0">
-        <v>430</v>
+        <v>4010.17</v>
       </c>
     </row>
     <row r="506">
@@ -10373,9 +10385,37 @@
         <v>1082</v>
       </c>
       <c r="C506" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="D506" s="0">
+        <v>3382.65</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="0" t="s">
+        <v>1083</v>
+      </c>
+      <c r="B507" s="0" t="s">
+        <v>1084</v>
+      </c>
+      <c r="C507" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="D507" s="0">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="0" t="s">
+        <v>1085</v>
+      </c>
+      <c r="B508" s="0" t="s">
+        <v>1086</v>
+      </c>
+      <c r="C508" s="0" t="s">
         <v>140</v>
       </c>
-      <c r="D506" s="0">
+      <c r="D508" s="0">
         <v>465</v>
       </c>
     </row>

</xml_diff>